<commit_message>
Auto: update momentum data - 2026-09-15 08:58 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ANOND-RE</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>146.25</v>
+        <v>21.2</v>
       </c>
       <c r="C2" t="n">
-        <v>180</v>
+        <v>25.44</v>
       </c>
       <c r="D2" t="n">
-        <v>23.08</v>
+        <v>20</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LADDERUP</t>
+          <t>MPEL-RE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61.93</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>73</v>
+        <v>2.4</v>
       </c>
       <c r="D3" t="n">
-        <v>17.88</v>
+        <v>20</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>TATACHEM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48.93</v>
+        <v>612.45</v>
       </c>
       <c r="C4" t="n">
-        <v>53.2</v>
+        <v>734.9</v>
       </c>
       <c r="D4" t="n">
-        <v>8.73</v>
+        <v>19.99</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.13</v>
+        <v>17.2</v>
       </c>
       <c r="C5" t="n">
-        <v>0.14</v>
+        <v>19.4</v>
       </c>
       <c r="D5" t="n">
-        <v>7.69</v>
+        <v>12.79</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>AFCONS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>94.95999999999999</v>
+        <v>253.8</v>
       </c>
       <c r="C6" t="n">
-        <v>101.15</v>
+        <v>281</v>
       </c>
       <c r="D6" t="n">
-        <v>6.52</v>
+        <v>10.72</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SHANKESH</t>
+          <t>PANCHMAHQ</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>98.41</v>
+        <v>280</v>
       </c>
       <c r="C7" t="n">
-        <v>104.4</v>
+        <v>309.8</v>
       </c>
       <c r="D7" t="n">
-        <v>6.09</v>
+        <v>10.64</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5.95</v>
+        <v>34.74</v>
       </c>
       <c r="C8" t="n">
-        <v>6.28</v>
+        <v>37.9</v>
       </c>
       <c r="D8" t="n">
-        <v>5.55</v>
+        <v>9.1</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRAVISSHO</t>
+          <t>LADDERUP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>35.59</v>
+        <v>74.31</v>
       </c>
       <c r="C9" t="n">
-        <v>37.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>5.37</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>QUICKHEAL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58.83</v>
+        <v>147.52</v>
       </c>
       <c r="C10" t="n">
-        <v>61.98</v>
+        <v>160</v>
       </c>
       <c r="D10" t="n">
-        <v>5.35</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7.03</v>
+        <v>494.05</v>
       </c>
       <c r="C11" t="n">
-        <v>7.4</v>
+        <v>535</v>
       </c>
       <c r="D11" t="n">
-        <v>5.26</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>17.56</v>
+        <v>2.1</v>
       </c>
       <c r="C12" t="n">
-        <v>18.48</v>
+        <v>2.27</v>
       </c>
       <c r="D12" t="n">
-        <v>5.24</v>
+        <v>8.1</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SOMICONVEY</t>
+          <t>GRAVISSHO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>92.76000000000001</v>
+        <v>42.7</v>
       </c>
       <c r="C13" t="n">
-        <v>97.59999999999999</v>
+        <v>46.15</v>
       </c>
       <c r="D13" t="n">
-        <v>5.22</v>
+        <v>8.08</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MVKAGRO</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>287.2</v>
+        <v>0.13</v>
       </c>
       <c r="C14" t="n">
-        <v>301.55</v>
+        <v>0.14</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>7.69</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SHANTIINOR</t>
+          <t>TATAINVEST</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>176.15</v>
+        <v>650.9</v>
       </c>
       <c r="C15" t="n">
-        <v>184.95</v>
+        <v>700.15</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>7.57</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TECHLABS</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>134.05</v>
+        <v>19.57</v>
       </c>
       <c r="C16" t="n">
-        <v>140.75</v>
+        <v>21.05</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>7.56</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KORE</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>165.05</v>
+        <v>14.96</v>
       </c>
       <c r="C17" t="n">
-        <v>173.3</v>
+        <v>16.03</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>7.15</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>ASIANTNE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>314.67</v>
+        <v>9.25</v>
       </c>
       <c r="C18" t="n">
-        <v>330.4</v>
+        <v>9.9</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>7.03</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SETL</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>445.9</v>
+        <v>301.1</v>
       </c>
       <c r="C19" t="n">
-        <v>468.15</v>
+        <v>320</v>
       </c>
       <c r="D19" t="n">
-        <v>4.99</v>
+        <v>6.28</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>181.3</v>
+        <v>15.01</v>
       </c>
       <c r="C20" t="n">
-        <v>190.35</v>
+        <v>15.94</v>
       </c>
       <c r="D20" t="n">
-        <v>4.99</v>
+        <v>6.2</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>81.53</v>
+        <v>4.28</v>
       </c>
       <c r="C21" t="n">
-        <v>85.59999999999999</v>
+        <v>4.54</v>
       </c>
       <c r="D21" t="n">
-        <v>4.99</v>
+        <v>6.07</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ATMASTCO</t>
+          <t>BALAXI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>128.6</v>
+        <v>23.39</v>
       </c>
       <c r="C22" t="n">
-        <v>135</v>
+        <v>24.8</v>
       </c>
       <c r="D22" t="n">
-        <v>4.98</v>
+        <v>6.03</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SUMAX</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>120.45</v>
+        <v>19.33</v>
       </c>
       <c r="C23" t="n">
-        <v>126.45</v>
+        <v>20.45</v>
       </c>
       <c r="D23" t="n">
-        <v>4.98</v>
+        <v>5.79</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>POLYSIL</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>85.40000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="C24" t="n">
-        <v>89.65000000000001</v>
+        <v>9.25</v>
       </c>
       <c r="D24" t="n">
-        <v>4.98</v>
+        <v>5.47</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAL</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>46.4</v>
+        <v>6.78</v>
       </c>
       <c r="C25" t="n">
-        <v>48.7</v>
+        <v>7.15</v>
       </c>
       <c r="D25" t="n">
-        <v>4.96</v>
+        <v>5.46</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>GILLANDERS</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>19.96</v>
+        <v>103.58</v>
       </c>
       <c r="C26" t="n">
-        <v>20.95</v>
+        <v>109</v>
       </c>
       <c r="D26" t="n">
-        <v>4.96</v>
+        <v>5.23</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16.78</v>
+        <v>67.08</v>
       </c>
       <c r="C27" t="n">
-        <v>17.61</v>
+        <v>70.5</v>
       </c>
       <c r="D27" t="n">
-        <v>4.95</v>
+        <v>5.1</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>YOGI</t>
+          <t>KEC</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>155.37</v>
+        <v>406.4</v>
       </c>
       <c r="C28" t="n">
-        <v>162.9</v>
+        <v>427.1</v>
       </c>
       <c r="D28" t="n">
-        <v>4.85</v>
+        <v>5.09</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>SUMEDHA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>67.84</v>
+        <v>41.4</v>
       </c>
       <c r="C29" t="n">
-        <v>71</v>
+        <v>43.49</v>
       </c>
       <c r="D29" t="n">
-        <v>4.66</v>
+        <v>5.05</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.43</v>
+        <v>125</v>
       </c>
       <c r="C30" t="n">
-        <v>0.45</v>
+        <v>131.25</v>
       </c>
       <c r="D30" t="n">
-        <v>4.65</v>
+        <v>5</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>COMPINFO</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1.08</v>
+        <v>526.3</v>
       </c>
       <c r="C31" t="n">
-        <v>1.13</v>
+        <v>552.6</v>
       </c>
       <c r="D31" t="n">
-        <v>4.63</v>
+        <v>5</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.73</v>
+        <v>206.64</v>
       </c>
       <c r="C32" t="n">
-        <v>1.81</v>
+        <v>216.97</v>
       </c>
       <c r="D32" t="n">
-        <v>4.62</v>
+        <v>5</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TOKYOPLAST</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>76.81</v>
+        <v>12.01</v>
       </c>
       <c r="C33" t="n">
-        <v>80.29000000000001</v>
+        <v>12.61</v>
       </c>
       <c r="D33" t="n">
-        <v>4.53</v>
+        <v>5</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TECHNOCRAF</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>439.4</v>
+        <v>330.4</v>
       </c>
       <c r="C34" t="n">
-        <v>459.15</v>
+        <v>346.92</v>
       </c>
       <c r="D34" t="n">
-        <v>4.49</v>
+        <v>5</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SETUINFRA</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.67</v>
+        <v>169.64</v>
       </c>
       <c r="C35" t="n">
-        <v>0.7</v>
+        <v>178.12</v>
       </c>
       <c r="D35" t="n">
-        <v>4.48</v>
+        <v>5</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>FIDEL</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>139.75</v>
+        <v>36.6</v>
       </c>
       <c r="C36" t="n">
-        <v>146</v>
+        <v>38.43</v>
       </c>
       <c r="D36" t="n">
-        <v>4.47</v>
+        <v>5</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OPTIFIN</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>14.57</v>
+        <v>17.61</v>
       </c>
       <c r="C37" t="n">
-        <v>15.22</v>
+        <v>18.49</v>
       </c>
       <c r="D37" t="n">
-        <v>4.46</v>
+        <v>5</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>ARCL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>24.33</v>
+        <v>249.9</v>
       </c>
       <c r="C38" t="n">
-        <v>25.4</v>
+        <v>262.39</v>
       </c>
       <c r="D38" t="n">
-        <v>4.4</v>
+        <v>5</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>SUMAX</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>189.49</v>
+        <v>126.45</v>
       </c>
       <c r="C39" t="n">
-        <v>197.75</v>
+        <v>132.75</v>
       </c>
       <c r="D39" t="n">
-        <v>4.36</v>
+        <v>4.98</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>8.029999999999999</v>
+        <v>26.14</v>
       </c>
       <c r="C40" t="n">
-        <v>8.380000000000001</v>
+        <v>27.44</v>
       </c>
       <c r="D40" t="n">
-        <v>4.36</v>
+        <v>4.97</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>SHANTIINOR</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1.15</v>
+        <v>184.95</v>
       </c>
       <c r="C41" t="n">
-        <v>1.2</v>
+        <v>194.15</v>
       </c>
       <c r="D41" t="n">
-        <v>4.35</v>
+        <v>4.97</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DIGJAMLMTD</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>61.84</v>
+        <v>20.95</v>
       </c>
       <c r="C42" t="n">
-        <v>64.5</v>
+        <v>21.99</v>
       </c>
       <c r="D42" t="n">
-        <v>4.3</v>
+        <v>4.96</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7.82</v>
+        <v>1.01</v>
       </c>
       <c r="C43" t="n">
-        <v>8.15</v>
+        <v>1.06</v>
       </c>
       <c r="D43" t="n">
-        <v>4.22</v>
+        <v>4.95</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>40.93</v>
+        <v>1.82</v>
       </c>
       <c r="C44" t="n">
-        <v>42.5</v>
+        <v>1.91</v>
       </c>
       <c r="D44" t="n">
-        <v>3.84</v>
+        <v>4.95</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>VIJSOLX</t>
+          <t>AARADHYA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>625.9</v>
+        <v>141.55</v>
       </c>
       <c r="C45" t="n">
-        <v>649.8</v>
+        <v>148.55</v>
       </c>
       <c r="D45" t="n">
-        <v>3.82</v>
+        <v>4.95</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>LEENEE</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2.36</v>
+        <v>7.9</v>
       </c>
       <c r="C46" t="n">
-        <v>2.45</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="D46" t="n">
-        <v>3.81</v>
+        <v>4.94</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>NTCIND</t>
+          <t>MAL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>131.7</v>
+        <v>48.7</v>
       </c>
       <c r="C47" t="n">
-        <v>136.7</v>
+        <v>51.1</v>
       </c>
       <c r="D47" t="n">
-        <v>3.8</v>
+        <v>4.93</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>35.79</v>
+        <v>16.87</v>
       </c>
       <c r="C48" t="n">
-        <v>37.09</v>
+        <v>17.68</v>
       </c>
       <c r="D48" t="n">
-        <v>3.63</v>
+        <v>4.8</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.28</v>
+        <v>1756.7</v>
       </c>
       <c r="C49" t="n">
-        <v>0.29</v>
+        <v>1841</v>
       </c>
       <c r="D49" t="n">
-        <v>3.57</v>
+        <v>4.8</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MEGASTAR</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>284.95</v>
+        <v>26.03</v>
       </c>
       <c r="C50" t="n">
-        <v>295</v>
+        <v>27.28</v>
       </c>
       <c r="D50" t="n">
-        <v>3.53</v>
+        <v>4.8</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.29</v>
+        <v>156.56</v>
       </c>
       <c r="C51" t="n">
-        <v>0.3</v>
+        <v>164</v>
       </c>
       <c r="D51" t="n">
-        <v>3.45</v>
+        <v>4.75</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CELEBRITY</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>6.72</v>
+        <v>38.38</v>
       </c>
       <c r="C52" t="n">
-        <v>6.95</v>
+        <v>40.2</v>
       </c>
       <c r="D52" t="n">
-        <v>3.42</v>
+        <v>4.74</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>4.97</v>
+        <v>13.31</v>
       </c>
       <c r="C53" t="n">
-        <v>5.14</v>
+        <v>13.94</v>
       </c>
       <c r="D53" t="n">
-        <v>3.42</v>
+        <v>4.73</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>RSDFIN</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1.49</v>
+        <v>94</v>
       </c>
       <c r="C54" t="n">
-        <v>1.54</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="D54" t="n">
-        <v>3.36</v>
+        <v>4.68</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>LAKPRE</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>175.14</v>
+        <v>6</v>
       </c>
       <c r="C55" t="n">
-        <v>180.99</v>
+        <v>6.28</v>
       </c>
       <c r="D55" t="n">
-        <v>3.34</v>
+        <v>4.67</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>CELEBRITY</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>10.87</v>
+        <v>6.85</v>
       </c>
       <c r="C56" t="n">
-        <v>11.23</v>
+        <v>7.17</v>
       </c>
       <c r="D56" t="n">
-        <v>3.31</v>
+        <v>4.67</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>BPLPHARMA</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>34.86</v>
+        <v>1505.1</v>
       </c>
       <c r="C57" t="n">
-        <v>36</v>
+        <v>1575</v>
       </c>
       <c r="D57" t="n">
-        <v>3.27</v>
+        <v>4.64</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DEVIT</t>
+          <t>DCAL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>23.97</v>
+        <v>167.25</v>
       </c>
       <c r="C58" t="n">
-        <v>24.75</v>
+        <v>174.99</v>
       </c>
       <c r="D58" t="n">
-        <v>3.25</v>
+        <v>4.63</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ACEINTEG</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>17.89</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="C59" t="n">
-        <v>18.47</v>
+        <v>8.59</v>
       </c>
       <c r="D59" t="n">
-        <v>3.24</v>
+        <v>4.63</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>18.45</v>
+        <v>34.41</v>
       </c>
       <c r="C60" t="n">
-        <v>19.04</v>
+        <v>36</v>
       </c>
       <c r="D60" t="n">
-        <v>3.2</v>
+        <v>4.62</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2878.6</v>
+        <v>1037.7</v>
       </c>
       <c r="C61" t="n">
-        <v>2970</v>
+        <v>1085</v>
       </c>
       <c r="D61" t="n">
-        <v>3.18</v>
+        <v>4.56</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SHIVAUM</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>461.45</v>
+        <v>0.66</v>
       </c>
       <c r="C62" t="n">
-        <v>476</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D62" t="n">
-        <v>3.15</v>
+        <v>4.55</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.97</v>
+        <v>16.74</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>17.5</v>
       </c>
       <c r="D63" t="n">
-        <v>3.09</v>
+        <v>4.54</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>NAHARPOLY</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>233.77</v>
+        <v>2.44</v>
       </c>
       <c r="C64" t="n">
-        <v>240.92</v>
+        <v>2.55</v>
       </c>
       <c r="D64" t="n">
-        <v>3.06</v>
+        <v>4.51</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>SHREEDHAR</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>44.55</v>
+        <v>135.8</v>
       </c>
       <c r="C65" t="n">
-        <v>45.9</v>
+        <v>141.9</v>
       </c>
       <c r="D65" t="n">
-        <v>3.03</v>
+        <v>4.49</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MONOLITH</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1446.4</v>
+        <v>0.45</v>
       </c>
       <c r="C66" t="n">
-        <v>1490</v>
+        <v>0.47</v>
       </c>
       <c r="D66" t="n">
-        <v>3.01</v>
+        <v>4.44</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>LAMOSAIC</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>154.5</v>
+        <v>53.1</v>
       </c>
       <c r="C67" t="n">
-        <v>159</v>
+        <v>55.45</v>
       </c>
       <c r="D67" t="n">
-        <v>2.91</v>
+        <v>4.43</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>30.04</v>
+        <v>6.2</v>
       </c>
       <c r="C68" t="n">
-        <v>30.9</v>
+        <v>6.47</v>
       </c>
       <c r="D68" t="n">
-        <v>2.86</v>
+        <v>4.35</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>DIGISPICE</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>16.53</v>
+        <v>5.75</v>
       </c>
       <c r="C69" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D69" t="n">
-        <v>2.84</v>
+        <v>4.35</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LOTUSDEV</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>207.88</v>
+        <v>13.42</v>
       </c>
       <c r="C70" t="n">
-        <v>213.7</v>
+        <v>14</v>
       </c>
       <c r="D70" t="n">
-        <v>2.8</v>
+        <v>4.32</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ORIENTLTD</t>
+          <t>A2ZINFRA</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>81.73</v>
+        <v>15.33</v>
       </c>
       <c r="C71" t="n">
-        <v>84</v>
+        <v>15.99</v>
       </c>
       <c r="D71" t="n">
-        <v>2.78</v>
+        <v>4.31</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>FLFL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.72</v>
+        <v>1.16</v>
       </c>
       <c r="C72" t="n">
-        <v>0.74</v>
+        <v>1.21</v>
       </c>
       <c r="D72" t="n">
-        <v>2.78</v>
+        <v>4.31</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>AKASH</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>3.99</v>
+        <v>24.86</v>
       </c>
       <c r="C73" t="n">
-        <v>4.1</v>
+        <v>25.93</v>
       </c>
       <c r="D73" t="n">
-        <v>2.76</v>
+        <v>4.3</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BIOFILCHEM</t>
+          <t>KRITI</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>36.79</v>
+        <v>61.4</v>
       </c>
       <c r="C74" t="n">
-        <v>37.8</v>
+        <v>64</v>
       </c>
       <c r="D74" t="n">
-        <v>2.75</v>
+        <v>4.23</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S&amp;SPOWER</t>
+          <t>SHRJAGP</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>342.6</v>
+        <v>647</v>
       </c>
       <c r="C75" t="n">
-        <v>352</v>
+        <v>673.95</v>
       </c>
       <c r="D75" t="n">
-        <v>2.74</v>
+        <v>4.17</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>15.97</v>
+        <v>297.1</v>
       </c>
       <c r="C76" t="n">
-        <v>16.4</v>
+        <v>309.25</v>
       </c>
       <c r="D76" t="n">
-        <v>2.69</v>
+        <v>4.09</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>AVIENCE</t>
+          <t>RRIL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>346.8</v>
+        <v>15.99</v>
       </c>
       <c r="C77" t="n">
-        <v>356.1</v>
+        <v>16.64</v>
       </c>
       <c r="D77" t="n">
-        <v>2.68</v>
+        <v>4.07</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>6.37</v>
+        <v>86.5</v>
       </c>
       <c r="C78" t="n">
-        <v>6.54</v>
+        <v>90</v>
       </c>
       <c r="D78" t="n">
-        <v>2.67</v>
+        <v>4.05</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>STEELXIND</t>
+          <t>PREMCO</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>12.17</v>
+        <v>394</v>
       </c>
       <c r="C79" t="n">
-        <v>12.49</v>
+        <v>409.95</v>
       </c>
       <c r="D79" t="n">
-        <v>2.63</v>
+        <v>4.05</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ORICONENT</t>
+          <t>NIMBSPROJ</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>51.65</v>
+        <v>165.25</v>
       </c>
       <c r="C80" t="n">
-        <v>53</v>
+        <v>171.86</v>
       </c>
       <c r="D80" t="n">
-        <v>2.61</v>
+        <v>4</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>4.29</v>
+        <v>785.05</v>
       </c>
       <c r="C81" t="n">
-        <v>4.4</v>
+        <v>816</v>
       </c>
       <c r="D81" t="n">
-        <v>2.56</v>
+        <v>3.94</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AARADHYA</t>
+          <t>PATELENG</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>140.95</v>
+        <v>26.61</v>
       </c>
       <c r="C82" t="n">
-        <v>144.5</v>
+        <v>27.65</v>
       </c>
       <c r="D82" t="n">
-        <v>2.52</v>
+        <v>3.91</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>PML</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>13.11</v>
+        <v>482.45</v>
       </c>
       <c r="C83" t="n">
-        <v>13.44</v>
+        <v>500.95</v>
       </c>
       <c r="D83" t="n">
-        <v>2.52</v>
+        <v>3.83</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1.2</v>
+        <v>3828.3</v>
       </c>
       <c r="C84" t="n">
-        <v>1.23</v>
+        <v>3974.6</v>
       </c>
       <c r="D84" t="n">
-        <v>2.5</v>
+        <v>3.82</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MAHAPEXLTD</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>56.23</v>
+        <v>1206.1</v>
       </c>
       <c r="C85" t="n">
-        <v>57.63</v>
+        <v>1252</v>
       </c>
       <c r="D85" t="n">
-        <v>2.49</v>
+        <v>3.81</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2.41</v>
+        <v>157.98</v>
       </c>
       <c r="C86" t="n">
-        <v>2.47</v>
+        <v>164</v>
       </c>
       <c r="D86" t="n">
-        <v>2.49</v>
+        <v>3.81</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>8.050000000000001</v>
+        <v>25.14</v>
       </c>
       <c r="C87" t="n">
-        <v>8.25</v>
+        <v>26.09</v>
       </c>
       <c r="D87" t="n">
-        <v>2.48</v>
+        <v>3.78</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>MOHITIND</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>16.3</v>
+        <v>23.23</v>
       </c>
       <c r="C88" t="n">
-        <v>16.7</v>
+        <v>24.1</v>
       </c>
       <c r="D88" t="n">
-        <v>2.45</v>
+        <v>3.75</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>36.61</v>
+        <v>1098.6</v>
       </c>
       <c r="C89" t="n">
-        <v>37.5</v>
+        <v>1139.8</v>
       </c>
       <c r="D89" t="n">
-        <v>2.43</v>
+        <v>3.75</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>178.67</v>
+        <v>43.28</v>
       </c>
       <c r="C90" t="n">
-        <v>182.99</v>
+        <v>44.89</v>
       </c>
       <c r="D90" t="n">
-        <v>2.42</v>
+        <v>3.72</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DHATRE</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>4.14</v>
+        <v>23.71</v>
       </c>
       <c r="C91" t="n">
-        <v>4.24</v>
+        <v>24.59</v>
       </c>
       <c r="D91" t="n">
-        <v>2.42</v>
+        <v>3.71</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>23.34</v>
+        <v>8.18</v>
       </c>
       <c r="C92" t="n">
-        <v>23.9</v>
+        <v>8.48</v>
       </c>
       <c r="D92" t="n">
-        <v>2.4</v>
+        <v>3.67</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MOLBIO</t>
+          <t>SUBAHOTELS</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1509.4</v>
+        <v>101.2</v>
       </c>
       <c r="C93" t="n">
-        <v>1545</v>
+        <v>104.9</v>
       </c>
       <c r="D93" t="n">
-        <v>2.36</v>
+        <v>3.66</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>DISHTV</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>5.99</v>
+        <v>2.5</v>
       </c>
       <c r="C94" t="n">
-        <v>6.13</v>
+        <v>2.59</v>
       </c>
       <c r="D94" t="n">
-        <v>2.34</v>
+        <v>3.6</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>AMDIND</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>590.2</v>
+        <v>64.03</v>
       </c>
       <c r="C95" t="n">
-        <v>604</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="D95" t="n">
-        <v>2.34</v>
+        <v>3.53</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ITDC</t>
+          <t>ENKEIWHEL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>664.6</v>
+        <v>399</v>
       </c>
       <c r="C96" t="n">
-        <v>679.95</v>
+        <v>412.95</v>
       </c>
       <c r="D96" t="n">
-        <v>2.31</v>
+        <v>3.5</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>KREBSBIO</t>
+          <t>YATHARTH</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>61.47</v>
+        <v>966.3</v>
       </c>
       <c r="C97" t="n">
-        <v>62.89</v>
+        <v>1000</v>
       </c>
       <c r="D97" t="n">
-        <v>2.31</v>
+        <v>3.49</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>FINKURVE</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>37.93</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="C98" t="n">
-        <v>38.8</v>
+        <v>75</v>
       </c>
       <c r="D98" t="n">
-        <v>2.29</v>
+        <v>3.46</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>254.25</v>
+        <v>12.74</v>
       </c>
       <c r="C99" t="n">
-        <v>260</v>
+        <v>13.18</v>
       </c>
       <c r="D99" t="n">
-        <v>2.26</v>
+        <v>3.45</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DCMSIL</t>
+          <t>MOHITE</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>72.36</v>
+        <v>2.63</v>
       </c>
       <c r="C100" t="n">
-        <v>73.98999999999999</v>
+        <v>2.72</v>
       </c>
       <c r="D100" t="n">
-        <v>2.25</v>
+        <v>3.42</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>ESDS</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>162.34</v>
+        <v>1740.4</v>
       </c>
       <c r="C101" t="n">
-        <v>165.9</v>
+        <v>1800</v>
       </c>
       <c r="D101" t="n">
-        <v>2.19</v>
+        <v>3.42</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>RELCHEMQ</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>7.8</v>
+        <v>110.23</v>
       </c>
       <c r="C102" t="n">
-        <v>7.97</v>
+        <v>114</v>
       </c>
       <c r="D102" t="n">
-        <v>2.18</v>
+        <v>3.42</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>TRANSCOR</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>135.95</v>
+        <v>25.39</v>
       </c>
       <c r="C103" t="n">
-        <v>138.9</v>
+        <v>26.25</v>
       </c>
       <c r="D103" t="n">
-        <v>2.17</v>
+        <v>3.39</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>43.07</v>
+        <v>2200.8</v>
       </c>
       <c r="C104" t="n">
-        <v>44</v>
+        <v>2275.5</v>
       </c>
       <c r="D104" t="n">
-        <v>2.16</v>
+        <v>3.39</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SONAMLTD</t>
+          <t>NTCIND</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>73.54000000000001</v>
+        <v>134.91</v>
       </c>
       <c r="C105" t="n">
-        <v>75.09999999999999</v>
+        <v>139.45</v>
       </c>
       <c r="D105" t="n">
-        <v>2.12</v>
+        <v>3.37</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BRNL</t>
+          <t>CHAVDA</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>16.65</v>
+        <v>125.3</v>
       </c>
       <c r="C106" t="n">
-        <v>17</v>
+        <v>129.5</v>
       </c>
       <c r="D106" t="n">
-        <v>2.1</v>
+        <v>3.35</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TECHD</t>
+          <t>SONATSOFTW</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>601.4</v>
+        <v>265.85</v>
       </c>
       <c r="C107" t="n">
-        <v>614</v>
+        <v>274.75</v>
       </c>
       <c r="D107" t="n">
-        <v>2.1</v>
+        <v>3.35</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>6.21</v>
+        <v>156.75</v>
       </c>
       <c r="C108" t="n">
-        <v>6.34</v>
+        <v>162</v>
       </c>
       <c r="D108" t="n">
-        <v>2.09</v>
+        <v>3.35</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>BSOFT</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1.91</v>
+        <v>281.65</v>
       </c>
       <c r="C109" t="n">
-        <v>1.95</v>
+        <v>291</v>
       </c>
       <c r="D109" t="n">
-        <v>2.09</v>
+        <v>3.32</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>DHUNINV</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.48</v>
+        <v>995</v>
       </c>
       <c r="C110" t="n">
-        <v>0.49</v>
+        <v>1028</v>
       </c>
       <c r="D110" t="n">
-        <v>2.08</v>
+        <v>3.32</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CHENNPETRO</t>
+          <t>AZADIND</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>1626.4</v>
+        <v>87.13</v>
       </c>
       <c r="C111" t="n">
-        <v>1660</v>
+        <v>90</v>
       </c>
       <c r="D111" t="n">
-        <v>2.07</v>
+        <v>3.29</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>372.15</v>
+        <v>40.86</v>
       </c>
       <c r="C112" t="n">
-        <v>379.8</v>
+        <v>42.2</v>
       </c>
       <c r="D112" t="n">
-        <v>2.06</v>
+        <v>3.28</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>PSRAJ</t>
+          <t>ASHUTOSH</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>94.90000000000001</v>
+        <v>164.5</v>
       </c>
       <c r="C113" t="n">
-        <v>96.84999999999999</v>
+        <v>169.9</v>
       </c>
       <c r="D113" t="n">
-        <v>2.05</v>
+        <v>3.28</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>19.1</v>
+        <v>5375.5</v>
       </c>
       <c r="C114" t="n">
-        <v>19.49</v>
+        <v>5550</v>
       </c>
       <c r="D114" t="n">
-        <v>2.04</v>
+        <v>3.25</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>DIACABS</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>24.8</v>
+        <v>369.05</v>
       </c>
       <c r="C115" t="n">
-        <v>25.3</v>
+        <v>381</v>
       </c>
       <c r="D115" t="n">
-        <v>2.02</v>
+        <v>3.24</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>126.46</v>
+        <v>91.64</v>
       </c>
       <c r="C116" t="n">
-        <v>129</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="D116" t="n">
-        <v>2.01</v>
+        <v>3.23</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>MWL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>299.95</v>
+        <v>40.6</v>
       </c>
       <c r="C117" t="n">
-        <v>305.95</v>
+        <v>41.9</v>
       </c>
       <c r="D117" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>AMARJOTHI</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.5</v>
+        <v>150.14</v>
       </c>
       <c r="C118" t="n">
-        <v>0.51</v>
+        <v>154.93</v>
       </c>
       <c r="D118" t="n">
-        <v>2</v>
+        <v>3.19</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GYFTR</t>
+          <t>NOVAAGRI</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>185.32</v>
+        <v>22.7</v>
       </c>
       <c r="C119" t="n">
-        <v>189</v>
+        <v>23.42</v>
       </c>
       <c r="D119" t="n">
-        <v>1.99</v>
+        <v>3.17</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>KAMDHENU</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>39.22</v>
+        <v>16.13</v>
       </c>
       <c r="C120" t="n">
-        <v>40</v>
+        <v>16.64</v>
       </c>
       <c r="D120" t="n">
-        <v>1.99</v>
+        <v>3.16</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CTE</t>
+          <t>DECNGOLD</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>42.24</v>
+        <v>229.73</v>
       </c>
       <c r="C121" t="n">
-        <v>43.08</v>
+        <v>237</v>
       </c>
       <c r="D121" t="n">
-        <v>1.99</v>
+        <v>3.16</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RAMANEWS</t>
+          <t>WATERBASE</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>32.15</v>
+        <v>46.54</v>
       </c>
       <c r="C122" t="n">
-        <v>32.79</v>
+        <v>48</v>
       </c>
       <c r="D122" t="n">
-        <v>1.99</v>
+        <v>3.14</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>22.21</v>
+        <v>463.45</v>
       </c>
       <c r="C123" t="n">
-        <v>22.65</v>
+        <v>477.95</v>
       </c>
       <c r="D123" t="n">
-        <v>1.98</v>
+        <v>3.13</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>BALKRISHNA</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.51</v>
+        <v>16.1</v>
       </c>
       <c r="C124" t="n">
-        <v>0.52</v>
+        <v>16.6</v>
       </c>
       <c r="D124" t="n">
-        <v>1.96</v>
+        <v>3.11</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>TNPETRO</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>77.2</v>
+        <v>128.9</v>
       </c>
       <c r="C125" t="n">
-        <v>78.69</v>
+        <v>132.9</v>
       </c>
       <c r="D125" t="n">
-        <v>1.93</v>
+        <v>3.1</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ROML</t>
+          <t>AYE</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>42.13</v>
+        <v>179.46</v>
       </c>
       <c r="C126" t="n">
-        <v>42.94</v>
+        <v>185</v>
       </c>
       <c r="D126" t="n">
-        <v>1.92</v>
+        <v>3.09</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>NEUEON</t>
+          <t>MVKAGRO</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>12.05</v>
+        <v>299.8</v>
       </c>
       <c r="C127" t="n">
-        <v>12.28</v>
+        <v>309</v>
       </c>
       <c r="D127" t="n">
-        <v>1.91</v>
+        <v>3.07</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>JINDRILL</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>654.2</v>
+        <v>366.7</v>
       </c>
       <c r="C128" t="n">
-        <v>666.65</v>
+        <v>377.95</v>
       </c>
       <c r="D128" t="n">
-        <v>1.9</v>
+        <v>3.07</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>59.87</v>
+        <v>62.97</v>
       </c>
       <c r="C129" t="n">
-        <v>61</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D129" t="n">
-        <v>1.89</v>
+        <v>3.06</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>1.6</v>
+        <v>5.55</v>
       </c>
       <c r="C130" t="n">
-        <v>1.63</v>
+        <v>5.72</v>
       </c>
       <c r="D130" t="n">
-        <v>1.87</v>
+        <v>3.06</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>2.15</v>
+        <v>65.69</v>
       </c>
       <c r="C131" t="n">
-        <v>2.19</v>
+        <v>67.7</v>
       </c>
       <c r="D131" t="n">
-        <v>1.86</v>
+        <v>3.06</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MIIL</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>687.2</v>
+        <v>1541</v>
       </c>
       <c r="C132" t="n">
-        <v>699.95</v>
+        <v>1588</v>
       </c>
       <c r="D132" t="n">
-        <v>1.86</v>
+        <v>3.05</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>LTM</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>261</v>
+        <v>4275</v>
       </c>
       <c r="C133" t="n">
-        <v>265.8</v>
+        <v>4404.3</v>
       </c>
       <c r="D133" t="n">
-        <v>1.84</v>
+        <v>3.02</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>PANORAMA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>2.19</v>
+        <v>53.78</v>
       </c>
       <c r="C134" t="n">
-        <v>2.23</v>
+        <v>55.4</v>
       </c>
       <c r="D134" t="n">
-        <v>1.83</v>
+        <v>3.01</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GVKPIL</t>
+          <t>DCM</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>2.21</v>
+        <v>75</v>
       </c>
       <c r="C135" t="n">
-        <v>2.25</v>
+        <v>77.25</v>
       </c>
       <c r="D135" t="n">
-        <v>1.81</v>
+        <v>3</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SIKKO</t>
+          <t>CALSOFT</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>5.56</v>
+        <v>38.74</v>
       </c>
       <c r="C136" t="n">
-        <v>5.66</v>
+        <v>39.9</v>
       </c>
       <c r="D136" t="n">
-        <v>1.8</v>
+        <v>2.99</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3435,13 +3435,13 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>23.37</v>
+        <v>23.5</v>
       </c>
       <c r="C137" t="n">
-        <v>23.79</v>
+        <v>24.2</v>
       </c>
       <c r="D137" t="n">
-        <v>1.8</v>
+        <v>2.98</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>BSOFT</t>
+          <t>VALIANTORG</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>275.8</v>
+        <v>396.3</v>
       </c>
       <c r="C138" t="n">
-        <v>280.75</v>
+        <v>408</v>
       </c>
       <c r="D138" t="n">
-        <v>1.79</v>
+        <v>2.95</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>854.75</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="C139" t="n">
-        <v>870</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D139" t="n">
-        <v>1.78</v>
+        <v>2.94</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>SUDEEPPHRM</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1.69</v>
+        <v>1202.8</v>
       </c>
       <c r="C140" t="n">
-        <v>1.72</v>
+        <v>1238</v>
       </c>
       <c r="D140" t="n">
-        <v>1.78</v>
+        <v>2.93</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SHREERAMA</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>45.88</v>
+        <v>7.18</v>
       </c>
       <c r="C141" t="n">
-        <v>46.69</v>
+        <v>7.39</v>
       </c>
       <c r="D141" t="n">
-        <v>1.77</v>
+        <v>2.92</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.57</v>
+        <v>132.17</v>
       </c>
       <c r="C142" t="n">
-        <v>0.58</v>
+        <v>136</v>
       </c>
       <c r="D142" t="n">
-        <v>1.75</v>
+        <v>2.9</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>TENNIND</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>8.01</v>
+        <v>506.35</v>
       </c>
       <c r="C143" t="n">
-        <v>8.15</v>
+        <v>521</v>
       </c>
       <c r="D143" t="n">
-        <v>1.75</v>
+        <v>2.89</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>PRAMODINI</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>127.2</v>
+        <v>167.4</v>
       </c>
       <c r="C144" t="n">
-        <v>129.4</v>
+        <v>172.2</v>
       </c>
       <c r="D144" t="n">
-        <v>1.73</v>
+        <v>2.87</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>KALYANIFRG</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>973.2</v>
+        <v>10.19</v>
       </c>
       <c r="C145" t="n">
-        <v>990</v>
+        <v>10.48</v>
       </c>
       <c r="D145" t="n">
-        <v>1.73</v>
+        <v>2.85</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SINGERIND</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>74.02</v>
+        <v>364.65</v>
       </c>
       <c r="C146" t="n">
-        <v>75.3</v>
+        <v>375</v>
       </c>
       <c r="D146" t="n">
-        <v>1.73</v>
+        <v>2.84</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RPEL</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>1743.5</v>
+        <v>455.1</v>
       </c>
       <c r="C147" t="n">
-        <v>1773.5</v>
+        <v>468</v>
       </c>
       <c r="D147" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>NDL</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>2.9</v>
+        <v>583.55</v>
       </c>
       <c r="C148" t="n">
-        <v>2.95</v>
+        <v>600.05</v>
       </c>
       <c r="D148" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SAHYADRI</t>
+          <t>BIMETAL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>383.35</v>
+        <v>640.5</v>
       </c>
       <c r="C149" t="n">
-        <v>389.9</v>
+        <v>658.65</v>
       </c>
       <c r="D149" t="n">
-        <v>1.71</v>
+        <v>2.83</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>WOMANCART</t>
+          <t>ARROWGREEN</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>100</v>
+        <v>813</v>
       </c>
       <c r="C150" t="n">
-        <v>101.7</v>
+        <v>835.9</v>
       </c>
       <c r="D150" t="n">
-        <v>1.7</v>
+        <v>2.82</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>EMAMILTD</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1.78</v>
+        <v>363.8</v>
       </c>
       <c r="C151" t="n">
-        <v>1.81</v>
+        <v>374</v>
       </c>
       <c r="D151" t="n">
-        <v>1.69</v>
+        <v>2.8</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>14.75</v>
+        <v>5.72</v>
       </c>
       <c r="C152" t="n">
-        <v>15</v>
+        <v>5.88</v>
       </c>
       <c r="D152" t="n">
-        <v>1.69</v>
+        <v>2.8</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>11.31</v>
+        <v>466.9</v>
       </c>
       <c r="C153" t="n">
-        <v>11.5</v>
+        <v>479.9</v>
       </c>
       <c r="D153" t="n">
-        <v>1.68</v>
+        <v>2.78</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>MSPL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>5.37</v>
+        <v>33.96</v>
       </c>
       <c r="C154" t="n">
-        <v>5.46</v>
+        <v>34.9</v>
       </c>
       <c r="D154" t="n">
-        <v>1.68</v>
+        <v>2.77</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>14.15</v>
+        <v>4.33</v>
       </c>
       <c r="C155" t="n">
-        <v>14.38</v>
+        <v>4.45</v>
       </c>
       <c r="D155" t="n">
-        <v>1.63</v>
+        <v>2.77</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>24.11</v>
+        <v>540.45</v>
       </c>
       <c r="C156" t="n">
-        <v>24.5</v>
+        <v>555.3</v>
       </c>
       <c r="D156" t="n">
-        <v>1.62</v>
+        <v>2.75</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ANDREWYU</t>
+          <t>JAYBEE</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>26.77</v>
+        <v>83.7</v>
       </c>
       <c r="C157" t="n">
-        <v>27.2</v>
+        <v>86</v>
       </c>
       <c r="D157" t="n">
-        <v>1.61</v>
+        <v>2.75</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.63</v>
+        <v>78.3</v>
       </c>
       <c r="C158" t="n">
-        <v>0.64</v>
+        <v>80.43000000000001</v>
       </c>
       <c r="D158" t="n">
-        <v>1.59</v>
+        <v>2.72</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MOLDTECH</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>13.87</v>
+        <v>207.39</v>
       </c>
       <c r="C159" t="n">
-        <v>14.09</v>
+        <v>213</v>
       </c>
       <c r="D159" t="n">
-        <v>1.59</v>
+        <v>2.71</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>DENORA</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>1.9</v>
+        <v>798.45</v>
       </c>
       <c r="C160" t="n">
-        <v>1.93</v>
+        <v>820</v>
       </c>
       <c r="D160" t="n">
-        <v>1.58</v>
+        <v>2.7</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>1.9</v>
+        <v>0.37</v>
       </c>
       <c r="C161" t="n">
-        <v>1.93</v>
+        <v>0.38</v>
       </c>
       <c r="D161" t="n">
-        <v>1.58</v>
+        <v>2.7</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SWANDEF</t>
+          <t>TUTIALKA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>2662.8</v>
+        <v>59.19</v>
       </c>
       <c r="C162" t="n">
-        <v>2705</v>
+        <v>60.79</v>
       </c>
       <c r="D162" t="n">
-        <v>1.58</v>
+        <v>2.7</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>2.53</v>
+        <v>198.93</v>
       </c>
       <c r="C163" t="n">
-        <v>2.57</v>
+        <v>204.28</v>
       </c>
       <c r="D163" t="n">
-        <v>1.58</v>
+        <v>2.69</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>DHARIWAL</t>
+          <t>LOTUSDEV</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>29.05</v>
+        <v>209.27</v>
       </c>
       <c r="C164" t="n">
-        <v>29.5</v>
+        <v>214.88</v>
       </c>
       <c r="D164" t="n">
-        <v>1.55</v>
+        <v>2.68</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>SHERA</t>
+          <t>ITL</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>190.8</v>
+        <v>369.25</v>
       </c>
       <c r="C165" t="n">
-        <v>193.75</v>
+        <v>378.95</v>
       </c>
       <c r="D165" t="n">
-        <v>1.55</v>
+        <v>2.63</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>OIL</t>
+          <t>HLEGLAS</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>500.3</v>
+        <v>404.35</v>
       </c>
       <c r="C166" t="n">
-        <v>508</v>
+        <v>415</v>
       </c>
       <c r="D166" t="n">
-        <v>1.54</v>
+        <v>2.63</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ZTECH</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>452</v>
+        <v>2.28</v>
       </c>
       <c r="C167" t="n">
-        <v>458.95</v>
+        <v>2.34</v>
       </c>
       <c r="D167" t="n">
-        <v>1.54</v>
+        <v>2.63</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>DIACABS</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>351.5</v>
+        <v>646.3</v>
       </c>
       <c r="C168" t="n">
-        <v>356.8</v>
+        <v>663.2</v>
       </c>
       <c r="D168" t="n">
-        <v>1.51</v>
+        <v>2.61</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>ELANTAS</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>134.49</v>
+        <v>14513</v>
       </c>
       <c r="C169" t="n">
-        <v>136.5</v>
+        <v>14890</v>
       </c>
       <c r="D169" t="n">
-        <v>1.49</v>
+        <v>2.6</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>44.25</v>
+        <v>723.15</v>
       </c>
       <c r="C170" t="n">
-        <v>44.9</v>
+        <v>741.9</v>
       </c>
       <c r="D170" t="n">
-        <v>1.47</v>
+        <v>2.59</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MRPL</t>
+          <t>TECHD</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>181.32</v>
+        <v>605.3</v>
       </c>
       <c r="C171" t="n">
-        <v>183.99</v>
+        <v>621</v>
       </c>
       <c r="D171" t="n">
-        <v>1.47</v>
+        <v>2.59</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>MUKKA</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>55.89</v>
+        <v>32.17</v>
       </c>
       <c r="C172" t="n">
-        <v>56.7</v>
+        <v>33</v>
       </c>
       <c r="D172" t="n">
-        <v>1.45</v>
+        <v>2.58</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>CHEMCRUX</t>
+          <t>SHARDAMOTR</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>85.52</v>
+        <v>943.75</v>
       </c>
       <c r="C173" t="n">
-        <v>86.75</v>
+        <v>968</v>
       </c>
       <c r="D173" t="n">
-        <v>1.44</v>
+        <v>2.57</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>9.869999999999999</v>
+        <v>24.18</v>
       </c>
       <c r="C174" t="n">
-        <v>10.01</v>
+        <v>24.8</v>
       </c>
       <c r="D174" t="n">
-        <v>1.42</v>
+        <v>2.56</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>FAIRCHEMOR</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>98.61</v>
+        <v>623.95</v>
       </c>
       <c r="C175" t="n">
-        <v>100</v>
+        <v>639.9</v>
       </c>
       <c r="D175" t="n">
-        <v>1.41</v>
+        <v>2.56</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>517.1</v>
+        <v>118.98</v>
       </c>
       <c r="C176" t="n">
-        <v>524.4</v>
+        <v>122</v>
       </c>
       <c r="D176" t="n">
-        <v>1.41</v>
+        <v>2.54</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>BIL</t>
+          <t>ENIL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>1081.7</v>
+        <v>101.24</v>
       </c>
       <c r="C177" t="n">
-        <v>1097</v>
+        <v>103.8</v>
       </c>
       <c r="D177" t="n">
-        <v>1.41</v>
+        <v>2.53</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>MPHASIS</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>20.71</v>
+        <v>2295</v>
       </c>
       <c r="C178" t="n">
-        <v>21</v>
+        <v>2353</v>
       </c>
       <c r="D178" t="n">
-        <v>1.4</v>
+        <v>2.53</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>PERSISTENT</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>30.58</v>
+        <v>5516</v>
       </c>
       <c r="C179" t="n">
-        <v>31</v>
+        <v>5654</v>
       </c>
       <c r="D179" t="n">
-        <v>1.37</v>
+        <v>2.5</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>SWSOLAR</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.74</v>
+        <v>180.22</v>
       </c>
       <c r="C180" t="n">
-        <v>0.75</v>
+        <v>184.7</v>
       </c>
       <c r="D180" t="n">
-        <v>1.35</v>
+        <v>2.49</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>MANCREDIT</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>218.58</v>
+        <v>2.01</v>
       </c>
       <c r="C181" t="n">
-        <v>221.5</v>
+        <v>2.06</v>
       </c>
       <c r="D181" t="n">
-        <v>1.34</v>
+        <v>2.49</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ISGEC</t>
+          <t>BELLACASA</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>810.15</v>
+        <v>256.52</v>
       </c>
       <c r="C182" t="n">
-        <v>821</v>
+        <v>262.86</v>
       </c>
       <c r="D182" t="n">
-        <v>1.34</v>
+        <v>2.47</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>63.85</v>
+        <v>165.32</v>
       </c>
       <c r="C183" t="n">
-        <v>64.7</v>
+        <v>169.4</v>
       </c>
       <c r="D183" t="n">
-        <v>1.33</v>
+        <v>2.47</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MANAKSTEEL</t>
+          <t>HEIDELBERG</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>115.01</v>
+        <v>149.8</v>
       </c>
       <c r="C184" t="n">
-        <v>116.5</v>
+        <v>153.5</v>
       </c>
       <c r="D184" t="n">
-        <v>1.3</v>
+        <v>2.47</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>SPLIL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>384.5</v>
+        <v>30.05</v>
       </c>
       <c r="C185" t="n">
-        <v>389.45</v>
+        <v>30.79</v>
       </c>
       <c r="D185" t="n">
-        <v>1.29</v>
+        <v>2.46</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>37.69</v>
+        <v>16.69</v>
       </c>
       <c r="C186" t="n">
-        <v>38.17</v>
+        <v>17.1</v>
       </c>
       <c r="D186" t="n">
-        <v>1.27</v>
+        <v>2.46</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>7.11</v>
+        <v>39.46</v>
       </c>
       <c r="C187" t="n">
-        <v>7.2</v>
+        <v>40.43</v>
       </c>
       <c r="D187" t="n">
-        <v>1.27</v>
+        <v>2.46</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MARATHON</t>
+          <t>XTRANET</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>438.5</v>
+        <v>271.34</v>
       </c>
       <c r="C188" t="n">
-        <v>444</v>
+        <v>278</v>
       </c>
       <c r="D188" t="n">
-        <v>1.25</v>
+        <v>2.45</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ORIRAIL</t>
+          <t>VISHAL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>122.3</v>
+        <v>18.36</v>
       </c>
       <c r="C189" t="n">
-        <v>123.8</v>
+        <v>18.81</v>
       </c>
       <c r="D189" t="n">
-        <v>1.23</v>
+        <v>2.45</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ASTAR</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>587.75</v>
+        <v>45.88</v>
       </c>
       <c r="C190" t="n">
-        <v>595</v>
+        <v>47</v>
       </c>
       <c r="D190" t="n">
-        <v>1.23</v>
+        <v>2.44</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>AVANCE</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>0.82</v>
+        <v>190.35</v>
       </c>
       <c r="C191" t="n">
-        <v>0.83</v>
+        <v>195</v>
       </c>
       <c r="D191" t="n">
-        <v>1.22</v>
+        <v>2.44</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>AMNPLST</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>167.92</v>
+        <v>46.86</v>
       </c>
       <c r="C192" t="n">
-        <v>169.95</v>
+        <v>48</v>
       </c>
       <c r="D192" t="n">
-        <v>1.21</v>
+        <v>2.43</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>14.9</v>
+        <v>62.29</v>
       </c>
       <c r="C193" t="n">
-        <v>15.08</v>
+        <v>63.8</v>
       </c>
       <c r="D193" t="n">
-        <v>1.21</v>
+        <v>2.42</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>AXISCADES</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>71.05</v>
+        <v>1831.8</v>
       </c>
       <c r="C194" t="n">
-        <v>71.90000000000001</v>
+        <v>1876.2</v>
       </c>
       <c r="D194" t="n">
-        <v>1.2</v>
+        <v>2.42</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>SIGACHI</t>
+          <t>SIKKO</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>37.56</v>
+        <v>5.83</v>
       </c>
       <c r="C195" t="n">
-        <v>38</v>
+        <v>5.97</v>
       </c>
       <c r="D195" t="n">
-        <v>1.17</v>
+        <v>2.4</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>RUBFILA</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>68.09</v>
+        <v>135.08</v>
       </c>
       <c r="C196" t="n">
-        <v>68.89</v>
+        <v>138.32</v>
       </c>
       <c r="D196" t="n">
-        <v>1.17</v>
+        <v>2.4</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>ADVANIHOTR</t>
+          <t>SUBEXLTD</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>48.43</v>
+        <v>20.8</v>
       </c>
       <c r="C197" t="n">
-        <v>48.99</v>
+        <v>21.3</v>
       </c>
       <c r="D197" t="n">
-        <v>1.16</v>
+        <v>2.4</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>14.92</v>
+        <v>17.09</v>
       </c>
       <c r="C198" t="n">
-        <v>15.09</v>
+        <v>17.5</v>
       </c>
       <c r="D198" t="n">
-        <v>1.14</v>
+        <v>2.4</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>3.54</v>
+        <v>87.41</v>
       </c>
       <c r="C199" t="n">
-        <v>3.58</v>
+        <v>89.5</v>
       </c>
       <c r="D199" t="n">
-        <v>1.13</v>
+        <v>2.39</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ESDS</t>
+          <t>CMICABLES</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>1582.2</v>
+        <v>2.51</v>
       </c>
       <c r="C200" t="n">
-        <v>1600</v>
+        <v>2.57</v>
       </c>
       <c r="D200" t="n">
-        <v>1.13</v>
+        <v>2.39</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>MEGATHERM</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>34.9</v>
+        <v>251</v>
       </c>
       <c r="C201" t="n">
-        <v>35.29</v>
+        <v>257</v>
       </c>
       <c r="D201" t="n">
-        <v>1.12</v>
+        <v>2.39</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-16 08:51 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,14 +461,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>RCDL-RE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>21.2</v>
+        <v>2.5</v>
       </c>
       <c r="C2" t="n">
-        <v>25.44</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>20</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MPEL-RE</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>48.24</v>
       </c>
       <c r="C3" t="n">
-        <v>2.4</v>
+        <v>57.88</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>19.98</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TATACHEM</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>612.45</v>
+        <v>5.18</v>
       </c>
       <c r="C4" t="n">
-        <v>734.9</v>
+        <v>5.98</v>
       </c>
       <c r="D4" t="n">
-        <v>19.99</v>
+        <v>15.44</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>SHRADHA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17.2</v>
+        <v>29.97</v>
       </c>
       <c r="C5" t="n">
-        <v>19.4</v>
+        <v>33.88</v>
       </c>
       <c r="D5" t="n">
-        <v>12.79</v>
+        <v>13.05</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AFCONS</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>253.8</v>
+        <v>389.55</v>
       </c>
       <c r="C6" t="n">
-        <v>281</v>
+        <v>428.5</v>
       </c>
       <c r="D6" t="n">
-        <v>10.72</v>
+        <v>10</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PANCHMAHQ</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>280</v>
+        <v>44.94</v>
       </c>
       <c r="C7" t="n">
-        <v>309.8</v>
+        <v>49.43</v>
       </c>
       <c r="D7" t="n">
-        <v>10.64</v>
+        <v>9.99</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SUPREME</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>34.74</v>
+        <v>20.89</v>
       </c>
       <c r="C8" t="n">
-        <v>37.9</v>
+        <v>22.89</v>
       </c>
       <c r="D8" t="n">
-        <v>9.1</v>
+        <v>9.57</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LADDERUP</t>
+          <t>MPEL-RE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>74.31</v>
+        <v>1.6</v>
       </c>
       <c r="C9" t="n">
-        <v>80.90000000000001</v>
+        <v>1.75</v>
       </c>
       <c r="D9" t="n">
-        <v>8.869999999999999</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>QUICKHEAL</t>
+          <t>HBPOR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>147.52</v>
+        <v>59.99</v>
       </c>
       <c r="C10" t="n">
-        <v>160</v>
+        <v>65</v>
       </c>
       <c r="D10" t="n">
-        <v>8.460000000000001</v>
+        <v>8.35</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>494.05</v>
+        <v>4.53</v>
       </c>
       <c r="C11" t="n">
-        <v>535</v>
+        <v>4.9</v>
       </c>
       <c r="D11" t="n">
-        <v>8.289999999999999</v>
+        <v>8.17</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>SAICAPI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.1</v>
+        <v>154.5</v>
       </c>
       <c r="C12" t="n">
-        <v>2.27</v>
+        <v>167</v>
       </c>
       <c r="D12" t="n">
-        <v>8.1</v>
+        <v>8.09</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GRAVISSHO</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>42.7</v>
+        <v>0.13</v>
       </c>
       <c r="C13" t="n">
-        <v>46.15</v>
+        <v>0.14</v>
       </c>
       <c r="D13" t="n">
-        <v>8.08</v>
+        <v>7.69</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>PRAKASHSTL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.13</v>
+        <v>3.56</v>
       </c>
       <c r="C14" t="n">
-        <v>0.14</v>
+        <v>3.82</v>
       </c>
       <c r="D14" t="n">
-        <v>7.69</v>
+        <v>7.3</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TATAINVEST</t>
+          <t>HMAAGRO</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>650.9</v>
+        <v>23.41</v>
       </c>
       <c r="C15" t="n">
-        <v>700.15</v>
+        <v>24.99</v>
       </c>
       <c r="D15" t="n">
-        <v>7.57</v>
+        <v>6.75</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>RADIANTCMS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>19.57</v>
+        <v>35.89</v>
       </c>
       <c r="C16" t="n">
-        <v>21.05</v>
+        <v>38.24</v>
       </c>
       <c r="D16" t="n">
-        <v>7.56</v>
+        <v>6.55</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>14.96</v>
+        <v>200.86</v>
       </c>
       <c r="C17" t="n">
-        <v>16.03</v>
+        <v>213.99</v>
       </c>
       <c r="D17" t="n">
-        <v>7.15</v>
+        <v>6.54</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASIANTNE</t>
+          <t>RTSPOWR</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>9.25</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="C18" t="n">
-        <v>9.9</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="D18" t="n">
-        <v>7.03</v>
+        <v>6.39</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>301.1</v>
+        <v>1.58</v>
       </c>
       <c r="C19" t="n">
-        <v>320</v>
+        <v>1.68</v>
       </c>
       <c r="D19" t="n">
-        <v>6.28</v>
+        <v>6.33</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15.01</v>
+        <v>25.44</v>
       </c>
       <c r="C20" t="n">
-        <v>15.94</v>
+        <v>26.99</v>
       </c>
       <c r="D20" t="n">
-        <v>6.2</v>
+        <v>6.09</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4.28</v>
+        <v>29.34</v>
       </c>
       <c r="C21" t="n">
-        <v>4.54</v>
+        <v>31.1</v>
       </c>
       <c r="D21" t="n">
-        <v>6.07</v>
+        <v>6</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BALAXI</t>
+          <t>PAYTM</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>23.39</v>
+        <v>1730</v>
       </c>
       <c r="C22" t="n">
-        <v>24.8</v>
+        <v>1830</v>
       </c>
       <c r="D22" t="n">
-        <v>6.03</v>
+        <v>5.78</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>19.33</v>
+        <v>14.08</v>
       </c>
       <c r="C23" t="n">
-        <v>20.45</v>
+        <v>14.89</v>
       </c>
       <c r="D23" t="n">
-        <v>5.79</v>
+        <v>5.75</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8.77</v>
+        <v>1639.5</v>
       </c>
       <c r="C24" t="n">
-        <v>9.25</v>
+        <v>1730</v>
       </c>
       <c r="D24" t="n">
-        <v>5.47</v>
+        <v>5.52</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>CMSINFO</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6.78</v>
+        <v>222.91</v>
       </c>
       <c r="C25" t="n">
-        <v>7.15</v>
+        <v>235.08</v>
       </c>
       <c r="D25" t="n">
         <v>5.46</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GILLANDERS</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>103.58</v>
+        <v>592.85</v>
       </c>
       <c r="C26" t="n">
-        <v>109</v>
+        <v>625</v>
       </c>
       <c r="D26" t="n">
-        <v>5.23</v>
+        <v>5.42</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>67.08</v>
+        <v>0.19</v>
       </c>
       <c r="C27" t="n">
-        <v>70.5</v>
+        <v>0.2</v>
       </c>
       <c r="D27" t="n">
-        <v>5.1</v>
+        <v>5.26</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KEC</t>
+          <t>SILVER001</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>406.4</v>
+        <v>23</v>
       </c>
       <c r="C28" t="n">
-        <v>427.1</v>
+        <v>24.2</v>
       </c>
       <c r="D28" t="n">
-        <v>5.09</v>
+        <v>5.22</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SUMEDHA</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>41.4</v>
+        <v>279</v>
       </c>
       <c r="C29" t="n">
-        <v>43.49</v>
+        <v>292.95</v>
       </c>
       <c r="D29" t="n">
-        <v>5.05</v>
+        <v>5</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,14 +1077,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>ARCL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>125</v>
+        <v>262.39</v>
       </c>
       <c r="C30" t="n">
-        <v>131.25</v>
+        <v>275.5</v>
       </c>
       <c r="D30" t="n">
         <v>5</v>
@@ -1099,14 +1099,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>526.3</v>
+        <v>178.12</v>
       </c>
       <c r="C31" t="n">
-        <v>552.6</v>
+        <v>187.02</v>
       </c>
       <c r="D31" t="n">
         <v>5</v>
@@ -1121,14 +1121,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>206.64</v>
+        <v>346.92</v>
       </c>
       <c r="C32" t="n">
-        <v>216.97</v>
+        <v>364.26</v>
       </c>
       <c r="D32" t="n">
         <v>5</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>12.01</v>
+        <v>97.56999999999999</v>
       </c>
       <c r="C33" t="n">
-        <v>12.61</v>
+        <v>102.44</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>330.4</v>
+        <v>366.65</v>
       </c>
       <c r="C34" t="n">
-        <v>346.92</v>
+        <v>384.95</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>169.64</v>
+        <v>27.44</v>
       </c>
       <c r="C35" t="n">
-        <v>178.12</v>
+        <v>28.81</v>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>36.6</v>
+        <v>18.49</v>
       </c>
       <c r="C36" t="n">
-        <v>38.43</v>
+        <v>19.41</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>BIKEWO</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>17.61</v>
+        <v>105.2</v>
       </c>
       <c r="C37" t="n">
-        <v>18.49</v>
+        <v>110.4</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>4.94</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ARCL</t>
+          <t>FLEXITUFF</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>249.9</v>
+        <v>2.24</v>
       </c>
       <c r="C38" t="n">
-        <v>262.39</v>
+        <v>2.35</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>4.91</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SUMAX</t>
+          <t>SUNSHINE</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>126.45</v>
+        <v>333.95</v>
       </c>
       <c r="C39" t="n">
-        <v>132.75</v>
+        <v>350.15</v>
       </c>
       <c r="D39" t="n">
-        <v>4.98</v>
+        <v>4.85</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>26.14</v>
+        <v>15.27</v>
       </c>
       <c r="C40" t="n">
-        <v>27.44</v>
+        <v>15.99</v>
       </c>
       <c r="D40" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SHANTIINOR</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>184.95</v>
+        <v>20.98</v>
       </c>
       <c r="C41" t="n">
-        <v>194.15</v>
+        <v>21.97</v>
       </c>
       <c r="D41" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>SIEL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>20.95</v>
+        <v>31.5</v>
       </c>
       <c r="C42" t="n">
-        <v>21.99</v>
+        <v>32.98</v>
       </c>
       <c r="D42" t="n">
-        <v>4.96</v>
+        <v>4.7</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.01</v>
+        <v>3.65</v>
       </c>
       <c r="C43" t="n">
-        <v>1.06</v>
+        <v>3.82</v>
       </c>
       <c r="D43" t="n">
-        <v>4.95</v>
+        <v>4.66</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.82</v>
+        <v>14.98</v>
       </c>
       <c r="C44" t="n">
-        <v>1.91</v>
+        <v>15.67</v>
       </c>
       <c r="D44" t="n">
-        <v>4.95</v>
+        <v>4.61</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AARADHYA</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>141.55</v>
+        <v>169.21</v>
       </c>
       <c r="C45" t="n">
-        <v>148.55</v>
+        <v>176.99</v>
       </c>
       <c r="D45" t="n">
-        <v>4.95</v>
+        <v>4.6</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LEENEE</t>
+          <t>ESSARSHPNG</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>7.9</v>
+        <v>15.76</v>
       </c>
       <c r="C46" t="n">
-        <v>8.289999999999999</v>
+        <v>16.48</v>
       </c>
       <c r="D46" t="n">
-        <v>4.94</v>
+        <v>4.57</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MAL</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>48.7</v>
+        <v>16.84</v>
       </c>
       <c r="C47" t="n">
-        <v>51.1</v>
+        <v>17.6</v>
       </c>
       <c r="D47" t="n">
-        <v>4.93</v>
+        <v>4.51</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DIGISPICE</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>16.87</v>
+        <v>151.6</v>
       </c>
       <c r="C48" t="n">
-        <v>17.68</v>
+        <v>158.44</v>
       </c>
       <c r="D48" t="n">
-        <v>4.8</v>
+        <v>4.51</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>LAHOTIOV</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1756.7</v>
+        <v>39.28</v>
       </c>
       <c r="C49" t="n">
-        <v>1841</v>
+        <v>40.99</v>
       </c>
       <c r="D49" t="n">
-        <v>4.8</v>
+        <v>4.35</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>GRAVISSHO</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>26.03</v>
+        <v>46.97</v>
       </c>
       <c r="C50" t="n">
-        <v>27.28</v>
+        <v>49</v>
       </c>
       <c r="D50" t="n">
-        <v>4.8</v>
+        <v>4.32</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>GEECEE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>156.56</v>
+        <v>350.1</v>
       </c>
       <c r="C51" t="n">
-        <v>164</v>
+        <v>365</v>
       </c>
       <c r="D51" t="n">
-        <v>4.75</v>
+        <v>4.26</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>BANG</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>38.38</v>
+        <v>32.29</v>
       </c>
       <c r="C52" t="n">
-        <v>40.2</v>
+        <v>33.65</v>
       </c>
       <c r="D52" t="n">
-        <v>4.74</v>
+        <v>4.21</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>13.31</v>
+        <v>15.83</v>
       </c>
       <c r="C53" t="n">
-        <v>13.94</v>
+        <v>16.48</v>
       </c>
       <c r="D53" t="n">
-        <v>4.73</v>
+        <v>4.11</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RSDFIN</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>94</v>
+        <v>11.43</v>
       </c>
       <c r="C54" t="n">
-        <v>98.40000000000001</v>
+        <v>11.9</v>
       </c>
       <c r="D54" t="n">
-        <v>4.68</v>
+        <v>4.11</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LAKPRE</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6</v>
+        <v>22.31</v>
       </c>
       <c r="C55" t="n">
-        <v>6.28</v>
+        <v>23.2</v>
       </c>
       <c r="D55" t="n">
-        <v>4.67</v>
+        <v>3.99</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CELEBRITY</t>
+          <t>PANCHMAHQ</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>6.85</v>
+        <v>293.4</v>
       </c>
       <c r="C56" t="n">
-        <v>7.17</v>
+        <v>304.85</v>
       </c>
       <c r="D56" t="n">
-        <v>4.67</v>
+        <v>3.9</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BPLPHARMA</t>
+          <t>SNOWMAN</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1505.1</v>
+        <v>35.03</v>
       </c>
       <c r="C57" t="n">
-        <v>1575</v>
+        <v>36.39</v>
       </c>
       <c r="D57" t="n">
-        <v>4.64</v>
+        <v>3.88</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DCAL</t>
+          <t>JAYESH</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>167.25</v>
+        <v>125.1</v>
       </c>
       <c r="C58" t="n">
-        <v>174.99</v>
+        <v>129.95</v>
       </c>
       <c r="D58" t="n">
-        <v>4.63</v>
+        <v>3.88</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>8.210000000000001</v>
+        <v>42.75</v>
       </c>
       <c r="C59" t="n">
-        <v>8.59</v>
+        <v>44.4</v>
       </c>
       <c r="D59" t="n">
-        <v>4.63</v>
+        <v>3.86</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>34.41</v>
+        <v>12.47</v>
       </c>
       <c r="C60" t="n">
-        <v>36</v>
+        <v>12.95</v>
       </c>
       <c r="D60" t="n">
-        <v>4.62</v>
+        <v>3.85</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1037.7</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="C61" t="n">
-        <v>1085</v>
+        <v>84.5</v>
       </c>
       <c r="D61" t="n">
-        <v>4.56</v>
+        <v>3.81</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>SUNSHIEL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.66</v>
+        <v>1209.3</v>
       </c>
       <c r="C62" t="n">
-        <v>0.6899999999999999</v>
+        <v>1255</v>
       </c>
       <c r="D62" t="n">
-        <v>4.55</v>
+        <v>3.78</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>COMPINFO</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>16.74</v>
+        <v>1.06</v>
       </c>
       <c r="C63" t="n">
-        <v>17.5</v>
+        <v>1.1</v>
       </c>
       <c r="D63" t="n">
-        <v>4.54</v>
+        <v>3.77</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2.44</v>
+        <v>37.4</v>
       </c>
       <c r="C64" t="n">
-        <v>2.55</v>
+        <v>38.8</v>
       </c>
       <c r="D64" t="n">
-        <v>4.51</v>
+        <v>3.74</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SHREEDHAR</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>135.8</v>
+        <v>131.25</v>
       </c>
       <c r="C65" t="n">
-        <v>141.9</v>
+        <v>136.15</v>
       </c>
       <c r="D65" t="n">
-        <v>4.49</v>
+        <v>3.73</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.45</v>
+        <v>0.27</v>
       </c>
       <c r="C66" t="n">
-        <v>0.47</v>
+        <v>0.28</v>
       </c>
       <c r="D66" t="n">
-        <v>4.44</v>
+        <v>3.7</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LAMOSAIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>53.1</v>
+        <v>737.9</v>
       </c>
       <c r="C67" t="n">
-        <v>55.45</v>
+        <v>765</v>
       </c>
       <c r="D67" t="n">
-        <v>4.43</v>
+        <v>3.67</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>6.2</v>
+        <v>26.71</v>
       </c>
       <c r="C68" t="n">
-        <v>6.47</v>
+        <v>27.68</v>
       </c>
       <c r="D68" t="n">
-        <v>4.35</v>
+        <v>3.63</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>5.75</v>
+        <v>6.88</v>
       </c>
       <c r="C69" t="n">
-        <v>6</v>
+        <v>7.13</v>
       </c>
       <c r="D69" t="n">
-        <v>4.35</v>
+        <v>3.63</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>MIIL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>13.42</v>
+        <v>666.1</v>
       </c>
       <c r="C70" t="n">
-        <v>14</v>
+        <v>689.95</v>
       </c>
       <c r="D70" t="n">
-        <v>4.32</v>
+        <v>3.58</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>ANSALBU</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>15.33</v>
+        <v>84</v>
       </c>
       <c r="C71" t="n">
-        <v>15.99</v>
+        <v>86.98999999999999</v>
       </c>
       <c r="D71" t="n">
-        <v>4.31</v>
+        <v>3.56</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>KSR</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1.16</v>
+        <v>44.4</v>
       </c>
       <c r="C72" t="n">
-        <v>1.21</v>
+        <v>45.98</v>
       </c>
       <c r="D72" t="n">
-        <v>4.31</v>
+        <v>3.56</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AKASH</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>24.86</v>
+        <v>7.62</v>
       </c>
       <c r="C73" t="n">
-        <v>25.93</v>
+        <v>7.89</v>
       </c>
       <c r="D73" t="n">
-        <v>4.3</v>
+        <v>3.54</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>KRITI</t>
+          <t>BENARAS</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>61.4</v>
+        <v>11001</v>
       </c>
       <c r="C74" t="n">
-        <v>64</v>
+        <v>11390</v>
       </c>
       <c r="D74" t="n">
-        <v>4.23</v>
+        <v>3.54</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SHRJAGP</t>
+          <t>NTCIND</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>647</v>
+        <v>134.11</v>
       </c>
       <c r="C75" t="n">
-        <v>673.95</v>
+        <v>138.8</v>
       </c>
       <c r="D75" t="n">
-        <v>4.17</v>
+        <v>3.5</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>297.1</v>
+        <v>23.47</v>
       </c>
       <c r="C76" t="n">
-        <v>309.25</v>
+        <v>24.29</v>
       </c>
       <c r="D76" t="n">
-        <v>4.09</v>
+        <v>3.49</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>15.99</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="C77" t="n">
-        <v>16.64</v>
+        <v>81</v>
       </c>
       <c r="D77" t="n">
-        <v>4.07</v>
+        <v>3.46</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>86.5</v>
+        <v>37.2</v>
       </c>
       <c r="C78" t="n">
-        <v>90</v>
+        <v>38.45</v>
       </c>
       <c r="D78" t="n">
-        <v>4.05</v>
+        <v>3.36</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PREMCO</t>
+          <t>RKDL</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>394</v>
+        <v>18</v>
       </c>
       <c r="C79" t="n">
-        <v>409.95</v>
+        <v>18.59</v>
       </c>
       <c r="D79" t="n">
-        <v>4.05</v>
+        <v>3.28</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NIMBSPROJ</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>165.25</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="C80" t="n">
-        <v>171.86</v>
+        <v>8.9</v>
       </c>
       <c r="D80" t="n">
-        <v>4</v>
+        <v>3.25</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>DEEP</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>785.05</v>
+        <v>45.13</v>
       </c>
       <c r="C81" t="n">
-        <v>816</v>
+        <v>46.59</v>
       </c>
       <c r="D81" t="n">
-        <v>3.94</v>
+        <v>3.24</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PATELENG</t>
+          <t>HINDADH</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>26.61</v>
+        <v>371.95</v>
       </c>
       <c r="C82" t="n">
-        <v>27.65</v>
+        <v>384</v>
       </c>
       <c r="D82" t="n">
-        <v>3.91</v>
+        <v>3.24</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PML</t>
+          <t>DELTAMAGNT</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>482.45</v>
+        <v>55.65</v>
       </c>
       <c r="C83" t="n">
-        <v>500.95</v>
+        <v>57.45</v>
       </c>
       <c r="D83" t="n">
-        <v>3.83</v>
+        <v>3.23</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>3828.3</v>
+        <v>43.5</v>
       </c>
       <c r="C84" t="n">
-        <v>3974.6</v>
+        <v>44.9</v>
       </c>
       <c r="D84" t="n">
-        <v>3.82</v>
+        <v>3.22</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1206.1</v>
+        <v>16.94</v>
       </c>
       <c r="C85" t="n">
-        <v>1252</v>
+        <v>17.48</v>
       </c>
       <c r="D85" t="n">
-        <v>3.81</v>
+        <v>3.19</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>INDTERRAIN</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>157.98</v>
+        <v>28.01</v>
       </c>
       <c r="C86" t="n">
-        <v>164</v>
+        <v>28.9</v>
       </c>
       <c r="D86" t="n">
-        <v>3.81</v>
+        <v>3.18</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>25.14</v>
+        <v>5.67</v>
       </c>
       <c r="C87" t="n">
-        <v>26.09</v>
+        <v>5.85</v>
       </c>
       <c r="D87" t="n">
-        <v>3.78</v>
+        <v>3.17</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MOHITIND</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>23.23</v>
+        <v>255.9</v>
       </c>
       <c r="C88" t="n">
-        <v>24.1</v>
+        <v>263.9</v>
       </c>
       <c r="D88" t="n">
-        <v>3.75</v>
+        <v>3.13</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>RUDRA</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1098.6</v>
+        <v>20.16</v>
       </c>
       <c r="C89" t="n">
-        <v>1139.8</v>
+        <v>20.79</v>
       </c>
       <c r="D89" t="n">
-        <v>3.75</v>
+        <v>3.12</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>UNIENTER</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>43.28</v>
+        <v>89.22</v>
       </c>
       <c r="C90" t="n">
-        <v>44.89</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="D90" t="n">
-        <v>3.72</v>
+        <v>3.1</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>23.71</v>
+        <v>24.88</v>
       </c>
       <c r="C91" t="n">
-        <v>24.59</v>
+        <v>25.65</v>
       </c>
       <c r="D91" t="n">
-        <v>3.71</v>
+        <v>3.09</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>8.18</v>
+        <v>14.65</v>
       </c>
       <c r="C92" t="n">
-        <v>8.48</v>
+        <v>15.1</v>
       </c>
       <c r="D92" t="n">
-        <v>3.67</v>
+        <v>3.07</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SUBAHOTELS</t>
+          <t>KAUSHALYA</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>101.2</v>
+        <v>834.5</v>
       </c>
       <c r="C93" t="n">
-        <v>104.9</v>
+        <v>859.75</v>
       </c>
       <c r="D93" t="n">
-        <v>3.66</v>
+        <v>3.03</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>DISHTV</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>2.5</v>
+        <v>8.57</v>
       </c>
       <c r="C94" t="n">
-        <v>2.59</v>
+        <v>8.83</v>
       </c>
       <c r="D94" t="n">
-        <v>3.6</v>
+        <v>3.03</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AMDIND</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>64.03</v>
+        <v>237.78</v>
       </c>
       <c r="C95" t="n">
-        <v>66.29000000000001</v>
+        <v>244.9</v>
       </c>
       <c r="D95" t="n">
-        <v>3.53</v>
+        <v>2.99</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ENKEIWHEL</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>399</v>
+        <v>3.39</v>
       </c>
       <c r="C96" t="n">
-        <v>412.95</v>
+        <v>3.49</v>
       </c>
       <c r="D96" t="n">
-        <v>3.5</v>
+        <v>2.95</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>YATHARTH</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>966.3</v>
+        <v>88.3</v>
       </c>
       <c r="C97" t="n">
-        <v>1000</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="D97" t="n">
-        <v>3.49</v>
+        <v>2.94</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>FINKURVE</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>72.48999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="C98" t="n">
-        <v>75</v>
+        <v>0.7</v>
       </c>
       <c r="D98" t="n">
-        <v>3.46</v>
+        <v>2.94</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LANCER</t>
+          <t>ICDSLTD</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>12.74</v>
+        <v>63.15</v>
       </c>
       <c r="C99" t="n">
-        <v>13.18</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="D99" t="n">
-        <v>3.45</v>
+        <v>2.91</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MOHITE</t>
+          <t>SICAGEN</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>2.63</v>
+        <v>53.98</v>
       </c>
       <c r="C100" t="n">
-        <v>2.72</v>
+        <v>55.55</v>
       </c>
       <c r="D100" t="n">
-        <v>3.42</v>
+        <v>2.91</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ESDS</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1740.4</v>
+        <v>35.47</v>
       </c>
       <c r="C101" t="n">
-        <v>1800</v>
+        <v>36.49</v>
       </c>
       <c r="D101" t="n">
-        <v>3.42</v>
+        <v>2.88</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>RELCHEMQ</t>
+          <t>DEEPA</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>110.23</v>
+        <v>169.14</v>
       </c>
       <c r="C102" t="n">
-        <v>114</v>
+        <v>173.99</v>
       </c>
       <c r="D102" t="n">
-        <v>3.42</v>
+        <v>2.87</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>TRANSCOR</t>
+          <t>DIAMINESQ</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>25.39</v>
+        <v>251.8</v>
       </c>
       <c r="C103" t="n">
-        <v>26.25</v>
+        <v>259</v>
       </c>
       <c r="D103" t="n">
-        <v>3.39</v>
+        <v>2.86</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>2200.8</v>
+        <v>4.9</v>
       </c>
       <c r="C104" t="n">
-        <v>2275.5</v>
+        <v>5.04</v>
       </c>
       <c r="D104" t="n">
-        <v>3.39</v>
+        <v>2.86</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>NTCIND</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>134.91</v>
+        <v>1.06</v>
       </c>
       <c r="C105" t="n">
-        <v>139.45</v>
+        <v>1.09</v>
       </c>
       <c r="D105" t="n">
-        <v>3.37</v>
+        <v>2.83</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CHAVDA</t>
+          <t>KOHINOOR</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>125.3</v>
+        <v>29.58</v>
       </c>
       <c r="C106" t="n">
-        <v>129.5</v>
+        <v>30.4</v>
       </c>
       <c r="D106" t="n">
-        <v>3.35</v>
+        <v>2.77</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SONATSOFTW</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>265.85</v>
+        <v>5.83</v>
       </c>
       <c r="C107" t="n">
-        <v>274.75</v>
+        <v>5.99</v>
       </c>
       <c r="D107" t="n">
-        <v>3.35</v>
+        <v>2.74</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>156.75</v>
+        <v>5012.4</v>
       </c>
       <c r="C108" t="n">
-        <v>162</v>
+        <v>5148</v>
       </c>
       <c r="D108" t="n">
-        <v>3.35</v>
+        <v>2.71</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BSOFT</t>
+          <t>MAHSCOOTER</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>281.65</v>
+        <v>12882</v>
       </c>
       <c r="C109" t="n">
-        <v>291</v>
+        <v>13231</v>
       </c>
       <c r="D109" t="n">
-        <v>3.32</v>
+        <v>2.71</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>DHUNINV</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>995</v>
+        <v>225.91</v>
       </c>
       <c r="C110" t="n">
-        <v>1028</v>
+        <v>232</v>
       </c>
       <c r="D110" t="n">
-        <v>3.32</v>
+        <v>2.7</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AZADIND</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>87.13</v>
+        <v>0.37</v>
       </c>
       <c r="C111" t="n">
-        <v>90</v>
+        <v>0.38</v>
       </c>
       <c r="D111" t="n">
-        <v>3.29</v>
+        <v>2.7</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>PGIL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>40.86</v>
+        <v>1141.4</v>
       </c>
       <c r="C112" t="n">
-        <v>42.2</v>
+        <v>1171.6</v>
       </c>
       <c r="D112" t="n">
-        <v>3.28</v>
+        <v>2.65</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ASHUTOSH</t>
+          <t>AMBICAAGAR</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>164.5</v>
+        <v>24.94</v>
       </c>
       <c r="C113" t="n">
-        <v>169.9</v>
+        <v>25.6</v>
       </c>
       <c r="D113" t="n">
-        <v>3.28</v>
+        <v>2.65</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>SPLIL</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>5375.5</v>
+        <v>28.84</v>
       </c>
       <c r="C114" t="n">
-        <v>5550</v>
+        <v>29.6</v>
       </c>
       <c r="D114" t="n">
-        <v>3.25</v>
+        <v>2.64</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>DIACABS</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>369.05</v>
+        <v>0.77</v>
       </c>
       <c r="C115" t="n">
-        <v>381</v>
+        <v>0.79</v>
       </c>
       <c r="D115" t="n">
-        <v>3.24</v>
+        <v>2.6</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>LAKSHMIMIL</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>91.64</v>
+        <v>7565</v>
       </c>
       <c r="C116" t="n">
-        <v>94.59999999999999</v>
+        <v>7760</v>
       </c>
       <c r="D116" t="n">
-        <v>3.23</v>
+        <v>2.58</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MWL</t>
+          <t>DHATRE</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>40.6</v>
+        <v>4.29</v>
       </c>
       <c r="C117" t="n">
-        <v>41.9</v>
+        <v>4.4</v>
       </c>
       <c r="D117" t="n">
-        <v>3.2</v>
+        <v>2.56</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>AMARJOTHI</t>
+          <t>HGS</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>150.14</v>
+        <v>381.6</v>
       </c>
       <c r="C118" t="n">
-        <v>154.93</v>
+        <v>391.35</v>
       </c>
       <c r="D118" t="n">
-        <v>3.19</v>
+        <v>2.56</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NOVAAGRI</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>22.7</v>
+        <v>77.91</v>
       </c>
       <c r="C119" t="n">
-        <v>23.42</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="D119" t="n">
-        <v>3.17</v>
+        <v>2.55</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>FINOPB</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>16.13</v>
+        <v>137.73</v>
       </c>
       <c r="C120" t="n">
-        <v>16.64</v>
+        <v>141.23</v>
       </c>
       <c r="D120" t="n">
-        <v>3.16</v>
+        <v>2.54</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DECNGOLD</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>229.73</v>
+        <v>1431.9</v>
       </c>
       <c r="C121" t="n">
-        <v>237</v>
+        <v>1468.3</v>
       </c>
       <c r="D121" t="n">
-        <v>3.16</v>
+        <v>2.54</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>WATERBASE</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>46.54</v>
+        <v>132.68</v>
       </c>
       <c r="C122" t="n">
-        <v>48</v>
+        <v>136</v>
       </c>
       <c r="D122" t="n">
-        <v>3.14</v>
+        <v>2.5</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>RELCHEMQ</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>463.45</v>
+        <v>120.7</v>
       </c>
       <c r="C123" t="n">
-        <v>477.95</v>
+        <v>123.71</v>
       </c>
       <c r="D123" t="n">
-        <v>3.13</v>
+        <v>2.49</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>BALKRISHNA</t>
+          <t>WEL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>16.1</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="C124" t="n">
-        <v>16.6</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="D124" t="n">
-        <v>3.11</v>
+        <v>2.49</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>TNPETRO</t>
+          <t>ARVEE</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>128.9</v>
+        <v>168.6</v>
       </c>
       <c r="C125" t="n">
-        <v>132.9</v>
+        <v>172.8</v>
       </c>
       <c r="D125" t="n">
-        <v>3.1</v>
+        <v>2.49</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>AYE</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>179.46</v>
+        <v>6.44</v>
       </c>
       <c r="C126" t="n">
-        <v>185</v>
+        <v>6.6</v>
       </c>
       <c r="D126" t="n">
-        <v>3.09</v>
+        <v>2.48</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MVKAGRO</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>299.8</v>
+        <v>15.85</v>
       </c>
       <c r="C127" t="n">
-        <v>309</v>
+        <v>16.24</v>
       </c>
       <c r="D127" t="n">
-        <v>3.07</v>
+        <v>2.46</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>366.7</v>
+        <v>10.22</v>
       </c>
       <c r="C128" t="n">
-        <v>377.95</v>
+        <v>10.47</v>
       </c>
       <c r="D128" t="n">
-        <v>3.07</v>
+        <v>2.45</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>TRITONV</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>62.97</v>
+        <v>1051.5</v>
       </c>
       <c r="C129" t="n">
-        <v>64.90000000000001</v>
+        <v>1077</v>
       </c>
       <c r="D129" t="n">
-        <v>3.06</v>
+        <v>2.43</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>5.55</v>
+        <v>19.28</v>
       </c>
       <c r="C130" t="n">
-        <v>5.72</v>
+        <v>19.74</v>
       </c>
       <c r="D130" t="n">
-        <v>3.06</v>
+        <v>2.39</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>65.69</v>
+        <v>29.45</v>
       </c>
       <c r="C131" t="n">
-        <v>67.7</v>
+        <v>30.15</v>
       </c>
       <c r="D131" t="n">
-        <v>3.06</v>
+        <v>2.38</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>1541</v>
+        <v>89.84999999999999</v>
       </c>
       <c r="C132" t="n">
-        <v>1588</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="D132" t="n">
-        <v>3.05</v>
+        <v>2.38</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>LTM</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>4275</v>
+        <v>24.42</v>
       </c>
       <c r="C133" t="n">
-        <v>4404.3</v>
+        <v>25</v>
       </c>
       <c r="D133" t="n">
-        <v>3.02</v>
+        <v>2.38</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>PANORAMA</t>
+          <t>SONATSOFTW</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>53.78</v>
+        <v>281.3</v>
       </c>
       <c r="C134" t="n">
-        <v>55.4</v>
+        <v>287.95</v>
       </c>
       <c r="D134" t="n">
-        <v>3.01</v>
+        <v>2.36</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>DCM</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>75</v>
+        <v>1.71</v>
       </c>
       <c r="C135" t="n">
-        <v>77.25</v>
+        <v>1.75</v>
       </c>
       <c r="D135" t="n">
-        <v>3</v>
+        <v>2.34</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CALSOFT</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>38.74</v>
+        <v>7.77</v>
       </c>
       <c r="C136" t="n">
-        <v>39.9</v>
+        <v>7.95</v>
       </c>
       <c r="D136" t="n">
-        <v>2.99</v>
+        <v>2.32</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>STARPAPER</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>23.5</v>
+        <v>160.27</v>
       </c>
       <c r="C137" t="n">
-        <v>24.2</v>
+        <v>163.99</v>
       </c>
       <c r="D137" t="n">
-        <v>2.98</v>
+        <v>2.32</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>VALIANTORG</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>396.3</v>
+        <v>14.47</v>
       </c>
       <c r="C138" t="n">
-        <v>408</v>
+        <v>14.8</v>
       </c>
       <c r="D138" t="n">
-        <v>2.95</v>
+        <v>2.28</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>64.98999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="C139" t="n">
-        <v>66.90000000000001</v>
+        <v>8.99</v>
       </c>
       <c r="D139" t="n">
-        <v>2.94</v>
+        <v>2.28</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>GROWWSLVR</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1202.8</v>
+        <v>22</v>
       </c>
       <c r="C140" t="n">
-        <v>1238</v>
+        <v>22.5</v>
       </c>
       <c r="D140" t="n">
-        <v>2.93</v>
+        <v>2.27</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>SAKHTISUG</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>7.18</v>
+        <v>18.95</v>
       </c>
       <c r="C141" t="n">
-        <v>7.39</v>
+        <v>19.38</v>
       </c>
       <c r="D141" t="n">
-        <v>2.92</v>
+        <v>2.27</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>132.17</v>
+        <v>5.74</v>
       </c>
       <c r="C142" t="n">
-        <v>136</v>
+        <v>5.87</v>
       </c>
       <c r="D142" t="n">
-        <v>2.9</v>
+        <v>2.26</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TENNIND</t>
+          <t>HLVLTD</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>506.35</v>
+        <v>6.26</v>
       </c>
       <c r="C143" t="n">
-        <v>521</v>
+        <v>6.4</v>
       </c>
       <c r="D143" t="n">
-        <v>2.89</v>
+        <v>2.24</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>MHLXMIRU</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>167.4</v>
+        <v>156.39</v>
       </c>
       <c r="C144" t="n">
-        <v>172.2</v>
+        <v>159.9</v>
       </c>
       <c r="D144" t="n">
-        <v>2.87</v>
+        <v>2.24</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>10.19</v>
+        <v>63.09</v>
       </c>
       <c r="C145" t="n">
-        <v>10.48</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="D145" t="n">
-        <v>2.85</v>
+        <v>2.22</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>364.65</v>
+        <v>43.73</v>
       </c>
       <c r="C146" t="n">
-        <v>375</v>
+        <v>44.7</v>
       </c>
       <c r="D146" t="n">
-        <v>2.84</v>
+        <v>2.22</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>AAREYDRUGS</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>455.1</v>
+        <v>98.81999999999999</v>
       </c>
       <c r="C147" t="n">
-        <v>468</v>
+        <v>101</v>
       </c>
       <c r="D147" t="n">
-        <v>2.83</v>
+        <v>2.21</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>583.55</v>
+        <v>6.79</v>
       </c>
       <c r="C148" t="n">
-        <v>600.05</v>
+        <v>6.94</v>
       </c>
       <c r="D148" t="n">
-        <v>2.83</v>
+        <v>2.21</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>BIMETAL</t>
+          <t>YESBANK</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>640.5</v>
+        <v>23.07</v>
       </c>
       <c r="C149" t="n">
-        <v>658.65</v>
+        <v>23.58</v>
       </c>
       <c r="D149" t="n">
-        <v>2.83</v>
+        <v>2.21</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ARROWGREEN</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>813</v>
+        <v>10.47</v>
       </c>
       <c r="C150" t="n">
-        <v>835.9</v>
+        <v>10.7</v>
       </c>
       <c r="D150" t="n">
-        <v>2.82</v>
+        <v>2.2</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>EMAMILTD</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>363.8</v>
+        <v>46.58</v>
       </c>
       <c r="C151" t="n">
-        <v>374</v>
+        <v>47.6</v>
       </c>
       <c r="D151" t="n">
-        <v>2.8</v>
+        <v>2.19</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CREATIVEYE</t>
+          <t>PINELABS</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>5.72</v>
+        <v>193.8</v>
       </c>
       <c r="C152" t="n">
-        <v>5.88</v>
+        <v>198</v>
       </c>
       <c r="D152" t="n">
-        <v>2.8</v>
+        <v>2.17</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>DTIL</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>466.9</v>
+        <v>138.3</v>
       </c>
       <c r="C153" t="n">
-        <v>479.9</v>
+        <v>141.3</v>
       </c>
       <c r="D153" t="n">
-        <v>2.78</v>
+        <v>2.17</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>MSPL</t>
+          <t>SURAJLTD</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>33.96</v>
+        <v>195.75</v>
       </c>
       <c r="C154" t="n">
-        <v>34.9</v>
+        <v>200</v>
       </c>
       <c r="D154" t="n">
-        <v>2.77</v>
+        <v>2.17</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>4.33</v>
+        <v>7.82</v>
       </c>
       <c r="C155" t="n">
-        <v>4.45</v>
+        <v>7.99</v>
       </c>
       <c r="D155" t="n">
-        <v>2.77</v>
+        <v>2.17</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>540.45</v>
+        <v>3.27</v>
       </c>
       <c r="C156" t="n">
-        <v>555.3</v>
+        <v>3.34</v>
       </c>
       <c r="D156" t="n">
-        <v>2.75</v>
+        <v>2.14</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>JAYBEE</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>83.7</v>
+        <v>4.22</v>
       </c>
       <c r="C157" t="n">
-        <v>86</v>
+        <v>4.31</v>
       </c>
       <c r="D157" t="n">
-        <v>2.75</v>
+        <v>2.13</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>RAJESHEXPO</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>78.3</v>
+        <v>2.35</v>
       </c>
       <c r="C158" t="n">
-        <v>80.43000000000001</v>
+        <v>2.4</v>
       </c>
       <c r="D158" t="n">
-        <v>2.72</v>
+        <v>2.13</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MOLDTECH</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>207.39</v>
+        <v>1.88</v>
       </c>
       <c r="C159" t="n">
-        <v>213</v>
+        <v>1.92</v>
       </c>
       <c r="D159" t="n">
-        <v>2.71</v>
+        <v>2.13</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>DENORA</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>798.45</v>
+        <v>474.95</v>
       </c>
       <c r="C160" t="n">
-        <v>820</v>
+        <v>485</v>
       </c>
       <c r="D160" t="n">
-        <v>2.7</v>
+        <v>2.12</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.37</v>
+        <v>64.52</v>
       </c>
       <c r="C161" t="n">
-        <v>0.38</v>
+        <v>65.88</v>
       </c>
       <c r="D161" t="n">
-        <v>2.7</v>
+        <v>2.11</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>TUTIALKA</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>59.19</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="C162" t="n">
-        <v>60.79</v>
+        <v>101.5</v>
       </c>
       <c r="D162" t="n">
-        <v>2.7</v>
+        <v>2.11</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>NDTV</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>198.93</v>
+        <v>70.43000000000001</v>
       </c>
       <c r="C163" t="n">
-        <v>204.28</v>
+        <v>71.91</v>
       </c>
       <c r="D163" t="n">
-        <v>2.69</v>
+        <v>2.1</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>LOTUSDEV</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>209.27</v>
+        <v>4.28</v>
       </c>
       <c r="C164" t="n">
-        <v>214.88</v>
+        <v>4.37</v>
       </c>
       <c r="D164" t="n">
-        <v>2.68</v>
+        <v>2.1</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>369.25</v>
+        <v>2.38</v>
       </c>
       <c r="C165" t="n">
-        <v>378.95</v>
+        <v>2.43</v>
       </c>
       <c r="D165" t="n">
-        <v>2.63</v>
+        <v>2.1</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>HLEGLAS</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>404.35</v>
+        <v>20.57</v>
       </c>
       <c r="C166" t="n">
-        <v>415</v>
+        <v>21</v>
       </c>
       <c r="D166" t="n">
-        <v>2.63</v>
+        <v>2.09</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>2.28</v>
+        <v>12.91</v>
       </c>
       <c r="C167" t="n">
-        <v>2.34</v>
+        <v>13.18</v>
       </c>
       <c r="D167" t="n">
-        <v>2.63</v>
+        <v>2.09</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>MOLBIO</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>646.3</v>
+        <v>1356.8</v>
       </c>
       <c r="C168" t="n">
-        <v>663.2</v>
+        <v>1385</v>
       </c>
       <c r="D168" t="n">
-        <v>2.61</v>
+        <v>2.08</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ELANTAS</t>
+          <t>POEL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>14513</v>
+        <v>139.45</v>
       </c>
       <c r="C169" t="n">
-        <v>14890</v>
+        <v>142.35</v>
       </c>
       <c r="D169" t="n">
-        <v>2.6</v>
+        <v>2.08</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>BAGFILMS</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>723.15</v>
+        <v>4.35</v>
       </c>
       <c r="C170" t="n">
-        <v>741.9</v>
+        <v>4.44</v>
       </c>
       <c r="D170" t="n">
-        <v>2.59</v>
+        <v>2.07</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>TECHD</t>
+          <t>ACCURACY</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>605.3</v>
+        <v>4.38</v>
       </c>
       <c r="C171" t="n">
-        <v>621</v>
+        <v>4.47</v>
       </c>
       <c r="D171" t="n">
-        <v>2.59</v>
+        <v>2.05</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MUKKA</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>32.17</v>
+        <v>6.35</v>
       </c>
       <c r="C172" t="n">
-        <v>33</v>
+        <v>6.48</v>
       </c>
       <c r="D172" t="n">
-        <v>2.58</v>
+        <v>2.05</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SHARDAMOTR</t>
+          <t>MKPL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>943.75</v>
+        <v>3.92</v>
       </c>
       <c r="C173" t="n">
-        <v>968</v>
+        <v>4</v>
       </c>
       <c r="D173" t="n">
-        <v>2.57</v>
+        <v>2.04</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>24.18</v>
+        <v>9.82</v>
       </c>
       <c r="C174" t="n">
-        <v>24.8</v>
+        <v>10.02</v>
       </c>
       <c r="D174" t="n">
-        <v>2.56</v>
+        <v>2.04</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>FAIRCHEMOR</t>
+          <t>TITAGARH</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>623.95</v>
+        <v>811.45</v>
       </c>
       <c r="C175" t="n">
-        <v>639.9</v>
+        <v>828</v>
       </c>
       <c r="D175" t="n">
-        <v>2.56</v>
+        <v>2.04</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>ITL</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>118.98</v>
+        <v>367.5</v>
       </c>
       <c r="C176" t="n">
-        <v>122</v>
+        <v>375</v>
       </c>
       <c r="D176" t="n">
-        <v>2.54</v>
+        <v>2.04</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ENIL</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>101.24</v>
+        <v>20.29</v>
       </c>
       <c r="C177" t="n">
-        <v>103.8</v>
+        <v>20.7</v>
       </c>
       <c r="D177" t="n">
-        <v>2.53</v>
+        <v>2.02</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>MPHASIS</t>
+          <t>STEELCITY</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>2295</v>
+        <v>86.12</v>
       </c>
       <c r="C178" t="n">
-        <v>2353</v>
+        <v>87.86</v>
       </c>
       <c r="D178" t="n">
-        <v>2.53</v>
+        <v>2.02</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>PERSISTENT</t>
+          <t>HINDALUMI</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>5516</v>
+        <v>95.09</v>
       </c>
       <c r="C179" t="n">
-        <v>5654</v>
+        <v>97</v>
       </c>
       <c r="D179" t="n">
-        <v>2.5</v>
+        <v>2.01</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SWSOLAR</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>180.22</v>
+        <v>34.02</v>
       </c>
       <c r="C180" t="n">
-        <v>184.7</v>
+        <v>34.7</v>
       </c>
       <c r="D180" t="n">
-        <v>2.49</v>
+        <v>2</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>2.01</v>
+        <v>2.5</v>
       </c>
       <c r="C181" t="n">
-        <v>2.06</v>
+        <v>2.55</v>
       </c>
       <c r="D181" t="n">
-        <v>2.49</v>
+        <v>2</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>BELLACASA</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>256.52</v>
+        <v>277.45</v>
       </c>
       <c r="C182" t="n">
-        <v>262.86</v>
+        <v>282.95</v>
       </c>
       <c r="D182" t="n">
-        <v>2.47</v>
+        <v>1.98</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>XCHANGING</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>165.32</v>
+        <v>64.5</v>
       </c>
       <c r="C183" t="n">
-        <v>169.4</v>
+        <v>65.78</v>
       </c>
       <c r="D183" t="n">
-        <v>2.47</v>
+        <v>1.98</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>HEIDELBERG</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>149.8</v>
+        <v>357.9</v>
       </c>
       <c r="C184" t="n">
-        <v>153.5</v>
+        <v>364.95</v>
       </c>
       <c r="D184" t="n">
-        <v>2.47</v>
+        <v>1.97</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SPLIL</t>
+          <t>CPEDU</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>30.05</v>
+        <v>176.34</v>
       </c>
       <c r="C185" t="n">
-        <v>30.79</v>
+        <v>179.8</v>
       </c>
       <c r="D185" t="n">
-        <v>2.46</v>
+        <v>1.96</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>WARDINMOBI</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>16.69</v>
+        <v>5.62</v>
       </c>
       <c r="C186" t="n">
-        <v>17.1</v>
+        <v>5.73</v>
       </c>
       <c r="D186" t="n">
-        <v>2.46</v>
+        <v>1.96</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>JMA</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>39.46</v>
+        <v>88.95999999999999</v>
       </c>
       <c r="C187" t="n">
-        <v>40.43</v>
+        <v>90.7</v>
       </c>
       <c r="D187" t="n">
-        <v>2.46</v>
+        <v>1.96</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>XTRANET</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>271.34</v>
+        <v>12.26</v>
       </c>
       <c r="C188" t="n">
-        <v>278</v>
+        <v>12.5</v>
       </c>
       <c r="D188" t="n">
-        <v>2.45</v>
+        <v>1.96</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>VISHAL</t>
+          <t>PROZONER</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>18.36</v>
+        <v>52.72</v>
       </c>
       <c r="C189" t="n">
-        <v>18.81</v>
+        <v>53.75</v>
       </c>
       <c r="D189" t="n">
-        <v>2.45</v>
+        <v>1.95</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>45.88</v>
+        <v>1693</v>
       </c>
       <c r="C190" t="n">
-        <v>47</v>
+        <v>1725.9</v>
       </c>
       <c r="D190" t="n">
-        <v>2.44</v>
+        <v>1.94</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>LEENEE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>190.35</v>
+        <v>7.74</v>
       </c>
       <c r="C191" t="n">
-        <v>195</v>
+        <v>7.89</v>
       </c>
       <c r="D191" t="n">
-        <v>2.44</v>
+        <v>1.94</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>SAMPANN</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>46.86</v>
+        <v>23.91</v>
       </c>
       <c r="C192" t="n">
-        <v>48</v>
+        <v>24.37</v>
       </c>
       <c r="D192" t="n">
-        <v>2.43</v>
+        <v>1.92</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>62.29</v>
+        <v>0.52</v>
       </c>
       <c r="C193" t="n">
-        <v>63.8</v>
+        <v>0.53</v>
       </c>
       <c r="D193" t="n">
-        <v>2.42</v>
+        <v>1.92</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>AXISCADES</t>
+          <t>RAJOOENG</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>1831.8</v>
+        <v>53.96</v>
       </c>
       <c r="C194" t="n">
-        <v>1876.2</v>
+        <v>54.99</v>
       </c>
       <c r="D194" t="n">
-        <v>2.42</v>
+        <v>1.91</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>SIKKO</t>
+          <t>BEPL</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>5.83</v>
+        <v>120.69</v>
       </c>
       <c r="C195" t="n">
-        <v>5.97</v>
+        <v>122.98</v>
       </c>
       <c r="D195" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>135.08</v>
+        <v>5.28</v>
       </c>
       <c r="C196" t="n">
-        <v>138.32</v>
+        <v>5.38</v>
       </c>
       <c r="D196" t="n">
-        <v>2.4</v>
+        <v>1.89</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>SUBEXLTD</t>
+          <t>HEXATRADEX</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>20.8</v>
+        <v>156.06</v>
       </c>
       <c r="C197" t="n">
-        <v>21.3</v>
+        <v>158.99</v>
       </c>
       <c r="D197" t="n">
-        <v>2.4</v>
+        <v>1.88</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>17.09</v>
+        <v>24.46</v>
       </c>
       <c r="C198" t="n">
-        <v>17.5</v>
+        <v>24.92</v>
       </c>
       <c r="D198" t="n">
-        <v>2.4</v>
+        <v>1.88</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>87.41</v>
+        <v>47.11</v>
       </c>
       <c r="C199" t="n">
-        <v>89.5</v>
+        <v>47.99</v>
       </c>
       <c r="D199" t="n">
-        <v>2.39</v>
+        <v>1.87</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>CMICABLES</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>2.51</v>
+        <v>5.41</v>
       </c>
       <c r="C200" t="n">
-        <v>2.57</v>
+        <v>5.51</v>
       </c>
       <c r="D200" t="n">
-        <v>2.39</v>
+        <v>1.85</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>MEGATHERM</t>
+          <t>OSWALGREEN</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>251</v>
+        <v>19.59</v>
       </c>
       <c r="C201" t="n">
-        <v>257</v>
+        <v>19.95</v>
       </c>
       <c r="D201" t="n">
-        <v>2.39</v>
+        <v>1.84</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-17 08:55 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RCDL-RE</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>10.68</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>16.09</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48.24</v>
+        <v>57.88</v>
       </c>
       <c r="C3" t="n">
-        <v>57.88</v>
+        <v>63.66</v>
       </c>
       <c r="D3" t="n">
-        <v>19.98</v>
+        <v>9.99</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>RIR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5.18</v>
+        <v>179.77</v>
       </c>
       <c r="C4" t="n">
-        <v>5.98</v>
+        <v>194.74</v>
       </c>
       <c r="D4" t="n">
-        <v>15.44</v>
+        <v>8.33</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SHRADHA</t>
+          <t>MGEL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29.97</v>
+        <v>15.6</v>
       </c>
       <c r="C5" t="n">
-        <v>33.88</v>
+        <v>16.8</v>
       </c>
       <c r="D5" t="n">
-        <v>13.05</v>
+        <v>7.69</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>389.55</v>
+        <v>0.13</v>
       </c>
       <c r="C6" t="n">
-        <v>428.5</v>
+        <v>0.14</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>7.69</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>KHAITANLTD</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44.94</v>
+        <v>149.37</v>
       </c>
       <c r="C7" t="n">
-        <v>49.43</v>
+        <v>159.95</v>
       </c>
       <c r="D7" t="n">
-        <v>9.99</v>
+        <v>7.08</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20.89</v>
+        <v>21.49</v>
       </c>
       <c r="C8" t="n">
-        <v>22.89</v>
+        <v>23</v>
       </c>
       <c r="D8" t="n">
-        <v>9.57</v>
+        <v>7.03</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MPEL-RE</t>
+          <t>ASTAR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.6</v>
+        <v>560.7</v>
       </c>
       <c r="C9" t="n">
-        <v>1.75</v>
+        <v>598</v>
       </c>
       <c r="D9" t="n">
-        <v>9.369999999999999</v>
+        <v>6.65</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HBPOR</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59.99</v>
+        <v>2.45</v>
       </c>
       <c r="C10" t="n">
-        <v>65</v>
+        <v>2.6</v>
       </c>
       <c r="D10" t="n">
-        <v>8.35</v>
+        <v>6.12</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.53</v>
+        <v>150.68</v>
       </c>
       <c r="C11" t="n">
-        <v>4.9</v>
+        <v>159.74</v>
       </c>
       <c r="D11" t="n">
-        <v>8.17</v>
+        <v>6.01</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SAICAPI</t>
+          <t>INNOVANA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>154.5</v>
+        <v>301.3</v>
       </c>
       <c r="C12" t="n">
-        <v>167</v>
+        <v>319</v>
       </c>
       <c r="D12" t="n">
-        <v>8.09</v>
+        <v>5.87</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.13</v>
+        <v>5.49</v>
       </c>
       <c r="C13" t="n">
-        <v>0.14</v>
+        <v>5.8</v>
       </c>
       <c r="D13" t="n">
-        <v>7.69</v>
+        <v>5.65</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PRAKASHSTL</t>
+          <t>ASIANTNE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.56</v>
+        <v>9.19</v>
       </c>
       <c r="C14" t="n">
-        <v>3.82</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>7.3</v>
+        <v>5.55</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HMAAGRO</t>
+          <t>AROGRANITE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23.41</v>
+        <v>22.55</v>
       </c>
       <c r="C15" t="n">
-        <v>24.99</v>
+        <v>23.8</v>
       </c>
       <c r="D15" t="n">
-        <v>6.75</v>
+        <v>5.54</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RADIANTCMS</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>35.89</v>
+        <v>6.06</v>
       </c>
       <c r="C16" t="n">
-        <v>38.24</v>
+        <v>6.39</v>
       </c>
       <c r="D16" t="n">
-        <v>6.55</v>
+        <v>5.45</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>SUVIDHAA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>200.86</v>
+        <v>2.21</v>
       </c>
       <c r="C17" t="n">
-        <v>213.99</v>
+        <v>2.33</v>
       </c>
       <c r="D17" t="n">
-        <v>6.54</v>
+        <v>5.43</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RTSPOWR</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>86.09999999999999</v>
+        <v>12.53</v>
       </c>
       <c r="C18" t="n">
-        <v>91.59999999999999</v>
+        <v>13.21</v>
       </c>
       <c r="D18" t="n">
-        <v>6.39</v>
+        <v>5.43</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.58</v>
+        <v>19.77</v>
       </c>
       <c r="C19" t="n">
-        <v>1.68</v>
+        <v>20.79</v>
       </c>
       <c r="D19" t="n">
-        <v>6.33</v>
+        <v>5.16</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>KRSNAA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>25.44</v>
+        <v>536.4</v>
       </c>
       <c r="C20" t="n">
-        <v>26.99</v>
+        <v>563.9</v>
       </c>
       <c r="D20" t="n">
-        <v>6.09</v>
+        <v>5.13</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>29.34</v>
+        <v>42.56</v>
       </c>
       <c r="C21" t="n">
-        <v>31.1</v>
+        <v>44.7</v>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>5.03</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PAYTM</t>
+          <t>ONMOBILE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1730</v>
+        <v>51.81</v>
       </c>
       <c r="C22" t="n">
-        <v>1830</v>
+        <v>54.4</v>
       </c>
       <c r="D22" t="n">
-        <v>5.78</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>14.08</v>
+        <v>649.25</v>
       </c>
       <c r="C23" t="n">
-        <v>14.89</v>
+        <v>681.7</v>
       </c>
       <c r="D23" t="n">
-        <v>5.75</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1639.5</v>
+        <v>364.26</v>
       </c>
       <c r="C24" t="n">
-        <v>1730</v>
+        <v>382.47</v>
       </c>
       <c r="D24" t="n">
-        <v>5.52</v>
+        <v>5</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CMSINFO</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>222.91</v>
+        <v>49.43</v>
       </c>
       <c r="C25" t="n">
-        <v>235.08</v>
+        <v>51.9</v>
       </c>
       <c r="D25" t="n">
-        <v>5.46</v>
+        <v>5</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>592.85</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="C26" t="n">
-        <v>625</v>
+        <v>103</v>
       </c>
       <c r="D26" t="n">
-        <v>5.42</v>
+        <v>4.99</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.19</v>
+        <v>23.08</v>
       </c>
       <c r="C27" t="n">
-        <v>0.2</v>
+        <v>24.23</v>
       </c>
       <c r="D27" t="n">
-        <v>5.26</v>
+        <v>4.98</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SILVER001</t>
+          <t>BURNPUR</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>23</v>
+        <v>16.67</v>
       </c>
       <c r="C28" t="n">
-        <v>24.2</v>
+        <v>17.5</v>
       </c>
       <c r="D28" t="n">
-        <v>5.22</v>
+        <v>4.98</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>GSMFOILS</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>279</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="C29" t="n">
-        <v>292.95</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ARCL</t>
+          <t>FELDVR</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>262.39</v>
+        <v>2.05</v>
       </c>
       <c r="C30" t="n">
-        <v>275.5</v>
+        <v>2.15</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4.88</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>178.12</v>
+        <v>476.9</v>
       </c>
       <c r="C31" t="n">
-        <v>187.02</v>
+        <v>500</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>4.84</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>346.92</v>
+        <v>290.95</v>
       </c>
       <c r="C32" t="n">
-        <v>364.26</v>
+        <v>304.95</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>4.81</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>97.56999999999999</v>
+        <v>3.13</v>
       </c>
       <c r="C33" t="n">
-        <v>102.44</v>
+        <v>3.28</v>
       </c>
       <c r="D33" t="n">
-        <v>4.99</v>
+        <v>4.79</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>366.65</v>
+        <v>3.83</v>
       </c>
       <c r="C34" t="n">
-        <v>384.95</v>
+        <v>4.01</v>
       </c>
       <c r="D34" t="n">
-        <v>4.99</v>
+        <v>4.7</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>INDIANCARD</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>27.44</v>
+        <v>214.96</v>
       </c>
       <c r="C35" t="n">
-        <v>28.81</v>
+        <v>225</v>
       </c>
       <c r="D35" t="n">
-        <v>4.99</v>
+        <v>4.67</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>POEL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>18.49</v>
+        <v>137.47</v>
       </c>
       <c r="C36" t="n">
-        <v>19.41</v>
+        <v>143.79</v>
       </c>
       <c r="D36" t="n">
-        <v>4.98</v>
+        <v>4.6</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BIKEWO</t>
+          <t>MLKFOOD</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>105.2</v>
+        <v>75.59</v>
       </c>
       <c r="C37" t="n">
-        <v>110.4</v>
+        <v>79</v>
       </c>
       <c r="D37" t="n">
-        <v>4.94</v>
+        <v>4.51</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FLEXITUFF</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2.24</v>
+        <v>5.19</v>
       </c>
       <c r="C38" t="n">
-        <v>2.35</v>
+        <v>5.42</v>
       </c>
       <c r="D38" t="n">
-        <v>4.91</v>
+        <v>4.43</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SUNSHINE</t>
+          <t>MGSL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>333.95</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="C39" t="n">
-        <v>350.15</v>
+        <v>69</v>
       </c>
       <c r="D39" t="n">
-        <v>4.85</v>
+        <v>4.39</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ANMOL</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>15.27</v>
+        <v>1.83</v>
       </c>
       <c r="C40" t="n">
-        <v>15.99</v>
+        <v>1.91</v>
       </c>
       <c r="D40" t="n">
-        <v>4.72</v>
+        <v>4.37</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>SADBHIN</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>20.98</v>
+        <v>2.55</v>
       </c>
       <c r="C41" t="n">
-        <v>21.97</v>
+        <v>2.66</v>
       </c>
       <c r="D41" t="n">
-        <v>4.72</v>
+        <v>4.31</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SIEL</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>31.5</v>
+        <v>0.71</v>
       </c>
       <c r="C42" t="n">
-        <v>32.98</v>
+        <v>0.74</v>
       </c>
       <c r="D42" t="n">
-        <v>4.7</v>
+        <v>4.23</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>GLASSWALL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3.65</v>
+        <v>214.85</v>
       </c>
       <c r="C43" t="n">
-        <v>3.82</v>
+        <v>223.75</v>
       </c>
       <c r="D43" t="n">
-        <v>4.66</v>
+        <v>4.14</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>SOMICONVEY</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>14.98</v>
+        <v>94.11</v>
       </c>
       <c r="C44" t="n">
-        <v>15.67</v>
+        <v>98</v>
       </c>
       <c r="D44" t="n">
-        <v>4.61</v>
+        <v>4.13</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>KAMANWALA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>169.21</v>
+        <v>17.24</v>
       </c>
       <c r="C45" t="n">
-        <v>176.99</v>
+        <v>17.95</v>
       </c>
       <c r="D45" t="n">
-        <v>4.6</v>
+        <v>4.12</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ESSARSHPNG</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>15.76</v>
+        <v>16.33</v>
       </c>
       <c r="C46" t="n">
-        <v>16.48</v>
+        <v>17</v>
       </c>
       <c r="D46" t="n">
-        <v>4.57</v>
+        <v>4.1</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>LAXMICOT</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>16.84</v>
+        <v>13.22</v>
       </c>
       <c r="C47" t="n">
-        <v>17.6</v>
+        <v>13.76</v>
       </c>
       <c r="D47" t="n">
-        <v>4.51</v>
+        <v>4.08</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1477,13 +1477,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>151.6</v>
+        <v>155.58</v>
       </c>
       <c r="C48" t="n">
-        <v>158.44</v>
+        <v>161.88</v>
       </c>
       <c r="D48" t="n">
-        <v>4.51</v>
+        <v>4.05</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LAHOTIOV</t>
+          <t>HILINFRA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>39.28</v>
+        <v>43.83</v>
       </c>
       <c r="C49" t="n">
-        <v>40.99</v>
+        <v>45.6</v>
       </c>
       <c r="D49" t="n">
-        <v>4.35</v>
+        <v>4.04</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GRAVISSHO</t>
+          <t>HBPOR</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>46.97</v>
+        <v>62.3</v>
       </c>
       <c r="C50" t="n">
-        <v>49</v>
+        <v>64.75</v>
       </c>
       <c r="D50" t="n">
-        <v>4.32</v>
+        <v>3.93</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GEECEE</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>350.1</v>
+        <v>5.87</v>
       </c>
       <c r="C51" t="n">
-        <v>365</v>
+        <v>6.1</v>
       </c>
       <c r="D51" t="n">
-        <v>4.26</v>
+        <v>3.92</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BANG</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>32.29</v>
+        <v>384.95</v>
       </c>
       <c r="C52" t="n">
-        <v>33.65</v>
+        <v>399.9</v>
       </c>
       <c r="D52" t="n">
-        <v>4.21</v>
+        <v>3.88</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>15.83</v>
+        <v>10.08</v>
       </c>
       <c r="C53" t="n">
-        <v>16.48</v>
+        <v>10.47</v>
       </c>
       <c r="D53" t="n">
-        <v>4.11</v>
+        <v>3.87</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>11.43</v>
+        <v>56.98</v>
       </c>
       <c r="C54" t="n">
-        <v>11.9</v>
+        <v>59.18</v>
       </c>
       <c r="D54" t="n">
-        <v>4.11</v>
+        <v>3.86</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>22.31</v>
+        <v>47.12</v>
       </c>
       <c r="C55" t="n">
-        <v>23.2</v>
+        <v>48.9</v>
       </c>
       <c r="D55" t="n">
-        <v>3.99</v>
+        <v>3.78</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PANCHMAHQ</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>293.4</v>
+        <v>19.71</v>
       </c>
       <c r="C56" t="n">
-        <v>304.85</v>
+        <v>20.45</v>
       </c>
       <c r="D56" t="n">
-        <v>3.9</v>
+        <v>3.75</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SNOWMAN</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>35.03</v>
+        <v>20.2</v>
       </c>
       <c r="C57" t="n">
-        <v>36.39</v>
+        <v>20.95</v>
       </c>
       <c r="D57" t="n">
-        <v>3.88</v>
+        <v>3.71</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>JAYESH</t>
+          <t>EMMBI</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>125.1</v>
+        <v>87.75</v>
       </c>
       <c r="C58" t="n">
-        <v>129.95</v>
+        <v>90.95</v>
       </c>
       <c r="D58" t="n">
-        <v>3.88</v>
+        <v>3.65</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>42.75</v>
+        <v>7.69</v>
       </c>
       <c r="C59" t="n">
-        <v>44.4</v>
+        <v>7.97</v>
       </c>
       <c r="D59" t="n">
-        <v>3.86</v>
+        <v>3.64</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LANCER</t>
+          <t>NEUEON</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>12.47</v>
+        <v>11.09</v>
       </c>
       <c r="C60" t="n">
-        <v>12.95</v>
+        <v>11.49</v>
       </c>
       <c r="D60" t="n">
-        <v>3.85</v>
+        <v>3.61</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>LATTEYS</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>81.40000000000001</v>
+        <v>20.65</v>
       </c>
       <c r="C61" t="n">
-        <v>84.5</v>
+        <v>21.39</v>
       </c>
       <c r="D61" t="n">
-        <v>3.81</v>
+        <v>3.58</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SUNSHIEL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1209.3</v>
+        <v>0.28</v>
       </c>
       <c r="C62" t="n">
-        <v>1255</v>
+        <v>0.29</v>
       </c>
       <c r="D62" t="n">
-        <v>3.78</v>
+        <v>3.57</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>COMPINFO</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1.06</v>
+        <v>13.52</v>
       </c>
       <c r="C63" t="n">
-        <v>1.1</v>
+        <v>14</v>
       </c>
       <c r="D63" t="n">
-        <v>3.77</v>
+        <v>3.55</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>GUJAPOLLO</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>37.4</v>
+        <v>338.1</v>
       </c>
       <c r="C64" t="n">
-        <v>38.8</v>
+        <v>349.85</v>
       </c>
       <c r="D64" t="n">
-        <v>3.74</v>
+        <v>3.48</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>SONAMLTD</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>131.25</v>
+        <v>71.44</v>
       </c>
       <c r="C65" t="n">
-        <v>136.15</v>
+        <v>73.89</v>
       </c>
       <c r="D65" t="n">
-        <v>3.73</v>
+        <v>3.43</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.27</v>
+        <v>2.34</v>
       </c>
       <c r="C66" t="n">
-        <v>0.28</v>
+        <v>2.42</v>
       </c>
       <c r="D66" t="n">
-        <v>3.7</v>
+        <v>3.42</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>MAKERSL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>737.9</v>
+        <v>177.92</v>
       </c>
       <c r="C67" t="n">
-        <v>765</v>
+        <v>184</v>
       </c>
       <c r="D67" t="n">
-        <v>3.67</v>
+        <v>3.42</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>26.71</v>
+        <v>18.01</v>
       </c>
       <c r="C68" t="n">
-        <v>27.68</v>
+        <v>18.6</v>
       </c>
       <c r="D68" t="n">
-        <v>3.63</v>
+        <v>3.28</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>6.88</v>
+        <v>31.79</v>
       </c>
       <c r="C69" t="n">
-        <v>7.13</v>
+        <v>32.83</v>
       </c>
       <c r="D69" t="n">
-        <v>3.63</v>
+        <v>3.27</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MIIL</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>666.1</v>
+        <v>994.45</v>
       </c>
       <c r="C70" t="n">
-        <v>689.95</v>
+        <v>1026.95</v>
       </c>
       <c r="D70" t="n">
-        <v>3.58</v>
+        <v>3.27</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ANSALBU</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>84</v>
+        <v>133.61</v>
       </c>
       <c r="C71" t="n">
-        <v>86.98999999999999</v>
+        <v>137.95</v>
       </c>
       <c r="D71" t="n">
-        <v>3.56</v>
+        <v>3.25</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>44.4</v>
+        <v>61.02</v>
       </c>
       <c r="C72" t="n">
-        <v>45.98</v>
+        <v>62.99</v>
       </c>
       <c r="D72" t="n">
-        <v>3.56</v>
+        <v>3.23</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>KSR</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>7.62</v>
+        <v>46.52</v>
       </c>
       <c r="C73" t="n">
-        <v>7.89</v>
+        <v>47.99</v>
       </c>
       <c r="D73" t="n">
-        <v>3.54</v>
+        <v>3.16</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BENARAS</t>
+          <t>EMAMIREAL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>11001</v>
+        <v>66.31</v>
       </c>
       <c r="C74" t="n">
-        <v>11390</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D74" t="n">
-        <v>3.54</v>
+        <v>3.15</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>NTCIND</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>134.11</v>
+        <v>23.76</v>
       </c>
       <c r="C75" t="n">
-        <v>138.8</v>
+        <v>24.5</v>
       </c>
       <c r="D75" t="n">
-        <v>3.5</v>
+        <v>3.11</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>23.47</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="C76" t="n">
-        <v>24.29</v>
+        <v>8.99</v>
       </c>
       <c r="D76" t="n">
-        <v>3.49</v>
+        <v>3.1</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>LAMBODHARA</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>78.29000000000001</v>
+        <v>117.76</v>
       </c>
       <c r="C77" t="n">
-        <v>81</v>
+        <v>121.4</v>
       </c>
       <c r="D77" t="n">
-        <v>3.46</v>
+        <v>3.09</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>37.2</v>
+        <v>24.59</v>
       </c>
       <c r="C78" t="n">
-        <v>38.45</v>
+        <v>25.35</v>
       </c>
       <c r="D78" t="n">
-        <v>3.36</v>
+        <v>3.09</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>RKDL</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>18</v>
+        <v>16.95</v>
       </c>
       <c r="C79" t="n">
-        <v>18.59</v>
+        <v>17.47</v>
       </c>
       <c r="D79" t="n">
-        <v>3.28</v>
+        <v>3.07</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>8.619999999999999</v>
+        <v>12.48</v>
       </c>
       <c r="C80" t="n">
-        <v>8.9</v>
+        <v>12.86</v>
       </c>
       <c r="D80" t="n">
-        <v>3.25</v>
+        <v>3.04</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>DEEP</t>
+          <t>PRANAV</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>45.13</v>
+        <v>106.81</v>
       </c>
       <c r="C81" t="n">
-        <v>46.59</v>
+        <v>110</v>
       </c>
       <c r="D81" t="n">
-        <v>3.24</v>
+        <v>2.99</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>HINDADH</t>
+          <t>RUBFILA</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>371.95</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="C82" t="n">
-        <v>384</v>
+        <v>66.95999999999999</v>
       </c>
       <c r="D82" t="n">
-        <v>3.24</v>
+        <v>2.95</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>DELTAMAGNT</t>
+          <t>KOTHARIPRO</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>55.65</v>
+        <v>64.14</v>
       </c>
       <c r="C83" t="n">
-        <v>57.45</v>
+        <v>66</v>
       </c>
       <c r="D83" t="n">
-        <v>3.23</v>
+        <v>2.9</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>43.5</v>
+        <v>93.34999999999999</v>
       </c>
       <c r="C84" t="n">
-        <v>44.9</v>
+        <v>96</v>
       </c>
       <c r="D84" t="n">
-        <v>3.22</v>
+        <v>2.84</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>MANAKSTEEL</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>16.94</v>
+        <v>106.42</v>
       </c>
       <c r="C85" t="n">
-        <v>17.48</v>
+        <v>109.4</v>
       </c>
       <c r="D85" t="n">
-        <v>3.19</v>
+        <v>2.8</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>INDTERRAIN</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>28.01</v>
+        <v>74.62</v>
       </c>
       <c r="C86" t="n">
-        <v>28.9</v>
+        <v>76.7</v>
       </c>
       <c r="D86" t="n">
-        <v>3.18</v>
+        <v>2.79</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>5.67</v>
+        <v>96.22</v>
       </c>
       <c r="C87" t="n">
-        <v>5.85</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="D87" t="n">
-        <v>3.17</v>
+        <v>2.79</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>255.9</v>
+        <v>0.36</v>
       </c>
       <c r="C88" t="n">
-        <v>263.9</v>
+        <v>0.37</v>
       </c>
       <c r="D88" t="n">
-        <v>3.13</v>
+        <v>2.78</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RUDRA</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>20.16</v>
+        <v>65.17</v>
       </c>
       <c r="C89" t="n">
-        <v>20.79</v>
+        <v>66.94</v>
       </c>
       <c r="D89" t="n">
-        <v>3.12</v>
+        <v>2.72</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>UNIENTER</t>
+          <t>ALPINETEX</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>89.22</v>
+        <v>52.33</v>
       </c>
       <c r="C90" t="n">
-        <v>91.98999999999999</v>
+        <v>53.75</v>
       </c>
       <c r="D90" t="n">
-        <v>3.1</v>
+        <v>2.71</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>24.88</v>
+        <v>37</v>
       </c>
       <c r="C91" t="n">
-        <v>25.65</v>
+        <v>38</v>
       </c>
       <c r="D91" t="n">
-        <v>3.09</v>
+        <v>2.7</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>WEWIN</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>14.65</v>
+        <v>41.87</v>
       </c>
       <c r="C92" t="n">
-        <v>15.1</v>
+        <v>43</v>
       </c>
       <c r="D92" t="n">
-        <v>3.07</v>
+        <v>2.7</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>KAUSHALYA</t>
+          <t>JINDWORLD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>834.5</v>
+        <v>49.16</v>
       </c>
       <c r="C93" t="n">
-        <v>859.75</v>
+        <v>50.48</v>
       </c>
       <c r="D93" t="n">
-        <v>3.03</v>
+        <v>2.69</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>8.57</v>
+        <v>22.99</v>
       </c>
       <c r="C94" t="n">
-        <v>8.83</v>
+        <v>23.6</v>
       </c>
       <c r="D94" t="n">
-        <v>3.03</v>
+        <v>2.65</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>S&amp;SPOWER</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>237.78</v>
+        <v>321.35</v>
       </c>
       <c r="C95" t="n">
-        <v>244.9</v>
+        <v>329.8</v>
       </c>
       <c r="D95" t="n">
-        <v>2.99</v>
+        <v>2.63</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>BPLPHARMA</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>3.39</v>
+        <v>1509.8</v>
       </c>
       <c r="C96" t="n">
-        <v>3.49</v>
+        <v>1549.2</v>
       </c>
       <c r="D96" t="n">
-        <v>2.95</v>
+        <v>2.61</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>88.3</v>
+        <v>13.06</v>
       </c>
       <c r="C97" t="n">
-        <v>90.90000000000001</v>
+        <v>13.4</v>
       </c>
       <c r="D97" t="n">
-        <v>2.94</v>
+        <v>2.6</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.68</v>
+        <v>17.52</v>
       </c>
       <c r="C98" t="n">
-        <v>0.7</v>
+        <v>17.97</v>
       </c>
       <c r="D98" t="n">
-        <v>2.94</v>
+        <v>2.57</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ICDSLTD</t>
+          <t>TURTLEMINT</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>63.15</v>
+        <v>127.74</v>
       </c>
       <c r="C99" t="n">
-        <v>64.98999999999999</v>
+        <v>131</v>
       </c>
       <c r="D99" t="n">
-        <v>2.91</v>
+        <v>2.55</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SICAGEN</t>
+          <t>AAREYDRUGS</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>53.98</v>
+        <v>99.94</v>
       </c>
       <c r="C100" t="n">
-        <v>55.55</v>
+        <v>102.49</v>
       </c>
       <c r="D100" t="n">
-        <v>2.91</v>
+        <v>2.55</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>35.47</v>
+        <v>51.98</v>
       </c>
       <c r="C101" t="n">
-        <v>36.49</v>
+        <v>53.3</v>
       </c>
       <c r="D101" t="n">
-        <v>2.88</v>
+        <v>2.54</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DEEPA</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>169.14</v>
+        <v>26.52</v>
       </c>
       <c r="C102" t="n">
-        <v>173.99</v>
+        <v>27.18</v>
       </c>
       <c r="D102" t="n">
-        <v>2.87</v>
+        <v>2.49</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>DIAMINESQ</t>
+          <t>IVC</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>251.8</v>
+        <v>7.76</v>
       </c>
       <c r="C103" t="n">
-        <v>259</v>
+        <v>7.95</v>
       </c>
       <c r="D103" t="n">
-        <v>2.86</v>
+        <v>2.45</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>ARENTERP</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>4.9</v>
+        <v>32.6</v>
       </c>
       <c r="C104" t="n">
-        <v>5.04</v>
+        <v>33.4</v>
       </c>
       <c r="D104" t="n">
-        <v>2.86</v>
+        <v>2.45</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1.06</v>
+        <v>39.39</v>
       </c>
       <c r="C105" t="n">
-        <v>1.09</v>
+        <v>40.35</v>
       </c>
       <c r="D105" t="n">
-        <v>2.83</v>
+        <v>2.44</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>KOHINOOR</t>
+          <t>DHATRE</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>29.58</v>
+        <v>4.11</v>
       </c>
       <c r="C106" t="n">
-        <v>30.4</v>
+        <v>4.21</v>
       </c>
       <c r="D106" t="n">
-        <v>2.77</v>
+        <v>2.43</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>DREAMFOLKS</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>5.83</v>
+        <v>65.33</v>
       </c>
       <c r="C107" t="n">
-        <v>5.99</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D107" t="n">
-        <v>2.74</v>
+        <v>2.4</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>KARMAENG</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>5012.4</v>
+        <v>38.72</v>
       </c>
       <c r="C108" t="n">
-        <v>5148</v>
+        <v>39.65</v>
       </c>
       <c r="D108" t="n">
-        <v>2.71</v>
+        <v>2.4</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MAHSCOOTER</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>12882</v>
+        <v>1902.6</v>
       </c>
       <c r="C109" t="n">
-        <v>13231</v>
+        <v>1948</v>
       </c>
       <c r="D109" t="n">
-        <v>2.71</v>
+        <v>2.39</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>SILVER001</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>225.91</v>
+        <v>23.12</v>
       </c>
       <c r="C110" t="n">
-        <v>232</v>
+        <v>23.67</v>
       </c>
       <c r="D110" t="n">
-        <v>2.7</v>
+        <v>2.38</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>ISFT</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.37</v>
+        <v>75.22</v>
       </c>
       <c r="C111" t="n">
-        <v>0.38</v>
+        <v>77</v>
       </c>
       <c r="D111" t="n">
-        <v>2.7</v>
+        <v>2.37</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>PGIL</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1141.4</v>
+        <v>250.95</v>
       </c>
       <c r="C112" t="n">
-        <v>1171.6</v>
+        <v>256.85</v>
       </c>
       <c r="D112" t="n">
-        <v>2.65</v>
+        <v>2.35</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AMBICAAGAR</t>
+          <t>RAMAPHO</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>24.94</v>
+        <v>115.18</v>
       </c>
       <c r="C113" t="n">
-        <v>25.6</v>
+        <v>117.89</v>
       </c>
       <c r="D113" t="n">
-        <v>2.65</v>
+        <v>2.35</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SPLIL</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>28.84</v>
+        <v>3.41</v>
       </c>
       <c r="C114" t="n">
-        <v>29.6</v>
+        <v>3.49</v>
       </c>
       <c r="D114" t="n">
-        <v>2.64</v>
+        <v>2.35</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>RPPINFRA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.77</v>
+        <v>53.56</v>
       </c>
       <c r="C115" t="n">
-        <v>0.79</v>
+        <v>54.8</v>
       </c>
       <c r="D115" t="n">
-        <v>2.6</v>
+        <v>2.32</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>LAKSHMIMIL</t>
+          <t>MALUPAPER</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>7565</v>
+        <v>31.66</v>
       </c>
       <c r="C116" t="n">
-        <v>7760</v>
+        <v>32.39</v>
       </c>
       <c r="D116" t="n">
-        <v>2.58</v>
+        <v>2.31</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>DHATRE</t>
+          <t>KANOHAR</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>4.29</v>
+        <v>751.5</v>
       </c>
       <c r="C117" t="n">
-        <v>4.4</v>
+        <v>768.7</v>
       </c>
       <c r="D117" t="n">
-        <v>2.56</v>
+        <v>2.29</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>HGS</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>381.6</v>
+        <v>107.54</v>
       </c>
       <c r="C118" t="n">
-        <v>391.35</v>
+        <v>110</v>
       </c>
       <c r="D118" t="n">
-        <v>2.56</v>
+        <v>2.29</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>MAHEPC</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>77.91</v>
+        <v>101.18</v>
       </c>
       <c r="C119" t="n">
-        <v>79.90000000000001</v>
+        <v>103.49</v>
       </c>
       <c r="D119" t="n">
-        <v>2.55</v>
+        <v>2.28</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>FINOPB</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>137.73</v>
+        <v>162.29</v>
       </c>
       <c r="C120" t="n">
-        <v>141.23</v>
+        <v>165.99</v>
       </c>
       <c r="D120" t="n">
-        <v>2.54</v>
+        <v>2.28</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>1431.9</v>
+        <v>24.69</v>
       </c>
       <c r="C121" t="n">
-        <v>1468.3</v>
+        <v>25.25</v>
       </c>
       <c r="D121" t="n">
-        <v>2.54</v>
+        <v>2.27</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>132.68</v>
+        <v>220.37</v>
       </c>
       <c r="C122" t="n">
-        <v>136</v>
+        <v>225.37</v>
       </c>
       <c r="D122" t="n">
-        <v>2.5</v>
+        <v>2.27</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RELCHEMQ</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>120.7</v>
+        <v>1515.8</v>
       </c>
       <c r="C123" t="n">
-        <v>123.71</v>
+        <v>1550</v>
       </c>
       <c r="D123" t="n">
-        <v>2.49</v>
+        <v>2.26</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>WEL</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>69.18000000000001</v>
+        <v>1.33</v>
       </c>
       <c r="C124" t="n">
-        <v>70.90000000000001</v>
+        <v>1.36</v>
       </c>
       <c r="D124" t="n">
-        <v>2.49</v>
+        <v>2.26</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ARVEE</t>
+          <t>SALONA</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>168.6</v>
+        <v>264</v>
       </c>
       <c r="C125" t="n">
-        <v>172.8</v>
+        <v>269.95</v>
       </c>
       <c r="D125" t="n">
-        <v>2.49</v>
+        <v>2.25</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>MALLCOM</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>6.44</v>
+        <v>924.3</v>
       </c>
       <c r="C126" t="n">
-        <v>6.6</v>
+        <v>945</v>
       </c>
       <c r="D126" t="n">
-        <v>2.48</v>
+        <v>2.24</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>15.85</v>
+        <v>11.2</v>
       </c>
       <c r="C127" t="n">
-        <v>16.24</v>
+        <v>11.45</v>
       </c>
       <c r="D127" t="n">
-        <v>2.46</v>
+        <v>2.23</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>10.22</v>
+        <v>5.86</v>
       </c>
       <c r="C128" t="n">
-        <v>10.47</v>
+        <v>5.99</v>
       </c>
       <c r="D128" t="n">
-        <v>2.45</v>
+        <v>2.22</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>TRITONV</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>1051.5</v>
+        <v>428.4</v>
       </c>
       <c r="C129" t="n">
-        <v>1077</v>
+        <v>437.85</v>
       </c>
       <c r="D129" t="n">
-        <v>2.43</v>
+        <v>2.21</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>19.28</v>
+        <v>46.73</v>
       </c>
       <c r="C130" t="n">
-        <v>19.74</v>
+        <v>47.75</v>
       </c>
       <c r="D130" t="n">
-        <v>2.39</v>
+        <v>2.18</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>JUNIPER</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>29.45</v>
+        <v>214.32</v>
       </c>
       <c r="C131" t="n">
-        <v>30.15</v>
+        <v>219</v>
       </c>
       <c r="D131" t="n">
-        <v>2.38</v>
+        <v>2.18</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>GANGESSECU</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>89.84999999999999</v>
+        <v>115.01</v>
       </c>
       <c r="C132" t="n">
-        <v>91.98999999999999</v>
+        <v>117.49</v>
       </c>
       <c r="D132" t="n">
-        <v>2.38</v>
+        <v>2.16</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>24.42</v>
+        <v>2.79</v>
       </c>
       <c r="C133" t="n">
-        <v>25</v>
+        <v>2.85</v>
       </c>
       <c r="D133" t="n">
-        <v>2.38</v>
+        <v>2.15</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SONATSOFTW</t>
+          <t>AKSHOPTFBR</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>281.3</v>
+        <v>7.96</v>
       </c>
       <c r="C134" t="n">
-        <v>287.95</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="D134" t="n">
-        <v>2.36</v>
+        <v>2.14</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>MVKAGRO</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1.71</v>
+        <v>270.65</v>
       </c>
       <c r="C135" t="n">
-        <v>1.75</v>
+        <v>276.4</v>
       </c>
       <c r="D135" t="n">
-        <v>2.34</v>
+        <v>2.12</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>7.77</v>
+        <v>68.06999999999999</v>
       </c>
       <c r="C136" t="n">
-        <v>7.95</v>
+        <v>69.48999999999999</v>
       </c>
       <c r="D136" t="n">
-        <v>2.32</v>
+        <v>2.09</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>STARPAPER</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>160.27</v>
+        <v>30.56</v>
       </c>
       <c r="C137" t="n">
-        <v>163.99</v>
+        <v>31.2</v>
       </c>
       <c r="D137" t="n">
-        <v>2.32</v>
+        <v>2.09</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>14.47</v>
+        <v>7.74</v>
       </c>
       <c r="C138" t="n">
-        <v>14.8</v>
+        <v>7.9</v>
       </c>
       <c r="D138" t="n">
-        <v>2.28</v>
+        <v>2.07</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>ADVIKCA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>8.789999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="C139" t="n">
-        <v>8.99</v>
+        <v>0.99</v>
       </c>
       <c r="D139" t="n">
-        <v>2.28</v>
+        <v>2.06</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GROWWSLVR</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>22</v>
+        <v>2.44</v>
       </c>
       <c r="C140" t="n">
-        <v>22.5</v>
+        <v>2.49</v>
       </c>
       <c r="D140" t="n">
-        <v>2.27</v>
+        <v>2.05</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SAKHTISUG</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>18.95</v>
+        <v>0.98</v>
       </c>
       <c r="C141" t="n">
-        <v>19.38</v>
+        <v>1</v>
       </c>
       <c r="D141" t="n">
-        <v>2.27</v>
+        <v>2.04</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CREATIVEYE</t>
+          <t>APOLSINHOT</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>5.74</v>
+        <v>1185.8</v>
       </c>
       <c r="C142" t="n">
-        <v>5.87</v>
+        <v>1210</v>
       </c>
       <c r="D142" t="n">
-        <v>2.26</v>
+        <v>2.04</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>HLVLTD</t>
+          <t>RAMASTEEL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>6.26</v>
+        <v>3.92</v>
       </c>
       <c r="C143" t="n">
-        <v>6.4</v>
+        <v>4</v>
       </c>
       <c r="D143" t="n">
-        <v>2.24</v>
+        <v>2.04</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>MHLXMIRU</t>
+          <t>AASTHA</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>156.39</v>
+        <v>74.33</v>
       </c>
       <c r="C144" t="n">
-        <v>159.9</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="D144" t="n">
-        <v>2.24</v>
+        <v>2.04</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>63.09</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="C145" t="n">
-        <v>64.48999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="D145" t="n">
-        <v>2.22</v>
+        <v>2.03</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ISHANCH</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>43.73</v>
+        <v>3.96</v>
       </c>
       <c r="C146" t="n">
-        <v>44.7</v>
+        <v>4.04</v>
       </c>
       <c r="D146" t="n">
-        <v>2.22</v>
+        <v>2.02</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>AAREYDRUGS</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>98.81999999999999</v>
+        <v>25.68</v>
       </c>
       <c r="C147" t="n">
-        <v>101</v>
+        <v>26.2</v>
       </c>
       <c r="D147" t="n">
-        <v>2.21</v>
+        <v>2.02</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>NECLIFE</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>6.79</v>
+        <v>10.9</v>
       </c>
       <c r="C148" t="n">
-        <v>6.94</v>
+        <v>11.12</v>
       </c>
       <c r="D148" t="n">
-        <v>2.21</v>
+        <v>2.02</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>YESBANK</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>23.07</v>
+        <v>74.20999999999999</v>
       </c>
       <c r="C149" t="n">
-        <v>23.58</v>
+        <v>75.70999999999999</v>
       </c>
       <c r="D149" t="n">
-        <v>2.21</v>
+        <v>2.02</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>10.47</v>
+        <v>21.42</v>
       </c>
       <c r="C150" t="n">
-        <v>10.7</v>
+        <v>21.85</v>
       </c>
       <c r="D150" t="n">
-        <v>2.2</v>
+        <v>2.01</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>CRSL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>46.58</v>
+        <v>2.49</v>
       </c>
       <c r="C151" t="n">
-        <v>47.6</v>
+        <v>2.54</v>
       </c>
       <c r="D151" t="n">
-        <v>2.19</v>
+        <v>2.01</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PINELABS</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>193.8</v>
+        <v>14.5</v>
       </c>
       <c r="C152" t="n">
-        <v>198</v>
+        <v>14.79</v>
       </c>
       <c r="D152" t="n">
-        <v>2.17</v>
+        <v>2</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>DTIL</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>138.3</v>
+        <v>103.49</v>
       </c>
       <c r="C153" t="n">
-        <v>141.3</v>
+        <v>105.55</v>
       </c>
       <c r="D153" t="n">
-        <v>2.17</v>
+        <v>1.99</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SURAJLTD</t>
+          <t>AUSTENG</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>195.75</v>
+        <v>126.95</v>
       </c>
       <c r="C154" t="n">
-        <v>200</v>
+        <v>129.48</v>
       </c>
       <c r="D154" t="n">
-        <v>2.17</v>
+        <v>1.99</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>VTMLTD</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>7.82</v>
+        <v>48.83</v>
       </c>
       <c r="C155" t="n">
-        <v>7.99</v>
+        <v>49.8</v>
       </c>
       <c r="D155" t="n">
-        <v>2.17</v>
+        <v>1.99</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>CMSINFO</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>3.27</v>
+        <v>232.39</v>
       </c>
       <c r="C156" t="n">
-        <v>3.34</v>
+        <v>237</v>
       </c>
       <c r="D156" t="n">
-        <v>2.14</v>
+        <v>1.98</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>GENUSPAPER</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>4.22</v>
+        <v>11.11</v>
       </c>
       <c r="C157" t="n">
-        <v>4.31</v>
+        <v>11.33</v>
       </c>
       <c r="D157" t="n">
-        <v>2.13</v>
+        <v>1.98</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>2.35</v>
+        <v>19.3</v>
       </c>
       <c r="C158" t="n">
-        <v>2.4</v>
+        <v>19.68</v>
       </c>
       <c r="D158" t="n">
-        <v>2.13</v>
+        <v>1.97</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>1.88</v>
+        <v>7.11</v>
       </c>
       <c r="C159" t="n">
-        <v>1.92</v>
+        <v>7.25</v>
       </c>
       <c r="D159" t="n">
-        <v>2.13</v>
+        <v>1.97</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>MEIL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>474.95</v>
+        <v>268.6</v>
       </c>
       <c r="C160" t="n">
-        <v>485</v>
+        <v>273.9</v>
       </c>
       <c r="D160" t="n">
-        <v>2.12</v>
+        <v>1.97</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>64.52</v>
+        <v>8.68</v>
       </c>
       <c r="C161" t="n">
-        <v>65.88</v>
+        <v>8.85</v>
       </c>
       <c r="D161" t="n">
-        <v>2.11</v>
+        <v>1.96</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>99.40000000000001</v>
+        <v>5121.2</v>
       </c>
       <c r="C162" t="n">
-        <v>101.5</v>
+        <v>5220</v>
       </c>
       <c r="D162" t="n">
-        <v>2.11</v>
+        <v>1.93</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>NDTV</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>70.43000000000001</v>
+        <v>45.6</v>
       </c>
       <c r="C163" t="n">
-        <v>71.91</v>
+        <v>46.48</v>
       </c>
       <c r="D163" t="n">
-        <v>2.1</v>
+        <v>1.93</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>4.28</v>
+        <v>547.5</v>
       </c>
       <c r="C164" t="n">
-        <v>4.37</v>
+        <v>558</v>
       </c>
       <c r="D164" t="n">
-        <v>2.1</v>
+        <v>1.92</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>HRYNSHP</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>2.38</v>
+        <v>100</v>
       </c>
       <c r="C165" t="n">
-        <v>2.43</v>
+        <v>101.9</v>
       </c>
       <c r="D165" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>21STCENMGM</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>20.57</v>
+        <v>38.37</v>
       </c>
       <c r="C166" t="n">
-        <v>21</v>
+        <v>39.1</v>
       </c>
       <c r="D166" t="n">
-        <v>2.09</v>
+        <v>1.9</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>12.91</v>
+        <v>164.29</v>
       </c>
       <c r="C167" t="n">
-        <v>13.18</v>
+        <v>167.4</v>
       </c>
       <c r="D167" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MOLBIO</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>1356.8</v>
+        <v>42.55</v>
       </c>
       <c r="C168" t="n">
-        <v>1385</v>
+        <v>43.35</v>
       </c>
       <c r="D168" t="n">
-        <v>2.08</v>
+        <v>1.88</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>POEL</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>139.45</v>
+        <v>12.84</v>
       </c>
       <c r="C169" t="n">
-        <v>142.35</v>
+        <v>13.08</v>
       </c>
       <c r="D169" t="n">
-        <v>2.08</v>
+        <v>1.87</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>BAGFILMS</t>
+          <t>MUNJALSHOW</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>4.35</v>
+        <v>124.67</v>
       </c>
       <c r="C170" t="n">
-        <v>4.44</v>
+        <v>127</v>
       </c>
       <c r="D170" t="n">
-        <v>2.07</v>
+        <v>1.87</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ACCURACY</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>4.38</v>
+        <v>14.48</v>
       </c>
       <c r="C171" t="n">
-        <v>4.47</v>
+        <v>14.75</v>
       </c>
       <c r="D171" t="n">
-        <v>2.05</v>
+        <v>1.86</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>6.35</v>
+        <v>5.38</v>
       </c>
       <c r="C172" t="n">
-        <v>6.48</v>
+        <v>5.48</v>
       </c>
       <c r="D172" t="n">
-        <v>2.05</v>
+        <v>1.86</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>MVGJL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>3.92</v>
+        <v>207.16</v>
       </c>
       <c r="C173" t="n">
-        <v>4</v>
+        <v>211</v>
       </c>
       <c r="D173" t="n">
-        <v>2.04</v>
+        <v>1.85</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>9.82</v>
+        <v>41.29</v>
       </c>
       <c r="C174" t="n">
-        <v>10.02</v>
+        <v>42.05</v>
       </c>
       <c r="D174" t="n">
-        <v>2.04</v>
+        <v>1.84</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>TITAGARH</t>
+          <t>TEJA</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>811.45</v>
+        <v>207.2</v>
       </c>
       <c r="C175" t="n">
-        <v>828</v>
+        <v>211</v>
       </c>
       <c r="D175" t="n">
-        <v>2.04</v>
+        <v>1.83</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>367.5</v>
+        <v>1995.5</v>
       </c>
       <c r="C176" t="n">
-        <v>375</v>
+        <v>2032</v>
       </c>
       <c r="D176" t="n">
-        <v>2.04</v>
+        <v>1.83</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>20.29</v>
+        <v>204.77</v>
       </c>
       <c r="C177" t="n">
-        <v>20.7</v>
+        <v>208.49</v>
       </c>
       <c r="D177" t="n">
-        <v>2.02</v>
+        <v>1.82</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>STEELCITY</t>
+          <t>AVALON</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>86.12</v>
+        <v>2216.1</v>
       </c>
       <c r="C178" t="n">
-        <v>87.86</v>
+        <v>2256</v>
       </c>
       <c r="D178" t="n">
-        <v>2.02</v>
+        <v>1.8</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HINDALUMI</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>95.09</v>
+        <v>1.67</v>
       </c>
       <c r="C179" t="n">
-        <v>97</v>
+        <v>1.7</v>
       </c>
       <c r="D179" t="n">
-        <v>2.01</v>
+        <v>1.8</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>MANOMAY</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>34.02</v>
+        <v>223.85</v>
       </c>
       <c r="C180" t="n">
-        <v>34.7</v>
+        <v>227.89</v>
       </c>
       <c r="D180" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>2.5</v>
+        <v>712.05</v>
       </c>
       <c r="C181" t="n">
-        <v>2.55</v>
+        <v>724.8</v>
       </c>
       <c r="D181" t="n">
-        <v>2</v>
+        <v>1.79</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>277.45</v>
+        <v>6846.5</v>
       </c>
       <c r="C182" t="n">
-        <v>282.95</v>
+        <v>6968</v>
       </c>
       <c r="D182" t="n">
-        <v>1.98</v>
+        <v>1.77</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>XCHANGING</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>64.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="C183" t="n">
-        <v>65.78</v>
+        <v>89.15000000000001</v>
       </c>
       <c r="D183" t="n">
-        <v>1.98</v>
+        <v>1.77</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>CHEMCON</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>357.9</v>
+        <v>212.1</v>
       </c>
       <c r="C184" t="n">
-        <v>364.95</v>
+        <v>215.8</v>
       </c>
       <c r="D184" t="n">
-        <v>1.97</v>
+        <v>1.74</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CPEDU</t>
+          <t>SWANDEF</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>176.34</v>
+        <v>2687.2</v>
       </c>
       <c r="C185" t="n">
-        <v>179.8</v>
+        <v>2734</v>
       </c>
       <c r="D185" t="n">
-        <v>1.96</v>
+        <v>1.74</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>WARDINMOBI</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>5.62</v>
+        <v>16.15</v>
       </c>
       <c r="C186" t="n">
-        <v>5.73</v>
+        <v>16.43</v>
       </c>
       <c r="D186" t="n">
-        <v>1.96</v>
+        <v>1.73</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>JMA</t>
+          <t>HINDADH</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>88.95999999999999</v>
+        <v>378.45</v>
       </c>
       <c r="C187" t="n">
-        <v>90.7</v>
+        <v>384.95</v>
       </c>
       <c r="D187" t="n">
-        <v>1.96</v>
+        <v>1.72</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>GVKPIL</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>12.26</v>
+        <v>2.33</v>
       </c>
       <c r="C188" t="n">
-        <v>12.5</v>
+        <v>2.37</v>
       </c>
       <c r="D188" t="n">
-        <v>1.96</v>
+        <v>1.72</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PROZONER</t>
+          <t>VILAS</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>52.72</v>
+        <v>316.25</v>
       </c>
       <c r="C189" t="n">
-        <v>53.75</v>
+        <v>321.7</v>
       </c>
       <c r="D189" t="n">
-        <v>1.95</v>
+        <v>1.72</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>BSL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>1693</v>
+        <v>117.97</v>
       </c>
       <c r="C190" t="n">
-        <v>1725.9</v>
+        <v>119.99</v>
       </c>
       <c r="D190" t="n">
-        <v>1.94</v>
+        <v>1.71</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>LEENEE</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>7.74</v>
+        <v>1.17</v>
       </c>
       <c r="C191" t="n">
-        <v>7.89</v>
+        <v>1.19</v>
       </c>
       <c r="D191" t="n">
-        <v>1.94</v>
+        <v>1.71</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>23.91</v>
+        <v>7.07</v>
       </c>
       <c r="C192" t="n">
-        <v>24.37</v>
+        <v>7.19</v>
       </c>
       <c r="D192" t="n">
-        <v>1.92</v>
+        <v>1.7</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>PARSVNATH</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>0.52</v>
+        <v>1.78</v>
       </c>
       <c r="C193" t="n">
-        <v>0.53</v>
+        <v>1.81</v>
       </c>
       <c r="D193" t="n">
-        <v>1.92</v>
+        <v>1.69</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>RAJOOENG</t>
+          <t>AWL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>53.96</v>
+        <v>181.94</v>
       </c>
       <c r="C194" t="n">
-        <v>54.99</v>
+        <v>185</v>
       </c>
       <c r="D194" t="n">
-        <v>1.91</v>
+        <v>1.68</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>BEPL</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>120.69</v>
+        <v>4.21</v>
       </c>
       <c r="C195" t="n">
-        <v>122.98</v>
+        <v>4.28</v>
       </c>
       <c r="D195" t="n">
-        <v>1.9</v>
+        <v>1.66</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>5.28</v>
+        <v>4.23</v>
       </c>
       <c r="C196" t="n">
-        <v>5.38</v>
+        <v>4.3</v>
       </c>
       <c r="D196" t="n">
-        <v>1.89</v>
+        <v>1.65</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>HEXATRADEX</t>
+          <t>GTPL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>156.06</v>
+        <v>56.46</v>
       </c>
       <c r="C197" t="n">
-        <v>158.99</v>
+        <v>57.39</v>
       </c>
       <c r="D197" t="n">
-        <v>1.88</v>
+        <v>1.65</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>24.46</v>
+        <v>42.7</v>
       </c>
       <c r="C198" t="n">
-        <v>24.92</v>
+        <v>43.4</v>
       </c>
       <c r="D198" t="n">
-        <v>1.88</v>
+        <v>1.64</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>47.11</v>
+        <v>1.84</v>
       </c>
       <c r="C199" t="n">
-        <v>47.99</v>
+        <v>1.87</v>
       </c>
       <c r="D199" t="n">
-        <v>1.87</v>
+        <v>1.63</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>GRAPHITE</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>5.41</v>
+        <v>805.05</v>
       </c>
       <c r="C200" t="n">
-        <v>5.51</v>
+        <v>818</v>
       </c>
       <c r="D200" t="n">
-        <v>1.85</v>
+        <v>1.61</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>OSWALGREEN</t>
+          <t>MEDICO</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>19.59</v>
+        <v>35.33</v>
       </c>
       <c r="C201" t="n">
-        <v>19.95</v>
+        <v>35.9</v>
       </c>
       <c r="D201" t="n">
-        <v>1.84</v>
+        <v>1.61</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-18 08:30 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>ASTAR</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9.199999999999999</v>
+        <v>672.8</v>
       </c>
       <c r="C2" t="n">
-        <v>10.68</v>
+        <v>807.3</v>
       </c>
       <c r="D2" t="n">
-        <v>16.09</v>
+        <v>19.99</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>ISFT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>57.88</v>
+        <v>90.26000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>63.66</v>
+        <v>98.97</v>
       </c>
       <c r="D3" t="n">
-        <v>9.99</v>
+        <v>9.65</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RIR</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>179.77</v>
+        <v>8.26</v>
       </c>
       <c r="C4" t="n">
-        <v>194.74</v>
+        <v>8.99</v>
       </c>
       <c r="D4" t="n">
-        <v>8.33</v>
+        <v>8.84</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,14 +527,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MGEL</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15.6</v>
+        <v>0.13</v>
       </c>
       <c r="C5" t="n">
-        <v>16.8</v>
+        <v>0.14</v>
       </c>
       <c r="D5" t="n">
         <v>7.69</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.13</v>
+        <v>31.97</v>
       </c>
       <c r="C6" t="n">
-        <v>0.14</v>
+        <v>34.4</v>
       </c>
       <c r="D6" t="n">
-        <v>7.69</v>
+        <v>7.6</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KHAITANLTD</t>
+          <t>SKYWAYS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>149.37</v>
+        <v>117.98</v>
       </c>
       <c r="C7" t="n">
-        <v>159.95</v>
+        <v>126.9</v>
       </c>
       <c r="D7" t="n">
-        <v>7.08</v>
+        <v>7.56</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21.49</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>23</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>7.03</v>
+        <v>7.05</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ASTAR</t>
+          <t>DHATRE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>560.7</v>
+        <v>4.12</v>
       </c>
       <c r="C9" t="n">
-        <v>598</v>
+        <v>4.4</v>
       </c>
       <c r="D9" t="n">
-        <v>6.65</v>
+        <v>6.8</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>RENTOMOJO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.45</v>
+        <v>534.25</v>
       </c>
       <c r="C10" t="n">
-        <v>2.6</v>
+        <v>570</v>
       </c>
       <c r="D10" t="n">
-        <v>6.12</v>
+        <v>6.69</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>150.68</v>
+        <v>6.85</v>
       </c>
       <c r="C11" t="n">
-        <v>159.74</v>
+        <v>7.3</v>
       </c>
       <c r="D11" t="n">
-        <v>6.01</v>
+        <v>6.57</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INNOVANA</t>
+          <t>OSWALAGRO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>301.3</v>
+        <v>33.91</v>
       </c>
       <c r="C12" t="n">
-        <v>319</v>
+        <v>35.99</v>
       </c>
       <c r="D12" t="n">
-        <v>5.87</v>
+        <v>6.13</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.49</v>
+        <v>63.66</v>
       </c>
       <c r="C13" t="n">
-        <v>5.8</v>
+        <v>67.52</v>
       </c>
       <c r="D13" t="n">
-        <v>5.65</v>
+        <v>6.06</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ASIANTNE</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9.19</v>
+        <v>1.84</v>
       </c>
       <c r="C14" t="n">
-        <v>9.699999999999999</v>
+        <v>1.95</v>
       </c>
       <c r="D14" t="n">
-        <v>5.55</v>
+        <v>5.98</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AROGRANITE</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22.55</v>
+        <v>2.31</v>
       </c>
       <c r="C15" t="n">
-        <v>23.8</v>
+        <v>2.44</v>
       </c>
       <c r="D15" t="n">
-        <v>5.54</v>
+        <v>5.63</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6.06</v>
+        <v>0.18</v>
       </c>
       <c r="C16" t="n">
-        <v>6.39</v>
+        <v>0.19</v>
       </c>
       <c r="D16" t="n">
-        <v>5.45</v>
+        <v>5.56</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.21</v>
+        <v>56.56</v>
       </c>
       <c r="C17" t="n">
-        <v>2.33</v>
+        <v>59.6</v>
       </c>
       <c r="D17" t="n">
-        <v>5.43</v>
+        <v>5.37</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12.53</v>
+        <v>81.63</v>
       </c>
       <c r="C18" t="n">
-        <v>13.21</v>
+        <v>86</v>
       </c>
       <c r="D18" t="n">
-        <v>5.43</v>
+        <v>5.35</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>19.77</v>
+        <v>5.59</v>
       </c>
       <c r="C19" t="n">
-        <v>20.79</v>
+        <v>5.88</v>
       </c>
       <c r="D19" t="n">
-        <v>5.16</v>
+        <v>5.19</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KRSNAA</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>536.4</v>
+        <v>5.29</v>
       </c>
       <c r="C20" t="n">
-        <v>563.9</v>
+        <v>5.56</v>
       </c>
       <c r="D20" t="n">
-        <v>5.13</v>
+        <v>5.1</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>KRITI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>42.56</v>
+        <v>59.95</v>
       </c>
       <c r="C21" t="n">
-        <v>44.7</v>
+        <v>62.99</v>
       </c>
       <c r="D21" t="n">
-        <v>5.03</v>
+        <v>5.07</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,14 +901,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ONMOBILE</t>
+          <t>BI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>51.81</v>
+        <v>102.5</v>
       </c>
       <c r="C22" t="n">
-        <v>54.4</v>
+        <v>107.62</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -923,14 +923,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>649.25</v>
+        <v>382.47</v>
       </c>
       <c r="C23" t="n">
-        <v>681.7</v>
+        <v>401.59</v>
       </c>
       <c r="D23" t="n">
         <v>5</v>
@@ -945,14 +945,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>364.26</v>
+        <v>145.01</v>
       </c>
       <c r="C24" t="n">
-        <v>382.47</v>
+        <v>152.26</v>
       </c>
       <c r="D24" t="n">
         <v>5</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>KRITINUT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>49.43</v>
+        <v>80.45</v>
       </c>
       <c r="C25" t="n">
-        <v>51.9</v>
+        <v>84.47</v>
       </c>
       <c r="D25" t="n">
         <v>5</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>98.09999999999999</v>
+        <v>51.9</v>
       </c>
       <c r="C26" t="n">
-        <v>103</v>
+        <v>54.49</v>
       </c>
       <c r="D26" t="n">
         <v>4.99</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>23.08</v>
+        <v>500.7</v>
       </c>
       <c r="C27" t="n">
-        <v>24.23</v>
+        <v>525.7</v>
       </c>
       <c r="D27" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BURNPUR</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>16.67</v>
+        <v>318.85</v>
       </c>
       <c r="C28" t="n">
-        <v>17.5</v>
+        <v>334.75</v>
       </c>
       <c r="D28" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GSMFOILS</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>85.84999999999999</v>
+        <v>24.23</v>
       </c>
       <c r="C29" t="n">
-        <v>90.09999999999999</v>
+        <v>25.44</v>
       </c>
       <c r="D29" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FELDVR</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2.05</v>
+        <v>40.91</v>
       </c>
       <c r="C30" t="n">
-        <v>2.15</v>
+        <v>42.95</v>
       </c>
       <c r="D30" t="n">
-        <v>4.88</v>
+        <v>4.99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>476.9</v>
+        <v>574.85</v>
       </c>
       <c r="C31" t="n">
-        <v>500</v>
+        <v>603.55</v>
       </c>
       <c r="D31" t="n">
-        <v>4.84</v>
+        <v>4.99</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>290.95</v>
+        <v>5.82</v>
       </c>
       <c r="C32" t="n">
-        <v>304.95</v>
+        <v>6.11</v>
       </c>
       <c r="D32" t="n">
-        <v>4.81</v>
+        <v>4.98</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3.13</v>
+        <v>57.47</v>
       </c>
       <c r="C33" t="n">
-        <v>3.28</v>
+        <v>60.33</v>
       </c>
       <c r="D33" t="n">
-        <v>4.79</v>
+        <v>4.98</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>BURNPUR</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3.83</v>
+        <v>17.5</v>
       </c>
       <c r="C34" t="n">
-        <v>4.01</v>
+        <v>18.37</v>
       </c>
       <c r="D34" t="n">
-        <v>4.7</v>
+        <v>4.97</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>INDIANCARD</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>214.96</v>
+        <v>125.95</v>
       </c>
       <c r="C35" t="n">
-        <v>225</v>
+        <v>132.2</v>
       </c>
       <c r="D35" t="n">
-        <v>4.67</v>
+        <v>4.96</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>POEL</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>137.47</v>
+        <v>113.56</v>
       </c>
       <c r="C36" t="n">
-        <v>143.79</v>
+        <v>119.17</v>
       </c>
       <c r="D36" t="n">
-        <v>4.6</v>
+        <v>4.94</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MLKFOOD</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>75.59</v>
+        <v>79.09</v>
       </c>
       <c r="C37" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D37" t="n">
-        <v>4.51</v>
+        <v>4.94</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>CLSL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>5.19</v>
+        <v>74.95</v>
       </c>
       <c r="C38" t="n">
-        <v>5.42</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="D38" t="n">
-        <v>4.43</v>
+        <v>4.94</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MGSL</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>66.09999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="C39" t="n">
-        <v>69</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="D39" t="n">
-        <v>4.39</v>
+        <v>4.92</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>MLKFOOD</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1.83</v>
+        <v>79.12</v>
       </c>
       <c r="C40" t="n">
-        <v>1.91</v>
+        <v>83</v>
       </c>
       <c r="D40" t="n">
-        <v>4.37</v>
+        <v>4.9</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SADBHIN</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2.55</v>
+        <v>3.28</v>
       </c>
       <c r="C41" t="n">
-        <v>2.66</v>
+        <v>3.44</v>
       </c>
       <c r="D41" t="n">
-        <v>4.31</v>
+        <v>4.88</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>TIPSFILMS</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.71</v>
+        <v>318.5</v>
       </c>
       <c r="C42" t="n">
-        <v>0.74</v>
+        <v>333.95</v>
       </c>
       <c r="D42" t="n">
-        <v>4.23</v>
+        <v>4.85</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GLASSWALL</t>
+          <t>KARAMTARA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>214.85</v>
+        <v>352</v>
       </c>
       <c r="C43" t="n">
-        <v>223.75</v>
+        <v>369</v>
       </c>
       <c r="D43" t="n">
-        <v>4.14</v>
+        <v>4.83</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SOMICONVEY</t>
+          <t>ABCOTS</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>94.11</v>
+        <v>210.83</v>
       </c>
       <c r="C44" t="n">
-        <v>98</v>
+        <v>221</v>
       </c>
       <c r="D44" t="n">
-        <v>4.13</v>
+        <v>4.82</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>KAMANWALA</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>17.24</v>
+        <v>21</v>
       </c>
       <c r="C45" t="n">
-        <v>17.95</v>
+        <v>22</v>
       </c>
       <c r="D45" t="n">
-        <v>4.12</v>
+        <v>4.76</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>16.33</v>
+        <v>4.01</v>
       </c>
       <c r="C46" t="n">
-        <v>17</v>
+        <v>4.2</v>
       </c>
       <c r="D46" t="n">
-        <v>4.1</v>
+        <v>4.74</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LAXMICOT</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>13.22</v>
+        <v>24.11</v>
       </c>
       <c r="C47" t="n">
-        <v>13.76</v>
+        <v>25.25</v>
       </c>
       <c r="D47" t="n">
-        <v>4.08</v>
+        <v>4.73</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>155.58</v>
+        <v>5.11</v>
       </c>
       <c r="C48" t="n">
-        <v>161.88</v>
+        <v>5.35</v>
       </c>
       <c r="D48" t="n">
-        <v>4.05</v>
+        <v>4.7</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HILINFRA</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>43.83</v>
+        <v>6.86</v>
       </c>
       <c r="C49" t="n">
-        <v>45.6</v>
+        <v>7.18</v>
       </c>
       <c r="D49" t="n">
-        <v>4.04</v>
+        <v>4.66</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>HBPOR</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>62.3</v>
+        <v>32.97</v>
       </c>
       <c r="C50" t="n">
-        <v>64.75</v>
+        <v>34.49</v>
       </c>
       <c r="D50" t="n">
-        <v>3.93</v>
+        <v>4.61</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5.87</v>
+        <v>1.32</v>
       </c>
       <c r="C51" t="n">
-        <v>6.1</v>
+        <v>1.38</v>
       </c>
       <c r="D51" t="n">
-        <v>3.92</v>
+        <v>4.55</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>384.95</v>
+        <v>18.41</v>
       </c>
       <c r="C52" t="n">
-        <v>399.9</v>
+        <v>19.24</v>
       </c>
       <c r="D52" t="n">
-        <v>3.88</v>
+        <v>4.51</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>SHREEDHAR</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>10.08</v>
+        <v>153.35</v>
       </c>
       <c r="C53" t="n">
-        <v>10.47</v>
+        <v>160.25</v>
       </c>
       <c r="D53" t="n">
-        <v>3.87</v>
+        <v>4.5</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>56.98</v>
+        <v>81.37</v>
       </c>
       <c r="C54" t="n">
-        <v>59.18</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="D54" t="n">
-        <v>3.86</v>
+        <v>4.34</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ISHANCH</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>47.12</v>
+        <v>0.7</v>
       </c>
       <c r="C55" t="n">
-        <v>48.9</v>
+        <v>0.73</v>
       </c>
       <c r="D55" t="n">
-        <v>3.78</v>
+        <v>4.29</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>SRGHFL</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>19.71</v>
+        <v>126.65</v>
       </c>
       <c r="C56" t="n">
-        <v>20.45</v>
+        <v>132.05</v>
       </c>
       <c r="D56" t="n">
-        <v>3.75</v>
+        <v>4.26</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>NEPHROCARE</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>20.2</v>
+        <v>91.65000000000001</v>
       </c>
       <c r="C57" t="n">
-        <v>20.95</v>
+        <v>95.55</v>
       </c>
       <c r="D57" t="n">
-        <v>3.71</v>
+        <v>4.26</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>EMMBI</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>87.75</v>
+        <v>14.62</v>
       </c>
       <c r="C58" t="n">
-        <v>90.95</v>
+        <v>15.24</v>
       </c>
       <c r="D58" t="n">
-        <v>3.65</v>
+        <v>4.24</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>7.69</v>
+        <v>21.68</v>
       </c>
       <c r="C59" t="n">
-        <v>7.97</v>
+        <v>22.6</v>
       </c>
       <c r="D59" t="n">
-        <v>3.64</v>
+        <v>4.24</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>NEUEON</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>11.09</v>
+        <v>0.48</v>
       </c>
       <c r="C60" t="n">
-        <v>11.49</v>
+        <v>0.5</v>
       </c>
       <c r="D60" t="n">
-        <v>3.61</v>
+        <v>4.17</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LATTEYS</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>20.65</v>
+        <v>446.5</v>
       </c>
       <c r="C61" t="n">
-        <v>21.39</v>
+        <v>465</v>
       </c>
       <c r="D61" t="n">
-        <v>3.58</v>
+        <v>4.14</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>ALPHAGEO</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.28</v>
+        <v>294.95</v>
       </c>
       <c r="C62" t="n">
-        <v>0.29</v>
+        <v>306.95</v>
       </c>
       <c r="D62" t="n">
-        <v>3.57</v>
+        <v>4.07</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>AAATECH</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>13.52</v>
+        <v>84.56999999999999</v>
       </c>
       <c r="C63" t="n">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="D63" t="n">
-        <v>3.55</v>
+        <v>4.06</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>GUJAPOLLO</t>
+          <t>MADHAV</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>338.1</v>
+        <v>34.5</v>
       </c>
       <c r="C64" t="n">
-        <v>349.85</v>
+        <v>35.9</v>
       </c>
       <c r="D64" t="n">
-        <v>3.48</v>
+        <v>4.06</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SONAMLTD</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>71.44</v>
+        <v>0.74</v>
       </c>
       <c r="C65" t="n">
-        <v>73.89</v>
+        <v>0.77</v>
       </c>
       <c r="D65" t="n">
-        <v>3.43</v>
+        <v>4.05</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2.34</v>
+        <v>23.44</v>
       </c>
       <c r="C66" t="n">
-        <v>2.42</v>
+        <v>24.38</v>
       </c>
       <c r="D66" t="n">
-        <v>3.42</v>
+        <v>4.01</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MAKERSL</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>177.92</v>
+        <v>34.94</v>
       </c>
       <c r="C67" t="n">
-        <v>184</v>
+        <v>36.33</v>
       </c>
       <c r="D67" t="n">
-        <v>3.42</v>
+        <v>3.98</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>18.01</v>
+        <v>631.9</v>
       </c>
       <c r="C68" t="n">
-        <v>18.6</v>
+        <v>657</v>
       </c>
       <c r="D68" t="n">
-        <v>3.28</v>
+        <v>3.97</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>GLASSWALL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>31.79</v>
+        <v>257.82</v>
       </c>
       <c r="C69" t="n">
-        <v>32.83</v>
+        <v>267.98</v>
       </c>
       <c r="D69" t="n">
-        <v>3.27</v>
+        <v>3.94</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>LAGNAM</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>994.45</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="C70" t="n">
-        <v>1026.95</v>
+        <v>73</v>
       </c>
       <c r="D70" t="n">
-        <v>3.27</v>
+        <v>3.93</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>LKPSEC</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>133.61</v>
+        <v>15.06</v>
       </c>
       <c r="C71" t="n">
-        <v>137.95</v>
+        <v>15.65</v>
       </c>
       <c r="D71" t="n">
-        <v>3.25</v>
+        <v>3.92</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>SHEMAROO</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>61.02</v>
+        <v>115.5</v>
       </c>
       <c r="C72" t="n">
-        <v>62.99</v>
+        <v>120</v>
       </c>
       <c r="D72" t="n">
-        <v>3.23</v>
+        <v>3.9</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>BATLIBOI</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>46.52</v>
+        <v>78.73</v>
       </c>
       <c r="C73" t="n">
-        <v>47.99</v>
+        <v>81.8</v>
       </c>
       <c r="D73" t="n">
-        <v>3.16</v>
+        <v>3.9</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>EMAMIREAL</t>
+          <t>NAGREEKCAP</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>66.31</v>
+        <v>27.92</v>
       </c>
       <c r="C74" t="n">
-        <v>68.40000000000001</v>
+        <v>29</v>
       </c>
       <c r="D74" t="n">
-        <v>3.15</v>
+        <v>3.87</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>23.76</v>
+        <v>56.6</v>
       </c>
       <c r="C75" t="n">
-        <v>24.5</v>
+        <v>58.79</v>
       </c>
       <c r="D75" t="n">
-        <v>3.11</v>
+        <v>3.87</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>8.720000000000001</v>
+        <v>6.97</v>
       </c>
       <c r="C76" t="n">
-        <v>8.99</v>
+        <v>7.24</v>
       </c>
       <c r="D76" t="n">
-        <v>3.1</v>
+        <v>3.87</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LAMBODHARA</t>
+          <t>GREENPOWER</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>117.76</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="C77" t="n">
-        <v>121.4</v>
+        <v>9.4</v>
       </c>
       <c r="D77" t="n">
-        <v>3.09</v>
+        <v>3.87</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>24.59</v>
+        <v>21.84</v>
       </c>
       <c r="C78" t="n">
-        <v>25.35</v>
+        <v>22.68</v>
       </c>
       <c r="D78" t="n">
-        <v>3.09</v>
+        <v>3.85</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>SHAHALLOYS</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>16.95</v>
+        <v>92.47</v>
       </c>
       <c r="C79" t="n">
-        <v>17.47</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="D79" t="n">
-        <v>3.07</v>
+        <v>3.81</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>AVPINFRA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>12.48</v>
+        <v>57.8</v>
       </c>
       <c r="C80" t="n">
-        <v>12.86</v>
+        <v>60</v>
       </c>
       <c r="D80" t="n">
-        <v>3.04</v>
+        <v>3.81</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PRANAV</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>106.81</v>
+        <v>530.45</v>
       </c>
       <c r="C81" t="n">
-        <v>110</v>
+        <v>550.45</v>
       </c>
       <c r="D81" t="n">
-        <v>2.99</v>
+        <v>3.77</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>RUBFILA</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>65.04000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="C82" t="n">
-        <v>66.95999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="D82" t="n">
-        <v>2.95</v>
+        <v>3.77</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>KOTHARIPRO</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>64.14</v>
+        <v>16.73</v>
       </c>
       <c r="C83" t="n">
-        <v>66</v>
+        <v>17.36</v>
       </c>
       <c r="D83" t="n">
-        <v>2.9</v>
+        <v>3.77</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>DEEP</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>93.34999999999999</v>
+        <v>47.23</v>
       </c>
       <c r="C84" t="n">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="D84" t="n">
-        <v>2.84</v>
+        <v>3.75</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MANAKSTEEL</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>106.42</v>
+        <v>315.2</v>
       </c>
       <c r="C85" t="n">
-        <v>109.4</v>
+        <v>327</v>
       </c>
       <c r="D85" t="n">
-        <v>2.8</v>
+        <v>3.74</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>ICELCO</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>74.62</v>
+        <v>121.5</v>
       </c>
       <c r="C86" t="n">
-        <v>76.7</v>
+        <v>125.95</v>
       </c>
       <c r="D86" t="n">
-        <v>2.79</v>
+        <v>3.66</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>96.22</v>
+        <v>7.67</v>
       </c>
       <c r="C87" t="n">
-        <v>98.90000000000001</v>
+        <v>7.95</v>
       </c>
       <c r="D87" t="n">
-        <v>2.79</v>
+        <v>3.65</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>GAUDIUMIVF</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.36</v>
+        <v>114.79</v>
       </c>
       <c r="C88" t="n">
-        <v>0.37</v>
+        <v>118.96</v>
       </c>
       <c r="D88" t="n">
-        <v>2.78</v>
+        <v>3.63</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>65.17</v>
+        <v>122.75</v>
       </c>
       <c r="C89" t="n">
-        <v>66.94</v>
+        <v>127.15</v>
       </c>
       <c r="D89" t="n">
-        <v>2.72</v>
+        <v>3.58</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ALPINETEX</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>52.33</v>
+        <v>3.35</v>
       </c>
       <c r="C90" t="n">
-        <v>53.75</v>
+        <v>3.47</v>
       </c>
       <c r="D90" t="n">
-        <v>2.71</v>
+        <v>3.58</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>37</v>
+        <v>34.71</v>
       </c>
       <c r="C91" t="n">
-        <v>38</v>
+        <v>35.95</v>
       </c>
       <c r="D91" t="n">
-        <v>2.7</v>
+        <v>3.57</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>WEWIN</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>41.87</v>
+        <v>2.8</v>
       </c>
       <c r="C92" t="n">
-        <v>43</v>
+        <v>2.9</v>
       </c>
       <c r="D92" t="n">
-        <v>2.7</v>
+        <v>3.57</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>JINDWORLD</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>49.16</v>
+        <v>7.05</v>
       </c>
       <c r="C93" t="n">
-        <v>50.48</v>
+        <v>7.3</v>
       </c>
       <c r="D93" t="n">
-        <v>2.69</v>
+        <v>3.55</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>HTMEDIA</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>22.99</v>
+        <v>19.28</v>
       </c>
       <c r="C94" t="n">
-        <v>23.6</v>
+        <v>19.95</v>
       </c>
       <c r="D94" t="n">
-        <v>2.65</v>
+        <v>3.48</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>S&amp;SPOWER</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>321.35</v>
+        <v>33.31</v>
       </c>
       <c r="C95" t="n">
-        <v>329.8</v>
+        <v>34.45</v>
       </c>
       <c r="D95" t="n">
-        <v>2.63</v>
+        <v>3.42</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BPLPHARMA</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>1509.8</v>
+        <v>4.11</v>
       </c>
       <c r="C96" t="n">
-        <v>1549.2</v>
+        <v>4.25</v>
       </c>
       <c r="D96" t="n">
-        <v>2.61</v>
+        <v>3.41</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>13.06</v>
+        <v>441.95</v>
       </c>
       <c r="C97" t="n">
-        <v>13.4</v>
+        <v>457</v>
       </c>
       <c r="D97" t="n">
-        <v>2.6</v>
+        <v>3.41</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>MOHITIND</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>17.52</v>
+        <v>23.2</v>
       </c>
       <c r="C98" t="n">
-        <v>17.97</v>
+        <v>23.99</v>
       </c>
       <c r="D98" t="n">
-        <v>2.57</v>
+        <v>3.41</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TURTLEMINT</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>127.74</v>
+        <v>25.15</v>
       </c>
       <c r="C99" t="n">
-        <v>131</v>
+        <v>26</v>
       </c>
       <c r="D99" t="n">
-        <v>2.55</v>
+        <v>3.38</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>AAREYDRUGS</t>
+          <t>IRMENERGY</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>99.94</v>
+        <v>269.1</v>
       </c>
       <c r="C100" t="n">
-        <v>102.49</v>
+        <v>278.15</v>
       </c>
       <c r="D100" t="n">
-        <v>2.55</v>
+        <v>3.36</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>AONESILVER</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>51.98</v>
+        <v>8.66</v>
       </c>
       <c r="C101" t="n">
-        <v>53.3</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="D101" t="n">
-        <v>2.54</v>
+        <v>3.35</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>26.52</v>
+        <v>1008.6</v>
       </c>
       <c r="C102" t="n">
-        <v>27.18</v>
+        <v>1042.4</v>
       </c>
       <c r="D102" t="n">
-        <v>2.49</v>
+        <v>3.35</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IVC</t>
+          <t>VIRAT</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>7.76</v>
+        <v>382.25</v>
       </c>
       <c r="C103" t="n">
-        <v>7.95</v>
+        <v>394.9</v>
       </c>
       <c r="D103" t="n">
-        <v>2.45</v>
+        <v>3.31</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ARENTERP</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>32.6</v>
+        <v>7.25</v>
       </c>
       <c r="C104" t="n">
-        <v>33.4</v>
+        <v>7.49</v>
       </c>
       <c r="D104" t="n">
-        <v>2.45</v>
+        <v>3.31</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>URJA</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>39.39</v>
+        <v>9.1</v>
       </c>
       <c r="C105" t="n">
-        <v>40.35</v>
+        <v>9.4</v>
       </c>
       <c r="D105" t="n">
-        <v>2.44</v>
+        <v>3.3</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>DHATRE</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>4.11</v>
+        <v>401.65</v>
       </c>
       <c r="C106" t="n">
-        <v>4.21</v>
+        <v>414.85</v>
       </c>
       <c r="D106" t="n">
-        <v>2.43</v>
+        <v>3.29</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>DREAMFOLKS</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>65.33</v>
+        <v>6.1</v>
       </c>
       <c r="C107" t="n">
-        <v>66.90000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="D107" t="n">
-        <v>2.4</v>
+        <v>3.28</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>KARMAENG</t>
+          <t>ARENTERP</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>38.72</v>
+        <v>34.2</v>
       </c>
       <c r="C108" t="n">
-        <v>39.65</v>
+        <v>35.3</v>
       </c>
       <c r="D108" t="n">
-        <v>2.4</v>
+        <v>3.22</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>NAHARCAP</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1902.6</v>
+        <v>250</v>
       </c>
       <c r="C109" t="n">
-        <v>1948</v>
+        <v>257.95</v>
       </c>
       <c r="D109" t="n">
-        <v>2.39</v>
+        <v>3.18</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SILVER001</t>
+          <t>WOMANCART</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>23.12</v>
+        <v>101</v>
       </c>
       <c r="C110" t="n">
-        <v>23.67</v>
+        <v>104.2</v>
       </c>
       <c r="D110" t="n">
-        <v>2.38</v>
+        <v>3.17</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ISFT</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>75.22</v>
+        <v>5.99</v>
       </c>
       <c r="C111" t="n">
-        <v>77</v>
+        <v>6.18</v>
       </c>
       <c r="D111" t="n">
-        <v>2.37</v>
+        <v>3.17</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>ORISSAMINE</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>250.95</v>
+        <v>3896.4</v>
       </c>
       <c r="C112" t="n">
-        <v>256.85</v>
+        <v>4020</v>
       </c>
       <c r="D112" t="n">
-        <v>2.35</v>
+        <v>3.17</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>RAMAPHO</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>115.18</v>
+        <v>63</v>
       </c>
       <c r="C113" t="n">
-        <v>117.89</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="D113" t="n">
-        <v>2.35</v>
+        <v>3.16</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>SOMICONVEY</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>3.41</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="C114" t="n">
-        <v>3.49</v>
+        <v>97.59</v>
       </c>
       <c r="D114" t="n">
-        <v>2.35</v>
+        <v>3.16</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>RPPINFRA</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>53.56</v>
+        <v>42.46</v>
       </c>
       <c r="C115" t="n">
-        <v>54.8</v>
+        <v>43.8</v>
       </c>
       <c r="D115" t="n">
-        <v>2.32</v>
+        <v>3.16</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MALUPAPER</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>31.66</v>
+        <v>16.19</v>
       </c>
       <c r="C116" t="n">
-        <v>32.39</v>
+        <v>16.7</v>
       </c>
       <c r="D116" t="n">
-        <v>2.31</v>
+        <v>3.15</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>KANOHAR</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>751.5</v>
+        <v>243.45</v>
       </c>
       <c r="C117" t="n">
-        <v>768.7</v>
+        <v>251</v>
       </c>
       <c r="D117" t="n">
-        <v>2.29</v>
+        <v>3.1</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>KELLTONTEC</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>107.54</v>
+        <v>13.57</v>
       </c>
       <c r="C118" t="n">
-        <v>110</v>
+        <v>13.99</v>
       </c>
       <c r="D118" t="n">
-        <v>2.29</v>
+        <v>3.1</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MAHEPC</t>
+          <t>GUJAPOLLO</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>101.18</v>
+        <v>324</v>
       </c>
       <c r="C119" t="n">
-        <v>103.49</v>
+        <v>333.95</v>
       </c>
       <c r="D119" t="n">
-        <v>2.28</v>
+        <v>3.07</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>162.29</v>
+        <v>22.27</v>
       </c>
       <c r="C120" t="n">
-        <v>165.99</v>
+        <v>22.94</v>
       </c>
       <c r="D120" t="n">
-        <v>2.28</v>
+        <v>3.01</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>24.69</v>
+        <v>827.45</v>
       </c>
       <c r="C121" t="n">
-        <v>25.25</v>
+        <v>852</v>
       </c>
       <c r="D121" t="n">
-        <v>2.27</v>
+        <v>2.97</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>220.37</v>
+        <v>1392.8</v>
       </c>
       <c r="C122" t="n">
-        <v>225.37</v>
+        <v>1434</v>
       </c>
       <c r="D122" t="n">
-        <v>2.27</v>
+        <v>2.96</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1515.8</v>
+        <v>1.37</v>
       </c>
       <c r="C123" t="n">
-        <v>1550</v>
+        <v>1.41</v>
       </c>
       <c r="D123" t="n">
-        <v>2.26</v>
+        <v>2.92</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>CPL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>1.33</v>
+        <v>65.39</v>
       </c>
       <c r="C124" t="n">
-        <v>1.36</v>
+        <v>67.3</v>
       </c>
       <c r="D124" t="n">
-        <v>2.26</v>
+        <v>2.92</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SALONA</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>264</v>
+        <v>8.59</v>
       </c>
       <c r="C125" t="n">
-        <v>269.95</v>
+        <v>8.84</v>
       </c>
       <c r="D125" t="n">
-        <v>2.25</v>
+        <v>2.91</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>MALLCOM</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>924.3</v>
+        <v>25.78</v>
       </c>
       <c r="C126" t="n">
-        <v>945</v>
+        <v>26.52</v>
       </c>
       <c r="D126" t="n">
-        <v>2.24</v>
+        <v>2.87</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>11.2</v>
+        <v>220.25</v>
       </c>
       <c r="C127" t="n">
-        <v>11.45</v>
+        <v>226.5</v>
       </c>
       <c r="D127" t="n">
-        <v>2.23</v>
+        <v>2.84</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>VALIANTORG</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>5.86</v>
+        <v>408.45</v>
       </c>
       <c r="C128" t="n">
-        <v>5.99</v>
+        <v>420</v>
       </c>
       <c r="D128" t="n">
-        <v>2.22</v>
+        <v>2.83</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>VILAS</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>428.4</v>
+        <v>331.6</v>
       </c>
       <c r="C129" t="n">
-        <v>437.85</v>
+        <v>341</v>
       </c>
       <c r="D129" t="n">
-        <v>2.21</v>
+        <v>2.83</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>LANCORHOL</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>46.73</v>
+        <v>35.2</v>
       </c>
       <c r="C130" t="n">
-        <v>47.75</v>
+        <v>36.19</v>
       </c>
       <c r="D130" t="n">
-        <v>2.18</v>
+        <v>2.81</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>JUNIPER</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>214.32</v>
+        <v>48.66</v>
       </c>
       <c r="C131" t="n">
-        <v>219</v>
+        <v>50</v>
       </c>
       <c r="D131" t="n">
-        <v>2.18</v>
+        <v>2.75</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>GANGESSECU</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>115.01</v>
+        <v>5.83</v>
       </c>
       <c r="C132" t="n">
-        <v>117.49</v>
+        <v>5.99</v>
       </c>
       <c r="D132" t="n">
-        <v>2.16</v>
+        <v>2.74</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>RHL</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>2.79</v>
+        <v>173.74</v>
       </c>
       <c r="C133" t="n">
-        <v>2.85</v>
+        <v>178.5</v>
       </c>
       <c r="D133" t="n">
-        <v>2.15</v>
+        <v>2.74</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>AKSHOPTFBR</t>
+          <t>RIR</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>7.96</v>
+        <v>197.63</v>
       </c>
       <c r="C134" t="n">
-        <v>8.130000000000001</v>
+        <v>203</v>
       </c>
       <c r="D134" t="n">
-        <v>2.14</v>
+        <v>2.72</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MVKAGRO</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>270.65</v>
+        <v>13.04</v>
       </c>
       <c r="C135" t="n">
-        <v>276.4</v>
+        <v>13.39</v>
       </c>
       <c r="D135" t="n">
-        <v>2.12</v>
+        <v>2.68</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>RUDRA</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>68.06999999999999</v>
+        <v>20.36</v>
       </c>
       <c r="C136" t="n">
-        <v>69.48999999999999</v>
+        <v>20.9</v>
       </c>
       <c r="D136" t="n">
-        <v>2.09</v>
+        <v>2.65</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>30.56</v>
+        <v>30.2</v>
       </c>
       <c r="C137" t="n">
-        <v>31.2</v>
+        <v>31</v>
       </c>
       <c r="D137" t="n">
-        <v>2.09</v>
+        <v>2.65</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>SUPERHOUSE</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>7.74</v>
+        <v>167.58</v>
       </c>
       <c r="C138" t="n">
-        <v>7.9</v>
+        <v>171.95</v>
       </c>
       <c r="D138" t="n">
-        <v>2.07</v>
+        <v>2.61</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ADVIKCA</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.97</v>
+        <v>35.97</v>
       </c>
       <c r="C139" t="n">
-        <v>0.99</v>
+        <v>36.9</v>
       </c>
       <c r="D139" t="n">
-        <v>2.06</v>
+        <v>2.59</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>2.44</v>
+        <v>10.02</v>
       </c>
       <c r="C140" t="n">
-        <v>2.49</v>
+        <v>10.28</v>
       </c>
       <c r="D140" t="n">
-        <v>2.05</v>
+        <v>2.59</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>XELPMOC</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.98</v>
+        <v>74.08</v>
       </c>
       <c r="C141" t="n">
-        <v>1</v>
+        <v>75.98999999999999</v>
       </c>
       <c r="D141" t="n">
-        <v>2.04</v>
+        <v>2.58</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>APOLSINHOT</t>
+          <t>PAISALO</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>1185.8</v>
+        <v>88.73</v>
       </c>
       <c r="C142" t="n">
-        <v>1210</v>
+        <v>91</v>
       </c>
       <c r="D142" t="n">
-        <v>2.04</v>
+        <v>2.56</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>RAMASTEEL</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>3.92</v>
+        <v>7.07</v>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>7.25</v>
       </c>
       <c r="D143" t="n">
-        <v>2.04</v>
+        <v>2.55</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>AASTHA</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>74.33</v>
+        <v>1456</v>
       </c>
       <c r="C144" t="n">
-        <v>75.84999999999999</v>
+        <v>1493</v>
       </c>
       <c r="D144" t="n">
-        <v>2.04</v>
+        <v>2.54</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>8.369999999999999</v>
+        <v>5.14</v>
       </c>
       <c r="C145" t="n">
-        <v>8.539999999999999</v>
+        <v>5.27</v>
       </c>
       <c r="D145" t="n">
-        <v>2.03</v>
+        <v>2.53</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>NOIDATOLL</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>3.96</v>
+        <v>5.13</v>
       </c>
       <c r="C146" t="n">
-        <v>4.04</v>
+        <v>5.26</v>
       </c>
       <c r="D146" t="n">
-        <v>2.02</v>
+        <v>2.53</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>25.68</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="C147" t="n">
-        <v>26.2</v>
+        <v>9</v>
       </c>
       <c r="D147" t="n">
-        <v>2.02</v>
+        <v>2.51</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>NECLIFE</t>
+          <t>AEROFLEX</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>10.9</v>
+        <v>497.6</v>
       </c>
       <c r="C148" t="n">
-        <v>11.12</v>
+        <v>510</v>
       </c>
       <c r="D148" t="n">
-        <v>2.02</v>
+        <v>2.49</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>74.20999999999999</v>
+        <v>6.05</v>
       </c>
       <c r="C149" t="n">
-        <v>75.70999999999999</v>
+        <v>6.2</v>
       </c>
       <c r="D149" t="n">
-        <v>2.02</v>
+        <v>2.48</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>INDOWIND</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>21.42</v>
+        <v>8.93</v>
       </c>
       <c r="C150" t="n">
-        <v>21.85</v>
+        <v>9.15</v>
       </c>
       <c r="D150" t="n">
-        <v>2.01</v>
+        <v>2.46</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CRSL</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>2.49</v>
+        <v>0.41</v>
       </c>
       <c r="C151" t="n">
-        <v>2.54</v>
+        <v>0.42</v>
       </c>
       <c r="D151" t="n">
-        <v>2.01</v>
+        <v>2.44</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>SHIVASHRIT</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>14.5</v>
+        <v>115.2</v>
       </c>
       <c r="C152" t="n">
-        <v>14.79</v>
+        <v>118</v>
       </c>
       <c r="D152" t="n">
-        <v>2</v>
+        <v>2.43</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>103.49</v>
+        <v>37.05</v>
       </c>
       <c r="C153" t="n">
-        <v>105.55</v>
+        <v>37.95</v>
       </c>
       <c r="D153" t="n">
-        <v>1.99</v>
+        <v>2.43</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>AUSTENG</t>
+          <t>YATHARTH</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>126.95</v>
+        <v>1072.4</v>
       </c>
       <c r="C154" t="n">
-        <v>129.48</v>
+        <v>1098</v>
       </c>
       <c r="D154" t="n">
-        <v>1.99</v>
+        <v>2.39</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>VTMLTD</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>48.83</v>
+        <v>72.05</v>
       </c>
       <c r="C155" t="n">
-        <v>49.8</v>
+        <v>73.75</v>
       </c>
       <c r="D155" t="n">
-        <v>1.99</v>
+        <v>2.36</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>CMSINFO</t>
+          <t>SILVERCASE</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>232.39</v>
+        <v>22.95</v>
       </c>
       <c r="C156" t="n">
-        <v>237</v>
+        <v>23.48</v>
       </c>
       <c r="D156" t="n">
-        <v>1.98</v>
+        <v>2.31</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>GENUSPAPER</t>
+          <t>GOACARBON</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>11.11</v>
+        <v>378.3</v>
       </c>
       <c r="C157" t="n">
-        <v>11.33</v>
+        <v>387</v>
       </c>
       <c r="D157" t="n">
-        <v>1.98</v>
+        <v>2.3</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>19.3</v>
+        <v>4.35</v>
       </c>
       <c r="C158" t="n">
-        <v>19.68</v>
+        <v>4.45</v>
       </c>
       <c r="D158" t="n">
-        <v>1.97</v>
+        <v>2.3</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>NECCLTD</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>7.11</v>
+        <v>18.82</v>
       </c>
       <c r="C159" t="n">
-        <v>7.25</v>
+        <v>19.25</v>
       </c>
       <c r="D159" t="n">
-        <v>1.97</v>
+        <v>2.28</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MEIL</t>
+          <t>RAMBHAJO</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>268.6</v>
+        <v>266.17</v>
       </c>
       <c r="C160" t="n">
-        <v>273.9</v>
+        <v>272.18</v>
       </c>
       <c r="D160" t="n">
-        <v>1.97</v>
+        <v>2.26</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>MUFTI</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>8.68</v>
+        <v>73.37</v>
       </c>
       <c r="C161" t="n">
-        <v>8.85</v>
+        <v>75.02</v>
       </c>
       <c r="D161" t="n">
-        <v>1.96</v>
+        <v>2.25</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>MINDTECK</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>5121.2</v>
+        <v>156.84</v>
       </c>
       <c r="C162" t="n">
-        <v>5220</v>
+        <v>160.36</v>
       </c>
       <c r="D162" t="n">
-        <v>1.93</v>
+        <v>2.24</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>TATSILV</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>45.6</v>
+        <v>21.99</v>
       </c>
       <c r="C163" t="n">
-        <v>46.48</v>
+        <v>22.48</v>
       </c>
       <c r="D163" t="n">
-        <v>1.93</v>
+        <v>2.23</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>BBNPPGOLD</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>547.5</v>
+        <v>145.45</v>
       </c>
       <c r="C164" t="n">
-        <v>558</v>
+        <v>148.7</v>
       </c>
       <c r="D164" t="n">
-        <v>1.92</v>
+        <v>2.23</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HRYNSHP</t>
+          <t>HDFCSILVER</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>100</v>
+        <v>216.47</v>
       </c>
       <c r="C165" t="n">
-        <v>101.9</v>
+        <v>221.28</v>
       </c>
       <c r="D165" t="n">
-        <v>1.9</v>
+        <v>2.22</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>21STCENMGM</t>
+          <t>SILVERIETF</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>38.37</v>
+        <v>226.19</v>
       </c>
       <c r="C166" t="n">
-        <v>39.1</v>
+        <v>231.22</v>
       </c>
       <c r="D166" t="n">
-        <v>1.9</v>
+        <v>2.22</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>MERCURYEV</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>164.29</v>
+        <v>40.84</v>
       </c>
       <c r="C167" t="n">
-        <v>167.4</v>
+        <v>41.74</v>
       </c>
       <c r="D167" t="n">
-        <v>1.89</v>
+        <v>2.2</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>42.55</v>
+        <v>305.05</v>
       </c>
       <c r="C168" t="n">
-        <v>43.35</v>
+        <v>311.75</v>
       </c>
       <c r="D168" t="n">
-        <v>1.88</v>
+        <v>2.2</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>HALDYNGL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>12.84</v>
+        <v>140.41</v>
       </c>
       <c r="C169" t="n">
-        <v>13.08</v>
+        <v>143.5</v>
       </c>
       <c r="D169" t="n">
-        <v>1.87</v>
+        <v>2.2</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MUNJALSHOW</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>124.67</v>
+        <v>6</v>
       </c>
       <c r="C170" t="n">
-        <v>127</v>
+        <v>6.13</v>
       </c>
       <c r="D170" t="n">
-        <v>1.87</v>
+        <v>2.17</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>SILVER</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>14.48</v>
+        <v>226.36</v>
       </c>
       <c r="C171" t="n">
-        <v>14.75</v>
+        <v>231.24</v>
       </c>
       <c r="D171" t="n">
-        <v>1.86</v>
+        <v>2.16</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>DCM</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>5.38</v>
+        <v>76.36</v>
       </c>
       <c r="C172" t="n">
-        <v>5.48</v>
+        <v>78</v>
       </c>
       <c r="D172" t="n">
-        <v>1.86</v>
+        <v>2.15</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MVGJL</t>
+          <t>SHINDL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>207.16</v>
+        <v>161.05</v>
       </c>
       <c r="C173" t="n">
-        <v>211</v>
+        <v>164.5</v>
       </c>
       <c r="D173" t="n">
-        <v>1.85</v>
+        <v>2.14</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>SBISILVER</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>41.29</v>
+        <v>222.1</v>
       </c>
       <c r="C174" t="n">
-        <v>42.05</v>
+        <v>226.86</v>
       </c>
       <c r="D174" t="n">
-        <v>1.84</v>
+        <v>2.14</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>TEJA</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>207.2</v>
+        <v>46.8</v>
       </c>
       <c r="C175" t="n">
-        <v>211</v>
+        <v>47.8</v>
       </c>
       <c r="D175" t="n">
-        <v>1.83</v>
+        <v>2.14</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>1995.5</v>
+        <v>209.45</v>
       </c>
       <c r="C176" t="n">
-        <v>2032</v>
+        <v>213.9</v>
       </c>
       <c r="D176" t="n">
-        <v>1.83</v>
+        <v>2.12</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>204.77</v>
+        <v>78.34999999999999</v>
       </c>
       <c r="C177" t="n">
-        <v>208.49</v>
+        <v>80.01000000000001</v>
       </c>
       <c r="D177" t="n">
-        <v>1.82</v>
+        <v>2.12</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>AVALON</t>
+          <t>SILVERAXIS</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>2216.1</v>
+        <v>225.27</v>
       </c>
       <c r="C178" t="n">
-        <v>2256</v>
+        <v>230.05</v>
       </c>
       <c r="D178" t="n">
-        <v>1.8</v>
+        <v>2.12</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>VINYLINDIA</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>1.67</v>
+        <v>214.17</v>
       </c>
       <c r="C179" t="n">
-        <v>1.7</v>
+        <v>218.7</v>
       </c>
       <c r="D179" t="n">
-        <v>1.8</v>
+        <v>2.12</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MANOMAY</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>223.85</v>
+        <v>159.63</v>
       </c>
       <c r="C180" t="n">
-        <v>227.89</v>
+        <v>163.01</v>
       </c>
       <c r="D180" t="n">
-        <v>1.8</v>
+        <v>2.12</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>LUMINO</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>712.05</v>
+        <v>107.14</v>
       </c>
       <c r="C181" t="n">
-        <v>724.8</v>
+        <v>109.4</v>
       </c>
       <c r="D181" t="n">
-        <v>1.79</v>
+        <v>2.11</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>6846.5</v>
+        <v>1.91</v>
       </c>
       <c r="C182" t="n">
-        <v>6968</v>
+        <v>1.95</v>
       </c>
       <c r="D182" t="n">
-        <v>1.77</v>
+        <v>2.09</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>87.59999999999999</v>
+        <v>12</v>
       </c>
       <c r="C183" t="n">
-        <v>89.15000000000001</v>
+        <v>12.25</v>
       </c>
       <c r="D183" t="n">
-        <v>1.77</v>
+        <v>2.08</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>CHEMCON</t>
+          <t>AIMTRON</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>212.1</v>
+        <v>1616.45</v>
       </c>
       <c r="C184" t="n">
-        <v>215.8</v>
+        <v>1650</v>
       </c>
       <c r="D184" t="n">
-        <v>1.74</v>
+        <v>2.08</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SWANDEF</t>
+          <t>SILVERBEES</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>2687.2</v>
+        <v>216.64</v>
       </c>
       <c r="C185" t="n">
-        <v>2734</v>
+        <v>221.1</v>
       </c>
       <c r="D185" t="n">
-        <v>1.74</v>
+        <v>2.06</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>16.15</v>
+        <v>0.97</v>
       </c>
       <c r="C186" t="n">
-        <v>16.43</v>
+        <v>0.99</v>
       </c>
       <c r="D186" t="n">
-        <v>1.73</v>
+        <v>2.06</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>HINDADH</t>
+          <t>SAHYADRI</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>378.45</v>
+        <v>359.25</v>
       </c>
       <c r="C187" t="n">
-        <v>384.95</v>
+        <v>366.6</v>
       </c>
       <c r="D187" t="n">
-        <v>1.72</v>
+        <v>2.05</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>GVKPIL</t>
+          <t>VICTORYEV</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>2.33</v>
+        <v>14.6</v>
       </c>
       <c r="C188" t="n">
-        <v>2.37</v>
+        <v>14.9</v>
       </c>
       <c r="D188" t="n">
-        <v>1.72</v>
+        <v>2.05</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>VILAS</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>316.25</v>
+        <v>5.87</v>
       </c>
       <c r="C189" t="n">
-        <v>321.7</v>
+        <v>5.99</v>
       </c>
       <c r="D189" t="n">
-        <v>1.72</v>
+        <v>2.04</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>BSL</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>117.97</v>
+        <v>24.64</v>
       </c>
       <c r="C190" t="n">
-        <v>119.99</v>
+        <v>25.14</v>
       </c>
       <c r="D190" t="n">
-        <v>1.71</v>
+        <v>2.03</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>ALPA</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>1.17</v>
+        <v>59.64</v>
       </c>
       <c r="C191" t="n">
-        <v>1.19</v>
+        <v>60.85</v>
       </c>
       <c r="D191" t="n">
-        <v>1.71</v>
+        <v>2.03</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>7.07</v>
+        <v>37.07</v>
       </c>
       <c r="C192" t="n">
-        <v>7.19</v>
+        <v>37.82</v>
       </c>
       <c r="D192" t="n">
-        <v>1.7</v>
+        <v>2.02</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>1.78</v>
+        <v>5.44</v>
       </c>
       <c r="C193" t="n">
-        <v>1.81</v>
+        <v>5.55</v>
       </c>
       <c r="D193" t="n">
-        <v>1.69</v>
+        <v>2.02</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>AWL</t>
+          <t>CRSL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>181.94</v>
+        <v>2.47</v>
       </c>
       <c r="C194" t="n">
-        <v>185</v>
+        <v>2.52</v>
       </c>
       <c r="D194" t="n">
-        <v>1.68</v>
+        <v>2.02</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>4.21</v>
+        <v>57.05</v>
       </c>
       <c r="C195" t="n">
-        <v>4.28</v>
+        <v>58.2</v>
       </c>
       <c r="D195" t="n">
-        <v>1.66</v>
+        <v>2.02</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>4.23</v>
+        <v>35.46</v>
       </c>
       <c r="C196" t="n">
-        <v>4.3</v>
+        <v>36.17</v>
       </c>
       <c r="D196" t="n">
-        <v>1.65</v>
+        <v>2</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>GTPL</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>56.46</v>
+        <v>359.6</v>
       </c>
       <c r="C197" t="n">
-        <v>57.39</v>
+        <v>366.8</v>
       </c>
       <c r="D197" t="n">
-        <v>1.65</v>
+        <v>2</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>ADVAIT</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>42.7</v>
+        <v>1990.4</v>
       </c>
       <c r="C198" t="n">
-        <v>43.4</v>
+        <v>2030</v>
       </c>
       <c r="D198" t="n">
-        <v>1.64</v>
+        <v>1.99</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>1.84</v>
+        <v>15.55</v>
       </c>
       <c r="C199" t="n">
-        <v>1.87</v>
+        <v>15.86</v>
       </c>
       <c r="D199" t="n">
-        <v>1.63</v>
+        <v>1.99</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>GRAPHITE</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>805.05</v>
+        <v>26.66</v>
       </c>
       <c r="C200" t="n">
-        <v>818</v>
+        <v>27.19</v>
       </c>
       <c r="D200" t="n">
-        <v>1.61</v>
+        <v>1.99</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>MEDICO</t>
+          <t>ANSALAPI</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>35.33</v>
+        <v>3.52</v>
       </c>
       <c r="C201" t="n">
-        <v>35.9</v>
+        <v>3.59</v>
       </c>
       <c r="D201" t="n">
-        <v>1.61</v>
+        <v>1.99</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-21 09:18 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASTAR</t>
+          <t>TOUCHWOOD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>672.8</v>
+        <v>60.93</v>
       </c>
       <c r="C2" t="n">
-        <v>807.3</v>
+        <v>68.95</v>
       </c>
       <c r="D2" t="n">
-        <v>19.99</v>
+        <v>13.16</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ISFT</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>90.26000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="C3" t="n">
-        <v>98.97</v>
+        <v>6.05</v>
       </c>
       <c r="D3" t="n">
-        <v>9.65</v>
+        <v>10</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>RRECL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8.26</v>
+        <v>138.89</v>
       </c>
       <c r="C4" t="n">
-        <v>8.99</v>
+        <v>152</v>
       </c>
       <c r="D4" t="n">
-        <v>8.84</v>
+        <v>9.44</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ENCOMPAS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.13</v>
+        <v>238.85</v>
       </c>
       <c r="C5" t="n">
-        <v>0.14</v>
+        <v>259.5</v>
       </c>
       <c r="D5" t="n">
-        <v>7.69</v>
+        <v>8.65</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>MPEL-RE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31.97</v>
+        <v>1.8</v>
       </c>
       <c r="C6" t="n">
-        <v>34.4</v>
+        <v>1.95</v>
       </c>
       <c r="D6" t="n">
-        <v>7.6</v>
+        <v>8.33</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SKYWAYS</t>
+          <t>ALKALI</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>117.98</v>
+        <v>87.66</v>
       </c>
       <c r="C7" t="n">
-        <v>126.9</v>
+        <v>94.95</v>
       </c>
       <c r="D7" t="n">
-        <v>7.56</v>
+        <v>8.32</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>SHAILY</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8.369999999999999</v>
+        <v>3149.8</v>
       </c>
       <c r="C8" t="n">
-        <v>8.960000000000001</v>
+        <v>3396.9</v>
       </c>
       <c r="D8" t="n">
-        <v>7.05</v>
+        <v>7.84</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DHATRE</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.12</v>
+        <v>0.14</v>
       </c>
       <c r="C9" t="n">
-        <v>4.4</v>
+        <v>0.15</v>
       </c>
       <c r="D9" t="n">
-        <v>6.8</v>
+        <v>7.14</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RENTOMOJO</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>534.25</v>
+        <v>97.84999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>570</v>
+        <v>104.7</v>
       </c>
       <c r="D10" t="n">
-        <v>6.69</v>
+        <v>7</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.85</v>
+        <v>236.6</v>
       </c>
       <c r="C11" t="n">
-        <v>7.3</v>
+        <v>253</v>
       </c>
       <c r="D11" t="n">
-        <v>6.57</v>
+        <v>6.93</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OSWALAGRO</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>33.91</v>
+        <v>15.92</v>
       </c>
       <c r="C12" t="n">
-        <v>35.99</v>
+        <v>17</v>
       </c>
       <c r="D12" t="n">
-        <v>6.13</v>
+        <v>6.78</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>ORIANA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>63.66</v>
+        <v>271.75</v>
       </c>
       <c r="C13" t="n">
-        <v>67.52</v>
+        <v>290</v>
       </c>
       <c r="D13" t="n">
-        <v>6.06</v>
+        <v>6.72</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.84</v>
+        <v>19.42</v>
       </c>
       <c r="C14" t="n">
-        <v>1.95</v>
+        <v>20.7</v>
       </c>
       <c r="D14" t="n">
-        <v>5.98</v>
+        <v>6.59</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>PRECOT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.31</v>
+        <v>659.65</v>
       </c>
       <c r="C15" t="n">
-        <v>2.44</v>
+        <v>700</v>
       </c>
       <c r="D15" t="n">
-        <v>5.63</v>
+        <v>6.12</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.18</v>
+        <v>14.13</v>
       </c>
       <c r="C16" t="n">
-        <v>0.19</v>
+        <v>14.98</v>
       </c>
       <c r="D16" t="n">
-        <v>5.56</v>
+        <v>6.02</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>56.56</v>
+        <v>0.17</v>
       </c>
       <c r="C17" t="n">
-        <v>59.6</v>
+        <v>0.18</v>
       </c>
       <c r="D17" t="n">
-        <v>5.37</v>
+        <v>5.88</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>THACKER</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>81.63</v>
+        <v>1030</v>
       </c>
       <c r="C18" t="n">
-        <v>86</v>
+        <v>1090</v>
       </c>
       <c r="D18" t="n">
-        <v>5.35</v>
+        <v>5.83</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CREATIVEYE</t>
+          <t>SVGLOBAL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5.59</v>
+        <v>147.92</v>
       </c>
       <c r="C19" t="n">
-        <v>5.88</v>
+        <v>156.5</v>
       </c>
       <c r="D19" t="n">
-        <v>5.19</v>
+        <v>5.8</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5.29</v>
+        <v>521.15</v>
       </c>
       <c r="C20" t="n">
-        <v>5.56</v>
+        <v>551</v>
       </c>
       <c r="D20" t="n">
-        <v>5.1</v>
+        <v>5.73</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KRITI</t>
+          <t>LAXMICOT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>59.95</v>
+        <v>12.72</v>
       </c>
       <c r="C21" t="n">
-        <v>62.99</v>
+        <v>13.44</v>
       </c>
       <c r="D21" t="n">
-        <v>5.07</v>
+        <v>5.66</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>102.5</v>
+        <v>0.18</v>
       </c>
       <c r="C22" t="n">
-        <v>107.62</v>
+        <v>0.19</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>5.56</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>382.47</v>
+        <v>37.2</v>
       </c>
       <c r="C23" t="n">
-        <v>401.59</v>
+        <v>39.2</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>5.38</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>145.01</v>
+        <v>1.86</v>
       </c>
       <c r="C24" t="n">
-        <v>152.26</v>
+        <v>1.96</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>5.38</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KRITINUT</t>
+          <t>SHIVALIK</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>80.45</v>
+        <v>372.1</v>
       </c>
       <c r="C25" t="n">
-        <v>84.47</v>
+        <v>392</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>5.35</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>DHATRE</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>51.9</v>
+        <v>4.18</v>
       </c>
       <c r="C26" t="n">
-        <v>54.49</v>
+        <v>4.4</v>
       </c>
       <c r="D26" t="n">
-        <v>4.99</v>
+        <v>5.26</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>500.7</v>
+        <v>18.09</v>
       </c>
       <c r="C27" t="n">
-        <v>525.7</v>
+        <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>4.99</v>
+        <v>5.03</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>318.85</v>
+        <v>336.1</v>
       </c>
       <c r="C28" t="n">
-        <v>334.75</v>
+        <v>352.9</v>
       </c>
       <c r="D28" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>24.23</v>
+        <v>401.59</v>
       </c>
       <c r="C29" t="n">
-        <v>25.44</v>
+        <v>421.66</v>
       </c>
       <c r="D29" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>STALLION</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>40.91</v>
+        <v>220.49</v>
       </c>
       <c r="C30" t="n">
-        <v>42.95</v>
+        <v>231.51</v>
       </c>
       <c r="D30" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SHREEDHAR</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>574.85</v>
+        <v>161</v>
       </c>
       <c r="C31" t="n">
-        <v>603.55</v>
+        <v>169.05</v>
       </c>
       <c r="D31" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>CTE</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>5.82</v>
+        <v>40.7</v>
       </c>
       <c r="C32" t="n">
-        <v>6.11</v>
+        <v>42.73</v>
       </c>
       <c r="D32" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>57.47</v>
+        <v>25.44</v>
       </c>
       <c r="C33" t="n">
-        <v>60.33</v>
+        <v>26.71</v>
       </c>
       <c r="D33" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BURNPUR</t>
+          <t>APEXECO</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>17.5</v>
+        <v>262.5</v>
       </c>
       <c r="C34" t="n">
-        <v>18.37</v>
+        <v>275.6</v>
       </c>
       <c r="D34" t="n">
-        <v>4.97</v>
+        <v>4.99</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>125.95</v>
+        <v>54.49</v>
       </c>
       <c r="C35" t="n">
-        <v>132.2</v>
+        <v>57.21</v>
       </c>
       <c r="D35" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>113.56</v>
+        <v>44.33</v>
       </c>
       <c r="C36" t="n">
-        <v>119.17</v>
+        <v>46.54</v>
       </c>
       <c r="D36" t="n">
-        <v>4.94</v>
+        <v>4.99</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>79.09</v>
+        <v>303.4</v>
       </c>
       <c r="C37" t="n">
-        <v>83</v>
+        <v>318.55</v>
       </c>
       <c r="D37" t="n">
-        <v>4.94</v>
+        <v>4.99</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CLSL</t>
+          <t>TIRUPATIFL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>74.95</v>
+        <v>67.68000000000001</v>
       </c>
       <c r="C38" t="n">
-        <v>78.65000000000001</v>
+        <v>71.06</v>
       </c>
       <c r="D38" t="n">
-        <v>4.94</v>
+        <v>4.99</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>APOORVA</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8.539999999999999</v>
+        <v>31.05</v>
       </c>
       <c r="C39" t="n">
-        <v>8.960000000000001</v>
+        <v>32.6</v>
       </c>
       <c r="D39" t="n">
-        <v>4.92</v>
+        <v>4.99</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MLKFOOD</t>
+          <t>AKANKSHA</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>79.12</v>
+        <v>139.65</v>
       </c>
       <c r="C40" t="n">
-        <v>83</v>
+        <v>146.6</v>
       </c>
       <c r="D40" t="n">
-        <v>4.9</v>
+        <v>4.98</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3.28</v>
+        <v>42.95</v>
       </c>
       <c r="C41" t="n">
-        <v>3.44</v>
+        <v>45.09</v>
       </c>
       <c r="D41" t="n">
-        <v>4.88</v>
+        <v>4.98</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TIPSFILMS</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>318.5</v>
+        <v>25.2</v>
       </c>
       <c r="C42" t="n">
-        <v>333.95</v>
+        <v>26.45</v>
       </c>
       <c r="D42" t="n">
-        <v>4.85</v>
+        <v>4.96</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>KARAMTARA</t>
+          <t>AMEYA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>352</v>
+        <v>142.55</v>
       </c>
       <c r="C43" t="n">
-        <v>369</v>
+        <v>149.6</v>
       </c>
       <c r="D43" t="n">
-        <v>4.83</v>
+        <v>4.95</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ABCOTS</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>210.83</v>
+        <v>3.44</v>
       </c>
       <c r="C44" t="n">
-        <v>221</v>
+        <v>3.61</v>
       </c>
       <c r="D44" t="n">
-        <v>4.82</v>
+        <v>4.94</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>BGLOBAL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>21</v>
+        <v>3.05</v>
       </c>
       <c r="C45" t="n">
-        <v>22</v>
+        <v>3.2</v>
       </c>
       <c r="D45" t="n">
-        <v>4.76</v>
+        <v>4.92</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4.01</v>
+        <v>70.02</v>
       </c>
       <c r="C46" t="n">
-        <v>4.2</v>
+        <v>73.45</v>
       </c>
       <c r="D46" t="n">
-        <v>4.74</v>
+        <v>4.9</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>REFRACTORY</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>24.11</v>
+        <v>31.65</v>
       </c>
       <c r="C47" t="n">
-        <v>25.25</v>
+        <v>33.2</v>
       </c>
       <c r="D47" t="n">
-        <v>4.73</v>
+        <v>4.9</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>5.11</v>
+        <v>1287</v>
       </c>
       <c r="C48" t="n">
-        <v>5.35</v>
+        <v>1350</v>
       </c>
       <c r="D48" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6.86</v>
+        <v>22.29</v>
       </c>
       <c r="C49" t="n">
-        <v>7.18</v>
+        <v>23.38</v>
       </c>
       <c r="D49" t="n">
-        <v>4.66</v>
+        <v>4.89</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>FELDVR</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>32.97</v>
+        <v>2.05</v>
       </c>
       <c r="C50" t="n">
-        <v>34.49</v>
+        <v>2.15</v>
       </c>
       <c r="D50" t="n">
-        <v>4.61</v>
+        <v>4.88</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1.32</v>
+        <v>334.75</v>
       </c>
       <c r="C51" t="n">
-        <v>1.38</v>
+        <v>351.05</v>
       </c>
       <c r="D51" t="n">
-        <v>4.55</v>
+        <v>4.87</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>18.41</v>
+        <v>273.7</v>
       </c>
       <c r="C52" t="n">
-        <v>19.24</v>
+        <v>286.95</v>
       </c>
       <c r="D52" t="n">
-        <v>4.51</v>
+        <v>4.84</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SHREEDHAR</t>
+          <t>KLL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>153.35</v>
+        <v>32.4</v>
       </c>
       <c r="C53" t="n">
-        <v>160.25</v>
+        <v>33.95</v>
       </c>
       <c r="D53" t="n">
-        <v>4.5</v>
+        <v>4.78</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>CONSOFINVT</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>81.37</v>
+        <v>302.2</v>
       </c>
       <c r="C54" t="n">
-        <v>84.90000000000001</v>
+        <v>316.6</v>
       </c>
       <c r="D54" t="n">
-        <v>4.34</v>
+        <v>4.77</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.7</v>
+        <v>4.2</v>
       </c>
       <c r="C55" t="n">
-        <v>0.73</v>
+        <v>4.4</v>
       </c>
       <c r="D55" t="n">
-        <v>4.29</v>
+        <v>4.76</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SRGHFL</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>126.65</v>
+        <v>2.75</v>
       </c>
       <c r="C56" t="n">
-        <v>132.05</v>
+        <v>2.88</v>
       </c>
       <c r="D56" t="n">
-        <v>4.26</v>
+        <v>4.73</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NEPHROCARE</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>91.65000000000001</v>
+        <v>1.69</v>
       </c>
       <c r="C57" t="n">
-        <v>95.55</v>
+        <v>1.77</v>
       </c>
       <c r="D57" t="n">
-        <v>4.26</v>
+        <v>4.73</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>KALANA</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>14.62</v>
+        <v>18.5</v>
       </c>
       <c r="C58" t="n">
-        <v>15.24</v>
+        <v>19.35</v>
       </c>
       <c r="D58" t="n">
-        <v>4.24</v>
+        <v>4.59</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>GLOBALE</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>21.68</v>
+        <v>11</v>
       </c>
       <c r="C59" t="n">
-        <v>22.6</v>
+        <v>11.5</v>
       </c>
       <c r="D59" t="n">
-        <v>4.24</v>
+        <v>4.55</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>ORIENTLTD</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.48</v>
+        <v>80.81999999999999</v>
       </c>
       <c r="C60" t="n">
-        <v>0.5</v>
+        <v>84.5</v>
       </c>
       <c r="D60" t="n">
-        <v>4.17</v>
+        <v>4.55</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>446.5</v>
+        <v>7.48</v>
       </c>
       <c r="C61" t="n">
-        <v>465</v>
+        <v>7.82</v>
       </c>
       <c r="D61" t="n">
-        <v>4.14</v>
+        <v>4.55</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ALPHAGEO</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>294.95</v>
+        <v>2.43</v>
       </c>
       <c r="C62" t="n">
-        <v>306.95</v>
+        <v>2.54</v>
       </c>
       <c r="D62" t="n">
-        <v>4.07</v>
+        <v>4.53</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AAATECH</t>
+          <t>CARBORUNIV</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>84.56999999999999</v>
+        <v>1124.4</v>
       </c>
       <c r="C63" t="n">
-        <v>88</v>
+        <v>1175</v>
       </c>
       <c r="D63" t="n">
-        <v>4.06</v>
+        <v>4.5</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MADHAV</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>34.5</v>
+        <v>2.24</v>
       </c>
       <c r="C64" t="n">
-        <v>35.9</v>
+        <v>2.34</v>
       </c>
       <c r="D64" t="n">
-        <v>4.06</v>
+        <v>4.46</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>CRAVATEX</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.74</v>
+        <v>324.55</v>
       </c>
       <c r="C65" t="n">
-        <v>0.77</v>
+        <v>338.95</v>
       </c>
       <c r="D65" t="n">
-        <v>4.05</v>
+        <v>4.44</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>JPPOWER</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>23.44</v>
+        <v>15.37</v>
       </c>
       <c r="C66" t="n">
-        <v>24.38</v>
+        <v>16.05</v>
       </c>
       <c r="D66" t="n">
-        <v>4.01</v>
+        <v>4.42</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>34.94</v>
+        <v>10.47</v>
       </c>
       <c r="C67" t="n">
-        <v>36.33</v>
+        <v>10.93</v>
       </c>
       <c r="D67" t="n">
-        <v>3.98</v>
+        <v>4.39</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>631.9</v>
+        <v>4.39</v>
       </c>
       <c r="C68" t="n">
-        <v>657</v>
+        <v>4.58</v>
       </c>
       <c r="D68" t="n">
-        <v>3.97</v>
+        <v>4.33</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GLASSWALL</t>
+          <t>LKPSEC</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>257.82</v>
+        <v>15.01</v>
       </c>
       <c r="C69" t="n">
-        <v>267.98</v>
+        <v>15.66</v>
       </c>
       <c r="D69" t="n">
-        <v>3.94</v>
+        <v>4.33</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LAGNAM</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>70.23999999999999</v>
+        <v>1.16</v>
       </c>
       <c r="C70" t="n">
-        <v>73</v>
+        <v>1.21</v>
       </c>
       <c r="D70" t="n">
-        <v>3.93</v>
+        <v>4.31</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LKPSEC</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>15.06</v>
+        <v>177.36</v>
       </c>
       <c r="C71" t="n">
-        <v>15.65</v>
+        <v>185</v>
       </c>
       <c r="D71" t="n">
-        <v>3.92</v>
+        <v>4.31</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SHEMAROO</t>
+          <t>SRIKPRIND</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>115.5</v>
+        <v>27.98</v>
       </c>
       <c r="C72" t="n">
-        <v>120</v>
+        <v>29.18</v>
       </c>
       <c r="D72" t="n">
-        <v>3.9</v>
+        <v>4.29</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BATLIBOI</t>
+          <t>APTECHT</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>78.73</v>
+        <v>92.05</v>
       </c>
       <c r="C73" t="n">
-        <v>81.8</v>
+        <v>96</v>
       </c>
       <c r="D73" t="n">
-        <v>3.9</v>
+        <v>4.29</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>NAGREEKCAP</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>27.92</v>
+        <v>21.48</v>
       </c>
       <c r="C74" t="n">
-        <v>29</v>
+        <v>22.4</v>
       </c>
       <c r="D74" t="n">
-        <v>3.87</v>
+        <v>4.28</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>56.6</v>
+        <v>11.57</v>
       </c>
       <c r="C75" t="n">
-        <v>58.79</v>
+        <v>12.06</v>
       </c>
       <c r="D75" t="n">
-        <v>3.87</v>
+        <v>4.24</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>UCAL</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>6.97</v>
+        <v>138.15</v>
       </c>
       <c r="C76" t="n">
-        <v>7.24</v>
+        <v>144</v>
       </c>
       <c r="D76" t="n">
-        <v>3.87</v>
+        <v>4.23</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GREENPOWER</t>
+          <t>KHAITANLTD</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>9.050000000000001</v>
+        <v>152.13</v>
       </c>
       <c r="C77" t="n">
-        <v>9.4</v>
+        <v>158.5</v>
       </c>
       <c r="D77" t="n">
-        <v>3.87</v>
+        <v>4.19</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>21.84</v>
+        <v>0.48</v>
       </c>
       <c r="C78" t="n">
-        <v>22.68</v>
+        <v>0.5</v>
       </c>
       <c r="D78" t="n">
-        <v>3.85</v>
+        <v>4.17</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SHAHALLOYS</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>92.47</v>
+        <v>61.06</v>
       </c>
       <c r="C79" t="n">
-        <v>95.98999999999999</v>
+        <v>63.6</v>
       </c>
       <c r="D79" t="n">
-        <v>3.81</v>
+        <v>4.16</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AVPINFRA</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>57.8</v>
+        <v>0.73</v>
       </c>
       <c r="C80" t="n">
-        <v>60</v>
+        <v>0.76</v>
       </c>
       <c r="D80" t="n">
-        <v>3.81</v>
+        <v>4.11</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>BI</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>530.45</v>
+        <v>107.62</v>
       </c>
       <c r="C81" t="n">
-        <v>550.45</v>
+        <v>112</v>
       </c>
       <c r="D81" t="n">
-        <v>3.77</v>
+        <v>4.07</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>MLKFOOD</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.53</v>
+        <v>79.81999999999999</v>
       </c>
       <c r="C82" t="n">
-        <v>0.55</v>
+        <v>83</v>
       </c>
       <c r="D82" t="n">
-        <v>3.77</v>
+        <v>3.98</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>16.73</v>
+        <v>2.78</v>
       </c>
       <c r="C83" t="n">
-        <v>17.36</v>
+        <v>2.89</v>
       </c>
       <c r="D83" t="n">
-        <v>3.77</v>
+        <v>3.96</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DEEP</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>47.23</v>
+        <v>46.47</v>
       </c>
       <c r="C84" t="n">
-        <v>49</v>
+        <v>48.3</v>
       </c>
       <c r="D84" t="n">
-        <v>3.75</v>
+        <v>3.94</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>315.2</v>
+        <v>6.11</v>
       </c>
       <c r="C85" t="n">
-        <v>327</v>
+        <v>6.35</v>
       </c>
       <c r="D85" t="n">
-        <v>3.74</v>
+        <v>3.93</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ICELCO</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>121.5</v>
+        <v>0.77</v>
       </c>
       <c r="C86" t="n">
-        <v>125.95</v>
+        <v>0.8</v>
       </c>
       <c r="D86" t="n">
-        <v>3.66</v>
+        <v>3.9</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>VGCL</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>7.67</v>
+        <v>48.42</v>
       </c>
       <c r="C87" t="n">
-        <v>7.95</v>
+        <v>50.29</v>
       </c>
       <c r="D87" t="n">
-        <v>3.65</v>
+        <v>3.86</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GAUDIUMIVF</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>114.79</v>
+        <v>2.07</v>
       </c>
       <c r="C88" t="n">
-        <v>118.96</v>
+        <v>2.15</v>
       </c>
       <c r="D88" t="n">
-        <v>3.63</v>
+        <v>3.86</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>122.75</v>
+        <v>7.8</v>
       </c>
       <c r="C89" t="n">
-        <v>127.15</v>
+        <v>8.1</v>
       </c>
       <c r="D89" t="n">
-        <v>3.58</v>
+        <v>3.85</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>3.35</v>
+        <v>38.04</v>
       </c>
       <c r="C90" t="n">
-        <v>3.47</v>
+        <v>39.5</v>
       </c>
       <c r="D90" t="n">
-        <v>3.58</v>
+        <v>3.84</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>34.71</v>
+        <v>30.09</v>
       </c>
       <c r="C91" t="n">
-        <v>35.95</v>
+        <v>31.23</v>
       </c>
       <c r="D91" t="n">
-        <v>3.57</v>
+        <v>3.79</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>2.8</v>
+        <v>5.06</v>
       </c>
       <c r="C92" t="n">
-        <v>2.9</v>
+        <v>5.25</v>
       </c>
       <c r="D92" t="n">
-        <v>3.57</v>
+        <v>3.75</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>GENCON</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>7.05</v>
+        <v>40.01</v>
       </c>
       <c r="C93" t="n">
-        <v>7.3</v>
+        <v>41.5</v>
       </c>
       <c r="D93" t="n">
-        <v>3.55</v>
+        <v>3.72</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>19.28</v>
+        <v>271.85</v>
       </c>
       <c r="C94" t="n">
-        <v>19.95</v>
+        <v>281.95</v>
       </c>
       <c r="D94" t="n">
-        <v>3.48</v>
+        <v>3.72</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>33.31</v>
+        <v>2660.1</v>
       </c>
       <c r="C95" t="n">
-        <v>34.45</v>
+        <v>2758</v>
       </c>
       <c r="D95" t="n">
-        <v>3.42</v>
+        <v>3.68</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>PAVNAIND</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>4.11</v>
+        <v>15.67</v>
       </c>
       <c r="C96" t="n">
-        <v>4.25</v>
+        <v>16.24</v>
       </c>
       <c r="D96" t="n">
-        <v>3.41</v>
+        <v>3.64</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>KMEW</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>441.95</v>
+        <v>2885.6</v>
       </c>
       <c r="C97" t="n">
-        <v>457</v>
+        <v>2990</v>
       </c>
       <c r="D97" t="n">
-        <v>3.41</v>
+        <v>3.62</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MOHITIND</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>23.2</v>
+        <v>0.28</v>
       </c>
       <c r="C98" t="n">
-        <v>23.99</v>
+        <v>0.29</v>
       </c>
       <c r="D98" t="n">
-        <v>3.41</v>
+        <v>3.57</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>25.15</v>
+        <v>22.21</v>
       </c>
       <c r="C99" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D99" t="n">
-        <v>3.38</v>
+        <v>3.56</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IRMENERGY</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>269.1</v>
+        <v>40.56</v>
       </c>
       <c r="C100" t="n">
-        <v>278.15</v>
+        <v>42</v>
       </c>
       <c r="D100" t="n">
-        <v>3.36</v>
+        <v>3.55</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AONESILVER</t>
+          <t>PRADPME</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>8.66</v>
+        <v>453.5</v>
       </c>
       <c r="C101" t="n">
-        <v>8.949999999999999</v>
+        <v>469.5</v>
       </c>
       <c r="D101" t="n">
-        <v>3.35</v>
+        <v>3.53</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>WEIZMANIND</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1008.6</v>
+        <v>71.48</v>
       </c>
       <c r="C102" t="n">
-        <v>1042.4</v>
+        <v>74</v>
       </c>
       <c r="D102" t="n">
-        <v>3.35</v>
+        <v>3.53</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>VIRAT</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>382.25</v>
+        <v>3.13</v>
       </c>
       <c r="C103" t="n">
-        <v>394.9</v>
+        <v>3.24</v>
       </c>
       <c r="D103" t="n">
-        <v>3.31</v>
+        <v>3.51</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>7.25</v>
+        <v>7.99</v>
       </c>
       <c r="C104" t="n">
-        <v>7.49</v>
+        <v>8.27</v>
       </c>
       <c r="D104" t="n">
-        <v>3.31</v>
+        <v>3.5</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>URJA</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>9.1</v>
+        <v>14</v>
       </c>
       <c r="C105" t="n">
-        <v>9.4</v>
+        <v>14.49</v>
       </c>
       <c r="D105" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>401.65</v>
+        <v>33.56</v>
       </c>
       <c r="C106" t="n">
-        <v>414.85</v>
+        <v>34.73</v>
       </c>
       <c r="D106" t="n">
-        <v>3.29</v>
+        <v>3.49</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>KARMAENG</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>6.1</v>
+        <v>41.27</v>
       </c>
       <c r="C107" t="n">
-        <v>6.3</v>
+        <v>42.7</v>
       </c>
       <c r="D107" t="n">
-        <v>3.28</v>
+        <v>3.46</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ARENTERP</t>
+          <t>GCHOTELS</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>34.2</v>
+        <v>115.05</v>
       </c>
       <c r="C108" t="n">
-        <v>35.3</v>
+        <v>119</v>
       </c>
       <c r="D108" t="n">
-        <v>3.22</v>
+        <v>3.43</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>NAHARCAP</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>250</v>
+        <v>4.09</v>
       </c>
       <c r="C109" t="n">
-        <v>257.95</v>
+        <v>4.23</v>
       </c>
       <c r="D109" t="n">
-        <v>3.18</v>
+        <v>3.42</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>WOMANCART</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>101</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="C110" t="n">
-        <v>104.2</v>
+        <v>9.09</v>
       </c>
       <c r="D110" t="n">
-        <v>3.17</v>
+        <v>3.41</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>5.99</v>
+        <v>17.06</v>
       </c>
       <c r="C111" t="n">
-        <v>6.18</v>
+        <v>17.64</v>
       </c>
       <c r="D111" t="n">
-        <v>3.17</v>
+        <v>3.4</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ORISSAMINE</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>3896.4</v>
+        <v>8.6</v>
       </c>
       <c r="C112" t="n">
-        <v>4020</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="D112" t="n">
-        <v>3.17</v>
+        <v>3.37</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>VETO</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>63</v>
+        <v>139.15</v>
       </c>
       <c r="C113" t="n">
-        <v>64.98999999999999</v>
+        <v>143.8</v>
       </c>
       <c r="D113" t="n">
-        <v>3.16</v>
+        <v>3.34</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SOMICONVEY</t>
+          <t>HINDALUMI</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>94.59999999999999</v>
+        <v>94.27</v>
       </c>
       <c r="C114" t="n">
-        <v>97.59</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="D114" t="n">
-        <v>3.16</v>
+        <v>3.32</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>VRAJ</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>42.46</v>
+        <v>127.74</v>
       </c>
       <c r="C115" t="n">
-        <v>43.8</v>
+        <v>131.94</v>
       </c>
       <c r="D115" t="n">
-        <v>3.16</v>
+        <v>3.29</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>16.19</v>
+        <v>525.7</v>
       </c>
       <c r="C116" t="n">
-        <v>16.7</v>
+        <v>543</v>
       </c>
       <c r="D116" t="n">
-        <v>3.15</v>
+        <v>3.29</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>243.45</v>
+        <v>32.45</v>
       </c>
       <c r="C117" t="n">
-        <v>251</v>
+        <v>33.5</v>
       </c>
       <c r="D117" t="n">
-        <v>3.1</v>
+        <v>3.24</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>KELLTONTEC</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>13.57</v>
+        <v>126.31</v>
       </c>
       <c r="C118" t="n">
-        <v>13.99</v>
+        <v>130.38</v>
       </c>
       <c r="D118" t="n">
-        <v>3.1</v>
+        <v>3.22</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GUJAPOLLO</t>
+          <t>SAPPL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>324</v>
+        <v>276.15</v>
       </c>
       <c r="C119" t="n">
-        <v>333.95</v>
+        <v>285</v>
       </c>
       <c r="D119" t="n">
-        <v>3.07</v>
+        <v>3.2</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>22.27</v>
+        <v>6.01</v>
       </c>
       <c r="C120" t="n">
-        <v>22.94</v>
+        <v>6.2</v>
       </c>
       <c r="D120" t="n">
-        <v>3.01</v>
+        <v>3.16</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>KMCSHIL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>827.45</v>
+        <v>150.26</v>
       </c>
       <c r="C121" t="n">
-        <v>852</v>
+        <v>155</v>
       </c>
       <c r="D121" t="n">
-        <v>2.97</v>
+        <v>3.15</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>SHRADHA</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>1392.8</v>
+        <v>30</v>
       </c>
       <c r="C122" t="n">
-        <v>1434</v>
+        <v>30.94</v>
       </c>
       <c r="D122" t="n">
-        <v>2.96</v>
+        <v>3.13</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1.37</v>
+        <v>39.48</v>
       </c>
       <c r="C123" t="n">
-        <v>1.41</v>
+        <v>40.7</v>
       </c>
       <c r="D123" t="n">
-        <v>2.92</v>
+        <v>3.09</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CPL</t>
+          <t>AURUS</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>65.39</v>
+        <v>4.87</v>
       </c>
       <c r="C124" t="n">
-        <v>67.3</v>
+        <v>5.02</v>
       </c>
       <c r="D124" t="n">
-        <v>2.92</v>
+        <v>3.08</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>LAMBODHARA</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>8.59</v>
+        <v>120.21</v>
       </c>
       <c r="C125" t="n">
-        <v>8.84</v>
+        <v>123.9</v>
       </c>
       <c r="D125" t="n">
-        <v>2.91</v>
+        <v>3.07</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>25.78</v>
+        <v>193.1</v>
       </c>
       <c r="C126" t="n">
-        <v>26.52</v>
+        <v>199</v>
       </c>
       <c r="D126" t="n">
-        <v>2.87</v>
+        <v>3.06</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>KONSTELEC</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>220.25</v>
+        <v>59.05</v>
       </c>
       <c r="C127" t="n">
-        <v>226.5</v>
+        <v>60.85</v>
       </c>
       <c r="D127" t="n">
-        <v>2.84</v>
+        <v>3.05</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>VALIANTORG</t>
+          <t>MOTOGENFIN</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>408.45</v>
+        <v>26.19</v>
       </c>
       <c r="C128" t="n">
-        <v>420</v>
+        <v>26.99</v>
       </c>
       <c r="D128" t="n">
-        <v>2.83</v>
+        <v>3.05</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>VILAS</t>
+          <t>MODINATUR</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>331.6</v>
+        <v>359.05</v>
       </c>
       <c r="C129" t="n">
-        <v>341</v>
+        <v>370</v>
       </c>
       <c r="D129" t="n">
-        <v>2.83</v>
+        <v>3.05</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>35.2</v>
+        <v>2.96</v>
       </c>
       <c r="C130" t="n">
-        <v>36.19</v>
+        <v>3.05</v>
       </c>
       <c r="D130" t="n">
-        <v>2.81</v>
+        <v>3.04</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>LAHOTIOV</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>48.66</v>
+        <v>39.26</v>
       </c>
       <c r="C131" t="n">
-        <v>50</v>
+        <v>40.45</v>
       </c>
       <c r="D131" t="n">
-        <v>2.75</v>
+        <v>3.03</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>5.83</v>
+        <v>33.15</v>
       </c>
       <c r="C132" t="n">
-        <v>5.99</v>
+        <v>34.14</v>
       </c>
       <c r="D132" t="n">
-        <v>2.74</v>
+        <v>2.99</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>RHL</t>
+          <t>SUNLITE</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>173.74</v>
+        <v>644.9</v>
       </c>
       <c r="C133" t="n">
-        <v>178.5</v>
+        <v>663.95</v>
       </c>
       <c r="D133" t="n">
-        <v>2.74</v>
+        <v>2.95</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>RIR</t>
+          <t>HAZOOR</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>197.63</v>
+        <v>19.3</v>
       </c>
       <c r="C134" t="n">
-        <v>203</v>
+        <v>19.86</v>
       </c>
       <c r="D134" t="n">
-        <v>2.72</v>
+        <v>2.9</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>LEAPIND</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>13.04</v>
+        <v>140.47</v>
       </c>
       <c r="C135" t="n">
-        <v>13.39</v>
+        <v>144.52</v>
       </c>
       <c r="D135" t="n">
-        <v>2.68</v>
+        <v>2.88</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RUDRA</t>
+          <t>MIRZAINT</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>20.36</v>
+        <v>29.14</v>
       </c>
       <c r="C136" t="n">
-        <v>20.9</v>
+        <v>29.98</v>
       </c>
       <c r="D136" t="n">
-        <v>2.65</v>
+        <v>2.88</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>30.2</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="C137" t="n">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="D137" t="n">
-        <v>2.65</v>
+        <v>2.87</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SUPERHOUSE</t>
+          <t>HEG</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>167.58</v>
+        <v>237.05</v>
       </c>
       <c r="C138" t="n">
-        <v>171.95</v>
+        <v>243.85</v>
       </c>
       <c r="D138" t="n">
-        <v>2.61</v>
+        <v>2.87</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>ABH</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>35.97</v>
+        <v>43.75</v>
       </c>
       <c r="C139" t="n">
-        <v>36.9</v>
+        <v>45</v>
       </c>
       <c r="D139" t="n">
-        <v>2.59</v>
+        <v>2.86</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>LANCORHOL</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>10.02</v>
+        <v>35</v>
       </c>
       <c r="C140" t="n">
-        <v>10.28</v>
+        <v>36</v>
       </c>
       <c r="D140" t="n">
-        <v>2.59</v>
+        <v>2.86</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>XELPMOC</t>
+          <t>PRESSTONIC</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>74.08</v>
+        <v>29.95</v>
       </c>
       <c r="C141" t="n">
-        <v>75.98999999999999</v>
+        <v>30.8</v>
       </c>
       <c r="D141" t="n">
-        <v>2.58</v>
+        <v>2.84</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>PAISALO</t>
+          <t>ONIDA</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>88.73</v>
+        <v>32.89</v>
       </c>
       <c r="C142" t="n">
-        <v>91</v>
+        <v>33.82</v>
       </c>
       <c r="D142" t="n">
-        <v>2.56</v>
+        <v>2.83</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>7.07</v>
+        <v>6.71</v>
       </c>
       <c r="C143" t="n">
-        <v>7.25</v>
+        <v>6.9</v>
       </c>
       <c r="D143" t="n">
-        <v>2.55</v>
+        <v>2.83</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>VITAL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>1456</v>
+        <v>55.4</v>
       </c>
       <c r="C144" t="n">
-        <v>1493</v>
+        <v>56.95</v>
       </c>
       <c r="D144" t="n">
-        <v>2.54</v>
+        <v>2.8</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>CONCORDBIO</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>5.14</v>
+        <v>1494.4</v>
       </c>
       <c r="C145" t="n">
-        <v>5.27</v>
+        <v>1536</v>
       </c>
       <c r="D145" t="n">
-        <v>2.53</v>
+        <v>2.78</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>5.13</v>
+        <v>13.72</v>
       </c>
       <c r="C146" t="n">
-        <v>5.26</v>
+        <v>14.1</v>
       </c>
       <c r="D146" t="n">
-        <v>2.53</v>
+        <v>2.77</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>BEEKAY</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>8.779999999999999</v>
+        <v>430.05</v>
       </c>
       <c r="C147" t="n">
-        <v>9</v>
+        <v>441.9</v>
       </c>
       <c r="D147" t="n">
-        <v>2.51</v>
+        <v>2.76</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>AEROFLEX</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>497.6</v>
+        <v>446.7</v>
       </c>
       <c r="C148" t="n">
-        <v>510</v>
+        <v>458.9</v>
       </c>
       <c r="D148" t="n">
-        <v>2.49</v>
+        <v>2.73</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>6.05</v>
+        <v>172.31</v>
       </c>
       <c r="C149" t="n">
-        <v>6.2</v>
+        <v>177</v>
       </c>
       <c r="D149" t="n">
-        <v>2.48</v>
+        <v>2.72</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>INDOWIND</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>8.93</v>
+        <v>13.63</v>
       </c>
       <c r="C150" t="n">
-        <v>9.15</v>
+        <v>14</v>
       </c>
       <c r="D150" t="n">
-        <v>2.46</v>
+        <v>2.71</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>BIL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.41</v>
+        <v>1040.85</v>
       </c>
       <c r="C151" t="n">
-        <v>0.42</v>
+        <v>1069</v>
       </c>
       <c r="D151" t="n">
-        <v>2.44</v>
+        <v>2.7</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SHIVASHRIT</t>
+          <t>WEL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>115.2</v>
+        <v>72.94</v>
       </c>
       <c r="C152" t="n">
-        <v>118</v>
+        <v>74.89</v>
       </c>
       <c r="D152" t="n">
-        <v>2.43</v>
+        <v>2.67</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>SWARNSAR</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>37.05</v>
+        <v>38.96</v>
       </c>
       <c r="C153" t="n">
-        <v>37.95</v>
+        <v>40</v>
       </c>
       <c r="D153" t="n">
-        <v>2.43</v>
+        <v>2.67</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>YATHARTH</t>
+          <t>VISHWARAJ</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>1072.4</v>
+        <v>5.31</v>
       </c>
       <c r="C154" t="n">
-        <v>1098</v>
+        <v>5.45</v>
       </c>
       <c r="D154" t="n">
-        <v>2.39</v>
+        <v>2.64</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>KAYA</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>72.05</v>
+        <v>341</v>
       </c>
       <c r="C155" t="n">
-        <v>73.75</v>
+        <v>350</v>
       </c>
       <c r="D155" t="n">
-        <v>2.36</v>
+        <v>2.64</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SILVERCASE</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>22.95</v>
+        <v>10.37</v>
       </c>
       <c r="C156" t="n">
-        <v>23.48</v>
+        <v>10.64</v>
       </c>
       <c r="D156" t="n">
-        <v>2.31</v>
+        <v>2.6</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>GOACARBON</t>
+          <t>NILASPACES</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>378.3</v>
+        <v>12.3</v>
       </c>
       <c r="C157" t="n">
-        <v>387</v>
+        <v>12.62</v>
       </c>
       <c r="D157" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>4.35</v>
+        <v>1.93</v>
       </c>
       <c r="C158" t="n">
-        <v>4.45</v>
+        <v>1.98</v>
       </c>
       <c r="D158" t="n">
-        <v>2.3</v>
+        <v>2.59</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>NECCLTD</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>18.82</v>
+        <v>61.42</v>
       </c>
       <c r="C159" t="n">
-        <v>19.25</v>
+        <v>63</v>
       </c>
       <c r="D159" t="n">
-        <v>2.28</v>
+        <v>2.57</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RAMBHAJO</t>
+          <t>LEENEE</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>266.17</v>
+        <v>7.8</v>
       </c>
       <c r="C160" t="n">
-        <v>272.18</v>
+        <v>8</v>
       </c>
       <c r="D160" t="n">
-        <v>2.26</v>
+        <v>2.56</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MUFTI</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>73.37</v>
+        <v>23.64</v>
       </c>
       <c r="C161" t="n">
-        <v>75.02</v>
+        <v>24.24</v>
       </c>
       <c r="D161" t="n">
-        <v>2.25</v>
+        <v>2.54</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MINDTECK</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>156.84</v>
+        <v>7.12</v>
       </c>
       <c r="C162" t="n">
-        <v>160.36</v>
+        <v>7.3</v>
       </c>
       <c r="D162" t="n">
-        <v>2.24</v>
+        <v>2.53</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>TATSILV</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>21.99</v>
+        <v>20.8</v>
       </c>
       <c r="C163" t="n">
-        <v>22.48</v>
+        <v>21.32</v>
       </c>
       <c r="D163" t="n">
-        <v>2.23</v>
+        <v>2.5</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>BBNPPGOLD</t>
+          <t>MITCON</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>145.45</v>
+        <v>80.01000000000001</v>
       </c>
       <c r="C164" t="n">
-        <v>148.7</v>
+        <v>82</v>
       </c>
       <c r="D164" t="n">
-        <v>2.23</v>
+        <v>2.49</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HDFCSILVER</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>216.47</v>
+        <v>152.26</v>
       </c>
       <c r="C165" t="n">
-        <v>221.28</v>
+        <v>156.05</v>
       </c>
       <c r="D165" t="n">
-        <v>2.22</v>
+        <v>2.49</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>SILVERIETF</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>226.19</v>
+        <v>66.15000000000001</v>
       </c>
       <c r="C166" t="n">
-        <v>231.22</v>
+        <v>67.8</v>
       </c>
       <c r="D166" t="n">
-        <v>2.22</v>
+        <v>2.49</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MERCURYEV</t>
+          <t>HILINFRA</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>40.84</v>
+        <v>43.92</v>
       </c>
       <c r="C167" t="n">
-        <v>41.74</v>
+        <v>45</v>
       </c>
       <c r="D167" t="n">
-        <v>2.2</v>
+        <v>2.46</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>AMBICAAGAR</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>305.05</v>
+        <v>24.89</v>
       </c>
       <c r="C168" t="n">
-        <v>311.75</v>
+        <v>25.5</v>
       </c>
       <c r="D168" t="n">
-        <v>2.2</v>
+        <v>2.45</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>HALDYNGL</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>140.41</v>
+        <v>207.35</v>
       </c>
       <c r="C169" t="n">
-        <v>143.5</v>
+        <v>212.4</v>
       </c>
       <c r="D169" t="n">
-        <v>2.2</v>
+        <v>2.44</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>6</v>
+        <v>54.57</v>
       </c>
       <c r="C170" t="n">
-        <v>6.13</v>
+        <v>55.9</v>
       </c>
       <c r="D170" t="n">
-        <v>2.17</v>
+        <v>2.44</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>SILVER</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>226.36</v>
+        <v>2.06</v>
       </c>
       <c r="C171" t="n">
-        <v>231.24</v>
+        <v>2.11</v>
       </c>
       <c r="D171" t="n">
-        <v>2.16</v>
+        <v>2.43</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>DCM</t>
+          <t>ABHAPOWER</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>76.36</v>
+        <v>24.65</v>
       </c>
       <c r="C172" t="n">
-        <v>78</v>
+        <v>25.25</v>
       </c>
       <c r="D172" t="n">
-        <v>2.15</v>
+        <v>2.43</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SHINDL</t>
+          <t>NACLIND</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>161.05</v>
+        <v>146.75</v>
       </c>
       <c r="C173" t="n">
-        <v>164.5</v>
+        <v>150.3</v>
       </c>
       <c r="D173" t="n">
-        <v>2.14</v>
+        <v>2.42</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SBISILVER</t>
+          <t>ABCOTS</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>222.1</v>
+        <v>209.85</v>
       </c>
       <c r="C174" t="n">
-        <v>226.86</v>
+        <v>214.9</v>
       </c>
       <c r="D174" t="n">
-        <v>2.14</v>
+        <v>2.41</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>46.8</v>
+        <v>0.83</v>
       </c>
       <c r="C175" t="n">
-        <v>47.8</v>
+        <v>0.85</v>
       </c>
       <c r="D175" t="n">
-        <v>2.14</v>
+        <v>2.41</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>NDLVENTURE</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>209.45</v>
+        <v>123</v>
       </c>
       <c r="C176" t="n">
-        <v>213.9</v>
+        <v>125.95</v>
       </c>
       <c r="D176" t="n">
-        <v>2.12</v>
+        <v>2.4</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>78.34999999999999</v>
+        <v>7.07</v>
       </c>
       <c r="C177" t="n">
-        <v>80.01000000000001</v>
+        <v>7.24</v>
       </c>
       <c r="D177" t="n">
-        <v>2.12</v>
+        <v>2.4</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SILVERAXIS</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>225.27</v>
+        <v>147.57</v>
       </c>
       <c r="C178" t="n">
-        <v>230.05</v>
+        <v>151.1</v>
       </c>
       <c r="D178" t="n">
-        <v>2.12</v>
+        <v>2.39</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>VINYLINDIA</t>
+          <t>TVVISION</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>214.17</v>
+        <v>2.53</v>
       </c>
       <c r="C179" t="n">
-        <v>218.7</v>
+        <v>2.59</v>
       </c>
       <c r="D179" t="n">
-        <v>2.12</v>
+        <v>2.37</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>159.63</v>
+        <v>55.65</v>
       </c>
       <c r="C180" t="n">
-        <v>163.01</v>
+        <v>56.97</v>
       </c>
       <c r="D180" t="n">
-        <v>2.12</v>
+        <v>2.37</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>LUMINO</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>107.14</v>
+        <v>1104.85</v>
       </c>
       <c r="C181" t="n">
-        <v>109.4</v>
+        <v>1131</v>
       </c>
       <c r="D181" t="n">
-        <v>2.11</v>
+        <v>2.37</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>1.91</v>
+        <v>61.35</v>
       </c>
       <c r="C182" t="n">
-        <v>1.95</v>
+        <v>62.8</v>
       </c>
       <c r="D182" t="n">
-        <v>2.09</v>
+        <v>2.36</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>AAATECH</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>12</v>
+        <v>86.95</v>
       </c>
       <c r="C183" t="n">
-        <v>12.25</v>
+        <v>88.98</v>
       </c>
       <c r="D183" t="n">
-        <v>2.08</v>
+        <v>2.33</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>AIMTRON</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>1616.45</v>
+        <v>467.1</v>
       </c>
       <c r="C184" t="n">
-        <v>1650</v>
+        <v>477.95</v>
       </c>
       <c r="D184" t="n">
-        <v>2.08</v>
+        <v>2.32</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SILVERBEES</t>
+          <t>OSWALGREEN</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>216.64</v>
+        <v>19.44</v>
       </c>
       <c r="C185" t="n">
-        <v>221.1</v>
+        <v>19.89</v>
       </c>
       <c r="D185" t="n">
-        <v>2.06</v>
+        <v>2.31</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>0.97</v>
+        <v>24.24</v>
       </c>
       <c r="C186" t="n">
-        <v>0.99</v>
+        <v>24.8</v>
       </c>
       <c r="D186" t="n">
-        <v>2.06</v>
+        <v>2.31</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SAHYADRI</t>
+          <t>BSHSL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>359.25</v>
+        <v>87.87</v>
       </c>
       <c r="C187" t="n">
-        <v>366.6</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="D187" t="n">
-        <v>2.05</v>
+        <v>2.31</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>VICTORYEV</t>
+          <t>INTENTECH</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>14.6</v>
+        <v>78.14</v>
       </c>
       <c r="C188" t="n">
-        <v>14.9</v>
+        <v>79.94</v>
       </c>
       <c r="D188" t="n">
-        <v>2.05</v>
+        <v>2.3</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>5.87</v>
+        <v>145.19</v>
       </c>
       <c r="C189" t="n">
-        <v>5.99</v>
+        <v>148.5</v>
       </c>
       <c r="D189" t="n">
-        <v>2.04</v>
+        <v>2.28</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>24.64</v>
+        <v>575.1</v>
       </c>
       <c r="C190" t="n">
-        <v>25.14</v>
+        <v>588</v>
       </c>
       <c r="D190" t="n">
-        <v>2.03</v>
+        <v>2.24</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ALPA</t>
+          <t>CFEL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>59.64</v>
+        <v>46.95</v>
       </c>
       <c r="C191" t="n">
-        <v>60.85</v>
+        <v>48</v>
       </c>
       <c r="D191" t="n">
-        <v>2.03</v>
+        <v>2.24</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>DENORA</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>37.07</v>
+        <v>782.25</v>
       </c>
       <c r="C192" t="n">
-        <v>37.82</v>
+        <v>799.65</v>
       </c>
       <c r="D192" t="n">
-        <v>2.02</v>
+        <v>2.22</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>EASTWEST</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>5.44</v>
+        <v>2.25</v>
       </c>
       <c r="C193" t="n">
-        <v>5.55</v>
+        <v>2.3</v>
       </c>
       <c r="D193" t="n">
-        <v>2.02</v>
+        <v>2.22</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>CRSL</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>2.47</v>
+        <v>4.96</v>
       </c>
       <c r="C194" t="n">
-        <v>2.52</v>
+        <v>5.07</v>
       </c>
       <c r="D194" t="n">
-        <v>2.02</v>
+        <v>2.22</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>57.05</v>
+        <v>613.45</v>
       </c>
       <c r="C195" t="n">
-        <v>58.2</v>
+        <v>627</v>
       </c>
       <c r="D195" t="n">
-        <v>2.02</v>
+        <v>2.21</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>GEECEE</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>35.46</v>
+        <v>371.85</v>
       </c>
       <c r="C196" t="n">
-        <v>36.17</v>
+        <v>380</v>
       </c>
       <c r="D196" t="n">
-        <v>2</v>
+        <v>2.19</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>359.6</v>
+        <v>316.85</v>
       </c>
       <c r="C197" t="n">
-        <v>366.8</v>
+        <v>323.75</v>
       </c>
       <c r="D197" t="n">
-        <v>2</v>
+        <v>2.18</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ADVAIT</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>1990.4</v>
+        <v>16.13</v>
       </c>
       <c r="C198" t="n">
-        <v>2030</v>
+        <v>16.48</v>
       </c>
       <c r="D198" t="n">
-        <v>1.99</v>
+        <v>2.17</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>ANNU</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>15.55</v>
+        <v>50.46</v>
       </c>
       <c r="C199" t="n">
-        <v>15.86</v>
+        <v>51.55</v>
       </c>
       <c r="D199" t="n">
-        <v>1.99</v>
+        <v>2.16</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>26.66</v>
+        <v>19.19</v>
       </c>
       <c r="C200" t="n">
-        <v>27.19</v>
+        <v>19.6</v>
       </c>
       <c r="D200" t="n">
-        <v>1.99</v>
+        <v>2.14</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ANSALAPI</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>3.52</v>
+        <v>82.26000000000001</v>
       </c>
       <c r="C201" t="n">
-        <v>3.59</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="D201" t="n">
-        <v>1.99</v>
+        <v>2.13</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-22 08:49 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TOUCHWOOD</t>
+          <t>TRANSCOR</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60.93</v>
+        <v>24.97</v>
       </c>
       <c r="C2" t="n">
-        <v>68.95</v>
+        <v>29</v>
       </c>
       <c r="D2" t="n">
-        <v>13.16</v>
+        <v>16.14</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5.5</v>
+        <v>317.45</v>
       </c>
       <c r="C3" t="n">
-        <v>6.05</v>
+        <v>365</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>14.98</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RRECL</t>
+          <t>ORIRAIL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>138.89</v>
+        <v>116.41</v>
       </c>
       <c r="C4" t="n">
-        <v>152</v>
+        <v>128.75</v>
       </c>
       <c r="D4" t="n">
-        <v>9.44</v>
+        <v>10.6</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ENCOMPAS</t>
+          <t>PRESSTONIC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>238.85</v>
+        <v>35.9</v>
       </c>
       <c r="C5" t="n">
-        <v>259.5</v>
+        <v>39.5</v>
       </c>
       <c r="D5" t="n">
-        <v>8.65</v>
+        <v>10.03</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MPEL-RE</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.8</v>
+        <v>4.9</v>
       </c>
       <c r="C6" t="n">
-        <v>1.95</v>
+        <v>5.39</v>
       </c>
       <c r="D6" t="n">
-        <v>8.33</v>
+        <v>10</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>87.66</v>
+        <v>6.05</v>
       </c>
       <c r="C7" t="n">
-        <v>94.95</v>
+        <v>6.65</v>
       </c>
       <c r="D7" t="n">
-        <v>8.32</v>
+        <v>9.92</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SHAILY</t>
+          <t>ARVEE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3149.8</v>
+        <v>208.87</v>
       </c>
       <c r="C8" t="n">
-        <v>3396.9</v>
+        <v>224.9</v>
       </c>
       <c r="D8" t="n">
-        <v>7.84</v>
+        <v>7.67</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.14</v>
+        <v>177.2</v>
       </c>
       <c r="C9" t="n">
-        <v>0.15</v>
+        <v>190</v>
       </c>
       <c r="D9" t="n">
-        <v>7.14</v>
+        <v>7.22</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>97.84999999999999</v>
+        <v>9.24</v>
       </c>
       <c r="C10" t="n">
-        <v>104.7</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>7.03</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>236.6</v>
+        <v>154.86</v>
       </c>
       <c r="C11" t="n">
-        <v>253</v>
+        <v>165.5</v>
       </c>
       <c r="D11" t="n">
-        <v>6.93</v>
+        <v>6.87</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>RHIM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15.92</v>
+        <v>368</v>
       </c>
       <c r="C12" t="n">
-        <v>17</v>
+        <v>392.6</v>
       </c>
       <c r="D12" t="n">
-        <v>6.78</v>
+        <v>6.68</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ORIANA</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>271.75</v>
+        <v>1.33</v>
       </c>
       <c r="C13" t="n">
-        <v>290</v>
+        <v>1.41</v>
       </c>
       <c r="D13" t="n">
-        <v>6.72</v>
+        <v>6.02</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>MARCO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19.42</v>
+        <v>27.85</v>
       </c>
       <c r="C14" t="n">
-        <v>20.7</v>
+        <v>29.5</v>
       </c>
       <c r="D14" t="n">
-        <v>6.59</v>
+        <v>5.92</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PRECOT</t>
+          <t>SRHHYPOLTD</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>659.65</v>
+        <v>627.7</v>
       </c>
       <c r="C15" t="n">
-        <v>700</v>
+        <v>664.7</v>
       </c>
       <c r="D15" t="n">
-        <v>6.12</v>
+        <v>5.89</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>14.13</v>
+        <v>0.17</v>
       </c>
       <c r="C16" t="n">
-        <v>14.98</v>
+        <v>0.18</v>
       </c>
       <c r="D16" t="n">
-        <v>6.02</v>
+        <v>5.88</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>FEDDERSHOL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.17</v>
+        <v>61.49</v>
       </c>
       <c r="C17" t="n">
-        <v>0.18</v>
+        <v>65</v>
       </c>
       <c r="D17" t="n">
-        <v>5.88</v>
+        <v>5.71</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>THACKER</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1030</v>
+        <v>17.89</v>
       </c>
       <c r="C18" t="n">
-        <v>1090</v>
+        <v>18.89</v>
       </c>
       <c r="D18" t="n">
-        <v>5.83</v>
+        <v>5.59</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SVGLOBAL</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>147.92</v>
+        <v>31.96</v>
       </c>
       <c r="C19" t="n">
-        <v>156.5</v>
+        <v>33.7</v>
       </c>
       <c r="D19" t="n">
-        <v>5.8</v>
+        <v>5.44</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>521.15</v>
+        <v>0.19</v>
       </c>
       <c r="C20" t="n">
-        <v>551</v>
+        <v>0.2</v>
       </c>
       <c r="D20" t="n">
-        <v>5.73</v>
+        <v>5.26</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LAXMICOT</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12.72</v>
+        <v>26.24</v>
       </c>
       <c r="C21" t="n">
-        <v>13.44</v>
+        <v>27.6</v>
       </c>
       <c r="D21" t="n">
-        <v>5.66</v>
+        <v>5.18</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>ASIANTNE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.18</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C22" t="n">
-        <v>0.19</v>
+        <v>9.67</v>
       </c>
       <c r="D22" t="n">
-        <v>5.56</v>
+        <v>5.11</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>37.2</v>
+        <v>5.31</v>
       </c>
       <c r="C23" t="n">
-        <v>39.2</v>
+        <v>5.58</v>
       </c>
       <c r="D23" t="n">
-        <v>5.38</v>
+        <v>5.08</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.86</v>
+        <v>62.24</v>
       </c>
       <c r="C24" t="n">
-        <v>1.96</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="D24" t="n">
-        <v>5.38</v>
+        <v>5</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SHIVALIK</t>
+          <t>TIRUPATIFL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>372.1</v>
+        <v>71.06</v>
       </c>
       <c r="C25" t="n">
-        <v>392</v>
+        <v>74.61</v>
       </c>
       <c r="D25" t="n">
-        <v>5.35</v>
+        <v>5</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DHATRE</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4.18</v>
+        <v>57.21</v>
       </c>
       <c r="C26" t="n">
-        <v>4.4</v>
+        <v>60.07</v>
       </c>
       <c r="D26" t="n">
-        <v>5.26</v>
+        <v>5</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>NAMAN</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18.09</v>
+        <v>40</v>
       </c>
       <c r="C27" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="D27" t="n">
-        <v>5.03</v>
+        <v>5</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,14 +1033,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>ESDS</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>336.1</v>
+        <v>1642.75</v>
       </c>
       <c r="C28" t="n">
-        <v>352.9</v>
+        <v>1724.85</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
@@ -1055,14 +1055,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>KILITCH</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>401.59</v>
+        <v>201.02</v>
       </c>
       <c r="C29" t="n">
-        <v>421.66</v>
+        <v>211.07</v>
       </c>
       <c r="D29" t="n">
         <v>5</v>
@@ -1077,14 +1077,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>STALLION</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>220.49</v>
+        <v>0.8</v>
       </c>
       <c r="C30" t="n">
-        <v>231.51</v>
+        <v>0.84</v>
       </c>
       <c r="D30" t="n">
         <v>5</v>
@@ -1099,14 +1099,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SHREEDHAR</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>161</v>
+        <v>950.4</v>
       </c>
       <c r="C31" t="n">
-        <v>169.05</v>
+        <v>997.9</v>
       </c>
       <c r="D31" t="n">
         <v>5</v>
@@ -1121,14 +1121,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CTE</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>40.7</v>
+        <v>352.9</v>
       </c>
       <c r="C32" t="n">
-        <v>42.73</v>
+        <v>370.5</v>
       </c>
       <c r="D32" t="n">
         <v>4.99</v>
@@ -1143,14 +1143,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>DEEP</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>25.44</v>
+        <v>46.28</v>
       </c>
       <c r="C33" t="n">
-        <v>26.71</v>
+        <v>48.59</v>
       </c>
       <c r="D33" t="n">
         <v>4.99</v>
@@ -1165,14 +1165,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>APEXECO</t>
+          <t>SILKFLEX</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>262.5</v>
+        <v>294.35</v>
       </c>
       <c r="C34" t="n">
-        <v>275.6</v>
+        <v>309.05</v>
       </c>
       <c r="D34" t="n">
         <v>4.99</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>54.49</v>
+        <v>50.2</v>
       </c>
       <c r="C35" t="n">
-        <v>57.21</v>
+        <v>52.7</v>
       </c>
       <c r="D35" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>44.33</v>
+        <v>26.71</v>
       </c>
       <c r="C36" t="n">
-        <v>46.54</v>
+        <v>28.04</v>
       </c>
       <c r="D36" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>303.4</v>
+        <v>202.75</v>
       </c>
       <c r="C37" t="n">
-        <v>318.55</v>
+        <v>212.85</v>
       </c>
       <c r="D37" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TIRUPATIFL</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>67.68000000000001</v>
+        <v>22.55</v>
       </c>
       <c r="C38" t="n">
-        <v>71.06</v>
+        <v>23.67</v>
       </c>
       <c r="D38" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>APOORVA</t>
+          <t>GCHOTELS</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>31.05</v>
+        <v>120.8</v>
       </c>
       <c r="C39" t="n">
-        <v>32.6</v>
+        <v>126.8</v>
       </c>
       <c r="D39" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AKANKSHA</t>
+          <t>RFBL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>139.65</v>
+        <v>88.5</v>
       </c>
       <c r="C40" t="n">
-        <v>146.6</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="D40" t="n">
-        <v>4.98</v>
+        <v>4.97</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>SUPTANERY</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>42.95</v>
+        <v>9.67</v>
       </c>
       <c r="C41" t="n">
-        <v>45.09</v>
+        <v>10.15</v>
       </c>
       <c r="D41" t="n">
-        <v>4.98</v>
+        <v>4.96</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>DCXINDIA</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>25.2</v>
+        <v>162.02</v>
       </c>
       <c r="C42" t="n">
-        <v>26.45</v>
+        <v>170</v>
       </c>
       <c r="D42" t="n">
-        <v>4.96</v>
+        <v>4.93</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AMEYA</t>
+          <t>LEENEE</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>142.55</v>
+        <v>7.5</v>
       </c>
       <c r="C43" t="n">
-        <v>149.6</v>
+        <v>7.87</v>
       </c>
       <c r="D43" t="n">
-        <v>4.95</v>
+        <v>4.93</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3.44</v>
+        <v>17.94</v>
       </c>
       <c r="C44" t="n">
-        <v>3.61</v>
+        <v>18.82</v>
       </c>
       <c r="D44" t="n">
-        <v>4.94</v>
+        <v>4.91</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BGLOBAL</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3.05</v>
+        <v>26.45</v>
       </c>
       <c r="C45" t="n">
-        <v>3.2</v>
+        <v>27.75</v>
       </c>
       <c r="D45" t="n">
-        <v>4.92</v>
+        <v>4.91</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,14 +1429,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>ICDSLTD</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>70.02</v>
+        <v>58.96</v>
       </c>
       <c r="C46" t="n">
-        <v>73.45</v>
+        <v>61.85</v>
       </c>
       <c r="D46" t="n">
         <v>4.9</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>REFRACTORY</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>31.65</v>
+        <v>4.4</v>
       </c>
       <c r="C47" t="n">
-        <v>33.2</v>
+        <v>4.61</v>
       </c>
       <c r="D47" t="n">
-        <v>4.9</v>
+        <v>4.77</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>NEELAM</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1287</v>
+        <v>7.35</v>
       </c>
       <c r="C48" t="n">
-        <v>1350</v>
+        <v>7.7</v>
       </c>
       <c r="D48" t="n">
-        <v>4.9</v>
+        <v>4.76</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>TAMBOLIIN</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>22.29</v>
+        <v>292.2</v>
       </c>
       <c r="C49" t="n">
-        <v>23.38</v>
+        <v>305.9</v>
       </c>
       <c r="D49" t="n">
-        <v>4.89</v>
+        <v>4.69</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>FELDVR</t>
+          <t>TANAA</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.05</v>
+        <v>319.6</v>
       </c>
       <c r="C50" t="n">
-        <v>2.15</v>
+        <v>334.5</v>
       </c>
       <c r="D50" t="n">
-        <v>4.88</v>
+        <v>4.66</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>VIJSOLX</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>334.75</v>
+        <v>634.95</v>
       </c>
       <c r="C51" t="n">
-        <v>351.05</v>
+        <v>664.4</v>
       </c>
       <c r="D51" t="n">
-        <v>4.87</v>
+        <v>4.64</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>GSTL</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>273.7</v>
+        <v>11.9</v>
       </c>
       <c r="C52" t="n">
-        <v>286.95</v>
+        <v>12.45</v>
       </c>
       <c r="D52" t="n">
-        <v>4.84</v>
+        <v>4.62</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KLL</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>32.4</v>
+        <v>6.41</v>
       </c>
       <c r="C53" t="n">
-        <v>33.95</v>
+        <v>6.7</v>
       </c>
       <c r="D53" t="n">
-        <v>4.78</v>
+        <v>4.52</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CONSOFINVT</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>302.2</v>
+        <v>27.44</v>
       </c>
       <c r="C54" t="n">
-        <v>316.6</v>
+        <v>28.68</v>
       </c>
       <c r="D54" t="n">
-        <v>4.77</v>
+        <v>4.52</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4.2</v>
+        <v>4297</v>
       </c>
       <c r="C55" t="n">
-        <v>4.4</v>
+        <v>4489.9</v>
       </c>
       <c r="D55" t="n">
-        <v>4.76</v>
+        <v>4.49</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SADHNANIQ</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2.75</v>
+        <v>4.02</v>
       </c>
       <c r="C56" t="n">
-        <v>2.88</v>
+        <v>4.2</v>
       </c>
       <c r="D56" t="n">
-        <v>4.73</v>
+        <v>4.48</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1.69</v>
+        <v>7.13</v>
       </c>
       <c r="C57" t="n">
-        <v>1.77</v>
+        <v>7.44</v>
       </c>
       <c r="D57" t="n">
-        <v>4.73</v>
+        <v>4.35</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>KALANA</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>18.5</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="C58" t="n">
-        <v>19.35</v>
+        <v>98</v>
       </c>
       <c r="D58" t="n">
-        <v>4.59</v>
+        <v>4.27</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GLOBALE</t>
+          <t>NIMBSPROJ</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>11</v>
+        <v>186.85</v>
       </c>
       <c r="C59" t="n">
-        <v>11.5</v>
+        <v>194.8</v>
       </c>
       <c r="D59" t="n">
-        <v>4.55</v>
+        <v>4.25</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ORIENTLTD</t>
+          <t>BIL</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>80.81999999999999</v>
+        <v>1044.35</v>
       </c>
       <c r="C60" t="n">
-        <v>84.5</v>
+        <v>1088</v>
       </c>
       <c r="D60" t="n">
-        <v>4.55</v>
+        <v>4.18</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>7.48</v>
+        <v>0.48</v>
       </c>
       <c r="C61" t="n">
-        <v>7.82</v>
+        <v>0.5</v>
       </c>
       <c r="D61" t="n">
-        <v>4.55</v>
+        <v>4.17</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2.43</v>
+        <v>60.28</v>
       </c>
       <c r="C62" t="n">
-        <v>2.54</v>
+        <v>62.78</v>
       </c>
       <c r="D62" t="n">
-        <v>4.53</v>
+        <v>4.15</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CARBORUNIV</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1124.4</v>
+        <v>10.03</v>
       </c>
       <c r="C63" t="n">
-        <v>1175</v>
+        <v>10.44</v>
       </c>
       <c r="D63" t="n">
-        <v>4.5</v>
+        <v>4.09</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2.24</v>
+        <v>42.08</v>
       </c>
       <c r="C64" t="n">
-        <v>2.34</v>
+        <v>43.8</v>
       </c>
       <c r="D64" t="n">
-        <v>4.46</v>
+        <v>4.09</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CRAVATEX</t>
+          <t>DHRUV</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>324.55</v>
+        <v>20.95</v>
       </c>
       <c r="C65" t="n">
-        <v>338.95</v>
+        <v>21.79</v>
       </c>
       <c r="D65" t="n">
-        <v>4.44</v>
+        <v>4.01</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>JPPOWER</t>
+          <t>ABH</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>15.37</v>
+        <v>48.1</v>
       </c>
       <c r="C66" t="n">
-        <v>16.05</v>
+        <v>50</v>
       </c>
       <c r="D66" t="n">
-        <v>4.42</v>
+        <v>3.95</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>10.47</v>
+        <v>24.04</v>
       </c>
       <c r="C67" t="n">
-        <v>10.93</v>
+        <v>24.99</v>
       </c>
       <c r="D67" t="n">
-        <v>4.39</v>
+        <v>3.95</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>4.39</v>
+        <v>0.76</v>
       </c>
       <c r="C68" t="n">
-        <v>4.58</v>
+        <v>0.79</v>
       </c>
       <c r="D68" t="n">
-        <v>4.33</v>
+        <v>3.95</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LKPSEC</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>15.01</v>
+        <v>21.47</v>
       </c>
       <c r="C69" t="n">
-        <v>15.66</v>
+        <v>22.3</v>
       </c>
       <c r="D69" t="n">
-        <v>4.33</v>
+        <v>3.87</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>TGBHOTELS</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1.16</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="C70" t="n">
-        <v>1.21</v>
+        <v>9.9</v>
       </c>
       <c r="D70" t="n">
-        <v>4.31</v>
+        <v>3.77</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>VITAL</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>177.36</v>
+        <v>54.9</v>
       </c>
       <c r="C71" t="n">
-        <v>185</v>
+        <v>56.9</v>
       </c>
       <c r="D71" t="n">
-        <v>4.31</v>
+        <v>3.64</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SRIKPRIND</t>
+          <t>CONSOFINVT</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>27.98</v>
+        <v>301.8</v>
       </c>
       <c r="C72" t="n">
-        <v>29.18</v>
+        <v>312.75</v>
       </c>
       <c r="D72" t="n">
-        <v>4.29</v>
+        <v>3.63</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>APTECHT</t>
+          <t>EMBDL</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>92.05</v>
+        <v>58.89</v>
       </c>
       <c r="C73" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="D73" t="n">
-        <v>4.29</v>
+        <v>3.58</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>KEYFINSERV</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>21.48</v>
+        <v>241.45</v>
       </c>
       <c r="C74" t="n">
-        <v>22.4</v>
+        <v>250</v>
       </c>
       <c r="D74" t="n">
-        <v>4.28</v>
+        <v>3.54</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>11.57</v>
+        <v>108.19</v>
       </c>
       <c r="C75" t="n">
-        <v>12.06</v>
+        <v>112</v>
       </c>
       <c r="D75" t="n">
-        <v>4.24</v>
+        <v>3.52</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>UCAL</t>
+          <t>ADISOFT</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>138.15</v>
+        <v>252.3</v>
       </c>
       <c r="C76" t="n">
-        <v>144</v>
+        <v>261.1</v>
       </c>
       <c r="D76" t="n">
-        <v>4.23</v>
+        <v>3.49</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>KHAITANLTD</t>
+          <t>NDGL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>152.13</v>
+        <v>2580.6</v>
       </c>
       <c r="C77" t="n">
-        <v>158.5</v>
+        <v>2670</v>
       </c>
       <c r="D77" t="n">
-        <v>4.19</v>
+        <v>3.46</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.48</v>
+        <v>0.87</v>
       </c>
       <c r="C78" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="D78" t="n">
-        <v>4.17</v>
+        <v>3.45</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>61.06</v>
+        <v>16.44</v>
       </c>
       <c r="C79" t="n">
-        <v>63.6</v>
+        <v>17</v>
       </c>
       <c r="D79" t="n">
-        <v>4.16</v>
+        <v>3.41</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>PHOENXINTL</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.73</v>
+        <v>27.95</v>
       </c>
       <c r="C80" t="n">
-        <v>0.76</v>
+        <v>28.9</v>
       </c>
       <c r="D80" t="n">
-        <v>4.11</v>
+        <v>3.4</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>107.62</v>
+        <v>13.35</v>
       </c>
       <c r="C81" t="n">
-        <v>112</v>
+        <v>13.79</v>
       </c>
       <c r="D81" t="n">
-        <v>4.07</v>
+        <v>3.3</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MLKFOOD</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>79.81999999999999</v>
+        <v>6.09</v>
       </c>
       <c r="C82" t="n">
-        <v>83</v>
+        <v>6.29</v>
       </c>
       <c r="D82" t="n">
-        <v>3.98</v>
+        <v>3.28</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>2.78</v>
+        <v>2.45</v>
       </c>
       <c r="C83" t="n">
-        <v>2.89</v>
+        <v>2.53</v>
       </c>
       <c r="D83" t="n">
-        <v>3.96</v>
+        <v>3.27</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>PRAKASHSTL</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>46.47</v>
+        <v>3.69</v>
       </c>
       <c r="C84" t="n">
-        <v>48.3</v>
+        <v>3.81</v>
       </c>
       <c r="D84" t="n">
-        <v>3.94</v>
+        <v>3.25</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>6.11</v>
+        <v>13.24</v>
       </c>
       <c r="C85" t="n">
-        <v>6.35</v>
+        <v>13.67</v>
       </c>
       <c r="D85" t="n">
-        <v>3.93</v>
+        <v>3.25</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>SWSOLAR</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.77</v>
+        <v>173.27</v>
       </c>
       <c r="C86" t="n">
-        <v>0.8</v>
+        <v>178.89</v>
       </c>
       <c r="D86" t="n">
-        <v>3.9</v>
+        <v>3.24</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>VGCL</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>48.42</v>
+        <v>69.45</v>
       </c>
       <c r="C87" t="n">
-        <v>50.29</v>
+        <v>71.7</v>
       </c>
       <c r="D87" t="n">
-        <v>3.86</v>
+        <v>3.24</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>NAGREEKCAP</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>2.07</v>
+        <v>29.06</v>
       </c>
       <c r="C88" t="n">
-        <v>2.15</v>
+        <v>30</v>
       </c>
       <c r="D88" t="n">
-        <v>3.86</v>
+        <v>3.23</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>7.8</v>
+        <v>10.82</v>
       </c>
       <c r="C89" t="n">
-        <v>8.1</v>
+        <v>11.17</v>
       </c>
       <c r="D89" t="n">
-        <v>3.85</v>
+        <v>3.23</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>DAICHI</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>38.04</v>
+        <v>319.7</v>
       </c>
       <c r="C90" t="n">
-        <v>39.5</v>
+        <v>330</v>
       </c>
       <c r="D90" t="n">
-        <v>3.84</v>
+        <v>3.22</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>30.09</v>
+        <v>1.88</v>
       </c>
       <c r="C91" t="n">
-        <v>31.23</v>
+        <v>1.94</v>
       </c>
       <c r="D91" t="n">
-        <v>3.79</v>
+        <v>3.19</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>SHRADHA</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>5.06</v>
+        <v>29.99</v>
       </c>
       <c r="C92" t="n">
-        <v>5.25</v>
+        <v>30.94</v>
       </c>
       <c r="D92" t="n">
-        <v>3.75</v>
+        <v>3.17</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>GENCON</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>40.01</v>
+        <v>46.54</v>
       </c>
       <c r="C93" t="n">
-        <v>41.5</v>
+        <v>48</v>
       </c>
       <c r="D93" t="n">
-        <v>3.72</v>
+        <v>3.14</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>271.85</v>
+        <v>12.79</v>
       </c>
       <c r="C94" t="n">
-        <v>281.95</v>
+        <v>13.19</v>
       </c>
       <c r="D94" t="n">
-        <v>3.72</v>
+        <v>3.13</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>2660.1</v>
+        <v>5.12</v>
       </c>
       <c r="C95" t="n">
-        <v>2758</v>
+        <v>5.28</v>
       </c>
       <c r="D95" t="n">
-        <v>3.68</v>
+        <v>3.13</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PAVNAIND</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>15.67</v>
+        <v>2.25</v>
       </c>
       <c r="C96" t="n">
-        <v>16.24</v>
+        <v>2.32</v>
       </c>
       <c r="D96" t="n">
-        <v>3.64</v>
+        <v>3.11</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>KMEW</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>2885.6</v>
+        <v>5.48</v>
       </c>
       <c r="C97" t="n">
-        <v>2990</v>
+        <v>5.65</v>
       </c>
       <c r="D97" t="n">
-        <v>3.62</v>
+        <v>3.1</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>XTRANET</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.28</v>
+        <v>341.43</v>
       </c>
       <c r="C98" t="n">
-        <v>0.29</v>
+        <v>352</v>
       </c>
       <c r="D98" t="n">
-        <v>3.57</v>
+        <v>3.1</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>BOROSCI</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>22.21</v>
+        <v>119.11</v>
       </c>
       <c r="C99" t="n">
-        <v>23</v>
+        <v>122.75</v>
       </c>
       <c r="D99" t="n">
-        <v>3.56</v>
+        <v>3.06</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>GLASSWALL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>40.56</v>
+        <v>295.21</v>
       </c>
       <c r="C100" t="n">
-        <v>42</v>
+        <v>304.15</v>
       </c>
       <c r="D100" t="n">
-        <v>3.55</v>
+        <v>3.03</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PRADPME</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>453.5</v>
+        <v>34.94</v>
       </c>
       <c r="C101" t="n">
-        <v>469.5</v>
+        <v>35.99</v>
       </c>
       <c r="D101" t="n">
-        <v>3.53</v>
+        <v>3.01</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>WEIZMANIND</t>
+          <t>RAMASTEEL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>71.48</v>
+        <v>4.38</v>
       </c>
       <c r="C102" t="n">
-        <v>74</v>
+        <v>4.51</v>
       </c>
       <c r="D102" t="n">
-        <v>3.53</v>
+        <v>2.97</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>3.13</v>
+        <v>5.72</v>
       </c>
       <c r="C103" t="n">
-        <v>3.24</v>
+        <v>5.89</v>
       </c>
       <c r="D103" t="n">
-        <v>3.51</v>
+        <v>2.97</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>7.99</v>
+        <v>49.54</v>
       </c>
       <c r="C104" t="n">
-        <v>8.27</v>
+        <v>50.99</v>
       </c>
       <c r="D104" t="n">
-        <v>3.5</v>
+        <v>2.93</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>14</v>
+        <v>3191.5</v>
       </c>
       <c r="C105" t="n">
-        <v>14.49</v>
+        <v>3285</v>
       </c>
       <c r="D105" t="n">
-        <v>3.5</v>
+        <v>2.93</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>MAHAPEXLTD</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>33.56</v>
+        <v>54.36</v>
       </c>
       <c r="C106" t="n">
-        <v>34.73</v>
+        <v>55.95</v>
       </c>
       <c r="D106" t="n">
-        <v>3.49</v>
+        <v>2.92</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>KARMAENG</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>41.27</v>
+        <v>7.91</v>
       </c>
       <c r="C107" t="n">
-        <v>42.7</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="D107" t="n">
-        <v>3.46</v>
+        <v>2.91</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>GCHOTELS</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>115.05</v>
+        <v>38.34</v>
       </c>
       <c r="C108" t="n">
-        <v>119</v>
+        <v>39.45</v>
       </c>
       <c r="D108" t="n">
-        <v>3.43</v>
+        <v>2.9</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>4.09</v>
+        <v>36.93</v>
       </c>
       <c r="C109" t="n">
-        <v>4.23</v>
+        <v>37.99</v>
       </c>
       <c r="D109" t="n">
-        <v>3.42</v>
+        <v>2.87</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>TREJHARA</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>8.789999999999999</v>
+        <v>132.25</v>
       </c>
       <c r="C110" t="n">
-        <v>9.09</v>
+        <v>136</v>
       </c>
       <c r="D110" t="n">
-        <v>3.41</v>
+        <v>2.84</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>JMA</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>17.06</v>
+        <v>88.3</v>
       </c>
       <c r="C111" t="n">
-        <v>17.64</v>
+        <v>90.79000000000001</v>
       </c>
       <c r="D111" t="n">
-        <v>3.4</v>
+        <v>2.82</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>KOTHARIPRO</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>8.6</v>
+        <v>63.23</v>
       </c>
       <c r="C112" t="n">
-        <v>8.890000000000001</v>
+        <v>65</v>
       </c>
       <c r="D112" t="n">
-        <v>3.37</v>
+        <v>2.8</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>VETO</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>139.15</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="C113" t="n">
-        <v>143.8</v>
+        <v>8.85</v>
       </c>
       <c r="D113" t="n">
-        <v>3.34</v>
+        <v>2.79</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>HINDALUMI</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>94.27</v>
+        <v>150.81</v>
       </c>
       <c r="C114" t="n">
-        <v>97.40000000000001</v>
+        <v>155</v>
       </c>
       <c r="D114" t="n">
-        <v>3.32</v>
+        <v>2.78</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>VRAJ</t>
+          <t>PRECOT</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>127.74</v>
+        <v>689.85</v>
       </c>
       <c r="C115" t="n">
-        <v>131.94</v>
+        <v>709</v>
       </c>
       <c r="D115" t="n">
-        <v>3.29</v>
+        <v>2.78</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>525.7</v>
+        <v>26.95</v>
       </c>
       <c r="C116" t="n">
-        <v>543</v>
+        <v>27.7</v>
       </c>
       <c r="D116" t="n">
-        <v>3.29</v>
+        <v>2.78</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>SHALPAINTS</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>32.45</v>
+        <v>80.16</v>
       </c>
       <c r="C117" t="n">
-        <v>33.5</v>
+        <v>82.36</v>
       </c>
       <c r="D117" t="n">
-        <v>3.24</v>
+        <v>2.74</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>CTE</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>126.31</v>
+        <v>42.73</v>
       </c>
       <c r="C118" t="n">
-        <v>130.38</v>
+        <v>43.89</v>
       </c>
       <c r="D118" t="n">
-        <v>3.22</v>
+        <v>2.71</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SAPPL</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>276.15</v>
+        <v>3.35</v>
       </c>
       <c r="C119" t="n">
-        <v>285</v>
+        <v>3.44</v>
       </c>
       <c r="D119" t="n">
-        <v>3.2</v>
+        <v>2.69</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>6.01</v>
+        <v>521</v>
       </c>
       <c r="C120" t="n">
-        <v>6.2</v>
+        <v>535</v>
       </c>
       <c r="D120" t="n">
-        <v>3.16</v>
+        <v>2.69</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>KMCSHIL</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>150.26</v>
+        <v>6.77</v>
       </c>
       <c r="C121" t="n">
-        <v>155</v>
+        <v>6.95</v>
       </c>
       <c r="D121" t="n">
-        <v>3.15</v>
+        <v>2.66</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SHRADHA</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>30</v>
+        <v>28.69</v>
       </c>
       <c r="C122" t="n">
-        <v>30.94</v>
+        <v>29.45</v>
       </c>
       <c r="D122" t="n">
-        <v>3.13</v>
+        <v>2.65</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>39.48</v>
+        <v>24.21</v>
       </c>
       <c r="C123" t="n">
-        <v>40.7</v>
+        <v>24.85</v>
       </c>
       <c r="D123" t="n">
-        <v>3.09</v>
+        <v>2.64</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AURUS</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>4.87</v>
+        <v>0.76</v>
       </c>
       <c r="C124" t="n">
-        <v>5.02</v>
+        <v>0.78</v>
       </c>
       <c r="D124" t="n">
-        <v>3.08</v>
+        <v>2.63</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LAMBODHARA</t>
+          <t>LCCPROJECT</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>120.21</v>
+        <v>141.33</v>
       </c>
       <c r="C125" t="n">
-        <v>123.9</v>
+        <v>145</v>
       </c>
       <c r="D125" t="n">
-        <v>3.07</v>
+        <v>2.6</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>LKPSEC</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>193.1</v>
+        <v>15.06</v>
       </c>
       <c r="C126" t="n">
-        <v>199</v>
+        <v>15.45</v>
       </c>
       <c r="D126" t="n">
-        <v>3.06</v>
+        <v>2.59</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>KONSTELEC</t>
+          <t>KLL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>59.05</v>
+        <v>36.8</v>
       </c>
       <c r="C127" t="n">
-        <v>60.85</v>
+        <v>37.75</v>
       </c>
       <c r="D127" t="n">
-        <v>3.05</v>
+        <v>2.58</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MOTOGENFIN</t>
+          <t>STEAMHOUSE</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>26.19</v>
+        <v>105.05</v>
       </c>
       <c r="C128" t="n">
-        <v>26.99</v>
+        <v>107.75</v>
       </c>
       <c r="D128" t="n">
-        <v>3.05</v>
+        <v>2.57</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MODINATUR</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>359.05</v>
+        <v>633.7</v>
       </c>
       <c r="C129" t="n">
-        <v>370</v>
+        <v>650</v>
       </c>
       <c r="D129" t="n">
-        <v>3.05</v>
+        <v>2.57</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>2.96</v>
+        <v>185.25</v>
       </c>
       <c r="C130" t="n">
-        <v>3.05</v>
+        <v>190</v>
       </c>
       <c r="D130" t="n">
-        <v>3.04</v>
+        <v>2.56</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>LAHOTIOV</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>39.26</v>
+        <v>1725.8</v>
       </c>
       <c r="C131" t="n">
-        <v>40.45</v>
+        <v>1770</v>
       </c>
       <c r="D131" t="n">
-        <v>3.03</v>
+        <v>2.56</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>RKSWAMY</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>33.15</v>
+        <v>88.79000000000001</v>
       </c>
       <c r="C132" t="n">
-        <v>34.14</v>
+        <v>91.05</v>
       </c>
       <c r="D132" t="n">
-        <v>2.99</v>
+        <v>2.55</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SUNLITE</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>644.9</v>
+        <v>477.7</v>
       </c>
       <c r="C133" t="n">
-        <v>663.95</v>
+        <v>489.9</v>
       </c>
       <c r="D133" t="n">
-        <v>2.95</v>
+        <v>2.55</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>HAZOOR</t>
+          <t>PANORAMA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>19.3</v>
+        <v>54.89</v>
       </c>
       <c r="C134" t="n">
-        <v>19.86</v>
+        <v>56.29</v>
       </c>
       <c r="D134" t="n">
-        <v>2.9</v>
+        <v>2.55</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LEAPIND</t>
+          <t>LINC</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>140.47</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="C135" t="n">
-        <v>144.52</v>
+        <v>93.89</v>
       </c>
       <c r="D135" t="n">
-        <v>2.88</v>
+        <v>2.53</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>MIRZAINT</t>
+          <t>PRADPME</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>29.14</v>
+        <v>475.1</v>
       </c>
       <c r="C136" t="n">
-        <v>29.98</v>
+        <v>487</v>
       </c>
       <c r="D136" t="n">
-        <v>2.88</v>
+        <v>2.5</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>SERVICE</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>69.98999999999999</v>
+        <v>66.05</v>
       </c>
       <c r="C137" t="n">
-        <v>72</v>
+        <v>67.7</v>
       </c>
       <c r="D137" t="n">
-        <v>2.87</v>
+        <v>2.5</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>HEG</t>
+          <t>WARDINMOBI</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>237.05</v>
+        <v>5.61</v>
       </c>
       <c r="C138" t="n">
-        <v>243.85</v>
+        <v>5.75</v>
       </c>
       <c r="D138" t="n">
-        <v>2.87</v>
+        <v>2.5</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ABH</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>43.75</v>
+        <v>2.01</v>
       </c>
       <c r="C139" t="n">
-        <v>45</v>
+        <v>2.06</v>
       </c>
       <c r="D139" t="n">
-        <v>2.86</v>
+        <v>2.49</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>35</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="C140" t="n">
-        <v>36</v>
+        <v>9.09</v>
       </c>
       <c r="D140" t="n">
-        <v>2.86</v>
+        <v>2.48</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>PRESSTONIC</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>29.95</v>
+        <v>171.75</v>
       </c>
       <c r="C141" t="n">
-        <v>30.8</v>
+        <v>176</v>
       </c>
       <c r="D141" t="n">
-        <v>2.84</v>
+        <v>2.47</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ONIDA</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>32.89</v>
+        <v>0.41</v>
       </c>
       <c r="C142" t="n">
-        <v>33.82</v>
+        <v>0.42</v>
       </c>
       <c r="D142" t="n">
-        <v>2.83</v>
+        <v>2.44</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>6.71</v>
+        <v>230.26</v>
       </c>
       <c r="C143" t="n">
-        <v>6.9</v>
+        <v>235.8</v>
       </c>
       <c r="D143" t="n">
-        <v>2.83</v>
+        <v>2.41</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>VITAL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>55.4</v>
+        <v>414.7</v>
       </c>
       <c r="C144" t="n">
-        <v>56.95</v>
+        <v>424.7</v>
       </c>
       <c r="D144" t="n">
-        <v>2.8</v>
+        <v>2.41</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CONCORDBIO</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1494.4</v>
+        <v>198.29</v>
       </c>
       <c r="C145" t="n">
-        <v>1536</v>
+        <v>202.99</v>
       </c>
       <c r="D145" t="n">
-        <v>2.78</v>
+        <v>2.37</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>CRSL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>13.72</v>
+        <v>2.53</v>
       </c>
       <c r="C146" t="n">
-        <v>14.1</v>
+        <v>2.59</v>
       </c>
       <c r="D146" t="n">
-        <v>2.77</v>
+        <v>2.37</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>BEEKAY</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>430.05</v>
+        <v>4.22</v>
       </c>
       <c r="C147" t="n">
-        <v>441.9</v>
+        <v>4.32</v>
       </c>
       <c r="D147" t="n">
-        <v>2.76</v>
+        <v>2.37</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>446.7</v>
+        <v>1.7</v>
       </c>
       <c r="C148" t="n">
-        <v>458.9</v>
+        <v>1.74</v>
       </c>
       <c r="D148" t="n">
-        <v>2.73</v>
+        <v>2.35</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>MANORG</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>172.31</v>
+        <v>464.15</v>
       </c>
       <c r="C149" t="n">
-        <v>177</v>
+        <v>475</v>
       </c>
       <c r="D149" t="n">
-        <v>2.72</v>
+        <v>2.34</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>AGIIL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>13.63</v>
+        <v>271.15</v>
       </c>
       <c r="C150" t="n">
-        <v>14</v>
+        <v>277.5</v>
       </c>
       <c r="D150" t="n">
-        <v>2.71</v>
+        <v>2.34</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>BIL</t>
+          <t>RTSPOWR</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1040.85</v>
+        <v>87.95999999999999</v>
       </c>
       <c r="C151" t="n">
-        <v>1069</v>
+        <v>90</v>
       </c>
       <c r="D151" t="n">
-        <v>2.7</v>
+        <v>2.32</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>WEL</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>72.94</v>
+        <v>168.63</v>
       </c>
       <c r="C152" t="n">
-        <v>74.89</v>
+        <v>172.5</v>
       </c>
       <c r="D152" t="n">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SWARNSAR</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>38.96</v>
+        <v>156.9</v>
       </c>
       <c r="C153" t="n">
-        <v>40</v>
+        <v>160.5</v>
       </c>
       <c r="D153" t="n">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>VISHWARAJ</t>
+          <t>ATAM</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>5.31</v>
+        <v>59.05</v>
       </c>
       <c r="C154" t="n">
-        <v>5.45</v>
+        <v>60.4</v>
       </c>
       <c r="D154" t="n">
-        <v>2.64</v>
+        <v>2.29</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>KAYA</t>
+          <t>VIVOBIOT</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>341</v>
+        <v>16.21</v>
       </c>
       <c r="C155" t="n">
-        <v>350</v>
+        <v>16.58</v>
       </c>
       <c r="D155" t="n">
-        <v>2.64</v>
+        <v>2.28</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>HLEGLAS</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>10.37</v>
+        <v>469.2</v>
       </c>
       <c r="C156" t="n">
-        <v>10.64</v>
+        <v>479.9</v>
       </c>
       <c r="D156" t="n">
-        <v>2.6</v>
+        <v>2.28</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>NILASPACES</t>
+          <t>CHEMFAB</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>12.3</v>
+        <v>359.3</v>
       </c>
       <c r="C157" t="n">
-        <v>12.62</v>
+        <v>367.45</v>
       </c>
       <c r="D157" t="n">
-        <v>2.6</v>
+        <v>2.27</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>ZOTA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1.93</v>
+        <v>1287.8</v>
       </c>
       <c r="C158" t="n">
-        <v>1.98</v>
+        <v>1317</v>
       </c>
       <c r="D158" t="n">
-        <v>2.59</v>
+        <v>2.27</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>INDSWFTLAB</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>61.42</v>
+        <v>379.4</v>
       </c>
       <c r="C159" t="n">
-        <v>63</v>
+        <v>388</v>
       </c>
       <c r="D159" t="n">
-        <v>2.57</v>
+        <v>2.27</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LEENEE</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>7.8</v>
+        <v>14.57</v>
       </c>
       <c r="C160" t="n">
-        <v>8</v>
+        <v>14.9</v>
       </c>
       <c r="D160" t="n">
-        <v>2.56</v>
+        <v>2.26</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>ANNAPURNA</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>23.64</v>
+        <v>130.56</v>
       </c>
       <c r="C161" t="n">
-        <v>24.24</v>
+        <v>133.5</v>
       </c>
       <c r="D161" t="n">
-        <v>2.54</v>
+        <v>2.25</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>7.12</v>
+        <v>29.44</v>
       </c>
       <c r="C162" t="n">
-        <v>7.3</v>
+        <v>30.09</v>
       </c>
       <c r="D162" t="n">
-        <v>2.53</v>
+        <v>2.21</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>INDOAMIN</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>20.8</v>
+        <v>132.87</v>
       </c>
       <c r="C163" t="n">
-        <v>21.32</v>
+        <v>135.8</v>
       </c>
       <c r="D163" t="n">
-        <v>2.5</v>
+        <v>2.21</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MITCON</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>80.01000000000001</v>
+        <v>5.97</v>
       </c>
       <c r="C164" t="n">
-        <v>82</v>
+        <v>6.1</v>
       </c>
       <c r="D164" t="n">
-        <v>2.49</v>
+        <v>2.18</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>152.26</v>
+        <v>202.63</v>
       </c>
       <c r="C165" t="n">
-        <v>156.05</v>
+        <v>207</v>
       </c>
       <c r="D165" t="n">
-        <v>2.49</v>
+        <v>2.16</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>66.15000000000001</v>
+        <v>2.78</v>
       </c>
       <c r="C166" t="n">
-        <v>67.8</v>
+        <v>2.84</v>
       </c>
       <c r="D166" t="n">
-        <v>2.49</v>
+        <v>2.16</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4095,13 +4095,13 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>43.92</v>
+        <v>43.37</v>
       </c>
       <c r="C167" t="n">
-        <v>45</v>
+        <v>44.3</v>
       </c>
       <c r="D167" t="n">
-        <v>2.46</v>
+        <v>2.14</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>AMBICAAGAR</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>24.89</v>
+        <v>1032.9</v>
       </c>
       <c r="C168" t="n">
-        <v>25.5</v>
+        <v>1055</v>
       </c>
       <c r="D168" t="n">
-        <v>2.45</v>
+        <v>2.14</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>207.35</v>
+        <v>2.37</v>
       </c>
       <c r="C169" t="n">
-        <v>212.4</v>
+        <v>2.42</v>
       </c>
       <c r="D169" t="n">
-        <v>2.44</v>
+        <v>2.11</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>54.57</v>
+        <v>577.8</v>
       </c>
       <c r="C170" t="n">
-        <v>55.9</v>
+        <v>590</v>
       </c>
       <c r="D170" t="n">
-        <v>2.44</v>
+        <v>2.11</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>ESSARSHPNG</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>2.06</v>
+        <v>16.15</v>
       </c>
       <c r="C171" t="n">
+        <v>16.49</v>
+      </c>
+      <c r="D171" t="n">
         <v>2.11</v>
-      </c>
-      <c r="D171" t="n">
-        <v>2.43</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>ABHAPOWER</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>24.65</v>
+        <v>160.92</v>
       </c>
       <c r="C172" t="n">
-        <v>25.25</v>
+        <v>164.3</v>
       </c>
       <c r="D172" t="n">
-        <v>2.43</v>
+        <v>2.1</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NACLIND</t>
+          <t>POWERICA</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>146.75</v>
+        <v>568.1</v>
       </c>
       <c r="C173" t="n">
-        <v>150.3</v>
+        <v>579.95</v>
       </c>
       <c r="D173" t="n">
-        <v>2.42</v>
+        <v>2.09</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ABCOTS</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>209.85</v>
+        <v>128.32</v>
       </c>
       <c r="C174" t="n">
-        <v>214.9</v>
+        <v>131</v>
       </c>
       <c r="D174" t="n">
-        <v>2.41</v>
+        <v>2.09</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0.83</v>
+        <v>6.21</v>
       </c>
       <c r="C175" t="n">
-        <v>0.85</v>
+        <v>6.34</v>
       </c>
       <c r="D175" t="n">
-        <v>2.41</v>
+        <v>2.09</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>HINDADH</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>123</v>
+        <v>383.9</v>
       </c>
       <c r="C176" t="n">
-        <v>125.95</v>
+        <v>391.9</v>
       </c>
       <c r="D176" t="n">
-        <v>2.4</v>
+        <v>2.08</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>VIRINCHI</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>7.07</v>
+        <v>13.98</v>
       </c>
       <c r="C177" t="n">
-        <v>7.24</v>
+        <v>14.27</v>
       </c>
       <c r="D177" t="n">
-        <v>2.4</v>
+        <v>2.07</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>APEX</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>147.57</v>
+        <v>351.65</v>
       </c>
       <c r="C178" t="n">
-        <v>151.1</v>
+        <v>358.9</v>
       </c>
       <c r="D178" t="n">
-        <v>2.39</v>
+        <v>2.06</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>PARAGMILK</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>2.53</v>
+        <v>272.4</v>
       </c>
       <c r="C179" t="n">
-        <v>2.59</v>
+        <v>278</v>
       </c>
       <c r="D179" t="n">
-        <v>2.37</v>
+        <v>2.06</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>XELPMOC</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>55.65</v>
+        <v>73.88</v>
       </c>
       <c r="C180" t="n">
-        <v>56.97</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="D180" t="n">
-        <v>2.37</v>
+        <v>2.06</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>1104.85</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="C181" t="n">
-        <v>1131</v>
+        <v>8.9</v>
       </c>
       <c r="D181" t="n">
-        <v>2.37</v>
+        <v>2.06</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>AUTOIND</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>61.35</v>
+        <v>83.76000000000001</v>
       </c>
       <c r="C182" t="n">
-        <v>62.8</v>
+        <v>85.48</v>
       </c>
       <c r="D182" t="n">
-        <v>2.36</v>
+        <v>2.05</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>AAATECH</t>
+          <t>ISFT</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>86.95</v>
+        <v>92.09</v>
       </c>
       <c r="C183" t="n">
-        <v>88.98</v>
+        <v>93.98</v>
       </c>
       <c r="D183" t="n">
-        <v>2.33</v>
+        <v>2.05</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>467.1</v>
+        <v>96.02</v>
       </c>
       <c r="C184" t="n">
-        <v>477.95</v>
+        <v>97.98999999999999</v>
       </c>
       <c r="D184" t="n">
-        <v>2.32</v>
+        <v>2.05</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>OSWALGREEN</t>
+          <t>ARIHANT</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>19.44</v>
+        <v>957.35</v>
       </c>
       <c r="C185" t="n">
-        <v>19.89</v>
+        <v>977</v>
       </c>
       <c r="D185" t="n">
-        <v>2.31</v>
+        <v>2.05</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>24.24</v>
+        <v>1371.1</v>
       </c>
       <c r="C186" t="n">
-        <v>24.8</v>
+        <v>1399</v>
       </c>
       <c r="D186" t="n">
-        <v>2.31</v>
+        <v>2.03</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>BSHSL</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>87.87</v>
+        <v>186.22</v>
       </c>
       <c r="C187" t="n">
-        <v>89.90000000000001</v>
+        <v>190</v>
       </c>
       <c r="D187" t="n">
-        <v>2.31</v>
+        <v>2.03</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>INTENTECH</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>78.14</v>
+        <v>15.94</v>
       </c>
       <c r="C188" t="n">
-        <v>79.94</v>
+        <v>16.26</v>
       </c>
       <c r="D188" t="n">
-        <v>2.3</v>
+        <v>2.01</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>145.19</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="C189" t="n">
-        <v>148.5</v>
+        <v>102</v>
       </c>
       <c r="D189" t="n">
-        <v>2.28</v>
+        <v>2.01</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>KECL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>575.1</v>
+        <v>118.43</v>
       </c>
       <c r="C190" t="n">
-        <v>588</v>
+        <v>120.8</v>
       </c>
       <c r="D190" t="n">
-        <v>2.24</v>
+        <v>2</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>CFEL</t>
+          <t>HPAL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>46.95</v>
+        <v>35.93</v>
       </c>
       <c r="C191" t="n">
-        <v>48</v>
+        <v>36.65</v>
       </c>
       <c r="D191" t="n">
-        <v>2.24</v>
+        <v>2</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>DENORA</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>782.25</v>
+        <v>421.66</v>
       </c>
       <c r="C192" t="n">
-        <v>799.65</v>
+        <v>430.09</v>
       </c>
       <c r="D192" t="n">
-        <v>2.22</v>
+        <v>2</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>EASTWEST</t>
+          <t>GHCLTEXTIL</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>2.25</v>
+        <v>129.52</v>
       </c>
       <c r="C193" t="n">
-        <v>2.3</v>
+        <v>132.1</v>
       </c>
       <c r="D193" t="n">
-        <v>2.22</v>
+        <v>1.99</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>SUDARCOLOR</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>4.96</v>
+        <v>402</v>
       </c>
       <c r="C194" t="n">
-        <v>5.07</v>
+        <v>410</v>
       </c>
       <c r="D194" t="n">
-        <v>2.22</v>
+        <v>1.99</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>613.45</v>
+        <v>24.13</v>
       </c>
       <c r="C195" t="n">
-        <v>627</v>
+        <v>24.61</v>
       </c>
       <c r="D195" t="n">
-        <v>2.21</v>
+        <v>1.99</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>GEECEE</t>
+          <t>INOXINDIA</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>371.85</v>
+        <v>2089.2</v>
       </c>
       <c r="C196" t="n">
-        <v>380</v>
+        <v>2130.7</v>
       </c>
       <c r="D196" t="n">
-        <v>2.19</v>
+        <v>1.99</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>316.85</v>
+        <v>39.61</v>
       </c>
       <c r="C197" t="n">
-        <v>323.75</v>
+        <v>40.4</v>
       </c>
       <c r="D197" t="n">
-        <v>2.18</v>
+        <v>1.99</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>SKYWAYS</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>16.13</v>
+        <v>126.03</v>
       </c>
       <c r="C198" t="n">
-        <v>16.48</v>
+        <v>128.54</v>
       </c>
       <c r="D198" t="n">
-        <v>2.17</v>
+        <v>1.99</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ANNU</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>50.46</v>
+        <v>97.17</v>
       </c>
       <c r="C199" t="n">
-        <v>51.55</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="D199" t="n">
-        <v>2.16</v>
+        <v>1.99</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>SGRL</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>19.19</v>
+        <v>720.75</v>
       </c>
       <c r="C200" t="n">
-        <v>19.6</v>
+        <v>735</v>
       </c>
       <c r="D200" t="n">
-        <v>2.14</v>
+        <v>1.98</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>TRITONV</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>82.26000000000001</v>
+        <v>1063.9</v>
       </c>
       <c r="C201" t="n">
-        <v>84.01000000000001</v>
+        <v>1085</v>
       </c>
       <c r="D201" t="n">
-        <v>2.13</v>
+        <v>1.98</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-23 08:50 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TRANSCOR</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24.97</v>
+        <v>104.85</v>
       </c>
       <c r="C2" t="n">
-        <v>29</v>
+        <v>125.82</v>
       </c>
       <c r="D2" t="n">
-        <v>16.14</v>
+        <v>20</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>317.45</v>
+        <v>119.98</v>
       </c>
       <c r="C3" t="n">
-        <v>365</v>
+        <v>143.97</v>
       </c>
       <c r="D3" t="n">
-        <v>14.98</v>
+        <v>19.99</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORIRAIL</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>116.41</v>
+        <v>708.9</v>
       </c>
       <c r="C4" t="n">
-        <v>128.75</v>
+        <v>800</v>
       </c>
       <c r="D4" t="n">
-        <v>10.6</v>
+        <v>12.85</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PRESSTONIC</t>
+          <t>REGENCERAM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35.9</v>
+        <v>33.3</v>
       </c>
       <c r="C5" t="n">
-        <v>39.5</v>
+        <v>36.75</v>
       </c>
       <c r="D5" t="n">
-        <v>10.03</v>
+        <v>10.36</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.9</v>
+        <v>23.16</v>
       </c>
       <c r="C6" t="n">
-        <v>5.39</v>
+        <v>25.4</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>9.67</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>PROSTARM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.05</v>
+        <v>127.84</v>
       </c>
       <c r="C7" t="n">
-        <v>6.65</v>
+        <v>139.4</v>
       </c>
       <c r="D7" t="n">
-        <v>9.92</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ARVEE</t>
+          <t>SCODATUBES</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>208.87</v>
+        <v>128.85</v>
       </c>
       <c r="C8" t="n">
-        <v>224.9</v>
+        <v>139.95</v>
       </c>
       <c r="D8" t="n">
-        <v>7.67</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>ANSALBU</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>177.2</v>
+        <v>90.12</v>
       </c>
       <c r="C9" t="n">
-        <v>190</v>
+        <v>97.75</v>
       </c>
       <c r="D9" t="n">
-        <v>7.22</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9.24</v>
+        <v>6.65</v>
       </c>
       <c r="C10" t="n">
-        <v>9.890000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="D10" t="n">
-        <v>7.03</v>
+        <v>8.27</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>154.86</v>
+        <v>1.46</v>
       </c>
       <c r="C11" t="n">
-        <v>165.5</v>
+        <v>1.57</v>
       </c>
       <c r="D11" t="n">
-        <v>6.87</v>
+        <v>7.53</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RHIM</t>
+          <t>ASIANTNE</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>368</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="C12" t="n">
-        <v>392.6</v>
+        <v>10.08</v>
       </c>
       <c r="D12" t="n">
-        <v>6.68</v>
+        <v>7.46</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>AUSTENG</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.33</v>
+        <v>162.85</v>
       </c>
       <c r="C13" t="n">
-        <v>1.41</v>
+        <v>174.8</v>
       </c>
       <c r="D13" t="n">
-        <v>6.02</v>
+        <v>7.34</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MARCO</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>27.85</v>
+        <v>6.25</v>
       </c>
       <c r="C14" t="n">
-        <v>29.5</v>
+        <v>6.68</v>
       </c>
       <c r="D14" t="n">
-        <v>5.92</v>
+        <v>6.88</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>AVIENCE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>627.7</v>
+        <v>345.85</v>
       </c>
       <c r="C15" t="n">
-        <v>664.7</v>
+        <v>369.5</v>
       </c>
       <c r="D15" t="n">
-        <v>5.89</v>
+        <v>6.84</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>BEWLTD</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.17</v>
+        <v>61.35</v>
       </c>
       <c r="C16" t="n">
-        <v>0.18</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>5.88</v>
+        <v>6.52</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FEDDERSHOL</t>
+          <t>ARVSMART</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>61.49</v>
+        <v>588.2</v>
       </c>
       <c r="C17" t="n">
-        <v>65</v>
+        <v>625</v>
       </c>
       <c r="D17" t="n">
-        <v>5.71</v>
+        <v>6.26</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>OSWALPUMPS</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>17.89</v>
+        <v>273.6</v>
       </c>
       <c r="C18" t="n">
-        <v>18.89</v>
+        <v>290.1</v>
       </c>
       <c r="D18" t="n">
-        <v>5.59</v>
+        <v>6.03</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SUPREME</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>31.96</v>
+        <v>0.17</v>
       </c>
       <c r="C19" t="n">
-        <v>33.7</v>
+        <v>0.18</v>
       </c>
       <c r="D19" t="n">
-        <v>5.44</v>
+        <v>5.88</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>SINTERCOM</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.19</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="C20" t="n">
-        <v>0.2</v>
+        <v>84.98</v>
       </c>
       <c r="D20" t="n">
-        <v>5.26</v>
+        <v>5.58</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>26.24</v>
+        <v>80.5</v>
       </c>
       <c r="C21" t="n">
-        <v>27.6</v>
+        <v>84.89</v>
       </c>
       <c r="D21" t="n">
-        <v>5.18</v>
+        <v>5.45</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ASIANTNE</t>
+          <t>AMJLAND</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>9.199999999999999</v>
+        <v>37.75</v>
       </c>
       <c r="C22" t="n">
-        <v>9.67</v>
+        <v>39.75</v>
       </c>
       <c r="D22" t="n">
-        <v>5.11</v>
+        <v>5.3</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5.31</v>
+        <v>7.02</v>
       </c>
       <c r="C23" t="n">
-        <v>5.58</v>
+        <v>7.39</v>
       </c>
       <c r="D23" t="n">
-        <v>5.08</v>
+        <v>5.27</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>KRITI</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>62.24</v>
+        <v>59.75</v>
       </c>
       <c r="C24" t="n">
-        <v>65.34999999999999</v>
+        <v>62.89</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>5.26</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TIRUPATIFL</t>
+          <t>CLEANMAX</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>71.06</v>
+        <v>1367.5</v>
       </c>
       <c r="C25" t="n">
-        <v>74.61</v>
+        <v>1439</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>5.23</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>57.21</v>
+        <v>5.56</v>
       </c>
       <c r="C26" t="n">
-        <v>60.07</v>
+        <v>5.84</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>5.04</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,14 +1011,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NAMAN</t>
+          <t>AMEYA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>40</v>
+        <v>157.1</v>
       </c>
       <c r="C27" t="n">
-        <v>42</v>
+        <v>164.95</v>
       </c>
       <c r="D27" t="n">
         <v>5</v>
@@ -1033,14 +1033,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ESDS</t>
+          <t>TIRUPATIFL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1642.75</v>
+        <v>74.61</v>
       </c>
       <c r="C28" t="n">
-        <v>1724.85</v>
+        <v>78.34</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
@@ -1059,10 +1059,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>201.02</v>
+        <v>211.07</v>
       </c>
       <c r="C29" t="n">
-        <v>211.07</v>
+        <v>221.62</v>
       </c>
       <c r="D29" t="n">
         <v>5</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.8</v>
+        <v>334.45</v>
       </c>
       <c r="C30" t="n">
-        <v>0.84</v>
+        <v>351.15</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>950.4</v>
+        <v>370.5</v>
       </c>
       <c r="C31" t="n">
-        <v>997.9</v>
+        <v>389</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,14 +1121,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>352.9</v>
+        <v>28.04</v>
       </c>
       <c r="C32" t="n">
-        <v>370.5</v>
+        <v>29.44</v>
       </c>
       <c r="D32" t="n">
         <v>4.99</v>
@@ -1143,14 +1143,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DEEP</t>
+          <t>DEEM</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>46.28</v>
+        <v>45.05</v>
       </c>
       <c r="C33" t="n">
-        <v>48.59</v>
+        <v>47.3</v>
       </c>
       <c r="D33" t="n">
         <v>4.99</v>
@@ -1165,14 +1165,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SILKFLEX</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>294.35</v>
+        <v>72.92</v>
       </c>
       <c r="C34" t="n">
-        <v>309.05</v>
+        <v>76.56</v>
       </c>
       <c r="D34" t="n">
         <v>4.99</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>50.2</v>
+        <v>28.86</v>
       </c>
       <c r="C35" t="n">
-        <v>52.7</v>
+        <v>30.3</v>
       </c>
       <c r="D35" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,14 +1209,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>26.71</v>
+        <v>33.16</v>
       </c>
       <c r="C36" t="n">
-        <v>28.04</v>
+        <v>34.81</v>
       </c>
       <c r="D36" t="n">
         <v>4.98</v>
@@ -1231,14 +1231,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>NEUEON</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>202.75</v>
+        <v>12.44</v>
       </c>
       <c r="C37" t="n">
-        <v>212.85</v>
+        <v>13.06</v>
       </c>
       <c r="D37" t="n">
         <v>4.98</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>22.55</v>
+        <v>44.15</v>
       </c>
       <c r="C38" t="n">
-        <v>23.67</v>
+        <v>46.35</v>
       </c>
       <c r="D38" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GCHOTELS</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>120.8</v>
+        <v>212.85</v>
       </c>
       <c r="C39" t="n">
-        <v>126.8</v>
+        <v>223.45</v>
       </c>
       <c r="D39" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RFBL</t>
+          <t>AUROIMPEX</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>88.5</v>
+        <v>37.15</v>
       </c>
       <c r="C40" t="n">
-        <v>92.90000000000001</v>
+        <v>39</v>
       </c>
       <c r="D40" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SUPTANERY</t>
+          <t>SMARTEN</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>9.67</v>
+        <v>59.3</v>
       </c>
       <c r="C41" t="n">
-        <v>10.15</v>
+        <v>62.25</v>
       </c>
       <c r="D41" t="n">
-        <v>4.96</v>
+        <v>4.97</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DCXINDIA</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>162.02</v>
+        <v>10.53</v>
       </c>
       <c r="C42" t="n">
-        <v>170</v>
+        <v>11.05</v>
       </c>
       <c r="D42" t="n">
-        <v>4.93</v>
+        <v>4.94</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,14 +1363,14 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LEENEE</t>
+          <t>HPTL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7.5</v>
+        <v>446</v>
       </c>
       <c r="C43" t="n">
-        <v>7.87</v>
+        <v>468</v>
       </c>
       <c r="D43" t="n">
         <v>4.93</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>17.94</v>
+        <v>3.66</v>
       </c>
       <c r="C44" t="n">
-        <v>18.82</v>
+        <v>3.84</v>
       </c>
       <c r="D44" t="n">
-        <v>4.91</v>
+        <v>4.92</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>ARCL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>26.45</v>
+        <v>262.06</v>
       </c>
       <c r="C45" t="n">
-        <v>27.75</v>
+        <v>274.95</v>
       </c>
       <c r="D45" t="n">
-        <v>4.91</v>
+        <v>4.92</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,14 +1429,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ICDSLTD</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>58.96</v>
+        <v>997.9</v>
       </c>
       <c r="C46" t="n">
-        <v>61.85</v>
+        <v>1046.8</v>
       </c>
       <c r="D46" t="n">
         <v>4.9</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4.4</v>
+        <v>47.34</v>
       </c>
       <c r="C47" t="n">
-        <v>4.61</v>
+        <v>49.65</v>
       </c>
       <c r="D47" t="n">
-        <v>4.77</v>
+        <v>4.88</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>NEELAM</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7.35</v>
+        <v>27.75</v>
       </c>
       <c r="C48" t="n">
-        <v>7.7</v>
+        <v>29.1</v>
       </c>
       <c r="D48" t="n">
-        <v>4.76</v>
+        <v>4.86</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>292.2</v>
+        <v>23.67</v>
       </c>
       <c r="C49" t="n">
-        <v>305.9</v>
+        <v>24.82</v>
       </c>
       <c r="D49" t="n">
-        <v>4.69</v>
+        <v>4.86</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TANAA</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>319.6</v>
+        <v>52.7</v>
       </c>
       <c r="C50" t="n">
-        <v>334.5</v>
+        <v>55.25</v>
       </c>
       <c r="D50" t="n">
-        <v>4.66</v>
+        <v>4.84</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>VIJSOLX</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>634.95</v>
+        <v>5.37</v>
       </c>
       <c r="C51" t="n">
-        <v>664.4</v>
+        <v>5.63</v>
       </c>
       <c r="D51" t="n">
-        <v>4.64</v>
+        <v>4.84</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GSTL</t>
+          <t>EASTWEST</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>11.9</v>
+        <v>2.3</v>
       </c>
       <c r="C52" t="n">
-        <v>12.45</v>
+        <v>2.41</v>
       </c>
       <c r="D52" t="n">
-        <v>4.62</v>
+        <v>4.78</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>6.41</v>
+        <v>4.61</v>
       </c>
       <c r="C53" t="n">
-        <v>6.7</v>
+        <v>4.83</v>
       </c>
       <c r="D53" t="n">
-        <v>4.52</v>
+        <v>4.77</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>27.44</v>
+        <v>39.04</v>
       </c>
       <c r="C54" t="n">
-        <v>28.68</v>
+        <v>40.9</v>
       </c>
       <c r="D54" t="n">
-        <v>4.52</v>
+        <v>4.76</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4297</v>
+        <v>0.84</v>
       </c>
       <c r="C55" t="n">
-        <v>4489.9</v>
+        <v>0.88</v>
       </c>
       <c r="D55" t="n">
-        <v>4.49</v>
+        <v>4.76</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>TVVISION</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4.02</v>
+        <v>2.78</v>
       </c>
       <c r="C56" t="n">
-        <v>4.2</v>
+        <v>2.91</v>
       </c>
       <c r="D56" t="n">
-        <v>4.48</v>
+        <v>4.68</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>7.13</v>
+        <v>6.26</v>
       </c>
       <c r="C57" t="n">
-        <v>7.44</v>
+        <v>6.55</v>
       </c>
       <c r="D57" t="n">
-        <v>4.35</v>
+        <v>4.63</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>METALIC</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>93.98999999999999</v>
+        <v>155.8</v>
       </c>
       <c r="C58" t="n">
-        <v>98</v>
+        <v>163</v>
       </c>
       <c r="D58" t="n">
-        <v>4.27</v>
+        <v>4.62</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NIMBSPROJ</t>
+          <t>HIGREEN</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>186.85</v>
+        <v>108.9</v>
       </c>
       <c r="C59" t="n">
-        <v>194.8</v>
+        <v>113.9</v>
       </c>
       <c r="D59" t="n">
-        <v>4.25</v>
+        <v>4.59</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BIL</t>
+          <t>PARNAXLAB</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1044.35</v>
+        <v>129.22</v>
       </c>
       <c r="C60" t="n">
-        <v>1088</v>
+        <v>134.98</v>
       </c>
       <c r="D60" t="n">
-        <v>4.18</v>
+        <v>4.46</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.48</v>
+        <v>21.8</v>
       </c>
       <c r="C61" t="n">
-        <v>0.5</v>
+        <v>22.75</v>
       </c>
       <c r="D61" t="n">
-        <v>4.17</v>
+        <v>4.36</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>SRGHFL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>60.28</v>
+        <v>143.75</v>
       </c>
       <c r="C62" t="n">
-        <v>62.78</v>
+        <v>150</v>
       </c>
       <c r="D62" t="n">
-        <v>4.15</v>
+        <v>4.35</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>10.03</v>
+        <v>2.1</v>
       </c>
       <c r="C63" t="n">
-        <v>10.44</v>
+        <v>2.19</v>
       </c>
       <c r="D63" t="n">
-        <v>4.09</v>
+        <v>4.29</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>ICDSLTD</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>42.08</v>
+        <v>61.9</v>
       </c>
       <c r="C64" t="n">
-        <v>43.8</v>
+        <v>64.5</v>
       </c>
       <c r="D64" t="n">
-        <v>4.09</v>
+        <v>4.2</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DHRUV</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>20.95</v>
+        <v>666.25</v>
       </c>
       <c r="C65" t="n">
-        <v>21.79</v>
+        <v>693.95</v>
       </c>
       <c r="D65" t="n">
-        <v>4.01</v>
+        <v>4.16</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ABH</t>
+          <t>SONAMLTD</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>48.1</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="C66" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D66" t="n">
-        <v>3.95</v>
+        <v>4.15</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>CRESTO</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>24.04</v>
+        <v>19.21</v>
       </c>
       <c r="C67" t="n">
-        <v>24.99</v>
+        <v>20</v>
       </c>
       <c r="D67" t="n">
-        <v>3.95</v>
+        <v>4.11</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.76</v>
+        <v>6.87</v>
       </c>
       <c r="C68" t="n">
-        <v>0.79</v>
+        <v>7.15</v>
       </c>
       <c r="D68" t="n">
-        <v>3.95</v>
+        <v>4.08</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>21.47</v>
+        <v>7.39</v>
       </c>
       <c r="C69" t="n">
-        <v>22.3</v>
+        <v>7.69</v>
       </c>
       <c r="D69" t="n">
-        <v>3.87</v>
+        <v>4.06</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TGBHOTELS</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>9.539999999999999</v>
+        <v>124.96</v>
       </c>
       <c r="C70" t="n">
-        <v>9.9</v>
+        <v>130</v>
       </c>
       <c r="D70" t="n">
-        <v>3.77</v>
+        <v>4.03</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>VITAL</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>54.9</v>
+        <v>8.74</v>
       </c>
       <c r="C71" t="n">
-        <v>56.9</v>
+        <v>9.09</v>
       </c>
       <c r="D71" t="n">
-        <v>3.64</v>
+        <v>4</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CONSOFINVT</t>
+          <t>SAHAJSOLAR</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>301.8</v>
+        <v>90.2</v>
       </c>
       <c r="C72" t="n">
-        <v>312.75</v>
+        <v>93.8</v>
       </c>
       <c r="D72" t="n">
-        <v>3.63</v>
+        <v>3.99</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>EMBDL</t>
+          <t>CORDSCABLE</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>58.89</v>
+        <v>382.9</v>
       </c>
       <c r="C73" t="n">
-        <v>61</v>
+        <v>398</v>
       </c>
       <c r="D73" t="n">
-        <v>3.58</v>
+        <v>3.94</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>KEYFINSERV</t>
+          <t>ATLASCYCLE</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>241.45</v>
+        <v>93.55</v>
       </c>
       <c r="C74" t="n">
-        <v>250</v>
+        <v>97.15000000000001</v>
       </c>
       <c r="D74" t="n">
-        <v>3.54</v>
+        <v>3.85</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>108.19</v>
+        <v>36.6</v>
       </c>
       <c r="C75" t="n">
-        <v>112</v>
+        <v>38</v>
       </c>
       <c r="D75" t="n">
-        <v>3.52</v>
+        <v>3.83</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ADISOFT</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>252.3</v>
+        <v>12.29</v>
       </c>
       <c r="C76" t="n">
-        <v>261.1</v>
+        <v>12.76</v>
       </c>
       <c r="D76" t="n">
-        <v>3.49</v>
+        <v>3.82</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>NDGL</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2580.6</v>
+        <v>20.22</v>
       </c>
       <c r="C77" t="n">
-        <v>2670</v>
+        <v>20.99</v>
       </c>
       <c r="D77" t="n">
-        <v>3.46</v>
+        <v>3.81</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.87</v>
+        <v>0.79</v>
       </c>
       <c r="C78" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="D78" t="n">
-        <v>3.45</v>
+        <v>3.8</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>16.44</v>
+        <v>5.01</v>
       </c>
       <c r="C79" t="n">
-        <v>17</v>
+        <v>5.2</v>
       </c>
       <c r="D79" t="n">
-        <v>3.41</v>
+        <v>3.79</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PHOENXINTL</t>
+          <t>RCDL</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>27.95</v>
+        <v>14.8</v>
       </c>
       <c r="C80" t="n">
-        <v>28.9</v>
+        <v>15.35</v>
       </c>
       <c r="D80" t="n">
-        <v>3.4</v>
+        <v>3.72</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>RAPPID</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>13.35</v>
+        <v>346.1</v>
       </c>
       <c r="C81" t="n">
-        <v>13.79</v>
+        <v>358.95</v>
       </c>
       <c r="D81" t="n">
-        <v>3.3</v>
+        <v>3.71</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>AGIIL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>6.09</v>
+        <v>269.3</v>
       </c>
       <c r="C82" t="n">
-        <v>6.29</v>
+        <v>279.15</v>
       </c>
       <c r="D82" t="n">
-        <v>3.28</v>
+        <v>3.66</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>2.45</v>
+        <v>636.8</v>
       </c>
       <c r="C83" t="n">
-        <v>2.53</v>
+        <v>660</v>
       </c>
       <c r="D83" t="n">
-        <v>3.27</v>
+        <v>3.64</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PRAKASHSTL</t>
+          <t>PRADPME</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>3.69</v>
+        <v>498.85</v>
       </c>
       <c r="C84" t="n">
-        <v>3.81</v>
+        <v>517</v>
       </c>
       <c r="D84" t="n">
-        <v>3.25</v>
+        <v>3.64</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>DPWIRES</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>13.24</v>
+        <v>154.23</v>
       </c>
       <c r="C85" t="n">
-        <v>13.67</v>
+        <v>159.8</v>
       </c>
       <c r="D85" t="n">
-        <v>3.25</v>
+        <v>3.61</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SWSOLAR</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>173.27</v>
+        <v>6.42</v>
       </c>
       <c r="C86" t="n">
-        <v>178.89</v>
+        <v>6.65</v>
       </c>
       <c r="D86" t="n">
-        <v>3.24</v>
+        <v>3.58</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>LOYALTEX</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>69.45</v>
+        <v>214.95</v>
       </c>
       <c r="C87" t="n">
-        <v>71.7</v>
+        <v>222.55</v>
       </c>
       <c r="D87" t="n">
-        <v>3.24</v>
+        <v>3.54</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>NAGREEKCAP</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>29.06</v>
+        <v>30.91</v>
       </c>
       <c r="C88" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D88" t="n">
-        <v>3.23</v>
+        <v>3.53</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>10.82</v>
+        <v>158.35</v>
       </c>
       <c r="C89" t="n">
-        <v>11.17</v>
+        <v>163.9</v>
       </c>
       <c r="D89" t="n">
-        <v>3.23</v>
+        <v>3.5</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>DAICHI</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>319.7</v>
+        <v>88.7</v>
       </c>
       <c r="C90" t="n">
-        <v>330</v>
+        <v>91.8</v>
       </c>
       <c r="D90" t="n">
-        <v>3.22</v>
+        <v>3.49</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1.88</v>
+        <v>50.06</v>
       </c>
       <c r="C91" t="n">
-        <v>1.94</v>
+        <v>51.8</v>
       </c>
       <c r="D91" t="n">
-        <v>3.19</v>
+        <v>3.48</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SHRADHA</t>
+          <t>WELSPUNLIV</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>29.99</v>
+        <v>221.51</v>
       </c>
       <c r="C92" t="n">
-        <v>30.94</v>
+        <v>229.2</v>
       </c>
       <c r="D92" t="n">
-        <v>3.17</v>
+        <v>3.47</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>LAXMICOT</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>46.54</v>
+        <v>13.05</v>
       </c>
       <c r="C93" t="n">
-        <v>48</v>
+        <v>13.5</v>
       </c>
       <c r="D93" t="n">
-        <v>3.14</v>
+        <v>3.45</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>12.79</v>
+        <v>94.8</v>
       </c>
       <c r="C94" t="n">
-        <v>13.19</v>
+        <v>98</v>
       </c>
       <c r="D94" t="n">
-        <v>3.13</v>
+        <v>3.38</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>5.12</v>
+        <v>12.47</v>
       </c>
       <c r="C95" t="n">
-        <v>5.28</v>
+        <v>12.89</v>
       </c>
       <c r="D95" t="n">
-        <v>3.13</v>
+        <v>3.37</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2.25</v>
+        <v>151.7</v>
       </c>
       <c r="C96" t="n">
-        <v>2.32</v>
+        <v>156.79</v>
       </c>
       <c r="D96" t="n">
-        <v>3.11</v>
+        <v>3.36</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>5.48</v>
+        <v>0.91</v>
       </c>
       <c r="C97" t="n">
-        <v>5.65</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D97" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>XTRANET</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>341.43</v>
+        <v>33.35</v>
       </c>
       <c r="C98" t="n">
-        <v>352</v>
+        <v>34.45</v>
       </c>
       <c r="D98" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>BOROSCI</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>119.11</v>
+        <v>14.51</v>
       </c>
       <c r="C99" t="n">
-        <v>122.75</v>
+        <v>14.98</v>
       </c>
       <c r="D99" t="n">
-        <v>3.06</v>
+        <v>3.24</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GLASSWALL</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>295.21</v>
+        <v>1022.2</v>
       </c>
       <c r="C100" t="n">
-        <v>304.15</v>
+        <v>1055</v>
       </c>
       <c r="D100" t="n">
-        <v>3.03</v>
+        <v>3.21</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>34.94</v>
+        <v>18.65</v>
       </c>
       <c r="C101" t="n">
-        <v>35.99</v>
+        <v>19.24</v>
       </c>
       <c r="D101" t="n">
-        <v>3.01</v>
+        <v>3.16</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>RAMASTEEL</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>4.38</v>
+        <v>867.65</v>
       </c>
       <c r="C102" t="n">
-        <v>4.51</v>
+        <v>895</v>
       </c>
       <c r="D102" t="n">
-        <v>2.97</v>
+        <v>3.15</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>5.72</v>
+        <v>28.81</v>
       </c>
       <c r="C103" t="n">
-        <v>5.89</v>
+        <v>29.7</v>
       </c>
       <c r="D103" t="n">
-        <v>2.97</v>
+        <v>3.09</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>49.54</v>
+        <v>663.55</v>
       </c>
       <c r="C104" t="n">
-        <v>50.99</v>
+        <v>684</v>
       </c>
       <c r="D104" t="n">
-        <v>2.93</v>
+        <v>3.08</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>3191.5</v>
+        <v>12.17</v>
       </c>
       <c r="C105" t="n">
-        <v>3285</v>
+        <v>12.54</v>
       </c>
       <c r="D105" t="n">
-        <v>2.93</v>
+        <v>3.04</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MAHAPEXLTD</t>
+          <t>KEN</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>54.36</v>
+        <v>43</v>
       </c>
       <c r="C106" t="n">
-        <v>55.95</v>
+        <v>44.3</v>
       </c>
       <c r="D106" t="n">
-        <v>2.92</v>
+        <v>3.02</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>7.91</v>
+        <v>133.41</v>
       </c>
       <c r="C107" t="n">
-        <v>8.140000000000001</v>
+        <v>137.41</v>
       </c>
       <c r="D107" t="n">
-        <v>2.91</v>
+        <v>3</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>38.34</v>
+        <v>5.34</v>
       </c>
       <c r="C108" t="n">
-        <v>39.45</v>
+        <v>5.5</v>
       </c>
       <c r="D108" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>36.93</v>
+        <v>19.8</v>
       </c>
       <c r="C109" t="n">
-        <v>37.99</v>
+        <v>20.39</v>
       </c>
       <c r="D109" t="n">
-        <v>2.87</v>
+        <v>2.98</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>TREJHARA</t>
+          <t>ARROWGREEN</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>132.25</v>
+        <v>913.05</v>
       </c>
       <c r="C110" t="n">
-        <v>136</v>
+        <v>940.05</v>
       </c>
       <c r="D110" t="n">
-        <v>2.84</v>
+        <v>2.96</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>JMA</t>
+          <t>MANINDS</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>88.3</v>
+        <v>849.9</v>
       </c>
       <c r="C111" t="n">
-        <v>90.79000000000001</v>
+        <v>875</v>
       </c>
       <c r="D111" t="n">
-        <v>2.82</v>
+        <v>2.95</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>KOTHARIPRO</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>63.23</v>
+        <v>665.35</v>
       </c>
       <c r="C112" t="n">
-        <v>65</v>
+        <v>685</v>
       </c>
       <c r="D112" t="n">
-        <v>2.8</v>
+        <v>2.95</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>SOLEX</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>8.609999999999999</v>
+        <v>678.95</v>
       </c>
       <c r="C113" t="n">
-        <v>8.85</v>
+        <v>698.95</v>
       </c>
       <c r="D113" t="n">
-        <v>2.79</v>
+        <v>2.95</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>INNOVANA</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>150.81</v>
+        <v>295.3</v>
       </c>
       <c r="C114" t="n">
-        <v>155</v>
+        <v>304</v>
       </c>
       <c r="D114" t="n">
-        <v>2.78</v>
+        <v>2.95</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>PRECOT</t>
+          <t>ABH</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>689.85</v>
+        <v>52.85</v>
       </c>
       <c r="C115" t="n">
-        <v>709</v>
+        <v>54.4</v>
       </c>
       <c r="D115" t="n">
-        <v>2.78</v>
+        <v>2.93</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>COOLCAPS</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>26.95</v>
+        <v>18.43</v>
       </c>
       <c r="C116" t="n">
-        <v>27.7</v>
+        <v>18.97</v>
       </c>
       <c r="D116" t="n">
-        <v>2.78</v>
+        <v>2.93</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SHALPAINTS</t>
+          <t>SHIVAAGRO</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>80.16</v>
+        <v>40.03</v>
       </c>
       <c r="C117" t="n">
-        <v>82.36</v>
+        <v>41.2</v>
       </c>
       <c r="D117" t="n">
-        <v>2.74</v>
+        <v>2.92</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CTE</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>42.73</v>
+        <v>1996.7</v>
       </c>
       <c r="C118" t="n">
-        <v>43.89</v>
+        <v>2055</v>
       </c>
       <c r="D118" t="n">
-        <v>2.71</v>
+        <v>2.92</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>SAMPANN</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>3.35</v>
+        <v>24.1</v>
       </c>
       <c r="C119" t="n">
-        <v>3.44</v>
+        <v>24.8</v>
       </c>
       <c r="D119" t="n">
-        <v>2.69</v>
+        <v>2.9</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>521</v>
+        <v>39.65</v>
       </c>
       <c r="C120" t="n">
-        <v>535</v>
+        <v>40.79</v>
       </c>
       <c r="D120" t="n">
-        <v>2.69</v>
+        <v>2.88</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>6.77</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="C121" t="n">
-        <v>6.95</v>
+        <v>70</v>
       </c>
       <c r="D121" t="n">
-        <v>2.66</v>
+        <v>2.88</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>REGAAL</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>28.69</v>
+        <v>97.20999999999999</v>
       </c>
       <c r="C122" t="n">
-        <v>29.45</v>
+        <v>100</v>
       </c>
       <c r="D122" t="n">
-        <v>2.65</v>
+        <v>2.87</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>24.21</v>
+        <v>59.09</v>
       </c>
       <c r="C123" t="n">
-        <v>24.85</v>
+        <v>60.74</v>
       </c>
       <c r="D123" t="n">
-        <v>2.64</v>
+        <v>2.79</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.76</v>
+        <v>33.08</v>
       </c>
       <c r="C124" t="n">
-        <v>0.78</v>
+        <v>34</v>
       </c>
       <c r="D124" t="n">
-        <v>2.63</v>
+        <v>2.78</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LCCPROJECT</t>
+          <t>BAGFILMS</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>141.33</v>
+        <v>4.31</v>
       </c>
       <c r="C125" t="n">
-        <v>145</v>
+        <v>4.43</v>
       </c>
       <c r="D125" t="n">
-        <v>2.6</v>
+        <v>2.78</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>LKPSEC</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>15.06</v>
+        <v>0.36</v>
       </c>
       <c r="C126" t="n">
-        <v>15.45</v>
+        <v>0.37</v>
       </c>
       <c r="D126" t="n">
-        <v>2.59</v>
+        <v>2.78</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>KLL</t>
+          <t>AKG</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>36.8</v>
+        <v>10.2</v>
       </c>
       <c r="C127" t="n">
-        <v>37.75</v>
+        <v>10.48</v>
       </c>
       <c r="D127" t="n">
-        <v>2.58</v>
+        <v>2.75</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>STEAMHOUSE</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>105.05</v>
+        <v>32.9</v>
       </c>
       <c r="C128" t="n">
-        <v>107.75</v>
+        <v>33.8</v>
       </c>
       <c r="D128" t="n">
-        <v>2.57</v>
+        <v>2.74</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>STYLAMIND</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>633.7</v>
+        <v>3309.4</v>
       </c>
       <c r="C129" t="n">
-        <v>650</v>
+        <v>3400</v>
       </c>
       <c r="D129" t="n">
-        <v>2.57</v>
+        <v>2.74</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>NRAIL</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>185.25</v>
+        <v>652.1</v>
       </c>
       <c r="C130" t="n">
-        <v>190</v>
+        <v>669.85</v>
       </c>
       <c r="D130" t="n">
-        <v>2.56</v>
+        <v>2.72</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>1725.8</v>
+        <v>24.35</v>
       </c>
       <c r="C131" t="n">
-        <v>1770</v>
+        <v>25</v>
       </c>
       <c r="D131" t="n">
-        <v>2.56</v>
+        <v>2.67</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>RKSWAMY</t>
+          <t>THEMISMED</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>88.79000000000001</v>
+        <v>122.6</v>
       </c>
       <c r="C132" t="n">
-        <v>91.05</v>
+        <v>125.85</v>
       </c>
       <c r="D132" t="n">
-        <v>2.55</v>
+        <v>2.65</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>477.7</v>
+        <v>254.45</v>
       </c>
       <c r="C133" t="n">
-        <v>489.9</v>
+        <v>261.2</v>
       </c>
       <c r="D133" t="n">
-        <v>2.55</v>
+        <v>2.65</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>PANORAMA</t>
+          <t>TEXINFRA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>54.89</v>
+        <v>115.02</v>
       </c>
       <c r="C134" t="n">
-        <v>56.29</v>
+        <v>118.05</v>
       </c>
       <c r="D134" t="n">
-        <v>2.55</v>
+        <v>2.63</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LINC</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>91.56999999999999</v>
+        <v>52.82</v>
       </c>
       <c r="C135" t="n">
-        <v>93.89</v>
+        <v>54.2</v>
       </c>
       <c r="D135" t="n">
-        <v>2.53</v>
+        <v>2.61</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PRADPME</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>475.1</v>
+        <v>9.31</v>
       </c>
       <c r="C136" t="n">
-        <v>487</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="D136" t="n">
-        <v>2.5</v>
+        <v>2.58</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SERVICE</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>66.05</v>
+        <v>1008.8</v>
       </c>
       <c r="C137" t="n">
-        <v>67.7</v>
+        <v>1034.7</v>
       </c>
       <c r="D137" t="n">
-        <v>2.5</v>
+        <v>2.57</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>WARDINMOBI</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>5.61</v>
+        <v>45.57</v>
       </c>
       <c r="C138" t="n">
-        <v>5.75</v>
+        <v>46.74</v>
       </c>
       <c r="D138" t="n">
-        <v>2.5</v>
+        <v>2.57</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>KAYA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>2.01</v>
+        <v>338.35</v>
       </c>
       <c r="C139" t="n">
-        <v>2.06</v>
+        <v>347</v>
       </c>
       <c r="D139" t="n">
-        <v>2.49</v>
+        <v>2.56</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>8.869999999999999</v>
+        <v>1062.8</v>
       </c>
       <c r="C140" t="n">
-        <v>9.09</v>
+        <v>1089.9</v>
       </c>
       <c r="D140" t="n">
-        <v>2.48</v>
+        <v>2.55</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>171.75</v>
+        <v>500.25</v>
       </c>
       <c r="C141" t="n">
-        <v>176</v>
+        <v>513</v>
       </c>
       <c r="D141" t="n">
-        <v>2.47</v>
+        <v>2.55</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.41</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C142" t="n">
-        <v>0.42</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="D142" t="n">
-        <v>2.44</v>
+        <v>2.51</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>NATCAPSUQ</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>230.26</v>
+        <v>169</v>
       </c>
       <c r="C143" t="n">
-        <v>235.8</v>
+        <v>173.2</v>
       </c>
       <c r="D143" t="n">
-        <v>2.41</v>
+        <v>2.49</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>MCLOUD</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>414.7</v>
+        <v>25.18</v>
       </c>
       <c r="C144" t="n">
-        <v>424.7</v>
+        <v>25.8</v>
       </c>
       <c r="D144" t="n">
-        <v>2.41</v>
+        <v>2.46</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>RKSWAMY</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>198.29</v>
+        <v>87.8</v>
       </c>
       <c r="C145" t="n">
-        <v>202.99</v>
+        <v>89.94</v>
       </c>
       <c r="D145" t="n">
-        <v>2.37</v>
+        <v>2.44</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>CRSL</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>2.53</v>
+        <v>80.98</v>
       </c>
       <c r="C146" t="n">
-        <v>2.59</v>
+        <v>82.95</v>
       </c>
       <c r="D146" t="n">
-        <v>2.37</v>
+        <v>2.43</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>TATACAP</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>4.22</v>
+        <v>341.1</v>
       </c>
       <c r="C147" t="n">
-        <v>4.32</v>
+        <v>349.35</v>
       </c>
       <c r="D147" t="n">
-        <v>2.37</v>
+        <v>2.42</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>1.7</v>
+        <v>192.77</v>
       </c>
       <c r="C148" t="n">
-        <v>1.74</v>
+        <v>197.44</v>
       </c>
       <c r="D148" t="n">
-        <v>2.35</v>
+        <v>2.42</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MANORG</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>464.15</v>
+        <v>28.95</v>
       </c>
       <c r="C149" t="n">
-        <v>475</v>
+        <v>29.65</v>
       </c>
       <c r="D149" t="n">
-        <v>2.34</v>
+        <v>2.42</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>AGIIL</t>
+          <t>BSHSL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>271.15</v>
+        <v>85.64</v>
       </c>
       <c r="C150" t="n">
-        <v>277.5</v>
+        <v>87.7</v>
       </c>
       <c r="D150" t="n">
-        <v>2.34</v>
+        <v>2.41</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>RTSPOWR</t>
+          <t>DRONE</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>87.95999999999999</v>
+        <v>33.15</v>
       </c>
       <c r="C151" t="n">
-        <v>90</v>
+        <v>33.95</v>
       </c>
       <c r="D151" t="n">
-        <v>2.32</v>
+        <v>2.41</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>168.63</v>
+        <v>24.41</v>
       </c>
       <c r="C152" t="n">
-        <v>172.5</v>
+        <v>24.99</v>
       </c>
       <c r="D152" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>SAFEENTP</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>156.9</v>
+        <v>248.1</v>
       </c>
       <c r="C153" t="n">
-        <v>160.5</v>
+        <v>254</v>
       </c>
       <c r="D153" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ATAM</t>
+          <t>TECHD</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>59.05</v>
+        <v>556.8</v>
       </c>
       <c r="C154" t="n">
-        <v>60.4</v>
+        <v>570</v>
       </c>
       <c r="D154" t="n">
-        <v>2.29</v>
+        <v>2.37</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>VIVOBIOT</t>
+          <t>IRB</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>16.21</v>
+        <v>17.98</v>
       </c>
       <c r="C155" t="n">
-        <v>16.58</v>
+        <v>18.4</v>
       </c>
       <c r="D155" t="n">
-        <v>2.28</v>
+        <v>2.34</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>HLEGLAS</t>
+          <t>SHRIAHIMSA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>469.2</v>
+        <v>473.95</v>
       </c>
       <c r="C156" t="n">
-        <v>479.9</v>
+        <v>485</v>
       </c>
       <c r="D156" t="n">
-        <v>2.28</v>
+        <v>2.33</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>359.3</v>
+        <v>40.07</v>
       </c>
       <c r="C157" t="n">
-        <v>367.45</v>
+        <v>41</v>
       </c>
       <c r="D157" t="n">
-        <v>2.27</v>
+        <v>2.32</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>ROHLTD</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1287.8</v>
+        <v>306</v>
       </c>
       <c r="C158" t="n">
-        <v>1317</v>
+        <v>313</v>
       </c>
       <c r="D158" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>INDSWFTLAB</t>
+          <t>EBIX</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>379.4</v>
+        <v>18.43</v>
       </c>
       <c r="C159" t="n">
-        <v>388</v>
+        <v>18.85</v>
       </c>
       <c r="D159" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>14.57</v>
+        <v>34.81</v>
       </c>
       <c r="C160" t="n">
-        <v>14.9</v>
+        <v>35.6</v>
       </c>
       <c r="D160" t="n">
-        <v>2.26</v>
+        <v>2.27</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ANNAPURNA</t>
+          <t>MARALOVER</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>130.56</v>
+        <v>61.11</v>
       </c>
       <c r="C161" t="n">
-        <v>133.5</v>
+        <v>62.5</v>
       </c>
       <c r="D161" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>MANBA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>29.44</v>
+        <v>136.41</v>
       </c>
       <c r="C162" t="n">
-        <v>30.09</v>
+        <v>139.48</v>
       </c>
       <c r="D162" t="n">
-        <v>2.21</v>
+        <v>2.25</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>INDOAMIN</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>132.87</v>
+        <v>2.22</v>
       </c>
       <c r="C163" t="n">
-        <v>135.8</v>
+        <v>2.27</v>
       </c>
       <c r="D163" t="n">
-        <v>2.21</v>
+        <v>2.25</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>DICIND</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>5.97</v>
+        <v>654.25</v>
       </c>
       <c r="C164" t="n">
-        <v>6.1</v>
+        <v>669</v>
       </c>
       <c r="D164" t="n">
-        <v>2.18</v>
+        <v>2.25</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>202.63</v>
+        <v>5.8</v>
       </c>
       <c r="C165" t="n">
-        <v>207</v>
+        <v>5.93</v>
       </c>
       <c r="D165" t="n">
-        <v>2.16</v>
+        <v>2.24</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>3BBLACKBIO</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>2.78</v>
+        <v>1369.3</v>
       </c>
       <c r="C166" t="n">
-        <v>2.84</v>
+        <v>1400</v>
       </c>
       <c r="D166" t="n">
-        <v>2.16</v>
+        <v>2.24</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>HILINFRA</t>
+          <t>GUJAPOLLO</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>43.37</v>
+        <v>337.4</v>
       </c>
       <c r="C167" t="n">
-        <v>44.3</v>
+        <v>344.95</v>
       </c>
       <c r="D167" t="n">
-        <v>2.14</v>
+        <v>2.24</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>1032.9</v>
+        <v>15.26</v>
       </c>
       <c r="C168" t="n">
-        <v>1055</v>
+        <v>15.6</v>
       </c>
       <c r="D168" t="n">
-        <v>2.14</v>
+        <v>2.23</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>2.37</v>
+        <v>2.26</v>
       </c>
       <c r="C169" t="n">
-        <v>2.42</v>
+        <v>2.31</v>
       </c>
       <c r="D169" t="n">
-        <v>2.11</v>
+        <v>2.21</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>ARIHANTCAP</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>577.8</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="C170" t="n">
-        <v>590</v>
+        <v>93</v>
       </c>
       <c r="D170" t="n">
-        <v>2.11</v>
+        <v>2.21</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ESSARSHPNG</t>
+          <t>THAKDEV</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>16.15</v>
+        <v>126.36</v>
       </c>
       <c r="C171" t="n">
-        <v>16.49</v>
+        <v>129.15</v>
       </c>
       <c r="D171" t="n">
-        <v>2.11</v>
+        <v>2.21</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>160.92</v>
+        <v>32.24</v>
       </c>
       <c r="C172" t="n">
-        <v>164.3</v>
+        <v>32.95</v>
       </c>
       <c r="D172" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>POWERICA</t>
+          <t>PRESSTONIC</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>568.1</v>
+        <v>41.05</v>
       </c>
       <c r="C173" t="n">
-        <v>579.95</v>
+        <v>41.95</v>
       </c>
       <c r="D173" t="n">
-        <v>2.09</v>
+        <v>2.19</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>128.32</v>
+        <v>5.04</v>
       </c>
       <c r="C174" t="n">
-        <v>131</v>
+        <v>5.15</v>
       </c>
       <c r="D174" t="n">
-        <v>2.09</v>
+        <v>2.18</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>ASHUTOSH</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>6.21</v>
+        <v>150.1</v>
       </c>
       <c r="C175" t="n">
-        <v>6.34</v>
+        <v>153.35</v>
       </c>
       <c r="D175" t="n">
-        <v>2.09</v>
+        <v>2.17</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>HINDADH</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>383.9</v>
+        <v>1.84</v>
       </c>
       <c r="C176" t="n">
-        <v>391.9</v>
+        <v>1.88</v>
       </c>
       <c r="D176" t="n">
-        <v>2.08</v>
+        <v>2.17</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>VIRINCHI</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>13.98</v>
+        <v>0.46</v>
       </c>
       <c r="C177" t="n">
-        <v>14.27</v>
+        <v>0.47</v>
       </c>
       <c r="D177" t="n">
-        <v>2.07</v>
+        <v>2.17</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>APEX</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>351.65</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="C178" t="n">
-        <v>358.9</v>
+        <v>72.5</v>
       </c>
       <c r="D178" t="n">
-        <v>2.06</v>
+        <v>2.17</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>PARAGMILK</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>272.4</v>
+        <v>12.58</v>
       </c>
       <c r="C179" t="n">
-        <v>278</v>
+        <v>12.85</v>
       </c>
       <c r="D179" t="n">
-        <v>2.06</v>
+        <v>2.15</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>XELPMOC</t>
+          <t>NDRAUTO</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>73.88</v>
+        <v>753.2</v>
       </c>
       <c r="C180" t="n">
-        <v>75.40000000000001</v>
+        <v>769.4</v>
       </c>
       <c r="D180" t="n">
-        <v>2.06</v>
+        <v>2.15</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>8.720000000000001</v>
+        <v>1.86</v>
       </c>
       <c r="C181" t="n">
-        <v>8.9</v>
+        <v>1.9</v>
       </c>
       <c r="D181" t="n">
-        <v>2.06</v>
+        <v>2.15</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>AUTOIND</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>83.76000000000001</v>
+        <v>13.6</v>
       </c>
       <c r="C182" t="n">
-        <v>85.48</v>
+        <v>13.89</v>
       </c>
       <c r="D182" t="n">
-        <v>2.05</v>
+        <v>2.13</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ISFT</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>92.09</v>
+        <v>2.83</v>
       </c>
       <c r="C183" t="n">
-        <v>93.98</v>
+        <v>2.89</v>
       </c>
       <c r="D183" t="n">
-        <v>2.05</v>
+        <v>2.12</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>96.02</v>
+        <v>17.91</v>
       </c>
       <c r="C184" t="n">
-        <v>97.98999999999999</v>
+        <v>18.29</v>
       </c>
       <c r="D184" t="n">
-        <v>2.05</v>
+        <v>2.12</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ARIHANT</t>
+          <t>PANORAMA</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>957.35</v>
+        <v>55.32</v>
       </c>
       <c r="C185" t="n">
-        <v>977</v>
+        <v>56.48</v>
       </c>
       <c r="D185" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>ANDHRAPAP</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1371.1</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="C186" t="n">
-        <v>1399</v>
+        <v>72.92</v>
       </c>
       <c r="D186" t="n">
-        <v>2.03</v>
+        <v>2.09</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>186.22</v>
+        <v>78.93000000000001</v>
       </c>
       <c r="C187" t="n">
-        <v>190</v>
+        <v>80.58</v>
       </c>
       <c r="D187" t="n">
-        <v>2.03</v>
+        <v>2.09</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ASHIMASYN</t>
+          <t>KANOHAR</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>15.94</v>
+        <v>870.5</v>
       </c>
       <c r="C188" t="n">
-        <v>16.26</v>
+        <v>888.7</v>
       </c>
       <c r="D188" t="n">
-        <v>2.01</v>
+        <v>2.09</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>99.98999999999999</v>
+        <v>30.14</v>
       </c>
       <c r="C189" t="n">
-        <v>102</v>
+        <v>30.77</v>
       </c>
       <c r="D189" t="n">
-        <v>2.01</v>
+        <v>2.09</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>KECL</t>
+          <t>NILASPACES</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>118.43</v>
+        <v>12.02</v>
       </c>
       <c r="C190" t="n">
-        <v>120.8</v>
+        <v>12.27</v>
       </c>
       <c r="D190" t="n">
-        <v>2</v>
+        <v>2.08</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>35.93</v>
+        <v>4.35</v>
       </c>
       <c r="C191" t="n">
-        <v>36.65</v>
+        <v>4.44</v>
       </c>
       <c r="D191" t="n">
-        <v>2</v>
+        <v>2.07</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>421.66</v>
+        <v>15.68</v>
       </c>
       <c r="C192" t="n">
-        <v>430.09</v>
+        <v>16</v>
       </c>
       <c r="D192" t="n">
-        <v>2</v>
+        <v>2.04</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>GHCLTEXTIL</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>129.52</v>
+        <v>38.19</v>
       </c>
       <c r="C193" t="n">
-        <v>132.1</v>
+        <v>38.97</v>
       </c>
       <c r="D193" t="n">
-        <v>1.99</v>
+        <v>2.04</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SUDARCOLOR</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>402</v>
+        <v>2096.5</v>
       </c>
       <c r="C194" t="n">
-        <v>410</v>
+        <v>2139</v>
       </c>
       <c r="D194" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>24.13</v>
+        <v>22.69</v>
       </c>
       <c r="C195" t="n">
-        <v>24.61</v>
+        <v>23.15</v>
       </c>
       <c r="D195" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>INOXINDIA</t>
+          <t>DIAMINESQ</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>2089.2</v>
+        <v>254.85</v>
       </c>
       <c r="C196" t="n">
-        <v>2130.7</v>
+        <v>260</v>
       </c>
       <c r="D196" t="n">
-        <v>1.99</v>
+        <v>2.02</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>MOHITE</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>39.61</v>
+        <v>2.47</v>
       </c>
       <c r="C197" t="n">
-        <v>40.4</v>
+        <v>2.52</v>
       </c>
       <c r="D197" t="n">
-        <v>1.99</v>
+        <v>2.02</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SKYWAYS</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>126.03</v>
+        <v>462.75</v>
       </c>
       <c r="C198" t="n">
-        <v>128.54</v>
+        <v>472.1</v>
       </c>
       <c r="D198" t="n">
-        <v>1.99</v>
+        <v>2.02</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>97.17</v>
+        <v>107.67</v>
       </c>
       <c r="C199" t="n">
-        <v>99.09999999999999</v>
+        <v>109.85</v>
       </c>
       <c r="D199" t="n">
-        <v>1.99</v>
+        <v>2.02</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>SGRL</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>720.75</v>
+        <v>23.34</v>
       </c>
       <c r="C200" t="n">
-        <v>735</v>
+        <v>23.81</v>
       </c>
       <c r="D200" t="n">
-        <v>1.98</v>
+        <v>2.01</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TRITONV</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>1063.9</v>
+        <v>5.97</v>
       </c>
       <c r="C201" t="n">
-        <v>1085</v>
+        <v>6.09</v>
       </c>
       <c r="D201" t="n">
-        <v>1.98</v>
+        <v>2.01</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-24 08:45 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>POLYSPIN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>104.85</v>
+        <v>30.78</v>
       </c>
       <c r="C2" t="n">
-        <v>125.82</v>
+        <v>36.49</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>18.55</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>119.98</v>
+        <v>125.82</v>
       </c>
       <c r="C3" t="n">
-        <v>143.97</v>
+        <v>138.4</v>
       </c>
       <c r="D3" t="n">
-        <v>19.99</v>
+        <v>10</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>CRESTO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>708.9</v>
+        <v>20.14</v>
       </c>
       <c r="C4" t="n">
-        <v>800</v>
+        <v>21.8</v>
       </c>
       <c r="D4" t="n">
-        <v>12.85</v>
+        <v>8.24</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REGENCERAM</t>
+          <t>TGBHOTELS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33.3</v>
+        <v>9.43</v>
       </c>
       <c r="C5" t="n">
-        <v>36.75</v>
+        <v>10.14</v>
       </c>
       <c r="D5" t="n">
-        <v>10.36</v>
+        <v>7.53</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>MITCON</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23.16</v>
+        <v>82.62</v>
       </c>
       <c r="C6" t="n">
-        <v>25.4</v>
+        <v>88.5</v>
       </c>
       <c r="D6" t="n">
-        <v>9.67</v>
+        <v>7.12</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PROSTARM</t>
+          <t>AASTHA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>127.84</v>
+        <v>89.77</v>
       </c>
       <c r="C7" t="n">
-        <v>139.4</v>
+        <v>96</v>
       </c>
       <c r="D7" t="n">
-        <v>9.039999999999999</v>
+        <v>6.94</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SCODATUBES</t>
+          <t>GKB</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>128.85</v>
+        <v>69.73</v>
       </c>
       <c r="C8" t="n">
-        <v>139.95</v>
+        <v>74</v>
       </c>
       <c r="D8" t="n">
-        <v>8.609999999999999</v>
+        <v>6.12</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ANSALBU</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>90.12</v>
+        <v>0.18</v>
       </c>
       <c r="C9" t="n">
-        <v>97.75</v>
+        <v>0.19</v>
       </c>
       <c r="D9" t="n">
-        <v>8.470000000000001</v>
+        <v>5.56</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>ASIANTNE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.65</v>
+        <v>9.24</v>
       </c>
       <c r="C10" t="n">
-        <v>7.2</v>
+        <v>9.75</v>
       </c>
       <c r="D10" t="n">
-        <v>8.27</v>
+        <v>5.52</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.46</v>
+        <v>389</v>
       </c>
       <c r="C11" t="n">
-        <v>1.57</v>
+        <v>408.45</v>
       </c>
       <c r="D11" t="n">
-        <v>7.53</v>
+        <v>5</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ASIANTNE</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.380000000000001</v>
+        <v>126</v>
       </c>
       <c r="C12" t="n">
-        <v>10.08</v>
+        <v>132.3</v>
       </c>
       <c r="D12" t="n">
-        <v>7.46</v>
+        <v>5</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AUSTENG</t>
+          <t>AKANKSHA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>162.85</v>
+        <v>151.1</v>
       </c>
       <c r="C13" t="n">
-        <v>174.8</v>
+        <v>158.65</v>
       </c>
       <c r="D13" t="n">
-        <v>7.34</v>
+        <v>5</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CREATIVEYE</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.25</v>
+        <v>152.1</v>
       </c>
       <c r="C14" t="n">
-        <v>6.68</v>
+        <v>159.7</v>
       </c>
       <c r="D14" t="n">
-        <v>6.88</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AVIENCE</t>
+          <t>SWARAJ</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>345.85</v>
+        <v>307.15</v>
       </c>
       <c r="C15" t="n">
-        <v>369.5</v>
+        <v>322.5</v>
       </c>
       <c r="D15" t="n">
-        <v>6.84</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BEWLTD</t>
+          <t>AUROIMPEX</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>61.35</v>
+        <v>39</v>
       </c>
       <c r="C16" t="n">
-        <v>65.34999999999999</v>
+        <v>40.95</v>
       </c>
       <c r="D16" t="n">
-        <v>6.52</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ARVSMART</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>588.2</v>
+        <v>84.58</v>
       </c>
       <c r="C17" t="n">
-        <v>625</v>
+        <v>88.8</v>
       </c>
       <c r="D17" t="n">
-        <v>6.26</v>
+        <v>4.99</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OSWALPUMPS</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>273.6</v>
+        <v>49.7</v>
       </c>
       <c r="C18" t="n">
-        <v>290.1</v>
+        <v>52.18</v>
       </c>
       <c r="D18" t="n">
-        <v>6.03</v>
+        <v>4.99</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.17</v>
+        <v>29.44</v>
       </c>
       <c r="C19" t="n">
-        <v>0.18</v>
+        <v>30.91</v>
       </c>
       <c r="D19" t="n">
-        <v>5.88</v>
+        <v>4.99</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SINTERCOM</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>80.48999999999999</v>
+        <v>11.05</v>
       </c>
       <c r="C20" t="n">
-        <v>84.98</v>
+        <v>11.6</v>
       </c>
       <c r="D20" t="n">
-        <v>5.58</v>
+        <v>4.98</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>80.5</v>
+        <v>29.1</v>
       </c>
       <c r="C21" t="n">
-        <v>84.89</v>
+        <v>30.55</v>
       </c>
       <c r="D21" t="n">
-        <v>5.45</v>
+        <v>4.98</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AMJLAND</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>37.75</v>
+        <v>5.83</v>
       </c>
       <c r="C22" t="n">
-        <v>39.75</v>
+        <v>6.12</v>
       </c>
       <c r="D22" t="n">
-        <v>5.3</v>
+        <v>4.97</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>DEEM</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>7.02</v>
+        <v>47.3</v>
       </c>
       <c r="C23" t="n">
-        <v>7.39</v>
+        <v>49.65</v>
       </c>
       <c r="D23" t="n">
-        <v>5.27</v>
+        <v>4.97</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KRITI</t>
+          <t>ARCL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59.75</v>
+        <v>255.79</v>
       </c>
       <c r="C24" t="n">
-        <v>62.89</v>
+        <v>268.5</v>
       </c>
       <c r="D24" t="n">
-        <v>5.26</v>
+        <v>4.97</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CLEANMAX</t>
+          <t>MARC</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1367.5</v>
+        <v>148.05</v>
       </c>
       <c r="C25" t="n">
-        <v>1439</v>
+        <v>155.4</v>
       </c>
       <c r="D25" t="n">
-        <v>5.23</v>
+        <v>4.96</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5.56</v>
+        <v>46.35</v>
       </c>
       <c r="C26" t="n">
-        <v>5.84</v>
+        <v>48.65</v>
       </c>
       <c r="D26" t="n">
-        <v>5.04</v>
+        <v>4.96</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMEYA</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>157.1</v>
+        <v>3.84</v>
       </c>
       <c r="C27" t="n">
-        <v>164.95</v>
+        <v>4.03</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TIRUPATIFL</t>
+          <t>ARMOUR</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>74.61</v>
+        <v>18.25</v>
       </c>
       <c r="C28" t="n">
-        <v>78.34</v>
+        <v>19.15</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>4.93</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1059,13 +1059,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>211.07</v>
+        <v>221.62</v>
       </c>
       <c r="C29" t="n">
-        <v>221.62</v>
+        <v>232.5</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4.91</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>RCDL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>334.45</v>
+        <v>15.5</v>
       </c>
       <c r="C30" t="n">
-        <v>351.15</v>
+        <v>16.25</v>
       </c>
       <c r="D30" t="n">
-        <v>4.99</v>
+        <v>4.84</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>370.5</v>
+        <v>34.81</v>
       </c>
       <c r="C31" t="n">
-        <v>389</v>
+        <v>36.48</v>
       </c>
       <c r="D31" t="n">
-        <v>4.99</v>
+        <v>4.8</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>28.04</v>
+        <v>55.3</v>
       </c>
       <c r="C32" t="n">
-        <v>29.44</v>
+        <v>57.95</v>
       </c>
       <c r="D32" t="n">
-        <v>4.99</v>
+        <v>4.79</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DEEM</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>45.05</v>
+        <v>4.83</v>
       </c>
       <c r="C33" t="n">
-        <v>47.3</v>
+        <v>5.06</v>
       </c>
       <c r="D33" t="n">
-        <v>4.99</v>
+        <v>4.76</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>NAGREEKEXP</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>72.92</v>
+        <v>24.21</v>
       </c>
       <c r="C34" t="n">
-        <v>76.56</v>
+        <v>25.35</v>
       </c>
       <c r="D34" t="n">
-        <v>4.99</v>
+        <v>4.71</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>HEROMOTORS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>28.86</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="C35" t="n">
-        <v>30.3</v>
+        <v>103</v>
       </c>
       <c r="D35" t="n">
-        <v>4.99</v>
+        <v>4.67</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>AVANTEL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>33.16</v>
+        <v>146.17</v>
       </c>
       <c r="C36" t="n">
-        <v>34.81</v>
+        <v>153</v>
       </c>
       <c r="D36" t="n">
-        <v>4.98</v>
+        <v>4.67</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NEUEON</t>
+          <t>GOLDSTAR</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>12.44</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C37" t="n">
-        <v>13.06</v>
+        <v>10.15</v>
       </c>
       <c r="D37" t="n">
-        <v>4.98</v>
+        <v>4.64</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>SUPTANERY</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>44.15</v>
+        <v>10.65</v>
       </c>
       <c r="C38" t="n">
-        <v>46.35</v>
+        <v>11.14</v>
       </c>
       <c r="D38" t="n">
-        <v>4.98</v>
+        <v>4.6</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>212.85</v>
+        <v>2.19</v>
       </c>
       <c r="C39" t="n">
-        <v>223.45</v>
+        <v>2.29</v>
       </c>
       <c r="D39" t="n">
-        <v>4.98</v>
+        <v>4.57</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AUROIMPEX</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>37.15</v>
+        <v>2.85</v>
       </c>
       <c r="C40" t="n">
-        <v>39</v>
+        <v>2.98</v>
       </c>
       <c r="D40" t="n">
-        <v>4.98</v>
+        <v>4.56</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SMARTEN</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>59.3</v>
+        <v>0.88</v>
       </c>
       <c r="C41" t="n">
-        <v>62.25</v>
+        <v>0.92</v>
       </c>
       <c r="D41" t="n">
-        <v>4.97</v>
+        <v>4.55</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>10.53</v>
+        <v>491.85</v>
       </c>
       <c r="C42" t="n">
-        <v>11.05</v>
+        <v>513</v>
       </c>
       <c r="D42" t="n">
-        <v>4.94</v>
+        <v>4.3</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HPTL</t>
+          <t>SMARTEN</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>446</v>
+        <v>62.25</v>
       </c>
       <c r="C43" t="n">
-        <v>468</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D43" t="n">
-        <v>4.93</v>
+        <v>4.26</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>VIKRAN</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3.66</v>
+        <v>56.14</v>
       </c>
       <c r="C44" t="n">
-        <v>3.84</v>
+        <v>58.5</v>
       </c>
       <c r="D44" t="n">
-        <v>4.92</v>
+        <v>4.2</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ARCL</t>
+          <t>LOYALTEX</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>262.06</v>
+        <v>231.23</v>
       </c>
       <c r="C45" t="n">
-        <v>274.95</v>
+        <v>240.9</v>
       </c>
       <c r="D45" t="n">
-        <v>4.92</v>
+        <v>4.18</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>997.9</v>
+        <v>411.85</v>
       </c>
       <c r="C46" t="n">
-        <v>1046.8</v>
+        <v>429</v>
       </c>
       <c r="D46" t="n">
-        <v>4.9</v>
+        <v>4.16</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>47.34</v>
+        <v>640.6</v>
       </c>
       <c r="C47" t="n">
-        <v>49.65</v>
+        <v>667</v>
       </c>
       <c r="D47" t="n">
-        <v>4.88</v>
+        <v>4.12</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>HITECHGEAR</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>27.75</v>
+        <v>560.95</v>
       </c>
       <c r="C48" t="n">
-        <v>29.1</v>
+        <v>584</v>
       </c>
       <c r="D48" t="n">
-        <v>4.86</v>
+        <v>4.11</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>FRONTSP</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>23.67</v>
+        <v>1394.6</v>
       </c>
       <c r="C49" t="n">
-        <v>24.82</v>
+        <v>1451.8</v>
       </c>
       <c r="D49" t="n">
-        <v>4.86</v>
+        <v>4.1</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>52.7</v>
+        <v>2.44</v>
       </c>
       <c r="C50" t="n">
-        <v>55.25</v>
+        <v>2.54</v>
       </c>
       <c r="D50" t="n">
-        <v>4.84</v>
+        <v>4.1</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5.37</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="C51" t="n">
-        <v>5.63</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="D51" t="n">
-        <v>4.84</v>
+        <v>4.08</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>EASTWEST</t>
+          <t>LAKSHYA</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2.3</v>
+        <v>98</v>
       </c>
       <c r="C52" t="n">
-        <v>2.41</v>
+        <v>102</v>
       </c>
       <c r="D52" t="n">
-        <v>4.78</v>
+        <v>4.08</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>RELTD</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>4.61</v>
+        <v>149.36</v>
       </c>
       <c r="C53" t="n">
-        <v>4.83</v>
+        <v>155.4</v>
       </c>
       <c r="D53" t="n">
-        <v>4.77</v>
+        <v>4.04</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>TIRUPATIFL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>39.04</v>
+        <v>78.34</v>
       </c>
       <c r="C54" t="n">
-        <v>40.9</v>
+        <v>81.5</v>
       </c>
       <c r="D54" t="n">
-        <v>4.76</v>
+        <v>4.03</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.84</v>
+        <v>5.25</v>
       </c>
       <c r="C55" t="n">
-        <v>0.88</v>
+        <v>5.46</v>
       </c>
       <c r="D55" t="n">
-        <v>4.76</v>
+        <v>4</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>EASTSILK</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2.78</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="C56" t="n">
-        <v>2.91</v>
+        <v>71.25</v>
       </c>
       <c r="D56" t="n">
-        <v>4.68</v>
+        <v>4</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>REFRACTORY</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6.26</v>
+        <v>36.55</v>
       </c>
       <c r="C57" t="n">
-        <v>6.55</v>
+        <v>38</v>
       </c>
       <c r="D57" t="n">
-        <v>4.63</v>
+        <v>3.97</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>METALIC</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>155.8</v>
+        <v>6.74</v>
       </c>
       <c r="C58" t="n">
-        <v>163</v>
+        <v>7</v>
       </c>
       <c r="D58" t="n">
-        <v>4.62</v>
+        <v>3.86</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>HIGREEN</t>
+          <t>AURUS</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>108.9</v>
+        <v>4.67</v>
       </c>
       <c r="C59" t="n">
-        <v>113.9</v>
+        <v>4.85</v>
       </c>
       <c r="D59" t="n">
-        <v>4.59</v>
+        <v>3.85</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PARNAXLAB</t>
+          <t>AZADIND</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>129.22</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="C60" t="n">
-        <v>134.98</v>
+        <v>84</v>
       </c>
       <c r="D60" t="n">
-        <v>4.46</v>
+        <v>3.79</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>APOORVA</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>21.8</v>
+        <v>34.32</v>
       </c>
       <c r="C61" t="n">
-        <v>22.75</v>
+        <v>35.58</v>
       </c>
       <c r="D61" t="n">
-        <v>4.36</v>
+        <v>3.67</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SRGHFL</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>143.75</v>
+        <v>40.47</v>
       </c>
       <c r="C62" t="n">
-        <v>150</v>
+        <v>41.94</v>
       </c>
       <c r="D62" t="n">
-        <v>4.35</v>
+        <v>3.63</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>VGCL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2.1</v>
+        <v>47.18</v>
       </c>
       <c r="C63" t="n">
-        <v>2.19</v>
+        <v>48.89</v>
       </c>
       <c r="D63" t="n">
-        <v>4.29</v>
+        <v>3.62</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ICDSLTD</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>61.9</v>
+        <v>29.93</v>
       </c>
       <c r="C64" t="n">
-        <v>64.5</v>
+        <v>31</v>
       </c>
       <c r="D64" t="n">
-        <v>4.2</v>
+        <v>3.58</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>666.25</v>
+        <v>0.28</v>
       </c>
       <c r="C65" t="n">
-        <v>693.95</v>
+        <v>0.29</v>
       </c>
       <c r="D65" t="n">
-        <v>4.16</v>
+        <v>3.57</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SONAMLTD</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>67.20999999999999</v>
+        <v>5.7</v>
       </c>
       <c r="C66" t="n">
-        <v>70</v>
+        <v>5.9</v>
       </c>
       <c r="D66" t="n">
-        <v>4.15</v>
+        <v>3.51</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CRESTO</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>19.21</v>
+        <v>18.22</v>
       </c>
       <c r="C67" t="n">
-        <v>20</v>
+        <v>18.84</v>
       </c>
       <c r="D67" t="n">
-        <v>4.11</v>
+        <v>3.4</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TIJARIA</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>6.87</v>
+        <v>30.25</v>
       </c>
       <c r="C68" t="n">
-        <v>7.15</v>
+        <v>31.25</v>
       </c>
       <c r="D68" t="n">
-        <v>4.08</v>
+        <v>3.31</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>7.39</v>
+        <v>19.04</v>
       </c>
       <c r="C69" t="n">
-        <v>7.69</v>
+        <v>19.67</v>
       </c>
       <c r="D69" t="n">
-        <v>4.06</v>
+        <v>3.31</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>124.96</v>
+        <v>4.28</v>
       </c>
       <c r="C70" t="n">
-        <v>130</v>
+        <v>4.42</v>
       </c>
       <c r="D70" t="n">
-        <v>4.03</v>
+        <v>3.27</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>8.74</v>
+        <v>12.5</v>
       </c>
       <c r="C71" t="n">
-        <v>9.09</v>
+        <v>12.9</v>
       </c>
       <c r="D71" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SAHAJSOLAR</t>
+          <t>ANSALBU</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>90.2</v>
+        <v>100.14</v>
       </c>
       <c r="C72" t="n">
-        <v>93.8</v>
+        <v>103.3</v>
       </c>
       <c r="D72" t="n">
-        <v>3.99</v>
+        <v>3.16</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CORDSCABLE</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>382.9</v>
+        <v>23.52</v>
       </c>
       <c r="C73" t="n">
-        <v>398</v>
+        <v>24.26</v>
       </c>
       <c r="D73" t="n">
-        <v>3.94</v>
+        <v>3.15</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ATLASCYCLE</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>93.55</v>
+        <v>254.85</v>
       </c>
       <c r="C74" t="n">
-        <v>97.15000000000001</v>
+        <v>262.8</v>
       </c>
       <c r="D74" t="n">
-        <v>3.85</v>
+        <v>3.12</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>SSRETAIL</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>36.6</v>
+        <v>748.8</v>
       </c>
       <c r="C75" t="n">
-        <v>38</v>
+        <v>771.95</v>
       </c>
       <c r="D75" t="n">
-        <v>3.83</v>
+        <v>3.09</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>12.29</v>
+        <v>44.08</v>
       </c>
       <c r="C76" t="n">
-        <v>12.76</v>
+        <v>45.44</v>
       </c>
       <c r="D76" t="n">
-        <v>3.82</v>
+        <v>3.09</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>20.22</v>
+        <v>68.41</v>
       </c>
       <c r="C77" t="n">
-        <v>20.99</v>
+        <v>70.5</v>
       </c>
       <c r="D77" t="n">
-        <v>3.81</v>
+        <v>3.06</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.79</v>
+        <v>24.85</v>
       </c>
       <c r="C78" t="n">
-        <v>0.82</v>
+        <v>25.6</v>
       </c>
       <c r="D78" t="n">
-        <v>3.8</v>
+        <v>3.02</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>5.01</v>
+        <v>24.95</v>
       </c>
       <c r="C79" t="n">
-        <v>5.2</v>
+        <v>25.7</v>
       </c>
       <c r="D79" t="n">
-        <v>3.79</v>
+        <v>3.01</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>RCDL</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>14.8</v>
+        <v>223.45</v>
       </c>
       <c r="C80" t="n">
-        <v>15.35</v>
+        <v>230</v>
       </c>
       <c r="D80" t="n">
-        <v>3.72</v>
+        <v>2.93</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>RAPPID</t>
+          <t>KSE</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>346.1</v>
+        <v>178.79</v>
       </c>
       <c r="C81" t="n">
-        <v>358.95</v>
+        <v>184</v>
       </c>
       <c r="D81" t="n">
-        <v>3.71</v>
+        <v>2.91</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AGIIL</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>269.3</v>
+        <v>26.87</v>
       </c>
       <c r="C82" t="n">
-        <v>279.15</v>
+        <v>27.65</v>
       </c>
       <c r="D82" t="n">
-        <v>3.66</v>
+        <v>2.9</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>MURUDCERA</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>636.8</v>
+        <v>29.06</v>
       </c>
       <c r="C83" t="n">
-        <v>660</v>
+        <v>29.9</v>
       </c>
       <c r="D83" t="n">
-        <v>3.64</v>
+        <v>2.89</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PRADPME</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>498.85</v>
+        <v>19.88</v>
       </c>
       <c r="C84" t="n">
-        <v>517</v>
+        <v>20.45</v>
       </c>
       <c r="D84" t="n">
-        <v>3.64</v>
+        <v>2.87</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DPWIRES</t>
+          <t>MAXESTATES</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>154.23</v>
+        <v>603.2</v>
       </c>
       <c r="C85" t="n">
-        <v>159.8</v>
+        <v>620.35</v>
       </c>
       <c r="D85" t="n">
-        <v>3.61</v>
+        <v>2.84</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>TECHNVISN</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>6.42</v>
+        <v>4181.5</v>
       </c>
       <c r="C86" t="n">
-        <v>6.65</v>
+        <v>4300</v>
       </c>
       <c r="D86" t="n">
-        <v>3.58</v>
+        <v>2.83</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LOYALTEX</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>214.95</v>
+        <v>0.71</v>
       </c>
       <c r="C87" t="n">
-        <v>222.55</v>
+        <v>0.73</v>
       </c>
       <c r="D87" t="n">
-        <v>3.54</v>
+        <v>2.82</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>30.91</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="C88" t="n">
-        <v>32</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="D88" t="n">
-        <v>3.53</v>
+        <v>2.8</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>PRIORITY</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>158.35</v>
+        <v>263.35</v>
       </c>
       <c r="C89" t="n">
-        <v>163.9</v>
+        <v>270.6</v>
       </c>
       <c r="D89" t="n">
-        <v>3.5</v>
+        <v>2.75</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>WCIL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>88.7</v>
+        <v>97.33</v>
       </c>
       <c r="C90" t="n">
-        <v>91.8</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="D90" t="n">
-        <v>3.49</v>
+        <v>2.73</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>50.06</v>
+        <v>1.83</v>
       </c>
       <c r="C91" t="n">
-        <v>51.8</v>
+        <v>1.88</v>
       </c>
       <c r="D91" t="n">
-        <v>3.48</v>
+        <v>2.73</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>WELSPUNLIV</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>221.51</v>
+        <v>5.92</v>
       </c>
       <c r="C92" t="n">
-        <v>229.2</v>
+        <v>6.08</v>
       </c>
       <c r="D92" t="n">
-        <v>3.47</v>
+        <v>2.7</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LAXMICOT</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>13.05</v>
+        <v>126.49</v>
       </c>
       <c r="C93" t="n">
-        <v>13.5</v>
+        <v>129.9</v>
       </c>
       <c r="D93" t="n">
-        <v>3.45</v>
+        <v>2.7</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>94.8</v>
+        <v>34.82</v>
       </c>
       <c r="C94" t="n">
-        <v>98</v>
+        <v>35.75</v>
       </c>
       <c r="D94" t="n">
-        <v>3.38</v>
+        <v>2.67</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>12.47</v>
+        <v>6.82</v>
       </c>
       <c r="C95" t="n">
-        <v>12.89</v>
+        <v>7</v>
       </c>
       <c r="D95" t="n">
-        <v>3.37</v>
+        <v>2.64</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>151.7</v>
+        <v>14.03</v>
       </c>
       <c r="C96" t="n">
-        <v>156.79</v>
+        <v>14.4</v>
       </c>
       <c r="D96" t="n">
-        <v>3.36</v>
+        <v>2.64</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.91</v>
+        <v>99.87</v>
       </c>
       <c r="C97" t="n">
-        <v>0.9399999999999999</v>
+        <v>102.5</v>
       </c>
       <c r="D97" t="n">
-        <v>3.3</v>
+        <v>2.63</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>33.35</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="C98" t="n">
-        <v>34.45</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="D98" t="n">
-        <v>3.3</v>
+        <v>2.63</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>14.51</v>
+        <v>21.34</v>
       </c>
       <c r="C99" t="n">
-        <v>14.98</v>
+        <v>21.9</v>
       </c>
       <c r="D99" t="n">
-        <v>3.24</v>
+        <v>2.62</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1022.2</v>
+        <v>13.53</v>
       </c>
       <c r="C100" t="n">
-        <v>1055</v>
+        <v>13.88</v>
       </c>
       <c r="D100" t="n">
-        <v>3.21</v>
+        <v>2.59</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>DCMSIL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>18.65</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="C101" t="n">
-        <v>19.24</v>
+        <v>79.45</v>
       </c>
       <c r="D101" t="n">
-        <v>3.16</v>
+        <v>2.57</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>LIBERTSHOE</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>867.65</v>
+        <v>235.48</v>
       </c>
       <c r="C102" t="n">
-        <v>895</v>
+        <v>241.4</v>
       </c>
       <c r="D102" t="n">
-        <v>3.15</v>
+        <v>2.51</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>MOLDTECH</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>28.81</v>
+        <v>199.88</v>
       </c>
       <c r="C103" t="n">
-        <v>29.7</v>
+        <v>204.9</v>
       </c>
       <c r="D103" t="n">
-        <v>3.09</v>
+        <v>2.51</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>663.55</v>
+        <v>1.6</v>
       </c>
       <c r="C104" t="n">
-        <v>684</v>
+        <v>1.64</v>
       </c>
       <c r="D104" t="n">
-        <v>3.08</v>
+        <v>2.5</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>JAYBARMARU</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>12.17</v>
+        <v>116.1</v>
       </c>
       <c r="C105" t="n">
-        <v>12.54</v>
+        <v>119</v>
       </c>
       <c r="D105" t="n">
-        <v>3.04</v>
+        <v>2.5</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>KEN</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>43</v>
+        <v>33.17</v>
       </c>
       <c r="C106" t="n">
-        <v>44.3</v>
+        <v>33.99</v>
       </c>
       <c r="D106" t="n">
-        <v>3.02</v>
+        <v>2.47</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>133.41</v>
+        <v>5.34</v>
       </c>
       <c r="C107" t="n">
-        <v>137.41</v>
+        <v>5.47</v>
       </c>
       <c r="D107" t="n">
-        <v>3</v>
+        <v>2.43</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>CYBERMEDIA</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>5.34</v>
+        <v>20.67</v>
       </c>
       <c r="C108" t="n">
-        <v>5.5</v>
+        <v>21.16</v>
       </c>
       <c r="D108" t="n">
-        <v>3</v>
+        <v>2.37</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>HBSL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>19.8</v>
+        <v>55.68</v>
       </c>
       <c r="C109" t="n">
-        <v>20.39</v>
+        <v>57</v>
       </c>
       <c r="D109" t="n">
-        <v>2.98</v>
+        <v>2.37</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ARROWGREEN</t>
+          <t>BIRLAPREC</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>913.05</v>
+        <v>56.67</v>
       </c>
       <c r="C110" t="n">
-        <v>940.05</v>
+        <v>58</v>
       </c>
       <c r="D110" t="n">
-        <v>2.96</v>
+        <v>2.35</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MANINDS</t>
+          <t>NATIONSTD</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>849.9</v>
+        <v>113.38</v>
       </c>
       <c r="C111" t="n">
-        <v>875</v>
+        <v>116</v>
       </c>
       <c r="D111" t="n">
-        <v>2.95</v>
+        <v>2.31</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>OMAXAUTO</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>665.35</v>
+        <v>209.94</v>
       </c>
       <c r="C112" t="n">
-        <v>685</v>
+        <v>214.69</v>
       </c>
       <c r="D112" t="n">
-        <v>2.95</v>
+        <v>2.26</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SOLEX</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>678.95</v>
+        <v>7.67</v>
       </c>
       <c r="C113" t="n">
-        <v>698.95</v>
+        <v>7.84</v>
       </c>
       <c r="D113" t="n">
-        <v>2.95</v>
+        <v>2.22</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>INNOVANA</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>295.3</v>
+        <v>0.45</v>
       </c>
       <c r="C114" t="n">
-        <v>304</v>
+        <v>0.46</v>
       </c>
       <c r="D114" t="n">
-        <v>2.95</v>
+        <v>2.22</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ABH</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>52.85</v>
+        <v>6.38</v>
       </c>
       <c r="C115" t="n">
-        <v>54.4</v>
+        <v>6.52</v>
       </c>
       <c r="D115" t="n">
-        <v>2.93</v>
+        <v>2.19</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>ORIANA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>18.43</v>
+        <v>308.3</v>
       </c>
       <c r="C116" t="n">
-        <v>18.97</v>
+        <v>315</v>
       </c>
       <c r="D116" t="n">
-        <v>2.93</v>
+        <v>2.17</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SHIVAAGRO</t>
+          <t>DANISH</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>40.03</v>
+        <v>1003.2</v>
       </c>
       <c r="C117" t="n">
-        <v>41.2</v>
+        <v>1025</v>
       </c>
       <c r="D117" t="n">
-        <v>2.92</v>
+        <v>2.17</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>SCPL</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>1996.7</v>
+        <v>650</v>
       </c>
       <c r="C118" t="n">
-        <v>2055</v>
+        <v>663.95</v>
       </c>
       <c r="D118" t="n">
-        <v>2.92</v>
+        <v>2.15</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>24.1</v>
+        <v>7.15</v>
       </c>
       <c r="C119" t="n">
-        <v>24.8</v>
+        <v>7.3</v>
       </c>
       <c r="D119" t="n">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>39.65</v>
+        <v>272.25</v>
       </c>
       <c r="C120" t="n">
-        <v>40.79</v>
+        <v>277.95</v>
       </c>
       <c r="D120" t="n">
-        <v>2.88</v>
+        <v>2.09</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>68.04000000000001</v>
+        <v>85.02</v>
       </c>
       <c r="C121" t="n">
-        <v>70</v>
+        <v>86.8</v>
       </c>
       <c r="D121" t="n">
-        <v>2.88</v>
+        <v>2.09</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>REGAAL</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>97.20999999999999</v>
+        <v>0.48</v>
       </c>
       <c r="C122" t="n">
-        <v>100</v>
+        <v>0.49</v>
       </c>
       <c r="D122" t="n">
-        <v>2.87</v>
+        <v>2.08</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>RPSGVENT</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>59.09</v>
+        <v>851.75</v>
       </c>
       <c r="C123" t="n">
-        <v>60.74</v>
+        <v>869</v>
       </c>
       <c r="D123" t="n">
-        <v>2.79</v>
+        <v>2.03</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>LKPSEC</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>33.08</v>
+        <v>15.27</v>
       </c>
       <c r="C124" t="n">
-        <v>34</v>
+        <v>15.58</v>
       </c>
       <c r="D124" t="n">
-        <v>2.78</v>
+        <v>2.03</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>BAGFILMS</t>
+          <t>DEVIT</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>4.31</v>
+        <v>23.24</v>
       </c>
       <c r="C125" t="n">
-        <v>4.43</v>
+        <v>23.71</v>
       </c>
       <c r="D125" t="n">
-        <v>2.78</v>
+        <v>2.02</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.36</v>
+        <v>5.98</v>
       </c>
       <c r="C126" t="n">
-        <v>0.37</v>
+        <v>6.1</v>
       </c>
       <c r="D126" t="n">
-        <v>2.78</v>
+        <v>2.01</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>AKG</t>
+          <t>STEELXIND</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>10.2</v>
+        <v>12.01</v>
       </c>
       <c r="C127" t="n">
-        <v>10.48</v>
+        <v>12.25</v>
       </c>
       <c r="D127" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>MALUPAPER</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>32.9</v>
+        <v>31.99</v>
       </c>
       <c r="C128" t="n">
-        <v>33.8</v>
+        <v>32.63</v>
       </c>
       <c r="D128" t="n">
-        <v>2.74</v>
+        <v>2</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>STYLAMIND</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>3309.4</v>
+        <v>438.69</v>
       </c>
       <c r="C129" t="n">
-        <v>3400</v>
+        <v>447.46</v>
       </c>
       <c r="D129" t="n">
-        <v>2.74</v>
+        <v>2</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>NRAIL</t>
+          <t>KALPATARU</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>652.1</v>
+        <v>272.55</v>
       </c>
       <c r="C130" t="n">
-        <v>669.85</v>
+        <v>278</v>
       </c>
       <c r="D130" t="n">
-        <v>2.72</v>
+        <v>2</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>MAHASTEEL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>24.35</v>
+        <v>1156.8</v>
       </c>
       <c r="C131" t="n">
-        <v>25</v>
+        <v>1179.8</v>
       </c>
       <c r="D131" t="n">
-        <v>2.67</v>
+        <v>1.99</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>THEMISMED</t>
+          <t>GVKPIL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>122.6</v>
+        <v>2.53</v>
       </c>
       <c r="C132" t="n">
-        <v>125.85</v>
+        <v>2.58</v>
       </c>
       <c r="D132" t="n">
-        <v>2.65</v>
+        <v>1.98</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>HINDADH</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>254.45</v>
+        <v>380.4</v>
       </c>
       <c r="C133" t="n">
-        <v>261.2</v>
+        <v>387.9</v>
       </c>
       <c r="D133" t="n">
-        <v>2.65</v>
+        <v>1.97</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>TEXINFRA</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>115.02</v>
+        <v>7.13</v>
       </c>
       <c r="C134" t="n">
-        <v>118.05</v>
+        <v>7.27</v>
       </c>
       <c r="D134" t="n">
-        <v>2.63</v>
+        <v>1.96</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>52.82</v>
+        <v>187.39</v>
       </c>
       <c r="C135" t="n">
-        <v>54.2</v>
+        <v>191</v>
       </c>
       <c r="D135" t="n">
-        <v>2.61</v>
+        <v>1.93</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>VOEPL</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>9.31</v>
+        <v>515.1</v>
       </c>
       <c r="C136" t="n">
-        <v>9.550000000000001</v>
+        <v>525</v>
       </c>
       <c r="D136" t="n">
-        <v>2.58</v>
+        <v>1.92</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1008.8</v>
+        <v>69.47</v>
       </c>
       <c r="C137" t="n">
-        <v>1034.7</v>
+        <v>70.8</v>
       </c>
       <c r="D137" t="n">
-        <v>2.57</v>
+        <v>1.91</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>LORDSCHLO</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>45.57</v>
+        <v>137.38</v>
       </c>
       <c r="C138" t="n">
-        <v>46.74</v>
+        <v>140</v>
       </c>
       <c r="D138" t="n">
-        <v>2.57</v>
+        <v>1.91</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>KAYA</t>
+          <t>AGL</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>338.35</v>
+        <v>14.22</v>
       </c>
       <c r="C139" t="n">
-        <v>347</v>
+        <v>14.49</v>
       </c>
       <c r="D139" t="n">
-        <v>2.56</v>
+        <v>1.9</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>BYKE</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1062.8</v>
+        <v>30.35</v>
       </c>
       <c r="C140" t="n">
-        <v>1089.9</v>
+        <v>30.92</v>
       </c>
       <c r="D140" t="n">
-        <v>2.55</v>
+        <v>1.88</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>PRAKASHSTL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>500.25</v>
+        <v>3.72</v>
       </c>
       <c r="C141" t="n">
-        <v>513</v>
+        <v>3.79</v>
       </c>
       <c r="D141" t="n">
-        <v>2.55</v>
+        <v>1.88</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>65.34999999999999</v>
+        <v>5.91</v>
       </c>
       <c r="C142" t="n">
-        <v>66.98999999999999</v>
+        <v>6.02</v>
       </c>
       <c r="D142" t="n">
-        <v>2.51</v>
+        <v>1.86</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>NATCAPSUQ</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>169</v>
+        <v>2.7</v>
       </c>
       <c r="C143" t="n">
-        <v>173.2</v>
+        <v>2.75</v>
       </c>
       <c r="D143" t="n">
-        <v>2.49</v>
+        <v>1.85</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>MCLOUD</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>25.18</v>
+        <v>0.54</v>
       </c>
       <c r="C144" t="n">
-        <v>25.8</v>
+        <v>0.55</v>
       </c>
       <c r="D144" t="n">
-        <v>2.46</v>
+        <v>1.85</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RKSWAMY</t>
+          <t>MILKYMIST</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>87.8</v>
+        <v>317.25</v>
       </c>
       <c r="C145" t="n">
-        <v>89.94</v>
+        <v>323</v>
       </c>
       <c r="D145" t="n">
-        <v>2.44</v>
+        <v>1.81</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>80.98</v>
+        <v>45.09</v>
       </c>
       <c r="C146" t="n">
-        <v>82.95</v>
+        <v>45.9</v>
       </c>
       <c r="D146" t="n">
-        <v>2.43</v>
+        <v>1.8</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>TATACAP</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>341.1</v>
+        <v>26.86</v>
       </c>
       <c r="C147" t="n">
-        <v>349.35</v>
+        <v>27.34</v>
       </c>
       <c r="D147" t="n">
-        <v>2.42</v>
+        <v>1.79</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>192.77</v>
+        <v>2.24</v>
       </c>
       <c r="C148" t="n">
-        <v>197.44</v>
+        <v>2.28</v>
       </c>
       <c r="D148" t="n">
-        <v>2.42</v>
+        <v>1.79</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>TRITONV</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>28.95</v>
+        <v>1133.8</v>
       </c>
       <c r="C149" t="n">
-        <v>29.65</v>
+        <v>1154</v>
       </c>
       <c r="D149" t="n">
-        <v>2.42</v>
+        <v>1.78</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>BSHSL</t>
+          <t>MANOMAY</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>85.64</v>
+        <v>224.48</v>
       </c>
       <c r="C150" t="n">
-        <v>87.7</v>
+        <v>228.48</v>
       </c>
       <c r="D150" t="n">
-        <v>2.41</v>
+        <v>1.78</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>DRONE</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>33.15</v>
+        <v>100.25</v>
       </c>
       <c r="C151" t="n">
-        <v>33.95</v>
+        <v>102</v>
       </c>
       <c r="D151" t="n">
-        <v>2.41</v>
+        <v>1.75</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>24.41</v>
+        <v>8.57</v>
       </c>
       <c r="C152" t="n">
-        <v>24.99</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="D152" t="n">
-        <v>2.38</v>
+        <v>1.75</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SAFEENTP</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>248.1</v>
+        <v>60.64</v>
       </c>
       <c r="C153" t="n">
-        <v>254</v>
+        <v>61.7</v>
       </c>
       <c r="D153" t="n">
-        <v>2.38</v>
+        <v>1.75</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>TECHD</t>
+          <t>EKI</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>556.8</v>
+        <v>82.54000000000001</v>
       </c>
       <c r="C154" t="n">
-        <v>570</v>
+        <v>83.98</v>
       </c>
       <c r="D154" t="n">
-        <v>2.37</v>
+        <v>1.74</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>IRB</t>
+          <t>LALITHAA</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>17.98</v>
+        <v>352.9</v>
       </c>
       <c r="C155" t="n">
-        <v>18.4</v>
+        <v>359</v>
       </c>
       <c r="D155" t="n">
-        <v>2.34</v>
+        <v>1.73</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SHRIAHIMSA</t>
+          <t>GAUDIUMIVF</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>473.95</v>
+        <v>117.69</v>
       </c>
       <c r="C156" t="n">
-        <v>485</v>
+        <v>119.7</v>
       </c>
       <c r="D156" t="n">
-        <v>2.33</v>
+        <v>1.71</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>40.07</v>
+        <v>1.17</v>
       </c>
       <c r="C157" t="n">
-        <v>41</v>
+        <v>1.19</v>
       </c>
       <c r="D157" t="n">
-        <v>2.32</v>
+        <v>1.71</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ROHLTD</t>
+          <t>ZUARIIND</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>306</v>
+        <v>278.9</v>
       </c>
       <c r="C158" t="n">
-        <v>313</v>
+        <v>283.65</v>
       </c>
       <c r="D158" t="n">
-        <v>2.29</v>
+        <v>1.7</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>EBIX</t>
+          <t>ATMASTCO</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>18.43</v>
+        <v>121.6</v>
       </c>
       <c r="C159" t="n">
-        <v>18.85</v>
+        <v>123.65</v>
       </c>
       <c r="D159" t="n">
-        <v>2.28</v>
+        <v>1.69</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>EMMBI</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>34.81</v>
+        <v>88.70999999999999</v>
       </c>
       <c r="C160" t="n">
-        <v>35.6</v>
+        <v>90.19</v>
       </c>
       <c r="D160" t="n">
-        <v>2.27</v>
+        <v>1.67</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MARALOVER</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>61.11</v>
+        <v>6.04</v>
       </c>
       <c r="C161" t="n">
-        <v>62.5</v>
+        <v>6.14</v>
       </c>
       <c r="D161" t="n">
-        <v>2.27</v>
+        <v>1.66</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MANBA</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>136.41</v>
+        <v>1780.6</v>
       </c>
       <c r="C162" t="n">
-        <v>139.48</v>
+        <v>1809.9</v>
       </c>
       <c r="D162" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>2.22</v>
+        <v>6.66</v>
       </c>
       <c r="C163" t="n">
-        <v>2.27</v>
+        <v>6.77</v>
       </c>
       <c r="D163" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>DICIND</t>
+          <t>KIRANVYPAR</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>654.25</v>
+        <v>215.1</v>
       </c>
       <c r="C164" t="n">
-        <v>669</v>
+        <v>218.65</v>
       </c>
       <c r="D164" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>ORIENTTECH</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>5.8</v>
+        <v>238.06</v>
       </c>
       <c r="C165" t="n">
-        <v>5.93</v>
+        <v>241.95</v>
       </c>
       <c r="D165" t="n">
-        <v>2.24</v>
+        <v>1.63</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>3BBLACKBIO</t>
+          <t>RKSWAMY</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>1369.3</v>
+        <v>92.45</v>
       </c>
       <c r="C166" t="n">
-        <v>1400</v>
+        <v>93.95</v>
       </c>
       <c r="D166" t="n">
-        <v>2.24</v>
+        <v>1.62</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>GUJAPOLLO</t>
+          <t>AMEYA</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>337.4</v>
+        <v>161.9</v>
       </c>
       <c r="C167" t="n">
-        <v>344.95</v>
+        <v>164.5</v>
       </c>
       <c r="D167" t="n">
-        <v>2.24</v>
+        <v>1.61</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>15.26</v>
+        <v>122.53</v>
       </c>
       <c r="C168" t="n">
-        <v>15.6</v>
+        <v>124.5</v>
       </c>
       <c r="D168" t="n">
-        <v>2.23</v>
+        <v>1.61</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>2.26</v>
+        <v>154.55</v>
       </c>
       <c r="C169" t="n">
-        <v>2.31</v>
+        <v>157</v>
       </c>
       <c r="D169" t="n">
-        <v>2.21</v>
+        <v>1.59</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ARIHANTCAP</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>90.98999999999999</v>
+        <v>543.35</v>
       </c>
       <c r="C170" t="n">
-        <v>93</v>
+        <v>552</v>
       </c>
       <c r="D170" t="n">
-        <v>2.21</v>
+        <v>1.59</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>THAKDEV</t>
+          <t>SIGNPOST</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>126.36</v>
+        <v>273.9</v>
       </c>
       <c r="C171" t="n">
-        <v>129.15</v>
+        <v>278.2</v>
       </c>
       <c r="D171" t="n">
-        <v>2.21</v>
+        <v>1.57</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>SURANAT&amp;P</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>32.24</v>
+        <v>16.04</v>
       </c>
       <c r="C172" t="n">
-        <v>32.95</v>
+        <v>16.29</v>
       </c>
       <c r="D172" t="n">
-        <v>2.2</v>
+        <v>1.56</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>PRESSTONIC</t>
+          <t>VIRAT</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>41.05</v>
+        <v>371.2</v>
       </c>
       <c r="C173" t="n">
-        <v>41.95</v>
+        <v>377</v>
       </c>
       <c r="D173" t="n">
-        <v>2.19</v>
+        <v>1.56</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>OSELDEVICE</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>5.04</v>
+        <v>404.65</v>
       </c>
       <c r="C174" t="n">
-        <v>5.15</v>
+        <v>410.95</v>
       </c>
       <c r="D174" t="n">
-        <v>2.18</v>
+        <v>1.56</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ASHUTOSH</t>
+          <t>SARLAPOLY</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>150.1</v>
+        <v>100.03</v>
       </c>
       <c r="C175" t="n">
-        <v>153.35</v>
+        <v>101.59</v>
       </c>
       <c r="D175" t="n">
-        <v>2.17</v>
+        <v>1.56</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>SILVER001</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>1.84</v>
+        <v>23.19</v>
       </c>
       <c r="C176" t="n">
-        <v>1.88</v>
+        <v>23.55</v>
       </c>
       <c r="D176" t="n">
-        <v>2.17</v>
+        <v>1.55</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>0.46</v>
+        <v>211.63</v>
       </c>
       <c r="C177" t="n">
-        <v>0.47</v>
+        <v>214.9</v>
       </c>
       <c r="D177" t="n">
-        <v>2.17</v>
+        <v>1.55</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>PARSVNATH</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>70.95999999999999</v>
+        <v>1.93</v>
       </c>
       <c r="C178" t="n">
-        <v>72.5</v>
+        <v>1.96</v>
       </c>
       <c r="D178" t="n">
-        <v>2.17</v>
+        <v>1.55</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>12.58</v>
+        <v>7.13</v>
       </c>
       <c r="C179" t="n">
-        <v>12.85</v>
+        <v>7.24</v>
       </c>
       <c r="D179" t="n">
-        <v>2.15</v>
+        <v>1.54</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>NDRAUTO</t>
+          <t>HLVLTD</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>753.2</v>
+        <v>6.59</v>
       </c>
       <c r="C180" t="n">
-        <v>769.4</v>
+        <v>6.69</v>
       </c>
       <c r="D180" t="n">
-        <v>2.15</v>
+        <v>1.52</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>1.86</v>
+        <v>27.78</v>
       </c>
       <c r="C181" t="n">
-        <v>1.9</v>
+        <v>28.2</v>
       </c>
       <c r="D181" t="n">
-        <v>2.15</v>
+        <v>1.51</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>HPAL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>13.6</v>
+        <v>35.65</v>
       </c>
       <c r="C182" t="n">
-        <v>13.89</v>
+        <v>36.19</v>
       </c>
       <c r="D182" t="n">
-        <v>2.13</v>
+        <v>1.51</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>KRISHANA</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>2.83</v>
+        <v>188.15</v>
       </c>
       <c r="C183" t="n">
-        <v>2.89</v>
+        <v>190.98</v>
       </c>
       <c r="D183" t="n">
-        <v>2.12</v>
+        <v>1.5</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>AERONEU</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>17.91</v>
+        <v>67.2</v>
       </c>
       <c r="C184" t="n">
-        <v>18.29</v>
+        <v>68.2</v>
       </c>
       <c r="D184" t="n">
-        <v>2.12</v>
+        <v>1.49</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>PANORAMA</t>
+          <t>VENTIVE</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>55.32</v>
+        <v>578.35</v>
       </c>
       <c r="C185" t="n">
-        <v>56.48</v>
+        <v>586.9</v>
       </c>
       <c r="D185" t="n">
-        <v>2.1</v>
+        <v>1.48</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ANDHRAPAP</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>71.43000000000001</v>
+        <v>137.46</v>
       </c>
       <c r="C186" t="n">
-        <v>72.92</v>
+        <v>139.5</v>
       </c>
       <c r="D186" t="n">
-        <v>2.09</v>
+        <v>1.48</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>OMINFRAL</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>78.93000000000001</v>
+        <v>3.39</v>
       </c>
       <c r="C187" t="n">
-        <v>80.58</v>
+        <v>3.44</v>
       </c>
       <c r="D187" t="n">
-        <v>2.09</v>
+        <v>1.47</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>KANOHAR</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>870.5</v>
+        <v>1.37</v>
       </c>
       <c r="C188" t="n">
-        <v>888.7</v>
+        <v>1.39</v>
       </c>
       <c r="D188" t="n">
-        <v>2.09</v>
+        <v>1.46</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>LANCORHOL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>30.14</v>
+        <v>34.97</v>
       </c>
       <c r="C189" t="n">
-        <v>30.77</v>
+        <v>35.48</v>
       </c>
       <c r="D189" t="n">
-        <v>2.09</v>
+        <v>1.46</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NILASPACES</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>12.02</v>
+        <v>35.96</v>
       </c>
       <c r="C190" t="n">
-        <v>12.27</v>
+        <v>36.48</v>
       </c>
       <c r="D190" t="n">
-        <v>2.08</v>
+        <v>1.45</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>JAYBEE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>4.35</v>
+        <v>95.05</v>
       </c>
       <c r="C191" t="n">
-        <v>4.44</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="D191" t="n">
-        <v>2.07</v>
+        <v>1.42</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ASHIMASYN</t>
+          <t>GHCL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>15.68</v>
+        <v>424</v>
       </c>
       <c r="C192" t="n">
-        <v>16</v>
+        <v>430</v>
       </c>
       <c r="D192" t="n">
-        <v>2.04</v>
+        <v>1.42</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>38.19</v>
+        <v>7.09</v>
       </c>
       <c r="C193" t="n">
-        <v>38.97</v>
+        <v>7.19</v>
       </c>
       <c r="D193" t="n">
-        <v>2.04</v>
+        <v>1.41</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>FERMENTA</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>2096.5</v>
+        <v>475.5</v>
       </c>
       <c r="C194" t="n">
-        <v>2139</v>
+        <v>482.2</v>
       </c>
       <c r="D194" t="n">
-        <v>2.03</v>
+        <v>1.41</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>AFSL</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>22.69</v>
+        <v>204.56</v>
       </c>
       <c r="C195" t="n">
-        <v>23.15</v>
+        <v>207.4</v>
       </c>
       <c r="D195" t="n">
-        <v>2.03</v>
+        <v>1.39</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>DIAMINESQ</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>254.85</v>
+        <v>5.02</v>
       </c>
       <c r="C196" t="n">
-        <v>260</v>
+        <v>5.09</v>
       </c>
       <c r="D196" t="n">
-        <v>2.02</v>
+        <v>1.39</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>MOHITE</t>
+          <t>AXITA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>2.47</v>
+        <v>8</v>
       </c>
       <c r="C197" t="n">
-        <v>2.52</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="D197" t="n">
-        <v>2.02</v>
+        <v>1.37</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>RAMAPHO</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>462.75</v>
+        <v>123.21</v>
       </c>
       <c r="C198" t="n">
-        <v>472.1</v>
+        <v>124.9</v>
       </c>
       <c r="D198" t="n">
-        <v>2.02</v>
+        <v>1.37</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>QUALIANCE</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>107.67</v>
+        <v>182.5</v>
       </c>
       <c r="C199" t="n">
-        <v>109.85</v>
+        <v>185</v>
       </c>
       <c r="D199" t="n">
-        <v>2.02</v>
+        <v>1.37</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>23.34</v>
+        <v>33.52</v>
       </c>
       <c r="C200" t="n">
-        <v>23.81</v>
+        <v>33.98</v>
       </c>
       <c r="D200" t="n">
-        <v>2.01</v>
+        <v>1.37</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>STERTOOLS</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>5.97</v>
+        <v>221.96</v>
       </c>
       <c r="C201" t="n">
-        <v>6.09</v>
+        <v>224.98</v>
       </c>
       <c r="D201" t="n">
-        <v>2.01</v>
+        <v>1.36</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-25 09:06 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POLYSPIN</t>
+          <t>CENTEXT-RE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>30.78</v>
+        <v>1.92</v>
       </c>
       <c r="C2" t="n">
-        <v>36.49</v>
+        <v>2.25</v>
       </c>
       <c r="D2" t="n">
-        <v>18.55</v>
+        <v>17.19</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>AERONEU</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>125.82</v>
+        <v>80.64</v>
       </c>
       <c r="C3" t="n">
-        <v>138.4</v>
+        <v>93</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>15.33</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CRESTO</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20.14</v>
+        <v>22.84</v>
       </c>
       <c r="C4" t="n">
-        <v>21.8</v>
+        <v>26</v>
       </c>
       <c r="D4" t="n">
-        <v>8.24</v>
+        <v>13.84</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TGBHOTELS</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.43</v>
+        <v>7.87</v>
       </c>
       <c r="C5" t="n">
-        <v>10.14</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>7.53</v>
+        <v>12.83</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MITCON</t>
+          <t>PANCHMAHQ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>82.62</v>
+        <v>305</v>
       </c>
       <c r="C6" t="n">
-        <v>88.5</v>
+        <v>339</v>
       </c>
       <c r="D6" t="n">
-        <v>7.12</v>
+        <v>11.15</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AASTHA</t>
+          <t>VASCONEQ</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>89.77</v>
+        <v>33.29</v>
       </c>
       <c r="C7" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="D7" t="n">
-        <v>6.94</v>
+        <v>11.14</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GKB</t>
+          <t>PARIN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>69.73</v>
+        <v>715</v>
       </c>
       <c r="C8" t="n">
-        <v>74</v>
+        <v>789</v>
       </c>
       <c r="D8" t="n">
-        <v>6.12</v>
+        <v>10.35</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>HEROMOTORS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.18</v>
+        <v>118.08</v>
       </c>
       <c r="C9" t="n">
-        <v>0.19</v>
+        <v>128</v>
       </c>
       <c r="D9" t="n">
-        <v>5.56</v>
+        <v>8.4</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ASIANTNE</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9.24</v>
+        <v>67.23999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>9.75</v>
+        <v>72.7</v>
       </c>
       <c r="D10" t="n">
-        <v>5.52</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>389</v>
+        <v>16.72</v>
       </c>
       <c r="C11" t="n">
-        <v>408.45</v>
+        <v>17.98</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>7.54</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126</v>
+        <v>0.14</v>
       </c>
       <c r="C12" t="n">
-        <v>132.3</v>
+        <v>0.15</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>7.14</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AKANKSHA</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>151.1</v>
+        <v>138.4</v>
       </c>
       <c r="C13" t="n">
-        <v>158.65</v>
+        <v>147.9</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>6.86</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>DUGLOBAL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>152.1</v>
+        <v>20.05</v>
       </c>
       <c r="C14" t="n">
-        <v>159.7</v>
+        <v>21.4</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>6.73</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SWARAJ</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>307.15</v>
+        <v>34.29</v>
       </c>
       <c r="C15" t="n">
-        <v>322.5</v>
+        <v>36.49</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>6.42</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AUROIMPEX</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>39</v>
+        <v>2.97</v>
       </c>
       <c r="C16" t="n">
-        <v>40.95</v>
+        <v>3.16</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>6.4</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>84.58</v>
+        <v>5.13</v>
       </c>
       <c r="C17" t="n">
-        <v>88.8</v>
+        <v>5.44</v>
       </c>
       <c r="D17" t="n">
-        <v>4.99</v>
+        <v>6.04</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>49.7</v>
+        <v>23.15</v>
       </c>
       <c r="C18" t="n">
-        <v>52.18</v>
+        <v>24.49</v>
       </c>
       <c r="D18" t="n">
-        <v>4.99</v>
+        <v>5.79</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>NAGREEKEXP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>29.44</v>
+        <v>24.02</v>
       </c>
       <c r="C19" t="n">
-        <v>30.91</v>
+        <v>25.4</v>
       </c>
       <c r="D19" t="n">
-        <v>4.99</v>
+        <v>5.75</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>11.05</v>
+        <v>60.62</v>
       </c>
       <c r="C20" t="n">
-        <v>11.6</v>
+        <v>64.05</v>
       </c>
       <c r="D20" t="n">
-        <v>4.98</v>
+        <v>5.66</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>29.1</v>
+        <v>0.18</v>
       </c>
       <c r="C21" t="n">
-        <v>30.55</v>
+        <v>0.19</v>
       </c>
       <c r="D21" t="n">
-        <v>4.98</v>
+        <v>5.56</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>ASIANTNE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5.83</v>
+        <v>9.19</v>
       </c>
       <c r="C22" t="n">
-        <v>6.12</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>4.97</v>
+        <v>5.55</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DEEM</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>47.3</v>
+        <v>66.3</v>
       </c>
       <c r="C23" t="n">
-        <v>49.65</v>
+        <v>69.92</v>
       </c>
       <c r="D23" t="n">
-        <v>4.97</v>
+        <v>5.46</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ARCL</t>
+          <t>LAMBODHARA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>255.79</v>
+        <v>139.46</v>
       </c>
       <c r="C24" t="n">
-        <v>268.5</v>
+        <v>147</v>
       </c>
       <c r="D24" t="n">
-        <v>4.97</v>
+        <v>5.41</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MARC</t>
+          <t>EKI</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>148.05</v>
+        <v>99.04000000000001</v>
       </c>
       <c r="C25" t="n">
-        <v>155.4</v>
+        <v>104.39</v>
       </c>
       <c r="D25" t="n">
-        <v>4.96</v>
+        <v>5.4</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>46.35</v>
+        <v>14.86</v>
       </c>
       <c r="C26" t="n">
-        <v>48.65</v>
+        <v>15.64</v>
       </c>
       <c r="D26" t="n">
-        <v>4.96</v>
+        <v>5.25</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>TCI</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3.84</v>
+        <v>833.45</v>
       </c>
       <c r="C27" t="n">
-        <v>4.03</v>
+        <v>877</v>
       </c>
       <c r="D27" t="n">
-        <v>4.95</v>
+        <v>5.23</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ARMOUR</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18.25</v>
+        <v>806.1</v>
       </c>
       <c r="C28" t="n">
-        <v>19.15</v>
+        <v>846.4</v>
       </c>
       <c r="D28" t="n">
-        <v>4.93</v>
+        <v>5</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>KILITCH</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>221.62</v>
+        <v>132.3</v>
       </c>
       <c r="C29" t="n">
-        <v>232.5</v>
+        <v>138.91</v>
       </c>
       <c r="D29" t="n">
-        <v>4.91</v>
+        <v>5</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RCDL</t>
+          <t>LALITHAA</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>15.5</v>
+        <v>370.5</v>
       </c>
       <c r="C30" t="n">
-        <v>16.25</v>
+        <v>389</v>
       </c>
       <c r="D30" t="n">
-        <v>4.84</v>
+        <v>4.99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>SPECTRAA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>34.81</v>
+        <v>235.4</v>
       </c>
       <c r="C31" t="n">
-        <v>36.48</v>
+        <v>247.15</v>
       </c>
       <c r="D31" t="n">
-        <v>4.8</v>
+        <v>4.99</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>ONIXSOLAR</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>55.3</v>
+        <v>321.8</v>
       </c>
       <c r="C32" t="n">
-        <v>57.95</v>
+        <v>337.85</v>
       </c>
       <c r="D32" t="n">
-        <v>4.79</v>
+        <v>4.99</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4.83</v>
+        <v>10.42</v>
       </c>
       <c r="C33" t="n">
-        <v>5.06</v>
+        <v>10.94</v>
       </c>
       <c r="D33" t="n">
-        <v>4.76</v>
+        <v>4.99</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NAGREEKEXP</t>
+          <t>METALIC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>24.21</v>
+        <v>171.7</v>
       </c>
       <c r="C34" t="n">
-        <v>25.35</v>
+        <v>180.25</v>
       </c>
       <c r="D34" t="n">
-        <v>4.71</v>
+        <v>4.98</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HEROMOTORS</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>98.40000000000001</v>
+        <v>30.91</v>
       </c>
       <c r="C35" t="n">
-        <v>103</v>
+        <v>32.45</v>
       </c>
       <c r="D35" t="n">
-        <v>4.67</v>
+        <v>4.98</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AVANTEL</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>146.17</v>
+        <v>159.7</v>
       </c>
       <c r="C36" t="n">
-        <v>153</v>
+        <v>167.65</v>
       </c>
       <c r="D36" t="n">
-        <v>4.67</v>
+        <v>4.98</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GOLDSTAR</t>
+          <t>SHRIKANHA</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>9.699999999999999</v>
+        <v>22.1</v>
       </c>
       <c r="C37" t="n">
-        <v>10.15</v>
+        <v>23.2</v>
       </c>
       <c r="D37" t="n">
-        <v>4.64</v>
+        <v>4.98</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SUPTANERY</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>10.65</v>
+        <v>22.29</v>
       </c>
       <c r="C38" t="n">
-        <v>11.14</v>
+        <v>23.4</v>
       </c>
       <c r="D38" t="n">
-        <v>4.6</v>
+        <v>4.98</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>AKANKSHA</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2.19</v>
+        <v>158.65</v>
       </c>
       <c r="C39" t="n">
-        <v>2.29</v>
+        <v>166.55</v>
       </c>
       <c r="D39" t="n">
-        <v>4.57</v>
+        <v>4.98</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2.85</v>
+        <v>20.72</v>
       </c>
       <c r="C40" t="n">
-        <v>2.98</v>
+        <v>21.75</v>
       </c>
       <c r="D40" t="n">
-        <v>4.56</v>
+        <v>4.97</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>NEXTMEDIA</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.88</v>
+        <v>3.62</v>
       </c>
       <c r="C41" t="n">
-        <v>0.92</v>
+        <v>3.8</v>
       </c>
       <c r="D41" t="n">
-        <v>4.55</v>
+        <v>4.97</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>491.85</v>
+        <v>4.03</v>
       </c>
       <c r="C42" t="n">
-        <v>513</v>
+        <v>4.23</v>
       </c>
       <c r="D42" t="n">
-        <v>4.3</v>
+        <v>4.96</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SMARTEN</t>
+          <t>NEUEON</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>62.25</v>
+        <v>13.71</v>
       </c>
       <c r="C43" t="n">
-        <v>64.90000000000001</v>
+        <v>14.39</v>
       </c>
       <c r="D43" t="n">
-        <v>4.26</v>
+        <v>4.96</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>VIKRAN</t>
+          <t>LAKSHYA</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>56.14</v>
+        <v>107.8</v>
       </c>
       <c r="C44" t="n">
-        <v>58.5</v>
+        <v>113.15</v>
       </c>
       <c r="D44" t="n">
-        <v>4.2</v>
+        <v>4.96</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LOYALTEX</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>231.23</v>
+        <v>10.91</v>
       </c>
       <c r="C45" t="n">
-        <v>240.9</v>
+        <v>11.45</v>
       </c>
       <c r="D45" t="n">
-        <v>4.18</v>
+        <v>4.95</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>GOLDSTAR</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>411.85</v>
+        <v>10.15</v>
       </c>
       <c r="C46" t="n">
-        <v>429</v>
+        <v>10.65</v>
       </c>
       <c r="D46" t="n">
-        <v>4.16</v>
+        <v>4.93</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>640.6</v>
+        <v>48.65</v>
       </c>
       <c r="C47" t="n">
-        <v>667</v>
+        <v>51.05</v>
       </c>
       <c r="D47" t="n">
-        <v>4.12</v>
+        <v>4.93</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>HITECHGEAR</t>
+          <t>RCDL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>560.95</v>
+        <v>16.25</v>
       </c>
       <c r="C48" t="n">
-        <v>584</v>
+        <v>17.05</v>
       </c>
       <c r="D48" t="n">
-        <v>4.11</v>
+        <v>4.92</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>FRONTSP</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1394.6</v>
+        <v>30.55</v>
       </c>
       <c r="C49" t="n">
-        <v>1451.8</v>
+        <v>32.05</v>
       </c>
       <c r="D49" t="n">
-        <v>4.1</v>
+        <v>4.91</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.44</v>
+        <v>5.91</v>
       </c>
       <c r="C50" t="n">
-        <v>2.54</v>
+        <v>6.2</v>
       </c>
       <c r="D50" t="n">
-        <v>4.1</v>
+        <v>4.91</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>93.09999999999999</v>
+        <v>6.12</v>
       </c>
       <c r="C51" t="n">
-        <v>96.90000000000001</v>
+        <v>6.42</v>
       </c>
       <c r="D51" t="n">
-        <v>4.08</v>
+        <v>4.9</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LAKSHYA</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>98</v>
+        <v>12.21</v>
       </c>
       <c r="C52" t="n">
-        <v>102</v>
+        <v>12.8</v>
       </c>
       <c r="D52" t="n">
-        <v>4.08</v>
+        <v>4.83</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RELTD</t>
+          <t>SWARAJ</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>149.36</v>
+        <v>322.5</v>
       </c>
       <c r="C53" t="n">
-        <v>155.4</v>
+        <v>338</v>
       </c>
       <c r="D53" t="n">
-        <v>4.04</v>
+        <v>4.81</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TIRUPATIFL</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>78.34</v>
+        <v>46.28</v>
       </c>
       <c r="C54" t="n">
-        <v>81.5</v>
+        <v>48.5</v>
       </c>
       <c r="D54" t="n">
-        <v>4.03</v>
+        <v>4.8</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5.25</v>
+        <v>2.29</v>
       </c>
       <c r="C55" t="n">
-        <v>5.46</v>
+        <v>2.4</v>
       </c>
       <c r="D55" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>EASTSILK</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>68.51000000000001</v>
+        <v>52.01</v>
       </c>
       <c r="C56" t="n">
-        <v>71.25</v>
+        <v>54.5</v>
       </c>
       <c r="D56" t="n">
-        <v>4</v>
+        <v>4.79</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>REFRACTORY</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>36.55</v>
+        <v>111.12</v>
       </c>
       <c r="C57" t="n">
-        <v>38</v>
+        <v>116.4</v>
       </c>
       <c r="D57" t="n">
-        <v>3.97</v>
+        <v>4.75</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>VITAL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>6.74</v>
+        <v>54.37</v>
       </c>
       <c r="C58" t="n">
-        <v>7</v>
+        <v>56.94</v>
       </c>
       <c r="D58" t="n">
-        <v>3.86</v>
+        <v>4.73</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AURUS</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>4.67</v>
+        <v>1.69</v>
       </c>
       <c r="C59" t="n">
-        <v>4.85</v>
+        <v>1.77</v>
       </c>
       <c r="D59" t="n">
-        <v>3.85</v>
+        <v>4.73</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AZADIND</t>
+          <t>STERTOOLS</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>80.93000000000001</v>
+        <v>233.05</v>
       </c>
       <c r="C60" t="n">
-        <v>84</v>
+        <v>244</v>
       </c>
       <c r="D60" t="n">
-        <v>3.79</v>
+        <v>4.7</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>APOORVA</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>34.32</v>
+        <v>7.65</v>
       </c>
       <c r="C61" t="n">
-        <v>35.58</v>
+        <v>8</v>
       </c>
       <c r="D61" t="n">
-        <v>3.67</v>
+        <v>4.58</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AMBALALSA</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>40.47</v>
+        <v>4.45</v>
       </c>
       <c r="C62" t="n">
-        <v>41.94</v>
+        <v>4.65</v>
       </c>
       <c r="D62" t="n">
-        <v>3.63</v>
+        <v>4.49</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>VGCL</t>
+          <t>DELTAMAGNT</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>47.18</v>
+        <v>54.45</v>
       </c>
       <c r="C63" t="n">
-        <v>48.89</v>
+        <v>56.89</v>
       </c>
       <c r="D63" t="n">
-        <v>3.62</v>
+        <v>4.48</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>29.93</v>
+        <v>22.02</v>
       </c>
       <c r="C64" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D64" t="n">
-        <v>3.58</v>
+        <v>4.45</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>SUPERSPIN</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.28</v>
+        <v>7.65</v>
       </c>
       <c r="C65" t="n">
-        <v>0.29</v>
+        <v>7.99</v>
       </c>
       <c r="D65" t="n">
-        <v>3.57</v>
+        <v>4.44</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>5.7</v>
+        <v>12.68</v>
       </c>
       <c r="C66" t="n">
-        <v>5.9</v>
+        <v>13.24</v>
       </c>
       <c r="D66" t="n">
-        <v>3.51</v>
+        <v>4.42</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>LCCPROJECT</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>18.22</v>
+        <v>144.22</v>
       </c>
       <c r="C67" t="n">
-        <v>18.84</v>
+        <v>150.5</v>
       </c>
       <c r="D67" t="n">
-        <v>3.4</v>
+        <v>4.35</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>30.25</v>
+        <v>0.47</v>
       </c>
       <c r="C68" t="n">
-        <v>31.25</v>
+        <v>0.49</v>
       </c>
       <c r="D68" t="n">
-        <v>3.31</v>
+        <v>4.26</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>19.04</v>
+        <v>267.55</v>
       </c>
       <c r="C69" t="n">
-        <v>19.67</v>
+        <v>278.8</v>
       </c>
       <c r="D69" t="n">
-        <v>3.31</v>
+        <v>4.2</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>4.28</v>
+        <v>196.75</v>
       </c>
       <c r="C70" t="n">
-        <v>4.42</v>
+        <v>205</v>
       </c>
       <c r="D70" t="n">
-        <v>3.27</v>
+        <v>4.19</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>12.5</v>
+        <v>14.38</v>
       </c>
       <c r="C71" t="n">
-        <v>12.9</v>
+        <v>14.98</v>
       </c>
       <c r="D71" t="n">
-        <v>3.2</v>
+        <v>4.17</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ANSALBU</t>
+          <t>NAGREEKCAP</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>100.14</v>
+        <v>29.55</v>
       </c>
       <c r="C72" t="n">
-        <v>103.3</v>
+        <v>30.75</v>
       </c>
       <c r="D72" t="n">
-        <v>3.16</v>
+        <v>4.06</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>LANCORHOL</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>23.52</v>
+        <v>34.03</v>
       </c>
       <c r="C73" t="n">
-        <v>24.26</v>
+        <v>35.4</v>
       </c>
       <c r="D73" t="n">
-        <v>3.15</v>
+        <v>4.03</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>ARTEMISMED</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>254.85</v>
+        <v>332.7</v>
       </c>
       <c r="C74" t="n">
-        <v>262.8</v>
+        <v>346</v>
       </c>
       <c r="D74" t="n">
-        <v>3.12</v>
+        <v>4</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SSRETAIL</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>748.8</v>
+        <v>17.89</v>
       </c>
       <c r="C75" t="n">
-        <v>771.95</v>
+        <v>18.6</v>
       </c>
       <c r="D75" t="n">
-        <v>3.09</v>
+        <v>3.97</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>BLUECLOUDS</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>44.08</v>
+        <v>20.06</v>
       </c>
       <c r="C76" t="n">
-        <v>45.44</v>
+        <v>20.85</v>
       </c>
       <c r="D76" t="n">
-        <v>3.09</v>
+        <v>3.94</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>68.41</v>
+        <v>46.11</v>
       </c>
       <c r="C77" t="n">
-        <v>70.5</v>
+        <v>47.9</v>
       </c>
       <c r="D77" t="n">
-        <v>3.06</v>
+        <v>3.88</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>24.85</v>
+        <v>41.27</v>
       </c>
       <c r="C78" t="n">
-        <v>25.6</v>
+        <v>42.85</v>
       </c>
       <c r="D78" t="n">
-        <v>3.02</v>
+        <v>3.83</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>COOLCAPS</t>
+          <t>GENESYS</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>24.95</v>
+        <v>283.18</v>
       </c>
       <c r="C79" t="n">
-        <v>25.7</v>
+        <v>294.03</v>
       </c>
       <c r="D79" t="n">
-        <v>3.01</v>
+        <v>3.83</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>223.45</v>
+        <v>162.33</v>
       </c>
       <c r="C80" t="n">
-        <v>230</v>
+        <v>168.5</v>
       </c>
       <c r="D80" t="n">
-        <v>2.93</v>
+        <v>3.8</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>KSE</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>178.79</v>
+        <v>9.81</v>
       </c>
       <c r="C81" t="n">
-        <v>184</v>
+        <v>10.18</v>
       </c>
       <c r="D81" t="n">
-        <v>2.91</v>
+        <v>3.77</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>VTMLTD</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>26.87</v>
+        <v>42.13</v>
       </c>
       <c r="C82" t="n">
-        <v>27.65</v>
+        <v>43.7</v>
       </c>
       <c r="D82" t="n">
-        <v>2.9</v>
+        <v>3.73</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MURUDCERA</t>
+          <t>QUESTLAB</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>29.06</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="C83" t="n">
-        <v>29.9</v>
+        <v>93.45</v>
       </c>
       <c r="D83" t="n">
-        <v>2.89</v>
+        <v>3.72</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>VIRAT</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>19.88</v>
+        <v>361.55</v>
       </c>
       <c r="C84" t="n">
-        <v>20.45</v>
+        <v>374.9</v>
       </c>
       <c r="D84" t="n">
-        <v>2.87</v>
+        <v>3.69</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MAXESTATES</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>603.2</v>
+        <v>6.85</v>
       </c>
       <c r="C85" t="n">
-        <v>620.35</v>
+        <v>7.1</v>
       </c>
       <c r="D85" t="n">
-        <v>2.84</v>
+        <v>3.65</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TECHNVISN</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>4181.5</v>
+        <v>4.96</v>
       </c>
       <c r="C86" t="n">
-        <v>4300</v>
+        <v>5.14</v>
       </c>
       <c r="D86" t="n">
-        <v>2.83</v>
+        <v>3.63</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.71</v>
+        <v>2180.8</v>
       </c>
       <c r="C87" t="n">
-        <v>0.73</v>
+        <v>2260</v>
       </c>
       <c r="D87" t="n">
-        <v>2.82</v>
+        <v>3.63</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>8.220000000000001</v>
+        <v>0.28</v>
       </c>
       <c r="C88" t="n">
-        <v>8.449999999999999</v>
+        <v>0.29</v>
       </c>
       <c r="D88" t="n">
-        <v>2.8</v>
+        <v>3.57</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PRIORITY</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>263.35</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="C89" t="n">
-        <v>270.6</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="D89" t="n">
-        <v>2.75</v>
+        <v>3.56</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>WCIL</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>97.33</v>
+        <v>4.21</v>
       </c>
       <c r="C90" t="n">
-        <v>99.98999999999999</v>
+        <v>4.36</v>
       </c>
       <c r="D90" t="n">
-        <v>2.73</v>
+        <v>3.56</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>MAHASTEEL</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1.83</v>
+        <v>1211.9</v>
       </c>
       <c r="C91" t="n">
-        <v>1.88</v>
+        <v>1255</v>
       </c>
       <c r="D91" t="n">
-        <v>2.73</v>
+        <v>3.56</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>DURLAX</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>5.92</v>
+        <v>60.55</v>
       </c>
       <c r="C92" t="n">
-        <v>6.08</v>
+        <v>62.7</v>
       </c>
       <c r="D92" t="n">
-        <v>2.7</v>
+        <v>3.55</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>KOHINOOR</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>126.49</v>
+        <v>30.82</v>
       </c>
       <c r="C93" t="n">
-        <v>129.9</v>
+        <v>31.9</v>
       </c>
       <c r="D93" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>LOYALTEX</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>34.82</v>
+        <v>223.98</v>
       </c>
       <c r="C94" t="n">
-        <v>35.75</v>
+        <v>231.8</v>
       </c>
       <c r="D94" t="n">
-        <v>2.67</v>
+        <v>3.49</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>NILAINFRA</t>
+          <t>SWARNSAR</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>6.82</v>
+        <v>42.04</v>
       </c>
       <c r="C95" t="n">
-        <v>7</v>
+        <v>43.5</v>
       </c>
       <c r="D95" t="n">
-        <v>2.64</v>
+        <v>3.47</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SWISSMLTRY</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>14.03</v>
+        <v>70.56</v>
       </c>
       <c r="C96" t="n">
-        <v>14.4</v>
+        <v>73</v>
       </c>
       <c r="D96" t="n">
-        <v>2.64</v>
+        <v>3.46</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>99.87</v>
+        <v>7.02</v>
       </c>
       <c r="C97" t="n">
-        <v>102.5</v>
+        <v>7.26</v>
       </c>
       <c r="D97" t="n">
-        <v>2.63</v>
+        <v>3.42</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>9.130000000000001</v>
+        <v>10.25</v>
       </c>
       <c r="C98" t="n">
-        <v>9.369999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="D98" t="n">
-        <v>2.63</v>
+        <v>3.41</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>21.34</v>
+        <v>432.4</v>
       </c>
       <c r="C99" t="n">
-        <v>21.9</v>
+        <v>447</v>
       </c>
       <c r="D99" t="n">
-        <v>2.62</v>
+        <v>3.38</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>13.53</v>
+        <v>11.6</v>
       </c>
       <c r="C100" t="n">
-        <v>13.88</v>
+        <v>11.99</v>
       </c>
       <c r="D100" t="n">
-        <v>2.59</v>
+        <v>3.36</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DCMSIL</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>77.45999999999999</v>
+        <v>5.69</v>
       </c>
       <c r="C101" t="n">
-        <v>79.45</v>
+        <v>5.88</v>
       </c>
       <c r="D101" t="n">
-        <v>2.57</v>
+        <v>3.34</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>LIBERTSHOE</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>235.48</v>
+        <v>13.31</v>
       </c>
       <c r="C102" t="n">
-        <v>241.4</v>
+        <v>13.75</v>
       </c>
       <c r="D102" t="n">
-        <v>2.51</v>
+        <v>3.31</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MOLDTECH</t>
+          <t>DCMSIL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>199.88</v>
+        <v>85.2</v>
       </c>
       <c r="C103" t="n">
-        <v>204.9</v>
+        <v>88</v>
       </c>
       <c r="D103" t="n">
-        <v>2.51</v>
+        <v>3.29</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>NATIONSTD</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>1.6</v>
+        <v>115.11</v>
       </c>
       <c r="C104" t="n">
-        <v>1.64</v>
+        <v>118.9</v>
       </c>
       <c r="D104" t="n">
-        <v>2.5</v>
+        <v>3.29</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>JAYBARMARU</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>116.1</v>
+        <v>231.58</v>
       </c>
       <c r="C105" t="n">
-        <v>119</v>
+        <v>239</v>
       </c>
       <c r="D105" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>JAYBARMARU</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>33.17</v>
+        <v>121.9</v>
       </c>
       <c r="C106" t="n">
-        <v>33.99</v>
+        <v>125.8</v>
       </c>
       <c r="D106" t="n">
-        <v>2.47</v>
+        <v>3.2</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>5.34</v>
+        <v>177.35</v>
       </c>
       <c r="C107" t="n">
-        <v>5.47</v>
+        <v>183</v>
       </c>
       <c r="D107" t="n">
-        <v>2.43</v>
+        <v>3.19</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CYBERMEDIA</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>20.67</v>
+        <v>58.05</v>
       </c>
       <c r="C108" t="n">
-        <v>21.16</v>
+        <v>59.9</v>
       </c>
       <c r="D108" t="n">
-        <v>2.37</v>
+        <v>3.19</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>HBSL</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>55.68</v>
+        <v>12.31</v>
       </c>
       <c r="C109" t="n">
-        <v>57</v>
+        <v>12.7</v>
       </c>
       <c r="D109" t="n">
-        <v>2.37</v>
+        <v>3.17</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BIRLAPREC</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>56.67</v>
+        <v>249.6</v>
       </c>
       <c r="C110" t="n">
-        <v>58</v>
+        <v>257.45</v>
       </c>
       <c r="D110" t="n">
-        <v>2.35</v>
+        <v>3.15</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>NATIONSTD</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>113.38</v>
+        <v>17.13</v>
       </c>
       <c r="C111" t="n">
-        <v>116</v>
+        <v>17.67</v>
       </c>
       <c r="D111" t="n">
-        <v>2.31</v>
+        <v>3.15</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>DENTA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>209.94</v>
+        <v>270.1</v>
       </c>
       <c r="C112" t="n">
-        <v>214.69</v>
+        <v>278.55</v>
       </c>
       <c r="D112" t="n">
-        <v>2.26</v>
+        <v>3.13</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>7.67</v>
+        <v>153.13</v>
       </c>
       <c r="C113" t="n">
-        <v>7.84</v>
+        <v>157.9</v>
       </c>
       <c r="D113" t="n">
-        <v>2.22</v>
+        <v>3.12</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.45</v>
+        <v>49.9</v>
       </c>
       <c r="C114" t="n">
-        <v>0.46</v>
+        <v>51.4</v>
       </c>
       <c r="D114" t="n">
-        <v>2.22</v>
+        <v>3.01</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>6.38</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="C115" t="n">
-        <v>6.52</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D115" t="n">
-        <v>2.19</v>
+        <v>2.99</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ORIANA</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>308.3</v>
+        <v>659.4</v>
       </c>
       <c r="C116" t="n">
-        <v>315</v>
+        <v>679</v>
       </c>
       <c r="D116" t="n">
-        <v>2.17</v>
+        <v>2.97</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>DANISH</t>
+          <t>AJAXENGG</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>1003.2</v>
+        <v>575.2</v>
       </c>
       <c r="C117" t="n">
-        <v>1025</v>
+        <v>592</v>
       </c>
       <c r="D117" t="n">
-        <v>2.17</v>
+        <v>2.92</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SCPL</t>
+          <t>INDOMIM</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>650</v>
+        <v>1311.15</v>
       </c>
       <c r="C118" t="n">
-        <v>663.95</v>
+        <v>1349</v>
       </c>
       <c r="D118" t="n">
-        <v>2.15</v>
+        <v>2.89</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>7.15</v>
+        <v>5.93</v>
       </c>
       <c r="C119" t="n">
-        <v>7.3</v>
+        <v>6.1</v>
       </c>
       <c r="D119" t="n">
-        <v>2.1</v>
+        <v>2.87</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>PACIFICI</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>272.25</v>
+        <v>136.14</v>
       </c>
       <c r="C120" t="n">
-        <v>277.95</v>
+        <v>140</v>
       </c>
       <c r="D120" t="n">
-        <v>2.09</v>
+        <v>2.84</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>LAKSHMIMIL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>85.02</v>
+        <v>7780.5</v>
       </c>
       <c r="C121" t="n">
-        <v>86.8</v>
+        <v>8001</v>
       </c>
       <c r="D121" t="n">
-        <v>2.09</v>
+        <v>2.83</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>ATALREAL</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.48</v>
+        <v>14.6</v>
       </c>
       <c r="C122" t="n">
-        <v>0.49</v>
+        <v>15.01</v>
       </c>
       <c r="D122" t="n">
-        <v>2.08</v>
+        <v>2.81</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RPSGVENT</t>
+          <t>NGLFINE</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>851.75</v>
+        <v>2894.9</v>
       </c>
       <c r="C123" t="n">
-        <v>869</v>
+        <v>2975.5</v>
       </c>
       <c r="D123" t="n">
-        <v>2.03</v>
+        <v>2.78</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LKPSEC</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>15.27</v>
+        <v>0.36</v>
       </c>
       <c r="C124" t="n">
-        <v>15.58</v>
+        <v>0.37</v>
       </c>
       <c r="D124" t="n">
-        <v>2.03</v>
+        <v>2.78</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DEVIT</t>
+          <t>AEROPLANE</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>23.24</v>
+        <v>201.98</v>
       </c>
       <c r="C125" t="n">
-        <v>23.71</v>
+        <v>207.55</v>
       </c>
       <c r="D125" t="n">
-        <v>2.02</v>
+        <v>2.76</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5.98</v>
+        <v>306</v>
       </c>
       <c r="C126" t="n">
-        <v>6.1</v>
+        <v>314.4</v>
       </c>
       <c r="D126" t="n">
-        <v>2.01</v>
+        <v>2.75</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>STEELXIND</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>12.01</v>
+        <v>12.02</v>
       </c>
       <c r="C127" t="n">
-        <v>12.25</v>
+        <v>12.35</v>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MALUPAPER</t>
+          <t>XCHANGING</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>31.99</v>
+        <v>60.35</v>
       </c>
       <c r="C128" t="n">
-        <v>32.63</v>
+        <v>62</v>
       </c>
       <c r="D128" t="n">
-        <v>2</v>
+        <v>2.73</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>KANDARP</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>438.69</v>
+        <v>76.95</v>
       </c>
       <c r="C129" t="n">
-        <v>447.46</v>
+        <v>79.05</v>
       </c>
       <c r="D129" t="n">
-        <v>2</v>
+        <v>2.73</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>KALPATARU</t>
+          <t>JISLDVREQS</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>272.55</v>
+        <v>20.14</v>
       </c>
       <c r="C130" t="n">
-        <v>278</v>
+        <v>20.69</v>
       </c>
       <c r="D130" t="n">
-        <v>2</v>
+        <v>2.73</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MAHASTEEL</t>
+          <t>ALKALI</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>1156.8</v>
+        <v>96.37</v>
       </c>
       <c r="C131" t="n">
-        <v>1179.8</v>
+        <v>98.98999999999999</v>
       </c>
       <c r="D131" t="n">
-        <v>1.99</v>
+        <v>2.72</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>GVKPIL</t>
+          <t>NARMADA</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>2.53</v>
+        <v>13.24</v>
       </c>
       <c r="C132" t="n">
-        <v>2.58</v>
+        <v>13.6</v>
       </c>
       <c r="D132" t="n">
-        <v>1.98</v>
+        <v>2.72</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>HINDADH</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>380.4</v>
+        <v>18.99</v>
       </c>
       <c r="C133" t="n">
-        <v>387.9</v>
+        <v>19.5</v>
       </c>
       <c r="D133" t="n">
-        <v>1.97</v>
+        <v>2.69</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>LORDSCHLO</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>7.13</v>
+        <v>134.5</v>
       </c>
       <c r="C134" t="n">
-        <v>7.27</v>
+        <v>138.1</v>
       </c>
       <c r="D134" t="n">
-        <v>1.96</v>
+        <v>2.68</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>187.39</v>
+        <v>949.65</v>
       </c>
       <c r="C135" t="n">
-        <v>191</v>
+        <v>974.9</v>
       </c>
       <c r="D135" t="n">
-        <v>1.93</v>
+        <v>2.66</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VOEPL</t>
+          <t>HSBCGOLD</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>515.1</v>
+        <v>130.3</v>
       </c>
       <c r="C136" t="n">
-        <v>525</v>
+        <v>133.75</v>
       </c>
       <c r="D136" t="n">
-        <v>1.92</v>
+        <v>2.65</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>OMFREIGHT</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>69.47</v>
+        <v>91.83</v>
       </c>
       <c r="C137" t="n">
-        <v>70.8</v>
+        <v>94.25</v>
       </c>
       <c r="D137" t="n">
-        <v>1.91</v>
+        <v>2.64</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LORDSCHLO</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>137.38</v>
+        <v>49.59</v>
       </c>
       <c r="C138" t="n">
-        <v>140</v>
+        <v>50.9</v>
       </c>
       <c r="D138" t="n">
-        <v>1.91</v>
+        <v>2.64</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>AGL</t>
+          <t>STEAMHOUSE</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>14.22</v>
+        <v>113.71</v>
       </c>
       <c r="C139" t="n">
-        <v>14.49</v>
+        <v>116.7</v>
       </c>
       <c r="D139" t="n">
-        <v>1.9</v>
+        <v>2.63</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>BYKE</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>30.35</v>
+        <v>80.39</v>
       </c>
       <c r="C140" t="n">
-        <v>30.92</v>
+        <v>82.5</v>
       </c>
       <c r="D140" t="n">
-        <v>1.88</v>
+        <v>2.62</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>PRAKASHSTL</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>3.72</v>
+        <v>14.11</v>
       </c>
       <c r="C141" t="n">
-        <v>3.79</v>
+        <v>14.48</v>
       </c>
       <c r="D141" t="n">
-        <v>1.88</v>
+        <v>2.62</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>5.91</v>
+        <v>34.93</v>
       </c>
       <c r="C142" t="n">
-        <v>6.02</v>
+        <v>35.84</v>
       </c>
       <c r="D142" t="n">
-        <v>1.86</v>
+        <v>2.61</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>2.7</v>
+        <v>89.27</v>
       </c>
       <c r="C143" t="n">
-        <v>2.75</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="D143" t="n">
-        <v>1.85</v>
+        <v>2.61</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>0.54</v>
+        <v>33.82</v>
       </c>
       <c r="C144" t="n">
-        <v>0.55</v>
+        <v>34.7</v>
       </c>
       <c r="D144" t="n">
-        <v>1.85</v>
+        <v>2.6</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>MILKYMIST</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>317.25</v>
+        <v>53.9</v>
       </c>
       <c r="C145" t="n">
-        <v>323</v>
+        <v>55.3</v>
       </c>
       <c r="D145" t="n">
-        <v>1.81</v>
+        <v>2.6</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>45.09</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="C146" t="n">
-        <v>45.9</v>
+        <v>8.75</v>
       </c>
       <c r="D146" t="n">
-        <v>1.8</v>
+        <v>2.58</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>ZFSTEERING</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>26.86</v>
+        <v>746.1</v>
       </c>
       <c r="C147" t="n">
-        <v>27.34</v>
+        <v>765</v>
       </c>
       <c r="D147" t="n">
-        <v>1.79</v>
+        <v>2.53</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>2.24</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="C148" t="n">
-        <v>2.28</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="D148" t="n">
-        <v>1.79</v>
+        <v>2.52</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>TRITONV</t>
+          <t>AVANCE</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>1133.8</v>
+        <v>0.8</v>
       </c>
       <c r="C149" t="n">
-        <v>1154</v>
+        <v>0.82</v>
       </c>
       <c r="D149" t="n">
-        <v>1.78</v>
+        <v>2.5</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MANOMAY</t>
+          <t>WAKEFIT</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>224.48</v>
+        <v>142.83</v>
       </c>
       <c r="C150" t="n">
-        <v>228.48</v>
+        <v>146.37</v>
       </c>
       <c r="D150" t="n">
-        <v>1.78</v>
+        <v>2.48</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>100.25</v>
+        <v>12.19</v>
       </c>
       <c r="C151" t="n">
-        <v>102</v>
+        <v>12.49</v>
       </c>
       <c r="D151" t="n">
-        <v>1.75</v>
+        <v>2.46</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>ARCHIES</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>8.57</v>
+        <v>12.66</v>
       </c>
       <c r="C152" t="n">
-        <v>8.720000000000001</v>
+        <v>12.97</v>
       </c>
       <c r="D152" t="n">
-        <v>1.75</v>
+        <v>2.45</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>60.64</v>
+        <v>69.31</v>
       </c>
       <c r="C153" t="n">
-        <v>61.7</v>
+        <v>71</v>
       </c>
       <c r="D153" t="n">
-        <v>1.75</v>
+        <v>2.44</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>EKI</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>82.54000000000001</v>
+        <v>26.36</v>
       </c>
       <c r="C154" t="n">
-        <v>83.98</v>
+        <v>27</v>
       </c>
       <c r="D154" t="n">
-        <v>1.74</v>
+        <v>2.43</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>LALITHAA</t>
+          <t>VETO</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>352.9</v>
+        <v>143.04</v>
       </c>
       <c r="C155" t="n">
-        <v>359</v>
+        <v>146.5</v>
       </c>
       <c r="D155" t="n">
-        <v>1.73</v>
+        <v>2.42</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>GAUDIUMIVF</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>117.69</v>
+        <v>5.81</v>
       </c>
       <c r="C156" t="n">
-        <v>119.7</v>
+        <v>5.95</v>
       </c>
       <c r="D156" t="n">
-        <v>1.71</v>
+        <v>2.41</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>1.17</v>
+        <v>16.58</v>
       </c>
       <c r="C157" t="n">
-        <v>1.19</v>
+        <v>16.98</v>
       </c>
       <c r="D157" t="n">
-        <v>1.71</v>
+        <v>2.41</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ZUARIIND</t>
+          <t>MANOMAY</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>278.9</v>
+        <v>233.21</v>
       </c>
       <c r="C158" t="n">
-        <v>283.65</v>
+        <v>238.8</v>
       </c>
       <c r="D158" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ATMASTCO</t>
+          <t>ORIANA</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>121.6</v>
+        <v>303.7</v>
       </c>
       <c r="C159" t="n">
-        <v>123.65</v>
+        <v>311</v>
       </c>
       <c r="D159" t="n">
-        <v>1.69</v>
+        <v>2.4</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>EMMBI</t>
+          <t>DRONE</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>88.70999999999999</v>
+        <v>33.6</v>
       </c>
       <c r="C160" t="n">
-        <v>90.19</v>
+        <v>34.4</v>
       </c>
       <c r="D160" t="n">
-        <v>1.67</v>
+        <v>2.38</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>6.04</v>
+        <v>25.18</v>
       </c>
       <c r="C161" t="n">
-        <v>6.14</v>
+        <v>25.78</v>
       </c>
       <c r="D161" t="n">
-        <v>1.66</v>
+        <v>2.38</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SASKEN</t>
+          <t>KECL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>1780.6</v>
+        <v>122.75</v>
       </c>
       <c r="C162" t="n">
-        <v>1809.9</v>
+        <v>125.65</v>
       </c>
       <c r="D162" t="n">
-        <v>1.65</v>
+        <v>2.36</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>6.66</v>
+        <v>78.06</v>
       </c>
       <c r="C163" t="n">
-        <v>6.77</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="D163" t="n">
-        <v>1.65</v>
+        <v>2.36</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>KIRANVYPAR</t>
+          <t>INVENTURE</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>215.1</v>
+        <v>0.87</v>
       </c>
       <c r="C164" t="n">
-        <v>218.65</v>
+        <v>0.89</v>
       </c>
       <c r="D164" t="n">
-        <v>1.65</v>
+        <v>2.3</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ORIENTTECH</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>238.06</v>
+        <v>191.59</v>
       </c>
       <c r="C165" t="n">
-        <v>241.95</v>
+        <v>196</v>
       </c>
       <c r="D165" t="n">
-        <v>1.63</v>
+        <v>2.3</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>RKSWAMY</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>92.45</v>
+        <v>37</v>
       </c>
       <c r="C166" t="n">
-        <v>93.95</v>
+        <v>37.85</v>
       </c>
       <c r="D166" t="n">
-        <v>1.62</v>
+        <v>2.3</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>AMEYA</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>161.9</v>
+        <v>213.63</v>
       </c>
       <c r="C167" t="n">
-        <v>164.5</v>
+        <v>218.5</v>
       </c>
       <c r="D167" t="n">
-        <v>1.61</v>
+        <v>2.28</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>122.53</v>
+        <v>14.06</v>
       </c>
       <c r="C168" t="n">
-        <v>124.5</v>
+        <v>14.38</v>
       </c>
       <c r="D168" t="n">
-        <v>1.61</v>
+        <v>2.28</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>154.55</v>
+        <v>6.64</v>
       </c>
       <c r="C169" t="n">
-        <v>157</v>
+        <v>6.79</v>
       </c>
       <c r="D169" t="n">
-        <v>1.59</v>
+        <v>2.26</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>543.35</v>
+        <v>2692.2</v>
       </c>
       <c r="C170" t="n">
-        <v>552</v>
+        <v>2752.9</v>
       </c>
       <c r="D170" t="n">
-        <v>1.59</v>
+        <v>2.25</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>SIGNPOST</t>
+          <t>ALPINETEX</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>273.9</v>
+        <v>50.65</v>
       </c>
       <c r="C171" t="n">
-        <v>278.2</v>
+        <v>51.79</v>
       </c>
       <c r="D171" t="n">
-        <v>1.57</v>
+        <v>2.25</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SURANAT&amp;P</t>
+          <t>KCEIL</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>16.04</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="C172" t="n">
-        <v>16.29</v>
+        <v>84.25</v>
       </c>
       <c r="D172" t="n">
-        <v>1.56</v>
+        <v>2.25</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>VIRAT</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>371.2</v>
+        <v>1.35</v>
       </c>
       <c r="C173" t="n">
-        <v>377</v>
+        <v>1.38</v>
       </c>
       <c r="D173" t="n">
-        <v>1.56</v>
+        <v>2.22</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>OSELDEVICE</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>404.65</v>
+        <v>39.33</v>
       </c>
       <c r="C174" t="n">
-        <v>410.95</v>
+        <v>40.2</v>
       </c>
       <c r="D174" t="n">
-        <v>1.56</v>
+        <v>2.21</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SARLAPOLY</t>
+          <t>FEDDERSHOL</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>100.03</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="C175" t="n">
-        <v>101.59</v>
+        <v>66.14</v>
       </c>
       <c r="D175" t="n">
-        <v>1.56</v>
+        <v>2.21</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SILVER001</t>
+          <t>SWELECTES</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>23.19</v>
+        <v>561.65</v>
       </c>
       <c r="C176" t="n">
-        <v>23.55</v>
+        <v>573.95</v>
       </c>
       <c r="D176" t="n">
-        <v>1.55</v>
+        <v>2.19</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>SRHHYPOLTD</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>211.63</v>
+        <v>605.75</v>
       </c>
       <c r="C177" t="n">
-        <v>214.9</v>
+        <v>619</v>
       </c>
       <c r="D177" t="n">
-        <v>1.55</v>
+        <v>2.19</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>1.93</v>
+        <v>283.62</v>
       </c>
       <c r="C178" t="n">
-        <v>1.96</v>
+        <v>289.8</v>
       </c>
       <c r="D178" t="n">
-        <v>1.55</v>
+        <v>2.18</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>7.13</v>
+        <v>113.52</v>
       </c>
       <c r="C179" t="n">
-        <v>7.24</v>
+        <v>115.99</v>
       </c>
       <c r="D179" t="n">
-        <v>1.54</v>
+        <v>2.18</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>HLVLTD</t>
+          <t>DIGITIDE</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>6.59</v>
+        <v>79.76000000000001</v>
       </c>
       <c r="C180" t="n">
-        <v>6.69</v>
+        <v>81.5</v>
       </c>
       <c r="D180" t="n">
-        <v>1.52</v>
+        <v>2.18</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>CARTRADE</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>27.78</v>
+        <v>3004.8</v>
       </c>
       <c r="C181" t="n">
-        <v>28.2</v>
+        <v>3070</v>
       </c>
       <c r="D181" t="n">
-        <v>1.51</v>
+        <v>2.17</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>MUTHOOTCAP</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>35.65</v>
+        <v>231.03</v>
       </c>
       <c r="C182" t="n">
-        <v>36.19</v>
+        <v>236</v>
       </c>
       <c r="D182" t="n">
-        <v>1.51</v>
+        <v>2.15</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>KRISHANA</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>188.15</v>
+        <v>0.93</v>
       </c>
       <c r="C183" t="n">
-        <v>190.98</v>
+        <v>0.95</v>
       </c>
       <c r="D183" t="n">
-        <v>1.5</v>
+        <v>2.15</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>AERONEU</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>67.2</v>
+        <v>4.21</v>
       </c>
       <c r="C184" t="n">
-        <v>68.2</v>
+        <v>4.3</v>
       </c>
       <c r="D184" t="n">
-        <v>1.49</v>
+        <v>2.14</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>VENTIVE</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>578.35</v>
+        <v>37.68</v>
       </c>
       <c r="C185" t="n">
-        <v>586.9</v>
+        <v>38.47</v>
       </c>
       <c r="D185" t="n">
-        <v>1.48</v>
+        <v>2.1</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>137.46</v>
+        <v>16.63</v>
       </c>
       <c r="C186" t="n">
-        <v>139.5</v>
+        <v>16.98</v>
       </c>
       <c r="D186" t="n">
-        <v>1.48</v>
+        <v>2.1</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>ECORECO</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>3.39</v>
+        <v>419.25</v>
       </c>
       <c r="C187" t="n">
-        <v>3.44</v>
+        <v>428</v>
       </c>
       <c r="D187" t="n">
-        <v>1.47</v>
+        <v>2.09</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>ACCURACY</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>1.37</v>
+        <v>4.3</v>
       </c>
       <c r="C188" t="n">
-        <v>1.39</v>
+        <v>4.39</v>
       </c>
       <c r="D188" t="n">
-        <v>1.46</v>
+        <v>2.09</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>BIL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>34.97</v>
+        <v>1010.25</v>
       </c>
       <c r="C189" t="n">
-        <v>35.48</v>
+        <v>1031</v>
       </c>
       <c r="D189" t="n">
-        <v>1.46</v>
+        <v>2.05</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>35.96</v>
+        <v>9.25</v>
       </c>
       <c r="C190" t="n">
-        <v>36.48</v>
+        <v>9.44</v>
       </c>
       <c r="D190" t="n">
-        <v>1.45</v>
+        <v>2.05</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>JAYBEE</t>
+          <t>SHILPAMED</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>95.05</v>
+        <v>1007.3</v>
       </c>
       <c r="C191" t="n">
-        <v>96.40000000000001</v>
+        <v>1028</v>
       </c>
       <c r="D191" t="n">
-        <v>1.42</v>
+        <v>2.05</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>GHCL</t>
+          <t>INDOWIND</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>424</v>
+        <v>8.82</v>
       </c>
       <c r="C192" t="n">
-        <v>430</v>
+        <v>9</v>
       </c>
       <c r="D192" t="n">
-        <v>1.42</v>
+        <v>2.04</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>MYSORPETRO</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>7.09</v>
+        <v>127.2</v>
       </c>
       <c r="C193" t="n">
-        <v>7.19</v>
+        <v>129.8</v>
       </c>
       <c r="D193" t="n">
-        <v>1.41</v>
+        <v>2.04</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>FERMENTA</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>475.5</v>
+        <v>15.4</v>
       </c>
       <c r="C194" t="n">
-        <v>482.2</v>
+        <v>15.71</v>
       </c>
       <c r="D194" t="n">
-        <v>1.41</v>
+        <v>2.01</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>AFSL</t>
+          <t>MEDICO</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>204.56</v>
+        <v>32.5</v>
       </c>
       <c r="C195" t="n">
-        <v>207.4</v>
+        <v>33.15</v>
       </c>
       <c r="D195" t="n">
-        <v>1.39</v>
+        <v>2</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>BELLACASA</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>5.02</v>
+        <v>272.34</v>
       </c>
       <c r="C196" t="n">
-        <v>5.09</v>
+        <v>277.79</v>
       </c>
       <c r="D196" t="n">
-        <v>1.39</v>
+        <v>2</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>AXITA</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>8</v>
+        <v>447.46</v>
       </c>
       <c r="C197" t="n">
-        <v>8.109999999999999</v>
+        <v>456.4</v>
       </c>
       <c r="D197" t="n">
-        <v>1.37</v>
+        <v>2</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>RAMAPHO</t>
+          <t>SEYAIND</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>123.21</v>
+        <v>14.05</v>
       </c>
       <c r="C198" t="n">
-        <v>124.9</v>
+        <v>14.33</v>
       </c>
       <c r="D198" t="n">
-        <v>1.37</v>
+        <v>1.99</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>QUALIANCE</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>182.5</v>
+        <v>6.02</v>
       </c>
       <c r="C199" t="n">
-        <v>185</v>
+        <v>6.14</v>
       </c>
       <c r="D199" t="n">
-        <v>1.37</v>
+        <v>1.99</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>33.52</v>
+        <v>20.57</v>
       </c>
       <c r="C200" t="n">
-        <v>33.98</v>
+        <v>20.98</v>
       </c>
       <c r="D200" t="n">
-        <v>1.37</v>
+        <v>1.99</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>STERTOOLS</t>
+          <t>SBCL</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>221.96</v>
+        <v>1143.2</v>
       </c>
       <c r="C201" t="n">
-        <v>224.98</v>
+        <v>1166</v>
       </c>
       <c r="D201" t="n">
-        <v>1.36</v>
+        <v>1.99</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-28 10:10 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CENTEXT-RE</t>
+          <t>PBMPOLY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.92</v>
+        <v>59.91</v>
       </c>
       <c r="C2" t="n">
-        <v>2.25</v>
+        <v>70.8</v>
       </c>
       <c r="D2" t="n">
-        <v>17.19</v>
+        <v>18.18</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AERONEU</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80.64</v>
+        <v>0.62</v>
       </c>
       <c r="C3" t="n">
-        <v>93</v>
+        <v>0.72</v>
       </c>
       <c r="D3" t="n">
-        <v>15.33</v>
+        <v>16.13</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22.84</v>
+        <v>20.06</v>
       </c>
       <c r="C4" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
-        <v>13.84</v>
+        <v>14.66</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>RTSPOWR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.87</v>
+        <v>104.59</v>
       </c>
       <c r="C5" t="n">
-        <v>8.880000000000001</v>
+        <v>116.3</v>
       </c>
       <c r="D5" t="n">
-        <v>12.83</v>
+        <v>11.2</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PANCHMAHQ</t>
+          <t>BPLPHARMA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>305</v>
+        <v>1898</v>
       </c>
       <c r="C6" t="n">
-        <v>339</v>
+        <v>2093</v>
       </c>
       <c r="D6" t="n">
-        <v>11.15</v>
+        <v>10.27</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VASCONEQ</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>33.29</v>
+        <v>74.36</v>
       </c>
       <c r="C7" t="n">
-        <v>37</v>
+        <v>81.92</v>
       </c>
       <c r="D7" t="n">
-        <v>11.14</v>
+        <v>10.17</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PARIN</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>715</v>
+        <v>27.6</v>
       </c>
       <c r="C8" t="n">
-        <v>789</v>
+        <v>30.29</v>
       </c>
       <c r="D8" t="n">
-        <v>10.35</v>
+        <v>9.75</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HEROMOTORS</t>
+          <t>SUNDRMBRAK</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>118.08</v>
+        <v>670.1</v>
       </c>
       <c r="C9" t="n">
-        <v>128</v>
+        <v>734</v>
       </c>
       <c r="D9" t="n">
-        <v>8.4</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SDBL</t>
+          <t>XELPMOC</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>67.23999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="C10" t="n">
-        <v>72.7</v>
+        <v>97.47</v>
       </c>
       <c r="D10" t="n">
-        <v>8.119999999999999</v>
+        <v>8.91</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>SECMARK</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16.72</v>
+        <v>137.12</v>
       </c>
       <c r="C11" t="n">
-        <v>17.98</v>
+        <v>148.4</v>
       </c>
       <c r="D11" t="n">
-        <v>7.54</v>
+        <v>8.23</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.14</v>
+        <v>36.05</v>
       </c>
       <c r="C12" t="n">
-        <v>0.15</v>
+        <v>39</v>
       </c>
       <c r="D12" t="n">
-        <v>7.14</v>
+        <v>8.18</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>LORDSCHLO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>138.4</v>
+        <v>148.2</v>
       </c>
       <c r="C13" t="n">
-        <v>147.9</v>
+        <v>160</v>
       </c>
       <c r="D13" t="n">
-        <v>6.86</v>
+        <v>7.96</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DUGLOBAL</t>
+          <t>CRAVATEX</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>20.05</v>
+        <v>369.75</v>
       </c>
       <c r="C14" t="n">
-        <v>21.4</v>
+        <v>399</v>
       </c>
       <c r="D14" t="n">
-        <v>6.73</v>
+        <v>7.91</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>34.29</v>
+        <v>12.18</v>
       </c>
       <c r="C15" t="n">
-        <v>36.49</v>
+        <v>13.12</v>
       </c>
       <c r="D15" t="n">
-        <v>6.42</v>
+        <v>7.72</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>HEROMOTORS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.97</v>
+        <v>141.69</v>
       </c>
       <c r="C16" t="n">
-        <v>3.16</v>
+        <v>152.37</v>
       </c>
       <c r="D16" t="n">
-        <v>6.4</v>
+        <v>7.54</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5.13</v>
+        <v>115.52</v>
       </c>
       <c r="C17" t="n">
-        <v>5.44</v>
+        <v>124</v>
       </c>
       <c r="D17" t="n">
-        <v>6.04</v>
+        <v>7.34</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>23.15</v>
+        <v>0.14</v>
       </c>
       <c r="C18" t="n">
-        <v>24.49</v>
+        <v>0.15</v>
       </c>
       <c r="D18" t="n">
-        <v>5.79</v>
+        <v>7.14</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NAGREEKEXP</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>24.02</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="C19" t="n">
-        <v>25.4</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>5.75</v>
+        <v>6.76</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>60.62</v>
+        <v>235.62</v>
       </c>
       <c r="C20" t="n">
-        <v>64.05</v>
+        <v>250</v>
       </c>
       <c r="D20" t="n">
-        <v>5.66</v>
+        <v>6.1</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.18</v>
+        <v>147.79</v>
       </c>
       <c r="C21" t="n">
-        <v>0.19</v>
+        <v>156.65</v>
       </c>
       <c r="D21" t="n">
-        <v>5.56</v>
+        <v>5.99</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ASIANTNE</t>
+          <t>PANCHMAHQ</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>9.19</v>
+        <v>290.1</v>
       </c>
       <c r="C22" t="n">
-        <v>9.699999999999999</v>
+        <v>307</v>
       </c>
       <c r="D22" t="n">
-        <v>5.55</v>
+        <v>5.83</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>66.3</v>
+        <v>73.31</v>
       </c>
       <c r="C23" t="n">
-        <v>69.92</v>
+        <v>77.5</v>
       </c>
       <c r="D23" t="n">
-        <v>5.46</v>
+        <v>5.72</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LAMBODHARA</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>139.46</v>
+        <v>0.18</v>
       </c>
       <c r="C24" t="n">
-        <v>147</v>
+        <v>0.19</v>
       </c>
       <c r="D24" t="n">
-        <v>5.41</v>
+        <v>5.56</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>EKI</t>
+          <t>HALDYNGL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>99.04000000000001</v>
+        <v>145.46</v>
       </c>
       <c r="C25" t="n">
-        <v>104.39</v>
+        <v>153.47</v>
       </c>
       <c r="D25" t="n">
-        <v>5.4</v>
+        <v>5.51</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>ORBTEXP</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>14.86</v>
+        <v>226.9</v>
       </c>
       <c r="C26" t="n">
-        <v>15.64</v>
+        <v>239</v>
       </c>
       <c r="D26" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TCI</t>
+          <t>AEQUS</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>833.45</v>
+        <v>246.05</v>
       </c>
       <c r="C27" t="n">
-        <v>877</v>
+        <v>259</v>
       </c>
       <c r="D27" t="n">
-        <v>5.23</v>
+        <v>5.26</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>806.1</v>
+        <v>0.19</v>
       </c>
       <c r="C28" t="n">
-        <v>846.4</v>
+        <v>0.2</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>5.26</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>132.3</v>
+        <v>2062.5</v>
       </c>
       <c r="C29" t="n">
-        <v>138.91</v>
+        <v>2170</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>5.21</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LALITHAA</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>370.5</v>
+        <v>76.84</v>
       </c>
       <c r="C30" t="n">
-        <v>389</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="D30" t="n">
-        <v>4.99</v>
+        <v>5.14</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SPECTRAA</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>235.4</v>
+        <v>4.99</v>
       </c>
       <c r="C31" t="n">
-        <v>247.15</v>
+        <v>5.24</v>
       </c>
       <c r="D31" t="n">
-        <v>4.99</v>
+        <v>5.01</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ONIXSOLAR</t>
+          <t>TSC</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>321.8</v>
+        <v>51</v>
       </c>
       <c r="C32" t="n">
-        <v>337.85</v>
+        <v>53.55</v>
       </c>
       <c r="D32" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10.42</v>
+        <v>180.87</v>
       </c>
       <c r="C33" t="n">
-        <v>10.94</v>
+        <v>189.91</v>
       </c>
       <c r="D33" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>METALIC</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>171.7</v>
+        <v>6.2</v>
       </c>
       <c r="C34" t="n">
-        <v>180.25</v>
+        <v>6.51</v>
       </c>
       <c r="D34" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>30.91</v>
+        <v>196.64</v>
       </c>
       <c r="C35" t="n">
-        <v>32.45</v>
+        <v>206.47</v>
       </c>
       <c r="D35" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>EMAMIPAP</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>159.7</v>
+        <v>111.87</v>
       </c>
       <c r="C36" t="n">
-        <v>167.65</v>
+        <v>117.46</v>
       </c>
       <c r="D36" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SHRIKANHA</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>22.1</v>
+        <v>206.58</v>
       </c>
       <c r="C37" t="n">
-        <v>23.2</v>
+        <v>216.9</v>
       </c>
       <c r="D37" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>22.29</v>
+        <v>2.4</v>
       </c>
       <c r="C38" t="n">
-        <v>23.4</v>
+        <v>2.52</v>
       </c>
       <c r="D38" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AKANKSHA</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>158.65</v>
+        <v>51.05</v>
       </c>
       <c r="C39" t="n">
-        <v>166.55</v>
+        <v>53.6</v>
       </c>
       <c r="D39" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>20.72</v>
+        <v>167.67</v>
       </c>
       <c r="C40" t="n">
-        <v>21.75</v>
+        <v>176.05</v>
       </c>
       <c r="D40" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NEXTMEDIA</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3.62</v>
+        <v>846.4</v>
       </c>
       <c r="C41" t="n">
-        <v>3.8</v>
+        <v>888.7</v>
       </c>
       <c r="D41" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4.03</v>
+        <v>255.81</v>
       </c>
       <c r="C42" t="n">
-        <v>4.23</v>
+        <v>268.6</v>
       </c>
       <c r="D42" t="n">
-        <v>4.96</v>
+        <v>5</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>NEUEON</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>13.71</v>
+        <v>32.05</v>
       </c>
       <c r="C43" t="n">
-        <v>14.39</v>
+        <v>33.65</v>
       </c>
       <c r="D43" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>107.8</v>
+        <v>113.15</v>
       </c>
       <c r="C44" t="n">
-        <v>113.15</v>
+        <v>118.8</v>
       </c>
       <c r="D44" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>ESAFSFB</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>10.91</v>
+        <v>42.86</v>
       </c>
       <c r="C45" t="n">
-        <v>11.45</v>
+        <v>45</v>
       </c>
       <c r="D45" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GOLDSTAR</t>
+          <t>SWARAJ</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>10.15</v>
+        <v>338.6</v>
       </c>
       <c r="C46" t="n">
-        <v>10.65</v>
+        <v>355.5</v>
       </c>
       <c r="D46" t="n">
-        <v>4.93</v>
+        <v>4.99</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>AISL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>48.65</v>
+        <v>55.1</v>
       </c>
       <c r="C47" t="n">
-        <v>51.05</v>
+        <v>57.85</v>
       </c>
       <c r="D47" t="n">
-        <v>4.93</v>
+        <v>4.99</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>RCDL</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>16.25</v>
+        <v>32.45</v>
       </c>
       <c r="C48" t="n">
-        <v>17.05</v>
+        <v>34.07</v>
       </c>
       <c r="D48" t="n">
-        <v>4.92</v>
+        <v>4.99</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>RCDL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>30.55</v>
+        <v>17.05</v>
       </c>
       <c r="C49" t="n">
-        <v>32.05</v>
+        <v>17.9</v>
       </c>
       <c r="D49" t="n">
-        <v>4.91</v>
+        <v>4.99</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>ARMOUR</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>5.91</v>
+        <v>20.1</v>
       </c>
       <c r="C50" t="n">
-        <v>6.2</v>
+        <v>21.1</v>
       </c>
       <c r="D50" t="n">
-        <v>4.91</v>
+        <v>4.98</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>MVKAGRO</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6.12</v>
+        <v>230.9</v>
       </c>
       <c r="C51" t="n">
-        <v>6.42</v>
+        <v>242.4</v>
       </c>
       <c r="D51" t="n">
-        <v>4.9</v>
+        <v>4.98</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>12.21</v>
+        <v>167.65</v>
       </c>
       <c r="C52" t="n">
-        <v>12.8</v>
+        <v>176</v>
       </c>
       <c r="D52" t="n">
-        <v>4.83</v>
+        <v>4.98</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SWARAJ</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>322.5</v>
+        <v>6.42</v>
       </c>
       <c r="C53" t="n">
-        <v>338</v>
+        <v>6.74</v>
       </c>
       <c r="D53" t="n">
-        <v>4.81</v>
+        <v>4.98</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>46.28</v>
+        <v>27.39</v>
       </c>
       <c r="C54" t="n">
-        <v>48.5</v>
+        <v>28.75</v>
       </c>
       <c r="D54" t="n">
-        <v>4.8</v>
+        <v>4.97</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2.29</v>
+        <v>102.6</v>
       </c>
       <c r="C55" t="n">
-        <v>2.4</v>
+        <v>107.7</v>
       </c>
       <c r="D55" t="n">
-        <v>4.8</v>
+        <v>4.97</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>RSDFIN</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>52.01</v>
+        <v>94.48999999999999</v>
       </c>
       <c r="C56" t="n">
-        <v>54.5</v>
+        <v>99.17</v>
       </c>
       <c r="D56" t="n">
-        <v>4.79</v>
+        <v>4.95</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>111.12</v>
+        <v>21.06</v>
       </c>
       <c r="C57" t="n">
-        <v>116.4</v>
+        <v>22.1</v>
       </c>
       <c r="D57" t="n">
-        <v>4.75</v>
+        <v>4.94</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>VITAL</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>54.37</v>
+        <v>10.76</v>
       </c>
       <c r="C58" t="n">
-        <v>56.94</v>
+        <v>11.29</v>
       </c>
       <c r="D58" t="n">
-        <v>4.73</v>
+        <v>4.93</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1.69</v>
+        <v>60.95</v>
       </c>
       <c r="C59" t="n">
-        <v>1.77</v>
+        <v>63.95</v>
       </c>
       <c r="D59" t="n">
-        <v>4.73</v>
+        <v>4.92</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>STERTOOLS</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>233.05</v>
+        <v>17.16</v>
       </c>
       <c r="C60" t="n">
-        <v>244</v>
+        <v>18</v>
       </c>
       <c r="D60" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>REFRACTORY</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>7.65</v>
+        <v>37.9</v>
       </c>
       <c r="C61" t="n">
-        <v>8</v>
+        <v>39.75</v>
       </c>
       <c r="D61" t="n">
-        <v>4.58</v>
+        <v>4.88</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>KAKATCEM</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>4.45</v>
+        <v>106.72</v>
       </c>
       <c r="C62" t="n">
-        <v>4.65</v>
+        <v>111.9</v>
       </c>
       <c r="D62" t="n">
-        <v>4.49</v>
+        <v>4.85</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DELTAMAGNT</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>54.45</v>
+        <v>36.05</v>
       </c>
       <c r="C63" t="n">
-        <v>56.89</v>
+        <v>37.8</v>
       </c>
       <c r="D63" t="n">
-        <v>4.48</v>
+        <v>4.85</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>22.02</v>
+        <v>834.7</v>
       </c>
       <c r="C64" t="n">
-        <v>23</v>
+        <v>875</v>
       </c>
       <c r="D64" t="n">
-        <v>4.45</v>
+        <v>4.83</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SUPERSPIN</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>7.65</v>
+        <v>538.75</v>
       </c>
       <c r="C65" t="n">
-        <v>7.99</v>
+        <v>564.65</v>
       </c>
       <c r="D65" t="n">
-        <v>4.44</v>
+        <v>4.81</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>12.68</v>
+        <v>425.55</v>
       </c>
       <c r="C66" t="n">
-        <v>13.24</v>
+        <v>446</v>
       </c>
       <c r="D66" t="n">
-        <v>4.42</v>
+        <v>4.81</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LCCPROJECT</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>144.22</v>
+        <v>13.25</v>
       </c>
       <c r="C67" t="n">
-        <v>150.5</v>
+        <v>13.88</v>
       </c>
       <c r="D67" t="n">
-        <v>4.35</v>
+        <v>4.75</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>WALPAR</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.47</v>
+        <v>27.45</v>
       </c>
       <c r="C68" t="n">
-        <v>0.49</v>
+        <v>28.75</v>
       </c>
       <c r="D68" t="n">
-        <v>4.26</v>
+        <v>4.74</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>267.55</v>
+        <v>30.56</v>
       </c>
       <c r="C69" t="n">
-        <v>278.8</v>
+        <v>32</v>
       </c>
       <c r="D69" t="n">
-        <v>4.2</v>
+        <v>4.71</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>196.75</v>
+        <v>116.8</v>
       </c>
       <c r="C70" t="n">
-        <v>205</v>
+        <v>122.29</v>
       </c>
       <c r="D70" t="n">
-        <v>4.19</v>
+        <v>4.7</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>14.38</v>
+        <v>49.19</v>
       </c>
       <c r="C71" t="n">
-        <v>14.98</v>
+        <v>51.5</v>
       </c>
       <c r="D71" t="n">
-        <v>4.17</v>
+        <v>4.7</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NAGREEKCAP</t>
+          <t>GOLDSTAR</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>29.55</v>
+        <v>10.65</v>
       </c>
       <c r="C72" t="n">
-        <v>30.75</v>
+        <v>11.15</v>
       </c>
       <c r="D72" t="n">
-        <v>4.06</v>
+        <v>4.69</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>34.03</v>
+        <v>7.71</v>
       </c>
       <c r="C73" t="n">
-        <v>35.4</v>
+        <v>8.07</v>
       </c>
       <c r="D73" t="n">
-        <v>4.03</v>
+        <v>4.67</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ARTEMISMED</t>
+          <t>BRIGHTBR</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>332.7</v>
+        <v>240.35</v>
       </c>
       <c r="C74" t="n">
-        <v>346</v>
+        <v>251.4</v>
       </c>
       <c r="D74" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>17.89</v>
+        <v>12.38</v>
       </c>
       <c r="C75" t="n">
-        <v>18.6</v>
+        <v>12.95</v>
       </c>
       <c r="D75" t="n">
-        <v>3.97</v>
+        <v>4.6</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BLUECLOUDS</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>20.06</v>
+        <v>28.11</v>
       </c>
       <c r="C76" t="n">
-        <v>20.85</v>
+        <v>29.4</v>
       </c>
       <c r="D76" t="n">
-        <v>3.94</v>
+        <v>4.59</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>MPEL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>46.11</v>
+        <v>25.25</v>
       </c>
       <c r="C77" t="n">
-        <v>47.9</v>
+        <v>26.4</v>
       </c>
       <c r="D77" t="n">
-        <v>3.88</v>
+        <v>4.55</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AMBALALSA</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>41.27</v>
+        <v>298.25</v>
       </c>
       <c r="C78" t="n">
-        <v>42.85</v>
+        <v>311.8</v>
       </c>
       <c r="D78" t="n">
-        <v>3.83</v>
+        <v>4.54</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GENESYS</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>283.18</v>
+        <v>23.7</v>
       </c>
       <c r="C79" t="n">
-        <v>294.03</v>
+        <v>24.77</v>
       </c>
       <c r="D79" t="n">
-        <v>3.83</v>
+        <v>4.51</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>BLACKROSE</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>162.33</v>
+        <v>115.82</v>
       </c>
       <c r="C80" t="n">
-        <v>168.5</v>
+        <v>121</v>
       </c>
       <c r="D80" t="n">
-        <v>3.8</v>
+        <v>4.47</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>9.81</v>
+        <v>59.94</v>
       </c>
       <c r="C81" t="n">
-        <v>10.18</v>
+        <v>62.6</v>
       </c>
       <c r="D81" t="n">
-        <v>3.77</v>
+        <v>4.44</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>VTMLTD</t>
+          <t>REPRO</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>42.13</v>
+        <v>288.25</v>
       </c>
       <c r="C82" t="n">
-        <v>43.7</v>
+        <v>301</v>
       </c>
       <c r="D82" t="n">
-        <v>3.73</v>
+        <v>4.42</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>QUESTLAB</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>90.09999999999999</v>
+        <v>479.8</v>
       </c>
       <c r="C83" t="n">
-        <v>93.45</v>
+        <v>501</v>
       </c>
       <c r="D83" t="n">
-        <v>3.72</v>
+        <v>4.42</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>VIRAT</t>
+          <t>SALONA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>361.55</v>
+        <v>274.75</v>
       </c>
       <c r="C84" t="n">
-        <v>374.9</v>
+        <v>286.9</v>
       </c>
       <c r="D84" t="n">
-        <v>3.69</v>
+        <v>4.42</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>AARNAV</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>6.85</v>
+        <v>36.05</v>
       </c>
       <c r="C85" t="n">
-        <v>7.1</v>
+        <v>37.6</v>
       </c>
       <c r="D85" t="n">
-        <v>3.65</v>
+        <v>4.3</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>SKIL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>4.96</v>
+        <v>0.93</v>
       </c>
       <c r="C86" t="n">
-        <v>5.14</v>
+        <v>0.97</v>
       </c>
       <c r="D86" t="n">
-        <v>3.63</v>
+        <v>4.3</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>2180.8</v>
+        <v>642.5</v>
       </c>
       <c r="C87" t="n">
-        <v>2260</v>
+        <v>670</v>
       </c>
       <c r="D87" t="n">
-        <v>3.63</v>
+        <v>4.28</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>GSMFOILS</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.28</v>
+        <v>77.55</v>
       </c>
       <c r="C88" t="n">
-        <v>0.29</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="D88" t="n">
-        <v>3.57</v>
+        <v>4.26</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>9.550000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="C89" t="n">
-        <v>9.890000000000001</v>
+        <v>8.44</v>
       </c>
       <c r="D89" t="n">
-        <v>3.56</v>
+        <v>4.2</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>SHRJAGP</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>4.21</v>
+        <v>660.25</v>
       </c>
       <c r="C90" t="n">
-        <v>4.36</v>
+        <v>688</v>
       </c>
       <c r="D90" t="n">
-        <v>3.56</v>
+        <v>4.2</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MAHASTEEL</t>
+          <t>VIRAT</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1211.9</v>
+        <v>364.7</v>
       </c>
       <c r="C91" t="n">
-        <v>1255</v>
+        <v>380</v>
       </c>
       <c r="D91" t="n">
-        <v>3.56</v>
+        <v>4.2</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>DURLAX</t>
+          <t>PARIN</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>60.55</v>
+        <v>736.8</v>
       </c>
       <c r="C92" t="n">
-        <v>62.7</v>
+        <v>767</v>
       </c>
       <c r="D92" t="n">
-        <v>3.55</v>
+        <v>4.1</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>KOHINOOR</t>
+          <t>EBIX</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>30.82</v>
+        <v>17.48</v>
       </c>
       <c r="C93" t="n">
-        <v>31.9</v>
+        <v>18.19</v>
       </c>
       <c r="D93" t="n">
-        <v>3.5</v>
+        <v>4.06</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LOYALTEX</t>
+          <t>NECCLTD</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>223.98</v>
+        <v>19.18</v>
       </c>
       <c r="C94" t="n">
-        <v>231.8</v>
+        <v>19.95</v>
       </c>
       <c r="D94" t="n">
-        <v>3.49</v>
+        <v>4.01</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SWARNSAR</t>
+          <t>TRANSCOR</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>42.04</v>
+        <v>24.05</v>
       </c>
       <c r="C95" t="n">
-        <v>43.5</v>
+        <v>25</v>
       </c>
       <c r="D95" t="n">
-        <v>3.47</v>
+        <v>3.95</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>KMSUGAR</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>70.56</v>
+        <v>32.46</v>
       </c>
       <c r="C96" t="n">
-        <v>73</v>
+        <v>33.74</v>
       </c>
       <c r="D96" t="n">
-        <v>3.46</v>
+        <v>3.94</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>7.02</v>
+        <v>39.5</v>
       </c>
       <c r="C97" t="n">
-        <v>7.26</v>
+        <v>41.05</v>
       </c>
       <c r="D97" t="n">
-        <v>3.42</v>
+        <v>3.92</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>SIMCA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>10.25</v>
+        <v>281.85</v>
       </c>
       <c r="C98" t="n">
-        <v>10.6</v>
+        <v>292.85</v>
       </c>
       <c r="D98" t="n">
-        <v>3.41</v>
+        <v>3.9</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>WIPL</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>432.4</v>
+        <v>168.46</v>
       </c>
       <c r="C99" t="n">
-        <v>447</v>
+        <v>175</v>
       </c>
       <c r="D99" t="n">
-        <v>3.38</v>
+        <v>3.88</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>11.6</v>
+        <v>11.07</v>
       </c>
       <c r="C100" t="n">
-        <v>11.99</v>
+        <v>11.5</v>
       </c>
       <c r="D100" t="n">
-        <v>3.36</v>
+        <v>3.88</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>BOROLTD</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>5.69</v>
+        <v>264.8</v>
       </c>
       <c r="C101" t="n">
-        <v>5.88</v>
+        <v>275</v>
       </c>
       <c r="D101" t="n">
-        <v>3.34</v>
+        <v>3.85</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>HBSL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>13.31</v>
+        <v>56.08</v>
       </c>
       <c r="C102" t="n">
-        <v>13.75</v>
+        <v>58.2</v>
       </c>
       <c r="D102" t="n">
-        <v>3.31</v>
+        <v>3.78</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>DCMSIL</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>85.2</v>
+        <v>428.85</v>
       </c>
       <c r="C103" t="n">
-        <v>88</v>
+        <v>445</v>
       </c>
       <c r="D103" t="n">
-        <v>3.29</v>
+        <v>3.77</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>NATIONSTD</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>115.11</v>
+        <v>191.99</v>
       </c>
       <c r="C104" t="n">
-        <v>118.9</v>
+        <v>199</v>
       </c>
       <c r="D104" t="n">
-        <v>3.29</v>
+        <v>3.65</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>ADDIND</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>231.58</v>
+        <v>77.2</v>
       </c>
       <c r="C105" t="n">
-        <v>239</v>
+        <v>80</v>
       </c>
       <c r="D105" t="n">
-        <v>3.2</v>
+        <v>3.63</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>JAYBARMARU</t>
+          <t>AVADHSUGAR</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>121.9</v>
+        <v>796.5</v>
       </c>
       <c r="C106" t="n">
-        <v>125.8</v>
+        <v>825.3</v>
       </c>
       <c r="D106" t="n">
-        <v>3.2</v>
+        <v>3.62</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>177.35</v>
+        <v>24.61</v>
       </c>
       <c r="C107" t="n">
-        <v>183</v>
+        <v>25.49</v>
       </c>
       <c r="D107" t="n">
-        <v>3.19</v>
+        <v>3.58</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>VIVOBIOT</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>58.05</v>
+        <v>16.79</v>
       </c>
       <c r="C108" t="n">
-        <v>59.9</v>
+        <v>17.39</v>
       </c>
       <c r="D108" t="n">
-        <v>3.19</v>
+        <v>3.57</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>12.31</v>
+        <v>0.28</v>
       </c>
       <c r="C109" t="n">
-        <v>12.7</v>
+        <v>0.29</v>
       </c>
       <c r="D109" t="n">
-        <v>3.17</v>
+        <v>3.57</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>FLFL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>249.6</v>
+        <v>1.12</v>
       </c>
       <c r="C110" t="n">
-        <v>257.45</v>
+        <v>1.16</v>
       </c>
       <c r="D110" t="n">
-        <v>3.15</v>
+        <v>3.57</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>17.13</v>
+        <v>16.85</v>
       </c>
       <c r="C111" t="n">
-        <v>17.67</v>
+        <v>17.45</v>
       </c>
       <c r="D111" t="n">
-        <v>3.15</v>
+        <v>3.56</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DENTA</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>270.1</v>
+        <v>17.82</v>
       </c>
       <c r="C112" t="n">
-        <v>278.55</v>
+        <v>18.45</v>
       </c>
       <c r="D112" t="n">
-        <v>3.13</v>
+        <v>3.54</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>153.13</v>
+        <v>23.2</v>
       </c>
       <c r="C113" t="n">
-        <v>157.9</v>
+        <v>24</v>
       </c>
       <c r="D113" t="n">
-        <v>3.12</v>
+        <v>3.45</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ISHANCH</t>
+          <t>CRESTO</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>49.9</v>
+        <v>22.03</v>
       </c>
       <c r="C114" t="n">
-        <v>51.4</v>
+        <v>22.79</v>
       </c>
       <c r="D114" t="n">
-        <v>3.01</v>
+        <v>3.45</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>8.039999999999999</v>
+        <v>57.29</v>
       </c>
       <c r="C115" t="n">
-        <v>8.279999999999999</v>
+        <v>59.26</v>
       </c>
       <c r="D115" t="n">
-        <v>2.99</v>
+        <v>3.44</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>SHRADDHA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>659.4</v>
+        <v>146.97</v>
       </c>
       <c r="C116" t="n">
-        <v>679</v>
+        <v>151.99</v>
       </c>
       <c r="D116" t="n">
-        <v>2.97</v>
+        <v>3.42</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AJAXENGG</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>575.2</v>
+        <v>298.51</v>
       </c>
       <c r="C117" t="n">
-        <v>592</v>
+        <v>308.7</v>
       </c>
       <c r="D117" t="n">
-        <v>2.92</v>
+        <v>3.41</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>INDOMIM</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>1311.15</v>
+        <v>10.59</v>
       </c>
       <c r="C118" t="n">
-        <v>1349</v>
+        <v>10.95</v>
       </c>
       <c r="D118" t="n">
-        <v>2.89</v>
+        <v>3.4</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>5.93</v>
+        <v>22.04</v>
       </c>
       <c r="C119" t="n">
-        <v>6.1</v>
+        <v>22.79</v>
       </c>
       <c r="D119" t="n">
-        <v>2.87</v>
+        <v>3.4</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>PACIFICI</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>136.14</v>
+        <v>6.87</v>
       </c>
       <c r="C120" t="n">
-        <v>140</v>
+        <v>7.1</v>
       </c>
       <c r="D120" t="n">
-        <v>2.84</v>
+        <v>3.35</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LAKSHMIMIL</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>7780.5</v>
+        <v>4.55</v>
       </c>
       <c r="C121" t="n">
-        <v>8001</v>
+        <v>4.7</v>
       </c>
       <c r="D121" t="n">
-        <v>2.83</v>
+        <v>3.3</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ATALREAL</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>14.6</v>
+        <v>556.6</v>
       </c>
       <c r="C122" t="n">
-        <v>15.01</v>
+        <v>574.95</v>
       </c>
       <c r="D122" t="n">
-        <v>2.81</v>
+        <v>3.3</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>NGLFINE</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>2894.9</v>
+        <v>16.7</v>
       </c>
       <c r="C123" t="n">
-        <v>2975.5</v>
+        <v>17.25</v>
       </c>
       <c r="D123" t="n">
-        <v>2.78</v>
+        <v>3.29</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.36</v>
+        <v>387.35</v>
       </c>
       <c r="C124" t="n">
-        <v>0.37</v>
+        <v>400</v>
       </c>
       <c r="D124" t="n">
-        <v>2.78</v>
+        <v>3.27</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>AEROPLANE</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>201.98</v>
+        <v>59.94</v>
       </c>
       <c r="C125" t="n">
-        <v>207.55</v>
+        <v>61.89</v>
       </c>
       <c r="D125" t="n">
-        <v>2.76</v>
+        <v>3.25</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>3BBLACKBIO</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>306</v>
+        <v>1456.2</v>
       </c>
       <c r="C126" t="n">
-        <v>314.4</v>
+        <v>1502.9</v>
       </c>
       <c r="D126" t="n">
-        <v>2.75</v>
+        <v>3.21</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>12.02</v>
+        <v>56.21</v>
       </c>
       <c r="C127" t="n">
-        <v>12.35</v>
+        <v>57.99</v>
       </c>
       <c r="D127" t="n">
-        <v>2.75</v>
+        <v>3.17</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>XCHANGING</t>
+          <t>TURTLEMINT</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>60.35</v>
+        <v>87.23999999999999</v>
       </c>
       <c r="C128" t="n">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="D128" t="n">
-        <v>2.73</v>
+        <v>3.16</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>KANDARP</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>76.95</v>
+        <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>79.05</v>
+        <v>8.25</v>
       </c>
       <c r="D129" t="n">
-        <v>2.73</v>
+        <v>3.12</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>JISLDVREQS</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>20.14</v>
+        <v>14.11</v>
       </c>
       <c r="C130" t="n">
-        <v>20.69</v>
+        <v>14.55</v>
       </c>
       <c r="D130" t="n">
-        <v>2.73</v>
+        <v>3.12</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>UGARSUGAR</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>96.37</v>
+        <v>64.03</v>
       </c>
       <c r="C131" t="n">
-        <v>98.98999999999999</v>
+        <v>66</v>
       </c>
       <c r="D131" t="n">
-        <v>2.72</v>
+        <v>3.08</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>NARMADA</t>
+          <t>VGL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>13.24</v>
+        <v>67.28</v>
       </c>
       <c r="C132" t="n">
-        <v>13.6</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="D132" t="n">
-        <v>2.72</v>
+        <v>3.08</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>18.99</v>
+        <v>45.61</v>
       </c>
       <c r="C133" t="n">
-        <v>19.5</v>
+        <v>47</v>
       </c>
       <c r="D133" t="n">
-        <v>2.69</v>
+        <v>3.05</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LORDSCHLO</t>
+          <t>GILLANDERS</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>134.5</v>
+        <v>108.69</v>
       </c>
       <c r="C134" t="n">
-        <v>138.1</v>
+        <v>112</v>
       </c>
       <c r="D134" t="n">
-        <v>2.68</v>
+        <v>3.05</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>949.65</v>
+        <v>12.18</v>
       </c>
       <c r="C135" t="n">
-        <v>974.9</v>
+        <v>12.55</v>
       </c>
       <c r="D135" t="n">
-        <v>2.66</v>
+        <v>3.04</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>HSBCGOLD</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>130.3</v>
+        <v>96.03</v>
       </c>
       <c r="C136" t="n">
-        <v>133.75</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="D136" t="n">
-        <v>2.65</v>
+        <v>2.99</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>OMFREIGHT</t>
+          <t>BENGALASM</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>91.83</v>
+        <v>6093</v>
       </c>
       <c r="C137" t="n">
-        <v>94.25</v>
+        <v>6275</v>
       </c>
       <c r="D137" t="n">
-        <v>2.64</v>
+        <v>2.99</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>49.59</v>
+        <v>90.54000000000001</v>
       </c>
       <c r="C138" t="n">
-        <v>50.9</v>
+        <v>93.23999999999999</v>
       </c>
       <c r="D138" t="n">
-        <v>2.64</v>
+        <v>2.98</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>STEAMHOUSE</t>
+          <t>PAKKA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>113.71</v>
+        <v>75.06</v>
       </c>
       <c r="C139" t="n">
-        <v>116.7</v>
+        <v>77.28</v>
       </c>
       <c r="D139" t="n">
-        <v>2.63</v>
+        <v>2.96</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>80.39</v>
+        <v>202.99</v>
       </c>
       <c r="C140" t="n">
-        <v>82.5</v>
+        <v>209</v>
       </c>
       <c r="D140" t="n">
-        <v>2.62</v>
+        <v>2.96</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>AIROLAM</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>14.11</v>
+        <v>92.29000000000001</v>
       </c>
       <c r="C141" t="n">
-        <v>14.48</v>
+        <v>95</v>
       </c>
       <c r="D141" t="n">
-        <v>2.62</v>
+        <v>2.94</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>34.93</v>
+        <v>2.4</v>
       </c>
       <c r="C142" t="n">
-        <v>35.84</v>
+        <v>2.47</v>
       </c>
       <c r="D142" t="n">
-        <v>2.61</v>
+        <v>2.92</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>CELEBRITY</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>89.27</v>
+        <v>6.63</v>
       </c>
       <c r="C143" t="n">
-        <v>91.59999999999999</v>
+        <v>6.82</v>
       </c>
       <c r="D143" t="n">
-        <v>2.61</v>
+        <v>2.87</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>33.82</v>
+        <v>18.47</v>
       </c>
       <c r="C144" t="n">
-        <v>34.7</v>
+        <v>19</v>
       </c>
       <c r="D144" t="n">
-        <v>2.6</v>
+        <v>2.87</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>53.9</v>
+        <v>25.28</v>
       </c>
       <c r="C145" t="n">
-        <v>55.3</v>
+        <v>26</v>
       </c>
       <c r="D145" t="n">
-        <v>2.6</v>
+        <v>2.85</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>8.529999999999999</v>
+        <v>7.03</v>
       </c>
       <c r="C146" t="n">
-        <v>8.75</v>
+        <v>7.23</v>
       </c>
       <c r="D146" t="n">
-        <v>2.58</v>
+        <v>2.84</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ZFSTEERING</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>746.1</v>
+        <v>15.97</v>
       </c>
       <c r="C147" t="n">
-        <v>765</v>
+        <v>16.42</v>
       </c>
       <c r="D147" t="n">
-        <v>2.53</v>
+        <v>2.82</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>IGPL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>9.140000000000001</v>
+        <v>593.15</v>
       </c>
       <c r="C148" t="n">
-        <v>9.369999999999999</v>
+        <v>609.9</v>
       </c>
       <c r="D148" t="n">
-        <v>2.52</v>
+        <v>2.82</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>AVANCE</t>
+          <t>SWARNSAR</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>0.8</v>
+        <v>41.68</v>
       </c>
       <c r="C149" t="n">
-        <v>0.82</v>
+        <v>42.85</v>
       </c>
       <c r="D149" t="n">
-        <v>2.5</v>
+        <v>2.81</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>WAKEFIT</t>
+          <t>SHEMAROO</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>142.83</v>
+        <v>124.51</v>
       </c>
       <c r="C150" t="n">
-        <v>146.37</v>
+        <v>128</v>
       </c>
       <c r="D150" t="n">
-        <v>2.48</v>
+        <v>2.8</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>FABTECH</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>12.19</v>
+        <v>145.83</v>
       </c>
       <c r="C151" t="n">
-        <v>12.49</v>
+        <v>149.9</v>
       </c>
       <c r="D151" t="n">
-        <v>2.46</v>
+        <v>2.79</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ARCHIES</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>12.66</v>
+        <v>4.67</v>
       </c>
       <c r="C152" t="n">
-        <v>12.97</v>
+        <v>4.8</v>
       </c>
       <c r="D152" t="n">
-        <v>2.45</v>
+        <v>2.78</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>69.31</v>
+        <v>0.36</v>
       </c>
       <c r="C153" t="n">
-        <v>71</v>
+        <v>0.37</v>
       </c>
       <c r="D153" t="n">
-        <v>2.44</v>
+        <v>2.78</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>26.36</v>
+        <v>164.06</v>
       </c>
       <c r="C154" t="n">
-        <v>27</v>
+        <v>168.6</v>
       </c>
       <c r="D154" t="n">
-        <v>2.43</v>
+        <v>2.77</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>VETO</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>143.04</v>
+        <v>36.29</v>
       </c>
       <c r="C155" t="n">
-        <v>146.5</v>
+        <v>37.29</v>
       </c>
       <c r="D155" t="n">
-        <v>2.42</v>
+        <v>2.76</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>FCSSOFT</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>5.81</v>
+        <v>1.46</v>
       </c>
       <c r="C156" t="n">
-        <v>5.95</v>
+        <v>1.5</v>
       </c>
       <c r="D156" t="n">
-        <v>2.41</v>
+        <v>2.74</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>WEL</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>16.58</v>
+        <v>74.62</v>
       </c>
       <c r="C157" t="n">
-        <v>16.98</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D157" t="n">
-        <v>2.41</v>
+        <v>2.72</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MANOMAY</t>
+          <t>MODIRUBBER</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>233.21</v>
+        <v>121.62</v>
       </c>
       <c r="C158" t="n">
-        <v>238.8</v>
+        <v>124.9</v>
       </c>
       <c r="D158" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ORIANA</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>303.7</v>
+        <v>1.85</v>
       </c>
       <c r="C159" t="n">
-        <v>311</v>
+        <v>1.9</v>
       </c>
       <c r="D159" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>DRONE</t>
+          <t>MAITREYA</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>33.6</v>
+        <v>112</v>
       </c>
       <c r="C160" t="n">
-        <v>34.4</v>
+        <v>115</v>
       </c>
       <c r="D160" t="n">
-        <v>2.38</v>
+        <v>2.68</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>KOHINOOR</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>25.18</v>
+        <v>31.05</v>
       </c>
       <c r="C161" t="n">
-        <v>25.78</v>
+        <v>31.88</v>
       </c>
       <c r="D161" t="n">
-        <v>2.38</v>
+        <v>2.67</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>KECL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>122.75</v>
+        <v>99.36</v>
       </c>
       <c r="C162" t="n">
-        <v>125.65</v>
+        <v>102</v>
       </c>
       <c r="D162" t="n">
-        <v>2.36</v>
+        <v>2.66</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>NOVAAGRI</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>78.06</v>
+        <v>22.9</v>
       </c>
       <c r="C163" t="n">
-        <v>79.90000000000001</v>
+        <v>23.5</v>
       </c>
       <c r="D163" t="n">
-        <v>2.36</v>
+        <v>2.62</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>INVENTURE</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.87</v>
+        <v>34.29</v>
       </c>
       <c r="C164" t="n">
-        <v>0.89</v>
+        <v>35.18</v>
       </c>
       <c r="D164" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>191.59</v>
+        <v>5.02</v>
       </c>
       <c r="C165" t="n">
-        <v>196</v>
+        <v>5.15</v>
       </c>
       <c r="D165" t="n">
-        <v>2.3</v>
+        <v>2.59</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>37</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="C166" t="n">
-        <v>37.85</v>
+        <v>96</v>
       </c>
       <c r="D166" t="n">
-        <v>2.3</v>
+        <v>2.56</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>213.63</v>
+        <v>32.65</v>
       </c>
       <c r="C167" t="n">
-        <v>218.5</v>
+        <v>33.48</v>
       </c>
       <c r="D167" t="n">
-        <v>2.28</v>
+        <v>2.54</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SWISSMLTRY</t>
+          <t>KAYA</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>14.06</v>
+        <v>316.8</v>
       </c>
       <c r="C168" t="n">
-        <v>14.38</v>
+        <v>324.85</v>
       </c>
       <c r="D168" t="n">
-        <v>2.28</v>
+        <v>2.54</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>6.64</v>
+        <v>21.38</v>
       </c>
       <c r="C169" t="n">
-        <v>6.79</v>
+        <v>21.92</v>
       </c>
       <c r="D169" t="n">
-        <v>2.26</v>
+        <v>2.53</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>2692.2</v>
+        <v>67.7</v>
       </c>
       <c r="C170" t="n">
-        <v>2752.9</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D170" t="n">
-        <v>2.25</v>
+        <v>2.51</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ALPINETEX</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>50.65</v>
+        <v>654.6</v>
       </c>
       <c r="C171" t="n">
-        <v>51.79</v>
+        <v>671</v>
       </c>
       <c r="D171" t="n">
-        <v>2.25</v>
+        <v>2.51</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>KCEIL</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>82.40000000000001</v>
+        <v>6.38</v>
       </c>
       <c r="C172" t="n">
-        <v>84.25</v>
+        <v>6.54</v>
       </c>
       <c r="D172" t="n">
-        <v>2.25</v>
+        <v>2.51</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>SUNDROP</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>1.35</v>
+        <v>745.75</v>
       </c>
       <c r="C173" t="n">
-        <v>1.38</v>
+        <v>764.4</v>
       </c>
       <c r="D173" t="n">
-        <v>2.22</v>
+        <v>2.5</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>39.33</v>
+        <v>8</v>
       </c>
       <c r="C174" t="n">
-        <v>40.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D174" t="n">
-        <v>2.21</v>
+        <v>2.5</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>FEDDERSHOL</t>
+          <t>ZIMLAB</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>64.70999999999999</v>
+        <v>138.48</v>
       </c>
       <c r="C175" t="n">
-        <v>66.14</v>
+        <v>141.94</v>
       </c>
       <c r="D175" t="n">
-        <v>2.21</v>
+        <v>2.5</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SWELECTES</t>
+          <t>IFBAGRO</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>561.65</v>
+        <v>858.6</v>
       </c>
       <c r="C176" t="n">
-        <v>573.95</v>
+        <v>880</v>
       </c>
       <c r="D176" t="n">
-        <v>2.19</v>
+        <v>2.49</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>STARTECK</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>605.75</v>
+        <v>262.5</v>
       </c>
       <c r="C177" t="n">
-        <v>619</v>
+        <v>269</v>
       </c>
       <c r="D177" t="n">
-        <v>2.19</v>
+        <v>2.48</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>HARDWYN</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>283.62</v>
+        <v>9.27</v>
       </c>
       <c r="C178" t="n">
-        <v>289.8</v>
+        <v>9.5</v>
       </c>
       <c r="D178" t="n">
-        <v>2.18</v>
+        <v>2.48</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>113.52</v>
+        <v>280.05</v>
       </c>
       <c r="C179" t="n">
-        <v>115.99</v>
+        <v>287</v>
       </c>
       <c r="D179" t="n">
-        <v>2.18</v>
+        <v>2.48</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>DIGITIDE</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>79.76000000000001</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C180" t="n">
-        <v>81.5</v>
+        <v>0.83</v>
       </c>
       <c r="D180" t="n">
-        <v>2.18</v>
+        <v>2.47</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>CARTRADE</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>3004.8</v>
+        <v>50.75</v>
       </c>
       <c r="C181" t="n">
-        <v>3070</v>
+        <v>52</v>
       </c>
       <c r="D181" t="n">
-        <v>2.17</v>
+        <v>2.46</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MUTHOOTCAP</t>
+          <t>SSEGL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>231.03</v>
+        <v>396.3</v>
       </c>
       <c r="C182" t="n">
-        <v>236</v>
+        <v>406</v>
       </c>
       <c r="D182" t="n">
-        <v>2.15</v>
+        <v>2.45</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.93</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C183" t="n">
-        <v>0.95</v>
+        <v>79.5</v>
       </c>
       <c r="D183" t="n">
-        <v>2.15</v>
+        <v>2.45</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>4.21</v>
+        <v>2.05</v>
       </c>
       <c r="C184" t="n">
-        <v>4.3</v>
+        <v>2.1</v>
       </c>
       <c r="D184" t="n">
-        <v>2.14</v>
+        <v>2.44</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>37.68</v>
+        <v>25.13</v>
       </c>
       <c r="C185" t="n">
-        <v>38.47</v>
+        <v>25.74</v>
       </c>
       <c r="D185" t="n">
-        <v>2.1</v>
+        <v>2.43</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>16.63</v>
+        <v>1737.8</v>
       </c>
       <c r="C186" t="n">
-        <v>16.98</v>
+        <v>1780</v>
       </c>
       <c r="D186" t="n">
-        <v>2.1</v>
+        <v>2.43</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ECORECO</t>
+          <t>AUGMONT</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>419.25</v>
+        <v>877.9</v>
       </c>
       <c r="C187" t="n">
-        <v>428</v>
+        <v>899</v>
       </c>
       <c r="D187" t="n">
-        <v>2.09</v>
+        <v>2.4</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ACCURACY</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>4.3</v>
+        <v>13.34</v>
       </c>
       <c r="C188" t="n">
-        <v>4.39</v>
+        <v>13.66</v>
       </c>
       <c r="D188" t="n">
-        <v>2.09</v>
+        <v>2.4</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>BIL</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>1010.25</v>
+        <v>4.19</v>
       </c>
       <c r="C189" t="n">
-        <v>1031</v>
+        <v>4.29</v>
       </c>
       <c r="D189" t="n">
-        <v>2.05</v>
+        <v>2.39</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>9.25</v>
+        <v>5.85</v>
       </c>
       <c r="C190" t="n">
-        <v>9.44</v>
+        <v>5.99</v>
       </c>
       <c r="D190" t="n">
-        <v>2.05</v>
+        <v>2.39</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>SHILPAMED</t>
+          <t>ESTER</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>1007.3</v>
+        <v>86.14</v>
       </c>
       <c r="C191" t="n">
-        <v>1028</v>
+        <v>88.2</v>
       </c>
       <c r="D191" t="n">
-        <v>2.05</v>
+        <v>2.39</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>INDOWIND</t>
+          <t>VIVIDEL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>8.82</v>
+        <v>1773.7</v>
       </c>
       <c r="C192" t="n">
-        <v>9</v>
+        <v>1816</v>
       </c>
       <c r="D192" t="n">
-        <v>2.04</v>
+        <v>2.38</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>MYSORPETRO</t>
+          <t>PRESSTONIC</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>127.2</v>
+        <v>52.5</v>
       </c>
       <c r="C193" t="n">
-        <v>129.8</v>
+        <v>53.75</v>
       </c>
       <c r="D193" t="n">
-        <v>2.04</v>
+        <v>2.38</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>15.4</v>
+        <v>29.44</v>
       </c>
       <c r="C194" t="n">
-        <v>15.71</v>
+        <v>30.14</v>
       </c>
       <c r="D194" t="n">
-        <v>2.01</v>
+        <v>2.38</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MEDICO</t>
+          <t>VETO</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>32.5</v>
+        <v>150.32</v>
       </c>
       <c r="C195" t="n">
-        <v>33.15</v>
+        <v>153.89</v>
       </c>
       <c r="D195" t="n">
-        <v>2</v>
+        <v>2.37</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>BELLACASA</t>
+          <t>ABDL</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>272.34</v>
+        <v>715.05</v>
       </c>
       <c r="C196" t="n">
-        <v>277.79</v>
+        <v>731.95</v>
       </c>
       <c r="D196" t="n">
-        <v>2</v>
+        <v>2.36</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>447.46</v>
+        <v>31.51</v>
       </c>
       <c r="C197" t="n">
-        <v>456.4</v>
+        <v>32.25</v>
       </c>
       <c r="D197" t="n">
-        <v>2</v>
+        <v>2.35</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SEYAIND</t>
+          <t>UNIDT</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>14.05</v>
+        <v>241.71</v>
       </c>
       <c r="C198" t="n">
-        <v>14.33</v>
+        <v>247.4</v>
       </c>
       <c r="D198" t="n">
-        <v>1.99</v>
+        <v>2.35</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>SUDEEPPHRM</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>6.02</v>
+        <v>1164.9</v>
       </c>
       <c r="C199" t="n">
-        <v>6.14</v>
+        <v>1192</v>
       </c>
       <c r="D199" t="n">
-        <v>1.99</v>
+        <v>2.33</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>20.57</v>
+        <v>167.05</v>
       </c>
       <c r="C200" t="n">
-        <v>20.98</v>
+        <v>170.95</v>
       </c>
       <c r="D200" t="n">
-        <v>1.99</v>
+        <v>2.33</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>SBCL</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>1143.2</v>
+        <v>13.18</v>
       </c>
       <c r="C201" t="n">
-        <v>1166</v>
+        <v>13.48</v>
       </c>
       <c r="D201" t="n">
-        <v>1.99</v>
+        <v>2.28</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-29 10:08 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PBMPOLY</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>59.91</v>
+        <v>24.07</v>
       </c>
       <c r="C2" t="n">
-        <v>70.8</v>
+        <v>28.88</v>
       </c>
       <c r="D2" t="n">
-        <v>18.18</v>
+        <v>19.98</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.62</v>
+        <v>0.74</v>
       </c>
       <c r="C3" t="n">
-        <v>0.72</v>
+        <v>0.85</v>
       </c>
       <c r="D3" t="n">
-        <v>16.13</v>
+        <v>14.86</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20.06</v>
+        <v>11.89</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>13.5</v>
       </c>
       <c r="D4" t="n">
-        <v>14.66</v>
+        <v>13.54</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RTSPOWR</t>
+          <t>REGENCERAM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>104.59</v>
+        <v>32.64</v>
       </c>
       <c r="C5" t="n">
-        <v>116.3</v>
+        <v>36.92</v>
       </c>
       <c r="D5" t="n">
-        <v>11.2</v>
+        <v>13.11</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BPLPHARMA</t>
+          <t>ELLEN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1898</v>
+        <v>359.05</v>
       </c>
       <c r="C6" t="n">
-        <v>2093</v>
+        <v>394.95</v>
       </c>
       <c r="D6" t="n">
-        <v>10.27</v>
+        <v>10</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SDBL</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>74.36</v>
+        <v>30.36</v>
       </c>
       <c r="C7" t="n">
-        <v>81.92</v>
+        <v>33.39</v>
       </c>
       <c r="D7" t="n">
-        <v>10.17</v>
+        <v>9.98</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27.6</v>
+        <v>26.97</v>
       </c>
       <c r="C8" t="n">
-        <v>30.29</v>
+        <v>29.66</v>
       </c>
       <c r="D8" t="n">
-        <v>9.75</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SUNDRMBRAK</t>
+          <t>RTSPOWR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>670.1</v>
+        <v>125.5</v>
       </c>
       <c r="C9" t="n">
-        <v>734</v>
+        <v>136.77</v>
       </c>
       <c r="D9" t="n">
-        <v>9.539999999999999</v>
+        <v>8.98</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>XELPMOC</t>
+          <t>COMPEAU</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>89.5</v>
+        <v>353.05</v>
       </c>
       <c r="C10" t="n">
-        <v>97.47</v>
+        <v>383.9</v>
       </c>
       <c r="D10" t="n">
-        <v>8.91</v>
+        <v>8.74</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SECMARK</t>
+          <t>STARTECK</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>137.12</v>
+        <v>314</v>
       </c>
       <c r="C11" t="n">
-        <v>148.4</v>
+        <v>340</v>
       </c>
       <c r="D11" t="n">
-        <v>8.23</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>AXISCADES</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>36.05</v>
+        <v>1879.5</v>
       </c>
       <c r="C12" t="n">
-        <v>39</v>
+        <v>2034</v>
       </c>
       <c r="D12" t="n">
-        <v>8.18</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LORDSCHLO</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>148.2</v>
+        <v>5.72</v>
       </c>
       <c r="C13" t="n">
-        <v>160</v>
+        <v>6.18</v>
       </c>
       <c r="D13" t="n">
-        <v>7.96</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CRAVATEX</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>369.75</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C14" t="n">
-        <v>399</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>7.91</v>
+        <v>7.46</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>VIVOBIOT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12.18</v>
+        <v>16.26</v>
       </c>
       <c r="C15" t="n">
-        <v>13.12</v>
+        <v>17.44</v>
       </c>
       <c r="D15" t="n">
-        <v>7.72</v>
+        <v>7.26</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HEROMOTORS</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>141.69</v>
+        <v>0.14</v>
       </c>
       <c r="C16" t="n">
-        <v>152.37</v>
+        <v>0.15</v>
       </c>
       <c r="D16" t="n">
-        <v>7.54</v>
+        <v>7.14</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADSL</t>
+          <t>THOMASCOTT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>115.52</v>
+        <v>238.35</v>
       </c>
       <c r="C17" t="n">
-        <v>124</v>
+        <v>255</v>
       </c>
       <c r="D17" t="n">
-        <v>7.34</v>
+        <v>6.99</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.14</v>
+        <v>72.17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.15</v>
+        <v>77</v>
       </c>
       <c r="D18" t="n">
-        <v>7.14</v>
+        <v>6.69</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>GILLANDERS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>9.029999999999999</v>
+        <v>107.38</v>
       </c>
       <c r="C19" t="n">
-        <v>9.640000000000001</v>
+        <v>114</v>
       </c>
       <c r="D19" t="n">
-        <v>6.76</v>
+        <v>6.17</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>235.62</v>
+        <v>81.52</v>
       </c>
       <c r="C20" t="n">
-        <v>250</v>
+        <v>86.52</v>
       </c>
       <c r="D20" t="n">
-        <v>6.1</v>
+        <v>6.13</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>DUCOL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>147.79</v>
+        <v>115</v>
       </c>
       <c r="C21" t="n">
-        <v>156.65</v>
+        <v>121.9</v>
       </c>
       <c r="D21" t="n">
-        <v>5.99</v>
+        <v>6</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PANCHMAHQ</t>
+          <t>AUGMONT</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>290.1</v>
+        <v>965.65</v>
       </c>
       <c r="C22" t="n">
-        <v>307</v>
+        <v>1022</v>
       </c>
       <c r="D22" t="n">
-        <v>5.83</v>
+        <v>5.84</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>73.31</v>
+        <v>0.18</v>
       </c>
       <c r="C23" t="n">
-        <v>77.5</v>
+        <v>0.19</v>
       </c>
       <c r="D23" t="n">
-        <v>5.72</v>
+        <v>5.56</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.18</v>
+        <v>165.91</v>
       </c>
       <c r="C24" t="n">
-        <v>0.19</v>
+        <v>175</v>
       </c>
       <c r="D24" t="n">
-        <v>5.56</v>
+        <v>5.48</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HALDYNGL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>145.46</v>
+        <v>275.21</v>
       </c>
       <c r="C25" t="n">
-        <v>153.47</v>
+        <v>290</v>
       </c>
       <c r="D25" t="n">
-        <v>5.51</v>
+        <v>5.37</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ORBTEXP</t>
+          <t>SHIGAN</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>226.9</v>
+        <v>60.55</v>
       </c>
       <c r="C26" t="n">
-        <v>239</v>
+        <v>63.8</v>
       </c>
       <c r="D26" t="n">
-        <v>5.33</v>
+        <v>5.37</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,14 +1011,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AEQUS</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>246.05</v>
+        <v>0.19</v>
       </c>
       <c r="C27" t="n">
-        <v>259</v>
+        <v>0.2</v>
       </c>
       <c r="D27" t="n">
         <v>5.26</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.19</v>
+        <v>18.87</v>
       </c>
       <c r="C28" t="n">
-        <v>0.2</v>
+        <v>19.85</v>
       </c>
       <c r="D28" t="n">
-        <v>5.26</v>
+        <v>5.19</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2062.5</v>
+        <v>10.26</v>
       </c>
       <c r="C29" t="n">
-        <v>2170</v>
+        <v>10.79</v>
       </c>
       <c r="D29" t="n">
-        <v>5.21</v>
+        <v>5.17</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>76.84</v>
+        <v>189.91</v>
       </c>
       <c r="C30" t="n">
-        <v>80.79000000000001</v>
+        <v>199.4</v>
       </c>
       <c r="D30" t="n">
-        <v>5.14</v>
+        <v>5</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4.99</v>
+        <v>216.9</v>
       </c>
       <c r="C31" t="n">
-        <v>5.24</v>
+        <v>227.74</v>
       </c>
       <c r="D31" t="n">
-        <v>5.01</v>
+        <v>5</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,14 +1121,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TSC</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>51</v>
+        <v>406.25</v>
       </c>
       <c r="C32" t="n">
-        <v>53.55</v>
+        <v>426.55</v>
       </c>
       <c r="D32" t="n">
         <v>5</v>
@@ -1143,14 +1143,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>180.87</v>
+        <v>145.85</v>
       </c>
       <c r="C33" t="n">
-        <v>189.91</v>
+        <v>153.14</v>
       </c>
       <c r="D33" t="n">
         <v>5</v>
@@ -1165,14 +1165,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6.2</v>
+        <v>206.47</v>
       </c>
       <c r="C34" t="n">
-        <v>6.51</v>
+        <v>216.79</v>
       </c>
       <c r="D34" t="n">
         <v>5</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>GFSTEELS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>196.64</v>
+        <v>34.07</v>
       </c>
       <c r="C35" t="n">
-        <v>206.47</v>
+        <v>35.77</v>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>EMAMIPAP</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>111.87</v>
+        <v>231.35</v>
       </c>
       <c r="C36" t="n">
-        <v>117.46</v>
+        <v>242.9</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>206.58</v>
+        <v>34.66</v>
       </c>
       <c r="C37" t="n">
-        <v>216.9</v>
+        <v>36.39</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>AKANKSHA</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2.4</v>
+        <v>159.7</v>
       </c>
       <c r="C38" t="n">
-        <v>2.52</v>
+        <v>167.65</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>51.05</v>
+        <v>159.6</v>
       </c>
       <c r="C39" t="n">
-        <v>53.6</v>
+        <v>167.55</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>BLUEWATER</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>167.67</v>
+        <v>561.45</v>
       </c>
       <c r="C40" t="n">
-        <v>176.05</v>
+        <v>589.4</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>ARMOUR</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>846.4</v>
+        <v>21.1</v>
       </c>
       <c r="C41" t="n">
-        <v>888.7</v>
+        <v>22.15</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>255.81</v>
+        <v>10.87</v>
       </c>
       <c r="C42" t="n">
-        <v>268.6</v>
+        <v>11.41</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>4.97</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>32.05</v>
+        <v>28.75</v>
       </c>
       <c r="C43" t="n">
-        <v>33.65</v>
+        <v>30.18</v>
       </c>
       <c r="D43" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LAKSHYA</t>
+          <t>NEUEON</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>113.15</v>
+        <v>15.1</v>
       </c>
       <c r="C44" t="n">
-        <v>118.8</v>
+        <v>15.85</v>
       </c>
       <c r="D44" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ESAFSFB</t>
+          <t>HITECHGEAR</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>42.86</v>
+        <v>648.85</v>
       </c>
       <c r="C45" t="n">
-        <v>45</v>
+        <v>680.9</v>
       </c>
       <c r="D45" t="n">
-        <v>4.99</v>
+        <v>4.94</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SWARAJ</t>
+          <t>GOLDSTAR</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>338.6</v>
+        <v>11.15</v>
       </c>
       <c r="C46" t="n">
-        <v>355.5</v>
+        <v>11.7</v>
       </c>
       <c r="D46" t="n">
-        <v>4.99</v>
+        <v>4.93</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AISL</t>
+          <t>MOMSBELIEF</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>55.1</v>
+        <v>223.01</v>
       </c>
       <c r="C47" t="n">
-        <v>57.85</v>
+        <v>234</v>
       </c>
       <c r="D47" t="n">
-        <v>4.99</v>
+        <v>4.93</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>LAKSHYA</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>32.45</v>
+        <v>118.8</v>
       </c>
       <c r="C48" t="n">
-        <v>34.07</v>
+        <v>124.65</v>
       </c>
       <c r="D48" t="n">
-        <v>4.99</v>
+        <v>4.92</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>RCDL</t>
+          <t>MPEL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>17.05</v>
+        <v>26.5</v>
       </c>
       <c r="C49" t="n">
-        <v>17.9</v>
+        <v>27.8</v>
       </c>
       <c r="D49" t="n">
-        <v>4.99</v>
+        <v>4.91</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ARMOUR</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>20.1</v>
+        <v>33.65</v>
       </c>
       <c r="C50" t="n">
-        <v>21.1</v>
+        <v>35.3</v>
       </c>
       <c r="D50" t="n">
-        <v>4.98</v>
+        <v>4.9</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MVKAGRO</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>230.9</v>
+        <v>6.74</v>
       </c>
       <c r="C51" t="n">
-        <v>242.4</v>
+        <v>7.07</v>
       </c>
       <c r="D51" t="n">
-        <v>4.98</v>
+        <v>4.9</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>RHETAN</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>167.65</v>
+        <v>15.91</v>
       </c>
       <c r="C52" t="n">
-        <v>176</v>
+        <v>16.69</v>
       </c>
       <c r="D52" t="n">
-        <v>4.98</v>
+        <v>4.9</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>6.42</v>
+        <v>2.29</v>
       </c>
       <c r="C53" t="n">
-        <v>6.74</v>
+        <v>2.4</v>
       </c>
       <c r="D53" t="n">
-        <v>4.98</v>
+        <v>4.8</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>QUADPRO</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>27.39</v>
+        <v>4.2</v>
       </c>
       <c r="C54" t="n">
-        <v>28.75</v>
+        <v>4.4</v>
       </c>
       <c r="D54" t="n">
-        <v>4.97</v>
+        <v>4.76</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>KORE</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>102.6</v>
+        <v>189.15</v>
       </c>
       <c r="C55" t="n">
-        <v>107.7</v>
+        <v>198.15</v>
       </c>
       <c r="D55" t="n">
-        <v>4.97</v>
+        <v>4.76</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RSDFIN</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>94.48999999999999</v>
+        <v>2.52</v>
       </c>
       <c r="C56" t="n">
-        <v>99.17</v>
+        <v>2.64</v>
       </c>
       <c r="D56" t="n">
-        <v>4.95</v>
+        <v>4.76</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>PRASOLCHEM</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>21.06</v>
+        <v>763.8</v>
       </c>
       <c r="C57" t="n">
-        <v>22.1</v>
+        <v>799.9</v>
       </c>
       <c r="D57" t="n">
-        <v>4.94</v>
+        <v>4.73</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>10.76</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C58" t="n">
-        <v>11.29</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="D58" t="n">
-        <v>4.93</v>
+        <v>4.71</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>SAPPL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>60.95</v>
+        <v>279.95</v>
       </c>
       <c r="C59" t="n">
-        <v>63.95</v>
+        <v>293</v>
       </c>
       <c r="D59" t="n">
-        <v>4.92</v>
+        <v>4.66</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>PARNAXLAB</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17.16</v>
+        <v>112.78</v>
       </c>
       <c r="C60" t="n">
-        <v>18</v>
+        <v>118</v>
       </c>
       <c r="D60" t="n">
-        <v>4.9</v>
+        <v>4.63</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>REFRACTORY</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>37.9</v>
+        <v>5.02</v>
       </c>
       <c r="C61" t="n">
-        <v>39.75</v>
+        <v>5.25</v>
       </c>
       <c r="D61" t="n">
-        <v>4.88</v>
+        <v>4.58</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>KAKATCEM</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>106.72</v>
+        <v>21.99</v>
       </c>
       <c r="C62" t="n">
-        <v>111.9</v>
+        <v>22.99</v>
       </c>
       <c r="D62" t="n">
-        <v>4.85</v>
+        <v>4.55</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>FERMENTA</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>36.05</v>
+        <v>479.3</v>
       </c>
       <c r="C63" t="n">
-        <v>37.8</v>
+        <v>501</v>
       </c>
       <c r="D63" t="n">
-        <v>4.85</v>
+        <v>4.53</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>DGCONTENT</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>834.7</v>
+        <v>23.37</v>
       </c>
       <c r="C64" t="n">
-        <v>875</v>
+        <v>24.4</v>
       </c>
       <c r="D64" t="n">
-        <v>4.83</v>
+        <v>4.41</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>538.75</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="C65" t="n">
-        <v>564.65</v>
+        <v>0.72</v>
       </c>
       <c r="D65" t="n">
-        <v>4.81</v>
+        <v>4.35</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>425.55</v>
+        <v>1.38</v>
       </c>
       <c r="C66" t="n">
-        <v>446</v>
+        <v>1.44</v>
       </c>
       <c r="D66" t="n">
-        <v>4.81</v>
+        <v>4.35</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ANMOL</t>
+          <t>GANESHBE</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>13.25</v>
+        <v>137.32</v>
       </c>
       <c r="C67" t="n">
-        <v>13.88</v>
+        <v>143</v>
       </c>
       <c r="D67" t="n">
-        <v>4.75</v>
+        <v>4.14</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>WALPAR</t>
+          <t>ARVEE</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>27.45</v>
+        <v>234.5</v>
       </c>
       <c r="C68" t="n">
-        <v>28.75</v>
+        <v>244</v>
       </c>
       <c r="D68" t="n">
-        <v>4.74</v>
+        <v>4.05</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>30.56</v>
+        <v>219.2</v>
       </c>
       <c r="C69" t="n">
-        <v>32</v>
+        <v>227.99</v>
       </c>
       <c r="D69" t="n">
-        <v>4.71</v>
+        <v>4.01</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>TIPSFILMS</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>116.8</v>
+        <v>331.8</v>
       </c>
       <c r="C70" t="n">
-        <v>122.29</v>
+        <v>345</v>
       </c>
       <c r="D70" t="n">
-        <v>4.7</v>
+        <v>3.98</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>49.19</v>
+        <v>15.37</v>
       </c>
       <c r="C71" t="n">
-        <v>51.5</v>
+        <v>15.98</v>
       </c>
       <c r="D71" t="n">
-        <v>4.7</v>
+        <v>3.97</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>GOLDSTAR</t>
+          <t>SAMPANN</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>10.65</v>
+        <v>24.29</v>
       </c>
       <c r="C72" t="n">
-        <v>11.15</v>
+        <v>25.25</v>
       </c>
       <c r="D72" t="n">
-        <v>4.69</v>
+        <v>3.95</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>7.71</v>
+        <v>4.94</v>
       </c>
       <c r="C73" t="n">
-        <v>8.07</v>
+        <v>5.13</v>
       </c>
       <c r="D73" t="n">
-        <v>4.67</v>
+        <v>3.85</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BRIGHTBR</t>
+          <t>SARTELE</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>240.35</v>
+        <v>84.8</v>
       </c>
       <c r="C74" t="n">
-        <v>251.4</v>
+        <v>88</v>
       </c>
       <c r="D74" t="n">
-        <v>4.6</v>
+        <v>3.77</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>ESSARSHPNG</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>12.38</v>
+        <v>15.63</v>
       </c>
       <c r="C75" t="n">
-        <v>12.95</v>
+        <v>16.21</v>
       </c>
       <c r="D75" t="n">
-        <v>4.6</v>
+        <v>3.71</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>MOTOGENFIN</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>28.11</v>
+        <v>25.7</v>
       </c>
       <c r="C76" t="n">
-        <v>29.4</v>
+        <v>26.65</v>
       </c>
       <c r="D76" t="n">
-        <v>4.59</v>
+        <v>3.7</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MPEL</t>
+          <t>HYBRIDFIN</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>25.25</v>
+        <v>17.36</v>
       </c>
       <c r="C77" t="n">
-        <v>26.4</v>
+        <v>18</v>
       </c>
       <c r="D77" t="n">
-        <v>4.55</v>
+        <v>3.69</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>298.25</v>
+        <v>58.81</v>
       </c>
       <c r="C78" t="n">
-        <v>311.8</v>
+        <v>60.9</v>
       </c>
       <c r="D78" t="n">
-        <v>4.54</v>
+        <v>3.55</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>23.7</v>
+        <v>53.6</v>
       </c>
       <c r="C79" t="n">
-        <v>24.77</v>
+        <v>55.5</v>
       </c>
       <c r="D79" t="n">
-        <v>4.51</v>
+        <v>3.54</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BLACKROSE</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>115.82</v>
+        <v>37</v>
       </c>
       <c r="C80" t="n">
-        <v>121</v>
+        <v>38.3</v>
       </c>
       <c r="D80" t="n">
-        <v>4.47</v>
+        <v>3.51</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>SSRETAIL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>59.94</v>
+        <v>716.95</v>
       </c>
       <c r="C81" t="n">
-        <v>62.6</v>
+        <v>742.15</v>
       </c>
       <c r="D81" t="n">
-        <v>4.44</v>
+        <v>3.51</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>REPRO</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>288.25</v>
+        <v>21.73</v>
       </c>
       <c r="C82" t="n">
-        <v>301</v>
+        <v>22.49</v>
       </c>
       <c r="D82" t="n">
-        <v>4.42</v>
+        <v>3.5</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>479.8</v>
+        <v>13.51</v>
       </c>
       <c r="C83" t="n">
-        <v>501</v>
+        <v>13.98</v>
       </c>
       <c r="D83" t="n">
-        <v>4.42</v>
+        <v>3.48</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SALONA</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>274.75</v>
+        <v>0.29</v>
       </c>
       <c r="C84" t="n">
-        <v>286.9</v>
+        <v>0.3</v>
       </c>
       <c r="D84" t="n">
-        <v>4.42</v>
+        <v>3.45</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AARNAV</t>
+          <t>DAICHI</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>36.05</v>
+        <v>316</v>
       </c>
       <c r="C85" t="n">
-        <v>37.6</v>
+        <v>326.85</v>
       </c>
       <c r="D85" t="n">
-        <v>4.3</v>
+        <v>3.43</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SKIL</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.93</v>
+        <v>7.9</v>
       </c>
       <c r="C86" t="n">
-        <v>0.97</v>
+        <v>8.17</v>
       </c>
       <c r="D86" t="n">
-        <v>4.3</v>
+        <v>3.42</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>642.5</v>
+        <v>0.88</v>
       </c>
       <c r="C87" t="n">
-        <v>670</v>
+        <v>0.91</v>
       </c>
       <c r="D87" t="n">
-        <v>4.28</v>
+        <v>3.41</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GSMFOILS</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>77.55</v>
+        <v>50.36</v>
       </c>
       <c r="C88" t="n">
-        <v>80.84999999999999</v>
+        <v>52.07</v>
       </c>
       <c r="D88" t="n">
-        <v>4.26</v>
+        <v>3.4</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>8.1</v>
+        <v>10.05</v>
       </c>
       <c r="C89" t="n">
-        <v>8.44</v>
+        <v>10.39</v>
       </c>
       <c r="D89" t="n">
-        <v>4.2</v>
+        <v>3.38</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SHRJAGP</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>660.25</v>
+        <v>107.7</v>
       </c>
       <c r="C90" t="n">
-        <v>688</v>
+        <v>111.3</v>
       </c>
       <c r="D90" t="n">
-        <v>4.2</v>
+        <v>3.34</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>VIRAT</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>364.7</v>
+        <v>4.84</v>
       </c>
       <c r="C91" t="n">
-        <v>380</v>
+        <v>5</v>
       </c>
       <c r="D91" t="n">
-        <v>4.2</v>
+        <v>3.31</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PARIN</t>
+          <t>MARALOVER</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>736.8</v>
+        <v>59.37</v>
       </c>
       <c r="C92" t="n">
-        <v>767</v>
+        <v>61.29</v>
       </c>
       <c r="D92" t="n">
-        <v>4.1</v>
+        <v>3.23</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>EBIX</t>
+          <t>ADDIND</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>17.48</v>
+        <v>77.5</v>
       </c>
       <c r="C93" t="n">
-        <v>18.19</v>
+        <v>80</v>
       </c>
       <c r="D93" t="n">
-        <v>4.06</v>
+        <v>3.23</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NECCLTD</t>
+          <t>KILITCH</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>19.18</v>
+        <v>217.05</v>
       </c>
       <c r="C94" t="n">
-        <v>19.95</v>
+        <v>224</v>
       </c>
       <c r="D94" t="n">
-        <v>4.01</v>
+        <v>3.2</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TRANSCOR</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>24.05</v>
+        <v>11.14</v>
       </c>
       <c r="C95" t="n">
-        <v>25</v>
+        <v>11.49</v>
       </c>
       <c r="D95" t="n">
-        <v>3.95</v>
+        <v>3.14</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>KMSUGAR</t>
+          <t>KMEW</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>32.46</v>
+        <v>2876.9</v>
       </c>
       <c r="C96" t="n">
-        <v>33.74</v>
+        <v>2965.1</v>
       </c>
       <c r="D96" t="n">
-        <v>3.94</v>
+        <v>3.07</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>39.5</v>
+        <v>28.13</v>
       </c>
       <c r="C97" t="n">
-        <v>41.05</v>
+        <v>28.99</v>
       </c>
       <c r="D97" t="n">
-        <v>3.92</v>
+        <v>3.06</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SIMCA</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>281.85</v>
+        <v>49.52</v>
       </c>
       <c r="C98" t="n">
-        <v>292.85</v>
+        <v>51</v>
       </c>
       <c r="D98" t="n">
-        <v>3.9</v>
+        <v>2.99</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>WIPL</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>168.46</v>
+        <v>34.39</v>
       </c>
       <c r="C99" t="n">
-        <v>175</v>
+        <v>35.4</v>
       </c>
       <c r="D99" t="n">
-        <v>3.88</v>
+        <v>2.94</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>11.07</v>
+        <v>3133.7</v>
       </c>
       <c r="C100" t="n">
-        <v>11.5</v>
+        <v>3225</v>
       </c>
       <c r="D100" t="n">
-        <v>3.88</v>
+        <v>2.91</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BOROLTD</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>264.8</v>
+        <v>92.81</v>
       </c>
       <c r="C101" t="n">
-        <v>275</v>
+        <v>95.48999999999999</v>
       </c>
       <c r="D101" t="n">
-        <v>3.85</v>
+        <v>2.89</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HBSL</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>56.08</v>
+        <v>26.4</v>
       </c>
       <c r="C102" t="n">
-        <v>58.2</v>
+        <v>27.16</v>
       </c>
       <c r="D102" t="n">
-        <v>3.78</v>
+        <v>2.88</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>SETL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>428.85</v>
+        <v>422.65</v>
       </c>
       <c r="C103" t="n">
-        <v>445</v>
+        <v>434.7</v>
       </c>
       <c r="D103" t="n">
-        <v>3.77</v>
+        <v>2.85</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>ORBTEXP</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>191.99</v>
+        <v>227.15</v>
       </c>
       <c r="C104" t="n">
-        <v>199</v>
+        <v>233.6</v>
       </c>
       <c r="D104" t="n">
-        <v>3.65</v>
+        <v>2.84</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ADDIND</t>
+          <t>ENIL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>77.2</v>
+        <v>96.01000000000001</v>
       </c>
       <c r="C105" t="n">
-        <v>80</v>
+        <v>98.73999999999999</v>
       </c>
       <c r="D105" t="n">
-        <v>3.63</v>
+        <v>2.84</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AVADHSUGAR</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>796.5</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="C106" t="n">
-        <v>825.3</v>
+        <v>70.98999999999999</v>
       </c>
       <c r="D106" t="n">
-        <v>3.62</v>
+        <v>2.82</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>SOMICONVEY</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>24.61</v>
+        <v>89.18000000000001</v>
       </c>
       <c r="C107" t="n">
-        <v>25.49</v>
+        <v>91.68000000000001</v>
       </c>
       <c r="D107" t="n">
-        <v>3.58</v>
+        <v>2.8</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>VIVOBIOT</t>
+          <t>INVPRECQ</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>16.79</v>
+        <v>1501.5</v>
       </c>
       <c r="C108" t="n">
-        <v>17.39</v>
+        <v>1543.6</v>
       </c>
       <c r="D108" t="n">
-        <v>3.57</v>
+        <v>2.8</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>RCDL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.28</v>
+        <v>17.9</v>
       </c>
       <c r="C109" t="n">
-        <v>0.29</v>
+        <v>18.4</v>
       </c>
       <c r="D109" t="n">
-        <v>3.57</v>
+        <v>2.79</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>ZFSTEERING</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1.12</v>
+        <v>729.7</v>
       </c>
       <c r="C110" t="n">
-        <v>1.16</v>
+        <v>750</v>
       </c>
       <c r="D110" t="n">
-        <v>3.57</v>
+        <v>2.78</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>16.85</v>
+        <v>5.06</v>
       </c>
       <c r="C111" t="n">
-        <v>17.45</v>
+        <v>5.2</v>
       </c>
       <c r="D111" t="n">
-        <v>3.56</v>
+        <v>2.77</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>17.82</v>
+        <v>5.8</v>
       </c>
       <c r="C112" t="n">
-        <v>18.45</v>
+        <v>5.96</v>
       </c>
       <c r="D112" t="n">
-        <v>3.54</v>
+        <v>2.76</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>LOKESHMACH</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>23.2</v>
+        <v>326.1</v>
       </c>
       <c r="C113" t="n">
-        <v>24</v>
+        <v>335</v>
       </c>
       <c r="D113" t="n">
-        <v>3.45</v>
+        <v>2.73</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CRESTO</t>
+          <t>HINDADH</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>22.03</v>
+        <v>384.45</v>
       </c>
       <c r="C114" t="n">
-        <v>22.79</v>
+        <v>394.95</v>
       </c>
       <c r="D114" t="n">
-        <v>3.45</v>
+        <v>2.73</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>57.29</v>
+        <v>486</v>
       </c>
       <c r="C115" t="n">
-        <v>59.26</v>
+        <v>499.2</v>
       </c>
       <c r="D115" t="n">
-        <v>3.44</v>
+        <v>2.72</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SHRADDHA</t>
+          <t>NCC</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>146.97</v>
+        <v>130.29</v>
       </c>
       <c r="C116" t="n">
-        <v>151.99</v>
+        <v>133.83</v>
       </c>
       <c r="D116" t="n">
-        <v>3.42</v>
+        <v>2.72</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>298.51</v>
+        <v>0.37</v>
       </c>
       <c r="C117" t="n">
-        <v>308.7</v>
+        <v>0.38</v>
       </c>
       <c r="D117" t="n">
-        <v>3.41</v>
+        <v>2.7</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>10.59</v>
+        <v>4.48</v>
       </c>
       <c r="C118" t="n">
-        <v>10.95</v>
+        <v>4.6</v>
       </c>
       <c r="D118" t="n">
-        <v>3.4</v>
+        <v>2.68</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>GLOSTERLTD</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>22.04</v>
+        <v>545.5</v>
       </c>
       <c r="C119" t="n">
-        <v>22.79</v>
+        <v>559.9</v>
       </c>
       <c r="D119" t="n">
-        <v>3.4</v>
+        <v>2.64</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>NILAINFRA</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>6.87</v>
+        <v>4.59</v>
       </c>
       <c r="C120" t="n">
-        <v>7.1</v>
+        <v>4.71</v>
       </c>
       <c r="D120" t="n">
-        <v>3.35</v>
+        <v>2.61</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>DCMSIL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>4.55</v>
+        <v>78.98</v>
       </c>
       <c r="C121" t="n">
-        <v>4.7</v>
+        <v>81</v>
       </c>
       <c r="D121" t="n">
-        <v>3.3</v>
+        <v>2.56</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>556.6</v>
+        <v>1.97</v>
       </c>
       <c r="C122" t="n">
-        <v>574.95</v>
+        <v>2.02</v>
       </c>
       <c r="D122" t="n">
-        <v>3.3</v>
+        <v>2.54</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>16.7</v>
+        <v>6.33</v>
       </c>
       <c r="C123" t="n">
-        <v>17.25</v>
+        <v>6.49</v>
       </c>
       <c r="D123" t="n">
-        <v>3.29</v>
+        <v>2.53</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>POEL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>387.35</v>
+        <v>141.35</v>
       </c>
       <c r="C124" t="n">
-        <v>400</v>
+        <v>144.91</v>
       </c>
       <c r="D124" t="n">
-        <v>3.27</v>
+        <v>2.52</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>MOHITE</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>59.94</v>
+        <v>2.4</v>
       </c>
       <c r="C125" t="n">
-        <v>61.89</v>
+        <v>2.46</v>
       </c>
       <c r="D125" t="n">
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>3BBLACKBIO</t>
+          <t>CENTEXT-RE</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1456.2</v>
+        <v>2</v>
       </c>
       <c r="C126" t="n">
-        <v>1502.9</v>
+        <v>2.05</v>
       </c>
       <c r="D126" t="n">
-        <v>3.21</v>
+        <v>2.5</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>SSEGL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>56.21</v>
+        <v>380.05</v>
       </c>
       <c r="C127" t="n">
-        <v>57.99</v>
+        <v>389.5</v>
       </c>
       <c r="D127" t="n">
-        <v>3.17</v>
+        <v>2.49</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TURTLEMINT</t>
+          <t>ONWARDTEC</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>87.23999999999999</v>
+        <v>285</v>
       </c>
       <c r="C128" t="n">
-        <v>90</v>
+        <v>292</v>
       </c>
       <c r="D128" t="n">
-        <v>3.16</v>
+        <v>2.46</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>AVIENCE</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>8</v>
+        <v>376.25</v>
       </c>
       <c r="C129" t="n">
-        <v>8.25</v>
+        <v>385.5</v>
       </c>
       <c r="D129" t="n">
-        <v>3.12</v>
+        <v>2.46</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>14.11</v>
+        <v>67.98</v>
       </c>
       <c r="C130" t="n">
-        <v>14.55</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D130" t="n">
-        <v>3.12</v>
+        <v>2.46</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>UGARSUGAR</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>64.03</v>
+        <v>48.65</v>
       </c>
       <c r="C131" t="n">
-        <v>66</v>
+        <v>49.84</v>
       </c>
       <c r="D131" t="n">
-        <v>3.08</v>
+        <v>2.45</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>VGL</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>67.28</v>
+        <v>93.03</v>
       </c>
       <c r="C132" t="n">
-        <v>69.34999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="D132" t="n">
-        <v>3.08</v>
+        <v>2.44</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>45.61</v>
+        <v>0.41</v>
       </c>
       <c r="C133" t="n">
-        <v>47</v>
+        <v>0.42</v>
       </c>
       <c r="D133" t="n">
-        <v>3.05</v>
+        <v>2.44</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>GILLANDERS</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>108.69</v>
+        <v>2.47</v>
       </c>
       <c r="C134" t="n">
-        <v>112</v>
+        <v>2.53</v>
       </c>
       <c r="D134" t="n">
-        <v>3.05</v>
+        <v>2.43</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>12.18</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="C135" t="n">
-        <v>12.55</v>
+        <v>8.84</v>
       </c>
       <c r="D135" t="n">
-        <v>3.04</v>
+        <v>2.43</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>96.03</v>
+        <v>118.97</v>
       </c>
       <c r="C136" t="n">
-        <v>98.90000000000001</v>
+        <v>121.85</v>
       </c>
       <c r="D136" t="n">
-        <v>2.99</v>
+        <v>2.42</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BENGALASM</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>6093</v>
+        <v>189.43</v>
       </c>
       <c r="C137" t="n">
-        <v>6275</v>
+        <v>194</v>
       </c>
       <c r="D137" t="n">
-        <v>2.99</v>
+        <v>2.41</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>90.54000000000001</v>
+        <v>34.08</v>
       </c>
       <c r="C138" t="n">
-        <v>93.23999999999999</v>
+        <v>34.9</v>
       </c>
       <c r="D138" t="n">
-        <v>2.98</v>
+        <v>2.41</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>PAKKA</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>75.06</v>
+        <v>5</v>
       </c>
       <c r="C139" t="n">
-        <v>77.28</v>
+        <v>5.12</v>
       </c>
       <c r="D139" t="n">
-        <v>2.96</v>
+        <v>2.4</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>VIKRAMSOLR</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>202.99</v>
+        <v>160.08</v>
       </c>
       <c r="C140" t="n">
-        <v>209</v>
+        <v>163.92</v>
       </c>
       <c r="D140" t="n">
-        <v>2.96</v>
+        <v>2.4</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>AIROLAM</t>
+          <t>MOLDTECH</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>92.29000000000001</v>
+        <v>197.29</v>
       </c>
       <c r="C141" t="n">
-        <v>95</v>
+        <v>202</v>
       </c>
       <c r="D141" t="n">
-        <v>2.94</v>
+        <v>2.39</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>2.4</v>
+        <v>150.22</v>
       </c>
       <c r="C142" t="n">
-        <v>2.47</v>
+        <v>153.8</v>
       </c>
       <c r="D142" t="n">
-        <v>2.92</v>
+        <v>2.38</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CELEBRITY</t>
+          <t>TVVISION</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>6.63</v>
+        <v>2.96</v>
       </c>
       <c r="C143" t="n">
-        <v>6.82</v>
+        <v>3.03</v>
       </c>
       <c r="D143" t="n">
-        <v>2.87</v>
+        <v>2.36</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>SURAJLTD</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>18.47</v>
+        <v>193.45</v>
       </c>
       <c r="C144" t="n">
-        <v>19</v>
+        <v>198</v>
       </c>
       <c r="D144" t="n">
-        <v>2.87</v>
+        <v>2.35</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>ACUTAAS</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>25.28</v>
+        <v>3214.4</v>
       </c>
       <c r="C145" t="n">
-        <v>26</v>
+        <v>3290</v>
       </c>
       <c r="D145" t="n">
-        <v>2.85</v>
+        <v>2.35</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>7.03</v>
+        <v>14.56</v>
       </c>
       <c r="C146" t="n">
-        <v>7.23</v>
+        <v>14.9</v>
       </c>
       <c r="D146" t="n">
-        <v>2.84</v>
+        <v>2.34</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>NURECA</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>15.97</v>
+        <v>362.55</v>
       </c>
       <c r="C147" t="n">
-        <v>16.42</v>
+        <v>371</v>
       </c>
       <c r="D147" t="n">
-        <v>2.82</v>
+        <v>2.33</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>IGPL</t>
+          <t>KOTARISUG</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>593.15</v>
+        <v>26.75</v>
       </c>
       <c r="C148" t="n">
-        <v>609.9</v>
+        <v>27.37</v>
       </c>
       <c r="D148" t="n">
-        <v>2.82</v>
+        <v>2.32</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SWARNSAR</t>
+          <t>CENTRUM</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>41.68</v>
+        <v>20.85</v>
       </c>
       <c r="C149" t="n">
-        <v>42.85</v>
+        <v>21.33</v>
       </c>
       <c r="D149" t="n">
-        <v>2.81</v>
+        <v>2.3</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SHEMAROO</t>
+          <t>PUNJABCHEM</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>124.51</v>
+        <v>1054.6</v>
       </c>
       <c r="C150" t="n">
-        <v>128</v>
+        <v>1078.9</v>
       </c>
       <c r="D150" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FABTECH</t>
+          <t>BLACKROSE</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>145.83</v>
+        <v>116.32</v>
       </c>
       <c r="C151" t="n">
-        <v>149.9</v>
+        <v>118.98</v>
       </c>
       <c r="D151" t="n">
-        <v>2.79</v>
+        <v>2.29</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>4.67</v>
+        <v>13.62</v>
       </c>
       <c r="C152" t="n">
-        <v>4.8</v>
+        <v>13.93</v>
       </c>
       <c r="D152" t="n">
-        <v>2.78</v>
+        <v>2.28</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>SUNFLAG</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>0.36</v>
+        <v>449.2</v>
       </c>
       <c r="C153" t="n">
-        <v>0.37</v>
+        <v>459.4</v>
       </c>
       <c r="D153" t="n">
-        <v>2.78</v>
+        <v>2.27</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>164.06</v>
+        <v>0.44</v>
       </c>
       <c r="C154" t="n">
-        <v>168.6</v>
+        <v>0.45</v>
       </c>
       <c r="D154" t="n">
-        <v>2.77</v>
+        <v>2.27</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>36.29</v>
+        <v>167.9</v>
       </c>
       <c r="C155" t="n">
-        <v>37.29</v>
+        <v>171.7</v>
       </c>
       <c r="D155" t="n">
-        <v>2.76</v>
+        <v>2.26</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>FCSSOFT</t>
+          <t>DCI</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>1.46</v>
+        <v>326.65</v>
       </c>
       <c r="C156" t="n">
-        <v>1.5</v>
+        <v>334</v>
       </c>
       <c r="D156" t="n">
-        <v>2.74</v>
+        <v>2.25</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>WEL</t>
+          <t>NDL</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>74.62</v>
+        <v>2.67</v>
       </c>
       <c r="C157" t="n">
-        <v>76.65000000000001</v>
+        <v>2.73</v>
       </c>
       <c r="D157" t="n">
-        <v>2.72</v>
+        <v>2.25</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MODIRUBBER</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>121.62</v>
+        <v>7.63</v>
       </c>
       <c r="C158" t="n">
-        <v>124.9</v>
+        <v>7.8</v>
       </c>
       <c r="D158" t="n">
-        <v>2.7</v>
+        <v>2.23</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>KAPSTON</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>1.85</v>
+        <v>537.8</v>
       </c>
       <c r="C159" t="n">
-        <v>1.9</v>
+        <v>549.6</v>
       </c>
       <c r="D159" t="n">
-        <v>2.7</v>
+        <v>2.19</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MAITREYA</t>
+          <t>AGIIL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>112</v>
+        <v>271.6</v>
       </c>
       <c r="C160" t="n">
-        <v>115</v>
+        <v>277.55</v>
       </c>
       <c r="D160" t="n">
-        <v>2.68</v>
+        <v>2.19</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>KOHINOOR</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>31.05</v>
+        <v>0.46</v>
       </c>
       <c r="C161" t="n">
-        <v>31.88</v>
+        <v>0.47</v>
       </c>
       <c r="D161" t="n">
-        <v>2.67</v>
+        <v>2.17</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDOBORAX</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>99.36</v>
+        <v>477.55</v>
       </c>
       <c r="C162" t="n">
-        <v>102</v>
+        <v>487.8</v>
       </c>
       <c r="D162" t="n">
-        <v>2.66</v>
+        <v>2.15</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>NOVAAGRI</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>22.9</v>
+        <v>450.25</v>
       </c>
       <c r="C163" t="n">
-        <v>23.5</v>
+        <v>459.95</v>
       </c>
       <c r="D163" t="n">
-        <v>2.62</v>
+        <v>2.15</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>34.29</v>
+        <v>31.33</v>
       </c>
       <c r="C164" t="n">
-        <v>35.18</v>
+        <v>32</v>
       </c>
       <c r="D164" t="n">
-        <v>2.6</v>
+        <v>2.14</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>5.02</v>
+        <v>36.18</v>
       </c>
       <c r="C165" t="n">
-        <v>5.15</v>
+        <v>36.95</v>
       </c>
       <c r="D165" t="n">
-        <v>2.59</v>
+        <v>2.13</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>93.59999999999999</v>
+        <v>12.18</v>
       </c>
       <c r="C166" t="n">
-        <v>96</v>
+        <v>12.44</v>
       </c>
       <c r="D166" t="n">
-        <v>2.56</v>
+        <v>2.13</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>32.65</v>
+        <v>39.94</v>
       </c>
       <c r="C167" t="n">
-        <v>33.48</v>
+        <v>40.78</v>
       </c>
       <c r="D167" t="n">
-        <v>2.54</v>
+        <v>2.1</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>KAYA</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>316.8</v>
+        <v>21.01</v>
       </c>
       <c r="C168" t="n">
-        <v>324.85</v>
+        <v>21.45</v>
       </c>
       <c r="D168" t="n">
-        <v>2.54</v>
+        <v>2.09</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>21.38</v>
+        <v>37.52</v>
       </c>
       <c r="C169" t="n">
-        <v>21.92</v>
+        <v>38.3</v>
       </c>
       <c r="D169" t="n">
-        <v>2.53</v>
+        <v>2.08</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>PARIN</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>67.7</v>
+        <v>720.1</v>
       </c>
       <c r="C170" t="n">
-        <v>69.40000000000001</v>
+        <v>735</v>
       </c>
       <c r="D170" t="n">
-        <v>2.51</v>
+        <v>2.07</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>654.6</v>
+        <v>203.81</v>
       </c>
       <c r="C171" t="n">
-        <v>671</v>
+        <v>208</v>
       </c>
       <c r="D171" t="n">
-        <v>2.51</v>
+        <v>2.06</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>ASMS</t>
+          <t>MADRASFERT</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>6.38</v>
+        <v>59.18</v>
       </c>
       <c r="C172" t="n">
-        <v>6.54</v>
+        <v>60.4</v>
       </c>
       <c r="D172" t="n">
-        <v>2.51</v>
+        <v>2.06</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SUNDROP</t>
+          <t>AZAD</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>745.75</v>
+        <v>2723.2</v>
       </c>
       <c r="C173" t="n">
-        <v>764.4</v>
+        <v>2779</v>
       </c>
       <c r="D173" t="n">
-        <v>2.5</v>
+        <v>2.05</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>MOKSH</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C174" t="n">
-        <v>8.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="D174" t="n">
-        <v>2.5</v>
+        <v>2.04</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ZIMLAB</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>138.48</v>
+        <v>8.81</v>
       </c>
       <c r="C175" t="n">
-        <v>141.94</v>
+        <v>8.99</v>
       </c>
       <c r="D175" t="n">
-        <v>2.5</v>
+        <v>2.04</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>IFBAGRO</t>
+          <t>WARDINMOBI</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>858.6</v>
+        <v>5.43</v>
       </c>
       <c r="C176" t="n">
-        <v>880</v>
+        <v>5.54</v>
       </c>
       <c r="D176" t="n">
-        <v>2.49</v>
+        <v>2.03</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>STARTECK</t>
+          <t>NAHARINDUS</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>262.5</v>
+        <v>127.47</v>
       </c>
       <c r="C177" t="n">
-        <v>269</v>
+        <v>130.05</v>
       </c>
       <c r="D177" t="n">
-        <v>2.48</v>
+        <v>2.02</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HARDWYN</t>
+          <t>MAANALU</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>9.27</v>
+        <v>100.86</v>
       </c>
       <c r="C178" t="n">
-        <v>9.5</v>
+        <v>102.9</v>
       </c>
       <c r="D178" t="n">
-        <v>2.48</v>
+        <v>2.02</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>SUNRAKSHAK</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>280.05</v>
+        <v>359.65</v>
       </c>
       <c r="C179" t="n">
-        <v>287</v>
+        <v>366.9</v>
       </c>
       <c r="D179" t="n">
-        <v>2.48</v>
+        <v>2.02</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.8100000000000001</v>
+        <v>27.9</v>
       </c>
       <c r="C180" t="n">
-        <v>0.83</v>
+        <v>28.46</v>
       </c>
       <c r="D180" t="n">
-        <v>2.47</v>
+        <v>2.01</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>TRACXN</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>50.75</v>
+        <v>32.33</v>
       </c>
       <c r="C181" t="n">
-        <v>52</v>
+        <v>32.98</v>
       </c>
       <c r="D181" t="n">
-        <v>2.46</v>
+        <v>2.01</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>SSEGL</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>396.3</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="C182" t="n">
-        <v>406</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="D182" t="n">
-        <v>2.45</v>
+        <v>2.01</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>ANSALAPI</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>77.59999999999999</v>
+        <v>4</v>
       </c>
       <c r="C183" t="n">
-        <v>79.5</v>
+        <v>4.08</v>
       </c>
       <c r="D183" t="n">
-        <v>2.45</v>
+        <v>2</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>2.05</v>
+        <v>113.72</v>
       </c>
       <c r="C184" t="n">
-        <v>2.1</v>
+        <v>115.99</v>
       </c>
       <c r="D184" t="n">
-        <v>2.44</v>
+        <v>2</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>25.13</v>
+        <v>465.52</v>
       </c>
       <c r="C185" t="n">
-        <v>25.74</v>
+        <v>474.83</v>
       </c>
       <c r="D185" t="n">
-        <v>2.43</v>
+        <v>2</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1737.8</v>
+        <v>6.54</v>
       </c>
       <c r="C186" t="n">
-        <v>1780</v>
+        <v>6.67</v>
       </c>
       <c r="D186" t="n">
-        <v>2.43</v>
+        <v>1.99</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>AUGMONT</t>
+          <t>PARSVNATH</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>877.9</v>
+        <v>2.01</v>
       </c>
       <c r="C187" t="n">
-        <v>899</v>
+        <v>2.05</v>
       </c>
       <c r="D187" t="n">
-        <v>2.4</v>
+        <v>1.99</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>13.34</v>
+        <v>117.27</v>
       </c>
       <c r="C188" t="n">
-        <v>13.66</v>
+        <v>119.6</v>
       </c>
       <c r="D188" t="n">
-        <v>2.4</v>
+        <v>1.99</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>ABAN</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>4.19</v>
+        <v>14.07</v>
       </c>
       <c r="C189" t="n">
-        <v>4.29</v>
+        <v>14.35</v>
       </c>
       <c r="D189" t="n">
-        <v>2.39</v>
+        <v>1.99</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>HUHTAMAKI</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>5.85</v>
+        <v>234.2</v>
       </c>
       <c r="C190" t="n">
-        <v>5.99</v>
+        <v>238.85</v>
       </c>
       <c r="D190" t="n">
-        <v>2.39</v>
+        <v>1.99</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ESTER</t>
+          <t>SEYAIND</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>86.14</v>
+        <v>13.6</v>
       </c>
       <c r="C191" t="n">
-        <v>88.2</v>
+        <v>13.87</v>
       </c>
       <c r="D191" t="n">
-        <v>2.39</v>
+        <v>1.99</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>VIVIDEL</t>
+          <t>LAHOTIOV</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>1773.7</v>
+        <v>40.2</v>
       </c>
       <c r="C192" t="n">
-        <v>1816</v>
+        <v>41</v>
       </c>
       <c r="D192" t="n">
-        <v>2.38</v>
+        <v>1.99</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>PRESSTONIC</t>
+          <t>SCHAND</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>52.5</v>
+        <v>144.65</v>
       </c>
       <c r="C193" t="n">
-        <v>53.75</v>
+        <v>147.5</v>
       </c>
       <c r="D193" t="n">
-        <v>2.38</v>
+        <v>1.97</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>29.44</v>
+        <v>5.09</v>
       </c>
       <c r="C194" t="n">
-        <v>30.14</v>
+        <v>5.19</v>
       </c>
       <c r="D194" t="n">
-        <v>2.38</v>
+        <v>1.96</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>VETO</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>150.32</v>
+        <v>130.05</v>
       </c>
       <c r="C195" t="n">
-        <v>153.89</v>
+        <v>132.6</v>
       </c>
       <c r="D195" t="n">
-        <v>2.37</v>
+        <v>1.96</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ABDL</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>715.05</v>
+        <v>22.93</v>
       </c>
       <c r="C196" t="n">
-        <v>731.95</v>
+        <v>23.38</v>
       </c>
       <c r="D196" t="n">
-        <v>2.36</v>
+        <v>1.96</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>31.51</v>
+        <v>6.65</v>
       </c>
       <c r="C197" t="n">
-        <v>32.25</v>
+        <v>6.78</v>
       </c>
       <c r="D197" t="n">
-        <v>2.35</v>
+        <v>1.95</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>UNIDT</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>241.71</v>
+        <v>2.06</v>
       </c>
       <c r="C198" t="n">
-        <v>247.4</v>
+        <v>2.1</v>
       </c>
       <c r="D198" t="n">
-        <v>2.35</v>
+        <v>1.94</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>1164.9</v>
+        <v>5.66</v>
       </c>
       <c r="C199" t="n">
-        <v>1192</v>
+        <v>5.77</v>
       </c>
       <c r="D199" t="n">
-        <v>2.33</v>
+        <v>1.94</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>167.05</v>
+        <v>6.26</v>
       </c>
       <c r="C200" t="n">
-        <v>170.95</v>
+        <v>6.38</v>
       </c>
       <c r="D200" t="n">
-        <v>2.33</v>
+        <v>1.92</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>LAMBODHARA</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>13.18</v>
+        <v>135.19</v>
       </c>
       <c r="C201" t="n">
-        <v>13.48</v>
+        <v>137.79</v>
       </c>
       <c r="D201" t="n">
-        <v>2.28</v>
+        <v>1.92</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-09-30 10:00 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>CENTEXT-RE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24.07</v>
+        <v>2.79</v>
       </c>
       <c r="C2" t="n">
-        <v>28.88</v>
+        <v>3.88</v>
       </c>
       <c r="D2" t="n">
-        <v>19.98</v>
+        <v>39.07</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.74</v>
+        <v>717</v>
       </c>
       <c r="C3" t="n">
-        <v>0.85</v>
+        <v>860.4</v>
       </c>
       <c r="D3" t="n">
-        <v>14.86</v>
+        <v>20</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11.89</v>
+        <v>92.72</v>
       </c>
       <c r="C4" t="n">
-        <v>13.5</v>
+        <v>111.26</v>
       </c>
       <c r="D4" t="n">
-        <v>13.54</v>
+        <v>20</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REGENCERAM</t>
+          <t>GENXAI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32.64</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>36.92</v>
+        <v>88.95</v>
       </c>
       <c r="D5" t="n">
-        <v>13.11</v>
+        <v>17.58</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ELLEN</t>
+          <t>JOCIL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>359.05</v>
+        <v>145.17</v>
       </c>
       <c r="C6" t="n">
-        <v>394.95</v>
+        <v>162</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>11.59</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,14 +571,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30.36</v>
+        <v>29.66</v>
       </c>
       <c r="C7" t="n">
-        <v>33.39</v>
+        <v>32.62</v>
       </c>
       <c r="D7" t="n">
         <v>9.98</v>
@@ -593,14 +593,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26.97</v>
+        <v>28.88</v>
       </c>
       <c r="C8" t="n">
-        <v>29.66</v>
+        <v>31.76</v>
       </c>
       <c r="D8" t="n">
         <v>9.970000000000001</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RTSPOWR</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>125.5</v>
+        <v>10.38</v>
       </c>
       <c r="C9" t="n">
-        <v>136.77</v>
+        <v>11.4</v>
       </c>
       <c r="D9" t="n">
-        <v>8.98</v>
+        <v>9.83</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>COMPEAU</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>353.05</v>
+        <v>0.88</v>
       </c>
       <c r="C10" t="n">
-        <v>383.9</v>
+        <v>0.96</v>
       </c>
       <c r="D10" t="n">
-        <v>8.74</v>
+        <v>9.09</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>STARTECK</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>314</v>
+        <v>77.83</v>
       </c>
       <c r="C11" t="n">
-        <v>340</v>
+        <v>84.75</v>
       </c>
       <c r="D11" t="n">
-        <v>8.279999999999999</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AXISCADES</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1879.5</v>
+        <v>22.31</v>
       </c>
       <c r="C12" t="n">
-        <v>2034</v>
+        <v>24</v>
       </c>
       <c r="D12" t="n">
-        <v>8.220000000000001</v>
+        <v>7.58</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CREATIVEYE</t>
+          <t>VIRAT</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.72</v>
+        <v>340.2</v>
       </c>
       <c r="C13" t="n">
-        <v>6.18</v>
+        <v>364.95</v>
       </c>
       <c r="D13" t="n">
-        <v>8.039999999999999</v>
+        <v>7.28</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9.119999999999999</v>
+        <v>0.14</v>
       </c>
       <c r="C14" t="n">
-        <v>9.800000000000001</v>
+        <v>0.15</v>
       </c>
       <c r="D14" t="n">
-        <v>7.46</v>
+        <v>7.14</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VIVOBIOT</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16.26</v>
+        <v>10.25</v>
       </c>
       <c r="C15" t="n">
-        <v>17.44</v>
+        <v>10.97</v>
       </c>
       <c r="D15" t="n">
-        <v>7.26</v>
+        <v>7.02</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ESTER</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.14</v>
+        <v>84.55</v>
       </c>
       <c r="C16" t="n">
-        <v>0.15</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>7.14</v>
+        <v>6.45</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>THOMASCOTT</t>
+          <t>KEYFINSERV</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>238.35</v>
+        <v>233</v>
       </c>
       <c r="C17" t="n">
-        <v>255</v>
+        <v>247.8</v>
       </c>
       <c r="D17" t="n">
-        <v>6.99</v>
+        <v>6.35</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>72.17</v>
+        <v>4.41</v>
       </c>
       <c r="C18" t="n">
-        <v>77</v>
+        <v>4.69</v>
       </c>
       <c r="D18" t="n">
-        <v>6.69</v>
+        <v>6.35</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GILLANDERS</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>107.38</v>
+        <v>149.26</v>
       </c>
       <c r="C19" t="n">
-        <v>114</v>
+        <v>158.2</v>
       </c>
       <c r="D19" t="n">
-        <v>6.17</v>
+        <v>5.99</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>MGSL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>81.52</v>
+        <v>63.25</v>
       </c>
       <c r="C20" t="n">
-        <v>86.52</v>
+        <v>66.95</v>
       </c>
       <c r="D20" t="n">
-        <v>6.13</v>
+        <v>5.85</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DUCOL</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>115</v>
+        <v>168.37</v>
       </c>
       <c r="C21" t="n">
-        <v>121.9</v>
+        <v>177.9</v>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>5.66</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AUGMONT</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>965.65</v>
+        <v>0.18</v>
       </c>
       <c r="C22" t="n">
-        <v>1022</v>
+        <v>0.19</v>
       </c>
       <c r="D22" t="n">
-        <v>5.84</v>
+        <v>5.56</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>TPLPLASTEH</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.18</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="C23" t="n">
-        <v>0.19</v>
+        <v>68.67</v>
       </c>
       <c r="D23" t="n">
-        <v>5.56</v>
+        <v>5.23</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>165.91</v>
+        <v>21.76</v>
       </c>
       <c r="C24" t="n">
-        <v>175</v>
+        <v>22.88</v>
       </c>
       <c r="D24" t="n">
-        <v>5.48</v>
+        <v>5.15</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>275.21</v>
+        <v>1665.8</v>
       </c>
       <c r="C25" t="n">
-        <v>290</v>
+        <v>1750</v>
       </c>
       <c r="D25" t="n">
-        <v>5.37</v>
+        <v>5.05</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SHIGAN</t>
+          <t>SHANKARA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>60.55</v>
+        <v>127.47</v>
       </c>
       <c r="C26" t="n">
-        <v>63.8</v>
+        <v>133.9</v>
       </c>
       <c r="D26" t="n">
-        <v>5.37</v>
+        <v>5.04</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>NEWJAISA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.19</v>
+        <v>18</v>
       </c>
       <c r="C27" t="n">
-        <v>0.2</v>
+        <v>18.9</v>
       </c>
       <c r="D27" t="n">
-        <v>5.26</v>
+        <v>5</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>MTARTECH</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18.87</v>
+        <v>7426</v>
       </c>
       <c r="C28" t="n">
-        <v>19.85</v>
+        <v>7797</v>
       </c>
       <c r="D28" t="n">
-        <v>5.19</v>
+        <v>5</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>10.26</v>
+        <v>866.6</v>
       </c>
       <c r="C29" t="n">
-        <v>10.79</v>
+        <v>909.9</v>
       </c>
       <c r="D29" t="n">
-        <v>5.17</v>
+        <v>5</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,14 +1077,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>189.91</v>
+        <v>216.21</v>
       </c>
       <c r="C30" t="n">
-        <v>199.4</v>
+        <v>227.02</v>
       </c>
       <c r="D30" t="n">
         <v>5</v>
@@ -1099,14 +1099,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>216.9</v>
+        <v>26.18</v>
       </c>
       <c r="C31" t="n">
-        <v>227.74</v>
+        <v>27.49</v>
       </c>
       <c r="D31" t="n">
         <v>5</v>
@@ -1125,13 +1125,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>406.25</v>
+        <v>426.55</v>
       </c>
       <c r="C32" t="n">
-        <v>426.55</v>
+        <v>447.85</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>AMEYA</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>145.85</v>
+        <v>146.2</v>
       </c>
       <c r="C33" t="n">
-        <v>153.14</v>
+        <v>153.5</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>206.47</v>
+        <v>49.46</v>
       </c>
       <c r="C34" t="n">
-        <v>216.79</v>
+        <v>51.93</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1191,13 +1191,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>34.07</v>
+        <v>35.77</v>
       </c>
       <c r="C35" t="n">
-        <v>35.77</v>
+        <v>37.55</v>
       </c>
       <c r="D35" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>BHADORA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>231.35</v>
+        <v>133.6</v>
       </c>
       <c r="C36" t="n">
-        <v>242.9</v>
+        <v>140.25</v>
       </c>
       <c r="D36" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>34.66</v>
+        <v>30.18</v>
       </c>
       <c r="C37" t="n">
-        <v>36.39</v>
+        <v>31.68</v>
       </c>
       <c r="D37" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AKANKSHA</t>
+          <t>PRIMECAB</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>159.7</v>
+        <v>187.1</v>
       </c>
       <c r="C38" t="n">
-        <v>167.65</v>
+        <v>196.4</v>
       </c>
       <c r="D38" t="n">
-        <v>4.98</v>
+        <v>4.97</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>RHETAN</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>159.6</v>
+        <v>16.69</v>
       </c>
       <c r="C39" t="n">
-        <v>167.55</v>
+        <v>17.52</v>
       </c>
       <c r="D39" t="n">
-        <v>4.98</v>
+        <v>4.97</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BLUEWATER</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>561.45</v>
+        <v>14.12</v>
       </c>
       <c r="C40" t="n">
-        <v>589.4</v>
+        <v>14.82</v>
       </c>
       <c r="D40" t="n">
-        <v>4.98</v>
+        <v>4.96</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ARMOUR</t>
+          <t>BIOPOL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>21.1</v>
+        <v>51.45</v>
       </c>
       <c r="C41" t="n">
-        <v>22.15</v>
+        <v>54</v>
       </c>
       <c r="D41" t="n">
-        <v>4.98</v>
+        <v>4.96</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>10.87</v>
+        <v>20.77</v>
       </c>
       <c r="C42" t="n">
-        <v>11.41</v>
+        <v>21.8</v>
       </c>
       <c r="D42" t="n">
-        <v>4.97</v>
+        <v>4.96</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>28.75</v>
+        <v>7.07</v>
       </c>
       <c r="C43" t="n">
-        <v>30.18</v>
+        <v>7.42</v>
       </c>
       <c r="D43" t="n">
-        <v>4.97</v>
+        <v>4.95</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>NEUEON</t>
+          <t>KORE</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>15.1</v>
+        <v>188.2</v>
       </c>
       <c r="C44" t="n">
-        <v>15.85</v>
+        <v>197.5</v>
       </c>
       <c r="D44" t="n">
-        <v>4.97</v>
+        <v>4.94</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>HITECHGEAR</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>648.85</v>
+        <v>50.95</v>
       </c>
       <c r="C45" t="n">
-        <v>680.9</v>
+        <v>53.45</v>
       </c>
       <c r="D45" t="n">
-        <v>4.94</v>
+        <v>4.91</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GOLDSTAR</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>11.15</v>
+        <v>7.34</v>
       </c>
       <c r="C46" t="n">
-        <v>11.7</v>
+        <v>7.7</v>
       </c>
       <c r="D46" t="n">
-        <v>4.93</v>
+        <v>4.9</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MOMSBELIEF</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>223.01</v>
+        <v>66.72</v>
       </c>
       <c r="C47" t="n">
-        <v>234</v>
+        <v>69.95</v>
       </c>
       <c r="D47" t="n">
-        <v>4.93</v>
+        <v>4.84</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LAKSHYA</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>118.8</v>
+        <v>23.32</v>
       </c>
       <c r="C48" t="n">
-        <v>124.65</v>
+        <v>24.44</v>
       </c>
       <c r="D48" t="n">
-        <v>4.92</v>
+        <v>4.8</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MPEL</t>
+          <t>LRRPL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>26.5</v>
+        <v>103.05</v>
       </c>
       <c r="C49" t="n">
-        <v>27.8</v>
+        <v>108</v>
       </c>
       <c r="D49" t="n">
-        <v>4.91</v>
+        <v>4.8</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>33.65</v>
+        <v>1.47</v>
       </c>
       <c r="C50" t="n">
-        <v>35.3</v>
+        <v>1.54</v>
       </c>
       <c r="D50" t="n">
-        <v>4.9</v>
+        <v>4.76</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6.74</v>
+        <v>8</v>
       </c>
       <c r="C51" t="n">
-        <v>7.07</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="D51" t="n">
-        <v>4.9</v>
+        <v>4.75</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RHETAN</t>
+          <t>CHEMFAB</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15.91</v>
+        <v>343.5</v>
       </c>
       <c r="C52" t="n">
-        <v>16.69</v>
+        <v>359.8</v>
       </c>
       <c r="D52" t="n">
-        <v>4.9</v>
+        <v>4.75</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2.29</v>
+        <v>5.27</v>
       </c>
       <c r="C53" t="n">
-        <v>2.4</v>
+        <v>5.52</v>
       </c>
       <c r="D53" t="n">
-        <v>4.8</v>
+        <v>4.74</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>QUADPRO</t>
+          <t>MOLBIO</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>4.2</v>
+        <v>1255.6</v>
       </c>
       <c r="C54" t="n">
-        <v>4.4</v>
+        <v>1314.9</v>
       </c>
       <c r="D54" t="n">
-        <v>4.76</v>
+        <v>4.72</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>KORE</t>
+          <t>VISL</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>189.15</v>
+        <v>32.85</v>
       </c>
       <c r="C55" t="n">
-        <v>198.15</v>
+        <v>34.4</v>
       </c>
       <c r="D55" t="n">
-        <v>4.76</v>
+        <v>4.72</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>GOLDSTAR</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2.52</v>
+        <v>11.7</v>
       </c>
       <c r="C56" t="n">
-        <v>2.64</v>
+        <v>12.25</v>
       </c>
       <c r="D56" t="n">
-        <v>4.76</v>
+        <v>4.7</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PRASOLCHEM</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>763.8</v>
+        <v>33.39</v>
       </c>
       <c r="C57" t="n">
-        <v>799.9</v>
+        <v>34.95</v>
       </c>
       <c r="D57" t="n">
-        <v>4.73</v>
+        <v>4.67</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>MASKINVEST</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>9.119999999999999</v>
+        <v>147.18</v>
       </c>
       <c r="C58" t="n">
-        <v>9.550000000000001</v>
+        <v>154</v>
       </c>
       <c r="D58" t="n">
-        <v>4.71</v>
+        <v>4.63</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SAPPL</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>279.95</v>
+        <v>43.56</v>
       </c>
       <c r="C59" t="n">
-        <v>293</v>
+        <v>45.55</v>
       </c>
       <c r="D59" t="n">
-        <v>4.66</v>
+        <v>4.57</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PARNAXLAB</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>112.78</v>
+        <v>51.08</v>
       </c>
       <c r="C60" t="n">
-        <v>118</v>
+        <v>53.39</v>
       </c>
       <c r="D60" t="n">
-        <v>4.63</v>
+        <v>4.52</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>5.02</v>
+        <v>26.79</v>
       </c>
       <c r="C61" t="n">
-        <v>5.25</v>
+        <v>27.99</v>
       </c>
       <c r="D61" t="n">
-        <v>4.58</v>
+        <v>4.48</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>21.99</v>
+        <v>243.95</v>
       </c>
       <c r="C62" t="n">
-        <v>22.99</v>
+        <v>254.85</v>
       </c>
       <c r="D62" t="n">
-        <v>4.55</v>
+        <v>4.47</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>FERMENTA</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>479.3</v>
+        <v>153.14</v>
       </c>
       <c r="C63" t="n">
-        <v>501</v>
+        <v>159.99</v>
       </c>
       <c r="D63" t="n">
-        <v>4.53</v>
+        <v>4.47</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DGCONTENT</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>23.37</v>
+        <v>93.19</v>
       </c>
       <c r="C64" t="n">
-        <v>24.4</v>
+        <v>97.2</v>
       </c>
       <c r="D64" t="n">
-        <v>4.41</v>
+        <v>4.3</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.6899999999999999</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="C65" t="n">
-        <v>0.72</v>
+        <v>8.75</v>
       </c>
       <c r="D65" t="n">
-        <v>4.35</v>
+        <v>4.29</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>KSB</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1.38</v>
+        <v>824.8</v>
       </c>
       <c r="C66" t="n">
-        <v>1.44</v>
+        <v>860</v>
       </c>
       <c r="D66" t="n">
-        <v>4.35</v>
+        <v>4.27</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GANESHBE</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>137.32</v>
+        <v>0.47</v>
       </c>
       <c r="C67" t="n">
-        <v>143</v>
+        <v>0.49</v>
       </c>
       <c r="D67" t="n">
-        <v>4.14</v>
+        <v>4.26</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ARVEE</t>
+          <t>ORBTEXP</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>234.5</v>
+        <v>262.01</v>
       </c>
       <c r="C68" t="n">
-        <v>244</v>
+        <v>272.85</v>
       </c>
       <c r="D68" t="n">
-        <v>4.05</v>
+        <v>4.14</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>KPIGREEN</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>219.2</v>
+        <v>371.25</v>
       </c>
       <c r="C69" t="n">
-        <v>227.99</v>
+        <v>386.4</v>
       </c>
       <c r="D69" t="n">
-        <v>4.01</v>
+        <v>4.08</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TIPSFILMS</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>331.8</v>
+        <v>139.25</v>
       </c>
       <c r="C70" t="n">
-        <v>345</v>
+        <v>144.9</v>
       </c>
       <c r="D70" t="n">
-        <v>3.98</v>
+        <v>4.06</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,14 +1979,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>DUGLOBAL</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>15.37</v>
+        <v>20.15</v>
       </c>
       <c r="C71" t="n">
-        <v>15.98</v>
+        <v>20.95</v>
       </c>
       <c r="D71" t="n">
         <v>3.97</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>24.29</v>
+        <v>36.88</v>
       </c>
       <c r="C72" t="n">
-        <v>25.25</v>
+        <v>38.34</v>
       </c>
       <c r="D72" t="n">
-        <v>3.95</v>
+        <v>3.96</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>EBIX</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>4.94</v>
+        <v>17.01</v>
       </c>
       <c r="C73" t="n">
-        <v>5.13</v>
+        <v>17.68</v>
       </c>
       <c r="D73" t="n">
-        <v>3.85</v>
+        <v>3.94</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SARTELE</t>
+          <t>VTMLTD</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>84.8</v>
+        <v>39.93</v>
       </c>
       <c r="C74" t="n">
-        <v>88</v>
+        <v>41.49</v>
       </c>
       <c r="D74" t="n">
-        <v>3.77</v>
+        <v>3.91</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ESSARSHPNG</t>
+          <t>PRIORITY</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>15.63</v>
+        <v>293.64</v>
       </c>
       <c r="C75" t="n">
-        <v>16.21</v>
+        <v>305</v>
       </c>
       <c r="D75" t="n">
-        <v>3.71</v>
+        <v>3.87</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MOTOGENFIN</t>
+          <t>POWERMECH</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>25.7</v>
+        <v>2397.2</v>
       </c>
       <c r="C76" t="n">
-        <v>26.65</v>
+        <v>2488.9</v>
       </c>
       <c r="D76" t="n">
-        <v>3.7</v>
+        <v>3.83</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HYBRIDFIN</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>17.36</v>
+        <v>502.85</v>
       </c>
       <c r="C77" t="n">
-        <v>18</v>
+        <v>522</v>
       </c>
       <c r="D77" t="n">
-        <v>3.69</v>
+        <v>3.81</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>58.81</v>
+        <v>22.93</v>
       </c>
       <c r="C78" t="n">
-        <v>60.9</v>
+        <v>23.8</v>
       </c>
       <c r="D78" t="n">
-        <v>3.55</v>
+        <v>3.79</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>53.6</v>
+        <v>13.47</v>
       </c>
       <c r="C79" t="n">
-        <v>55.5</v>
+        <v>13.98</v>
       </c>
       <c r="D79" t="n">
-        <v>3.54</v>
+        <v>3.79</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>EBGNG</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>37</v>
+        <v>674.8</v>
       </c>
       <c r="C80" t="n">
-        <v>38.3</v>
+        <v>700.05</v>
       </c>
       <c r="D80" t="n">
-        <v>3.51</v>
+        <v>3.74</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SSRETAIL</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>716.95</v>
+        <v>19.57</v>
       </c>
       <c r="C81" t="n">
-        <v>742.15</v>
+        <v>20.3</v>
       </c>
       <c r="D81" t="n">
-        <v>3.51</v>
+        <v>3.73</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>21.73</v>
+        <v>2.15</v>
       </c>
       <c r="C82" t="n">
-        <v>22.49</v>
+        <v>2.23</v>
       </c>
       <c r="D82" t="n">
-        <v>3.5</v>
+        <v>3.72</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>13.51</v>
+        <v>0.27</v>
       </c>
       <c r="C83" t="n">
-        <v>13.98</v>
+        <v>0.28</v>
       </c>
       <c r="D83" t="n">
-        <v>3.48</v>
+        <v>3.7</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>ARIS</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.29</v>
+        <v>135</v>
       </c>
       <c r="C84" t="n">
-        <v>0.3</v>
+        <v>140</v>
       </c>
       <c r="D84" t="n">
-        <v>3.45</v>
+        <v>3.7</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DAICHI</t>
+          <t>SAMPANN</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>316</v>
+        <v>23.82</v>
       </c>
       <c r="C85" t="n">
-        <v>326.85</v>
+        <v>24.7</v>
       </c>
       <c r="D85" t="n">
-        <v>3.43</v>
+        <v>3.69</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>7.9</v>
+        <v>30.74</v>
       </c>
       <c r="C86" t="n">
-        <v>8.17</v>
+        <v>31.87</v>
       </c>
       <c r="D86" t="n">
-        <v>3.42</v>
+        <v>3.68</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>NICCOPAR</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.88</v>
+        <v>81</v>
       </c>
       <c r="C87" t="n">
-        <v>0.91</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="D87" t="n">
-        <v>3.41</v>
+        <v>3.58</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>ESSARSHPNG</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>50.36</v>
+        <v>16.95</v>
       </c>
       <c r="C88" t="n">
-        <v>52.07</v>
+        <v>17.54</v>
       </c>
       <c r="D88" t="n">
-        <v>3.4</v>
+        <v>3.48</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>10.05</v>
+        <v>119.85</v>
       </c>
       <c r="C89" t="n">
-        <v>10.39</v>
+        <v>124</v>
       </c>
       <c r="D89" t="n">
-        <v>3.38</v>
+        <v>3.46</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>107.7</v>
+        <v>0.29</v>
       </c>
       <c r="C90" t="n">
-        <v>111.3</v>
+        <v>0.3</v>
       </c>
       <c r="D90" t="n">
-        <v>3.34</v>
+        <v>3.45</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>4.84</v>
+        <v>14.48</v>
       </c>
       <c r="C91" t="n">
-        <v>5</v>
+        <v>14.98</v>
       </c>
       <c r="D91" t="n">
-        <v>3.31</v>
+        <v>3.45</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MARALOVER</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>59.37</v>
+        <v>29.97</v>
       </c>
       <c r="C92" t="n">
-        <v>61.29</v>
+        <v>31</v>
       </c>
       <c r="D92" t="n">
-        <v>3.23</v>
+        <v>3.44</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ADDIND</t>
+          <t>LEENEE</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>77.5</v>
+        <v>7.58</v>
       </c>
       <c r="C93" t="n">
-        <v>80</v>
+        <v>7.84</v>
       </c>
       <c r="D93" t="n">
-        <v>3.23</v>
+        <v>3.43</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>KILITCH</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>217.05</v>
+        <v>21.77</v>
       </c>
       <c r="C94" t="n">
-        <v>224</v>
+        <v>22.5</v>
       </c>
       <c r="D94" t="n">
-        <v>3.2</v>
+        <v>3.35</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>PRASOLCHEM</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>11.14</v>
+        <v>840.15</v>
       </c>
       <c r="C95" t="n">
-        <v>11.49</v>
+        <v>868.25</v>
       </c>
       <c r="D95" t="n">
-        <v>3.14</v>
+        <v>3.34</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>KMEW</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2876.9</v>
+        <v>59.9</v>
       </c>
       <c r="C96" t="n">
-        <v>2965.1</v>
+        <v>61.88</v>
       </c>
       <c r="D96" t="n">
-        <v>3.07</v>
+        <v>3.31</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>28.13</v>
+        <v>18.4</v>
       </c>
       <c r="C97" t="n">
-        <v>28.99</v>
+        <v>19</v>
       </c>
       <c r="D97" t="n">
-        <v>3.06</v>
+        <v>3.26</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>49.52</v>
+        <v>14.23</v>
       </c>
       <c r="C98" t="n">
-        <v>51</v>
+        <v>14.69</v>
       </c>
       <c r="D98" t="n">
-        <v>2.99</v>
+        <v>3.23</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>YOGI</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>34.39</v>
+        <v>156.67</v>
       </c>
       <c r="C99" t="n">
-        <v>35.4</v>
+        <v>161.7</v>
       </c>
       <c r="D99" t="n">
-        <v>2.94</v>
+        <v>3.21</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>KHAITANLTD</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>3133.7</v>
+        <v>150.01</v>
       </c>
       <c r="C100" t="n">
-        <v>3225</v>
+        <v>154.79</v>
       </c>
       <c r="D100" t="n">
-        <v>2.91</v>
+        <v>3.19</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PREMIERPOL</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>92.81</v>
+        <v>69.52</v>
       </c>
       <c r="C101" t="n">
-        <v>95.48999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="D101" t="n">
-        <v>2.89</v>
+        <v>3.14</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>26.4</v>
+        <v>1190.5</v>
       </c>
       <c r="C102" t="n">
-        <v>27.16</v>
+        <v>1227.8</v>
       </c>
       <c r="D102" t="n">
-        <v>2.88</v>
+        <v>3.13</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SETL</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>422.65</v>
+        <v>6.73</v>
       </c>
       <c r="C103" t="n">
-        <v>434.7</v>
+        <v>6.94</v>
       </c>
       <c r="D103" t="n">
-        <v>2.85</v>
+        <v>3.12</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ORBTEXP</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>227.15</v>
+        <v>178.52</v>
       </c>
       <c r="C104" t="n">
-        <v>233.6</v>
+        <v>184</v>
       </c>
       <c r="D104" t="n">
-        <v>2.84</v>
+        <v>3.07</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ENIL</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>96.01000000000001</v>
+        <v>993</v>
       </c>
       <c r="C105" t="n">
-        <v>98.73999999999999</v>
+        <v>1023.5</v>
       </c>
       <c r="D105" t="n">
-        <v>2.84</v>
+        <v>3.07</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>69.04000000000001</v>
+        <v>113.05</v>
       </c>
       <c r="C106" t="n">
-        <v>70.98999999999999</v>
+        <v>116.5</v>
       </c>
       <c r="D106" t="n">
-        <v>2.82</v>
+        <v>3.05</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SOMICONVEY</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>89.18000000000001</v>
+        <v>1.32</v>
       </c>
       <c r="C107" t="n">
-        <v>91.68000000000001</v>
+        <v>1.36</v>
       </c>
       <c r="D107" t="n">
-        <v>2.8</v>
+        <v>3.03</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>INVPRECQ</t>
+          <t>LKPSEC</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>1501.5</v>
+        <v>14.27</v>
       </c>
       <c r="C108" t="n">
-        <v>1543.6</v>
+        <v>14.7</v>
       </c>
       <c r="D108" t="n">
-        <v>2.8</v>
+        <v>3.01</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>RCDL</t>
+          <t>BAJAJINDEF</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>17.9</v>
+        <v>213.11</v>
       </c>
       <c r="C109" t="n">
-        <v>18.4</v>
+        <v>219.44</v>
       </c>
       <c r="D109" t="n">
-        <v>2.79</v>
+        <v>2.97</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ZFSTEERING</t>
+          <t>VISHAL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>729.7</v>
+        <v>17.92</v>
       </c>
       <c r="C110" t="n">
-        <v>750</v>
+        <v>18.45</v>
       </c>
       <c r="D110" t="n">
-        <v>2.78</v>
+        <v>2.96</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>5.06</v>
+        <v>3720.9</v>
       </c>
       <c r="C111" t="n">
-        <v>5.2</v>
+        <v>3830</v>
       </c>
       <c r="D111" t="n">
-        <v>2.77</v>
+        <v>2.93</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>BIL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>5.8</v>
+        <v>1000.7</v>
       </c>
       <c r="C112" t="n">
-        <v>5.96</v>
+        <v>1030</v>
       </c>
       <c r="D112" t="n">
-        <v>2.76</v>
+        <v>2.93</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>LOKESHMACH</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>326.1</v>
+        <v>38.64</v>
       </c>
       <c r="C113" t="n">
-        <v>335</v>
+        <v>39.77</v>
       </c>
       <c r="D113" t="n">
-        <v>2.73</v>
+        <v>2.92</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>HINDADH</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>384.45</v>
+        <v>29.43</v>
       </c>
       <c r="C114" t="n">
-        <v>394.95</v>
+        <v>30.29</v>
       </c>
       <c r="D114" t="n">
-        <v>2.73</v>
+        <v>2.92</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>TCIEXP</t>
+          <t>SUYOG</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>486</v>
+        <v>689.95</v>
       </c>
       <c r="C115" t="n">
-        <v>499.2</v>
+        <v>710</v>
       </c>
       <c r="D115" t="n">
-        <v>2.72</v>
+        <v>2.91</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>NCC</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>130.29</v>
+        <v>5.19</v>
       </c>
       <c r="C116" t="n">
-        <v>133.83</v>
+        <v>5.34</v>
       </c>
       <c r="D116" t="n">
-        <v>2.72</v>
+        <v>2.89</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.37</v>
+        <v>5.88</v>
       </c>
       <c r="C117" t="n">
-        <v>0.38</v>
+        <v>6.05</v>
       </c>
       <c r="D117" t="n">
-        <v>2.7</v>
+        <v>2.89</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4.48</v>
+        <v>97.08</v>
       </c>
       <c r="C118" t="n">
-        <v>4.6</v>
+        <v>99.87</v>
       </c>
       <c r="D118" t="n">
-        <v>2.68</v>
+        <v>2.87</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GLOSTERLTD</t>
+          <t>SMARTWORKS</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>545.5</v>
+        <v>514.25</v>
       </c>
       <c r="C119" t="n">
-        <v>559.9</v>
+        <v>528.95</v>
       </c>
       <c r="D119" t="n">
-        <v>2.64</v>
+        <v>2.86</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>ABCOTS</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>4.59</v>
+        <v>198.84</v>
       </c>
       <c r="C120" t="n">
-        <v>4.71</v>
+        <v>204.5</v>
       </c>
       <c r="D120" t="n">
-        <v>2.61</v>
+        <v>2.85</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DCMSIL</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>78.98</v>
+        <v>38.9</v>
       </c>
       <c r="C121" t="n">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="D121" t="n">
-        <v>2.56</v>
+        <v>2.83</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>1.97</v>
+        <v>322.7</v>
       </c>
       <c r="C122" t="n">
-        <v>2.02</v>
+        <v>331.8</v>
       </c>
       <c r="D122" t="n">
-        <v>2.54</v>
+        <v>2.82</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ASMS</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>6.33</v>
+        <v>57.15</v>
       </c>
       <c r="C123" t="n">
-        <v>6.49</v>
+        <v>58.75</v>
       </c>
       <c r="D123" t="n">
-        <v>2.53</v>
+        <v>2.8</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>POEL</t>
+          <t>TIPSFILMS</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>141.35</v>
+        <v>339.55</v>
       </c>
       <c r="C124" t="n">
-        <v>144.91</v>
+        <v>348.95</v>
       </c>
       <c r="D124" t="n">
-        <v>2.52</v>
+        <v>2.77</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>MOHITE</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>2.4</v>
+        <v>35.55</v>
       </c>
       <c r="C125" t="n">
-        <v>2.46</v>
+        <v>36.53</v>
       </c>
       <c r="D125" t="n">
-        <v>2.5</v>
+        <v>2.76</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CENTEXT-RE</t>
+          <t>NKIND</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>2</v>
+        <v>61.99</v>
       </c>
       <c r="C126" t="n">
-        <v>2.05</v>
+        <v>63.7</v>
       </c>
       <c r="D126" t="n">
-        <v>2.5</v>
+        <v>2.76</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SSEGL</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>380.05</v>
+        <v>1675</v>
       </c>
       <c r="C127" t="n">
-        <v>389.5</v>
+        <v>1721</v>
       </c>
       <c r="D127" t="n">
-        <v>2.49</v>
+        <v>2.75</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ONWARDTEC</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>285</v>
+        <v>35.02</v>
       </c>
       <c r="C128" t="n">
-        <v>292</v>
+        <v>35.98</v>
       </c>
       <c r="D128" t="n">
-        <v>2.46</v>
+        <v>2.74</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>AVIENCE</t>
+          <t>REGENCERAM</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>376.25</v>
+        <v>32.51</v>
       </c>
       <c r="C129" t="n">
-        <v>385.5</v>
+        <v>33.4</v>
       </c>
       <c r="D129" t="n">
-        <v>2.46</v>
+        <v>2.74</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>WARDINMOBI</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>67.98</v>
+        <v>5.49</v>
       </c>
       <c r="C130" t="n">
-        <v>69.65000000000001</v>
+        <v>5.64</v>
       </c>
       <c r="D130" t="n">
-        <v>2.46</v>
+        <v>2.73</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>GLOSTERLTD</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>48.65</v>
+        <v>539.25</v>
       </c>
       <c r="C131" t="n">
-        <v>49.84</v>
+        <v>553.9</v>
       </c>
       <c r="D131" t="n">
-        <v>2.45</v>
+        <v>2.72</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>MITCON</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>93.03</v>
+        <v>82.66</v>
       </c>
       <c r="C132" t="n">
-        <v>95.3</v>
+        <v>84.89</v>
       </c>
       <c r="D132" t="n">
-        <v>2.44</v>
+        <v>2.7</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.41</v>
+        <v>194.55</v>
       </c>
       <c r="C133" t="n">
-        <v>0.42</v>
+        <v>199.7</v>
       </c>
       <c r="D133" t="n">
-        <v>2.44</v>
+        <v>2.65</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>2.47</v>
+        <v>1.9</v>
       </c>
       <c r="C134" t="n">
-        <v>2.53</v>
+        <v>1.95</v>
       </c>
       <c r="D134" t="n">
-        <v>2.43</v>
+        <v>2.63</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>8.630000000000001</v>
+        <v>0.38</v>
       </c>
       <c r="C135" t="n">
-        <v>8.84</v>
+        <v>0.39</v>
       </c>
       <c r="D135" t="n">
-        <v>2.43</v>
+        <v>2.63</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>118.97</v>
+        <v>32.14</v>
       </c>
       <c r="C136" t="n">
-        <v>121.85</v>
+        <v>32.98</v>
       </c>
       <c r="D136" t="n">
-        <v>2.42</v>
+        <v>2.61</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>SBCL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>189.43</v>
+        <v>1111.3</v>
       </c>
       <c r="C137" t="n">
-        <v>194</v>
+        <v>1140</v>
       </c>
       <c r="D137" t="n">
-        <v>2.41</v>
+        <v>2.58</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>MEDICO</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>34.08</v>
+        <v>21.84</v>
       </c>
       <c r="C138" t="n">
-        <v>34.9</v>
+        <v>22.4</v>
       </c>
       <c r="D138" t="n">
-        <v>2.41</v>
+        <v>2.56</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>5</v>
+        <v>3186.2</v>
       </c>
       <c r="C139" t="n">
-        <v>5.12</v>
+        <v>3267</v>
       </c>
       <c r="D139" t="n">
-        <v>2.4</v>
+        <v>2.54</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>VIKRAMSOLR</t>
+          <t>COSMOFIRST</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>160.08</v>
+        <v>834.8</v>
       </c>
       <c r="C140" t="n">
-        <v>163.92</v>
+        <v>856</v>
       </c>
       <c r="D140" t="n">
-        <v>2.4</v>
+        <v>2.54</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>MOLDTECH</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>197.29</v>
+        <v>60</v>
       </c>
       <c r="C141" t="n">
-        <v>202</v>
+        <v>61.5</v>
       </c>
       <c r="D141" t="n">
-        <v>2.39</v>
+        <v>2.5</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>150.22</v>
+        <v>199.92</v>
       </c>
       <c r="C142" t="n">
-        <v>153.8</v>
+        <v>204.9</v>
       </c>
       <c r="D142" t="n">
-        <v>2.38</v>
+        <v>2.49</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>KRISHIVAL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>2.96</v>
+        <v>403.95</v>
       </c>
       <c r="C143" t="n">
-        <v>3.03</v>
+        <v>414</v>
       </c>
       <c r="D143" t="n">
-        <v>2.36</v>
+        <v>2.49</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SURAJLTD</t>
+          <t>SADBHAV</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>193.45</v>
+        <v>6.93</v>
       </c>
       <c r="C144" t="n">
-        <v>198</v>
+        <v>7.1</v>
       </c>
       <c r="D144" t="n">
-        <v>2.35</v>
+        <v>2.45</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ACUTAAS</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>3214.4</v>
+        <v>175.61</v>
       </c>
       <c r="C145" t="n">
-        <v>3290</v>
+        <v>179.88</v>
       </c>
       <c r="D145" t="n">
-        <v>2.35</v>
+        <v>2.43</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>HALEOSLABS</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>14.56</v>
+        <v>1487.9</v>
       </c>
       <c r="C146" t="n">
-        <v>14.9</v>
+        <v>1524</v>
       </c>
       <c r="D146" t="n">
-        <v>2.34</v>
+        <v>2.43</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>NURECA</t>
+          <t>ARCHIES</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>362.55</v>
+        <v>12.43</v>
       </c>
       <c r="C147" t="n">
-        <v>371</v>
+        <v>12.73</v>
       </c>
       <c r="D147" t="n">
-        <v>2.33</v>
+        <v>2.41</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>KOTARISUG</t>
+          <t>KHAICHEM</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>26.75</v>
+        <v>49.22</v>
       </c>
       <c r="C148" t="n">
-        <v>27.37</v>
+        <v>50.4</v>
       </c>
       <c r="D148" t="n">
-        <v>2.32</v>
+        <v>2.4</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CENTRUM</t>
+          <t>UNIONBANK</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>20.85</v>
+        <v>166</v>
       </c>
       <c r="C149" t="n">
-        <v>21.33</v>
+        <v>169.98</v>
       </c>
       <c r="D149" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PUNJABCHEM</t>
+          <t>LALITHAA</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1054.6</v>
+        <v>375</v>
       </c>
       <c r="C150" t="n">
-        <v>1078.9</v>
+        <v>384</v>
       </c>
       <c r="D150" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>BLACKROSE</t>
+          <t>KAPSTON</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>116.32</v>
+        <v>555.7</v>
       </c>
       <c r="C151" t="n">
-        <v>118.98</v>
+        <v>569</v>
       </c>
       <c r="D151" t="n">
-        <v>2.29</v>
+        <v>2.39</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ANMOL</t>
+          <t>ALLCARGO</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>13.62</v>
+        <v>10.53</v>
       </c>
       <c r="C152" t="n">
-        <v>13.93</v>
+        <v>10.78</v>
       </c>
       <c r="D152" t="n">
-        <v>2.28</v>
+        <v>2.37</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SUNFLAG</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>449.2</v>
+        <v>150.35</v>
       </c>
       <c r="C153" t="n">
-        <v>459.4</v>
+        <v>153.9</v>
       </c>
       <c r="D153" t="n">
-        <v>2.27</v>
+        <v>2.36</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>SUNLITE</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>0.44</v>
+        <v>625.2</v>
       </c>
       <c r="C154" t="n">
-        <v>0.45</v>
+        <v>639.95</v>
       </c>
       <c r="D154" t="n">
-        <v>2.27</v>
+        <v>2.36</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>ELLEN</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>167.9</v>
+        <v>369.35</v>
       </c>
       <c r="C155" t="n">
-        <v>171.7</v>
+        <v>378</v>
       </c>
       <c r="D155" t="n">
-        <v>2.26</v>
+        <v>2.34</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>DCI</t>
+          <t>MAFATIND</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>326.65</v>
+        <v>115.29</v>
       </c>
       <c r="C156" t="n">
-        <v>334</v>
+        <v>117.98</v>
       </c>
       <c r="D156" t="n">
-        <v>2.25</v>
+        <v>2.33</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>NDL</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>2.67</v>
+        <v>21.5</v>
       </c>
       <c r="C157" t="n">
-        <v>2.73</v>
+        <v>22</v>
       </c>
       <c r="D157" t="n">
-        <v>2.25</v>
+        <v>2.33</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>7.63</v>
+        <v>103.44</v>
       </c>
       <c r="C158" t="n">
-        <v>7.8</v>
+        <v>105.85</v>
       </c>
       <c r="D158" t="n">
-        <v>2.23</v>
+        <v>2.33</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>KAPSTON</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>537.8</v>
+        <v>0.43</v>
       </c>
       <c r="C159" t="n">
-        <v>549.6</v>
+        <v>0.44</v>
       </c>
       <c r="D159" t="n">
-        <v>2.19</v>
+        <v>2.33</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>AGIIL</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>271.6</v>
+        <v>0.86</v>
       </c>
       <c r="C160" t="n">
-        <v>277.55</v>
+        <v>0.88</v>
       </c>
       <c r="D160" t="n">
-        <v>2.19</v>
+        <v>2.33</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.46</v>
+        <v>447.75</v>
       </c>
       <c r="C161" t="n">
-        <v>0.47</v>
+        <v>458.2</v>
       </c>
       <c r="D161" t="n">
-        <v>2.17</v>
+        <v>2.33</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>INDOBORAX</t>
+          <t>AAKASH</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>477.55</v>
+        <v>8.59</v>
       </c>
       <c r="C162" t="n">
-        <v>487.8</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="D162" t="n">
-        <v>2.15</v>
+        <v>2.33</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>SAGARDEEP</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>450.25</v>
+        <v>23.44</v>
       </c>
       <c r="C163" t="n">
-        <v>459.95</v>
+        <v>23.98</v>
       </c>
       <c r="D163" t="n">
-        <v>2.15</v>
+        <v>2.3</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>SAHAJSOLAR</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>31.33</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="C164" t="n">
-        <v>32</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="D164" t="n">
-        <v>2.14</v>
+        <v>2.28</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>CREST</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>36.18</v>
+        <v>356.9</v>
       </c>
       <c r="C165" t="n">
-        <v>36.95</v>
+        <v>364.95</v>
       </c>
       <c r="D165" t="n">
-        <v>2.13</v>
+        <v>2.26</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>12.18</v>
+        <v>205.36</v>
       </c>
       <c r="C166" t="n">
-        <v>12.44</v>
+        <v>209.99</v>
       </c>
       <c r="D166" t="n">
-        <v>2.13</v>
+        <v>2.25</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>39.94</v>
+        <v>13.36</v>
       </c>
       <c r="C167" t="n">
-        <v>40.78</v>
+        <v>13.66</v>
       </c>
       <c r="D167" t="n">
-        <v>2.1</v>
+        <v>2.25</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>21.01</v>
+        <v>11.2</v>
       </c>
       <c r="C168" t="n">
-        <v>21.45</v>
+        <v>11.45</v>
       </c>
       <c r="D168" t="n">
-        <v>2.09</v>
+        <v>2.23</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>ASHUTOSH</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>37.52</v>
+        <v>163.35</v>
       </c>
       <c r="C169" t="n">
-        <v>38.3</v>
+        <v>167</v>
       </c>
       <c r="D169" t="n">
-        <v>2.08</v>
+        <v>2.23</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>PARIN</t>
+          <t>KRITI</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>720.1</v>
+        <v>62.41</v>
       </c>
       <c r="C170" t="n">
-        <v>735</v>
+        <v>63.8</v>
       </c>
       <c r="D170" t="n">
-        <v>2.07</v>
+        <v>2.23</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>203.81</v>
+        <v>0.9</v>
       </c>
       <c r="C171" t="n">
-        <v>208</v>
+        <v>0.92</v>
       </c>
       <c r="D171" t="n">
-        <v>2.06</v>
+        <v>2.22</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MADRASFERT</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>59.18</v>
+        <v>10.84</v>
       </c>
       <c r="C172" t="n">
-        <v>60.4</v>
+        <v>11.08</v>
       </c>
       <c r="D172" t="n">
-        <v>2.06</v>
+        <v>2.21</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>AZAD</t>
+          <t>GALLANTT</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>2723.2</v>
+        <v>539.1</v>
       </c>
       <c r="C173" t="n">
-        <v>2779</v>
+        <v>551</v>
       </c>
       <c r="D173" t="n">
-        <v>2.05</v>
+        <v>2.21</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>9.800000000000001</v>
+        <v>49.64</v>
       </c>
       <c r="C174" t="n">
-        <v>10</v>
+        <v>50.73</v>
       </c>
       <c r="D174" t="n">
-        <v>2.04</v>
+        <v>2.2</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>8.81</v>
+        <v>20.06</v>
       </c>
       <c r="C175" t="n">
-        <v>8.99</v>
+        <v>20.5</v>
       </c>
       <c r="D175" t="n">
-        <v>2.04</v>
+        <v>2.19</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>WARDINMOBI</t>
+          <t>COMSYN</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>5.43</v>
+        <v>261.95</v>
       </c>
       <c r="C176" t="n">
-        <v>5.54</v>
+        <v>267.65</v>
       </c>
       <c r="D176" t="n">
-        <v>2.03</v>
+        <v>2.18</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>NAHARINDUS</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>127.47</v>
+        <v>57.07</v>
       </c>
       <c r="C177" t="n">
-        <v>130.05</v>
+        <v>58.3</v>
       </c>
       <c r="D177" t="n">
-        <v>2.02</v>
+        <v>2.16</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>MAANALU</t>
+          <t>NEXTMEDIA</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>100.86</v>
+        <v>3.7</v>
       </c>
       <c r="C178" t="n">
-        <v>102.9</v>
+        <v>3.78</v>
       </c>
       <c r="D178" t="n">
-        <v>2.02</v>
+        <v>2.16</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SUNRAKSHAK</t>
+          <t>HITECHGEAR</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>359.65</v>
+        <v>625.5</v>
       </c>
       <c r="C179" t="n">
-        <v>366.9</v>
+        <v>639</v>
       </c>
       <c r="D179" t="n">
-        <v>2.02</v>
+        <v>2.16</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>27.9</v>
+        <v>6.98</v>
       </c>
       <c r="C180" t="n">
-        <v>28.46</v>
+        <v>7.13</v>
       </c>
       <c r="D180" t="n">
-        <v>2.01</v>
+        <v>2.15</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>TRACXN</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>32.33</v>
+        <v>25.06</v>
       </c>
       <c r="C181" t="n">
-        <v>32.98</v>
+        <v>25.6</v>
       </c>
       <c r="D181" t="n">
-        <v>2.01</v>
+        <v>2.15</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>91.06999999999999</v>
+        <v>2.79</v>
       </c>
       <c r="C182" t="n">
-        <v>92.90000000000001</v>
+        <v>2.85</v>
       </c>
       <c r="D182" t="n">
-        <v>2.01</v>
+        <v>2.15</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ANSALAPI</t>
+          <t>ASTAR</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>4</v>
+        <v>685.35</v>
       </c>
       <c r="C183" t="n">
-        <v>4.08</v>
+        <v>700</v>
       </c>
       <c r="D183" t="n">
-        <v>2</v>
+        <v>2.14</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>113.72</v>
+        <v>36.39</v>
       </c>
       <c r="C184" t="n">
-        <v>115.99</v>
+        <v>37.17</v>
       </c>
       <c r="D184" t="n">
-        <v>2</v>
+        <v>2.14</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>465.52</v>
+        <v>6.09</v>
       </c>
       <c r="C185" t="n">
-        <v>474.83</v>
+        <v>6.22</v>
       </c>
       <c r="D185" t="n">
-        <v>2</v>
+        <v>2.13</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>PANORAMA</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>6.54</v>
+        <v>57.77</v>
       </c>
       <c r="C186" t="n">
-        <v>6.67</v>
+        <v>59</v>
       </c>
       <c r="D186" t="n">
-        <v>1.99</v>
+        <v>2.13</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>2.01</v>
+        <v>6660.5</v>
       </c>
       <c r="C187" t="n">
-        <v>2.05</v>
+        <v>6801</v>
       </c>
       <c r="D187" t="n">
-        <v>1.99</v>
+        <v>2.11</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>BOROLTD</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>117.27</v>
+        <v>276.21</v>
       </c>
       <c r="C188" t="n">
-        <v>119.6</v>
+        <v>282</v>
       </c>
       <c r="D188" t="n">
-        <v>1.99</v>
+        <v>2.1</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ABAN</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>14.07</v>
+        <v>95.89</v>
       </c>
       <c r="C189" t="n">
-        <v>14.35</v>
+        <v>97.89</v>
       </c>
       <c r="D189" t="n">
-        <v>1.99</v>
+        <v>2.09</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HUHTAMAKI</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>234.2</v>
+        <v>31.52</v>
       </c>
       <c r="C190" t="n">
-        <v>238.85</v>
+        <v>32.18</v>
       </c>
       <c r="D190" t="n">
-        <v>1.99</v>
+        <v>2.09</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>SEYAIND</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>13.6</v>
+        <v>40.16</v>
       </c>
       <c r="C191" t="n">
-        <v>13.87</v>
+        <v>41</v>
       </c>
       <c r="D191" t="n">
-        <v>1.99</v>
+        <v>2.09</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>LAHOTIOV</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>40.2</v>
+        <v>78.37</v>
       </c>
       <c r="C192" t="n">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="D192" t="n">
-        <v>1.99</v>
+        <v>2.08</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SCHAND</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>144.65</v>
+        <v>103.84</v>
       </c>
       <c r="C193" t="n">
-        <v>147.5</v>
+        <v>106</v>
       </c>
       <c r="D193" t="n">
-        <v>1.97</v>
+        <v>2.08</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>SURANAT&amp;P</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>5.09</v>
+        <v>15.87</v>
       </c>
       <c r="C194" t="n">
-        <v>5.19</v>
+        <v>16.2</v>
       </c>
       <c r="D194" t="n">
-        <v>1.96</v>
+        <v>2.08</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>BRIGHTBR</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>130.05</v>
+        <v>248.85</v>
       </c>
       <c r="C195" t="n">
-        <v>132.6</v>
+        <v>254</v>
       </c>
       <c r="D195" t="n">
-        <v>1.96</v>
+        <v>2.07</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>ANIKINDS</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>22.93</v>
+        <v>43.98</v>
       </c>
       <c r="C196" t="n">
-        <v>23.38</v>
+        <v>44.89</v>
       </c>
       <c r="D196" t="n">
-        <v>1.96</v>
+        <v>2.07</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>6.65</v>
+        <v>1722</v>
       </c>
       <c r="C197" t="n">
-        <v>6.78</v>
+        <v>1757.6</v>
       </c>
       <c r="D197" t="n">
-        <v>1.95</v>
+        <v>2.07</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>ALBERTDAVD</t>
         </is>
       </c>
       <c r="B198" t="n">
+        <v>876.35</v>
+      </c>
+      <c r="C198" t="n">
+        <v>894.4</v>
+      </c>
+      <c r="D198" t="n">
         <v>2.06</v>
-      </c>
-      <c r="C198" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="D198" t="n">
-        <v>1.94</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>ORICONENT</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>5.66</v>
+        <v>51.83</v>
       </c>
       <c r="C199" t="n">
-        <v>5.77</v>
+        <v>52.9</v>
       </c>
       <c r="D199" t="n">
-        <v>1.94</v>
+        <v>2.06</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>6.26</v>
+        <v>55.7</v>
       </c>
       <c r="C200" t="n">
-        <v>6.38</v>
+        <v>56.85</v>
       </c>
       <c r="D200" t="n">
-        <v>1.92</v>
+        <v>2.06</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>LAMBODHARA</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>135.19</v>
+        <v>2.93</v>
       </c>
       <c r="C201" t="n">
-        <v>137.79</v>
+        <v>2.99</v>
       </c>
       <c r="D201" t="n">
-        <v>1.92</v>
+        <v>2.05</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-01 10:28 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CENTEXT-RE</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.79</v>
+        <v>32.62</v>
       </c>
       <c r="C2" t="n">
-        <v>3.88</v>
+        <v>35.88</v>
       </c>
       <c r="D2" t="n">
-        <v>39.07</v>
+        <v>9.99</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>717</v>
+        <v>31.76</v>
       </c>
       <c r="C3" t="n">
-        <v>860.4</v>
+        <v>34.93</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>9.98</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>BAWEJA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>92.72</v>
+        <v>25.65</v>
       </c>
       <c r="C4" t="n">
-        <v>111.26</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>9.16</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GENXAI</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>75.65000000000001</v>
+        <v>14.3</v>
       </c>
       <c r="C5" t="n">
-        <v>88.95</v>
+        <v>15.5</v>
       </c>
       <c r="D5" t="n">
-        <v>17.58</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JOCIL</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>145.17</v>
+        <v>61.82</v>
       </c>
       <c r="C6" t="n">
-        <v>162</v>
+        <v>67</v>
       </c>
       <c r="D6" t="n">
-        <v>11.59</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29.66</v>
+        <v>12.45</v>
       </c>
       <c r="C7" t="n">
-        <v>32.62</v>
+        <v>13.47</v>
       </c>
       <c r="D7" t="n">
-        <v>9.98</v>
+        <v>8.19</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>SUNLOC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28.88</v>
+        <v>68.8</v>
       </c>
       <c r="C8" t="n">
-        <v>31.76</v>
+        <v>74</v>
       </c>
       <c r="D8" t="n">
-        <v>9.970000000000001</v>
+        <v>7.56</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>GENXAI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10.38</v>
+        <v>90.75</v>
       </c>
       <c r="C9" t="n">
-        <v>11.4</v>
+        <v>97.15000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>9.83</v>
+        <v>7.05</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>HILINFRA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.88</v>
+        <v>42.75</v>
       </c>
       <c r="C10" t="n">
-        <v>0.96</v>
+        <v>45.42</v>
       </c>
       <c r="D10" t="n">
-        <v>9.09</v>
+        <v>6.25</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>77.83</v>
+        <v>18.63</v>
       </c>
       <c r="C11" t="n">
-        <v>84.75</v>
+        <v>19.79</v>
       </c>
       <c r="D11" t="n">
-        <v>8.890000000000001</v>
+        <v>6.23</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>3PLAND</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22.31</v>
+        <v>31.01</v>
       </c>
       <c r="C12" t="n">
-        <v>24</v>
+        <v>32.7</v>
       </c>
       <c r="D12" t="n">
-        <v>7.58</v>
+        <v>5.45</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VIRAT</t>
+          <t>CRAVATEX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>340.2</v>
+        <v>359.85</v>
       </c>
       <c r="C13" t="n">
-        <v>364.95</v>
+        <v>379</v>
       </c>
       <c r="D13" t="n">
-        <v>7.28</v>
+        <v>5.32</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="C14" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="D14" t="n">
-        <v>7.14</v>
+        <v>5.26</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>EASTSILK</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10.25</v>
+        <v>73.81</v>
       </c>
       <c r="C15" t="n">
-        <v>10.97</v>
+        <v>77.5</v>
       </c>
       <c r="D15" t="n">
-        <v>7.02</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ESTER</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>84.55</v>
+        <v>21.8</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>22.89</v>
       </c>
       <c r="D16" t="n">
-        <v>6.45</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KEYFINSERV</t>
+          <t>MTARTECH</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>233</v>
+        <v>7797</v>
       </c>
       <c r="C17" t="n">
-        <v>247.8</v>
+        <v>8186.5</v>
       </c>
       <c r="D17" t="n">
-        <v>6.35</v>
+        <v>5</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4.41</v>
+        <v>909.9</v>
       </c>
       <c r="C18" t="n">
-        <v>4.69</v>
+        <v>955.35</v>
       </c>
       <c r="D18" t="n">
-        <v>6.35</v>
+        <v>5</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>149.26</v>
+        <v>227.02</v>
       </c>
       <c r="C19" t="n">
-        <v>158.2</v>
+        <v>238.37</v>
       </c>
       <c r="D19" t="n">
-        <v>5.99</v>
+        <v>5</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MGSL</t>
+          <t>ABAN</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>63.25</v>
+        <v>14.63</v>
       </c>
       <c r="C20" t="n">
-        <v>66.95</v>
+        <v>15.36</v>
       </c>
       <c r="D20" t="n">
-        <v>5.85</v>
+        <v>4.99</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>PRIMECAB</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>168.37</v>
+        <v>196.45</v>
       </c>
       <c r="C21" t="n">
-        <v>177.9</v>
+        <v>206.25</v>
       </c>
       <c r="D21" t="n">
-        <v>5.66</v>
+        <v>4.99</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>BHADORA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.18</v>
+        <v>140.25</v>
       </c>
       <c r="C22" t="n">
-        <v>0.19</v>
+        <v>147.25</v>
       </c>
       <c r="D22" t="n">
-        <v>5.56</v>
+        <v>4.99</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TPLPLASTEH</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>65.26000000000001</v>
+        <v>44.27</v>
       </c>
       <c r="C23" t="n">
-        <v>68.67</v>
+        <v>46.48</v>
       </c>
       <c r="D23" t="n">
-        <v>5.23</v>
+        <v>4.99</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>21.76</v>
+        <v>37.05</v>
       </c>
       <c r="C24" t="n">
-        <v>22.88</v>
+        <v>38.9</v>
       </c>
       <c r="D24" t="n">
-        <v>5.15</v>
+        <v>4.99</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1665.8</v>
+        <v>1025.7</v>
       </c>
       <c r="C25" t="n">
-        <v>1750</v>
+        <v>1076.9</v>
       </c>
       <c r="D25" t="n">
-        <v>5.05</v>
+        <v>4.99</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SHANKARA</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>127.47</v>
+        <v>7.42</v>
       </c>
       <c r="C26" t="n">
-        <v>133.9</v>
+        <v>7.79</v>
       </c>
       <c r="D26" t="n">
-        <v>5.04</v>
+        <v>4.99</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NEWJAISA</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>31.68</v>
       </c>
       <c r="C27" t="n">
-        <v>18.9</v>
+        <v>33.26</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MTARTECH</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>7426</v>
+        <v>5.44</v>
       </c>
       <c r="C28" t="n">
-        <v>7797</v>
+        <v>5.71</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>866.6</v>
+        <v>53.45</v>
       </c>
       <c r="C29" t="n">
-        <v>909.9</v>
+        <v>56.1</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>SRIKPRIND</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>216.21</v>
+        <v>26.25</v>
       </c>
       <c r="C30" t="n">
-        <v>227.02</v>
+        <v>27.55</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>26.18</v>
+        <v>36.77</v>
       </c>
       <c r="C31" t="n">
-        <v>27.49</v>
+        <v>38.59</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>MOHITIND</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>426.55</v>
+        <v>22.67</v>
       </c>
       <c r="C32" t="n">
-        <v>447.85</v>
+        <v>23.79</v>
       </c>
       <c r="D32" t="n">
-        <v>4.99</v>
+        <v>4.94</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AMEYA</t>
+          <t>DHARIWAL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>146.2</v>
+        <v>28.4</v>
       </c>
       <c r="C33" t="n">
-        <v>153.5</v>
+        <v>29.8</v>
       </c>
       <c r="D33" t="n">
-        <v>4.99</v>
+        <v>4.93</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>49.46</v>
+        <v>2.25</v>
       </c>
       <c r="C34" t="n">
-        <v>51.93</v>
+        <v>2.36</v>
       </c>
       <c r="D34" t="n">
-        <v>4.99</v>
+        <v>4.89</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GFSTEELS</t>
+          <t>HEROMOTORS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>35.77</v>
+        <v>152.55</v>
       </c>
       <c r="C35" t="n">
-        <v>37.55</v>
+        <v>159.99</v>
       </c>
       <c r="D35" t="n">
-        <v>4.98</v>
+        <v>4.88</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>BHADORA</t>
+          <t>AISL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>133.6</v>
+        <v>63.7</v>
       </c>
       <c r="C36" t="n">
-        <v>140.25</v>
+        <v>66.8</v>
       </c>
       <c r="D36" t="n">
-        <v>4.98</v>
+        <v>4.87</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>30.18</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="C37" t="n">
-        <v>31.68</v>
+        <v>79</v>
       </c>
       <c r="D37" t="n">
-        <v>4.97</v>
+        <v>4.77</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PRIMECAB</t>
+          <t>RNPL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>187.1</v>
+        <v>65.7</v>
       </c>
       <c r="C38" t="n">
-        <v>196.4</v>
+        <v>68.8</v>
       </c>
       <c r="D38" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RHETAN</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>16.69</v>
+        <v>22.43</v>
       </c>
       <c r="C39" t="n">
-        <v>17.52</v>
+        <v>23.48</v>
       </c>
       <c r="D39" t="n">
-        <v>4.97</v>
+        <v>4.68</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>ESCONET</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>14.12</v>
+        <v>235.05</v>
       </c>
       <c r="C40" t="n">
-        <v>14.82</v>
+        <v>246</v>
       </c>
       <c r="D40" t="n">
-        <v>4.96</v>
+        <v>4.66</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1323,13 +1323,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>51.45</v>
+        <v>54</v>
       </c>
       <c r="C41" t="n">
-        <v>54</v>
+        <v>56.5</v>
       </c>
       <c r="D41" t="n">
-        <v>4.96</v>
+        <v>4.63</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>20.77</v>
+        <v>2.38</v>
       </c>
       <c r="C42" t="n">
-        <v>21.8</v>
+        <v>2.49</v>
       </c>
       <c r="D42" t="n">
-        <v>4.96</v>
+        <v>4.62</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>BELLACASA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7.07</v>
+        <v>246.61</v>
       </c>
       <c r="C43" t="n">
-        <v>7.42</v>
+        <v>258</v>
       </c>
       <c r="D43" t="n">
-        <v>4.95</v>
+        <v>4.62</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>KORE</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>188.2</v>
+        <v>1.97</v>
       </c>
       <c r="C44" t="n">
-        <v>197.5</v>
+        <v>2.06</v>
       </c>
       <c r="D44" t="n">
-        <v>4.94</v>
+        <v>4.57</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>50.95</v>
+        <v>454.35</v>
       </c>
       <c r="C45" t="n">
-        <v>53.45</v>
+        <v>474.95</v>
       </c>
       <c r="D45" t="n">
-        <v>4.91</v>
+        <v>4.53</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>SACHEEROME</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>7.34</v>
+        <v>465</v>
       </c>
       <c r="C46" t="n">
-        <v>7.7</v>
+        <v>485.95</v>
       </c>
       <c r="D46" t="n">
-        <v>4.9</v>
+        <v>4.51</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>66.72</v>
+        <v>1796.1</v>
       </c>
       <c r="C47" t="n">
-        <v>69.95</v>
+        <v>1877</v>
       </c>
       <c r="D47" t="n">
-        <v>4.84</v>
+        <v>4.5</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>23.32</v>
+        <v>5.39</v>
       </c>
       <c r="C48" t="n">
-        <v>24.44</v>
+        <v>5.63</v>
       </c>
       <c r="D48" t="n">
-        <v>4.8</v>
+        <v>4.45</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LRRPL</t>
+          <t>SHRADDHA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>103.05</v>
+        <v>152.31</v>
       </c>
       <c r="C49" t="n">
-        <v>108</v>
+        <v>159</v>
       </c>
       <c r="D49" t="n">
-        <v>4.8</v>
+        <v>4.39</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1.47</v>
+        <v>669.8</v>
       </c>
       <c r="C50" t="n">
-        <v>1.54</v>
+        <v>698.9</v>
       </c>
       <c r="D50" t="n">
-        <v>4.76</v>
+        <v>4.34</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>8</v>
+        <v>68.73</v>
       </c>
       <c r="C51" t="n">
-        <v>8.380000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="D51" t="n">
-        <v>4.75</v>
+        <v>4.32</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>343.5</v>
+        <v>0.47</v>
       </c>
       <c r="C52" t="n">
-        <v>359.8</v>
+        <v>0.49</v>
       </c>
       <c r="D52" t="n">
-        <v>4.75</v>
+        <v>4.26</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>SADBHIN</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>5.27</v>
+        <v>2.6</v>
       </c>
       <c r="C53" t="n">
-        <v>5.52</v>
+        <v>2.71</v>
       </c>
       <c r="D53" t="n">
-        <v>4.74</v>
+        <v>4.23</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MOLBIO</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1255.6</v>
+        <v>1043.35</v>
       </c>
       <c r="C54" t="n">
-        <v>1314.9</v>
+        <v>1087</v>
       </c>
       <c r="D54" t="n">
-        <v>4.72</v>
+        <v>4.18</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>VISL</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>32.85</v>
+        <v>0.72</v>
       </c>
       <c r="C55" t="n">
-        <v>34.4</v>
+        <v>0.75</v>
       </c>
       <c r="D55" t="n">
-        <v>4.72</v>
+        <v>4.17</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GOLDSTAR</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>11.7</v>
+        <v>14.39</v>
       </c>
       <c r="C56" t="n">
-        <v>12.25</v>
+        <v>14.99</v>
       </c>
       <c r="D56" t="n">
-        <v>4.7</v>
+        <v>4.17</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>33.39</v>
+        <v>2.73</v>
       </c>
       <c r="C57" t="n">
-        <v>34.95</v>
+        <v>2.84</v>
       </c>
       <c r="D57" t="n">
-        <v>4.67</v>
+        <v>4.03</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MASKINVEST</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>147.18</v>
+        <v>98.17</v>
       </c>
       <c r="C58" t="n">
-        <v>154</v>
+        <v>102</v>
       </c>
       <c r="D58" t="n">
-        <v>4.63</v>
+        <v>3.9</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>43.56</v>
+        <v>78.84</v>
       </c>
       <c r="C59" t="n">
-        <v>45.55</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="D59" t="n">
-        <v>4.57</v>
+        <v>3.88</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>FALCONTECH</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>51.08</v>
+        <v>12.95</v>
       </c>
       <c r="C60" t="n">
-        <v>53.39</v>
+        <v>13.45</v>
       </c>
       <c r="D60" t="n">
-        <v>4.52</v>
+        <v>3.86</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>26.79</v>
+        <v>160.79</v>
       </c>
       <c r="C61" t="n">
-        <v>27.99</v>
+        <v>166.9</v>
       </c>
       <c r="D61" t="n">
-        <v>4.48</v>
+        <v>3.8</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>243.95</v>
+        <v>159.98</v>
       </c>
       <c r="C62" t="n">
-        <v>254.85</v>
+        <v>165.99</v>
       </c>
       <c r="D62" t="n">
-        <v>4.47</v>
+        <v>3.76</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>AMNPLST</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>153.14</v>
+        <v>171.57</v>
       </c>
       <c r="C63" t="n">
-        <v>159.99</v>
+        <v>178</v>
       </c>
       <c r="D63" t="n">
-        <v>4.47</v>
+        <v>3.75</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>93.19</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C64" t="n">
-        <v>97.2</v>
+        <v>0.84</v>
       </c>
       <c r="D64" t="n">
-        <v>4.3</v>
+        <v>3.7</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>8.390000000000001</v>
+        <v>175.65</v>
       </c>
       <c r="C65" t="n">
-        <v>8.75</v>
+        <v>182</v>
       </c>
       <c r="D65" t="n">
-        <v>4.29</v>
+        <v>3.62</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>KSB</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>824.8</v>
+        <v>527.9</v>
       </c>
       <c r="C66" t="n">
-        <v>860</v>
+        <v>546.95</v>
       </c>
       <c r="D66" t="n">
-        <v>4.27</v>
+        <v>3.61</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>IVC</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.47</v>
+        <v>7.8</v>
       </c>
       <c r="C67" t="n">
-        <v>0.49</v>
+        <v>8.08</v>
       </c>
       <c r="D67" t="n">
-        <v>4.26</v>
+        <v>3.59</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ORBTEXP</t>
+          <t>AAKASH</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>262.01</v>
+        <v>8.44</v>
       </c>
       <c r="C68" t="n">
-        <v>272.85</v>
+        <v>8.74</v>
       </c>
       <c r="D68" t="n">
-        <v>4.14</v>
+        <v>3.55</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>KPIGREEN</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>371.25</v>
+        <v>44.25</v>
       </c>
       <c r="C69" t="n">
-        <v>386.4</v>
+        <v>45.8</v>
       </c>
       <c r="D69" t="n">
-        <v>4.08</v>
+        <v>3.5</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>139.25</v>
+        <v>27.41</v>
       </c>
       <c r="C70" t="n">
-        <v>144.9</v>
+        <v>28.37</v>
       </c>
       <c r="D70" t="n">
-        <v>4.06</v>
+        <v>3.5</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>DUGLOBAL</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>20.15</v>
+        <v>70.45</v>
       </c>
       <c r="C71" t="n">
-        <v>20.95</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="D71" t="n">
-        <v>3.97</v>
+        <v>3.48</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>36.88</v>
+        <v>3846.1</v>
       </c>
       <c r="C72" t="n">
-        <v>38.34</v>
+        <v>3980</v>
       </c>
       <c r="D72" t="n">
-        <v>3.96</v>
+        <v>3.48</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>EBIX</t>
+          <t>ARVEE</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>17.01</v>
+        <v>225.16</v>
       </c>
       <c r="C73" t="n">
-        <v>17.68</v>
+        <v>232.99</v>
       </c>
       <c r="D73" t="n">
-        <v>3.94</v>
+        <v>3.48</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>VTMLTD</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>39.93</v>
+        <v>0.29</v>
       </c>
       <c r="C74" t="n">
-        <v>41.49</v>
+        <v>0.3</v>
       </c>
       <c r="D74" t="n">
-        <v>3.91</v>
+        <v>3.45</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>PRIORITY</t>
+          <t>JOCIL</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>293.64</v>
+        <v>146.86</v>
       </c>
       <c r="C75" t="n">
-        <v>305</v>
+        <v>151.9</v>
       </c>
       <c r="D75" t="n">
-        <v>3.87</v>
+        <v>3.43</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>POWERMECH</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2397.2</v>
+        <v>442.45</v>
       </c>
       <c r="C76" t="n">
-        <v>2488.9</v>
+        <v>457.5</v>
       </c>
       <c r="D76" t="n">
-        <v>3.83</v>
+        <v>3.4</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>502.85</v>
+        <v>129.66</v>
       </c>
       <c r="C77" t="n">
-        <v>522</v>
+        <v>134</v>
       </c>
       <c r="D77" t="n">
-        <v>3.81</v>
+        <v>3.35</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>TTML</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>22.93</v>
+        <v>34.3</v>
       </c>
       <c r="C78" t="n">
-        <v>23.8</v>
+        <v>35.44</v>
       </c>
       <c r="D78" t="n">
-        <v>3.79</v>
+        <v>3.32</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>13.47</v>
+        <v>52.28</v>
       </c>
       <c r="C79" t="n">
-        <v>13.98</v>
+        <v>53.99</v>
       </c>
       <c r="D79" t="n">
-        <v>3.79</v>
+        <v>3.27</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>EBGNG</t>
+          <t>ESSARSHPNG</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>674.8</v>
+        <v>18.89</v>
       </c>
       <c r="C80" t="n">
-        <v>700.05</v>
+        <v>19.5</v>
       </c>
       <c r="D80" t="n">
-        <v>3.74</v>
+        <v>3.23</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>LORDSCHLO</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>19.57</v>
+        <v>138.54</v>
       </c>
       <c r="C81" t="n">
-        <v>20.3</v>
+        <v>143</v>
       </c>
       <c r="D81" t="n">
-        <v>3.73</v>
+        <v>3.22</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>2.15</v>
+        <v>58.14</v>
       </c>
       <c r="C82" t="n">
-        <v>2.23</v>
+        <v>60</v>
       </c>
       <c r="D82" t="n">
-        <v>3.72</v>
+        <v>3.2</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>IFBAGRO</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.27</v>
+        <v>891.65</v>
       </c>
       <c r="C83" t="n">
-        <v>0.28</v>
+        <v>919.95</v>
       </c>
       <c r="D83" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ARIS</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>135</v>
+        <v>5.38</v>
       </c>
       <c r="C84" t="n">
-        <v>140</v>
+        <v>5.55</v>
       </c>
       <c r="D84" t="n">
-        <v>3.7</v>
+        <v>3.16</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>AKSHOPTFBR</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>23.82</v>
+        <v>6.97</v>
       </c>
       <c r="C85" t="n">
-        <v>24.7</v>
+        <v>7.19</v>
       </c>
       <c r="D85" t="n">
-        <v>3.69</v>
+        <v>3.16</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>PYRAMID</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>30.74</v>
+        <v>156.01</v>
       </c>
       <c r="C86" t="n">
-        <v>31.87</v>
+        <v>160.92</v>
       </c>
       <c r="D86" t="n">
-        <v>3.68</v>
+        <v>3.15</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>NICCOPAR</t>
+          <t>PVSL</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>81</v>
+        <v>95.5</v>
       </c>
       <c r="C87" t="n">
-        <v>83.90000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="D87" t="n">
-        <v>3.58</v>
+        <v>3.14</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ESSARSHPNG</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>16.95</v>
+        <v>6.4</v>
       </c>
       <c r="C88" t="n">
-        <v>17.54</v>
+        <v>6.6</v>
       </c>
       <c r="D88" t="n">
-        <v>3.48</v>
+        <v>3.12</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>119.85</v>
+        <v>9.99</v>
       </c>
       <c r="C89" t="n">
-        <v>124</v>
+        <v>10.3</v>
       </c>
       <c r="D89" t="n">
-        <v>3.46</v>
+        <v>3.1</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>HBSL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.29</v>
+        <v>55.89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.3</v>
+        <v>57.6</v>
       </c>
       <c r="D90" t="n">
-        <v>3.45</v>
+        <v>3.06</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>VALIANTORG</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>14.48</v>
+        <v>455.1</v>
       </c>
       <c r="C91" t="n">
-        <v>14.98</v>
+        <v>469</v>
       </c>
       <c r="D91" t="n">
-        <v>3.45</v>
+        <v>3.05</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>29.97</v>
+        <v>10.88</v>
       </c>
       <c r="C92" t="n">
-        <v>31</v>
+        <v>11.21</v>
       </c>
       <c r="D92" t="n">
-        <v>3.44</v>
+        <v>3.03</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LEENEE</t>
+          <t>SEPC</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>7.58</v>
+        <v>5.02</v>
       </c>
       <c r="C93" t="n">
-        <v>7.84</v>
+        <v>5.17</v>
       </c>
       <c r="D93" t="n">
-        <v>3.43</v>
+        <v>2.99</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>MLKFOOD</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>21.77</v>
+        <v>83.36</v>
       </c>
       <c r="C94" t="n">
-        <v>22.5</v>
+        <v>85.8</v>
       </c>
       <c r="D94" t="n">
-        <v>3.35</v>
+        <v>2.93</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PRASOLCHEM</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>840.15</v>
+        <v>132.96</v>
       </c>
       <c r="C95" t="n">
-        <v>868.25</v>
+        <v>136.85</v>
       </c>
       <c r="D95" t="n">
-        <v>3.34</v>
+        <v>2.93</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>SURANAT&amp;P</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>59.9</v>
+        <v>15.84</v>
       </c>
       <c r="C96" t="n">
-        <v>61.88</v>
+        <v>16.3</v>
       </c>
       <c r="D96" t="n">
-        <v>3.31</v>
+        <v>2.9</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>18.4</v>
+        <v>14.82</v>
       </c>
       <c r="C97" t="n">
-        <v>19</v>
+        <v>15.25</v>
       </c>
       <c r="D97" t="n">
-        <v>3.26</v>
+        <v>2.9</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>14.23</v>
+        <v>167.23</v>
       </c>
       <c r="C98" t="n">
-        <v>14.69</v>
+        <v>172</v>
       </c>
       <c r="D98" t="n">
-        <v>3.23</v>
+        <v>2.85</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>YOGI</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>156.67</v>
+        <v>10.94</v>
       </c>
       <c r="C99" t="n">
-        <v>161.7</v>
+        <v>11.25</v>
       </c>
       <c r="D99" t="n">
-        <v>3.21</v>
+        <v>2.83</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KHAITANLTD</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>150.01</v>
+        <v>4.59</v>
       </c>
       <c r="C100" t="n">
-        <v>154.79</v>
+        <v>4.72</v>
       </c>
       <c r="D100" t="n">
-        <v>3.19</v>
+        <v>2.83</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>IFGLEXPOR</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>69.52</v>
+        <v>191.45</v>
       </c>
       <c r="C101" t="n">
-        <v>71.7</v>
+        <v>196.8</v>
       </c>
       <c r="D101" t="n">
-        <v>3.14</v>
+        <v>2.79</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>FLFL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1190.5</v>
+        <v>1.09</v>
       </c>
       <c r="C102" t="n">
-        <v>1227.8</v>
+        <v>1.12</v>
       </c>
       <c r="D102" t="n">
-        <v>3.13</v>
+        <v>2.75</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>6.73</v>
+        <v>6.18</v>
       </c>
       <c r="C103" t="n">
-        <v>6.94</v>
+        <v>6.35</v>
       </c>
       <c r="D103" t="n">
-        <v>3.12</v>
+        <v>2.75</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>BSL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>178.52</v>
+        <v>118.28</v>
       </c>
       <c r="C104" t="n">
-        <v>184</v>
+        <v>121.5</v>
       </c>
       <c r="D104" t="n">
-        <v>3.07</v>
+        <v>2.72</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>993</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C105" t="n">
-        <v>1023.5</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="D105" t="n">
-        <v>3.07</v>
+        <v>2.71</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>113.05</v>
+        <v>58.12</v>
       </c>
       <c r="C106" t="n">
-        <v>116.5</v>
+        <v>59.69</v>
       </c>
       <c r="D106" t="n">
-        <v>3.05</v>
+        <v>2.7</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>NINSYS</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>1.32</v>
+        <v>766.35</v>
       </c>
       <c r="C107" t="n">
-        <v>1.36</v>
+        <v>787</v>
       </c>
       <c r="D107" t="n">
-        <v>3.03</v>
+        <v>2.69</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>LKPSEC</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>14.27</v>
+        <v>113.93</v>
       </c>
       <c r="C108" t="n">
-        <v>14.7</v>
+        <v>116.99</v>
       </c>
       <c r="D108" t="n">
-        <v>3.01</v>
+        <v>2.69</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BAJAJINDEF</t>
+          <t>PARIN</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>213.11</v>
+        <v>710.9</v>
       </c>
       <c r="C109" t="n">
-        <v>219.44</v>
+        <v>729.95</v>
       </c>
       <c r="D109" t="n">
-        <v>2.97</v>
+        <v>2.68</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>VISHAL</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>17.92</v>
+        <v>0.38</v>
       </c>
       <c r="C110" t="n">
-        <v>18.45</v>
+        <v>0.39</v>
       </c>
       <c r="D110" t="n">
-        <v>2.96</v>
+        <v>2.63</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>3720.9</v>
+        <v>33.52</v>
       </c>
       <c r="C111" t="n">
-        <v>3830</v>
+        <v>34.4</v>
       </c>
       <c r="D111" t="n">
-        <v>2.93</v>
+        <v>2.63</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BIL</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1000.7</v>
+        <v>1.92</v>
       </c>
       <c r="C112" t="n">
-        <v>1030</v>
+        <v>1.97</v>
       </c>
       <c r="D112" t="n">
-        <v>2.93</v>
+        <v>2.6</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>38.64</v>
+        <v>15.18</v>
       </c>
       <c r="C113" t="n">
-        <v>39.77</v>
+        <v>15.57</v>
       </c>
       <c r="D113" t="n">
-        <v>2.92</v>
+        <v>2.57</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>ONYX</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>29.43</v>
+        <v>37</v>
       </c>
       <c r="C114" t="n">
-        <v>30.29</v>
+        <v>37.95</v>
       </c>
       <c r="D114" t="n">
-        <v>2.92</v>
+        <v>2.57</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SUYOG</t>
+          <t>CHEMFAB</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>689.95</v>
+        <v>335.9</v>
       </c>
       <c r="C115" t="n">
-        <v>710</v>
+        <v>344.45</v>
       </c>
       <c r="D115" t="n">
-        <v>2.91</v>
+        <v>2.55</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>SJLOGISTIC</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>5.19</v>
+        <v>310.1</v>
       </c>
       <c r="C116" t="n">
-        <v>5.34</v>
+        <v>317.9</v>
       </c>
       <c r="D116" t="n">
-        <v>2.89</v>
+        <v>2.52</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>5.88</v>
+        <v>33.55</v>
       </c>
       <c r="C117" t="n">
-        <v>6.05</v>
+        <v>34.39</v>
       </c>
       <c r="D117" t="n">
-        <v>2.89</v>
+        <v>2.5</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>97.08</v>
+        <v>56.74</v>
       </c>
       <c r="C118" t="n">
-        <v>99.87</v>
+        <v>58.15</v>
       </c>
       <c r="D118" t="n">
-        <v>2.87</v>
+        <v>2.49</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SMARTWORKS</t>
+          <t>VEDAVAAG</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>514.25</v>
+        <v>22.24</v>
       </c>
       <c r="C119" t="n">
-        <v>528.95</v>
+        <v>22.79</v>
       </c>
       <c r="D119" t="n">
-        <v>2.86</v>
+        <v>2.47</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ABCOTS</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>198.84</v>
+        <v>20</v>
       </c>
       <c r="C120" t="n">
-        <v>204.5</v>
+        <v>20.49</v>
       </c>
       <c r="D120" t="n">
-        <v>2.85</v>
+        <v>2.45</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>38.9</v>
+        <v>6.14</v>
       </c>
       <c r="C121" t="n">
-        <v>40</v>
+        <v>6.29</v>
       </c>
       <c r="D121" t="n">
-        <v>2.83</v>
+        <v>2.44</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>SUVIDHAA</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>322.7</v>
+        <v>2.09</v>
       </c>
       <c r="C122" t="n">
-        <v>331.8</v>
+        <v>2.14</v>
       </c>
       <c r="D122" t="n">
-        <v>2.82</v>
+        <v>2.39</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>57.15</v>
+        <v>4.19</v>
       </c>
       <c r="C123" t="n">
-        <v>58.75</v>
+        <v>4.29</v>
       </c>
       <c r="D123" t="n">
-        <v>2.8</v>
+        <v>2.39</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TIPSFILMS</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>339.55</v>
+        <v>0.42</v>
       </c>
       <c r="C124" t="n">
-        <v>348.95</v>
+        <v>0.43</v>
       </c>
       <c r="D124" t="n">
-        <v>2.77</v>
+        <v>2.38</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>35.55</v>
+        <v>5.07</v>
       </c>
       <c r="C125" t="n">
-        <v>36.53</v>
+        <v>5.19</v>
       </c>
       <c r="D125" t="n">
-        <v>2.76</v>
+        <v>2.37</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>NKIND</t>
+          <t>INVPRECQ</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>61.99</v>
+        <v>1536.7</v>
       </c>
       <c r="C126" t="n">
-        <v>63.7</v>
+        <v>1573</v>
       </c>
       <c r="D126" t="n">
-        <v>2.76</v>
+        <v>2.36</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>INTERARCH</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1675</v>
+        <v>1673.4</v>
       </c>
       <c r="C127" t="n">
-        <v>1721</v>
+        <v>1712.9</v>
       </c>
       <c r="D127" t="n">
-        <v>2.75</v>
+        <v>2.36</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>35.02</v>
+        <v>37.52</v>
       </c>
       <c r="C128" t="n">
-        <v>35.98</v>
+        <v>38.4</v>
       </c>
       <c r="D128" t="n">
-        <v>2.74</v>
+        <v>2.35</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>REGENCERAM</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>32.51</v>
+        <v>6.83</v>
       </c>
       <c r="C129" t="n">
-        <v>33.4</v>
+        <v>6.99</v>
       </c>
       <c r="D129" t="n">
-        <v>2.74</v>
+        <v>2.34</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>WARDINMOBI</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>5.49</v>
+        <v>3</v>
       </c>
       <c r="C130" t="n">
-        <v>5.64</v>
+        <v>3.07</v>
       </c>
       <c r="D130" t="n">
-        <v>2.73</v>
+        <v>2.33</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GLOSTERLTD</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>539.25</v>
+        <v>187.44</v>
       </c>
       <c r="C131" t="n">
-        <v>553.9</v>
+        <v>191.79</v>
       </c>
       <c r="D131" t="n">
-        <v>2.72</v>
+        <v>2.32</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MITCON</t>
+          <t>HMT</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>82.66</v>
+        <v>60.1</v>
       </c>
       <c r="C132" t="n">
-        <v>84.89</v>
+        <v>61.49</v>
       </c>
       <c r="D132" t="n">
-        <v>2.7</v>
+        <v>2.31</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>194.55</v>
+        <v>287.59</v>
       </c>
       <c r="C133" t="n">
-        <v>199.7</v>
+        <v>294.2</v>
       </c>
       <c r="D133" t="n">
-        <v>2.65</v>
+        <v>2.3</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>1.9</v>
+        <v>40.08</v>
       </c>
       <c r="C134" t="n">
-        <v>1.95</v>
+        <v>41</v>
       </c>
       <c r="D134" t="n">
-        <v>2.63</v>
+        <v>2.3</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.38</v>
+        <v>406.45</v>
       </c>
       <c r="C135" t="n">
-        <v>0.39</v>
+        <v>415.8</v>
       </c>
       <c r="D135" t="n">
-        <v>2.63</v>
+        <v>2.3</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>32.14</v>
+        <v>1.32</v>
       </c>
       <c r="C136" t="n">
-        <v>32.98</v>
+        <v>1.35</v>
       </c>
       <c r="D136" t="n">
-        <v>2.61</v>
+        <v>2.27</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SBCL</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1111.3</v>
+        <v>0.44</v>
       </c>
       <c r="C137" t="n">
-        <v>1140</v>
+        <v>0.45</v>
       </c>
       <c r="D137" t="n">
-        <v>2.58</v>
+        <v>2.27</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MEDICO</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>21.84</v>
+        <v>1.76</v>
       </c>
       <c r="C138" t="n">
-        <v>22.4</v>
+        <v>1.8</v>
       </c>
       <c r="D138" t="n">
-        <v>2.56</v>
+        <v>2.27</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>STARTECK</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>3186.2</v>
+        <v>306.95</v>
       </c>
       <c r="C139" t="n">
-        <v>3267</v>
+        <v>313.9</v>
       </c>
       <c r="D139" t="n">
-        <v>2.54</v>
+        <v>2.26</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>COSMOFIRST</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>834.8</v>
+        <v>205.19</v>
       </c>
       <c r="C140" t="n">
-        <v>856</v>
+        <v>209.8</v>
       </c>
       <c r="D140" t="n">
-        <v>2.54</v>
+        <v>2.25</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>60</v>
+        <v>0.89</v>
       </c>
       <c r="C141" t="n">
-        <v>61.5</v>
+        <v>0.91</v>
       </c>
       <c r="D141" t="n">
-        <v>2.5</v>
+        <v>2.25</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>CENTEXT-RE</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>199.92</v>
+        <v>3.62</v>
       </c>
       <c r="C142" t="n">
-        <v>204.9</v>
+        <v>3.7</v>
       </c>
       <c r="D142" t="n">
-        <v>2.49</v>
+        <v>2.21</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>KRISHIVAL</t>
+          <t>SPECIALITY</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>403.95</v>
+        <v>154.1</v>
       </c>
       <c r="C143" t="n">
-        <v>414</v>
+        <v>157.5</v>
       </c>
       <c r="D143" t="n">
-        <v>2.49</v>
+        <v>2.21</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SADBHAV</t>
+          <t>OPTIFIN</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>6.93</v>
+        <v>15.45</v>
       </c>
       <c r="C144" t="n">
-        <v>7.1</v>
+        <v>15.79</v>
       </c>
       <c r="D144" t="n">
-        <v>2.45</v>
+        <v>2.2</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>175.61</v>
+        <v>2186.8</v>
       </c>
       <c r="C145" t="n">
-        <v>179.88</v>
+        <v>2235</v>
       </c>
       <c r="D145" t="n">
-        <v>2.43</v>
+        <v>2.2</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HALEOSLABS</t>
+          <t>BANG</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1487.9</v>
+        <v>32.27</v>
       </c>
       <c r="C146" t="n">
-        <v>1524</v>
+        <v>32.98</v>
       </c>
       <c r="D146" t="n">
-        <v>2.43</v>
+        <v>2.2</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ARCHIES</t>
+          <t>SAMPANN</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>12.43</v>
+        <v>24.17</v>
       </c>
       <c r="C147" t="n">
-        <v>12.73</v>
+        <v>24.7</v>
       </c>
       <c r="D147" t="n">
-        <v>2.41</v>
+        <v>2.19</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>KHAICHEM</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>49.22</v>
+        <v>148.08</v>
       </c>
       <c r="C148" t="n">
-        <v>50.4</v>
+        <v>151.3</v>
       </c>
       <c r="D148" t="n">
-        <v>2.4</v>
+        <v>2.17</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>UNIONBANK</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>166</v>
+        <v>417</v>
       </c>
       <c r="C149" t="n">
-        <v>169.98</v>
+        <v>426</v>
       </c>
       <c r="D149" t="n">
-        <v>2.4</v>
+        <v>2.16</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>LALITHAA</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>375</v>
+        <v>1.85</v>
       </c>
       <c r="C150" t="n">
-        <v>384</v>
+        <v>1.89</v>
       </c>
       <c r="D150" t="n">
-        <v>2.4</v>
+        <v>2.16</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>KAPSTON</t>
+          <t>ITL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>555.7</v>
+        <v>351.2</v>
       </c>
       <c r="C151" t="n">
-        <v>569</v>
+        <v>358.8</v>
       </c>
       <c r="D151" t="n">
-        <v>2.39</v>
+        <v>2.16</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ALLCARGO</t>
+          <t>BEEKAY</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>10.53</v>
+        <v>452.95</v>
       </c>
       <c r="C152" t="n">
-        <v>10.78</v>
+        <v>462.7</v>
       </c>
       <c r="D152" t="n">
-        <v>2.37</v>
+        <v>2.15</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>150.35</v>
+        <v>6.07</v>
       </c>
       <c r="C153" t="n">
-        <v>153.9</v>
+        <v>6.2</v>
       </c>
       <c r="D153" t="n">
-        <v>2.36</v>
+        <v>2.14</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SUNLITE</t>
+          <t>NIRLON</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>625.2</v>
+        <v>605</v>
       </c>
       <c r="C154" t="n">
-        <v>639.95</v>
+        <v>617.95</v>
       </c>
       <c r="D154" t="n">
-        <v>2.36</v>
+        <v>2.14</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ELLEN</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>369.35</v>
+        <v>228.67</v>
       </c>
       <c r="C155" t="n">
-        <v>378</v>
+        <v>233.5</v>
       </c>
       <c r="D155" t="n">
-        <v>2.34</v>
+        <v>2.11</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>MAFATIND</t>
+          <t>TRF</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>115.29</v>
+        <v>197.82</v>
       </c>
       <c r="C156" t="n">
-        <v>117.98</v>
+        <v>202</v>
       </c>
       <c r="D156" t="n">
-        <v>2.33</v>
+        <v>2.11</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>COOLCAPS</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>21.5</v>
+        <v>1672.7</v>
       </c>
       <c r="C157" t="n">
-        <v>22</v>
+        <v>1707.8</v>
       </c>
       <c r="D157" t="n">
-        <v>2.33</v>
+        <v>2.1</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>103.44</v>
+        <v>11.45</v>
       </c>
       <c r="C158" t="n">
-        <v>105.85</v>
+        <v>11.69</v>
       </c>
       <c r="D158" t="n">
-        <v>2.33</v>
+        <v>2.1</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>XTRANET</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>0.43</v>
+        <v>285.05</v>
       </c>
       <c r="C159" t="n">
-        <v>0.44</v>
+        <v>291</v>
       </c>
       <c r="D159" t="n">
-        <v>2.33</v>
+        <v>2.09</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>HLEGLAS</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>0.86</v>
+        <v>439.4</v>
       </c>
       <c r="C160" t="n">
-        <v>0.88</v>
+        <v>448.45</v>
       </c>
       <c r="D160" t="n">
-        <v>2.33</v>
+        <v>2.06</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>INDOAMIN</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>447.75</v>
+        <v>142.07</v>
       </c>
       <c r="C161" t="n">
-        <v>458.2</v>
+        <v>145</v>
       </c>
       <c r="D161" t="n">
-        <v>2.33</v>
+        <v>2.06</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AAKASH</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>8.59</v>
+        <v>25.2</v>
       </c>
       <c r="C162" t="n">
-        <v>8.789999999999999</v>
+        <v>25.72</v>
       </c>
       <c r="D162" t="n">
-        <v>2.33</v>
+        <v>2.06</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>23.44</v>
+        <v>5.86</v>
       </c>
       <c r="C163" t="n">
-        <v>23.98</v>
+        <v>5.98</v>
       </c>
       <c r="D163" t="n">
-        <v>2.3</v>
+        <v>2.05</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>SAHAJSOLAR</t>
+          <t>AUSTENG</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>87.90000000000001</v>
+        <v>171.52</v>
       </c>
       <c r="C164" t="n">
-        <v>89.90000000000001</v>
+        <v>175</v>
       </c>
       <c r="D164" t="n">
-        <v>2.28</v>
+        <v>2.03</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CREST</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>356.9</v>
+        <v>13.83</v>
       </c>
       <c r="C165" t="n">
-        <v>364.95</v>
+        <v>14.11</v>
       </c>
       <c r="D165" t="n">
-        <v>2.26</v>
+        <v>2.02</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>205.36</v>
+        <v>50.92</v>
       </c>
       <c r="C166" t="n">
-        <v>209.99</v>
+        <v>51.95</v>
       </c>
       <c r="D166" t="n">
-        <v>2.25</v>
+        <v>2.02</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>13.36</v>
+        <v>31.85</v>
       </c>
       <c r="C167" t="n">
-        <v>13.66</v>
+        <v>32.49</v>
       </c>
       <c r="D167" t="n">
-        <v>2.25</v>
+        <v>2.01</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>11.2</v>
+        <v>6.97</v>
       </c>
       <c r="C168" t="n">
-        <v>11.45</v>
+        <v>7.11</v>
       </c>
       <c r="D168" t="n">
-        <v>2.23</v>
+        <v>2.01</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ASHUTOSH</t>
+          <t>ONIXSOLAR</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>163.35</v>
+        <v>343.05</v>
       </c>
       <c r="C169" t="n">
-        <v>167</v>
+        <v>349.95</v>
       </c>
       <c r="D169" t="n">
-        <v>2.23</v>
+        <v>2.01</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>KRITI</t>
+          <t>MHLXMIRU</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>62.41</v>
+        <v>179.21</v>
       </c>
       <c r="C170" t="n">
-        <v>63.8</v>
+        <v>182.79</v>
       </c>
       <c r="D170" t="n">
-        <v>2.23</v>
+        <v>2</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>MBECL</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.9</v>
+        <v>484.32</v>
       </c>
       <c r="C171" t="n">
-        <v>0.92</v>
+        <v>494</v>
       </c>
       <c r="D171" t="n">
-        <v>2.22</v>
+        <v>2</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>10.84</v>
+        <v>0.5</v>
       </c>
       <c r="C172" t="n">
-        <v>11.08</v>
+        <v>0.51</v>
       </c>
       <c r="D172" t="n">
-        <v>2.21</v>
+        <v>2</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>GALLANTT</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>539.1</v>
+        <v>200.04</v>
       </c>
       <c r="C173" t="n">
-        <v>551</v>
+        <v>204.04</v>
       </c>
       <c r="D173" t="n">
-        <v>2.21</v>
+        <v>2</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>DENTALKART</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>49.64</v>
+        <v>460</v>
       </c>
       <c r="C174" t="n">
-        <v>50.73</v>
+        <v>469.2</v>
       </c>
       <c r="D174" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>RPEL</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>20.06</v>
+        <v>1809</v>
       </c>
       <c r="C175" t="n">
-        <v>20.5</v>
+        <v>1845</v>
       </c>
       <c r="D175" t="n">
-        <v>2.19</v>
+        <v>1.99</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>COMSYN</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>261.95</v>
+        <v>2.53</v>
       </c>
       <c r="C176" t="n">
-        <v>267.65</v>
+        <v>2.58</v>
       </c>
       <c r="D176" t="n">
-        <v>2.18</v>
+        <v>1.98</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>57.07</v>
+        <v>13.11</v>
       </c>
       <c r="C177" t="n">
-        <v>58.3</v>
+        <v>13.37</v>
       </c>
       <c r="D177" t="n">
-        <v>2.16</v>
+        <v>1.98</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>NEXTMEDIA</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>3.7</v>
+        <v>68.45</v>
       </c>
       <c r="C178" t="n">
-        <v>3.78</v>
+        <v>69.8</v>
       </c>
       <c r="D178" t="n">
-        <v>2.16</v>
+        <v>1.97</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HITECHGEAR</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>625.5</v>
+        <v>0.51</v>
       </c>
       <c r="C179" t="n">
-        <v>639</v>
+        <v>0.52</v>
       </c>
       <c r="D179" t="n">
-        <v>2.16</v>
+        <v>1.96</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>6.98</v>
+        <v>40.21</v>
       </c>
       <c r="C180" t="n">
-        <v>7.13</v>
+        <v>41</v>
       </c>
       <c r="D180" t="n">
-        <v>2.15</v>
+        <v>1.96</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>25.06</v>
+        <v>126.23</v>
       </c>
       <c r="C181" t="n">
-        <v>25.6</v>
+        <v>128.7</v>
       </c>
       <c r="D181" t="n">
-        <v>2.15</v>
+        <v>1.96</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>2.79</v>
+        <v>31.19</v>
       </c>
       <c r="C182" t="n">
-        <v>2.85</v>
+        <v>31.8</v>
       </c>
       <c r="D182" t="n">
-        <v>2.15</v>
+        <v>1.96</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ASTAR</t>
+          <t>EVERESTIND</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>685.35</v>
+        <v>455.6</v>
       </c>
       <c r="C183" t="n">
-        <v>700</v>
+        <v>464.5</v>
       </c>
       <c r="D183" t="n">
-        <v>2.14</v>
+        <v>1.95</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>BAGFILMS</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>36.39</v>
+        <v>4.1</v>
       </c>
       <c r="C184" t="n">
-        <v>37.17</v>
+        <v>4.18</v>
       </c>
       <c r="D184" t="n">
-        <v>2.14</v>
+        <v>1.95</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>GGBL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>6.09</v>
+        <v>222.7</v>
       </c>
       <c r="C185" t="n">
-        <v>6.22</v>
+        <v>227</v>
       </c>
       <c r="D185" t="n">
-        <v>2.13</v>
+        <v>1.93</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PANORAMA</t>
+          <t>ROHLTD</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>57.77</v>
+        <v>299.85</v>
       </c>
       <c r="C186" t="n">
-        <v>59</v>
+        <v>305.6</v>
       </c>
       <c r="D186" t="n">
-        <v>2.13</v>
+        <v>1.92</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>PRISMX</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>6660.5</v>
+        <v>0.52</v>
       </c>
       <c r="C187" t="n">
-        <v>6801</v>
+        <v>0.53</v>
       </c>
       <c r="D187" t="n">
-        <v>2.11</v>
+        <v>1.92</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>BOROLTD</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>276.21</v>
+        <v>127.58</v>
       </c>
       <c r="C188" t="n">
-        <v>282</v>
+        <v>130</v>
       </c>
       <c r="D188" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PREMIERPOL</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>95.89</v>
+        <v>16.34</v>
       </c>
       <c r="C189" t="n">
-        <v>97.89</v>
+        <v>16.65</v>
       </c>
       <c r="D189" t="n">
-        <v>2.09</v>
+        <v>1.9</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>31.52</v>
+        <v>3.18</v>
       </c>
       <c r="C190" t="n">
-        <v>32.18</v>
+        <v>3.24</v>
       </c>
       <c r="D190" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>WEL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>40.16</v>
+        <v>72.63</v>
       </c>
       <c r="C191" t="n">
-        <v>41</v>
+        <v>74</v>
       </c>
       <c r="D191" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>BESTAGRO</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>78.37</v>
+        <v>17.53</v>
       </c>
       <c r="C192" t="n">
-        <v>80</v>
+        <v>17.86</v>
       </c>
       <c r="D192" t="n">
-        <v>2.08</v>
+        <v>1.88</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>SOMICONVEY</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>103.84</v>
+        <v>89.31</v>
       </c>
       <c r="C193" t="n">
-        <v>106</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="D193" t="n">
-        <v>2.08</v>
+        <v>1.88</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SURANAT&amp;P</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>15.87</v>
+        <v>1919</v>
       </c>
       <c r="C194" t="n">
-        <v>16.2</v>
+        <v>1954.9</v>
       </c>
       <c r="D194" t="n">
-        <v>2.08</v>
+        <v>1.87</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>BRIGHTBR</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>248.85</v>
+        <v>6.97</v>
       </c>
       <c r="C195" t="n">
-        <v>254</v>
+        <v>7.1</v>
       </c>
       <c r="D195" t="n">
-        <v>2.07</v>
+        <v>1.87</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ANIKINDS</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>43.98</v>
+        <v>2096</v>
       </c>
       <c r="C196" t="n">
-        <v>44.89</v>
+        <v>2135</v>
       </c>
       <c r="D196" t="n">
-        <v>2.07</v>
+        <v>1.86</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>INNOVANA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>1722</v>
+        <v>292.55</v>
       </c>
       <c r="C197" t="n">
-        <v>1757.6</v>
+        <v>298</v>
       </c>
       <c r="D197" t="n">
-        <v>2.07</v>
+        <v>1.86</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ALBERTDAVD</t>
+          <t>MOLDTECH</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>876.35</v>
+        <v>206.16</v>
       </c>
       <c r="C198" t="n">
-        <v>894.4</v>
+        <v>210</v>
       </c>
       <c r="D198" t="n">
-        <v>2.06</v>
+        <v>1.86</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ORICONENT</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>51.83</v>
+        <v>40.69</v>
       </c>
       <c r="C199" t="n">
-        <v>52.9</v>
+        <v>41.44</v>
       </c>
       <c r="D199" t="n">
-        <v>2.06</v>
+        <v>1.84</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>PONNIERODE</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>55.7</v>
+        <v>372.2</v>
       </c>
       <c r="C200" t="n">
-        <v>56.85</v>
+        <v>379</v>
       </c>
       <c r="D200" t="n">
-        <v>2.06</v>
+        <v>1.83</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>BLUEDART</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>2.93</v>
+        <v>4629</v>
       </c>
       <c r="C201" t="n">
-        <v>2.99</v>
+        <v>4713.9</v>
       </c>
       <c r="D201" t="n">
-        <v>2.05</v>
+        <v>1.83</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-05 10:51 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>PARTY-RE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32.62</v>
+        <v>0.2</v>
       </c>
       <c r="C2" t="n">
-        <v>35.88</v>
+        <v>0.25</v>
       </c>
       <c r="D2" t="n">
-        <v>9.99</v>
+        <v>25</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>SURANI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31.76</v>
+        <v>100.05</v>
       </c>
       <c r="C3" t="n">
-        <v>34.93</v>
+        <v>114.9</v>
       </c>
       <c r="D3" t="n">
-        <v>9.98</v>
+        <v>14.84</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BAWEJA</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25.65</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>28</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>9.16</v>
+        <v>11.08</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>CENTEXT-RE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14.3</v>
+        <v>3.16</v>
       </c>
       <c r="C5" t="n">
-        <v>15.5</v>
+        <v>3.5</v>
       </c>
       <c r="D5" t="n">
-        <v>8.390000000000001</v>
+        <v>10.76</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>HRYNSHP</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>61.82</v>
+        <v>97.98</v>
       </c>
       <c r="C6" t="n">
-        <v>67</v>
+        <v>108</v>
       </c>
       <c r="D6" t="n">
-        <v>8.380000000000001</v>
+        <v>10.23</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>NIKITA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12.45</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>13.47</v>
+        <v>72.7</v>
       </c>
       <c r="D7" t="n">
-        <v>8.19</v>
+        <v>9.98</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SUNLOC</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>68.8</v>
+        <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>74</v>
+        <v>5.45</v>
       </c>
       <c r="D8" t="n">
-        <v>7.56</v>
+        <v>9</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GENXAI</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>90.75</v>
+        <v>380.8</v>
       </c>
       <c r="C9" t="n">
-        <v>97.15000000000001</v>
+        <v>414.95</v>
       </c>
       <c r="D9" t="n">
-        <v>7.05</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HILINFRA</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>42.75</v>
+        <v>5.42</v>
       </c>
       <c r="C10" t="n">
-        <v>45.42</v>
+        <v>5.88</v>
       </c>
       <c r="D10" t="n">
-        <v>6.25</v>
+        <v>8.49</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>CGVAK</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18.63</v>
+        <v>147.24</v>
       </c>
       <c r="C11" t="n">
-        <v>19.79</v>
+        <v>158.99</v>
       </c>
       <c r="D11" t="n">
-        <v>6.23</v>
+        <v>7.98</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3PLAND</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>31.01</v>
+        <v>47.76</v>
       </c>
       <c r="C12" t="n">
-        <v>32.7</v>
+        <v>51.5</v>
       </c>
       <c r="D12" t="n">
-        <v>5.45</v>
+        <v>7.83</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CRAVATEX</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>359.85</v>
+        <v>0.13</v>
       </c>
       <c r="C13" t="n">
-        <v>379</v>
+        <v>0.14</v>
       </c>
       <c r="D13" t="n">
-        <v>5.32</v>
+        <v>7.69</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>PANORAMA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.19</v>
+        <v>60.91</v>
       </c>
       <c r="C14" t="n">
-        <v>0.2</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>5.26</v>
+        <v>7.55</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EASTSILK</t>
+          <t>STLSTRINF</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73.81</v>
+        <v>21.52</v>
       </c>
       <c r="C15" t="n">
-        <v>77.5</v>
+        <v>22.99</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>6.83</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>21.8</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="C16" t="n">
-        <v>22.89</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MTARTECH</t>
+          <t>OMFREIGHT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7797</v>
+        <v>97.5</v>
       </c>
       <c r="C17" t="n">
-        <v>8186.5</v>
+        <v>103.99</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>6.66</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>PACIFICI</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>909.9</v>
+        <v>135.99</v>
       </c>
       <c r="C18" t="n">
-        <v>955.35</v>
+        <v>144.99</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>6.62</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>KDGREEN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>227.02</v>
+        <v>46.76</v>
       </c>
       <c r="C19" t="n">
-        <v>238.37</v>
+        <v>49.7</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>6.29</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABAN</t>
+          <t>MAHAPEXLTD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>14.63</v>
+        <v>50.18</v>
       </c>
       <c r="C20" t="n">
-        <v>15.36</v>
+        <v>53.3</v>
       </c>
       <c r="D20" t="n">
-        <v>4.99</v>
+        <v>6.22</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PRIMECAB</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>196.45</v>
+        <v>72.52</v>
       </c>
       <c r="C21" t="n">
-        <v>206.25</v>
+        <v>77</v>
       </c>
       <c r="D21" t="n">
-        <v>4.99</v>
+        <v>6.18</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BHADORA</t>
+          <t>AUSTENG</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>140.25</v>
+        <v>167.72</v>
       </c>
       <c r="C22" t="n">
-        <v>147.25</v>
+        <v>177.9</v>
       </c>
       <c r="D22" t="n">
-        <v>4.99</v>
+        <v>6.07</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>44.27</v>
+        <v>148.85</v>
       </c>
       <c r="C23" t="n">
-        <v>46.48</v>
+        <v>157.65</v>
       </c>
       <c r="D23" t="n">
-        <v>4.99</v>
+        <v>5.91</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>37.05</v>
+        <v>3.56</v>
       </c>
       <c r="C24" t="n">
-        <v>38.9</v>
+        <v>3.77</v>
       </c>
       <c r="D24" t="n">
-        <v>4.99</v>
+        <v>5.9</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>VTMLTD</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1025.7</v>
+        <v>38.15</v>
       </c>
       <c r="C25" t="n">
-        <v>1076.9</v>
+        <v>40.4</v>
       </c>
       <c r="D25" t="n">
-        <v>4.99</v>
+        <v>5.9</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>SACHEEROME</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>7.42</v>
+        <v>499.65</v>
       </c>
       <c r="C26" t="n">
-        <v>7.79</v>
+        <v>529</v>
       </c>
       <c r="D26" t="n">
-        <v>4.99</v>
+        <v>5.87</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>31.68</v>
+        <v>774.5</v>
       </c>
       <c r="C27" t="n">
-        <v>33.26</v>
+        <v>819.9</v>
       </c>
       <c r="D27" t="n">
-        <v>4.99</v>
+        <v>5.86</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>FAIRCHEMOR</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5.44</v>
+        <v>661.5</v>
       </c>
       <c r="C28" t="n">
-        <v>5.71</v>
+        <v>699.95</v>
       </c>
       <c r="D28" t="n">
-        <v>4.96</v>
+        <v>5.81</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>TGVSL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>53.45</v>
+        <v>116.38</v>
       </c>
       <c r="C29" t="n">
-        <v>56.1</v>
+        <v>123.12</v>
       </c>
       <c r="D29" t="n">
-        <v>4.96</v>
+        <v>5.79</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SRIKPRIND</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>26.25</v>
+        <v>25.41</v>
       </c>
       <c r="C30" t="n">
-        <v>27.55</v>
+        <v>26.85</v>
       </c>
       <c r="D30" t="n">
-        <v>4.95</v>
+        <v>5.67</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>SANGAMIND</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>36.77</v>
+        <v>634.55</v>
       </c>
       <c r="C31" t="n">
-        <v>38.59</v>
+        <v>670</v>
       </c>
       <c r="D31" t="n">
-        <v>4.95</v>
+        <v>5.59</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MOHITIND</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>22.67</v>
+        <v>0.18</v>
       </c>
       <c r="C32" t="n">
-        <v>23.79</v>
+        <v>0.19</v>
       </c>
       <c r="D32" t="n">
-        <v>4.94</v>
+        <v>5.56</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DHARIWAL</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>28.4</v>
+        <v>76.75</v>
       </c>
       <c r="C33" t="n">
-        <v>29.8</v>
+        <v>81</v>
       </c>
       <c r="D33" t="n">
-        <v>4.93</v>
+        <v>5.54</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>VOEPL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2.25</v>
+        <v>493</v>
       </c>
       <c r="C34" t="n">
-        <v>2.36</v>
+        <v>520</v>
       </c>
       <c r="D34" t="n">
-        <v>4.89</v>
+        <v>5.48</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HEROMOTORS</t>
+          <t>SUNLOC</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>152.55</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="C35" t="n">
-        <v>159.99</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D35" t="n">
-        <v>4.88</v>
+        <v>5.42</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AISL</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>63.7</v>
+        <v>31.32</v>
       </c>
       <c r="C36" t="n">
-        <v>66.8</v>
+        <v>32.98</v>
       </c>
       <c r="D36" t="n">
-        <v>4.87</v>
+        <v>5.3</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>TECHD</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>75.40000000000001</v>
+        <v>531.95</v>
       </c>
       <c r="C37" t="n">
-        <v>79</v>
+        <v>559.95</v>
       </c>
       <c r="D37" t="n">
-        <v>4.77</v>
+        <v>5.26</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>RNPL</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>65.7</v>
+        <v>0.19</v>
       </c>
       <c r="C38" t="n">
-        <v>68.8</v>
+        <v>0.2</v>
       </c>
       <c r="D38" t="n">
-        <v>4.72</v>
+        <v>5.26</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>SEDEMAC</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>22.43</v>
+        <v>3432.8</v>
       </c>
       <c r="C39" t="n">
-        <v>23.48</v>
+        <v>3607.8</v>
       </c>
       <c r="D39" t="n">
-        <v>4.68</v>
+        <v>5.1</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ESCONET</t>
+          <t>HEROMOTORS</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>235.05</v>
+        <v>167.8</v>
       </c>
       <c r="C40" t="n">
-        <v>246</v>
+        <v>176.34</v>
       </c>
       <c r="D40" t="n">
-        <v>4.66</v>
+        <v>5.09</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BIOPOL</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>54</v>
+        <v>4.57</v>
       </c>
       <c r="C41" t="n">
-        <v>56.5</v>
+        <v>4.8</v>
       </c>
       <c r="D41" t="n">
-        <v>4.63</v>
+        <v>5.03</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2.38</v>
+        <v>1076.9</v>
       </c>
       <c r="C42" t="n">
-        <v>2.49</v>
+        <v>1130.7</v>
       </c>
       <c r="D42" t="n">
-        <v>4.62</v>
+        <v>5</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BELLACASA</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>246.61</v>
+        <v>2.6</v>
       </c>
       <c r="C43" t="n">
-        <v>258</v>
+        <v>2.73</v>
       </c>
       <c r="D43" t="n">
-        <v>4.62</v>
+        <v>5</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.97</v>
+        <v>516.15</v>
       </c>
       <c r="C44" t="n">
-        <v>2.06</v>
+        <v>541.95</v>
       </c>
       <c r="D44" t="n">
-        <v>4.57</v>
+        <v>5</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>UNIVPHOTO</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>454.35</v>
+        <v>490</v>
       </c>
       <c r="C45" t="n">
-        <v>474.95</v>
+        <v>514.5</v>
       </c>
       <c r="D45" t="n">
-        <v>4.53</v>
+        <v>5</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SACHEEROME</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>465</v>
+        <v>168.82</v>
       </c>
       <c r="C46" t="n">
-        <v>485.95</v>
+        <v>177.26</v>
       </c>
       <c r="D46" t="n">
-        <v>4.51</v>
+        <v>5</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1796.1</v>
+        <v>46.48</v>
       </c>
       <c r="C47" t="n">
-        <v>1877</v>
+        <v>48.8</v>
       </c>
       <c r="D47" t="n">
-        <v>4.5</v>
+        <v>4.99</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>SPRL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>5.39</v>
+        <v>146.2</v>
       </c>
       <c r="C48" t="n">
-        <v>5.63</v>
+        <v>153.5</v>
       </c>
       <c r="D48" t="n">
-        <v>4.45</v>
+        <v>4.99</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SHRADDHA</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>152.31</v>
+        <v>35.88</v>
       </c>
       <c r="C49" t="n">
-        <v>159</v>
+        <v>37.67</v>
       </c>
       <c r="D49" t="n">
-        <v>4.39</v>
+        <v>4.99</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>669.8</v>
+        <v>464</v>
       </c>
       <c r="C50" t="n">
-        <v>698.9</v>
+        <v>487</v>
       </c>
       <c r="D50" t="n">
-        <v>4.34</v>
+        <v>4.96</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>ABAN</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>68.73</v>
+        <v>15.36</v>
       </c>
       <c r="C51" t="n">
-        <v>71.7</v>
+        <v>16.12</v>
       </c>
       <c r="D51" t="n">
-        <v>4.32</v>
+        <v>4.95</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.47</v>
+        <v>15.56</v>
       </c>
       <c r="C52" t="n">
-        <v>0.49</v>
+        <v>16.33</v>
       </c>
       <c r="D52" t="n">
-        <v>4.26</v>
+        <v>4.95</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SADBHIN</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2.6</v>
+        <v>449.8</v>
       </c>
       <c r="C53" t="n">
-        <v>2.71</v>
+        <v>472</v>
       </c>
       <c r="D53" t="n">
-        <v>4.23</v>
+        <v>4.94</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>WHBRADY</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1043.35</v>
+        <v>465.05</v>
       </c>
       <c r="C54" t="n">
-        <v>1087</v>
+        <v>488</v>
       </c>
       <c r="D54" t="n">
-        <v>4.18</v>
+        <v>4.93</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.72</v>
+        <v>6.72</v>
       </c>
       <c r="C55" t="n">
-        <v>0.75</v>
+        <v>7.05</v>
       </c>
       <c r="D55" t="n">
-        <v>4.17</v>
+        <v>4.91</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>14.39</v>
+        <v>5.71</v>
       </c>
       <c r="C56" t="n">
-        <v>14.99</v>
+        <v>5.99</v>
       </c>
       <c r="D56" t="n">
-        <v>4.17</v>
+        <v>4.9</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2.73</v>
+        <v>38.9</v>
       </c>
       <c r="C57" t="n">
-        <v>2.84</v>
+        <v>40.8</v>
       </c>
       <c r="D57" t="n">
-        <v>4.03</v>
+        <v>4.88</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>98.17</v>
+        <v>193.49</v>
       </c>
       <c r="C58" t="n">
-        <v>102</v>
+        <v>202.9</v>
       </c>
       <c r="D58" t="n">
-        <v>3.9</v>
+        <v>4.86</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>78.84</v>
+        <v>41.57</v>
       </c>
       <c r="C59" t="n">
-        <v>81.90000000000001</v>
+        <v>43.59</v>
       </c>
       <c r="D59" t="n">
-        <v>3.88</v>
+        <v>4.86</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FALCONTECH</t>
+          <t>APSISAERO</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>12.95</v>
+        <v>555</v>
       </c>
       <c r="C60" t="n">
-        <v>13.45</v>
+        <v>581.95</v>
       </c>
       <c r="D60" t="n">
-        <v>3.86</v>
+        <v>4.86</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>160.79</v>
+        <v>2.06</v>
       </c>
       <c r="C61" t="n">
-        <v>166.9</v>
+        <v>2.16</v>
       </c>
       <c r="D61" t="n">
-        <v>3.8</v>
+        <v>4.85</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>COMPEAU</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>159.98</v>
+        <v>362.45</v>
       </c>
       <c r="C62" t="n">
-        <v>165.99</v>
+        <v>380</v>
       </c>
       <c r="D62" t="n">
-        <v>3.76</v>
+        <v>4.84</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AMNPLST</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>171.57</v>
+        <v>35.91</v>
       </c>
       <c r="C63" t="n">
-        <v>178</v>
+        <v>37.64</v>
       </c>
       <c r="D63" t="n">
-        <v>3.75</v>
+        <v>4.82</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>AIROLAM</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.8100000000000001</v>
+        <v>89.58</v>
       </c>
       <c r="C64" t="n">
-        <v>0.84</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="D64" t="n">
-        <v>3.7</v>
+        <v>4.82</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>KILITCH</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>175.65</v>
+        <v>218.51</v>
       </c>
       <c r="C65" t="n">
-        <v>182</v>
+        <v>229</v>
       </c>
       <c r="D65" t="n">
-        <v>3.62</v>
+        <v>4.8</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>TEAMTECH</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>527.9</v>
+        <v>145.95</v>
       </c>
       <c r="C66" t="n">
-        <v>546.95</v>
+        <v>152.85</v>
       </c>
       <c r="D66" t="n">
-        <v>3.61</v>
+        <v>4.73</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>IVC</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>7.8</v>
+        <v>540.35</v>
       </c>
       <c r="C67" t="n">
-        <v>8.08</v>
+        <v>565.85</v>
       </c>
       <c r="D67" t="n">
-        <v>3.59</v>
+        <v>4.72</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AAKASH</t>
+          <t>TVVISION</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>8.44</v>
+        <v>2.55</v>
       </c>
       <c r="C68" t="n">
-        <v>8.74</v>
+        <v>2.67</v>
       </c>
       <c r="D68" t="n">
-        <v>3.55</v>
+        <v>4.71</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>AISL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>44.25</v>
+        <v>66.84999999999999</v>
       </c>
       <c r="C69" t="n">
-        <v>45.8</v>
+        <v>70</v>
       </c>
       <c r="D69" t="n">
-        <v>3.5</v>
+        <v>4.71</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>27.41</v>
+        <v>1.28</v>
       </c>
       <c r="C70" t="n">
-        <v>28.37</v>
+        <v>1.34</v>
       </c>
       <c r="D70" t="n">
-        <v>3.5</v>
+        <v>4.69</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>70.45</v>
+        <v>2.36</v>
       </c>
       <c r="C71" t="n">
-        <v>72.90000000000001</v>
+        <v>2.47</v>
       </c>
       <c r="D71" t="n">
-        <v>3.48</v>
+        <v>4.66</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>PELATRO</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3846.1</v>
+        <v>359.9</v>
       </c>
       <c r="C72" t="n">
-        <v>3980</v>
+        <v>376.5</v>
       </c>
       <c r="D72" t="n">
-        <v>3.48</v>
+        <v>4.61</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ARVEE</t>
+          <t>VISHAL</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>225.16</v>
+        <v>17.38</v>
       </c>
       <c r="C73" t="n">
-        <v>232.99</v>
+        <v>18.18</v>
       </c>
       <c r="D73" t="n">
-        <v>3.48</v>
+        <v>4.6</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.29</v>
+        <v>4.81</v>
       </c>
       <c r="C74" t="n">
-        <v>0.3</v>
+        <v>5.03</v>
       </c>
       <c r="D74" t="n">
-        <v>3.45</v>
+        <v>4.57</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>JOCIL</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>146.86</v>
+        <v>10.32</v>
       </c>
       <c r="C75" t="n">
-        <v>151.9</v>
+        <v>10.79</v>
       </c>
       <c r="D75" t="n">
-        <v>3.43</v>
+        <v>4.55</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>442.45</v>
+        <v>38.24</v>
       </c>
       <c r="C76" t="n">
-        <v>457.5</v>
+        <v>39.98</v>
       </c>
       <c r="D76" t="n">
-        <v>3.4</v>
+        <v>4.55</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>129.66</v>
+        <v>13.68</v>
       </c>
       <c r="C77" t="n">
-        <v>134</v>
+        <v>14.3</v>
       </c>
       <c r="D77" t="n">
-        <v>3.35</v>
+        <v>4.53</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TTML</t>
+          <t>MASKINVEST</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>34.3</v>
+        <v>143.41</v>
       </c>
       <c r="C78" t="n">
-        <v>35.44</v>
+        <v>149.9</v>
       </c>
       <c r="D78" t="n">
-        <v>3.32</v>
+        <v>4.53</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>52.28</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="C79" t="n">
-        <v>53.99</v>
+        <v>69.5</v>
       </c>
       <c r="D79" t="n">
-        <v>3.27</v>
+        <v>4.5</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ESSARSHPNG</t>
+          <t>QUINTEGRA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>18.89</v>
+        <v>1.34</v>
       </c>
       <c r="C80" t="n">
-        <v>19.5</v>
+        <v>1.4</v>
       </c>
       <c r="D80" t="n">
-        <v>3.23</v>
+        <v>4.48</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LORDSCHLO</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>138.54</v>
+        <v>1.37</v>
       </c>
       <c r="C81" t="n">
-        <v>143</v>
+        <v>1.43</v>
       </c>
       <c r="D81" t="n">
-        <v>3.22</v>
+        <v>4.38</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>58.14</v>
+        <v>89.95999999999999</v>
       </c>
       <c r="C82" t="n">
-        <v>60</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="D82" t="n">
-        <v>3.2</v>
+        <v>4.38</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>IFBAGRO</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>891.65</v>
+        <v>159.06</v>
       </c>
       <c r="C83" t="n">
-        <v>919.95</v>
+        <v>166</v>
       </c>
       <c r="D83" t="n">
-        <v>3.17</v>
+        <v>4.36</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>5.38</v>
+        <v>0.46</v>
       </c>
       <c r="C84" t="n">
-        <v>5.55</v>
+        <v>0.48</v>
       </c>
       <c r="D84" t="n">
-        <v>3.16</v>
+        <v>4.35</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AKSHOPTFBR</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>6.97</v>
+        <v>631.85</v>
       </c>
       <c r="C85" t="n">
-        <v>7.19</v>
+        <v>659.35</v>
       </c>
       <c r="D85" t="n">
-        <v>3.16</v>
+        <v>4.35</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PYRAMID</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>156.01</v>
+        <v>1243.2</v>
       </c>
       <c r="C86" t="n">
-        <v>160.92</v>
+        <v>1297</v>
       </c>
       <c r="D86" t="n">
-        <v>3.15</v>
+        <v>4.33</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PVSL</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>95.5</v>
+        <v>23</v>
       </c>
       <c r="C87" t="n">
-        <v>98.5</v>
+        <v>23.99</v>
       </c>
       <c r="D87" t="n">
-        <v>3.14</v>
+        <v>4.3</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>RFBL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>6.4</v>
+        <v>107.1</v>
       </c>
       <c r="C88" t="n">
-        <v>6.6</v>
+        <v>111.7</v>
       </c>
       <c r="D88" t="n">
-        <v>3.12</v>
+        <v>4.3</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>9.99</v>
+        <v>35.19</v>
       </c>
       <c r="C89" t="n">
-        <v>10.3</v>
+        <v>36.7</v>
       </c>
       <c r="D89" t="n">
-        <v>3.1</v>
+        <v>4.29</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>HBSL</t>
+          <t>INNOMET</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>55.89</v>
+        <v>280</v>
       </c>
       <c r="C90" t="n">
-        <v>57.6</v>
+        <v>292</v>
       </c>
       <c r="D90" t="n">
-        <v>3.06</v>
+        <v>4.29</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>VALIANTORG</t>
+          <t>ABCOTS</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>455.1</v>
+        <v>189.91</v>
       </c>
       <c r="C91" t="n">
-        <v>469</v>
+        <v>198</v>
       </c>
       <c r="D91" t="n">
-        <v>3.05</v>
+        <v>4.26</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>10.88</v>
+        <v>7.09</v>
       </c>
       <c r="C92" t="n">
-        <v>11.21</v>
+        <v>7.39</v>
       </c>
       <c r="D92" t="n">
-        <v>3.03</v>
+        <v>4.23</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SEPC</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>5.02</v>
+        <v>34.93</v>
       </c>
       <c r="C93" t="n">
-        <v>5.17</v>
+        <v>36.39</v>
       </c>
       <c r="D93" t="n">
-        <v>2.99</v>
+        <v>4.18</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MLKFOOD</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>83.36</v>
+        <v>10.56</v>
       </c>
       <c r="C94" t="n">
-        <v>85.8</v>
+        <v>11</v>
       </c>
       <c r="D94" t="n">
-        <v>2.93</v>
+        <v>4.17</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>132.96</v>
+        <v>580</v>
       </c>
       <c r="C95" t="n">
-        <v>136.85</v>
+        <v>604</v>
       </c>
       <c r="D95" t="n">
-        <v>2.93</v>
+        <v>4.14</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SURANAT&amp;P</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>15.84</v>
+        <v>5.32</v>
       </c>
       <c r="C96" t="n">
-        <v>16.3</v>
+        <v>5.54</v>
       </c>
       <c r="D96" t="n">
-        <v>2.9</v>
+        <v>4.14</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>14.82</v>
+        <v>253.35</v>
       </c>
       <c r="C97" t="n">
-        <v>15.25</v>
+        <v>263.8</v>
       </c>
       <c r="D97" t="n">
-        <v>2.9</v>
+        <v>4.12</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>BLACKROSE</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>167.23</v>
+        <v>110.45</v>
       </c>
       <c r="C98" t="n">
-        <v>172</v>
+        <v>115</v>
       </c>
       <c r="D98" t="n">
-        <v>2.85</v>
+        <v>4.12</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>MAANALU</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>10.94</v>
+        <v>99.34</v>
       </c>
       <c r="C99" t="n">
-        <v>11.25</v>
+        <v>103.4</v>
       </c>
       <c r="D99" t="n">
-        <v>2.83</v>
+        <v>4.09</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>4.59</v>
+        <v>17.09</v>
       </c>
       <c r="C100" t="n">
-        <v>4.72</v>
+        <v>17.78</v>
       </c>
       <c r="D100" t="n">
-        <v>2.83</v>
+        <v>4.04</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IFGLEXPOR</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>191.45</v>
+        <v>245.01</v>
       </c>
       <c r="C101" t="n">
-        <v>196.8</v>
+        <v>254.9</v>
       </c>
       <c r="D101" t="n">
-        <v>2.79</v>
+        <v>4.04</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>BESTAGRO</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1.09</v>
+        <v>17.47</v>
       </c>
       <c r="C102" t="n">
-        <v>1.12</v>
+        <v>18.17</v>
       </c>
       <c r="D102" t="n">
-        <v>2.75</v>
+        <v>4.01</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>6.18</v>
+        <v>15.34</v>
       </c>
       <c r="C103" t="n">
-        <v>6.35</v>
+        <v>15.95</v>
       </c>
       <c r="D103" t="n">
-        <v>2.75</v>
+        <v>3.98</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BSL</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>118.28</v>
+        <v>525.4</v>
       </c>
       <c r="C104" t="n">
-        <v>121.5</v>
+        <v>545.9</v>
       </c>
       <c r="D104" t="n">
-        <v>2.72</v>
+        <v>3.9</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>SPLIL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>73.90000000000001</v>
+        <v>28.5</v>
       </c>
       <c r="C105" t="n">
-        <v>75.90000000000001</v>
+        <v>29.6</v>
       </c>
       <c r="D105" t="n">
-        <v>2.71</v>
+        <v>3.86</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>58.12</v>
+        <v>1.3</v>
       </c>
       <c r="C106" t="n">
-        <v>59.69</v>
+        <v>1.35</v>
       </c>
       <c r="D106" t="n">
-        <v>2.7</v>
+        <v>3.85</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>NINSYS</t>
+          <t>MIDWESTLTD</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>766.35</v>
+        <v>904.15</v>
       </c>
       <c r="C107" t="n">
-        <v>787</v>
+        <v>938.85</v>
       </c>
       <c r="D107" t="n">
-        <v>2.69</v>
+        <v>3.84</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>113.93</v>
+        <v>67.42</v>
       </c>
       <c r="C108" t="n">
-        <v>116.99</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="D108" t="n">
-        <v>2.69</v>
+        <v>3.81</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>PARIN</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>710.9</v>
+        <v>1874</v>
       </c>
       <c r="C109" t="n">
-        <v>729.95</v>
+        <v>1945</v>
       </c>
       <c r="D109" t="n">
-        <v>2.68</v>
+        <v>3.79</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.38</v>
+        <v>21.19</v>
       </c>
       <c r="C110" t="n">
-        <v>0.39</v>
+        <v>21.99</v>
       </c>
       <c r="D110" t="n">
-        <v>2.63</v>
+        <v>3.78</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>PAVNAIND</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>33.52</v>
+        <v>15.36</v>
       </c>
       <c r="C111" t="n">
-        <v>34.4</v>
+        <v>15.94</v>
       </c>
       <c r="D111" t="n">
-        <v>2.63</v>
+        <v>3.78</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1.92</v>
+        <v>477.05</v>
       </c>
       <c r="C112" t="n">
-        <v>1.97</v>
+        <v>494.95</v>
       </c>
       <c r="D112" t="n">
-        <v>2.6</v>
+        <v>3.75</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>15.18</v>
+        <v>35.66</v>
       </c>
       <c r="C113" t="n">
-        <v>15.57</v>
+        <v>36.99</v>
       </c>
       <c r="D113" t="n">
-        <v>2.57</v>
+        <v>3.73</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ONYX</t>
+          <t>SMARTLINK</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>37</v>
+        <v>212.1</v>
       </c>
       <c r="C114" t="n">
-        <v>37.95</v>
+        <v>220</v>
       </c>
       <c r="D114" t="n">
-        <v>2.57</v>
+        <v>3.72</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>335.9</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C115" t="n">
-        <v>344.45</v>
+        <v>0.84</v>
       </c>
       <c r="D115" t="n">
-        <v>2.55</v>
+        <v>3.7</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SJLOGISTIC</t>
+          <t>MONEYVIEW</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>310.1</v>
+        <v>53.88</v>
       </c>
       <c r="C116" t="n">
-        <v>317.9</v>
+        <v>55.85</v>
       </c>
       <c r="D116" t="n">
-        <v>2.52</v>
+        <v>3.66</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>33.55</v>
+        <v>23.59</v>
       </c>
       <c r="C117" t="n">
-        <v>34.39</v>
+        <v>24.45</v>
       </c>
       <c r="D117" t="n">
-        <v>2.5</v>
+        <v>3.65</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>TUTIALKA</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>56.74</v>
+        <v>53.98</v>
       </c>
       <c r="C118" t="n">
-        <v>58.15</v>
+        <v>55.92</v>
       </c>
       <c r="D118" t="n">
-        <v>2.49</v>
+        <v>3.59</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>VEDAVAAG</t>
+          <t>NDL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>22.24</v>
+        <v>2.54</v>
       </c>
       <c r="C119" t="n">
-        <v>22.79</v>
+        <v>2.63</v>
       </c>
       <c r="D119" t="n">
-        <v>2.47</v>
+        <v>3.54</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>20</v>
+        <v>5.1</v>
       </c>
       <c r="C120" t="n">
-        <v>20.49</v>
+        <v>5.28</v>
       </c>
       <c r="D120" t="n">
-        <v>2.45</v>
+        <v>3.53</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>AAATECH</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>6.14</v>
+        <v>92.73999999999999</v>
       </c>
       <c r="C121" t="n">
-        <v>6.29</v>
+        <v>96</v>
       </c>
       <c r="D121" t="n">
-        <v>2.44</v>
+        <v>3.52</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>2.09</v>
+        <v>33.76</v>
       </c>
       <c r="C122" t="n">
-        <v>2.14</v>
+        <v>34.95</v>
       </c>
       <c r="D122" t="n">
-        <v>2.39</v>
+        <v>3.52</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>WATERBASE</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>4.19</v>
+        <v>45.4</v>
       </c>
       <c r="C123" t="n">
-        <v>4.29</v>
+        <v>47</v>
       </c>
       <c r="D123" t="n">
-        <v>2.39</v>
+        <v>3.52</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>RKSWAMY</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.42</v>
+        <v>86.45999999999999</v>
       </c>
       <c r="C124" t="n">
-        <v>0.43</v>
+        <v>89.5</v>
       </c>
       <c r="D124" t="n">
-        <v>2.38</v>
+        <v>3.52</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>PRADPME</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>5.07</v>
+        <v>449.25</v>
       </c>
       <c r="C125" t="n">
-        <v>5.19</v>
+        <v>465</v>
       </c>
       <c r="D125" t="n">
-        <v>2.37</v>
+        <v>3.51</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>INVPRECQ</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1536.7</v>
+        <v>205.77</v>
       </c>
       <c r="C126" t="n">
-        <v>1573</v>
+        <v>213</v>
       </c>
       <c r="D126" t="n">
-        <v>2.36</v>
+        <v>3.51</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>INTERARCH</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1673.4</v>
+        <v>36.24</v>
       </c>
       <c r="C127" t="n">
-        <v>1712.9</v>
+        <v>37.5</v>
       </c>
       <c r="D127" t="n">
-        <v>2.36</v>
+        <v>3.48</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>37.52</v>
+        <v>449.6</v>
       </c>
       <c r="C128" t="n">
-        <v>38.4</v>
+        <v>465</v>
       </c>
       <c r="D128" t="n">
-        <v>2.35</v>
+        <v>3.43</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>UNIENTER</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>6.83</v>
+        <v>87.02</v>
       </c>
       <c r="C129" t="n">
-        <v>6.99</v>
+        <v>90</v>
       </c>
       <c r="D129" t="n">
-        <v>2.34</v>
+        <v>3.42</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>3</v>
+        <v>34.8</v>
       </c>
       <c r="C130" t="n">
-        <v>3.07</v>
+        <v>35.99</v>
       </c>
       <c r="D130" t="n">
-        <v>2.33</v>
+        <v>3.42</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>187.44</v>
+        <v>6.16</v>
       </c>
       <c r="C131" t="n">
-        <v>191.79</v>
+        <v>6.37</v>
       </c>
       <c r="D131" t="n">
-        <v>2.32</v>
+        <v>3.41</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>HMT</t>
+          <t>MPIMANIPAL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>60.1</v>
+        <v>401.4</v>
       </c>
       <c r="C132" t="n">
-        <v>61.49</v>
+        <v>415</v>
       </c>
       <c r="D132" t="n">
-        <v>2.31</v>
+        <v>3.39</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>287.59</v>
+        <v>127.7</v>
       </c>
       <c r="C133" t="n">
-        <v>294.2</v>
+        <v>131.99</v>
       </c>
       <c r="D133" t="n">
-        <v>2.3</v>
+        <v>3.36</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>40.08</v>
+        <v>47.3</v>
       </c>
       <c r="C134" t="n">
-        <v>41</v>
+        <v>48.89</v>
       </c>
       <c r="D134" t="n">
-        <v>2.3</v>
+        <v>3.36</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>406.45</v>
+        <v>4.21</v>
       </c>
       <c r="C135" t="n">
-        <v>415.8</v>
+        <v>4.35</v>
       </c>
       <c r="D135" t="n">
-        <v>2.3</v>
+        <v>3.33</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>ESCONET</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1.32</v>
+        <v>246.8</v>
       </c>
       <c r="C136" t="n">
-        <v>1.35</v>
+        <v>255</v>
       </c>
       <c r="D136" t="n">
-        <v>2.27</v>
+        <v>3.32</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>KRITINUT</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.44</v>
+        <v>66.53</v>
       </c>
       <c r="C137" t="n">
-        <v>0.45</v>
+        <v>68.73999999999999</v>
       </c>
       <c r="D137" t="n">
-        <v>2.27</v>
+        <v>3.32</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>1.76</v>
+        <v>118.66</v>
       </c>
       <c r="C138" t="n">
-        <v>1.8</v>
+        <v>122.6</v>
       </c>
       <c r="D138" t="n">
-        <v>2.27</v>
+        <v>3.32</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>STARTECK</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>306.95</v>
+        <v>15.73</v>
       </c>
       <c r="C139" t="n">
-        <v>313.9</v>
+        <v>16.25</v>
       </c>
       <c r="D139" t="n">
-        <v>2.26</v>
+        <v>3.31</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SECMARK</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>205.19</v>
+        <v>137.48</v>
       </c>
       <c r="C140" t="n">
-        <v>209.8</v>
+        <v>142</v>
       </c>
       <c r="D140" t="n">
-        <v>2.25</v>
+        <v>3.29</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>JOCIL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.89</v>
+        <v>145.22</v>
       </c>
       <c r="C141" t="n">
-        <v>0.91</v>
+        <v>149.99</v>
       </c>
       <c r="D141" t="n">
-        <v>2.25</v>
+        <v>3.28</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CENTEXT-RE</t>
+          <t>RAJOOENG</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>3.62</v>
+        <v>53.21</v>
       </c>
       <c r="C142" t="n">
-        <v>3.7</v>
+        <v>54.95</v>
       </c>
       <c r="D142" t="n">
-        <v>2.21</v>
+        <v>3.27</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SPECIALITY</t>
+          <t>PHANTOMFX</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>154.1</v>
+        <v>86.2</v>
       </c>
       <c r="C143" t="n">
-        <v>157.5</v>
+        <v>89</v>
       </c>
       <c r="D143" t="n">
-        <v>2.21</v>
+        <v>3.25</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>OPTIFIN</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>15.45</v>
+        <v>10.85</v>
       </c>
       <c r="C144" t="n">
-        <v>15.79</v>
+        <v>11.2</v>
       </c>
       <c r="D144" t="n">
-        <v>2.2</v>
+        <v>3.23</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>2186.8</v>
+        <v>19.28</v>
       </c>
       <c r="C145" t="n">
-        <v>2235</v>
+        <v>19.9</v>
       </c>
       <c r="D145" t="n">
-        <v>2.2</v>
+        <v>3.22</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>BANG</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>32.27</v>
+        <v>6.21</v>
       </c>
       <c r="C146" t="n">
-        <v>32.98</v>
+        <v>6.41</v>
       </c>
       <c r="D146" t="n">
-        <v>2.2</v>
+        <v>3.22</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>SHRADDHA</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>24.17</v>
+        <v>155.1</v>
       </c>
       <c r="C147" t="n">
-        <v>24.7</v>
+        <v>160.1</v>
       </c>
       <c r="D147" t="n">
-        <v>2.19</v>
+        <v>3.22</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>148.08</v>
+        <v>1965</v>
       </c>
       <c r="C148" t="n">
-        <v>151.3</v>
+        <v>2027.7</v>
       </c>
       <c r="D148" t="n">
-        <v>2.17</v>
+        <v>3.19</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>AUTOIND</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>417</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="C149" t="n">
-        <v>426</v>
+        <v>84</v>
       </c>
       <c r="D149" t="n">
-        <v>2.16</v>
+        <v>3.19</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1.85</v>
+        <v>1622.7</v>
       </c>
       <c r="C150" t="n">
-        <v>1.89</v>
+        <v>1674.4</v>
       </c>
       <c r="D150" t="n">
-        <v>2.16</v>
+        <v>3.19</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>AURUS</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>351.2</v>
+        <v>4.4</v>
       </c>
       <c r="C151" t="n">
-        <v>358.8</v>
+        <v>4.54</v>
       </c>
       <c r="D151" t="n">
-        <v>2.16</v>
+        <v>3.18</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>BEEKAY</t>
+          <t>SPAL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>452.95</v>
+        <v>935.6</v>
       </c>
       <c r="C152" t="n">
-        <v>462.7</v>
+        <v>965.15</v>
       </c>
       <c r="D152" t="n">
-        <v>2.15</v>
+        <v>3.16</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>6.07</v>
+        <v>13.95</v>
       </c>
       <c r="C153" t="n">
-        <v>6.2</v>
+        <v>14.39</v>
       </c>
       <c r="D153" t="n">
-        <v>2.14</v>
+        <v>3.15</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>NIRLON</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>605</v>
+        <v>18.39</v>
       </c>
       <c r="C154" t="n">
-        <v>617.95</v>
+        <v>18.97</v>
       </c>
       <c r="D154" t="n">
-        <v>2.14</v>
+        <v>3.15</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>NINSYS</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>228.67</v>
+        <v>804.65</v>
       </c>
       <c r="C155" t="n">
-        <v>233.5</v>
+        <v>830</v>
       </c>
       <c r="D155" t="n">
-        <v>2.11</v>
+        <v>3.15</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TRF</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>197.82</v>
+        <v>208.4</v>
       </c>
       <c r="C156" t="n">
-        <v>202</v>
+        <v>214.95</v>
       </c>
       <c r="D156" t="n">
-        <v>2.11</v>
+        <v>3.14</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SASKEN</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>1672.7</v>
+        <v>1664.3</v>
       </c>
       <c r="C157" t="n">
-        <v>1707.8</v>
+        <v>1716.3</v>
       </c>
       <c r="D157" t="n">
-        <v>2.1</v>
+        <v>3.12</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>LANCER</t>
+          <t>NRAIL</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>11.45</v>
+        <v>659.5</v>
       </c>
       <c r="C158" t="n">
-        <v>11.69</v>
+        <v>680</v>
       </c>
       <c r="D158" t="n">
-        <v>2.1</v>
+        <v>3.11</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>XTRANET</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>285.05</v>
+        <v>574.15</v>
       </c>
       <c r="C159" t="n">
-        <v>291</v>
+        <v>592</v>
       </c>
       <c r="D159" t="n">
-        <v>2.09</v>
+        <v>3.11</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>HLEGLAS</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>439.4</v>
+        <v>14.52</v>
       </c>
       <c r="C160" t="n">
-        <v>448.45</v>
+        <v>14.97</v>
       </c>
       <c r="D160" t="n">
-        <v>2.06</v>
+        <v>3.1</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>INDOAMIN</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>142.07</v>
+        <v>324.95</v>
       </c>
       <c r="C161" t="n">
-        <v>145</v>
+        <v>335</v>
       </c>
       <c r="D161" t="n">
-        <v>2.06</v>
+        <v>3.09</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>BHADORA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>25.2</v>
+        <v>147.25</v>
       </c>
       <c r="C162" t="n">
-        <v>25.72</v>
+        <v>151.8</v>
       </c>
       <c r="D162" t="n">
-        <v>2.06</v>
+        <v>3.09</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>5.86</v>
+        <v>6.5</v>
       </c>
       <c r="C163" t="n">
-        <v>5.98</v>
+        <v>6.7</v>
       </c>
       <c r="D163" t="n">
-        <v>2.05</v>
+        <v>3.08</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>AUSTENG</t>
+          <t>MKPL</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>171.52</v>
+        <v>3.9</v>
       </c>
       <c r="C164" t="n">
-        <v>175</v>
+        <v>4.02</v>
       </c>
       <c r="D164" t="n">
-        <v>2.03</v>
+        <v>3.08</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>IVC</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>13.83</v>
+        <v>7.81</v>
       </c>
       <c r="C165" t="n">
-        <v>14.11</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="D165" t="n">
-        <v>2.02</v>
+        <v>3.07</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>50.92</v>
+        <v>44.34</v>
       </c>
       <c r="C166" t="n">
-        <v>51.95</v>
+        <v>45.7</v>
       </c>
       <c r="D166" t="n">
-        <v>2.02</v>
+        <v>3.07</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>EASTWEST</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>31.85</v>
+        <v>2.29</v>
       </c>
       <c r="C167" t="n">
-        <v>32.49</v>
+        <v>2.36</v>
       </c>
       <c r="D167" t="n">
-        <v>2.01</v>
+        <v>3.06</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>MANALIPETC</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>6.97</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="C168" t="n">
-        <v>7.11</v>
+        <v>80.53</v>
       </c>
       <c r="D168" t="n">
-        <v>2.01</v>
+        <v>3.05</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ONIXSOLAR</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>343.05</v>
+        <v>111.53</v>
       </c>
       <c r="C169" t="n">
-        <v>349.95</v>
+        <v>114.92</v>
       </c>
       <c r="D169" t="n">
-        <v>2.01</v>
+        <v>3.04</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MHLXMIRU</t>
+          <t>MVGJL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>179.21</v>
+        <v>206.69</v>
       </c>
       <c r="C170" t="n">
-        <v>182.79</v>
+        <v>212.94</v>
       </c>
       <c r="D170" t="n">
-        <v>2</v>
+        <v>3.02</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MBECL</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>484.32</v>
+        <v>125.08</v>
       </c>
       <c r="C171" t="n">
-        <v>494</v>
+        <v>128.85</v>
       </c>
       <c r="D171" t="n">
-        <v>2</v>
+        <v>3.01</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>EUROBOND</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.5</v>
+        <v>148.29</v>
       </c>
       <c r="C172" t="n">
-        <v>0.51</v>
+        <v>152.75</v>
       </c>
       <c r="D172" t="n">
-        <v>2</v>
+        <v>3.01</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>SCML</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>200.04</v>
+        <v>83.5</v>
       </c>
       <c r="C173" t="n">
-        <v>204.04</v>
+        <v>86</v>
       </c>
       <c r="D173" t="n">
-        <v>2</v>
+        <v>2.99</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>DENTALKART</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>460</v>
+        <v>679.5</v>
       </c>
       <c r="C174" t="n">
-        <v>469.2</v>
+        <v>699.8</v>
       </c>
       <c r="D174" t="n">
-        <v>2</v>
+        <v>2.99</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>RPEL</t>
+          <t>AKASH</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>1809</v>
+        <v>24.95</v>
       </c>
       <c r="C175" t="n">
-        <v>1845</v>
+        <v>25.69</v>
       </c>
       <c r="D175" t="n">
-        <v>1.99</v>
+        <v>2.97</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SADHNANIQ</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>2.53</v>
+        <v>31.08</v>
       </c>
       <c r="C176" t="n">
-        <v>2.58</v>
+        <v>32</v>
       </c>
       <c r="D176" t="n">
-        <v>1.98</v>
+        <v>2.96</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>13.11</v>
+        <v>51.38</v>
       </c>
       <c r="C177" t="n">
-        <v>13.37</v>
+        <v>52.9</v>
       </c>
       <c r="D177" t="n">
-        <v>1.98</v>
+        <v>2.96</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>68.45</v>
+        <v>190.4</v>
       </c>
       <c r="C178" t="n">
-        <v>69.8</v>
+        <v>196</v>
       </c>
       <c r="D178" t="n">
-        <v>1.97</v>
+        <v>2.94</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>RAMBHAJO</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.51</v>
+        <v>288.75</v>
       </c>
       <c r="C179" t="n">
-        <v>0.52</v>
+        <v>297.2</v>
       </c>
       <c r="D179" t="n">
-        <v>1.96</v>
+        <v>2.93</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>BVCL</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>40.21</v>
+        <v>41.39</v>
       </c>
       <c r="C180" t="n">
-        <v>41</v>
+        <v>42.6</v>
       </c>
       <c r="D180" t="n">
-        <v>1.96</v>
+        <v>2.92</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>CYBERTECH</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>126.23</v>
+        <v>135.95</v>
       </c>
       <c r="C181" t="n">
-        <v>128.7</v>
+        <v>139.9</v>
       </c>
       <c r="D181" t="n">
-        <v>1.96</v>
+        <v>2.91</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>ENKEIWHEL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>31.19</v>
+        <v>392.6</v>
       </c>
       <c r="C182" t="n">
-        <v>31.8</v>
+        <v>404</v>
       </c>
       <c r="D182" t="n">
-        <v>1.96</v>
+        <v>2.9</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>EVERESTIND</t>
+          <t>KALYANIFRG</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>455.6</v>
+        <v>944.75</v>
       </c>
       <c r="C183" t="n">
-        <v>464.5</v>
+        <v>972</v>
       </c>
       <c r="D183" t="n">
-        <v>1.95</v>
+        <v>2.88</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>BAGFILMS</t>
+          <t>PRANAV</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>4.1</v>
+        <v>97.20999999999999</v>
       </c>
       <c r="C184" t="n">
-        <v>4.18</v>
+        <v>100</v>
       </c>
       <c r="D184" t="n">
-        <v>1.95</v>
+        <v>2.87</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>GGBL</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>222.7</v>
+        <v>30.04</v>
       </c>
       <c r="C185" t="n">
-        <v>227</v>
+        <v>30.9</v>
       </c>
       <c r="D185" t="n">
-        <v>1.93</v>
+        <v>2.86</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ROHLTD</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>299.85</v>
+        <v>1.05</v>
       </c>
       <c r="C186" t="n">
-        <v>305.6</v>
+        <v>1.08</v>
       </c>
       <c r="D186" t="n">
-        <v>1.92</v>
+        <v>2.86</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>PRISMX</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>0.52</v>
+        <v>215.81</v>
       </c>
       <c r="C187" t="n">
-        <v>0.53</v>
+        <v>221.95</v>
       </c>
       <c r="D187" t="n">
-        <v>1.92</v>
+        <v>2.85</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>BPLPHARMA</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>127.58</v>
+        <v>1720.4</v>
       </c>
       <c r="C188" t="n">
-        <v>130</v>
+        <v>1769.2</v>
       </c>
       <c r="D188" t="n">
-        <v>1.9</v>
+        <v>2.84</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>KCK</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>16.34</v>
+        <v>14.1</v>
       </c>
       <c r="C189" t="n">
-        <v>16.65</v>
+        <v>14.5</v>
       </c>
       <c r="D189" t="n">
-        <v>1.9</v>
+        <v>2.84</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>INTLCONV</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>3.18</v>
+        <v>80.03</v>
       </c>
       <c r="C190" t="n">
-        <v>3.24</v>
+        <v>82.3</v>
       </c>
       <c r="D190" t="n">
-        <v>1.89</v>
+        <v>2.84</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>WEL</t>
+          <t>IWARE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>72.63</v>
+        <v>388</v>
       </c>
       <c r="C191" t="n">
-        <v>74</v>
+        <v>398.95</v>
       </c>
       <c r="D191" t="n">
-        <v>1.89</v>
+        <v>2.82</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>BESTAGRO</t>
+          <t>PRIMECAB</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>17.53</v>
+        <v>206.25</v>
       </c>
       <c r="C192" t="n">
-        <v>17.86</v>
+        <v>212</v>
       </c>
       <c r="D192" t="n">
-        <v>1.88</v>
+        <v>2.79</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SOMICONVEY</t>
+          <t>FEDDERSHOL</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>89.31</v>
+        <v>63.63</v>
       </c>
       <c r="C193" t="n">
-        <v>90.98999999999999</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D193" t="n">
-        <v>1.88</v>
+        <v>2.78</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>BSL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>1919</v>
+        <v>118.2</v>
       </c>
       <c r="C194" t="n">
-        <v>1954.9</v>
+        <v>121.49</v>
       </c>
       <c r="D194" t="n">
-        <v>1.87</v>
+        <v>2.78</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>6.97</v>
+        <v>3.24</v>
       </c>
       <c r="C195" t="n">
-        <v>7.1</v>
+        <v>3.33</v>
       </c>
       <c r="D195" t="n">
-        <v>1.87</v>
+        <v>2.78</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>2096</v>
+        <v>1.08</v>
       </c>
       <c r="C196" t="n">
-        <v>2135</v>
+        <v>1.11</v>
       </c>
       <c r="D196" t="n">
-        <v>1.86</v>
+        <v>2.78</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>INNOVANA</t>
+          <t>INVPRECQ</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>292.55</v>
+        <v>1595.2</v>
       </c>
       <c r="C197" t="n">
-        <v>298</v>
+        <v>1639</v>
       </c>
       <c r="D197" t="n">
-        <v>1.86</v>
+        <v>2.75</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>MOLDTECH</t>
+          <t>SUNSHIEL</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>206.16</v>
+        <v>1059</v>
       </c>
       <c r="C198" t="n">
-        <v>210</v>
+        <v>1088</v>
       </c>
       <c r="D198" t="n">
-        <v>1.86</v>
+        <v>2.74</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>BSOFT</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>40.69</v>
+        <v>269.75</v>
       </c>
       <c r="C199" t="n">
-        <v>41.44</v>
+        <v>277.15</v>
       </c>
       <c r="D199" t="n">
-        <v>1.84</v>
+        <v>2.74</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>PONNIERODE</t>
+          <t>SCHAND</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>372.2</v>
+        <v>143.57</v>
       </c>
       <c r="C200" t="n">
-        <v>379</v>
+        <v>147.5</v>
       </c>
       <c r="D200" t="n">
-        <v>1.83</v>
+        <v>2.74</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>BLUEDART</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>4629</v>
+        <v>776.7</v>
       </c>
       <c r="C201" t="n">
-        <v>4713.9</v>
+        <v>797.9</v>
       </c>
       <c r="D201" t="n">
-        <v>1.83</v>
+        <v>2.73</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-06 10:46 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PARTY-RE</t>
+          <t>SURANI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2</v>
+        <v>120.05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.25</v>
+        <v>144.05</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>19.99</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SURANI</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100.05</v>
+        <v>61.59</v>
       </c>
       <c r="C3" t="n">
-        <v>114.9</v>
+        <v>68</v>
       </c>
       <c r="D3" t="n">
-        <v>14.84</v>
+        <v>10.41</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>HBESD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74.18000000000001</v>
+        <v>78.13</v>
       </c>
       <c r="C4" t="n">
-        <v>82.40000000000001</v>
+        <v>86</v>
       </c>
       <c r="D4" t="n">
-        <v>11.08</v>
+        <v>10.07</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CENTEXT-RE</t>
+          <t>SAGARDEEP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.16</v>
+        <v>22.1</v>
       </c>
       <c r="C5" t="n">
-        <v>3.5</v>
+        <v>24</v>
       </c>
       <c r="D5" t="n">
-        <v>10.76</v>
+        <v>8.6</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HRYNSHP</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>97.98</v>
+        <v>2580</v>
       </c>
       <c r="C6" t="n">
-        <v>108</v>
+        <v>2800</v>
       </c>
       <c r="D6" t="n">
-        <v>10.23</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NIKITA</t>
+          <t>PRECOT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.09999999999999</v>
+        <v>605.1</v>
       </c>
       <c r="C7" t="n">
-        <v>72.7</v>
+        <v>653</v>
       </c>
       <c r="D7" t="n">
-        <v>9.98</v>
+        <v>7.92</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>LAGNAM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>5.45</v>
+        <v>76.7</v>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>7.88</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>DPWIRES</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>380.8</v>
+        <v>196.78</v>
       </c>
       <c r="C9" t="n">
-        <v>414.95</v>
+        <v>212.23</v>
       </c>
       <c r="D9" t="n">
-        <v>8.970000000000001</v>
+        <v>7.85</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5.42</v>
+        <v>1201</v>
       </c>
       <c r="C10" t="n">
-        <v>5.88</v>
+        <v>1294</v>
       </c>
       <c r="D10" t="n">
-        <v>8.49</v>
+        <v>7.74</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CGVAK</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>147.24</v>
+        <v>0.13</v>
       </c>
       <c r="C11" t="n">
-        <v>158.99</v>
+        <v>0.14</v>
       </c>
       <c r="D11" t="n">
-        <v>7.98</v>
+        <v>7.69</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47.76</v>
+        <v>37.16</v>
       </c>
       <c r="C12" t="n">
-        <v>51.5</v>
+        <v>39.87</v>
       </c>
       <c r="D12" t="n">
-        <v>7.83</v>
+        <v>7.29</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>STEAMHOUSE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.13</v>
+        <v>107.66</v>
       </c>
       <c r="C13" t="n">
-        <v>0.14</v>
+        <v>115</v>
       </c>
       <c r="D13" t="n">
-        <v>7.69</v>
+        <v>6.82</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PANORAMA</t>
+          <t>BALKRISHNA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>60.91</v>
+        <v>16</v>
       </c>
       <c r="C14" t="n">
-        <v>65.51000000000001</v>
+        <v>16.95</v>
       </c>
       <c r="D14" t="n">
-        <v>7.55</v>
+        <v>5.94</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>STLSTRINF</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21.52</v>
+        <v>8.84</v>
       </c>
       <c r="C15" t="n">
-        <v>22.99</v>
+        <v>9.35</v>
       </c>
       <c r="D15" t="n">
-        <v>6.83</v>
+        <v>5.77</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>TOLINS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8.380000000000001</v>
+        <v>85.12</v>
       </c>
       <c r="C16" t="n">
-        <v>8.949999999999999</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>6.8</v>
+        <v>5.73</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OMFREIGHT</t>
+          <t>AVANA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>97.5</v>
+        <v>139.25</v>
       </c>
       <c r="C17" t="n">
-        <v>103.99</v>
+        <v>146.9</v>
       </c>
       <c r="D17" t="n">
-        <v>6.66</v>
+        <v>5.49</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PACIFICI</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>135.99</v>
+        <v>0.19</v>
       </c>
       <c r="C18" t="n">
-        <v>144.99</v>
+        <v>0.2</v>
       </c>
       <c r="D18" t="n">
-        <v>6.62</v>
+        <v>5.26</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>KDGREEN</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>46.76</v>
+        <v>8</v>
       </c>
       <c r="C19" t="n">
-        <v>49.7</v>
+        <v>8.4</v>
       </c>
       <c r="D19" t="n">
-        <v>6.29</v>
+        <v>5</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAHAPEXLTD</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>50.18</v>
+        <v>232.95</v>
       </c>
       <c r="C20" t="n">
-        <v>53.3</v>
+        <v>244.59</v>
       </c>
       <c r="D20" t="n">
-        <v>6.22</v>
+        <v>5</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>KORE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>72.52</v>
+        <v>191</v>
       </c>
       <c r="C21" t="n">
-        <v>77</v>
+        <v>200.55</v>
       </c>
       <c r="D21" t="n">
-        <v>6.18</v>
+        <v>5</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AUSTENG</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>167.72</v>
+        <v>1253.7</v>
       </c>
       <c r="C22" t="n">
-        <v>177.9</v>
+        <v>1316.35</v>
       </c>
       <c r="D22" t="n">
-        <v>6.07</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>QUINTEGRA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>148.85</v>
+        <v>1.4</v>
       </c>
       <c r="C23" t="n">
-        <v>157.65</v>
+        <v>1.47</v>
       </c>
       <c r="D23" t="n">
-        <v>5.91</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NOIDATOLL</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.56</v>
+        <v>2410.9</v>
       </c>
       <c r="C24" t="n">
-        <v>3.77</v>
+        <v>2531.4</v>
       </c>
       <c r="D24" t="n">
-        <v>5.9</v>
+        <v>5</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VTMLTD</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>38.15</v>
+        <v>250.27</v>
       </c>
       <c r="C25" t="n">
-        <v>40.4</v>
+        <v>262.78</v>
       </c>
       <c r="D25" t="n">
-        <v>5.9</v>
+        <v>5</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SACHEEROME</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>499.65</v>
+        <v>177.26</v>
       </c>
       <c r="C26" t="n">
-        <v>529</v>
+        <v>186.12</v>
       </c>
       <c r="D26" t="n">
-        <v>5.87</v>
+        <v>5</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>774.5</v>
+        <v>472.25</v>
       </c>
       <c r="C27" t="n">
-        <v>819.9</v>
+        <v>495.85</v>
       </c>
       <c r="D27" t="n">
-        <v>5.86</v>
+        <v>5</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FAIRCHEMOR</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>661.5</v>
+        <v>48.8</v>
       </c>
       <c r="C28" t="n">
-        <v>699.95</v>
+        <v>51.24</v>
       </c>
       <c r="D28" t="n">
-        <v>5.81</v>
+        <v>5</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TGVSL</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>116.38</v>
+        <v>37.67</v>
       </c>
       <c r="C29" t="n">
-        <v>123.12</v>
+        <v>39.55</v>
       </c>
       <c r="D29" t="n">
-        <v>5.79</v>
+        <v>4.99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>25.41</v>
+        <v>5.21</v>
       </c>
       <c r="C30" t="n">
-        <v>26.85</v>
+        <v>5.47</v>
       </c>
       <c r="D30" t="n">
-        <v>5.67</v>
+        <v>4.99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SANGAMIND</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>634.55</v>
+        <v>541.95</v>
       </c>
       <c r="C31" t="n">
-        <v>670</v>
+        <v>569</v>
       </c>
       <c r="D31" t="n">
-        <v>5.59</v>
+        <v>4.99</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>BMISL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.18</v>
+        <v>115.5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.19</v>
+        <v>121.25</v>
       </c>
       <c r="D32" t="n">
-        <v>5.56</v>
+        <v>4.98</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>76.75</v>
+        <v>16.51</v>
       </c>
       <c r="C33" t="n">
-        <v>81</v>
+        <v>17.33</v>
       </c>
       <c r="D33" t="n">
-        <v>5.54</v>
+        <v>4.97</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>VOEPL</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>493</v>
+        <v>1.61</v>
       </c>
       <c r="C34" t="n">
-        <v>520</v>
+        <v>1.69</v>
       </c>
       <c r="D34" t="n">
-        <v>5.48</v>
+        <v>4.97</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUNLOC</t>
+          <t>AVATAR</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>70.09999999999999</v>
+        <v>159</v>
       </c>
       <c r="C35" t="n">
-        <v>73.90000000000001</v>
+        <v>166.9</v>
       </c>
       <c r="D35" t="n">
-        <v>5.42</v>
+        <v>4.97</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>31.32</v>
+        <v>10.89</v>
       </c>
       <c r="C36" t="n">
-        <v>32.98</v>
+        <v>11.43</v>
       </c>
       <c r="D36" t="n">
-        <v>5.3</v>
+        <v>4.96</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TECHD</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>531.95</v>
+        <v>16.33</v>
       </c>
       <c r="C37" t="n">
-        <v>559.95</v>
+        <v>17.14</v>
       </c>
       <c r="D37" t="n">
-        <v>5.26</v>
+        <v>4.96</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>ABAN</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.19</v>
+        <v>16.12</v>
       </c>
       <c r="C38" t="n">
-        <v>0.2</v>
+        <v>16.92</v>
       </c>
       <c r="D38" t="n">
-        <v>5.26</v>
+        <v>4.96</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SEDEMAC</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3432.8</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C39" t="n">
-        <v>3607.8</v>
+        <v>81.45</v>
       </c>
       <c r="D39" t="n">
-        <v>5.1</v>
+        <v>4.96</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HEROMOTORS</t>
+          <t>BURNPUR</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>167.8</v>
+        <v>13.18</v>
       </c>
       <c r="C40" t="n">
-        <v>176.34</v>
+        <v>13.83</v>
       </c>
       <c r="D40" t="n">
-        <v>5.09</v>
+        <v>4.93</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4.57</v>
+        <v>8.17</v>
       </c>
       <c r="C41" t="n">
-        <v>4.8</v>
+        <v>8.57</v>
       </c>
       <c r="D41" t="n">
-        <v>5.03</v>
+        <v>4.9</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>BIOPOL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1076.9</v>
+        <v>49.3</v>
       </c>
       <c r="C42" t="n">
-        <v>1130.7</v>
+        <v>51.7</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>4.87</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2.6</v>
+        <v>5.99</v>
       </c>
       <c r="C43" t="n">
-        <v>2.73</v>
+        <v>6.28</v>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>4.84</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>516.15</v>
+        <v>4.97</v>
       </c>
       <c r="C44" t="n">
-        <v>541.95</v>
+        <v>5.21</v>
       </c>
       <c r="D44" t="n">
-        <v>5</v>
+        <v>4.83</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>UNIVPHOTO</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>490</v>
+        <v>56.24</v>
       </c>
       <c r="C45" t="n">
-        <v>514.5</v>
+        <v>58.95</v>
       </c>
       <c r="D45" t="n">
-        <v>5</v>
+        <v>4.82</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>ABH</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>168.82</v>
+        <v>43.5</v>
       </c>
       <c r="C46" t="n">
-        <v>177.26</v>
+        <v>45.55</v>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>4.71</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>AKSHARCHEM</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>46.48</v>
+        <v>365.3</v>
       </c>
       <c r="C47" t="n">
-        <v>48.8</v>
+        <v>382.5</v>
       </c>
       <c r="D47" t="n">
-        <v>4.99</v>
+        <v>4.71</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SPRL</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>146.2</v>
+        <v>21.06</v>
       </c>
       <c r="C48" t="n">
-        <v>153.5</v>
+        <v>22.05</v>
       </c>
       <c r="D48" t="n">
-        <v>4.99</v>
+        <v>4.7</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>35.88</v>
+        <v>536.8</v>
       </c>
       <c r="C49" t="n">
-        <v>37.67</v>
+        <v>562</v>
       </c>
       <c r="D49" t="n">
-        <v>4.99</v>
+        <v>4.69</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>464</v>
+        <v>101.25</v>
       </c>
       <c r="C50" t="n">
-        <v>487</v>
+        <v>106</v>
       </c>
       <c r="D50" t="n">
-        <v>4.96</v>
+        <v>4.69</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ABAN</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>15.36</v>
+        <v>213.99</v>
       </c>
       <c r="C51" t="n">
-        <v>16.12</v>
+        <v>224</v>
       </c>
       <c r="D51" t="n">
-        <v>4.95</v>
+        <v>4.68</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15.56</v>
+        <v>50.64</v>
       </c>
       <c r="C52" t="n">
-        <v>16.33</v>
+        <v>53</v>
       </c>
       <c r="D52" t="n">
-        <v>4.95</v>
+        <v>4.66</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>KEYFINSERV</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>449.8</v>
+        <v>237.01</v>
       </c>
       <c r="C53" t="n">
-        <v>472</v>
+        <v>247.9</v>
       </c>
       <c r="D53" t="n">
-        <v>4.94</v>
+        <v>4.59</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>WHBRADY</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>465.05</v>
+        <v>12.49</v>
       </c>
       <c r="C54" t="n">
-        <v>488</v>
+        <v>13.06</v>
       </c>
       <c r="D54" t="n">
-        <v>4.93</v>
+        <v>4.56</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6.72</v>
+        <v>75.5</v>
       </c>
       <c r="C55" t="n">
-        <v>7.05</v>
+        <v>78.92</v>
       </c>
       <c r="D55" t="n">
-        <v>4.91</v>
+        <v>4.53</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>UNIENTER</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>5.71</v>
+        <v>86.17</v>
       </c>
       <c r="C56" t="n">
-        <v>5.99</v>
+        <v>90</v>
       </c>
       <c r="D56" t="n">
-        <v>4.9</v>
+        <v>4.44</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>MUTHOOTCAP</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>38.9</v>
+        <v>219.33</v>
       </c>
       <c r="C57" t="n">
-        <v>40.8</v>
+        <v>229.05</v>
       </c>
       <c r="D57" t="n">
-        <v>4.88</v>
+        <v>4.43</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>193.49</v>
+        <v>160.27</v>
       </c>
       <c r="C58" t="n">
-        <v>202.9</v>
+        <v>167.35</v>
       </c>
       <c r="D58" t="n">
-        <v>4.86</v>
+        <v>4.42</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>41.57</v>
+        <v>13.79</v>
       </c>
       <c r="C59" t="n">
-        <v>43.59</v>
+        <v>14.4</v>
       </c>
       <c r="D59" t="n">
-        <v>4.86</v>
+        <v>4.42</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>APSISAERO</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>555</v>
+        <v>1.36</v>
       </c>
       <c r="C60" t="n">
-        <v>581.95</v>
+        <v>1.42</v>
       </c>
       <c r="D60" t="n">
-        <v>4.86</v>
+        <v>4.41</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>KILITCH</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2.06</v>
+        <v>233.74</v>
       </c>
       <c r="C61" t="n">
-        <v>2.16</v>
+        <v>244</v>
       </c>
       <c r="D61" t="n">
-        <v>4.85</v>
+        <v>4.39</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>COMPEAU</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>362.45</v>
+        <v>4.78</v>
       </c>
       <c r="C62" t="n">
-        <v>380</v>
+        <v>4.99</v>
       </c>
       <c r="D62" t="n">
-        <v>4.84</v>
+        <v>4.39</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>RKDL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>35.91</v>
+        <v>17.05</v>
       </c>
       <c r="C63" t="n">
-        <v>37.64</v>
+        <v>17.79</v>
       </c>
       <c r="D63" t="n">
-        <v>4.82</v>
+        <v>4.34</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AIROLAM</t>
+          <t>ALPINETEX</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>89.58</v>
+        <v>45.82</v>
       </c>
       <c r="C64" t="n">
-        <v>93.90000000000001</v>
+        <v>47.8</v>
       </c>
       <c r="D64" t="n">
-        <v>4.82</v>
+        <v>4.32</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>KILITCH</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>218.51</v>
+        <v>114.5</v>
       </c>
       <c r="C65" t="n">
-        <v>229</v>
+        <v>119.4</v>
       </c>
       <c r="D65" t="n">
-        <v>4.8</v>
+        <v>4.28</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TEAMTECH</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>145.95</v>
+        <v>108.95</v>
       </c>
       <c r="C66" t="n">
-        <v>152.85</v>
+        <v>113.6</v>
       </c>
       <c r="D66" t="n">
-        <v>4.73</v>
+        <v>4.27</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>540.35</v>
+        <v>1.43</v>
       </c>
       <c r="C67" t="n">
-        <v>565.85</v>
+        <v>1.49</v>
       </c>
       <c r="D67" t="n">
-        <v>4.72</v>
+        <v>4.2</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2.55</v>
+        <v>224.7</v>
       </c>
       <c r="C68" t="n">
-        <v>2.67</v>
+        <v>233.9</v>
       </c>
       <c r="D68" t="n">
-        <v>4.71</v>
+        <v>4.09</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>AISL</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>66.84999999999999</v>
+        <v>143.02</v>
       </c>
       <c r="C69" t="n">
-        <v>70</v>
+        <v>148.8</v>
       </c>
       <c r="D69" t="n">
-        <v>4.71</v>
+        <v>4.04</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1.28</v>
+        <v>29.79</v>
       </c>
       <c r="C70" t="n">
-        <v>1.34</v>
+        <v>30.99</v>
       </c>
       <c r="D70" t="n">
-        <v>4.69</v>
+        <v>4.03</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>HITECH</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>2.36</v>
+        <v>70.05</v>
       </c>
       <c r="C71" t="n">
-        <v>2.47</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="D71" t="n">
-        <v>4.66</v>
+        <v>4</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PELATRO</t>
+          <t>HPIL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>359.9</v>
+        <v>110.64</v>
       </c>
       <c r="C72" t="n">
-        <v>376.5</v>
+        <v>115</v>
       </c>
       <c r="D72" t="n">
-        <v>4.61</v>
+        <v>3.94</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>VISHAL</t>
+          <t>CENTEXT-RE</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>17.38</v>
+        <v>2.79</v>
       </c>
       <c r="C73" t="n">
-        <v>18.18</v>
+        <v>2.9</v>
       </c>
       <c r="D73" t="n">
-        <v>4.6</v>
+        <v>3.94</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>4.81</v>
+        <v>4.85</v>
       </c>
       <c r="C74" t="n">
-        <v>5.03</v>
+        <v>5.04</v>
       </c>
       <c r="D74" t="n">
-        <v>4.57</v>
+        <v>3.92</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>10.32</v>
+        <v>15.58</v>
       </c>
       <c r="C75" t="n">
-        <v>10.79</v>
+        <v>16.19</v>
       </c>
       <c r="D75" t="n">
-        <v>4.55</v>
+        <v>3.92</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>38.24</v>
+        <v>126.05</v>
       </c>
       <c r="C76" t="n">
-        <v>39.98</v>
+        <v>130.95</v>
       </c>
       <c r="D76" t="n">
-        <v>4.55</v>
+        <v>3.89</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>13.68</v>
+        <v>54.24</v>
       </c>
       <c r="C77" t="n">
-        <v>14.3</v>
+        <v>56.34</v>
       </c>
       <c r="D77" t="n">
-        <v>4.53</v>
+        <v>3.87</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MASKINVEST</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>143.41</v>
+        <v>221.97</v>
       </c>
       <c r="C78" t="n">
-        <v>149.9</v>
+        <v>230.33</v>
       </c>
       <c r="D78" t="n">
-        <v>4.53</v>
+        <v>3.77</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>VTMLTD</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>66.51000000000001</v>
+        <v>38.27</v>
       </c>
       <c r="C79" t="n">
-        <v>69.5</v>
+        <v>39.7</v>
       </c>
       <c r="D79" t="n">
-        <v>4.5</v>
+        <v>3.74</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>QUINTEGRA</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1.34</v>
+        <v>197.18</v>
       </c>
       <c r="C80" t="n">
-        <v>1.4</v>
+        <v>204.49</v>
       </c>
       <c r="D80" t="n">
-        <v>4.48</v>
+        <v>3.71</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1.37</v>
+        <v>4.41</v>
       </c>
       <c r="C81" t="n">
-        <v>1.43</v>
+        <v>4.57</v>
       </c>
       <c r="D81" t="n">
-        <v>4.38</v>
+        <v>3.63</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>CYBERMEDIA</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>89.95999999999999</v>
+        <v>17.69</v>
       </c>
       <c r="C82" t="n">
-        <v>93.90000000000001</v>
+        <v>18.33</v>
       </c>
       <c r="D82" t="n">
-        <v>4.38</v>
+        <v>3.62</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>159.06</v>
+        <v>34.12</v>
       </c>
       <c r="C83" t="n">
-        <v>166</v>
+        <v>35.35</v>
       </c>
       <c r="D83" t="n">
-        <v>4.36</v>
+        <v>3.6</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>AVADHSUGAR</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.46</v>
+        <v>840.35</v>
       </c>
       <c r="C84" t="n">
-        <v>0.48</v>
+        <v>870.45</v>
       </c>
       <c r="D84" t="n">
-        <v>4.35</v>
+        <v>3.58</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>631.85</v>
+        <v>0.28</v>
       </c>
       <c r="C85" t="n">
-        <v>659.35</v>
+        <v>0.29</v>
       </c>
       <c r="D85" t="n">
-        <v>4.35</v>
+        <v>3.57</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>GILLANDERS</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>1243.2</v>
+        <v>115.73</v>
       </c>
       <c r="C86" t="n">
-        <v>1297</v>
+        <v>119.8</v>
       </c>
       <c r="D86" t="n">
-        <v>4.33</v>
+        <v>3.52</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>23</v>
+        <v>227.86</v>
       </c>
       <c r="C87" t="n">
-        <v>23.99</v>
+        <v>235.85</v>
       </c>
       <c r="D87" t="n">
-        <v>4.3</v>
+        <v>3.51</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>RFBL</t>
+          <t>EBIX</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>107.1</v>
+        <v>16.91</v>
       </c>
       <c r="C88" t="n">
-        <v>111.7</v>
+        <v>17.5</v>
       </c>
       <c r="D88" t="n">
-        <v>4.3</v>
+        <v>3.49</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>UGARSUGAR</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>35.19</v>
+        <v>58.84</v>
       </c>
       <c r="C89" t="n">
-        <v>36.7</v>
+        <v>60.89</v>
       </c>
       <c r="D89" t="n">
-        <v>4.29</v>
+        <v>3.48</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>INNOMET</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>280</v>
+        <v>1.46</v>
       </c>
       <c r="C90" t="n">
-        <v>292</v>
+        <v>1.51</v>
       </c>
       <c r="D90" t="n">
-        <v>4.29</v>
+        <v>3.42</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ABCOTS</t>
+          <t>WILLAMAGOR</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>189.91</v>
+        <v>21.67</v>
       </c>
       <c r="C91" t="n">
-        <v>198</v>
+        <v>22.4</v>
       </c>
       <c r="D91" t="n">
-        <v>4.26</v>
+        <v>3.37</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>7.09</v>
+        <v>1001.25</v>
       </c>
       <c r="C92" t="n">
-        <v>7.39</v>
+        <v>1034.4</v>
       </c>
       <c r="D92" t="n">
-        <v>4.23</v>
+        <v>3.31</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>TRANSRAILL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>34.93</v>
+        <v>462.75</v>
       </c>
       <c r="C93" t="n">
-        <v>36.39</v>
+        <v>478</v>
       </c>
       <c r="D93" t="n">
-        <v>4.18</v>
+        <v>3.3</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>ELECTHERM</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>10.56</v>
+        <v>702.4</v>
       </c>
       <c r="C94" t="n">
-        <v>11</v>
+        <v>725.4</v>
       </c>
       <c r="D94" t="n">
-        <v>4.17</v>
+        <v>3.27</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>580</v>
+        <v>15.98</v>
       </c>
       <c r="C95" t="n">
-        <v>604</v>
+        <v>16.5</v>
       </c>
       <c r="D95" t="n">
-        <v>4.14</v>
+        <v>3.25</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>5.32</v>
+        <v>22.76</v>
       </c>
       <c r="C96" t="n">
-        <v>5.54</v>
+        <v>23.5</v>
       </c>
       <c r="D96" t="n">
-        <v>4.14</v>
+        <v>3.25</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>GOKULAGRO</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>253.35</v>
+        <v>205.27</v>
       </c>
       <c r="C97" t="n">
-        <v>263.8</v>
+        <v>211.89</v>
       </c>
       <c r="D97" t="n">
-        <v>4.12</v>
+        <v>3.23</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BLACKROSE</t>
+          <t>ROXHITECH</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>110.45</v>
+        <v>62.45</v>
       </c>
       <c r="C98" t="n">
-        <v>115</v>
+        <v>64.45</v>
       </c>
       <c r="D98" t="n">
-        <v>4.12</v>
+        <v>3.2</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MAANALU</t>
+          <t>TRIVENI</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>99.34</v>
+        <v>237.22</v>
       </c>
       <c r="C99" t="n">
-        <v>103.4</v>
+        <v>244.8</v>
       </c>
       <c r="D99" t="n">
-        <v>4.09</v>
+        <v>3.2</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>17.09</v>
+        <v>11.58</v>
       </c>
       <c r="C100" t="n">
-        <v>17.78</v>
+        <v>11.95</v>
       </c>
       <c r="D100" t="n">
-        <v>4.04</v>
+        <v>3.2</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>245.01</v>
+        <v>199.92</v>
       </c>
       <c r="C101" t="n">
-        <v>254.9</v>
+        <v>206.3</v>
       </c>
       <c r="D101" t="n">
-        <v>4.04</v>
+        <v>3.19</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BESTAGRO</t>
+          <t>SKYTECH</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>17.47</v>
+        <v>40.7</v>
       </c>
       <c r="C102" t="n">
-        <v>18.17</v>
+        <v>42</v>
       </c>
       <c r="D102" t="n">
-        <v>4.01</v>
+        <v>3.19</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>15.34</v>
+        <v>173</v>
       </c>
       <c r="C103" t="n">
-        <v>15.95</v>
+        <v>178.5</v>
       </c>
       <c r="D103" t="n">
-        <v>3.98</v>
+        <v>3.18</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>525.4</v>
+        <v>28.09</v>
       </c>
       <c r="C104" t="n">
-        <v>545.9</v>
+        <v>28.98</v>
       </c>
       <c r="D104" t="n">
-        <v>3.9</v>
+        <v>3.17</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SPLIL</t>
+          <t>ARCHIES</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>28.5</v>
+        <v>12.35</v>
       </c>
       <c r="C105" t="n">
-        <v>29.6</v>
+        <v>12.74</v>
       </c>
       <c r="D105" t="n">
-        <v>3.86</v>
+        <v>3.16</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>PVSL</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1.3</v>
+        <v>91.08</v>
       </c>
       <c r="C106" t="n">
-        <v>1.35</v>
+        <v>93.95999999999999</v>
       </c>
       <c r="D106" t="n">
-        <v>3.85</v>
+        <v>3.16</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MIDWESTLTD</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>904.15</v>
+        <v>6.05</v>
       </c>
       <c r="C107" t="n">
-        <v>938.85</v>
+        <v>6.24</v>
       </c>
       <c r="D107" t="n">
-        <v>3.84</v>
+        <v>3.14</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>NATHBIOGEN</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>67.42</v>
+        <v>134.29</v>
       </c>
       <c r="C108" t="n">
-        <v>69.98999999999999</v>
+        <v>138.5</v>
       </c>
       <c r="D108" t="n">
-        <v>3.81</v>
+        <v>3.14</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1874</v>
+        <v>4.83</v>
       </c>
       <c r="C109" t="n">
-        <v>1945</v>
+        <v>4.98</v>
       </c>
       <c r="D109" t="n">
-        <v>3.79</v>
+        <v>3.11</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>21.19</v>
+        <v>54.8</v>
       </c>
       <c r="C110" t="n">
-        <v>21.99</v>
+        <v>56.5</v>
       </c>
       <c r="D110" t="n">
-        <v>3.78</v>
+        <v>3.1</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>PAVNAIND</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>15.36</v>
+        <v>5.8</v>
       </c>
       <c r="C111" t="n">
-        <v>15.94</v>
+        <v>5.98</v>
       </c>
       <c r="D111" t="n">
-        <v>3.78</v>
+        <v>3.1</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>477.05</v>
+        <v>290.8</v>
       </c>
       <c r="C112" t="n">
-        <v>494.95</v>
+        <v>299.8</v>
       </c>
       <c r="D112" t="n">
-        <v>3.75</v>
+        <v>3.09</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>35.66</v>
+        <v>36.97</v>
       </c>
       <c r="C113" t="n">
-        <v>36.99</v>
+        <v>38.1</v>
       </c>
       <c r="D113" t="n">
-        <v>3.73</v>
+        <v>3.06</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SMARTLINK</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>212.1</v>
+        <v>11.15</v>
       </c>
       <c r="C114" t="n">
-        <v>220</v>
+        <v>11.49</v>
       </c>
       <c r="D114" t="n">
-        <v>3.72</v>
+        <v>3.05</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.8100000000000001</v>
+        <v>1668.9</v>
       </c>
       <c r="C115" t="n">
-        <v>0.84</v>
+        <v>1719.8</v>
       </c>
       <c r="D115" t="n">
-        <v>3.7</v>
+        <v>3.05</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MONEYVIEW</t>
+          <t>RAJSREESUG</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>53.88</v>
+        <v>28.39</v>
       </c>
       <c r="C116" t="n">
-        <v>55.85</v>
+        <v>29.25</v>
       </c>
       <c r="D116" t="n">
-        <v>3.66</v>
+        <v>3.03</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>23.59</v>
+        <v>227.25</v>
       </c>
       <c r="C117" t="n">
-        <v>24.45</v>
+        <v>234</v>
       </c>
       <c r="D117" t="n">
-        <v>3.65</v>
+        <v>2.97</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>TUTIALKA</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>53.98</v>
+        <v>81.48</v>
       </c>
       <c r="C118" t="n">
-        <v>55.92</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="D118" t="n">
-        <v>3.59</v>
+        <v>2.97</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NDL</t>
+          <t>NTCIND</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>2.54</v>
+        <v>135.97</v>
       </c>
       <c r="C119" t="n">
-        <v>2.63</v>
+        <v>140</v>
       </c>
       <c r="D119" t="n">
-        <v>3.54</v>
+        <v>2.96</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>DHAMPURSUG</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>5.1</v>
+        <v>176.85</v>
       </c>
       <c r="C120" t="n">
-        <v>5.28</v>
+        <v>182</v>
       </c>
       <c r="D120" t="n">
-        <v>3.53</v>
+        <v>2.91</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AAATECH</t>
+          <t>BANSWRAS</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>92.73999999999999</v>
+        <v>102.93</v>
       </c>
       <c r="C121" t="n">
-        <v>96</v>
+        <v>105.93</v>
       </c>
       <c r="D121" t="n">
-        <v>3.52</v>
+        <v>2.91</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>33.76</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="C122" t="n">
-        <v>34.95</v>
+        <v>0.71</v>
       </c>
       <c r="D122" t="n">
-        <v>3.52</v>
+        <v>2.9</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>WATERBASE</t>
+          <t>ALLCARGO</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>45.4</v>
+        <v>10.03</v>
       </c>
       <c r="C123" t="n">
-        <v>47</v>
+        <v>10.32</v>
       </c>
       <c r="D123" t="n">
-        <v>3.52</v>
+        <v>2.89</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>RKSWAMY</t>
+          <t>APRAMEYA</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>86.45999999999999</v>
+        <v>102</v>
       </c>
       <c r="C124" t="n">
-        <v>89.5</v>
+        <v>104.95</v>
       </c>
       <c r="D124" t="n">
-        <v>3.52</v>
+        <v>2.89</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>PRADPME</t>
+          <t>RENUKA</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>449.25</v>
+        <v>21.76</v>
       </c>
       <c r="C125" t="n">
-        <v>465</v>
+        <v>22.38</v>
       </c>
       <c r="D125" t="n">
-        <v>3.51</v>
+        <v>2.85</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>ENIL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>205.77</v>
+        <v>91.69</v>
       </c>
       <c r="C126" t="n">
-        <v>213</v>
+        <v>94.3</v>
       </c>
       <c r="D126" t="n">
-        <v>3.51</v>
+        <v>2.85</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>36.24</v>
+        <v>15.46</v>
       </c>
       <c r="C127" t="n">
-        <v>37.5</v>
+        <v>15.9</v>
       </c>
       <c r="D127" t="n">
-        <v>3.48</v>
+        <v>2.85</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>BRNL</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>449.6</v>
+        <v>16.13</v>
       </c>
       <c r="C128" t="n">
-        <v>465</v>
+        <v>16.59</v>
       </c>
       <c r="D128" t="n">
-        <v>3.43</v>
+        <v>2.85</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>UNIENTER</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>87.02</v>
+        <v>7.05</v>
       </c>
       <c r="C129" t="n">
-        <v>90</v>
+        <v>7.25</v>
       </c>
       <c r="D129" t="n">
-        <v>3.42</v>
+        <v>2.84</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>PRABHA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>34.8</v>
+        <v>214.9</v>
       </c>
       <c r="C130" t="n">
-        <v>35.99</v>
+        <v>221</v>
       </c>
       <c r="D130" t="n">
-        <v>3.42</v>
+        <v>2.84</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>6.16</v>
+        <v>143.92</v>
       </c>
       <c r="C131" t="n">
-        <v>6.37</v>
+        <v>147.99</v>
       </c>
       <c r="D131" t="n">
-        <v>3.41</v>
+        <v>2.83</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MPIMANIPAL</t>
+          <t>TECHD</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>401.4</v>
+        <v>552</v>
       </c>
       <c r="C132" t="n">
-        <v>415</v>
+        <v>567.5</v>
       </c>
       <c r="D132" t="n">
-        <v>3.39</v>
+        <v>2.81</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>127.7</v>
+        <v>27.11</v>
       </c>
       <c r="C133" t="n">
-        <v>131.99</v>
+        <v>27.87</v>
       </c>
       <c r="D133" t="n">
-        <v>3.36</v>
+        <v>2.8</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ISHANCH</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>47.3</v>
+        <v>20.04</v>
       </c>
       <c r="C134" t="n">
-        <v>48.89</v>
+        <v>20.6</v>
       </c>
       <c r="D134" t="n">
-        <v>3.36</v>
+        <v>2.79</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>SHUKRAPHAR</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>4.21</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="C135" t="n">
-        <v>4.35</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D135" t="n">
-        <v>3.33</v>
+        <v>2.71</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ESCONET</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>246.8</v>
+        <v>19.96</v>
       </c>
       <c r="C136" t="n">
-        <v>255</v>
+        <v>20.5</v>
       </c>
       <c r="D136" t="n">
-        <v>3.32</v>
+        <v>2.71</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>KRITINUT</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>66.53</v>
+        <v>52.08</v>
       </c>
       <c r="C137" t="n">
-        <v>68.73999999999999</v>
+        <v>53.49</v>
       </c>
       <c r="D137" t="n">
-        <v>3.32</v>
+        <v>2.71</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>WATERBASE</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>118.66</v>
+        <v>45.57</v>
       </c>
       <c r="C138" t="n">
-        <v>122.6</v>
+        <v>46.79</v>
       </c>
       <c r="D138" t="n">
-        <v>3.32</v>
+        <v>2.68</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>15.73</v>
+        <v>9.32</v>
       </c>
       <c r="C139" t="n">
-        <v>16.25</v>
+        <v>9.57</v>
       </c>
       <c r="D139" t="n">
-        <v>3.31</v>
+        <v>2.68</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SECMARK</t>
+          <t>VOEPL</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>137.48</v>
+        <v>506.1</v>
       </c>
       <c r="C140" t="n">
-        <v>142</v>
+        <v>519.65</v>
       </c>
       <c r="D140" t="n">
-        <v>3.29</v>
+        <v>2.68</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>JOCIL</t>
+          <t>SHERA</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>145.22</v>
+        <v>187</v>
       </c>
       <c r="C141" t="n">
-        <v>149.99</v>
+        <v>192</v>
       </c>
       <c r="D141" t="n">
-        <v>3.28</v>
+        <v>2.67</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>RAJOOENG</t>
+          <t>NRAIL</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>53.21</v>
+        <v>661.35</v>
       </c>
       <c r="C142" t="n">
-        <v>54.95</v>
+        <v>679</v>
       </c>
       <c r="D142" t="n">
-        <v>3.27</v>
+        <v>2.67</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>PHANTOMFX</t>
+          <t>INVPRECQ</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>86.2</v>
+        <v>1612.1</v>
       </c>
       <c r="C143" t="n">
-        <v>89</v>
+        <v>1655</v>
       </c>
       <c r="D143" t="n">
-        <v>3.25</v>
+        <v>2.66</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>10.85</v>
+        <v>10.93</v>
       </c>
       <c r="C144" t="n">
-        <v>11.2</v>
+        <v>11.22</v>
       </c>
       <c r="D144" t="n">
-        <v>3.23</v>
+        <v>2.65</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>19.28</v>
+        <v>0.38</v>
       </c>
       <c r="C145" t="n">
-        <v>19.9</v>
+        <v>0.39</v>
       </c>
       <c r="D145" t="n">
-        <v>3.22</v>
+        <v>2.63</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>ANONDITA</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>6.21</v>
+        <v>1031</v>
       </c>
       <c r="C146" t="n">
-        <v>6.41</v>
+        <v>1057.95</v>
       </c>
       <c r="D146" t="n">
-        <v>3.22</v>
+        <v>2.61</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SHRADDHA</t>
+          <t>ACEVECTOR</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>155.1</v>
+        <v>26.08</v>
       </c>
       <c r="C147" t="n">
-        <v>160.1</v>
+        <v>26.75</v>
       </c>
       <c r="D147" t="n">
-        <v>3.22</v>
+        <v>2.57</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>GAUDIUMIVF</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>1965</v>
+        <v>103.25</v>
       </c>
       <c r="C148" t="n">
-        <v>2027.7</v>
+        <v>105.89</v>
       </c>
       <c r="D148" t="n">
-        <v>3.19</v>
+        <v>2.56</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>AUTOIND</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>81.40000000000001</v>
+        <v>19.99</v>
       </c>
       <c r="C149" t="n">
-        <v>84</v>
+        <v>20.5</v>
       </c>
       <c r="D149" t="n">
-        <v>3.19</v>
+        <v>2.55</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1622.7</v>
+        <v>5.9</v>
       </c>
       <c r="C150" t="n">
-        <v>1674.4</v>
+        <v>6.05</v>
       </c>
       <c r="D150" t="n">
-        <v>3.19</v>
+        <v>2.54</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AURUS</t>
+          <t>CENTRUM</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>4.4</v>
+        <v>19.7</v>
       </c>
       <c r="C151" t="n">
-        <v>4.54</v>
+        <v>20.2</v>
       </c>
       <c r="D151" t="n">
-        <v>3.18</v>
+        <v>2.54</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SPAL</t>
+          <t>AVANCE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>935.6</v>
+        <v>0.79</v>
       </c>
       <c r="C152" t="n">
-        <v>965.15</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D152" t="n">
-        <v>3.16</v>
+        <v>2.53</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SWISSMLTRY</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>13.95</v>
+        <v>5.55</v>
       </c>
       <c r="C153" t="n">
-        <v>14.39</v>
+        <v>5.69</v>
       </c>
       <c r="D153" t="n">
-        <v>3.15</v>
+        <v>2.52</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>INDOAMIN</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>18.39</v>
+        <v>143.31</v>
       </c>
       <c r="C154" t="n">
-        <v>18.97</v>
+        <v>146.9</v>
       </c>
       <c r="D154" t="n">
-        <v>3.15</v>
+        <v>2.51</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>NINSYS</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>804.65</v>
+        <v>24.8</v>
       </c>
       <c r="C155" t="n">
-        <v>830</v>
+        <v>25.42</v>
       </c>
       <c r="D155" t="n">
-        <v>3.15</v>
+        <v>2.5</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>PONNIERODE</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>208.4</v>
+        <v>368.4</v>
       </c>
       <c r="C156" t="n">
-        <v>214.95</v>
+        <v>377.5</v>
       </c>
       <c r="D156" t="n">
-        <v>3.14</v>
+        <v>2.47</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>1664.3</v>
+        <v>20.66</v>
       </c>
       <c r="C157" t="n">
-        <v>1716.3</v>
+        <v>21.17</v>
       </c>
       <c r="D157" t="n">
-        <v>3.12</v>
+        <v>2.47</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>NRAIL</t>
+          <t>MURUDCERA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>659.5</v>
+        <v>28.01</v>
       </c>
       <c r="C158" t="n">
-        <v>680</v>
+        <v>28.7</v>
       </c>
       <c r="D158" t="n">
-        <v>3.11</v>
+        <v>2.46</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>DOLATALGO</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>574.15</v>
+        <v>62.4</v>
       </c>
       <c r="C159" t="n">
-        <v>592</v>
+        <v>63.93</v>
       </c>
       <c r="D159" t="n">
-        <v>3.11</v>
+        <v>2.45</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>14.52</v>
+        <v>10.64</v>
       </c>
       <c r="C160" t="n">
-        <v>14.97</v>
+        <v>10.9</v>
       </c>
       <c r="D160" t="n">
-        <v>3.1</v>
+        <v>2.44</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>324.95</v>
+        <v>20.49</v>
       </c>
       <c r="C161" t="n">
-        <v>335</v>
+        <v>20.99</v>
       </c>
       <c r="D161" t="n">
-        <v>3.09</v>
+        <v>2.44</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>BHADORA</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>147.25</v>
+        <v>43.83</v>
       </c>
       <c r="C162" t="n">
-        <v>151.8</v>
+        <v>44.9</v>
       </c>
       <c r="D162" t="n">
-        <v>3.09</v>
+        <v>2.44</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>DWARKESH</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>6.5</v>
+        <v>44.08</v>
       </c>
       <c r="C163" t="n">
-        <v>6.7</v>
+        <v>45.15</v>
       </c>
       <c r="D163" t="n">
-        <v>3.08</v>
+        <v>2.43</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>OSWALAGRO</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>3.9</v>
+        <v>32.98</v>
       </c>
       <c r="C164" t="n">
-        <v>4.02</v>
+        <v>33.78</v>
       </c>
       <c r="D164" t="n">
-        <v>3.08</v>
+        <v>2.43</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>IVC</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>7.81</v>
+        <v>0.83</v>
       </c>
       <c r="C165" t="n">
-        <v>8.050000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="D165" t="n">
-        <v>3.07</v>
+        <v>2.41</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>44.34</v>
+        <v>4.15</v>
       </c>
       <c r="C166" t="n">
-        <v>45.7</v>
+        <v>4.25</v>
       </c>
       <c r="D166" t="n">
-        <v>3.07</v>
+        <v>2.41</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>EASTWEST</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>2.29</v>
+        <v>0.42</v>
       </c>
       <c r="C167" t="n">
-        <v>2.36</v>
+        <v>0.43</v>
       </c>
       <c r="D167" t="n">
-        <v>3.06</v>
+        <v>2.38</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MANALIPETC</t>
+          <t>WANBURY</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>78.15000000000001</v>
+        <v>190.46</v>
       </c>
       <c r="C168" t="n">
-        <v>80.53</v>
+        <v>194.99</v>
       </c>
       <c r="D168" t="n">
-        <v>3.05</v>
+        <v>2.38</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>AMJLAND</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>111.53</v>
+        <v>37.14</v>
       </c>
       <c r="C169" t="n">
-        <v>114.92</v>
+        <v>38.02</v>
       </c>
       <c r="D169" t="n">
-        <v>3.04</v>
+        <v>2.37</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MVGJL</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>206.69</v>
+        <v>197.79</v>
       </c>
       <c r="C170" t="n">
-        <v>212.94</v>
+        <v>202.45</v>
       </c>
       <c r="D170" t="n">
-        <v>3.02</v>
+        <v>2.36</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>SHANTIINOR</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>125.08</v>
+        <v>168.05</v>
       </c>
       <c r="C171" t="n">
-        <v>128.85</v>
+        <v>172</v>
       </c>
       <c r="D171" t="n">
-        <v>3.01</v>
+        <v>2.35</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>EUROBOND</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>148.29</v>
+        <v>14.16</v>
       </c>
       <c r="C172" t="n">
-        <v>152.75</v>
+        <v>14.49</v>
       </c>
       <c r="D172" t="n">
-        <v>3.01</v>
+        <v>2.33</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SCML</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>83.5</v>
+        <v>0.43</v>
       </c>
       <c r="C173" t="n">
-        <v>86</v>
+        <v>0.44</v>
       </c>
       <c r="D173" t="n">
-        <v>2.99</v>
+        <v>2.33</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>ARROWGREEN</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>679.5</v>
+        <v>858.55</v>
       </c>
       <c r="C174" t="n">
-        <v>699.8</v>
+        <v>878.5</v>
       </c>
       <c r="D174" t="n">
-        <v>2.99</v>
+        <v>2.32</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>AKASH</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>24.95</v>
+        <v>547.2</v>
       </c>
       <c r="C175" t="n">
-        <v>25.69</v>
+        <v>559.9</v>
       </c>
       <c r="D175" t="n">
-        <v>2.97</v>
+        <v>2.32</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SUPREME</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>31.08</v>
+        <v>3989.5</v>
       </c>
       <c r="C176" t="n">
-        <v>32</v>
+        <v>4082.1</v>
       </c>
       <c r="D176" t="n">
-        <v>2.96</v>
+        <v>2.32</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>51.38</v>
+        <v>515.1</v>
       </c>
       <c r="C177" t="n">
-        <v>52.9</v>
+        <v>526.95</v>
       </c>
       <c r="D177" t="n">
-        <v>2.96</v>
+        <v>2.3</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>AMANTA</t>
+          <t>HILINFRA</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>190.4</v>
+        <v>43.71</v>
       </c>
       <c r="C178" t="n">
-        <v>196</v>
+        <v>44.7</v>
       </c>
       <c r="D178" t="n">
-        <v>2.94</v>
+        <v>2.26</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>RAMBHAJO</t>
+          <t>KRISHANA</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>288.75</v>
+        <v>185.83</v>
       </c>
       <c r="C179" t="n">
-        <v>297.2</v>
+        <v>190</v>
       </c>
       <c r="D179" t="n">
-        <v>2.93</v>
+        <v>2.24</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>BVCL</t>
+          <t>JAIBALAJI</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>41.39</v>
+        <v>61.12</v>
       </c>
       <c r="C180" t="n">
-        <v>42.6</v>
+        <v>62.49</v>
       </c>
       <c r="D180" t="n">
-        <v>2.92</v>
+        <v>2.24</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>CYBERTECH</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>135.95</v>
+        <v>26.3</v>
       </c>
       <c r="C181" t="n">
-        <v>139.9</v>
+        <v>26.89</v>
       </c>
       <c r="D181" t="n">
-        <v>2.91</v>
+        <v>2.24</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ENKEIWHEL</t>
+          <t>GLOTTIS</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>392.6</v>
+        <v>56.72</v>
       </c>
       <c r="C182" t="n">
-        <v>404</v>
+        <v>57.99</v>
       </c>
       <c r="D182" t="n">
-        <v>2.9</v>
+        <v>2.24</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>KALYANIFRG</t>
+          <t>AKASH</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>944.75</v>
+        <v>24.64</v>
       </c>
       <c r="C183" t="n">
-        <v>972</v>
+        <v>25.19</v>
       </c>
       <c r="D183" t="n">
-        <v>2.88</v>
+        <v>2.23</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>PRANAV</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>97.20999999999999</v>
+        <v>46.47</v>
       </c>
       <c r="C184" t="n">
-        <v>100</v>
+        <v>47.5</v>
       </c>
       <c r="D184" t="n">
-        <v>2.87</v>
+        <v>2.22</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>30.04</v>
+        <v>1700.4</v>
       </c>
       <c r="C185" t="n">
-        <v>30.9</v>
+        <v>1738.1</v>
       </c>
       <c r="D185" t="n">
-        <v>2.86</v>
+        <v>2.22</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>ONIXSOLAR</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1.05</v>
+        <v>334.6</v>
       </c>
       <c r="C186" t="n">
-        <v>1.08</v>
+        <v>342</v>
       </c>
       <c r="D186" t="n">
-        <v>2.86</v>
+        <v>2.21</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>215.81</v>
+        <v>2206.6</v>
       </c>
       <c r="C187" t="n">
-        <v>221.95</v>
+        <v>2254.9</v>
       </c>
       <c r="D187" t="n">
-        <v>2.85</v>
+        <v>2.19</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>BPLPHARMA</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>1720.4</v>
+        <v>37.57</v>
       </c>
       <c r="C188" t="n">
-        <v>1769.2</v>
+        <v>38.39</v>
       </c>
       <c r="D188" t="n">
-        <v>2.84</v>
+        <v>2.18</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KCK</t>
+          <t>SUDEEPPHRM</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>14.1</v>
+        <v>1173.4</v>
       </c>
       <c r="C189" t="n">
-        <v>14.5</v>
+        <v>1199</v>
       </c>
       <c r="D189" t="n">
-        <v>2.84</v>
+        <v>2.18</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>INTLCONV</t>
+          <t>MANCREDIT</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>80.03</v>
+        <v>221.1</v>
       </c>
       <c r="C190" t="n">
-        <v>82.3</v>
+        <v>225.9</v>
       </c>
       <c r="D190" t="n">
-        <v>2.84</v>
+        <v>2.17</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>IWARE</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>388</v>
+        <v>641.6</v>
       </c>
       <c r="C191" t="n">
-        <v>398.95</v>
+        <v>655.45</v>
       </c>
       <c r="D191" t="n">
-        <v>2.82</v>
+        <v>2.16</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PRIMECAB</t>
+          <t>CORDELIA</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>206.25</v>
+        <v>100.83</v>
       </c>
       <c r="C192" t="n">
-        <v>212</v>
+        <v>103</v>
       </c>
       <c r="D192" t="n">
-        <v>2.79</v>
+        <v>2.15</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>FEDDERSHOL</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>63.63</v>
+        <v>204.89</v>
       </c>
       <c r="C193" t="n">
-        <v>65.40000000000001</v>
+        <v>209.28</v>
       </c>
       <c r="D193" t="n">
-        <v>2.78</v>
+        <v>2.14</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>BSL</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>118.2</v>
+        <v>0.47</v>
       </c>
       <c r="C194" t="n">
-        <v>121.49</v>
+        <v>0.48</v>
       </c>
       <c r="D194" t="n">
-        <v>2.78</v>
+        <v>2.13</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>URBAN</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>3.24</v>
+        <v>120.25</v>
       </c>
       <c r="C195" t="n">
-        <v>3.33</v>
+        <v>122.8</v>
       </c>
       <c r="D195" t="n">
-        <v>2.78</v>
+        <v>2.12</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1.08</v>
+        <v>1.89</v>
       </c>
       <c r="C196" t="n">
-        <v>1.11</v>
+        <v>1.93</v>
       </c>
       <c r="D196" t="n">
-        <v>2.78</v>
+        <v>2.12</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>INVPRECQ</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>1595.2</v>
+        <v>28.26</v>
       </c>
       <c r="C197" t="n">
-        <v>1639</v>
+        <v>28.86</v>
       </c>
       <c r="D197" t="n">
-        <v>2.75</v>
+        <v>2.12</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SUNSHIEL</t>
+          <t>METROPOLIS</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>1059</v>
+        <v>553.6</v>
       </c>
       <c r="C198" t="n">
-        <v>1088</v>
+        <v>565.35</v>
       </c>
       <c r="D198" t="n">
-        <v>2.74</v>
+        <v>2.12</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>BSOFT</t>
+          <t>VISHWARAJ</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>269.75</v>
+        <v>5.23</v>
       </c>
       <c r="C199" t="n">
-        <v>277.15</v>
+        <v>5.34</v>
       </c>
       <c r="D199" t="n">
-        <v>2.74</v>
+        <v>2.1</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>SCHAND</t>
+          <t>MODIS</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>143.57</v>
+        <v>372.25</v>
       </c>
       <c r="C200" t="n">
-        <v>147.5</v>
+        <v>380</v>
       </c>
       <c r="D200" t="n">
-        <v>2.74</v>
+        <v>2.08</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>776.7</v>
+        <v>1.94</v>
       </c>
       <c r="C201" t="n">
-        <v>797.9</v>
+        <v>1.98</v>
       </c>
       <c r="D201" t="n">
-        <v>2.73</v>
+        <v>2.06</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-07 10:35 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SURANI</t>
+          <t>PARTY-RE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>120.05</v>
+        <v>0.3</v>
       </c>
       <c r="C2" t="n">
-        <v>144.05</v>
+        <v>0.35</v>
       </c>
       <c r="D2" t="n">
-        <v>19.99</v>
+        <v>16.67</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>VALUE360</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61.59</v>
+        <v>61.55</v>
       </c>
       <c r="C3" t="n">
         <v>68</v>
       </c>
       <c r="D3" t="n">
-        <v>10.41</v>
+        <v>10.48</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HBESD</t>
+          <t>SURANI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>78.13</v>
+        <v>144.05</v>
       </c>
       <c r="C4" t="n">
-        <v>86</v>
+        <v>158.45</v>
       </c>
       <c r="D4" t="n">
-        <v>10.07</v>
+        <v>10</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>KANOHAR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22.1</v>
+        <v>942.5</v>
       </c>
       <c r="C5" t="n">
-        <v>24</v>
+        <v>1030</v>
       </c>
       <c r="D5" t="n">
-        <v>8.6</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SHKSIL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2580</v>
+        <v>30.45</v>
       </c>
       <c r="C6" t="n">
-        <v>2800</v>
+        <v>32.9</v>
       </c>
       <c r="D6" t="n">
-        <v>8.529999999999999</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PRECOT</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>605.1</v>
+        <v>17.41</v>
       </c>
       <c r="C7" t="n">
-        <v>653</v>
+        <v>18.8</v>
       </c>
       <c r="D7" t="n">
-        <v>7.92</v>
+        <v>7.98</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LAGNAM</t>
+          <t>KDGREEN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>71.09999999999999</v>
+        <v>49.19</v>
       </c>
       <c r="C8" t="n">
-        <v>76.7</v>
+        <v>52.99</v>
       </c>
       <c r="D8" t="n">
-        <v>7.88</v>
+        <v>7.73</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DPWIRES</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>196.78</v>
+        <v>242.14</v>
       </c>
       <c r="C9" t="n">
-        <v>212.23</v>
+        <v>260</v>
       </c>
       <c r="D9" t="n">
-        <v>7.85</v>
+        <v>7.38</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1201</v>
+        <v>0.14</v>
       </c>
       <c r="C10" t="n">
-        <v>1294</v>
+        <v>0.15</v>
       </c>
       <c r="D10" t="n">
-        <v>7.74</v>
+        <v>7.14</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>PRUDMOULI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.13</v>
+        <v>13.81</v>
       </c>
       <c r="C11" t="n">
-        <v>0.14</v>
+        <v>14.77</v>
       </c>
       <c r="D11" t="n">
-        <v>7.69</v>
+        <v>6.95</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>37.16</v>
+        <v>213.69</v>
       </c>
       <c r="C12" t="n">
-        <v>39.87</v>
+        <v>228</v>
       </c>
       <c r="D12" t="n">
-        <v>7.29</v>
+        <v>6.7</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>STEAMHOUSE</t>
+          <t>RPSGVENT</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>107.66</v>
+        <v>833.1</v>
       </c>
       <c r="C13" t="n">
-        <v>115</v>
+        <v>887</v>
       </c>
       <c r="D13" t="n">
-        <v>6.82</v>
+        <v>6.47</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BALKRISHNA</t>
+          <t>MYMUDRA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16</v>
+        <v>82.7</v>
       </c>
       <c r="C14" t="n">
-        <v>16.95</v>
+        <v>87.95</v>
       </c>
       <c r="D14" t="n">
-        <v>5.94</v>
+        <v>6.35</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8.84</v>
+        <v>8.09</v>
       </c>
       <c r="C15" t="n">
-        <v>9.35</v>
+        <v>8.6</v>
       </c>
       <c r="D15" t="n">
-        <v>5.77</v>
+        <v>6.3</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TOLINS</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>85.12</v>
+        <v>5.25</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>5.58</v>
       </c>
       <c r="D16" t="n">
-        <v>5.73</v>
+        <v>6.29</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AVANA</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>139.25</v>
+        <v>5.21</v>
       </c>
       <c r="C17" t="n">
-        <v>146.9</v>
+        <v>5.53</v>
       </c>
       <c r="D17" t="n">
-        <v>5.49</v>
+        <v>6.14</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>UTKARSHBNK</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.19</v>
+        <v>13.52</v>
       </c>
       <c r="C18" t="n">
-        <v>0.2</v>
+        <v>14.3</v>
       </c>
       <c r="D18" t="n">
-        <v>5.26</v>
+        <v>5.77</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>SHANTIINOR</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>8</v>
+        <v>201.65</v>
       </c>
       <c r="C19" t="n">
-        <v>8.4</v>
+        <v>213.1</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>5.68</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>KEYFINSERV</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>232.95</v>
+        <v>241.53</v>
       </c>
       <c r="C20" t="n">
-        <v>244.59</v>
+        <v>254.95</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>5.56</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KORE</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>191</v>
+        <v>153.5</v>
       </c>
       <c r="C21" t="n">
-        <v>200.55</v>
+        <v>162</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>5.54</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>NKIND</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1253.7</v>
+        <v>57.06</v>
       </c>
       <c r="C22" t="n">
-        <v>1316.35</v>
+        <v>60</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>5.15</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>QUINTEGRA</t>
+          <t>PRADPME</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.4</v>
+        <v>544.25</v>
       </c>
       <c r="C23" t="n">
-        <v>1.47</v>
+        <v>572.2</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>5.14</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2410.9</v>
+        <v>1.78</v>
       </c>
       <c r="C24" t="n">
-        <v>2531.4</v>
+        <v>1.87</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>5.06</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>250.27</v>
+        <v>7.4</v>
       </c>
       <c r="C25" t="n">
-        <v>262.78</v>
+        <v>7.77</v>
       </c>
       <c r="D25" t="n">
         <v>5</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>177.26</v>
+        <v>244.11</v>
       </c>
       <c r="C26" t="n">
-        <v>186.12</v>
+        <v>256.31</v>
       </c>
       <c r="D26" t="n">
         <v>5</v>
@@ -1011,14 +1011,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>472.25</v>
+        <v>186.12</v>
       </c>
       <c r="C27" t="n">
-        <v>495.85</v>
+        <v>195.42</v>
       </c>
       <c r="D27" t="n">
         <v>5</v>
@@ -1033,14 +1033,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>ESDS</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>48.8</v>
+        <v>1294.3</v>
       </c>
       <c r="C28" t="n">
-        <v>51.24</v>
+        <v>1359</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>37.67</v>
+        <v>262.78</v>
       </c>
       <c r="C29" t="n">
-        <v>39.55</v>
+        <v>275.91</v>
       </c>
       <c r="D29" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>CEDAAR</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5.21</v>
+        <v>11</v>
       </c>
       <c r="C30" t="n">
-        <v>5.47</v>
+        <v>11.55</v>
       </c>
       <c r="D30" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>541.95</v>
+        <v>1316.35</v>
       </c>
       <c r="C31" t="n">
-        <v>569</v>
+        <v>1382.15</v>
       </c>
       <c r="D31" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BMISL</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>115.5</v>
+        <v>51.24</v>
       </c>
       <c r="C32" t="n">
-        <v>121.25</v>
+        <v>53.8</v>
       </c>
       <c r="D32" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>16.51</v>
+        <v>2531.4</v>
       </c>
       <c r="C33" t="n">
-        <v>17.33</v>
+        <v>2657.9</v>
       </c>
       <c r="D33" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>SPECTRAA</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.61</v>
+        <v>259.6</v>
       </c>
       <c r="C34" t="n">
-        <v>1.69</v>
+        <v>272.55</v>
       </c>
       <c r="D34" t="n">
-        <v>4.97</v>
+        <v>4.99</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AVATAR</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>159</v>
+        <v>11.43</v>
       </c>
       <c r="C35" t="n">
-        <v>166.9</v>
+        <v>12</v>
       </c>
       <c r="D35" t="n">
-        <v>4.97</v>
+        <v>4.99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>JAIBALAJI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>10.89</v>
+        <v>64.17</v>
       </c>
       <c r="C36" t="n">
-        <v>11.43</v>
+        <v>67.37</v>
       </c>
       <c r="D36" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>16.33</v>
+        <v>50.34</v>
       </c>
       <c r="C37" t="n">
-        <v>17.14</v>
+        <v>52.85</v>
       </c>
       <c r="D37" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABAN</t>
+          <t>BMISL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>16.12</v>
+        <v>121.25</v>
       </c>
       <c r="C38" t="n">
-        <v>16.92</v>
+        <v>127.3</v>
       </c>
       <c r="D38" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>AVATAR</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>77.59999999999999</v>
+        <v>166.95</v>
       </c>
       <c r="C39" t="n">
-        <v>81.45</v>
+        <v>175.25</v>
       </c>
       <c r="D39" t="n">
-        <v>4.96</v>
+        <v>4.97</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BURNPUR</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>13.18</v>
+        <v>61.4</v>
       </c>
       <c r="C40" t="n">
-        <v>13.83</v>
+        <v>64.45</v>
       </c>
       <c r="D40" t="n">
-        <v>4.93</v>
+        <v>4.97</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>8.17</v>
+        <v>17.14</v>
       </c>
       <c r="C41" t="n">
-        <v>8.57</v>
+        <v>17.99</v>
       </c>
       <c r="D41" t="n">
-        <v>4.9</v>
+        <v>4.96</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BIOPOL</t>
+          <t>TECHNVISN</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>49.3</v>
+        <v>4012.9</v>
       </c>
       <c r="C42" t="n">
-        <v>51.7</v>
+        <v>4211.9</v>
       </c>
       <c r="D42" t="n">
-        <v>4.87</v>
+        <v>4.96</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>ABAN</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5.99</v>
+        <v>16.92</v>
       </c>
       <c r="C43" t="n">
-        <v>6.28</v>
+        <v>17.76</v>
       </c>
       <c r="D43" t="n">
-        <v>4.84</v>
+        <v>4.96</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>AUSOMENT</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>4.97</v>
+        <v>137.48</v>
       </c>
       <c r="C44" t="n">
-        <v>5.21</v>
+        <v>144.3</v>
       </c>
       <c r="D44" t="n">
-        <v>4.83</v>
+        <v>4.96</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>RHETAN</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>56.24</v>
+        <v>16.59</v>
       </c>
       <c r="C45" t="n">
-        <v>58.95</v>
+        <v>17.41</v>
       </c>
       <c r="D45" t="n">
-        <v>4.82</v>
+        <v>4.94</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ABH</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>43.5</v>
+        <v>6.28</v>
       </c>
       <c r="C46" t="n">
-        <v>45.55</v>
+        <v>6.59</v>
       </c>
       <c r="D46" t="n">
-        <v>4.71</v>
+        <v>4.94</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AKSHARCHEM</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>365.3</v>
+        <v>1.42</v>
       </c>
       <c r="C47" t="n">
-        <v>382.5</v>
+        <v>1.49</v>
       </c>
       <c r="D47" t="n">
-        <v>4.71</v>
+        <v>4.93</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>ARCIIL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>21.06</v>
+        <v>32.65</v>
       </c>
       <c r="C48" t="n">
-        <v>22.05</v>
+        <v>34.25</v>
       </c>
       <c r="D48" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>SWASTIKAIN</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>536.8</v>
+        <v>200.13</v>
       </c>
       <c r="C49" t="n">
-        <v>562</v>
+        <v>209.8</v>
       </c>
       <c r="D49" t="n">
-        <v>4.69</v>
+        <v>4.83</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>101.25</v>
+        <v>5.21</v>
       </c>
       <c r="C50" t="n">
-        <v>106</v>
+        <v>5.46</v>
       </c>
       <c r="D50" t="n">
-        <v>4.69</v>
+        <v>4.8</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>213.99</v>
+        <v>160.33</v>
       </c>
       <c r="C51" t="n">
-        <v>224</v>
+        <v>168</v>
       </c>
       <c r="D51" t="n">
-        <v>4.68</v>
+        <v>4.78</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>50.64</v>
+        <v>0.42</v>
       </c>
       <c r="C52" t="n">
-        <v>53</v>
+        <v>0.44</v>
       </c>
       <c r="D52" t="n">
-        <v>4.66</v>
+        <v>4.76</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KEYFINSERV</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>237.01</v>
+        <v>145.58</v>
       </c>
       <c r="C53" t="n">
-        <v>247.9</v>
+        <v>152.5</v>
       </c>
       <c r="D53" t="n">
-        <v>4.59</v>
+        <v>4.75</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>12.49</v>
+        <v>235.45</v>
       </c>
       <c r="C54" t="n">
-        <v>13.06</v>
+        <v>246.6</v>
       </c>
       <c r="D54" t="n">
-        <v>4.56</v>
+        <v>4.74</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>SOMATEX</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>75.5</v>
+        <v>79.09</v>
       </c>
       <c r="C55" t="n">
-        <v>78.92</v>
+        <v>82.8</v>
       </c>
       <c r="D55" t="n">
-        <v>4.53</v>
+        <v>4.69</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>UNIENTER</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>86.17</v>
+        <v>1.5</v>
       </c>
       <c r="C56" t="n">
-        <v>90</v>
+        <v>1.57</v>
       </c>
       <c r="D56" t="n">
-        <v>4.44</v>
+        <v>4.67</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MUTHOOTCAP</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>219.33</v>
+        <v>3.64</v>
       </c>
       <c r="C57" t="n">
-        <v>229.05</v>
+        <v>3.81</v>
       </c>
       <c r="D57" t="n">
-        <v>4.43</v>
+        <v>4.67</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>CRAVATEX</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>160.27</v>
+        <v>374.6</v>
       </c>
       <c r="C58" t="n">
-        <v>167.35</v>
+        <v>391.95</v>
       </c>
       <c r="D58" t="n">
-        <v>4.42</v>
+        <v>4.63</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>13.79</v>
+        <v>38.78</v>
       </c>
       <c r="C59" t="n">
-        <v>14.4</v>
+        <v>40.57</v>
       </c>
       <c r="D59" t="n">
-        <v>4.42</v>
+        <v>4.62</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1.36</v>
+        <v>47.92</v>
       </c>
       <c r="C60" t="n">
-        <v>1.42</v>
+        <v>50.04</v>
       </c>
       <c r="D60" t="n">
-        <v>4.41</v>
+        <v>4.42</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>KILITCH</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>233.74</v>
+        <v>45</v>
       </c>
       <c r="C61" t="n">
-        <v>244</v>
+        <v>46.99</v>
       </c>
       <c r="D61" t="n">
-        <v>4.39</v>
+        <v>4.42</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>4.78</v>
+        <v>4.12</v>
       </c>
       <c r="C62" t="n">
-        <v>4.99</v>
+        <v>4.3</v>
       </c>
       <c r="D62" t="n">
-        <v>4.39</v>
+        <v>4.37</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,14 +1803,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>RKDL</t>
+          <t>AKSHOPTFBR</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>17.05</v>
+        <v>7.37</v>
       </c>
       <c r="C63" t="n">
-        <v>17.79</v>
+        <v>7.69</v>
       </c>
       <c r="D63" t="n">
         <v>4.34</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ALPINETEX</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>45.82</v>
+        <v>29.72</v>
       </c>
       <c r="C64" t="n">
-        <v>47.8</v>
+        <v>30.99</v>
       </c>
       <c r="D64" t="n">
-        <v>4.32</v>
+        <v>4.27</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>MIDWESTLTD</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>114.5</v>
+        <v>1006.2</v>
       </c>
       <c r="C65" t="n">
-        <v>119.4</v>
+        <v>1049</v>
       </c>
       <c r="D65" t="n">
-        <v>4.28</v>
+        <v>4.25</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>VLINFRA</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>108.95</v>
+        <v>24.75</v>
       </c>
       <c r="C66" t="n">
-        <v>113.6</v>
+        <v>25.8</v>
       </c>
       <c r="D66" t="n">
-        <v>4.27</v>
+        <v>4.24</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1.43</v>
+        <v>20.98</v>
       </c>
       <c r="C67" t="n">
-        <v>1.49</v>
+        <v>21.84</v>
       </c>
       <c r="D67" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>ABH</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>224.7</v>
+        <v>45.65</v>
       </c>
       <c r="C68" t="n">
-        <v>233.9</v>
+        <v>47.5</v>
       </c>
       <c r="D68" t="n">
-        <v>4.09</v>
+        <v>4.05</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>143.02</v>
+        <v>0.25</v>
       </c>
       <c r="C69" t="n">
-        <v>148.8</v>
+        <v>0.26</v>
       </c>
       <c r="D69" t="n">
-        <v>4.04</v>
+        <v>4</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>29.79</v>
+        <v>16.33</v>
       </c>
       <c r="C70" t="n">
-        <v>30.99</v>
+        <v>16.98</v>
       </c>
       <c r="D70" t="n">
-        <v>4.03</v>
+        <v>3.98</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HITECH</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>70.05</v>
+        <v>85.55</v>
       </c>
       <c r="C71" t="n">
-        <v>72.84999999999999</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="D71" t="n">
-        <v>4</v>
+        <v>3.92</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>HPIL</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>110.64</v>
+        <v>59.66</v>
       </c>
       <c r="C72" t="n">
-        <v>115</v>
+        <v>61.98</v>
       </c>
       <c r="D72" t="n">
-        <v>3.94</v>
+        <v>3.89</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CENTEXT-RE</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2.79</v>
+        <v>18.64</v>
       </c>
       <c r="C73" t="n">
-        <v>2.9</v>
+        <v>19.36</v>
       </c>
       <c r="D73" t="n">
-        <v>3.94</v>
+        <v>3.86</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>4.85</v>
+        <v>495.85</v>
       </c>
       <c r="C74" t="n">
-        <v>5.04</v>
+        <v>515</v>
       </c>
       <c r="D74" t="n">
-        <v>3.92</v>
+        <v>3.86</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>MANIKA</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>15.58</v>
+        <v>51.52</v>
       </c>
       <c r="C75" t="n">
-        <v>16.19</v>
+        <v>53.5</v>
       </c>
       <c r="D75" t="n">
-        <v>3.92</v>
+        <v>3.84</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>126.05</v>
+        <v>206.65</v>
       </c>
       <c r="C76" t="n">
-        <v>130.95</v>
+        <v>214.55</v>
       </c>
       <c r="D76" t="n">
-        <v>3.89</v>
+        <v>3.82</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>54.24</v>
+        <v>16.6</v>
       </c>
       <c r="C77" t="n">
-        <v>56.34</v>
+        <v>17.23</v>
       </c>
       <c r="D77" t="n">
-        <v>3.87</v>
+        <v>3.8</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>DIGIKORE</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>221.97</v>
+        <v>36.15</v>
       </c>
       <c r="C78" t="n">
-        <v>230.33</v>
+        <v>37.5</v>
       </c>
       <c r="D78" t="n">
-        <v>3.77</v>
+        <v>3.73</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>VTMLTD</t>
+          <t>SUPTANERY</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>38.27</v>
+        <v>8.07</v>
       </c>
       <c r="C79" t="n">
-        <v>39.7</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="D79" t="n">
-        <v>3.74</v>
+        <v>3.72</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>NAGREEKCAP</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>197.18</v>
+        <v>27.25</v>
       </c>
       <c r="C80" t="n">
-        <v>204.49</v>
+        <v>28.25</v>
       </c>
       <c r="D80" t="n">
-        <v>3.71</v>
+        <v>3.67</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>4.41</v>
+        <v>30.27</v>
       </c>
       <c r="C81" t="n">
-        <v>4.57</v>
+        <v>31.35</v>
       </c>
       <c r="D81" t="n">
-        <v>3.63</v>
+        <v>3.57</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CYBERMEDIA</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>17.69</v>
+        <v>24.24</v>
       </c>
       <c r="C82" t="n">
-        <v>18.33</v>
+        <v>25.1</v>
       </c>
       <c r="D82" t="n">
-        <v>3.62</v>
+        <v>3.55</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>34.12</v>
+        <v>6.52</v>
       </c>
       <c r="C83" t="n">
-        <v>35.35</v>
+        <v>6.75</v>
       </c>
       <c r="D83" t="n">
-        <v>3.6</v>
+        <v>3.53</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>AVADHSUGAR</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>840.35</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="C84" t="n">
-        <v>870.45</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D84" t="n">
-        <v>3.58</v>
+        <v>3.52</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>MANCREDIT</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.28</v>
+        <v>231.9</v>
       </c>
       <c r="C85" t="n">
-        <v>0.29</v>
+        <v>239.99</v>
       </c>
       <c r="D85" t="n">
-        <v>3.57</v>
+        <v>3.49</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GILLANDERS</t>
+          <t>NELCAST</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>115.73</v>
+        <v>124.48</v>
       </c>
       <c r="C86" t="n">
-        <v>119.8</v>
+        <v>128.77</v>
       </c>
       <c r="D86" t="n">
-        <v>3.52</v>
+        <v>3.45</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>RELIABLE</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>227.86</v>
+        <v>139.3</v>
       </c>
       <c r="C87" t="n">
-        <v>235.85</v>
+        <v>144</v>
       </c>
       <c r="D87" t="n">
-        <v>3.51</v>
+        <v>3.37</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>EBIX</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>16.91</v>
+        <v>15.46</v>
       </c>
       <c r="C88" t="n">
-        <v>17.5</v>
+        <v>15.98</v>
       </c>
       <c r="D88" t="n">
-        <v>3.49</v>
+        <v>3.36</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>UGARSUGAR</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>58.84</v>
+        <v>172.06</v>
       </c>
       <c r="C89" t="n">
-        <v>60.89</v>
+        <v>177.8</v>
       </c>
       <c r="D89" t="n">
-        <v>3.48</v>
+        <v>3.34</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1.46</v>
+        <v>25.05</v>
       </c>
       <c r="C90" t="n">
-        <v>1.51</v>
+        <v>25.88</v>
       </c>
       <c r="D90" t="n">
-        <v>3.42</v>
+        <v>3.31</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>WILLAMAGOR</t>
+          <t>MODIRUBBER</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>21.67</v>
+        <v>118.58</v>
       </c>
       <c r="C91" t="n">
-        <v>22.4</v>
+        <v>122.49</v>
       </c>
       <c r="D91" t="n">
-        <v>3.37</v>
+        <v>3.3</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>GENCON</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1001.25</v>
+        <v>37.78</v>
       </c>
       <c r="C92" t="n">
-        <v>1034.4</v>
+        <v>39</v>
       </c>
       <c r="D92" t="n">
-        <v>3.31</v>
+        <v>3.23</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>TRANSRAILL</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>462.75</v>
+        <v>207.59</v>
       </c>
       <c r="C93" t="n">
-        <v>478</v>
+        <v>214.3</v>
       </c>
       <c r="D93" t="n">
-        <v>3.3</v>
+        <v>3.23</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ELECTHERM</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>702.4</v>
+        <v>11.51</v>
       </c>
       <c r="C94" t="n">
-        <v>725.4</v>
+        <v>11.88</v>
       </c>
       <c r="D94" t="n">
-        <v>3.27</v>
+        <v>3.21</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>SIEL</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>15.98</v>
+        <v>31</v>
       </c>
       <c r="C95" t="n">
-        <v>16.5</v>
+        <v>31.99</v>
       </c>
       <c r="D95" t="n">
-        <v>3.25</v>
+        <v>3.19</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>22.76</v>
+        <v>10.76</v>
       </c>
       <c r="C96" t="n">
-        <v>23.5</v>
+        <v>11.1</v>
       </c>
       <c r="D96" t="n">
-        <v>3.25</v>
+        <v>3.16</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>GOKULAGRO</t>
+          <t>MARSONS</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>205.27</v>
+        <v>119.24</v>
       </c>
       <c r="C97" t="n">
-        <v>211.89</v>
+        <v>123</v>
       </c>
       <c r="D97" t="n">
-        <v>3.23</v>
+        <v>3.15</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ROXHITECH</t>
+          <t>PTCIL</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>62.45</v>
+        <v>23125</v>
       </c>
       <c r="C98" t="n">
-        <v>64.45</v>
+        <v>23850</v>
       </c>
       <c r="D98" t="n">
-        <v>3.2</v>
+        <v>3.14</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TRIVENI</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>237.22</v>
+        <v>47.08</v>
       </c>
       <c r="C99" t="n">
-        <v>244.8</v>
+        <v>48.54</v>
       </c>
       <c r="D99" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>BIOPOL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>11.58</v>
+        <v>51.75</v>
       </c>
       <c r="C100" t="n">
-        <v>11.95</v>
+        <v>53.35</v>
       </c>
       <c r="D100" t="n">
-        <v>3.2</v>
+        <v>3.09</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AMANTA</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>199.92</v>
+        <v>48.49</v>
       </c>
       <c r="C101" t="n">
-        <v>206.3</v>
+        <v>49.99</v>
       </c>
       <c r="D101" t="n">
-        <v>3.19</v>
+        <v>3.09</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SKYTECH</t>
+          <t>NUCLEUS</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>40.7</v>
+        <v>638.05</v>
       </c>
       <c r="C102" t="n">
-        <v>42</v>
+        <v>657.7</v>
       </c>
       <c r="D102" t="n">
-        <v>3.19</v>
+        <v>3.08</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>173</v>
+        <v>1.63</v>
       </c>
       <c r="C103" t="n">
-        <v>178.5</v>
+        <v>1.68</v>
       </c>
       <c r="D103" t="n">
-        <v>3.18</v>
+        <v>3.07</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>PARAGON</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>28.09</v>
+        <v>49.2</v>
       </c>
       <c r="C104" t="n">
-        <v>28.98</v>
+        <v>50.7</v>
       </c>
       <c r="D104" t="n">
-        <v>3.17</v>
+        <v>3.05</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ARCHIES</t>
+          <t>PVRINOX</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>12.35</v>
+        <v>1249.4</v>
       </c>
       <c r="C105" t="n">
-        <v>12.74</v>
+        <v>1287</v>
       </c>
       <c r="D105" t="n">
-        <v>3.16</v>
+        <v>3.01</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PVSL</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>91.08</v>
+        <v>41.86</v>
       </c>
       <c r="C106" t="n">
-        <v>93.95999999999999</v>
+        <v>43.12</v>
       </c>
       <c r="D106" t="n">
-        <v>3.16</v>
+        <v>3.01</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>6.05</v>
+        <v>2</v>
       </c>
       <c r="C107" t="n">
-        <v>6.24</v>
+        <v>2.06</v>
       </c>
       <c r="D107" t="n">
-        <v>3.14</v>
+        <v>3</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>NATHBIOGEN</t>
+          <t>RRIL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>134.29</v>
+        <v>16.18</v>
       </c>
       <c r="C108" t="n">
-        <v>138.5</v>
+        <v>16.66</v>
       </c>
       <c r="D108" t="n">
-        <v>3.14</v>
+        <v>2.97</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>MARALOVER</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>4.83</v>
+        <v>57.99</v>
       </c>
       <c r="C109" t="n">
-        <v>4.98</v>
+        <v>59.7</v>
       </c>
       <c r="D109" t="n">
-        <v>3.11</v>
+        <v>2.95</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>54.8</v>
+        <v>233.12</v>
       </c>
       <c r="C110" t="n">
-        <v>56.5</v>
+        <v>240</v>
       </c>
       <c r="D110" t="n">
-        <v>3.1</v>
+        <v>2.95</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>5.8</v>
+        <v>11.55</v>
       </c>
       <c r="C111" t="n">
-        <v>5.98</v>
+        <v>11.89</v>
       </c>
       <c r="D111" t="n">
-        <v>3.1</v>
+        <v>2.94</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>290.8</v>
+        <v>1.36</v>
       </c>
       <c r="C112" t="n">
-        <v>299.8</v>
+        <v>1.4</v>
       </c>
       <c r="D112" t="n">
-        <v>3.09</v>
+        <v>2.94</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>SHRADHA</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>36.97</v>
+        <v>29.83</v>
       </c>
       <c r="C113" t="n">
-        <v>38.1</v>
+        <v>30.7</v>
       </c>
       <c r="D113" t="n">
-        <v>3.06</v>
+        <v>2.92</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LANCER</t>
+          <t>LOVABLE</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>11.15</v>
+        <v>69</v>
       </c>
       <c r="C114" t="n">
-        <v>11.49</v>
+        <v>71</v>
       </c>
       <c r="D114" t="n">
-        <v>3.05</v>
+        <v>2.9</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1668.9</v>
+        <v>22.78</v>
       </c>
       <c r="C115" t="n">
-        <v>1719.8</v>
+        <v>23.44</v>
       </c>
       <c r="D115" t="n">
-        <v>3.05</v>
+        <v>2.9</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>RAJSREESUG</t>
+          <t>ASTEC</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>28.39</v>
+        <v>704.7</v>
       </c>
       <c r="C116" t="n">
-        <v>29.25</v>
+        <v>724.95</v>
       </c>
       <c r="D116" t="n">
-        <v>3.03</v>
+        <v>2.87</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>227.25</v>
+        <v>76.70999999999999</v>
       </c>
       <c r="C117" t="n">
-        <v>234</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D117" t="n">
-        <v>2.97</v>
+        <v>2.85</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>KAVDEFENCE</t>
+          <t>MHLXMIRU</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>81.48</v>
+        <v>171.12</v>
       </c>
       <c r="C118" t="n">
-        <v>83.90000000000001</v>
+        <v>176</v>
       </c>
       <c r="D118" t="n">
-        <v>2.97</v>
+        <v>2.85</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NTCIND</t>
+          <t>KHERIAAUTO</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>135.97</v>
+        <v>89.45</v>
       </c>
       <c r="C119" t="n">
-        <v>140</v>
+        <v>92</v>
       </c>
       <c r="D119" t="n">
-        <v>2.96</v>
+        <v>2.85</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DHAMPURSUG</t>
+          <t>GAUDIUMIVF</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>176.85</v>
+        <v>109.28</v>
       </c>
       <c r="C120" t="n">
-        <v>182</v>
+        <v>112.38</v>
       </c>
       <c r="D120" t="n">
-        <v>2.91</v>
+        <v>2.84</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>BANSWRAS</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>102.93</v>
+        <v>8.17</v>
       </c>
       <c r="C121" t="n">
-        <v>105.93</v>
+        <v>8.4</v>
       </c>
       <c r="D121" t="n">
-        <v>2.91</v>
+        <v>2.82</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>VISHAL</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.6899999999999999</v>
+        <v>17.5</v>
       </c>
       <c r="C122" t="n">
-        <v>0.71</v>
+        <v>17.99</v>
       </c>
       <c r="D122" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ALLCARGO</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>10.03</v>
+        <v>1.44</v>
       </c>
       <c r="C123" t="n">
-        <v>10.32</v>
+        <v>1.48</v>
       </c>
       <c r="D123" t="n">
-        <v>2.89</v>
+        <v>2.78</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>APRAMEYA</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>102</v>
+        <v>0.37</v>
       </c>
       <c r="C124" t="n">
-        <v>104.95</v>
+        <v>0.38</v>
       </c>
       <c r="D124" t="n">
-        <v>2.89</v>
+        <v>2.7</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RENUKA</t>
+          <t>APOLSINHOT</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>21.76</v>
+        <v>1174.7</v>
       </c>
       <c r="C125" t="n">
-        <v>22.38</v>
+        <v>1205.9</v>
       </c>
       <c r="D125" t="n">
-        <v>2.85</v>
+        <v>2.66</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ENIL</t>
+          <t>SUNSHIEL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>91.69</v>
+        <v>1047.4</v>
       </c>
       <c r="C126" t="n">
-        <v>94.3</v>
+        <v>1075</v>
       </c>
       <c r="D126" t="n">
-        <v>2.85</v>
+        <v>2.64</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>BPLPHARMA</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>15.46</v>
+        <v>1836.4</v>
       </c>
       <c r="C127" t="n">
-        <v>15.9</v>
+        <v>1884.9</v>
       </c>
       <c r="D127" t="n">
-        <v>2.85</v>
+        <v>2.64</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>BRNL</t>
+          <t>PAUSHAKLTD</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>16.13</v>
+        <v>704.3</v>
       </c>
       <c r="C128" t="n">
-        <v>16.59</v>
+        <v>722.85</v>
       </c>
       <c r="D128" t="n">
-        <v>2.85</v>
+        <v>2.63</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>7.05</v>
+        <v>2.68</v>
       </c>
       <c r="C129" t="n">
-        <v>7.25</v>
+        <v>2.75</v>
       </c>
       <c r="D129" t="n">
-        <v>2.84</v>
+        <v>2.61</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PRABHA</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>214.9</v>
+        <v>13.15</v>
       </c>
       <c r="C130" t="n">
-        <v>221</v>
+        <v>13.48</v>
       </c>
       <c r="D130" t="n">
-        <v>2.84</v>
+        <v>2.51</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>RAMANEWS</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>143.92</v>
+        <v>28.88</v>
       </c>
       <c r="C131" t="n">
-        <v>147.99</v>
+        <v>29.59</v>
       </c>
       <c r="D131" t="n">
-        <v>2.83</v>
+        <v>2.46</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TECHD</t>
+          <t>KOKUYOCMLN</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>552</v>
+        <v>74.56999999999999</v>
       </c>
       <c r="C132" t="n">
-        <v>567.5</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D132" t="n">
-        <v>2.81</v>
+        <v>2.45</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>27.11</v>
+        <v>131.63</v>
       </c>
       <c r="C133" t="n">
-        <v>27.87</v>
+        <v>134.84</v>
       </c>
       <c r="D133" t="n">
-        <v>2.8</v>
+        <v>2.44</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>GINNIFILA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>20.04</v>
+        <v>40.96</v>
       </c>
       <c r="C134" t="n">
-        <v>20.6</v>
+        <v>41.95</v>
       </c>
       <c r="D134" t="n">
-        <v>2.79</v>
+        <v>2.42</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SHUKRAPHAR</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>70.48999999999999</v>
+        <v>16.09</v>
       </c>
       <c r="C135" t="n">
-        <v>72.40000000000001</v>
+        <v>16.48</v>
       </c>
       <c r="D135" t="n">
-        <v>2.71</v>
+        <v>2.42</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>SHAHALLOYS</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>19.96</v>
+        <v>81.03</v>
       </c>
       <c r="C136" t="n">
-        <v>20.5</v>
+        <v>82.94</v>
       </c>
       <c r="D136" t="n">
-        <v>2.71</v>
+        <v>2.36</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>52.08</v>
+        <v>14.16</v>
       </c>
       <c r="C137" t="n">
-        <v>53.49</v>
+        <v>14.49</v>
       </c>
       <c r="D137" t="n">
-        <v>2.71</v>
+        <v>2.33</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>WATERBASE</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>45.57</v>
+        <v>12.92</v>
       </c>
       <c r="C138" t="n">
-        <v>46.79</v>
+        <v>13.22</v>
       </c>
       <c r="D138" t="n">
-        <v>2.68</v>
+        <v>2.32</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>9.32</v>
+        <v>27.37</v>
       </c>
       <c r="C139" t="n">
-        <v>9.57</v>
+        <v>28</v>
       </c>
       <c r="D139" t="n">
-        <v>2.68</v>
+        <v>2.3</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>VOEPL</t>
+          <t>HARIOMPIPE</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>506.1</v>
+        <v>336.5</v>
       </c>
       <c r="C140" t="n">
-        <v>519.65</v>
+        <v>344.25</v>
       </c>
       <c r="D140" t="n">
-        <v>2.68</v>
+        <v>2.3</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SHERA</t>
+          <t>JSWCEMENT</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>187</v>
+        <v>113.2</v>
       </c>
       <c r="C141" t="n">
-        <v>192</v>
+        <v>115.77</v>
       </c>
       <c r="D141" t="n">
-        <v>2.67</v>
+        <v>2.27</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>NRAIL</t>
+          <t>ARCIL</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>661.35</v>
+        <v>145.74</v>
       </c>
       <c r="C142" t="n">
-        <v>679</v>
+        <v>149</v>
       </c>
       <c r="D142" t="n">
-        <v>2.67</v>
+        <v>2.24</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>INVPRECQ</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>1612.1</v>
+        <v>96.36</v>
       </c>
       <c r="C143" t="n">
-        <v>1655</v>
+        <v>98.5</v>
       </c>
       <c r="D143" t="n">
-        <v>2.66</v>
+        <v>2.22</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>10.93</v>
+        <v>35.22</v>
       </c>
       <c r="C144" t="n">
-        <v>11.22</v>
+        <v>36</v>
       </c>
       <c r="D144" t="n">
-        <v>2.65</v>
+        <v>2.21</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>ATAM</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.38</v>
+        <v>54.2</v>
       </c>
       <c r="C145" t="n">
-        <v>0.39</v>
+        <v>55.4</v>
       </c>
       <c r="D145" t="n">
-        <v>2.63</v>
+        <v>2.21</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ANONDITA</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1031</v>
+        <v>69.91</v>
       </c>
       <c r="C146" t="n">
-        <v>1057.95</v>
+        <v>71.45</v>
       </c>
       <c r="D146" t="n">
-        <v>2.61</v>
+        <v>2.2</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ACEVECTOR</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>26.08</v>
+        <v>110.55</v>
       </c>
       <c r="C147" t="n">
-        <v>26.75</v>
+        <v>112.97</v>
       </c>
       <c r="D147" t="n">
-        <v>2.57</v>
+        <v>2.19</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GAUDIUMIVF</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>103.25</v>
+        <v>36.15</v>
       </c>
       <c r="C148" t="n">
-        <v>105.89</v>
+        <v>36.94</v>
       </c>
       <c r="D148" t="n">
-        <v>2.56</v>
+        <v>2.19</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>ALOKINDS</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>19.99</v>
+        <v>7.83</v>
       </c>
       <c r="C149" t="n">
-        <v>20.5</v>
+        <v>8</v>
       </c>
       <c r="D149" t="n">
-        <v>2.55</v>
+        <v>2.17</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>5.9</v>
+        <v>54.82</v>
       </c>
       <c r="C150" t="n">
-        <v>6.05</v>
+        <v>56</v>
       </c>
       <c r="D150" t="n">
-        <v>2.54</v>
+        <v>2.15</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CENTRUM</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>19.7</v>
+        <v>92.86</v>
       </c>
       <c r="C151" t="n">
-        <v>20.2</v>
+        <v>94.84</v>
       </c>
       <c r="D151" t="n">
-        <v>2.54</v>
+        <v>2.13</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>AVANCE</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>0.79</v>
+        <v>51.88</v>
       </c>
       <c r="C152" t="n">
-        <v>0.8100000000000001</v>
+        <v>52.98</v>
       </c>
       <c r="D152" t="n">
-        <v>2.53</v>
+        <v>2.12</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>CORDSCABLE</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>5.55</v>
+        <v>314.35</v>
       </c>
       <c r="C153" t="n">
-        <v>5.69</v>
+        <v>321</v>
       </c>
       <c r="D153" t="n">
-        <v>2.52</v>
+        <v>2.12</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>INDOAMIN</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>143.31</v>
+        <v>1013.05</v>
       </c>
       <c r="C154" t="n">
-        <v>146.9</v>
+        <v>1034.4</v>
       </c>
       <c r="D154" t="n">
-        <v>2.51</v>
+        <v>2.11</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>DRONE</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>24.8</v>
+        <v>33.3</v>
       </c>
       <c r="C155" t="n">
-        <v>25.42</v>
+        <v>34</v>
       </c>
       <c r="D155" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PONNIERODE</t>
+          <t>AURUS</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>368.4</v>
+        <v>4.29</v>
       </c>
       <c r="C156" t="n">
-        <v>377.5</v>
+        <v>4.38</v>
       </c>
       <c r="D156" t="n">
-        <v>2.47</v>
+        <v>2.1</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>20.66</v>
+        <v>30.95</v>
       </c>
       <c r="C157" t="n">
-        <v>21.17</v>
+        <v>31.6</v>
       </c>
       <c r="D157" t="n">
-        <v>2.47</v>
+        <v>2.1</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MURUDCERA</t>
+          <t>BAJAJINDEF</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>28.01</v>
+        <v>207.21</v>
       </c>
       <c r="C158" t="n">
-        <v>28.7</v>
+        <v>211.5</v>
       </c>
       <c r="D158" t="n">
-        <v>2.46</v>
+        <v>2.07</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>DOLATALGO</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>62.4</v>
+        <v>1.94</v>
       </c>
       <c r="C159" t="n">
-        <v>63.93</v>
+        <v>1.98</v>
       </c>
       <c r="D159" t="n">
-        <v>2.45</v>
+        <v>2.06</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>ARIES</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>10.64</v>
+        <v>499</v>
       </c>
       <c r="C160" t="n">
-        <v>10.9</v>
+        <v>509.3</v>
       </c>
       <c r="D160" t="n">
-        <v>2.44</v>
+        <v>2.06</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>PRISMX</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>20.49</v>
+        <v>0.49</v>
       </c>
       <c r="C161" t="n">
-        <v>20.99</v>
+        <v>0.5</v>
       </c>
       <c r="D161" t="n">
-        <v>2.44</v>
+        <v>2.04</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>43.83</v>
+        <v>6.42</v>
       </c>
       <c r="C162" t="n">
-        <v>44.9</v>
+        <v>6.55</v>
       </c>
       <c r="D162" t="n">
-        <v>2.44</v>
+        <v>2.02</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>DWARKESH</t>
+          <t>MOLDTECH</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>44.08</v>
+        <v>216.72</v>
       </c>
       <c r="C163" t="n">
-        <v>45.15</v>
+        <v>221.1</v>
       </c>
       <c r="D163" t="n">
-        <v>2.43</v>
+        <v>2.02</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>OSWALAGRO</t>
+          <t>PPAP</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>32.98</v>
+        <v>239.81</v>
       </c>
       <c r="C164" t="n">
-        <v>33.78</v>
+        <v>244.6</v>
       </c>
       <c r="D164" t="n">
-        <v>2.43</v>
+        <v>2</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>ELECTHERM</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>0.83</v>
+        <v>735.25</v>
       </c>
       <c r="C165" t="n">
-        <v>0.85</v>
+        <v>749.9</v>
       </c>
       <c r="D165" t="n">
-        <v>2.41</v>
+        <v>1.99</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>4.15</v>
+        <v>14.07</v>
       </c>
       <c r="C166" t="n">
-        <v>4.25</v>
+        <v>14.35</v>
       </c>
       <c r="D166" t="n">
-        <v>2.41</v>
+        <v>1.99</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.42</v>
+        <v>31.86</v>
       </c>
       <c r="C167" t="n">
-        <v>0.43</v>
+        <v>32.49</v>
       </c>
       <c r="D167" t="n">
-        <v>2.38</v>
+        <v>1.98</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>WANBURY</t>
+          <t>3BBLACKBIO</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>190.46</v>
+        <v>1575.1</v>
       </c>
       <c r="C168" t="n">
-        <v>194.99</v>
+        <v>1606</v>
       </c>
       <c r="D168" t="n">
-        <v>2.38</v>
+        <v>1.96</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>AMJLAND</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>37.14</v>
+        <v>196.15</v>
       </c>
       <c r="C169" t="n">
-        <v>38.02</v>
+        <v>200</v>
       </c>
       <c r="D169" t="n">
-        <v>2.37</v>
+        <v>1.96</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>197.79</v>
+        <v>201.12</v>
       </c>
       <c r="C170" t="n">
-        <v>202.45</v>
+        <v>205</v>
       </c>
       <c r="D170" t="n">
-        <v>2.36</v>
+        <v>1.93</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>SHANTIINOR</t>
+          <t>TRACXN</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>168.05</v>
+        <v>34.34</v>
       </c>
       <c r="C171" t="n">
-        <v>172</v>
+        <v>35</v>
       </c>
       <c r="D171" t="n">
-        <v>2.35</v>
+        <v>1.92</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SWISSMLTRY</t>
+          <t>NCLIND</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>14.16</v>
+        <v>166.8</v>
       </c>
       <c r="C172" t="n">
-        <v>14.49</v>
+        <v>170</v>
       </c>
       <c r="D172" t="n">
-        <v>2.33</v>
+        <v>1.92</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>0.43</v>
+        <v>1668.1</v>
       </c>
       <c r="C173" t="n">
-        <v>0.44</v>
+        <v>1700</v>
       </c>
       <c r="D173" t="n">
-        <v>2.33</v>
+        <v>1.91</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ARROWGREEN</t>
+          <t>SONA</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>858.55</v>
+        <v>94.08</v>
       </c>
       <c r="C174" t="n">
-        <v>878.5</v>
+        <v>95.88</v>
       </c>
       <c r="D174" t="n">
-        <v>2.32</v>
+        <v>1.91</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>547.2</v>
+        <v>73.33</v>
       </c>
       <c r="C175" t="n">
-        <v>559.9</v>
+        <v>74.73</v>
       </c>
       <c r="D175" t="n">
-        <v>2.32</v>
+        <v>1.91</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>RTSPOWR</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>3989.5</v>
+        <v>103.78</v>
       </c>
       <c r="C176" t="n">
-        <v>4082.1</v>
+        <v>105.75</v>
       </c>
       <c r="D176" t="n">
-        <v>2.32</v>
+        <v>1.9</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>515.1</v>
+        <v>57.38</v>
       </c>
       <c r="C177" t="n">
-        <v>526.95</v>
+        <v>58.47</v>
       </c>
       <c r="D177" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HILINFRA</t>
+          <t>NATCAPSUQ</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>43.71</v>
+        <v>166.74</v>
       </c>
       <c r="C178" t="n">
-        <v>44.7</v>
+        <v>169.89</v>
       </c>
       <c r="D178" t="n">
-        <v>2.26</v>
+        <v>1.89</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>KRISHANA</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>185.83</v>
+        <v>73.81</v>
       </c>
       <c r="C179" t="n">
-        <v>190</v>
+        <v>75.2</v>
       </c>
       <c r="D179" t="n">
-        <v>2.24</v>
+        <v>1.88</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>JAIBALAJI</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>61.12</v>
+        <v>318.95</v>
       </c>
       <c r="C180" t="n">
-        <v>62.49</v>
+        <v>324.9</v>
       </c>
       <c r="D180" t="n">
-        <v>2.24</v>
+        <v>1.87</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>26.3</v>
+        <v>36.52</v>
       </c>
       <c r="C181" t="n">
-        <v>26.89</v>
+        <v>37.2</v>
       </c>
       <c r="D181" t="n">
-        <v>2.24</v>
+        <v>1.86</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>GLOTTIS</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>56.72</v>
+        <v>432.95</v>
       </c>
       <c r="C182" t="n">
-        <v>57.99</v>
+        <v>441</v>
       </c>
       <c r="D182" t="n">
-        <v>2.24</v>
+        <v>1.86</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>AKASH</t>
+          <t>WEL</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>24.64</v>
+        <v>74.62</v>
       </c>
       <c r="C183" t="n">
-        <v>25.19</v>
+        <v>76</v>
       </c>
       <c r="D183" t="n">
-        <v>2.23</v>
+        <v>1.85</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>GTPL</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>46.47</v>
+        <v>54.68</v>
       </c>
       <c r="C184" t="n">
-        <v>47.5</v>
+        <v>55.69</v>
       </c>
       <c r="D184" t="n">
-        <v>2.22</v>
+        <v>1.85</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SYRMA</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>1700.4</v>
+        <v>5.98</v>
       </c>
       <c r="C185" t="n">
-        <v>1738.1</v>
+        <v>6.09</v>
       </c>
       <c r="D185" t="n">
-        <v>2.22</v>
+        <v>1.84</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ONIXSOLAR</t>
+          <t>RKSWAMY</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>334.6</v>
+        <v>87.87</v>
       </c>
       <c r="C186" t="n">
-        <v>342</v>
+        <v>89.48</v>
       </c>
       <c r="D186" t="n">
-        <v>2.21</v>
+        <v>1.83</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>2206.6</v>
+        <v>4.98</v>
       </c>
       <c r="C187" t="n">
-        <v>2254.9</v>
+        <v>5.07</v>
       </c>
       <c r="D187" t="n">
-        <v>2.19</v>
+        <v>1.81</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>37.57</v>
+        <v>579.65</v>
       </c>
       <c r="C188" t="n">
-        <v>38.39</v>
+        <v>590</v>
       </c>
       <c r="D188" t="n">
-        <v>2.18</v>
+        <v>1.79</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>1173.4</v>
+        <v>55.95</v>
       </c>
       <c r="C189" t="n">
-        <v>1199</v>
+        <v>56.95</v>
       </c>
       <c r="D189" t="n">
-        <v>2.18</v>
+        <v>1.79</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>MANCREDIT</t>
+          <t>HMAAGRO</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>221.1</v>
+        <v>24.56</v>
       </c>
       <c r="C190" t="n">
-        <v>225.9</v>
+        <v>25</v>
       </c>
       <c r="D190" t="n">
-        <v>2.17</v>
+        <v>1.79</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>KSE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>641.6</v>
+        <v>176.86</v>
       </c>
       <c r="C191" t="n">
-        <v>655.45</v>
+        <v>180</v>
       </c>
       <c r="D191" t="n">
-        <v>2.16</v>
+        <v>1.78</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>CORDELIA</t>
+          <t>KAMATHOTEL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>100.83</v>
+        <v>258.82</v>
       </c>
       <c r="C192" t="n">
-        <v>103</v>
+        <v>263.4</v>
       </c>
       <c r="D192" t="n">
-        <v>2.15</v>
+        <v>1.77</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>BYKE</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>204.89</v>
+        <v>29.46</v>
       </c>
       <c r="C193" t="n">
-        <v>209.28</v>
+        <v>29.98</v>
       </c>
       <c r="D193" t="n">
-        <v>2.14</v>
+        <v>1.77</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0.47</v>
+        <v>7.35</v>
       </c>
       <c r="C194" t="n">
-        <v>0.48</v>
+        <v>7.48</v>
       </c>
       <c r="D194" t="n">
-        <v>2.13</v>
+        <v>1.77</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>URBAN</t>
+          <t>WARDINMOBI</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>120.25</v>
+        <v>5.11</v>
       </c>
       <c r="C195" t="n">
-        <v>122.8</v>
+        <v>5.2</v>
       </c>
       <c r="D195" t="n">
-        <v>2.12</v>
+        <v>1.76</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1.89</v>
+        <v>26.97</v>
       </c>
       <c r="C196" t="n">
-        <v>1.93</v>
+        <v>27.44</v>
       </c>
       <c r="D196" t="n">
-        <v>2.12</v>
+        <v>1.74</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>KOTYARK</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>28.26</v>
+        <v>22.5</v>
       </c>
       <c r="C197" t="n">
-        <v>28.86</v>
+        <v>22.89</v>
       </c>
       <c r="D197" t="n">
-        <v>2.12</v>
+        <v>1.73</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>METROPOLIS</t>
+          <t>ONIXSOLAR</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>553.6</v>
+        <v>338.2</v>
       </c>
       <c r="C198" t="n">
-        <v>565.35</v>
+        <v>344</v>
       </c>
       <c r="D198" t="n">
-        <v>2.12</v>
+        <v>1.71</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>VISHWARAJ</t>
+          <t>UNIDT</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>5.23</v>
+        <v>226.13</v>
       </c>
       <c r="C199" t="n">
-        <v>5.34</v>
+        <v>230</v>
       </c>
       <c r="D199" t="n">
-        <v>2.1</v>
+        <v>1.71</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MODIS</t>
+          <t>CSLFINANCE</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>372.25</v>
+        <v>207.48</v>
       </c>
       <c r="C200" t="n">
-        <v>380</v>
+        <v>211</v>
       </c>
       <c r="D200" t="n">
-        <v>2.08</v>
+        <v>1.7</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>JMA</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>1.94</v>
+        <v>86.92</v>
       </c>
       <c r="C201" t="n">
-        <v>1.98</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="D201" t="n">
-        <v>2.06</v>
+        <v>1.7</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-08 10:56 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PARTY-RE</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3</v>
+        <v>11.52</v>
       </c>
       <c r="C2" t="n">
-        <v>0.35</v>
+        <v>13.8</v>
       </c>
       <c r="D2" t="n">
-        <v>16.67</v>
+        <v>19.79</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61.55</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>68</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>10.48</v>
+        <v>16.99</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SURANI</t>
+          <t>AGL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>144.05</v>
+        <v>12.63</v>
       </c>
       <c r="C4" t="n">
-        <v>158.45</v>
+        <v>14.5</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>14.81</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KANOHAR</t>
+          <t>PARTY-RE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>942.5</v>
+        <v>0.35</v>
       </c>
       <c r="C5" t="n">
-        <v>1030</v>
+        <v>0.4</v>
       </c>
       <c r="D5" t="n">
-        <v>9.279999999999999</v>
+        <v>14.29</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SHKSIL</t>
+          <t>VIRAT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30.45</v>
+        <v>382.45</v>
       </c>
       <c r="C6" t="n">
-        <v>32.9</v>
+        <v>420.65</v>
       </c>
       <c r="D6" t="n">
-        <v>8.050000000000001</v>
+        <v>9.99</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17.41</v>
+        <v>17.99</v>
       </c>
       <c r="C7" t="n">
-        <v>18.8</v>
+        <v>19.78</v>
       </c>
       <c r="D7" t="n">
-        <v>7.98</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>KDGREEN</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>49.19</v>
+        <v>4.51</v>
       </c>
       <c r="C8" t="n">
-        <v>52.99</v>
+        <v>4.94</v>
       </c>
       <c r="D8" t="n">
-        <v>7.73</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>SURANI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>242.14</v>
+        <v>158.45</v>
       </c>
       <c r="C9" t="n">
-        <v>260</v>
+        <v>172</v>
       </c>
       <c r="D9" t="n">
-        <v>7.38</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.14</v>
+        <v>320.6</v>
       </c>
       <c r="C10" t="n">
-        <v>0.15</v>
+        <v>346.05</v>
       </c>
       <c r="D10" t="n">
-        <v>7.14</v>
+        <v>7.94</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PRUDMOULI</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13.81</v>
+        <v>11.45</v>
       </c>
       <c r="C11" t="n">
-        <v>14.77</v>
+        <v>12.34</v>
       </c>
       <c r="D11" t="n">
-        <v>6.95</v>
+        <v>7.77</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>PRUDMOULI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>213.69</v>
+        <v>13.54</v>
       </c>
       <c r="C12" t="n">
-        <v>228</v>
+        <v>14.49</v>
       </c>
       <c r="D12" t="n">
-        <v>6.7</v>
+        <v>7.02</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RPSGVENT</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>833.1</v>
+        <v>1.52</v>
       </c>
       <c r="C13" t="n">
-        <v>887</v>
+        <v>1.62</v>
       </c>
       <c r="D13" t="n">
-        <v>6.47</v>
+        <v>6.58</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MYMUDRA</t>
+          <t>MONEYVIEW</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>82.7</v>
+        <v>60.46</v>
       </c>
       <c r="C14" t="n">
-        <v>87.95</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>6.35</v>
+        <v>6.52</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8.09</v>
+        <v>34.82</v>
       </c>
       <c r="C15" t="n">
-        <v>8.6</v>
+        <v>36.99</v>
       </c>
       <c r="D15" t="n">
-        <v>6.3</v>
+        <v>6.23</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>KIRANVYPAR</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.25</v>
+        <v>191.35</v>
       </c>
       <c r="C16" t="n">
-        <v>5.58</v>
+        <v>203</v>
       </c>
       <c r="D16" t="n">
-        <v>6.29</v>
+        <v>6.09</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5.21</v>
+        <v>32.49</v>
       </c>
       <c r="C17" t="n">
-        <v>5.53</v>
+        <v>34.4</v>
       </c>
       <c r="D17" t="n">
-        <v>6.14</v>
+        <v>5.88</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UTKARSHBNK</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>13.52</v>
+        <v>7.32</v>
       </c>
       <c r="C18" t="n">
-        <v>14.3</v>
+        <v>7.75</v>
       </c>
       <c r="D18" t="n">
-        <v>5.77</v>
+        <v>5.87</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SHANTIINOR</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>201.65</v>
+        <v>0.18</v>
       </c>
       <c r="C19" t="n">
-        <v>213.1</v>
+        <v>0.19</v>
       </c>
       <c r="D19" t="n">
-        <v>5.68</v>
+        <v>5.56</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KEYFINSERV</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>241.53</v>
+        <v>4.98</v>
       </c>
       <c r="C20" t="n">
-        <v>254.95</v>
+        <v>5.23</v>
       </c>
       <c r="D20" t="n">
-        <v>5.56</v>
+        <v>5.02</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>RHETAN</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>153.5</v>
+        <v>17.4</v>
       </c>
       <c r="C21" t="n">
-        <v>162</v>
+        <v>18.27</v>
       </c>
       <c r="D21" t="n">
-        <v>5.54</v>
+        <v>5</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NKIND</t>
+          <t>ESDS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>57.06</v>
+        <v>1359</v>
       </c>
       <c r="C22" t="n">
-        <v>60</v>
+        <v>1426.9</v>
       </c>
       <c r="D22" t="n">
-        <v>5.15</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PRADPME</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>544.25</v>
+        <v>1382.15</v>
       </c>
       <c r="C23" t="n">
-        <v>572.2</v>
+        <v>1451.25</v>
       </c>
       <c r="D23" t="n">
-        <v>5.14</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.78</v>
+        <v>53.8</v>
       </c>
       <c r="C24" t="n">
-        <v>1.87</v>
+        <v>56.49</v>
       </c>
       <c r="D24" t="n">
-        <v>5.06</v>
+        <v>5</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>SWASTIKAIN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>7.4</v>
+        <v>210.13</v>
       </c>
       <c r="C25" t="n">
-        <v>7.77</v>
+        <v>220.63</v>
       </c>
       <c r="D25" t="n">
         <v>5</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>SPCON</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>244.11</v>
+        <v>180</v>
       </c>
       <c r="C26" t="n">
-        <v>256.31</v>
+        <v>189</v>
       </c>
       <c r="D26" t="n">
         <v>5</v>
@@ -1011,14 +1011,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>186.12</v>
+        <v>597.45</v>
       </c>
       <c r="C27" t="n">
-        <v>195.42</v>
+        <v>627.3</v>
       </c>
       <c r="D27" t="n">
         <v>5</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ESDS</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1294.3</v>
+        <v>3.81</v>
       </c>
       <c r="C28" t="n">
-        <v>1359</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>RUDRA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>262.78</v>
+        <v>19.46</v>
       </c>
       <c r="C29" t="n">
-        <v>275.91</v>
+        <v>20.43</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CEDAAR</t>
+          <t>POOJALOGIS</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>11</v>
+        <v>125.85</v>
       </c>
       <c r="C30" t="n">
-        <v>11.55</v>
+        <v>132.1</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4.97</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>NATIONSTD</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1316.35</v>
+        <v>110.21</v>
       </c>
       <c r="C31" t="n">
-        <v>1382.15</v>
+        <v>115.69</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>4.97</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>51.24</v>
+        <v>85.5</v>
       </c>
       <c r="C32" t="n">
-        <v>53.8</v>
+        <v>89.75</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>4.97</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>ARCL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2531.4</v>
+        <v>229.99</v>
       </c>
       <c r="C33" t="n">
-        <v>2657.9</v>
+        <v>241.4</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SPECTRAA</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>259.6</v>
+        <v>256.31</v>
       </c>
       <c r="C34" t="n">
-        <v>272.55</v>
+        <v>269</v>
       </c>
       <c r="D34" t="n">
-        <v>4.99</v>
+        <v>4.95</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>11.43</v>
+        <v>12.12</v>
       </c>
       <c r="C35" t="n">
-        <v>12</v>
+        <v>12.72</v>
       </c>
       <c r="D35" t="n">
-        <v>4.99</v>
+        <v>4.95</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>JAIBALAJI</t>
+          <t>ABAN</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>64.17</v>
+        <v>17.76</v>
       </c>
       <c r="C36" t="n">
-        <v>67.37</v>
+        <v>18.64</v>
       </c>
       <c r="D36" t="n">
-        <v>4.99</v>
+        <v>4.95</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>50.34</v>
+        <v>5.47</v>
       </c>
       <c r="C37" t="n">
-        <v>52.85</v>
+        <v>5.74</v>
       </c>
       <c r="D37" t="n">
-        <v>4.99</v>
+        <v>4.94</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BMISL</t>
+          <t>ARIES</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>121.25</v>
+        <v>494.55</v>
       </c>
       <c r="C38" t="n">
-        <v>127.3</v>
+        <v>519</v>
       </c>
       <c r="D38" t="n">
-        <v>4.99</v>
+        <v>4.94</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AVATAR</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>166.95</v>
+        <v>28.88</v>
       </c>
       <c r="C39" t="n">
-        <v>175.25</v>
+        <v>30.3</v>
       </c>
       <c r="D39" t="n">
-        <v>4.97</v>
+        <v>4.92</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>61.4</v>
+        <v>6.59</v>
       </c>
       <c r="C40" t="n">
-        <v>64.45</v>
+        <v>6.91</v>
       </c>
       <c r="D40" t="n">
-        <v>4.97</v>
+        <v>4.86</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>17.14</v>
+        <v>1.65</v>
       </c>
       <c r="C41" t="n">
-        <v>17.99</v>
+        <v>1.73</v>
       </c>
       <c r="D41" t="n">
-        <v>4.96</v>
+        <v>4.85</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHNVISN</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4012.9</v>
+        <v>40.71</v>
       </c>
       <c r="C42" t="n">
-        <v>4211.9</v>
+        <v>42.68</v>
       </c>
       <c r="D42" t="n">
-        <v>4.96</v>
+        <v>4.84</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ABAN</t>
+          <t>GLOBALE</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>16.92</v>
+        <v>10.49</v>
       </c>
       <c r="C43" t="n">
-        <v>17.76</v>
+        <v>10.99</v>
       </c>
       <c r="D43" t="n">
-        <v>4.96</v>
+        <v>4.77</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AUSOMENT</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>137.48</v>
+        <v>6.3</v>
       </c>
       <c r="C44" t="n">
-        <v>144.3</v>
+        <v>6.6</v>
       </c>
       <c r="D44" t="n">
-        <v>4.96</v>
+        <v>4.76</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>RHETAN</t>
+          <t>APSISAERO</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>16.59</v>
+        <v>582.1</v>
       </c>
       <c r="C45" t="n">
-        <v>17.41</v>
+        <v>609.75</v>
       </c>
       <c r="D45" t="n">
-        <v>4.94</v>
+        <v>4.75</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>6.28</v>
+        <v>1.49</v>
       </c>
       <c r="C46" t="n">
-        <v>6.59</v>
+        <v>1.56</v>
       </c>
       <c r="D46" t="n">
-        <v>4.94</v>
+        <v>4.7</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1.42</v>
+        <v>8.1</v>
       </c>
       <c r="C47" t="n">
-        <v>1.49</v>
+        <v>8.48</v>
       </c>
       <c r="D47" t="n">
-        <v>4.93</v>
+        <v>4.69</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ARCIIL</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>32.65</v>
+        <v>3</v>
       </c>
       <c r="C48" t="n">
-        <v>34.25</v>
+        <v>3.14</v>
       </c>
       <c r="D48" t="n">
-        <v>4.9</v>
+        <v>4.67</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SWASTIKAIN</t>
+          <t>VISAMAN</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>200.13</v>
+        <v>25.7</v>
       </c>
       <c r="C49" t="n">
-        <v>209.8</v>
+        <v>26.9</v>
       </c>
       <c r="D49" t="n">
-        <v>4.83</v>
+        <v>4.67</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>5.21</v>
+        <v>2.37</v>
       </c>
       <c r="C50" t="n">
-        <v>5.46</v>
+        <v>2.48</v>
       </c>
       <c r="D50" t="n">
-        <v>4.8</v>
+        <v>4.64</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>VGINFOTECH</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>160.33</v>
+        <v>136.6</v>
       </c>
       <c r="C51" t="n">
-        <v>168</v>
+        <v>142.75</v>
       </c>
       <c r="D51" t="n">
-        <v>4.78</v>
+        <v>4.5</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>ONYX</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.42</v>
+        <v>37.8</v>
       </c>
       <c r="C52" t="n">
-        <v>0.44</v>
+        <v>39.45</v>
       </c>
       <c r="D52" t="n">
-        <v>4.76</v>
+        <v>4.37</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>BEWLTD</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>145.58</v>
+        <v>58.45</v>
       </c>
       <c r="C53" t="n">
-        <v>152.5</v>
+        <v>61</v>
       </c>
       <c r="D53" t="n">
-        <v>4.75</v>
+        <v>4.36</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OPTIVALUE</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>235.45</v>
+        <v>9.48</v>
       </c>
       <c r="C54" t="n">
-        <v>246.6</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="D54" t="n">
-        <v>4.74</v>
+        <v>4.32</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SOMATEX</t>
+          <t>MARALOVER</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>79.09</v>
+        <v>58.48</v>
       </c>
       <c r="C55" t="n">
-        <v>82.8</v>
+        <v>61</v>
       </c>
       <c r="D55" t="n">
-        <v>4.69</v>
+        <v>4.31</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>SONA</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1.5</v>
+        <v>98.78</v>
       </c>
       <c r="C56" t="n">
-        <v>1.57</v>
+        <v>103</v>
       </c>
       <c r="D56" t="n">
-        <v>4.67</v>
+        <v>4.27</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>3.64</v>
+        <v>382.7</v>
       </c>
       <c r="C57" t="n">
-        <v>3.81</v>
+        <v>399</v>
       </c>
       <c r="D57" t="n">
-        <v>4.67</v>
+        <v>4.26</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CRAVATEX</t>
+          <t>TVVISION</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>374.6</v>
+        <v>2.59</v>
       </c>
       <c r="C58" t="n">
-        <v>391.95</v>
+        <v>2.7</v>
       </c>
       <c r="D58" t="n">
-        <v>4.63</v>
+        <v>4.25</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>ACEVECTOR</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>38.78</v>
+        <v>31.11</v>
       </c>
       <c r="C59" t="n">
-        <v>40.57</v>
+        <v>32.42</v>
       </c>
       <c r="D59" t="n">
-        <v>4.62</v>
+        <v>4.21</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ISHANCH</t>
+          <t>FINOPB</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>47.92</v>
+        <v>128.76</v>
       </c>
       <c r="C60" t="n">
-        <v>50.04</v>
+        <v>134</v>
       </c>
       <c r="D60" t="n">
-        <v>4.42</v>
+        <v>4.07</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>45</v>
+        <v>52.85</v>
       </c>
       <c r="C61" t="n">
-        <v>46.99</v>
+        <v>55</v>
       </c>
       <c r="D61" t="n">
-        <v>4.42</v>
+        <v>4.07</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>4.12</v>
+        <v>214.34</v>
       </c>
       <c r="C62" t="n">
-        <v>4.3</v>
+        <v>223</v>
       </c>
       <c r="D62" t="n">
-        <v>4.37</v>
+        <v>4.04</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AKSHOPTFBR</t>
+          <t>VIJAYPD</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>7.37</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="C63" t="n">
-        <v>7.69</v>
+        <v>99.95</v>
       </c>
       <c r="D63" t="n">
-        <v>4.34</v>
+        <v>4.01</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>29.72</v>
+        <v>22.02</v>
       </c>
       <c r="C64" t="n">
-        <v>30.99</v>
+        <v>22.9</v>
       </c>
       <c r="D64" t="n">
-        <v>4.27</v>
+        <v>4</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MIDWESTLTD</t>
+          <t>CHEMFAB</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1006.2</v>
+        <v>331.8</v>
       </c>
       <c r="C65" t="n">
-        <v>1049</v>
+        <v>345</v>
       </c>
       <c r="D65" t="n">
-        <v>4.25</v>
+        <v>3.98</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>VLINFRA</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>24.75</v>
+        <v>195.42</v>
       </c>
       <c r="C66" t="n">
-        <v>25.8</v>
+        <v>203.2</v>
       </c>
       <c r="D66" t="n">
-        <v>4.24</v>
+        <v>3.98</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>20.98</v>
+        <v>12.8</v>
       </c>
       <c r="C67" t="n">
-        <v>21.84</v>
+        <v>13.29</v>
       </c>
       <c r="D67" t="n">
-        <v>4.1</v>
+        <v>3.83</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ABH</t>
+          <t>SOMICONVEY</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>45.65</v>
+        <v>83.37</v>
       </c>
       <c r="C68" t="n">
-        <v>47.5</v>
+        <v>86.55</v>
       </c>
       <c r="D68" t="n">
-        <v>4.05</v>
+        <v>3.81</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>AZADIND</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.25</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="C69" t="n">
-        <v>0.26</v>
+        <v>85.98999999999999</v>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>3.79</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>16.33</v>
+        <v>19.26</v>
       </c>
       <c r="C70" t="n">
-        <v>16.98</v>
+        <v>19.99</v>
       </c>
       <c r="D70" t="n">
-        <v>3.98</v>
+        <v>3.79</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>KAVDEFENCE</t>
+          <t>SUPTANERY</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>85.55</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="C71" t="n">
-        <v>88.90000000000001</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="D71" t="n">
-        <v>3.92</v>
+        <v>3.78</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>59.66</v>
+        <v>4.51</v>
       </c>
       <c r="C72" t="n">
-        <v>61.98</v>
+        <v>4.68</v>
       </c>
       <c r="D72" t="n">
-        <v>3.89</v>
+        <v>3.77</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>UNITEDTEA</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>18.64</v>
+        <v>408.85</v>
       </c>
       <c r="C73" t="n">
-        <v>19.36</v>
+        <v>424</v>
       </c>
       <c r="D73" t="n">
-        <v>3.86</v>
+        <v>3.71</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>495.85</v>
+        <v>47.16</v>
       </c>
       <c r="C74" t="n">
-        <v>515</v>
+        <v>48.9</v>
       </c>
       <c r="D74" t="n">
-        <v>3.86</v>
+        <v>3.69</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MANIKA</t>
+          <t>NAGREEKCAP</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>51.52</v>
+        <v>27.25</v>
       </c>
       <c r="C75" t="n">
-        <v>53.5</v>
+        <v>28.25</v>
       </c>
       <c r="D75" t="n">
-        <v>3.84</v>
+        <v>3.67</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>SHIVALIK</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>206.65</v>
+        <v>365.05</v>
       </c>
       <c r="C76" t="n">
-        <v>214.55</v>
+        <v>378.3</v>
       </c>
       <c r="D76" t="n">
-        <v>3.82</v>
+        <v>3.63</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>TECHLABS</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>16.6</v>
+        <v>111.85</v>
       </c>
       <c r="C77" t="n">
-        <v>17.23</v>
+        <v>115.85</v>
       </c>
       <c r="D77" t="n">
-        <v>3.8</v>
+        <v>3.58</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DIGIKORE</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>36.15</v>
+        <v>680.55</v>
       </c>
       <c r="C78" t="n">
-        <v>37.5</v>
+        <v>704.9</v>
       </c>
       <c r="D78" t="n">
-        <v>3.73</v>
+        <v>3.58</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SUPTANERY</t>
+          <t>DHABRIYA</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>8.07</v>
+        <v>477.05</v>
       </c>
       <c r="C79" t="n">
-        <v>8.369999999999999</v>
+        <v>494</v>
       </c>
       <c r="D79" t="n">
-        <v>3.72</v>
+        <v>3.55</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NAGREEKCAP</t>
+          <t>MUTHOOTMF</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>27.25</v>
+        <v>172.91</v>
       </c>
       <c r="C80" t="n">
-        <v>28.25</v>
+        <v>179</v>
       </c>
       <c r="D80" t="n">
-        <v>3.67</v>
+        <v>3.52</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SUPREME</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>30.27</v>
+        <v>6.55</v>
       </c>
       <c r="C81" t="n">
-        <v>31.35</v>
+        <v>6.78</v>
       </c>
       <c r="D81" t="n">
-        <v>3.57</v>
+        <v>3.51</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>EXCELSOFT</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>24.24</v>
+        <v>81.70999999999999</v>
       </c>
       <c r="C82" t="n">
-        <v>25.1</v>
+        <v>84.56999999999999</v>
       </c>
       <c r="D82" t="n">
-        <v>3.55</v>
+        <v>3.5</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>OSWALGREEN</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>6.52</v>
+        <v>18.99</v>
       </c>
       <c r="C83" t="n">
-        <v>6.75</v>
+        <v>19.65</v>
       </c>
       <c r="D83" t="n">
-        <v>3.53</v>
+        <v>3.48</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>9.369999999999999</v>
+        <v>15.37</v>
       </c>
       <c r="C84" t="n">
-        <v>9.699999999999999</v>
+        <v>15.9</v>
       </c>
       <c r="D84" t="n">
-        <v>3.52</v>
+        <v>3.45</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MANCREDIT</t>
+          <t>ABH</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>231.9</v>
+        <v>47.85</v>
       </c>
       <c r="C85" t="n">
-        <v>239.99</v>
+        <v>49.5</v>
       </c>
       <c r="D85" t="n">
-        <v>3.49</v>
+        <v>3.45</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>NELCAST</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>124.48</v>
+        <v>4.95</v>
       </c>
       <c r="C86" t="n">
-        <v>128.77</v>
+        <v>5.12</v>
       </c>
       <c r="D86" t="n">
-        <v>3.45</v>
+        <v>3.43</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>139.3</v>
+        <v>157.4</v>
       </c>
       <c r="C87" t="n">
-        <v>144</v>
+        <v>162.8</v>
       </c>
       <c r="D87" t="n">
-        <v>3.37</v>
+        <v>3.43</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>15.46</v>
+        <v>15.62</v>
       </c>
       <c r="C88" t="n">
-        <v>15.98</v>
+        <v>16.15</v>
       </c>
       <c r="D88" t="n">
-        <v>3.36</v>
+        <v>3.39</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>172.06</v>
+        <v>101.23</v>
       </c>
       <c r="C89" t="n">
-        <v>177.8</v>
+        <v>104.6</v>
       </c>
       <c r="D89" t="n">
-        <v>3.34</v>
+        <v>3.33</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>25.05</v>
+        <v>580.95</v>
       </c>
       <c r="C90" t="n">
-        <v>25.88</v>
+        <v>600</v>
       </c>
       <c r="D90" t="n">
-        <v>3.31</v>
+        <v>3.28</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MODIRUBBER</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>118.58</v>
+        <v>76.31</v>
       </c>
       <c r="C91" t="n">
-        <v>122.49</v>
+        <v>78.8</v>
       </c>
       <c r="D91" t="n">
-        <v>3.3</v>
+        <v>3.26</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GENCON</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>37.78</v>
+        <v>585</v>
       </c>
       <c r="C92" t="n">
-        <v>39</v>
+        <v>604</v>
       </c>
       <c r="D92" t="n">
-        <v>3.23</v>
+        <v>3.25</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>207.59</v>
+        <v>31.2</v>
       </c>
       <c r="C93" t="n">
-        <v>214.3</v>
+        <v>32.2</v>
       </c>
       <c r="D93" t="n">
-        <v>3.23</v>
+        <v>3.21</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,14 +2485,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>11.51</v>
+        <v>58.33</v>
       </c>
       <c r="C94" t="n">
-        <v>11.88</v>
+        <v>60.2</v>
       </c>
       <c r="D94" t="n">
         <v>3.21</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SIEL</t>
+          <t>JAIBALAJI</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>31</v>
+        <v>67.37</v>
       </c>
       <c r="C95" t="n">
-        <v>31.99</v>
+        <v>69.5</v>
       </c>
       <c r="D95" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,14 +2529,14 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>BATLIBOI</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>10.76</v>
+        <v>94.8</v>
       </c>
       <c r="C96" t="n">
-        <v>11.1</v>
+        <v>97.8</v>
       </c>
       <c r="D96" t="n">
         <v>3.16</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MARSONS</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>119.24</v>
+        <v>6.01</v>
       </c>
       <c r="C97" t="n">
-        <v>123</v>
+        <v>6.2</v>
       </c>
       <c r="D97" t="n">
-        <v>3.15</v>
+        <v>3.16</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PTCIL</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>23125</v>
+        <v>32.2</v>
       </c>
       <c r="C98" t="n">
-        <v>23850</v>
+        <v>33.2</v>
       </c>
       <c r="D98" t="n">
-        <v>3.14</v>
+        <v>3.11</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>47.08</v>
+        <v>5.87</v>
       </c>
       <c r="C99" t="n">
-        <v>48.54</v>
+        <v>6.05</v>
       </c>
       <c r="D99" t="n">
-        <v>3.1</v>
+        <v>3.07</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BIOPOL</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>51.75</v>
+        <v>87.94</v>
       </c>
       <c r="C100" t="n">
-        <v>53.35</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="D100" t="n">
-        <v>3.09</v>
+        <v>3.02</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>CORDELIA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>48.49</v>
+        <v>109.52</v>
       </c>
       <c r="C101" t="n">
-        <v>49.99</v>
+        <v>112.76</v>
       </c>
       <c r="D101" t="n">
-        <v>3.09</v>
+        <v>2.96</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>NUCLEUS</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>638.05</v>
+        <v>1127</v>
       </c>
       <c r="C102" t="n">
-        <v>657.7</v>
+        <v>1159.9</v>
       </c>
       <c r="D102" t="n">
-        <v>3.08</v>
+        <v>2.92</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>1.63</v>
+        <v>7.53</v>
       </c>
       <c r="C103" t="n">
-        <v>1.68</v>
+        <v>7.75</v>
       </c>
       <c r="D103" t="n">
-        <v>3.07</v>
+        <v>2.92</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PARAGON</t>
+          <t>BELLACASA</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>49.2</v>
+        <v>251.77</v>
       </c>
       <c r="C104" t="n">
-        <v>50.7</v>
+        <v>259</v>
       </c>
       <c r="D104" t="n">
-        <v>3.05</v>
+        <v>2.87</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PVRINOX</t>
+          <t>ARCIL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1249.4</v>
+        <v>160.31</v>
       </c>
       <c r="C105" t="n">
-        <v>1287</v>
+        <v>164.9</v>
       </c>
       <c r="D105" t="n">
-        <v>3.01</v>
+        <v>2.86</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>41.86</v>
+        <v>100.62</v>
       </c>
       <c r="C106" t="n">
-        <v>43.12</v>
+        <v>103.5</v>
       </c>
       <c r="D106" t="n">
-        <v>3.01</v>
+        <v>2.86</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>2</v>
+        <v>723.3</v>
       </c>
       <c r="C107" t="n">
-        <v>2.06</v>
+        <v>744</v>
       </c>
       <c r="D107" t="n">
-        <v>3</v>
+        <v>2.86</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>16.18</v>
+        <v>0.71</v>
       </c>
       <c r="C108" t="n">
-        <v>16.66</v>
+        <v>0.73</v>
       </c>
       <c r="D108" t="n">
-        <v>2.97</v>
+        <v>2.82</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MARALOVER</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>57.99</v>
+        <v>45.71</v>
       </c>
       <c r="C109" t="n">
-        <v>59.7</v>
+        <v>47</v>
       </c>
       <c r="D109" t="n">
-        <v>2.95</v>
+        <v>2.82</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>233.12</v>
+        <v>1.43</v>
       </c>
       <c r="C110" t="n">
-        <v>240</v>
+        <v>1.47</v>
       </c>
       <c r="D110" t="n">
-        <v>2.95</v>
+        <v>2.8</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>11.55</v>
+        <v>12.5</v>
       </c>
       <c r="C111" t="n">
-        <v>11.89</v>
+        <v>12.85</v>
       </c>
       <c r="D111" t="n">
-        <v>2.94</v>
+        <v>2.8</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>HINDALUMI</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1.36</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="C112" t="n">
-        <v>1.4</v>
+        <v>92.5</v>
       </c>
       <c r="D112" t="n">
-        <v>2.94</v>
+        <v>2.79</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SHRADHA</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>29.83</v>
+        <v>35.22</v>
       </c>
       <c r="C113" t="n">
-        <v>30.7</v>
+        <v>36.2</v>
       </c>
       <c r="D113" t="n">
-        <v>2.92</v>
+        <v>2.78</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LOVABLE</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>69</v>
+        <v>0.36</v>
       </c>
       <c r="C114" t="n">
-        <v>71</v>
+        <v>0.37</v>
       </c>
       <c r="D114" t="n">
-        <v>2.9</v>
+        <v>2.78</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>JITFINFRA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>22.78</v>
+        <v>278.3</v>
       </c>
       <c r="C115" t="n">
-        <v>23.44</v>
+        <v>286</v>
       </c>
       <c r="D115" t="n">
-        <v>2.9</v>
+        <v>2.77</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ASTEC</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>704.7</v>
+        <v>2.18</v>
       </c>
       <c r="C116" t="n">
-        <v>724.95</v>
+        <v>2.24</v>
       </c>
       <c r="D116" t="n">
-        <v>2.87</v>
+        <v>2.75</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>JTLIND</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>76.70999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="C117" t="n">
-        <v>78.90000000000001</v>
+        <v>90.62</v>
       </c>
       <c r="D117" t="n">
-        <v>2.85</v>
+        <v>2.74</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MHLXMIRU</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>171.12</v>
+        <v>225.66</v>
       </c>
       <c r="C118" t="n">
-        <v>176</v>
+        <v>231.83</v>
       </c>
       <c r="D118" t="n">
-        <v>2.85</v>
+        <v>2.73</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KHERIAAUTO</t>
+          <t>KOKUYOCMLN</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>89.45</v>
+        <v>73</v>
       </c>
       <c r="C119" t="n">
-        <v>92</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="D119" t="n">
-        <v>2.85</v>
+        <v>2.73</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>GAUDIUMIVF</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>109.28</v>
+        <v>2657.9</v>
       </c>
       <c r="C120" t="n">
-        <v>112.38</v>
+        <v>2730</v>
       </c>
       <c r="D120" t="n">
-        <v>2.84</v>
+        <v>2.71</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>8.17</v>
+        <v>698.15</v>
       </c>
       <c r="C121" t="n">
-        <v>8.4</v>
+        <v>717</v>
       </c>
       <c r="D121" t="n">
-        <v>2.82</v>
+        <v>2.7</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>VISHAL</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>17.5</v>
+        <v>31.1</v>
       </c>
       <c r="C122" t="n">
-        <v>17.99</v>
+        <v>31.94</v>
       </c>
       <c r="D122" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1.44</v>
+        <v>57.75</v>
       </c>
       <c r="C123" t="n">
-        <v>1.48</v>
+        <v>59.29</v>
       </c>
       <c r="D123" t="n">
-        <v>2.78</v>
+        <v>2.67</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.37</v>
+        <v>13.14</v>
       </c>
       <c r="C124" t="n">
-        <v>0.38</v>
+        <v>13.49</v>
       </c>
       <c r="D124" t="n">
-        <v>2.7</v>
+        <v>2.66</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>APOLSINHOT</t>
+          <t>ASIANHOTNR</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1174.7</v>
+        <v>330.25</v>
       </c>
       <c r="C125" t="n">
-        <v>1205.9</v>
+        <v>339</v>
       </c>
       <c r="D125" t="n">
-        <v>2.66</v>
+        <v>2.65</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SUNSHIEL</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1047.4</v>
+        <v>498.8</v>
       </c>
       <c r="C126" t="n">
-        <v>1075</v>
+        <v>512</v>
       </c>
       <c r="D126" t="n">
-        <v>2.64</v>
+        <v>2.65</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,14 +3211,14 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BPLPHARMA</t>
+          <t>SICAGEN</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1836.4</v>
+        <v>51.53</v>
       </c>
       <c r="C127" t="n">
-        <v>1884.9</v>
+        <v>52.89</v>
       </c>
       <c r="D127" t="n">
         <v>2.64</v>
@@ -3233,14 +3233,14 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>PAUSHAKLTD</t>
+          <t>ELIN</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>704.3</v>
+        <v>77.06999999999999</v>
       </c>
       <c r="C128" t="n">
-        <v>722.85</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="D128" t="n">
         <v>2.63</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SADHNANIQ</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>2.68</v>
+        <v>33.14</v>
       </c>
       <c r="C129" t="n">
-        <v>2.75</v>
+        <v>34</v>
       </c>
       <c r="D129" t="n">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>13.15</v>
+        <v>142.71</v>
       </c>
       <c r="C130" t="n">
-        <v>13.48</v>
+        <v>146.4</v>
       </c>
       <c r="D130" t="n">
-        <v>2.51</v>
+        <v>2.59</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RAMANEWS</t>
+          <t>JAYBARMARU</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>28.88</v>
+        <v>132.78</v>
       </c>
       <c r="C131" t="n">
-        <v>29.59</v>
+        <v>136.2</v>
       </c>
       <c r="D131" t="n">
-        <v>2.46</v>
+        <v>2.58</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>KOKUYOCMLN</t>
+          <t>ALPEXSOLAR</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>74.56999999999999</v>
+        <v>815.1</v>
       </c>
       <c r="C132" t="n">
-        <v>76.40000000000001</v>
+        <v>836</v>
       </c>
       <c r="D132" t="n">
-        <v>2.45</v>
+        <v>2.56</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>131.63</v>
+        <v>165.75</v>
       </c>
       <c r="C133" t="n">
-        <v>134.84</v>
+        <v>170</v>
       </c>
       <c r="D133" t="n">
-        <v>2.44</v>
+        <v>2.56</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>GINNIFILA</t>
+          <t>NELCAST</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>40.96</v>
+        <v>146.29</v>
       </c>
       <c r="C134" t="n">
-        <v>41.95</v>
+        <v>150</v>
       </c>
       <c r="D134" t="n">
-        <v>2.42</v>
+        <v>2.54</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>CALSOFT</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>16.09</v>
+        <v>35.11</v>
       </c>
       <c r="C135" t="n">
-        <v>16.48</v>
+        <v>36</v>
       </c>
       <c r="D135" t="n">
-        <v>2.42</v>
+        <v>2.53</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SHAHALLOYS</t>
+          <t>ALOKINDS</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>81.03</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="C136" t="n">
-        <v>82.94</v>
+        <v>8.5</v>
       </c>
       <c r="D136" t="n">
-        <v>2.36</v>
+        <v>2.53</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>RENTOMOJO</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>14.16</v>
+        <v>618.95</v>
       </c>
       <c r="C137" t="n">
-        <v>14.49</v>
+        <v>634.5</v>
       </c>
       <c r="D137" t="n">
-        <v>2.33</v>
+        <v>2.51</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>12.92</v>
+        <v>377.55</v>
       </c>
       <c r="C138" t="n">
-        <v>13.22</v>
+        <v>387</v>
       </c>
       <c r="D138" t="n">
-        <v>2.32</v>
+        <v>2.5</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>HBPOR</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>27.37</v>
+        <v>62.36</v>
       </c>
       <c r="C139" t="n">
-        <v>28</v>
+        <v>63.91</v>
       </c>
       <c r="D139" t="n">
-        <v>2.3</v>
+        <v>2.49</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>HARIOMPIPE</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>336.5</v>
+        <v>3.22</v>
       </c>
       <c r="C140" t="n">
-        <v>344.25</v>
+        <v>3.3</v>
       </c>
       <c r="D140" t="n">
-        <v>2.3</v>
+        <v>2.48</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>JSWCEMENT</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>113.2</v>
+        <v>26.11</v>
       </c>
       <c r="C141" t="n">
-        <v>115.77</v>
+        <v>26.75</v>
       </c>
       <c r="D141" t="n">
-        <v>2.27</v>
+        <v>2.45</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ARCIL</t>
+          <t>RAJOOENG</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>145.74</v>
+        <v>62.37</v>
       </c>
       <c r="C142" t="n">
-        <v>149</v>
+        <v>63.9</v>
       </c>
       <c r="D142" t="n">
-        <v>2.24</v>
+        <v>2.45</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>BAIDFIN</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>96.36</v>
+        <v>10.21</v>
       </c>
       <c r="C143" t="n">
-        <v>98.5</v>
+        <v>10.46</v>
       </c>
       <c r="D143" t="n">
-        <v>2.22</v>
+        <v>2.45</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>THEINVEST</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>35.22</v>
+        <v>90.2</v>
       </c>
       <c r="C144" t="n">
-        <v>36</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="D144" t="n">
-        <v>2.21</v>
+        <v>2.44</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ATAM</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>54.2</v>
+        <v>0.84</v>
       </c>
       <c r="C145" t="n">
-        <v>55.4</v>
+        <v>0.86</v>
       </c>
       <c r="D145" t="n">
-        <v>2.21</v>
+        <v>2.38</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>69.91</v>
+        <v>49.43</v>
       </c>
       <c r="C146" t="n">
-        <v>71.45</v>
+        <v>50.6</v>
       </c>
       <c r="D146" t="n">
-        <v>2.2</v>
+        <v>2.37</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>110.55</v>
+        <v>1270.1</v>
       </c>
       <c r="C147" t="n">
-        <v>112.97</v>
+        <v>1300</v>
       </c>
       <c r="D147" t="n">
-        <v>2.19</v>
+        <v>2.35</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>36.15</v>
+        <v>1484.2</v>
       </c>
       <c r="C148" t="n">
-        <v>36.94</v>
+        <v>1519</v>
       </c>
       <c r="D148" t="n">
-        <v>2.19</v>
+        <v>2.34</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ALOKINDS</t>
+          <t>AURUS</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>7.83</v>
+        <v>4.29</v>
       </c>
       <c r="C149" t="n">
-        <v>8</v>
+        <v>4.39</v>
       </c>
       <c r="D149" t="n">
-        <v>2.17</v>
+        <v>2.33</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>54.82</v>
+        <v>199.38</v>
       </c>
       <c r="C150" t="n">
-        <v>56</v>
+        <v>204</v>
       </c>
       <c r="D150" t="n">
-        <v>2.15</v>
+        <v>2.32</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>MOMSBELIEF</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>92.86</v>
+        <v>229.68</v>
       </c>
       <c r="C151" t="n">
-        <v>94.84</v>
+        <v>234.89</v>
       </c>
       <c r="D151" t="n">
-        <v>2.13</v>
+        <v>2.27</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>51.88</v>
+        <v>91.81999999999999</v>
       </c>
       <c r="C152" t="n">
-        <v>52.98</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="D152" t="n">
-        <v>2.12</v>
+        <v>2.27</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CORDSCABLE</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>314.35</v>
+        <v>1.76</v>
       </c>
       <c r="C153" t="n">
-        <v>321</v>
+        <v>1.8</v>
       </c>
       <c r="D153" t="n">
-        <v>2.12</v>
+        <v>2.27</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>1013.05</v>
+        <v>0.44</v>
       </c>
       <c r="C154" t="n">
-        <v>1034.4</v>
+        <v>0.45</v>
       </c>
       <c r="D154" t="n">
-        <v>2.11</v>
+        <v>2.27</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>DRONE</t>
+          <t>MATRIMONY</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>33.3</v>
+        <v>517.5</v>
       </c>
       <c r="C155" t="n">
-        <v>34</v>
+        <v>529.05</v>
       </c>
       <c r="D155" t="n">
-        <v>2.1</v>
+        <v>2.23</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>AURUS</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>4.29</v>
+        <v>28.32</v>
       </c>
       <c r="C156" t="n">
-        <v>4.38</v>
+        <v>28.95</v>
       </c>
       <c r="D156" t="n">
-        <v>2.1</v>
+        <v>2.22</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>WEWIN</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>30.95</v>
+        <v>52.85</v>
       </c>
       <c r="C157" t="n">
-        <v>31.6</v>
+        <v>54</v>
       </c>
       <c r="D157" t="n">
-        <v>2.1</v>
+        <v>2.18</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>BAJAJINDEF</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>207.21</v>
+        <v>5.95</v>
       </c>
       <c r="C158" t="n">
-        <v>211.5</v>
+        <v>6.08</v>
       </c>
       <c r="D158" t="n">
-        <v>2.07</v>
+        <v>2.18</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>1.94</v>
+        <v>14.19</v>
       </c>
       <c r="C159" t="n">
-        <v>1.98</v>
+        <v>14.5</v>
       </c>
       <c r="D159" t="n">
-        <v>2.06</v>
+        <v>2.18</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ARIES</t>
+          <t>MERCURYEV</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>499</v>
+        <v>37.88</v>
       </c>
       <c r="C160" t="n">
-        <v>509.3</v>
+        <v>38.7</v>
       </c>
       <c r="D160" t="n">
-        <v>2.06</v>
+        <v>2.16</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>PRISMX</t>
+          <t>THOMASCOTT</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.49</v>
+        <v>278.85</v>
       </c>
       <c r="C161" t="n">
-        <v>0.5</v>
+        <v>284.85</v>
       </c>
       <c r="D161" t="n">
-        <v>2.04</v>
+        <v>2.15</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>TIJARIA</t>
+          <t>DRONE</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>6.42</v>
+        <v>33.05</v>
       </c>
       <c r="C162" t="n">
-        <v>6.55</v>
+        <v>33.75</v>
       </c>
       <c r="D162" t="n">
-        <v>2.02</v>
+        <v>2.12</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>MOLDTECH</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>216.72</v>
+        <v>4.25</v>
       </c>
       <c r="C163" t="n">
-        <v>221.1</v>
+        <v>4.34</v>
       </c>
       <c r="D163" t="n">
-        <v>2.02</v>
+        <v>2.12</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>PPAP</t>
+          <t>ZIMLAB</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>239.81</v>
+        <v>146.61</v>
       </c>
       <c r="C164" t="n">
-        <v>244.6</v>
+        <v>149.69</v>
       </c>
       <c r="D164" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ELECTHERM</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>735.25</v>
+        <v>1.91</v>
       </c>
       <c r="C165" t="n">
-        <v>749.9</v>
+        <v>1.95</v>
       </c>
       <c r="D165" t="n">
-        <v>1.99</v>
+        <v>2.09</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>SWISSMLTRY</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>14.07</v>
+        <v>58.78</v>
       </c>
       <c r="C166" t="n">
-        <v>14.35</v>
+        <v>60</v>
       </c>
       <c r="D166" t="n">
-        <v>1.99</v>
+        <v>2.08</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>31.86</v>
+        <v>13.11</v>
       </c>
       <c r="C167" t="n">
-        <v>32.49</v>
+        <v>13.38</v>
       </c>
       <c r="D167" t="n">
-        <v>1.98</v>
+        <v>2.06</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>3BBLACKBIO</t>
+          <t>ESAFSFB</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>1575.1</v>
+        <v>42.67</v>
       </c>
       <c r="C168" t="n">
-        <v>1606</v>
+        <v>43.54</v>
       </c>
       <c r="D168" t="n">
-        <v>1.96</v>
+        <v>2.04</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>ADVIKCA</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>196.15</v>
+        <v>0.98</v>
       </c>
       <c r="C169" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="D169" t="n">
-        <v>1.96</v>
+        <v>2.04</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>201.12</v>
+        <v>9.4</v>
       </c>
       <c r="C170" t="n">
-        <v>205</v>
+        <v>9.59</v>
       </c>
       <c r="D170" t="n">
-        <v>1.93</v>
+        <v>2.02</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>TRACXN</t>
+          <t>TGBHOTELS</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>34.34</v>
+        <v>9.4</v>
       </c>
       <c r="C171" t="n">
-        <v>35</v>
+        <v>9.59</v>
       </c>
       <c r="D171" t="n">
-        <v>1.92</v>
+        <v>2.02</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>NCLIND</t>
+          <t>ONWARDTEC</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>166.8</v>
+        <v>297.4</v>
       </c>
       <c r="C172" t="n">
-        <v>170</v>
+        <v>303.4</v>
       </c>
       <c r="D172" t="n">
-        <v>1.92</v>
+        <v>2.02</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>1668.1</v>
+        <v>12.96</v>
       </c>
       <c r="C173" t="n">
-        <v>1700</v>
+        <v>13.22</v>
       </c>
       <c r="D173" t="n">
-        <v>1.91</v>
+        <v>2.01</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SONA</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>94.08</v>
+        <v>367.6</v>
       </c>
       <c r="C174" t="n">
-        <v>95.88</v>
+        <v>375</v>
       </c>
       <c r="D174" t="n">
-        <v>1.91</v>
+        <v>2.01</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>OMINFRAL</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>73.33</v>
+        <v>26.36</v>
       </c>
       <c r="C175" t="n">
-        <v>74.73</v>
+        <v>26.89</v>
       </c>
       <c r="D175" t="n">
-        <v>1.91</v>
+        <v>2.01</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>RTSPOWR</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>103.78</v>
+        <v>16.91</v>
       </c>
       <c r="C176" t="n">
-        <v>105.75</v>
+        <v>17.25</v>
       </c>
       <c r="D176" t="n">
-        <v>1.9</v>
+        <v>2.01</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>57.38</v>
+        <v>50.48</v>
       </c>
       <c r="C177" t="n">
-        <v>58.47</v>
+        <v>51.49</v>
       </c>
       <c r="D177" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>NATCAPSUQ</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>166.74</v>
+        <v>13.03</v>
       </c>
       <c r="C178" t="n">
-        <v>169.89</v>
+        <v>13.29</v>
       </c>
       <c r="D178" t="n">
-        <v>1.89</v>
+        <v>2</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>73.81</v>
+        <v>92.64</v>
       </c>
       <c r="C179" t="n">
-        <v>75.2</v>
+        <v>94.48999999999999</v>
       </c>
       <c r="D179" t="n">
-        <v>1.88</v>
+        <v>2</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>SPECTRAA</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>318.95</v>
+        <v>272.55</v>
       </c>
       <c r="C180" t="n">
-        <v>324.9</v>
+        <v>278</v>
       </c>
       <c r="D180" t="n">
-        <v>1.87</v>
+        <v>2</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>BALPHARMA</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>36.52</v>
+        <v>98.62</v>
       </c>
       <c r="C181" t="n">
-        <v>37.2</v>
+        <v>100.59</v>
       </c>
       <c r="D181" t="n">
-        <v>1.86</v>
+        <v>2</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>432.95</v>
+        <v>33.09</v>
       </c>
       <c r="C182" t="n">
-        <v>441</v>
+        <v>33.75</v>
       </c>
       <c r="D182" t="n">
-        <v>1.86</v>
+        <v>1.99</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>WEL</t>
+          <t>MUTHOOTCAP</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>74.62</v>
+        <v>213.53</v>
       </c>
       <c r="C183" t="n">
-        <v>76</v>
+        <v>217.78</v>
       </c>
       <c r="D183" t="n">
-        <v>1.85</v>
+        <v>1.99</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>GTPL</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>54.68</v>
+        <v>24.18</v>
       </c>
       <c r="C184" t="n">
-        <v>55.69</v>
+        <v>24.66</v>
       </c>
       <c r="D184" t="n">
-        <v>1.85</v>
+        <v>1.99</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ASMS</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>5.98</v>
+        <v>173.9</v>
       </c>
       <c r="C185" t="n">
-        <v>6.09</v>
+        <v>177.35</v>
       </c>
       <c r="D185" t="n">
-        <v>1.84</v>
+        <v>1.98</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>RKSWAMY</t>
+          <t>LOVABLE</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>87.87</v>
+        <v>68.73</v>
       </c>
       <c r="C186" t="n">
-        <v>89.48</v>
+        <v>70.09</v>
       </c>
       <c r="D186" t="n">
-        <v>1.83</v>
+        <v>1.98</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>4.98</v>
+        <v>215.12</v>
       </c>
       <c r="C187" t="n">
-        <v>5.07</v>
+        <v>219.39</v>
       </c>
       <c r="D187" t="n">
-        <v>1.81</v>
+        <v>1.98</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>579.65</v>
+        <v>1665.1</v>
       </c>
       <c r="C188" t="n">
-        <v>590</v>
+        <v>1698</v>
       </c>
       <c r="D188" t="n">
-        <v>1.79</v>
+        <v>1.98</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>MEGASTAR</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>55.95</v>
+        <v>309.06</v>
       </c>
       <c r="C189" t="n">
-        <v>56.95</v>
+        <v>315.15</v>
       </c>
       <c r="D189" t="n">
-        <v>1.79</v>
+        <v>1.97</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HMAAGRO</t>
+          <t>ARCHIDPLY</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>24.56</v>
+        <v>102.73</v>
       </c>
       <c r="C190" t="n">
-        <v>25</v>
+        <v>104.75</v>
       </c>
       <c r="D190" t="n">
-        <v>1.79</v>
+        <v>1.97</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KSE</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>176.86</v>
+        <v>631</v>
       </c>
       <c r="C191" t="n">
-        <v>180</v>
+        <v>643.4</v>
       </c>
       <c r="D191" t="n">
-        <v>1.78</v>
+        <v>1.97</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>KAMATHOTEL</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>258.82</v>
+        <v>653.25</v>
       </c>
       <c r="C192" t="n">
-        <v>263.4</v>
+        <v>666</v>
       </c>
       <c r="D192" t="n">
-        <v>1.77</v>
+        <v>1.95</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>BYKE</t>
+          <t>CEMPRO</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>29.46</v>
+        <v>1137.8</v>
       </c>
       <c r="C193" t="n">
-        <v>29.98</v>
+        <v>1160</v>
       </c>
       <c r="D193" t="n">
-        <v>1.77</v>
+        <v>1.95</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>SARVESHWAR</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>7.35</v>
+        <v>3.61</v>
       </c>
       <c r="C194" t="n">
-        <v>7.48</v>
+        <v>3.68</v>
       </c>
       <c r="D194" t="n">
-        <v>1.77</v>
+        <v>1.94</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>WARDINMOBI</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>5.11</v>
+        <v>1.55</v>
       </c>
       <c r="C195" t="n">
-        <v>5.2</v>
+        <v>1.58</v>
       </c>
       <c r="D195" t="n">
-        <v>1.76</v>
+        <v>1.94</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>CRSL</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>26.97</v>
+        <v>2.06</v>
       </c>
       <c r="C196" t="n">
-        <v>27.44</v>
+        <v>2.1</v>
       </c>
       <c r="D196" t="n">
-        <v>1.74</v>
+        <v>1.94</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>22.5</v>
+        <v>31.37</v>
       </c>
       <c r="C197" t="n">
-        <v>22.89</v>
+        <v>31.98</v>
       </c>
       <c r="D197" t="n">
-        <v>1.73</v>
+        <v>1.94</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ONIXSOLAR</t>
+          <t>ITTL</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>338.2</v>
+        <v>61.9</v>
       </c>
       <c r="C198" t="n">
-        <v>344</v>
+        <v>63.1</v>
       </c>
       <c r="D198" t="n">
-        <v>1.71</v>
+        <v>1.94</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>UNIDT</t>
+          <t>CEIGALL</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>226.13</v>
+        <v>372.8</v>
       </c>
       <c r="C199" t="n">
-        <v>230</v>
+        <v>380</v>
       </c>
       <c r="D199" t="n">
-        <v>1.71</v>
+        <v>1.93</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>CSLFINANCE</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>207.48</v>
+        <v>1032.45</v>
       </c>
       <c r="C200" t="n">
-        <v>211</v>
+        <v>1052.4</v>
       </c>
       <c r="D200" t="n">
-        <v>1.7</v>
+        <v>1.93</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>JMA</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>86.92</v>
+        <v>56.5</v>
       </c>
       <c r="C201" t="n">
-        <v>88.40000000000001</v>
+        <v>57.59</v>
       </c>
       <c r="D201" t="n">
-        <v>1.7</v>
+        <v>1.93</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-09 10:55 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.52</v>
+        <v>13.82</v>
       </c>
       <c r="C2" t="n">
-        <v>13.8</v>
+        <v>16.4</v>
       </c>
       <c r="D2" t="n">
-        <v>19.79</v>
+        <v>18.67</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VALUE360</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73.84999999999999</v>
+        <v>1.41</v>
       </c>
       <c r="C3" t="n">
-        <v>86.40000000000001</v>
+        <v>1.59</v>
       </c>
       <c r="D3" t="n">
-        <v>16.99</v>
+        <v>12.77</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AGL</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12.63</v>
+        <v>5.61</v>
       </c>
       <c r="C4" t="n">
-        <v>14.5</v>
+        <v>6.14</v>
       </c>
       <c r="D4" t="n">
-        <v>14.81</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PARTY-RE</t>
+          <t>CEDAAR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.35</v>
+        <v>12.7</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4</v>
+        <v>13.9</v>
       </c>
       <c r="D5" t="n">
-        <v>14.29</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VIRAT</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>382.45</v>
+        <v>195.4</v>
       </c>
       <c r="C6" t="n">
-        <v>420.65</v>
+        <v>213</v>
       </c>
       <c r="D6" t="n">
-        <v>9.99</v>
+        <v>9.01</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>GLOBALE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17.99</v>
+        <v>11.53</v>
       </c>
       <c r="C7" t="n">
-        <v>19.78</v>
+        <v>12.55</v>
       </c>
       <c r="D7" t="n">
-        <v>9.949999999999999</v>
+        <v>8.85</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.51</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>4.94</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>9.529999999999999</v>
+        <v>7.83</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SURANI</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>158.45</v>
+        <v>0.13</v>
       </c>
       <c r="C9" t="n">
-        <v>172</v>
+        <v>0.14</v>
       </c>
       <c r="D9" t="n">
-        <v>8.550000000000001</v>
+        <v>7.69</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>BSHSL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>320.6</v>
+        <v>78.36</v>
       </c>
       <c r="C10" t="n">
-        <v>346.05</v>
+        <v>83.95</v>
       </c>
       <c r="D10" t="n">
-        <v>7.94</v>
+        <v>7.13</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>ITL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11.45</v>
+        <v>364.85</v>
       </c>
       <c r="C11" t="n">
-        <v>12.34</v>
+        <v>390</v>
       </c>
       <c r="D11" t="n">
-        <v>7.77</v>
+        <v>6.89</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PRUDMOULI</t>
+          <t>CUDML</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>13.54</v>
+        <v>87.2</v>
       </c>
       <c r="C12" t="n">
-        <v>14.49</v>
+        <v>93</v>
       </c>
       <c r="D12" t="n">
-        <v>7.02</v>
+        <v>6.65</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.52</v>
+        <v>20.63</v>
       </c>
       <c r="C13" t="n">
-        <v>1.62</v>
+        <v>22</v>
       </c>
       <c r="D13" t="n">
-        <v>6.58</v>
+        <v>6.64</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MONEYVIEW</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>60.46</v>
+        <v>16.84</v>
       </c>
       <c r="C14" t="n">
-        <v>64.40000000000001</v>
+        <v>17.76</v>
       </c>
       <c r="D14" t="n">
-        <v>6.52</v>
+        <v>5.46</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SHRIKRISH</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>34.82</v>
+        <v>28.45</v>
       </c>
       <c r="C15" t="n">
-        <v>36.99</v>
+        <v>30</v>
       </c>
       <c r="D15" t="n">
-        <v>6.23</v>
+        <v>5.45</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>KIRANVYPAR</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>191.35</v>
+        <v>1.31</v>
       </c>
       <c r="C16" t="n">
-        <v>203</v>
+        <v>1.38</v>
       </c>
       <c r="D16" t="n">
-        <v>6.09</v>
+        <v>5.34</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>AATMAJ</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>32.49</v>
+        <v>22.95</v>
       </c>
       <c r="C17" t="n">
-        <v>34.4</v>
+        <v>24.15</v>
       </c>
       <c r="D17" t="n">
-        <v>5.88</v>
+        <v>5.23</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>BNAGROCHEM</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7.32</v>
+        <v>199.39</v>
       </c>
       <c r="C18" t="n">
-        <v>7.75</v>
+        <v>209.65</v>
       </c>
       <c r="D18" t="n">
-        <v>5.87</v>
+        <v>5.15</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>SIMCA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.18</v>
+        <v>338</v>
       </c>
       <c r="C19" t="n">
-        <v>0.19</v>
+        <v>354.9</v>
       </c>
       <c r="D19" t="n">
-        <v>5.56</v>
+        <v>5</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4.98</v>
+        <v>89.05</v>
       </c>
       <c r="C20" t="n">
-        <v>5.23</v>
+        <v>93.5</v>
       </c>
       <c r="D20" t="n">
-        <v>5.02</v>
+        <v>5</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RHETAN</t>
+          <t>MOBILISE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>17.4</v>
+        <v>103.25</v>
       </c>
       <c r="C21" t="n">
-        <v>18.27</v>
+        <v>108.4</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ESDS</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1359</v>
+        <v>32.76</v>
       </c>
       <c r="C22" t="n">
-        <v>1426.9</v>
+        <v>34.39</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1382.15</v>
+        <v>3.83</v>
       </c>
       <c r="C23" t="n">
-        <v>1451.25</v>
+        <v>4.02</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>53.8</v>
+        <v>12.72</v>
       </c>
       <c r="C24" t="n">
-        <v>56.49</v>
+        <v>13.35</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SWASTIKAIN</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>210.13</v>
+        <v>41.4</v>
       </c>
       <c r="C25" t="n">
-        <v>220.63</v>
+        <v>43.45</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SPCON</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>180</v>
+        <v>6.91</v>
       </c>
       <c r="C26" t="n">
-        <v>189</v>
+        <v>7.25</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>4.92</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>597.45</v>
+        <v>8.15</v>
       </c>
       <c r="C27" t="n">
-        <v>627.3</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>4.91</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>ROXHITECH</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3.81</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>68.55</v>
       </c>
       <c r="D28" t="n">
-        <v>4.99</v>
+        <v>4.9</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RUDRA</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>19.46</v>
+        <v>7.34</v>
       </c>
       <c r="C29" t="n">
-        <v>20.43</v>
+        <v>7.7</v>
       </c>
       <c r="D29" t="n">
-        <v>4.98</v>
+        <v>4.9</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>POOJALOGIS</t>
+          <t>SINTERCOM</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>125.85</v>
+        <v>73.41</v>
       </c>
       <c r="C30" t="n">
-        <v>132.1</v>
+        <v>77</v>
       </c>
       <c r="D30" t="n">
-        <v>4.97</v>
+        <v>4.89</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NATIONSTD</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>110.21</v>
+        <v>7.99</v>
       </c>
       <c r="C31" t="n">
-        <v>115.69</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="D31" t="n">
-        <v>4.97</v>
+        <v>4.88</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>EMKAY</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>85.5</v>
+        <v>265.65</v>
       </c>
       <c r="C32" t="n">
-        <v>89.75</v>
+        <v>278.6</v>
       </c>
       <c r="D32" t="n">
-        <v>4.97</v>
+        <v>4.87</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ARCL</t>
+          <t>KICL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>229.99</v>
+        <v>4692</v>
       </c>
       <c r="C33" t="n">
-        <v>241.4</v>
+        <v>4919</v>
       </c>
       <c r="D33" t="n">
-        <v>4.96</v>
+        <v>4.84</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>256.31</v>
+        <v>2.48</v>
       </c>
       <c r="C34" t="n">
-        <v>269</v>
+        <v>2.6</v>
       </c>
       <c r="D34" t="n">
-        <v>4.95</v>
+        <v>4.84</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>STARTECK</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>12.12</v>
+        <v>264.25</v>
       </c>
       <c r="C35" t="n">
-        <v>12.72</v>
+        <v>276.95</v>
       </c>
       <c r="D35" t="n">
-        <v>4.95</v>
+        <v>4.81</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABAN</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>17.76</v>
+        <v>27.44</v>
       </c>
       <c r="C36" t="n">
-        <v>18.64</v>
+        <v>28.75</v>
       </c>
       <c r="D36" t="n">
-        <v>4.95</v>
+        <v>4.77</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>CEWATER</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>5.47</v>
+        <v>254.8</v>
       </c>
       <c r="C37" t="n">
-        <v>5.74</v>
+        <v>266.9</v>
       </c>
       <c r="D37" t="n">
-        <v>4.94</v>
+        <v>4.75</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ARIES</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>494.55</v>
+        <v>10.01</v>
       </c>
       <c r="C38" t="n">
-        <v>519</v>
+        <v>10.48</v>
       </c>
       <c r="D38" t="n">
-        <v>4.94</v>
+        <v>4.7</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>21STCENMGM</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>28.88</v>
+        <v>41.07</v>
       </c>
       <c r="C39" t="n">
-        <v>30.3</v>
+        <v>42.95</v>
       </c>
       <c r="D39" t="n">
-        <v>4.92</v>
+        <v>4.58</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6.59</v>
+        <v>45.92</v>
       </c>
       <c r="C40" t="n">
-        <v>6.91</v>
+        <v>48</v>
       </c>
       <c r="D40" t="n">
-        <v>4.86</v>
+        <v>4.53</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>HBPOR</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1.65</v>
+        <v>61.99</v>
       </c>
       <c r="C41" t="n">
-        <v>1.73</v>
+        <v>64.75</v>
       </c>
       <c r="D41" t="n">
-        <v>4.85</v>
+        <v>4.45</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>DOLPHIN</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>40.71</v>
+        <v>620.05</v>
       </c>
       <c r="C42" t="n">
-        <v>42.68</v>
+        <v>647.6</v>
       </c>
       <c r="D42" t="n">
-        <v>4.84</v>
+        <v>4.44</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GLOBALE</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>10.49</v>
+        <v>3.39</v>
       </c>
       <c r="C43" t="n">
-        <v>10.99</v>
+        <v>3.54</v>
       </c>
       <c r="D43" t="n">
-        <v>4.77</v>
+        <v>4.42</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>AXIOMGAS</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6.3</v>
+        <v>44.1</v>
       </c>
       <c r="C44" t="n">
-        <v>6.6</v>
+        <v>46</v>
       </c>
       <c r="D44" t="n">
-        <v>4.76</v>
+        <v>4.31</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>APSISAERO</t>
+          <t>DEEP</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>582.1</v>
+        <v>39.33</v>
       </c>
       <c r="C45" t="n">
-        <v>609.75</v>
+        <v>41</v>
       </c>
       <c r="D45" t="n">
-        <v>4.75</v>
+        <v>4.25</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>NCC</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.49</v>
+        <v>119.93</v>
       </c>
       <c r="C46" t="n">
-        <v>1.56</v>
+        <v>125</v>
       </c>
       <c r="D46" t="n">
-        <v>4.7</v>
+        <v>4.23</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>HEXT</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>8.1</v>
+        <v>511.4</v>
       </c>
       <c r="C47" t="n">
-        <v>8.48</v>
+        <v>533</v>
       </c>
       <c r="D47" t="n">
-        <v>4.69</v>
+        <v>4.22</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>MANIKA</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>55.46</v>
       </c>
       <c r="C48" t="n">
-        <v>3.14</v>
+        <v>57.8</v>
       </c>
       <c r="D48" t="n">
-        <v>4.67</v>
+        <v>4.22</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>VISAMAN</t>
+          <t>HIMALAYAN</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>25.7</v>
+        <v>76.8</v>
       </c>
       <c r="C49" t="n">
-        <v>26.9</v>
+        <v>80</v>
       </c>
       <c r="D49" t="n">
-        <v>4.67</v>
+        <v>4.17</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.37</v>
+        <v>0.73</v>
       </c>
       <c r="C50" t="n">
-        <v>2.48</v>
+        <v>0.76</v>
       </c>
       <c r="D50" t="n">
-        <v>4.64</v>
+        <v>4.11</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>VGINFOTECH</t>
+          <t>PNGJL</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>136.6</v>
+        <v>586.3</v>
       </c>
       <c r="C51" t="n">
-        <v>142.75</v>
+        <v>609.9</v>
       </c>
       <c r="D51" t="n">
-        <v>4.5</v>
+        <v>4.03</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ONYX</t>
+          <t>LAGNAM</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>37.8</v>
+        <v>71.14</v>
       </c>
       <c r="C52" t="n">
-        <v>39.45</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="D52" t="n">
-        <v>4.37</v>
+        <v>4.01</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BEWLTD</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>58.45</v>
+        <v>48.68</v>
       </c>
       <c r="C53" t="n">
-        <v>61</v>
+        <v>50.6</v>
       </c>
       <c r="D53" t="n">
-        <v>4.36</v>
+        <v>3.94</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>9.48</v>
+        <v>278.2</v>
       </c>
       <c r="C54" t="n">
-        <v>9.890000000000001</v>
+        <v>288.9</v>
       </c>
       <c r="D54" t="n">
-        <v>4.32</v>
+        <v>3.85</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MARALOVER</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>58.48</v>
+        <v>36.5</v>
       </c>
       <c r="C55" t="n">
-        <v>61</v>
+        <v>37.9</v>
       </c>
       <c r="D55" t="n">
-        <v>4.31</v>
+        <v>3.84</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SONA</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>98.78</v>
+        <v>161.85</v>
       </c>
       <c r="C56" t="n">
-        <v>103</v>
+        <v>168</v>
       </c>
       <c r="D56" t="n">
-        <v>4.27</v>
+        <v>3.8</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>AKCAPIT</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>382.7</v>
+        <v>1728.4</v>
       </c>
       <c r="C57" t="n">
-        <v>399</v>
+        <v>1793.9</v>
       </c>
       <c r="D57" t="n">
-        <v>4.26</v>
+        <v>3.79</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>AVPINFRA</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2.59</v>
+        <v>53.5</v>
       </c>
       <c r="C58" t="n">
-        <v>2.7</v>
+        <v>55.5</v>
       </c>
       <c r="D58" t="n">
-        <v>4.25</v>
+        <v>3.74</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ACEVECTOR</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>31.11</v>
+        <v>7666</v>
       </c>
       <c r="C59" t="n">
-        <v>32.42</v>
+        <v>7950</v>
       </c>
       <c r="D59" t="n">
-        <v>4.21</v>
+        <v>3.7</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FINOPB</t>
+          <t>KKCL</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>128.76</v>
+        <v>472.5</v>
       </c>
       <c r="C60" t="n">
-        <v>134</v>
+        <v>489.9</v>
       </c>
       <c r="D60" t="n">
-        <v>4.07</v>
+        <v>3.68</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>52.85</v>
+        <v>259.46</v>
       </c>
       <c r="C61" t="n">
-        <v>55</v>
+        <v>269</v>
       </c>
       <c r="D61" t="n">
-        <v>4.07</v>
+        <v>3.68</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>AERONEU</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>214.34</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="C62" t="n">
-        <v>223</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="D62" t="n">
-        <v>4.04</v>
+        <v>3.65</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>VIJAYPD</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>96.09999999999999</v>
+        <v>68.86</v>
       </c>
       <c r="C63" t="n">
-        <v>99.95</v>
+        <v>71.34</v>
       </c>
       <c r="D63" t="n">
-        <v>4.01</v>
+        <v>3.6</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>22.02</v>
+        <v>18.72</v>
       </c>
       <c r="C64" t="n">
-        <v>22.9</v>
+        <v>19.39</v>
       </c>
       <c r="D64" t="n">
-        <v>4</v>
+        <v>3.58</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>331.8</v>
+        <v>1.43</v>
       </c>
       <c r="C65" t="n">
-        <v>345</v>
+        <v>1.48</v>
       </c>
       <c r="D65" t="n">
-        <v>3.98</v>
+        <v>3.5</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>HEALTHX</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>195.42</v>
+        <v>292.9</v>
       </c>
       <c r="C66" t="n">
-        <v>203.2</v>
+        <v>303</v>
       </c>
       <c r="D66" t="n">
-        <v>3.98</v>
+        <v>3.45</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>OMAXAUTO</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>12.8</v>
+        <v>200.16</v>
       </c>
       <c r="C67" t="n">
-        <v>13.29</v>
+        <v>207</v>
       </c>
       <c r="D67" t="n">
-        <v>3.83</v>
+        <v>3.42</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SOMICONVEY</t>
+          <t>S&amp;SPOWER</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>83.37</v>
+        <v>275.2</v>
       </c>
       <c r="C68" t="n">
-        <v>86.55</v>
+        <v>284.6</v>
       </c>
       <c r="D68" t="n">
-        <v>3.81</v>
+        <v>3.42</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>AZADIND</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>82.84999999999999</v>
+        <v>2.05</v>
       </c>
       <c r="C69" t="n">
-        <v>85.98999999999999</v>
+        <v>2.12</v>
       </c>
       <c r="D69" t="n">
-        <v>3.79</v>
+        <v>3.41</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>19.26</v>
+        <v>25.63</v>
       </c>
       <c r="C70" t="n">
-        <v>19.99</v>
+        <v>26.5</v>
       </c>
       <c r="D70" t="n">
-        <v>3.79</v>
+        <v>3.39</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SUPTANERY</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>8.470000000000001</v>
+        <v>34.63</v>
       </c>
       <c r="C71" t="n">
-        <v>8.789999999999999</v>
+        <v>35.8</v>
       </c>
       <c r="D71" t="n">
-        <v>3.78</v>
+        <v>3.38</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>4.51</v>
+        <v>561.3</v>
       </c>
       <c r="C72" t="n">
-        <v>4.68</v>
+        <v>580</v>
       </c>
       <c r="D72" t="n">
-        <v>3.77</v>
+        <v>3.33</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>UNITEDTEA</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>408.85</v>
+        <v>763</v>
       </c>
       <c r="C73" t="n">
-        <v>424</v>
+        <v>788</v>
       </c>
       <c r="D73" t="n">
-        <v>3.71</v>
+        <v>3.28</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>47.16</v>
+        <v>207.2</v>
       </c>
       <c r="C74" t="n">
-        <v>48.9</v>
+        <v>214</v>
       </c>
       <c r="D74" t="n">
-        <v>3.69</v>
+        <v>3.28</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>NAGREEKCAP</t>
+          <t>DIFFNKG</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>27.25</v>
+        <v>427.25</v>
       </c>
       <c r="C75" t="n">
-        <v>28.25</v>
+        <v>441</v>
       </c>
       <c r="D75" t="n">
-        <v>3.67</v>
+        <v>3.22</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SHIVALIK</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>365.05</v>
+        <v>49.92</v>
       </c>
       <c r="C76" t="n">
-        <v>378.3</v>
+        <v>51.5</v>
       </c>
       <c r="D76" t="n">
-        <v>3.63</v>
+        <v>3.17</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TECHLABS</t>
+          <t>COFFEEDAY</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>111.85</v>
+        <v>30.53</v>
       </c>
       <c r="C77" t="n">
-        <v>115.85</v>
+        <v>31.49</v>
       </c>
       <c r="D77" t="n">
-        <v>3.58</v>
+        <v>3.14</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>BATLIBOI</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>680.55</v>
+        <v>93.98</v>
       </c>
       <c r="C78" t="n">
-        <v>704.9</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="D78" t="n">
-        <v>3.58</v>
+        <v>3.11</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DHABRIYA</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>477.05</v>
+        <v>14.94</v>
       </c>
       <c r="C79" t="n">
-        <v>494</v>
+        <v>15.4</v>
       </c>
       <c r="D79" t="n">
-        <v>3.55</v>
+        <v>3.08</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MUTHOOTMF</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>172.91</v>
+        <v>36</v>
       </c>
       <c r="C80" t="n">
-        <v>179</v>
+        <v>37.09</v>
       </c>
       <c r="D80" t="n">
-        <v>3.52</v>
+        <v>3.03</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>6.55</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C81" t="n">
-        <v>6.78</v>
+        <v>9.99</v>
       </c>
       <c r="D81" t="n">
-        <v>3.51</v>
+        <v>2.99</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>EXCELSOFT</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>81.70999999999999</v>
+        <v>14.08</v>
       </c>
       <c r="C82" t="n">
-        <v>84.56999999999999</v>
+        <v>14.5</v>
       </c>
       <c r="D82" t="n">
-        <v>3.5</v>
+        <v>2.98</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>OSWALGREEN</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>18.99</v>
+        <v>4.36</v>
       </c>
       <c r="C83" t="n">
-        <v>19.65</v>
+        <v>4.49</v>
       </c>
       <c r="D83" t="n">
-        <v>3.48</v>
+        <v>2.98</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>15.37</v>
+        <v>49.51</v>
       </c>
       <c r="C84" t="n">
-        <v>15.9</v>
+        <v>50.98</v>
       </c>
       <c r="D84" t="n">
-        <v>3.45</v>
+        <v>2.97</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ABH</t>
+          <t>KEC</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>47.85</v>
+        <v>349.6</v>
       </c>
       <c r="C85" t="n">
-        <v>49.5</v>
+        <v>360</v>
       </c>
       <c r="D85" t="n">
-        <v>3.45</v>
+        <v>2.97</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>4.95</v>
+        <v>1.69</v>
       </c>
       <c r="C86" t="n">
-        <v>5.12</v>
+        <v>1.74</v>
       </c>
       <c r="D86" t="n">
-        <v>3.43</v>
+        <v>2.96</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>157.4</v>
+        <v>18.11</v>
       </c>
       <c r="C87" t="n">
-        <v>162.8</v>
+        <v>18.64</v>
       </c>
       <c r="D87" t="n">
-        <v>3.43</v>
+        <v>2.93</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>15.62</v>
+        <v>23.71</v>
       </c>
       <c r="C88" t="n">
-        <v>16.15</v>
+        <v>24.39</v>
       </c>
       <c r="D88" t="n">
-        <v>3.39</v>
+        <v>2.87</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PREMIERPOL</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>101.23</v>
+        <v>136.1</v>
       </c>
       <c r="C89" t="n">
-        <v>104.6</v>
+        <v>140</v>
       </c>
       <c r="D89" t="n">
-        <v>3.33</v>
+        <v>2.87</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>JAINREC</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>580.95</v>
+        <v>281.05</v>
       </c>
       <c r="C90" t="n">
-        <v>600</v>
+        <v>289.1</v>
       </c>
       <c r="D90" t="n">
-        <v>3.28</v>
+        <v>2.86</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>COMPINFO</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>76.31</v>
+        <v>1.06</v>
       </c>
       <c r="C91" t="n">
-        <v>78.8</v>
+        <v>1.09</v>
       </c>
       <c r="D91" t="n">
-        <v>3.26</v>
+        <v>2.83</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>KERNEX</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>585</v>
+        <v>1700.5</v>
       </c>
       <c r="C92" t="n">
-        <v>604</v>
+        <v>1748.7</v>
       </c>
       <c r="D92" t="n">
-        <v>3.25</v>
+        <v>2.83</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>DECCANCE</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>31.2</v>
+        <v>532.95</v>
       </c>
       <c r="C93" t="n">
-        <v>32.2</v>
+        <v>548</v>
       </c>
       <c r="D93" t="n">
-        <v>3.21</v>
+        <v>2.82</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>58.33</v>
+        <v>7.18</v>
       </c>
       <c r="C94" t="n">
-        <v>60.2</v>
+        <v>7.38</v>
       </c>
       <c r="D94" t="n">
-        <v>3.21</v>
+        <v>2.79</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>JAIBALAJI</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>67.37</v>
+        <v>197</v>
       </c>
       <c r="C95" t="n">
-        <v>69.5</v>
+        <v>202.5</v>
       </c>
       <c r="D95" t="n">
-        <v>3.16</v>
+        <v>2.79</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BATLIBOI</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>94.8</v>
+        <v>1.44</v>
       </c>
       <c r="C96" t="n">
-        <v>97.8</v>
+        <v>1.48</v>
       </c>
       <c r="D96" t="n">
-        <v>3.16</v>
+        <v>2.78</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>6.01</v>
+        <v>18.77</v>
       </c>
       <c r="C97" t="n">
-        <v>6.2</v>
+        <v>19.29</v>
       </c>
       <c r="D97" t="n">
-        <v>3.16</v>
+        <v>2.77</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>32.2</v>
+        <v>252.6</v>
       </c>
       <c r="C98" t="n">
-        <v>33.2</v>
+        <v>259.5</v>
       </c>
       <c r="D98" t="n">
-        <v>3.11</v>
+        <v>2.73</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>5.87</v>
+        <v>1.83</v>
       </c>
       <c r="C99" t="n">
-        <v>6.05</v>
+        <v>1.88</v>
       </c>
       <c r="D99" t="n">
-        <v>3.07</v>
+        <v>2.73</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>87.94</v>
+        <v>1041.5</v>
       </c>
       <c r="C100" t="n">
-        <v>90.59999999999999</v>
+        <v>1069.8</v>
       </c>
       <c r="D100" t="n">
-        <v>3.02</v>
+        <v>2.72</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CORDELIA</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>109.52</v>
+        <v>873.4</v>
       </c>
       <c r="C101" t="n">
-        <v>112.76</v>
+        <v>896.8</v>
       </c>
       <c r="D101" t="n">
-        <v>2.96</v>
+        <v>2.68</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1127</v>
+        <v>14.6</v>
       </c>
       <c r="C102" t="n">
-        <v>1159.9</v>
+        <v>14.99</v>
       </c>
       <c r="D102" t="n">
-        <v>2.92</v>
+        <v>2.67</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>7.53</v>
+        <v>5.25</v>
       </c>
       <c r="C103" t="n">
-        <v>7.75</v>
+        <v>5.39</v>
       </c>
       <c r="D103" t="n">
-        <v>2.92</v>
+        <v>2.67</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BELLACASA</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>251.77</v>
+        <v>608.6</v>
       </c>
       <c r="C104" t="n">
-        <v>259</v>
+        <v>624.8</v>
       </c>
       <c r="D104" t="n">
-        <v>2.87</v>
+        <v>2.66</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ARCIL</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>160.31</v>
+        <v>19.97</v>
       </c>
       <c r="C105" t="n">
-        <v>164.9</v>
+        <v>20.5</v>
       </c>
       <c r="D105" t="n">
-        <v>2.86</v>
+        <v>2.65</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>TECHNVISN</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>100.62</v>
+        <v>4384.5</v>
       </c>
       <c r="C106" t="n">
-        <v>103.5</v>
+        <v>4500</v>
       </c>
       <c r="D106" t="n">
-        <v>2.86</v>
+        <v>2.63</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>MAFATIND</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>723.3</v>
+        <v>111.07</v>
       </c>
       <c r="C107" t="n">
-        <v>744</v>
+        <v>113.97</v>
       </c>
       <c r="D107" t="n">
-        <v>2.86</v>
+        <v>2.61</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.71</v>
+        <v>6.12</v>
       </c>
       <c r="C108" t="n">
-        <v>0.73</v>
+        <v>6.28</v>
       </c>
       <c r="D108" t="n">
-        <v>2.82</v>
+        <v>2.61</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>45.71</v>
+        <v>14.23</v>
       </c>
       <c r="C109" t="n">
-        <v>47</v>
+        <v>14.6</v>
       </c>
       <c r="D109" t="n">
-        <v>2.82</v>
+        <v>2.6</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1.43</v>
+        <v>25.14</v>
       </c>
       <c r="C110" t="n">
-        <v>1.47</v>
+        <v>25.79</v>
       </c>
       <c r="D110" t="n">
-        <v>2.8</v>
+        <v>2.59</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>GOACARBON</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>12.5</v>
+        <v>394.8</v>
       </c>
       <c r="C111" t="n">
-        <v>12.85</v>
+        <v>405</v>
       </c>
       <c r="D111" t="n">
-        <v>2.8</v>
+        <v>2.58</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>HINDALUMI</t>
+          <t>CENTRUM</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>89.98999999999999</v>
+        <v>19.44</v>
       </c>
       <c r="C112" t="n">
-        <v>92.5</v>
+        <v>19.94</v>
       </c>
       <c r="D112" t="n">
-        <v>2.79</v>
+        <v>2.57</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>35.22</v>
+        <v>177.5</v>
       </c>
       <c r="C113" t="n">
-        <v>36.2</v>
+        <v>182</v>
       </c>
       <c r="D113" t="n">
-        <v>2.78</v>
+        <v>2.54</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>GMBREW</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.36</v>
+        <v>887.45</v>
       </c>
       <c r="C114" t="n">
-        <v>0.37</v>
+        <v>910</v>
       </c>
       <c r="D114" t="n">
-        <v>2.78</v>
+        <v>2.54</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>JITFINFRA</t>
+          <t>BHANDARI</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>278.3</v>
+        <v>2.76</v>
       </c>
       <c r="C115" t="n">
-        <v>286</v>
+        <v>2.83</v>
       </c>
       <c r="D115" t="n">
-        <v>2.77</v>
+        <v>2.54</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2.18</v>
+        <v>152.17</v>
       </c>
       <c r="C116" t="n">
-        <v>2.24</v>
+        <v>156</v>
       </c>
       <c r="D116" t="n">
-        <v>2.75</v>
+        <v>2.52</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>JTLIND</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>88.2</v>
+        <v>31.22</v>
       </c>
       <c r="C117" t="n">
-        <v>90.62</v>
+        <v>32</v>
       </c>
       <c r="D117" t="n">
-        <v>2.74</v>
+        <v>2.5</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>PAUSHAKLTD</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>225.66</v>
+        <v>671.65</v>
       </c>
       <c r="C118" t="n">
-        <v>231.83</v>
+        <v>688.35</v>
       </c>
       <c r="D118" t="n">
-        <v>2.73</v>
+        <v>2.49</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KOKUYOCMLN</t>
+          <t>INVENTURE</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>73</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C119" t="n">
-        <v>74.98999999999999</v>
+        <v>0.83</v>
       </c>
       <c r="D119" t="n">
-        <v>2.73</v>
+        <v>2.47</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>DISHTV</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>2657.9</v>
+        <v>2.03</v>
       </c>
       <c r="C120" t="n">
-        <v>2730</v>
+        <v>2.08</v>
       </c>
       <c r="D120" t="n">
-        <v>2.71</v>
+        <v>2.46</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>AUSOMENT</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>698.15</v>
+        <v>143.29</v>
       </c>
       <c r="C121" t="n">
-        <v>717</v>
+        <v>146.8</v>
       </c>
       <c r="D121" t="n">
-        <v>2.7</v>
+        <v>2.45</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KOTYARK</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>31.1</v>
+        <v>6.23</v>
       </c>
       <c r="C122" t="n">
-        <v>31.94</v>
+        <v>6.38</v>
       </c>
       <c r="D122" t="n">
-        <v>2.7</v>
+        <v>2.41</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>BIRLACORPN</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>57.75</v>
+        <v>794.85</v>
       </c>
       <c r="C123" t="n">
-        <v>59.29</v>
+        <v>814</v>
       </c>
       <c r="D123" t="n">
-        <v>2.67</v>
+        <v>2.41</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>MOKSH</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>13.14</v>
+        <v>9.17</v>
       </c>
       <c r="C124" t="n">
-        <v>13.49</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="D124" t="n">
-        <v>2.66</v>
+        <v>2.4</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ASIANHOTNR</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>330.25</v>
+        <v>40.63</v>
       </c>
       <c r="C125" t="n">
-        <v>339</v>
+        <v>41.6</v>
       </c>
       <c r="D125" t="n">
-        <v>2.65</v>
+        <v>2.39</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>TCPLPACK</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>498.8</v>
+        <v>3994.4</v>
       </c>
       <c r="C126" t="n">
-        <v>512</v>
+        <v>4090</v>
       </c>
       <c r="D126" t="n">
-        <v>2.65</v>
+        <v>2.39</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SICAGEN</t>
+          <t>KHAICHEM</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>51.53</v>
+        <v>47.6</v>
       </c>
       <c r="C127" t="n">
-        <v>52.89</v>
+        <v>48.73</v>
       </c>
       <c r="D127" t="n">
-        <v>2.64</v>
+        <v>2.37</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ELIN</t>
+          <t>JITFINFRA</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>77.06999999999999</v>
+        <v>269.55</v>
       </c>
       <c r="C128" t="n">
-        <v>79.09999999999999</v>
+        <v>275.9</v>
       </c>
       <c r="D128" t="n">
-        <v>2.63</v>
+        <v>2.36</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>BAJAJST</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>33.14</v>
+        <v>324.3</v>
       </c>
       <c r="C129" t="n">
-        <v>34</v>
+        <v>331.95</v>
       </c>
       <c r="D129" t="n">
-        <v>2.6</v>
+        <v>2.36</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>ELECTHERM</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>142.71</v>
+        <v>683.75</v>
       </c>
       <c r="C130" t="n">
-        <v>146.4</v>
+        <v>699.9</v>
       </c>
       <c r="D130" t="n">
-        <v>2.59</v>
+        <v>2.36</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>JAYBARMARU</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>132.78</v>
+        <v>8.09</v>
       </c>
       <c r="C131" t="n">
-        <v>136.2</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D131" t="n">
-        <v>2.58</v>
+        <v>2.35</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ALPEXSOLAR</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>815.1</v>
+        <v>0.43</v>
       </c>
       <c r="C132" t="n">
-        <v>836</v>
+        <v>0.44</v>
       </c>
       <c r="D132" t="n">
-        <v>2.56</v>
+        <v>2.33</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>ARCHIES</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>165.75</v>
+        <v>12.01</v>
       </c>
       <c r="C133" t="n">
-        <v>170</v>
+        <v>12.29</v>
       </c>
       <c r="D133" t="n">
-        <v>2.56</v>
+        <v>2.33</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>NELCAST</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>146.29</v>
+        <v>0.87</v>
       </c>
       <c r="C134" t="n">
-        <v>150</v>
+        <v>0.89</v>
       </c>
       <c r="D134" t="n">
-        <v>2.54</v>
+        <v>2.3</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CALSOFT</t>
+          <t>BAJAJINDEF</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>35.11</v>
+        <v>199.24</v>
       </c>
       <c r="C135" t="n">
-        <v>36</v>
+        <v>203.8</v>
       </c>
       <c r="D135" t="n">
-        <v>2.53</v>
+        <v>2.29</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ALOKINDS</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>8.289999999999999</v>
+        <v>12.79</v>
       </c>
       <c r="C136" t="n">
-        <v>8.5</v>
+        <v>13.08</v>
       </c>
       <c r="D136" t="n">
-        <v>2.53</v>
+        <v>2.27</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>RENTOMOJO</t>
+          <t>AVATAR</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>618.95</v>
+        <v>183.75</v>
       </c>
       <c r="C137" t="n">
-        <v>634.5</v>
+        <v>187.9</v>
       </c>
       <c r="D137" t="n">
-        <v>2.51</v>
+        <v>2.26</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>MMTC</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>377.55</v>
+        <v>54.27</v>
       </c>
       <c r="C138" t="n">
-        <v>387</v>
+        <v>55.49</v>
       </c>
       <c r="D138" t="n">
-        <v>2.5</v>
+        <v>2.25</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>HBPOR</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>62.36</v>
+        <v>3.13</v>
       </c>
       <c r="C139" t="n">
-        <v>63.91</v>
+        <v>3.2</v>
       </c>
       <c r="D139" t="n">
-        <v>2.49</v>
+        <v>2.24</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>3.22</v>
+        <v>13.9</v>
       </c>
       <c r="C140" t="n">
-        <v>3.3</v>
+        <v>14.21</v>
       </c>
       <c r="D140" t="n">
-        <v>2.48</v>
+        <v>2.23</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>26.11</v>
+        <v>1.8</v>
       </c>
       <c r="C141" t="n">
-        <v>26.75</v>
+        <v>1.84</v>
       </c>
       <c r="D141" t="n">
-        <v>2.45</v>
+        <v>2.22</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>RAJOOENG</t>
+          <t>CRIZAC</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>62.37</v>
+        <v>159.97</v>
       </c>
       <c r="C142" t="n">
-        <v>63.9</v>
+        <v>163.5</v>
       </c>
       <c r="D142" t="n">
-        <v>2.45</v>
+        <v>2.21</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>BAIDFIN</t>
+          <t>EPACKPEB</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>10.21</v>
+        <v>256.33</v>
       </c>
       <c r="C143" t="n">
-        <v>10.46</v>
+        <v>262</v>
       </c>
       <c r="D143" t="n">
-        <v>2.45</v>
+        <v>2.21</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>THEINVEST</t>
+          <t>TRIVENI</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>90.2</v>
+        <v>237.86</v>
       </c>
       <c r="C144" t="n">
-        <v>92.40000000000001</v>
+        <v>243.1</v>
       </c>
       <c r="D144" t="n">
-        <v>2.44</v>
+        <v>2.2</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>VEEGALAND</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.84</v>
+        <v>136.9</v>
       </c>
       <c r="C145" t="n">
-        <v>0.86</v>
+        <v>139.9</v>
       </c>
       <c r="D145" t="n">
-        <v>2.38</v>
+        <v>2.19</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>MOHITIND</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>49.43</v>
+        <v>22.01</v>
       </c>
       <c r="C146" t="n">
-        <v>50.6</v>
+        <v>22.49</v>
       </c>
       <c r="D146" t="n">
-        <v>2.37</v>
+        <v>2.18</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>TOLINS</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>1270.1</v>
+        <v>86.56</v>
       </c>
       <c r="C147" t="n">
-        <v>1300</v>
+        <v>88.45</v>
       </c>
       <c r="D147" t="n">
-        <v>2.35</v>
+        <v>2.18</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>1484.2</v>
+        <v>0.46</v>
       </c>
       <c r="C148" t="n">
-        <v>1519</v>
+        <v>0.47</v>
       </c>
       <c r="D148" t="n">
-        <v>2.34</v>
+        <v>2.17</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>AURUS</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>4.29</v>
+        <v>46.44</v>
       </c>
       <c r="C149" t="n">
-        <v>4.39</v>
+        <v>47.45</v>
       </c>
       <c r="D149" t="n">
-        <v>2.33</v>
+        <v>2.17</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>199.38</v>
+        <v>1.84</v>
       </c>
       <c r="C150" t="n">
-        <v>204</v>
+        <v>1.88</v>
       </c>
       <c r="D150" t="n">
-        <v>2.32</v>
+        <v>2.17</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MOMSBELIEF</t>
+          <t>AUTOIND</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>229.68</v>
+        <v>80.06</v>
       </c>
       <c r="C151" t="n">
-        <v>234.89</v>
+        <v>81.8</v>
       </c>
       <c r="D151" t="n">
-        <v>2.27</v>
+        <v>2.17</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>DIGIDRIVE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>91.81999999999999</v>
+        <v>17.51</v>
       </c>
       <c r="C152" t="n">
-        <v>93.90000000000001</v>
+        <v>17.89</v>
       </c>
       <c r="D152" t="n">
-        <v>2.27</v>
+        <v>2.17</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>MANBA</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>1.76</v>
+        <v>146.82</v>
       </c>
       <c r="C153" t="n">
-        <v>1.8</v>
+        <v>150</v>
       </c>
       <c r="D153" t="n">
-        <v>2.27</v>
+        <v>2.17</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>0.44</v>
+        <v>5.56</v>
       </c>
       <c r="C154" t="n">
-        <v>0.45</v>
+        <v>5.68</v>
       </c>
       <c r="D154" t="n">
-        <v>2.27</v>
+        <v>2.16</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>MATRIMONY</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>517.5</v>
+        <v>861.4</v>
       </c>
       <c r="C155" t="n">
-        <v>529.05</v>
+        <v>880</v>
       </c>
       <c r="D155" t="n">
-        <v>2.23</v>
+        <v>2.16</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>28.32</v>
+        <v>44.48</v>
       </c>
       <c r="C156" t="n">
-        <v>28.95</v>
+        <v>45.44</v>
       </c>
       <c r="D156" t="n">
-        <v>2.22</v>
+        <v>2.16</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>WEWIN</t>
+          <t>APEXECO</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>52.85</v>
+        <v>246.3</v>
       </c>
       <c r="C157" t="n">
-        <v>54</v>
+        <v>251.6</v>
       </c>
       <c r="D157" t="n">
-        <v>2.18</v>
+        <v>2.15</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ASMS</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>5.95</v>
+        <v>20.55</v>
       </c>
       <c r="C158" t="n">
-        <v>6.08</v>
+        <v>20.99</v>
       </c>
       <c r="D158" t="n">
-        <v>2.18</v>
+        <v>2.14</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SWISSMLTRY</t>
+          <t>SAMPANN</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>14.19</v>
+        <v>23.78</v>
       </c>
       <c r="C159" t="n">
-        <v>14.5</v>
+        <v>24.29</v>
       </c>
       <c r="D159" t="n">
-        <v>2.18</v>
+        <v>2.14</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MERCURYEV</t>
+          <t>SWSOLAR</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>37.88</v>
+        <v>160.09</v>
       </c>
       <c r="C160" t="n">
-        <v>38.7</v>
+        <v>163.5</v>
       </c>
       <c r="D160" t="n">
-        <v>2.16</v>
+        <v>2.13</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>THOMASCOTT</t>
+          <t>GALLANTT</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>278.85</v>
+        <v>503.15</v>
       </c>
       <c r="C161" t="n">
-        <v>284.85</v>
+        <v>513.8</v>
       </c>
       <c r="D161" t="n">
-        <v>2.15</v>
+        <v>2.12</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,14 +3981,14 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>DRONE</t>
+          <t>CENTUM</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>33.05</v>
+        <v>4142.1</v>
       </c>
       <c r="C162" t="n">
-        <v>33.75</v>
+        <v>4230</v>
       </c>
       <c r="D162" t="n">
         <v>2.12</v>
@@ -4003,14 +4003,14 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>4.25</v>
+        <v>108.11</v>
       </c>
       <c r="C163" t="n">
-        <v>4.34</v>
+        <v>110.4</v>
       </c>
       <c r="D163" t="n">
         <v>2.12</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ZIMLAB</t>
+          <t>MUFTI</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>146.61</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="C164" t="n">
-        <v>149.69</v>
+        <v>69.7</v>
       </c>
       <c r="D164" t="n">
-        <v>2.1</v>
+        <v>2.11</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>1.91</v>
+        <v>37.21</v>
       </c>
       <c r="C165" t="n">
-        <v>1.95</v>
+        <v>37.99</v>
       </c>
       <c r="D165" t="n">
-        <v>2.09</v>
+        <v>2.1</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>CENTEXT</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>58.78</v>
+        <v>18.6</v>
       </c>
       <c r="C166" t="n">
-        <v>60</v>
+        <v>18.99</v>
       </c>
       <c r="D166" t="n">
-        <v>2.08</v>
+        <v>2.1</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>13.11</v>
+        <v>31.63</v>
       </c>
       <c r="C167" t="n">
-        <v>13.38</v>
+        <v>32.29</v>
       </c>
       <c r="D167" t="n">
-        <v>2.06</v>
+        <v>2.09</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ESAFSFB</t>
+          <t>GTL</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>42.67</v>
+        <v>6.71</v>
       </c>
       <c r="C168" t="n">
-        <v>43.54</v>
+        <v>6.85</v>
       </c>
       <c r="D168" t="n">
-        <v>2.04</v>
+        <v>2.09</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ADVIKCA</t>
+          <t>HIGREEN</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0.98</v>
+        <v>119.35</v>
       </c>
       <c r="C169" t="n">
-        <v>1</v>
+        <v>121.8</v>
       </c>
       <c r="D169" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>ADVIKCA</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>9.4</v>
+        <v>0.98</v>
       </c>
       <c r="C170" t="n">
-        <v>9.59</v>
+        <v>1</v>
       </c>
       <c r="D170" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>TGBHOTELS</t>
+          <t>PRISMX</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>9.4</v>
+        <v>0.49</v>
       </c>
       <c r="C171" t="n">
-        <v>9.59</v>
+        <v>0.5</v>
       </c>
       <c r="D171" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>ONWARDTEC</t>
+          <t>THERMAX</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>297.4</v>
+        <v>3138.1</v>
       </c>
       <c r="C172" t="n">
-        <v>303.4</v>
+        <v>3202</v>
       </c>
       <c r="D172" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>MIDWESTLTD</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>12.96</v>
+        <v>989.8</v>
       </c>
       <c r="C173" t="n">
-        <v>13.22</v>
+        <v>1010</v>
       </c>
       <c r="D173" t="n">
-        <v>2.01</v>
+        <v>2.04</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>367.6</v>
+        <v>20.17</v>
       </c>
       <c r="C174" t="n">
-        <v>375</v>
+        <v>20.58</v>
       </c>
       <c r="D174" t="n">
-        <v>2.01</v>
+        <v>2.03</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>26.36</v>
+        <v>15.77</v>
       </c>
       <c r="C175" t="n">
-        <v>26.89</v>
+        <v>16.09</v>
       </c>
       <c r="D175" t="n">
-        <v>2.01</v>
+        <v>2.03</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>AUGMONT</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>16.91</v>
+        <v>1274.1</v>
       </c>
       <c r="C176" t="n">
-        <v>17.25</v>
+        <v>1300</v>
       </c>
       <c r="D176" t="n">
-        <v>2.01</v>
+        <v>2.03</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>50.48</v>
+        <v>11.91</v>
       </c>
       <c r="C177" t="n">
-        <v>51.49</v>
+        <v>12.15</v>
       </c>
       <c r="D177" t="n">
-        <v>2</v>
+        <v>2.02</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ANMOL</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>13.03</v>
+        <v>199.47</v>
       </c>
       <c r="C178" t="n">
-        <v>13.29</v>
+        <v>203.5</v>
       </c>
       <c r="D178" t="n">
-        <v>2</v>
+        <v>2.02</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>92.64</v>
+        <v>53.75</v>
       </c>
       <c r="C179" t="n">
-        <v>94.48999999999999</v>
+        <v>54.83</v>
       </c>
       <c r="D179" t="n">
-        <v>2</v>
+        <v>2.01</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SPECTRAA</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>272.55</v>
+        <v>76.26000000000001</v>
       </c>
       <c r="C180" t="n">
-        <v>278</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="D180" t="n">
-        <v>2</v>
+        <v>2.01</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,14 +4399,14 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>BALPHARMA</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>98.62</v>
+        <v>0.5</v>
       </c>
       <c r="C181" t="n">
-        <v>100.59</v>
+        <v>0.51</v>
       </c>
       <c r="D181" t="n">
         <v>2</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>NOVAAGRI</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>33.09</v>
+        <v>21.95</v>
       </c>
       <c r="C182" t="n">
-        <v>33.75</v>
+        <v>22.39</v>
       </c>
       <c r="D182" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MUTHOOTCAP</t>
+          <t>GEECEE</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>213.53</v>
+        <v>352.7</v>
       </c>
       <c r="C183" t="n">
-        <v>217.78</v>
+        <v>359.75</v>
       </c>
       <c r="D183" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,14 +4465,14 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>24.18</v>
+        <v>483.25</v>
       </c>
       <c r="C184" t="n">
-        <v>24.66</v>
+        <v>492.85</v>
       </c>
       <c r="D184" t="n">
         <v>1.99</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>VHL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>173.9</v>
+        <v>3578.8</v>
       </c>
       <c r="C185" t="n">
-        <v>177.35</v>
+        <v>3650</v>
       </c>
       <c r="D185" t="n">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>LOVABLE</t>
+          <t>ORIENTCABL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>68.73</v>
+        <v>386.85</v>
       </c>
       <c r="C186" t="n">
-        <v>70.09</v>
+        <v>394.55</v>
       </c>
       <c r="D186" t="n">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>AMJLAND</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>215.12</v>
+        <v>36.66</v>
       </c>
       <c r="C187" t="n">
-        <v>219.39</v>
+        <v>37.39</v>
       </c>
       <c r="D187" t="n">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,14 +4553,14 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SASKEN</t>
+          <t>MSL</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>1665.1</v>
+        <v>136.69</v>
       </c>
       <c r="C188" t="n">
-        <v>1698</v>
+        <v>139.39</v>
       </c>
       <c r="D188" t="n">
         <v>1.98</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>MEGASTAR</t>
+          <t>PHOENXINTL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>309.06</v>
+        <v>27.84</v>
       </c>
       <c r="C189" t="n">
-        <v>315.15</v>
+        <v>28.39</v>
       </c>
       <c r="D189" t="n">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ARCHIDPLY</t>
+          <t>EFCIL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>102.73</v>
+        <v>167.07</v>
       </c>
       <c r="C190" t="n">
-        <v>104.75</v>
+        <v>170.38</v>
       </c>
       <c r="D190" t="n">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>631</v>
+        <v>7.58</v>
       </c>
       <c r="C191" t="n">
-        <v>643.4</v>
+        <v>7.73</v>
       </c>
       <c r="D191" t="n">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>653.25</v>
+        <v>54.9</v>
       </c>
       <c r="C192" t="n">
-        <v>666</v>
+        <v>55.98</v>
       </c>
       <c r="D192" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>CEMPRO</t>
+          <t>CGVAK</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>1137.8</v>
+        <v>137.73</v>
       </c>
       <c r="C193" t="n">
-        <v>1160</v>
+        <v>140.45</v>
       </c>
       <c r="D193" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>NTCIND</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>3.61</v>
+        <v>135.03</v>
       </c>
       <c r="C194" t="n">
-        <v>3.68</v>
+        <v>137.69</v>
       </c>
       <c r="D194" t="n">
-        <v>1.94</v>
+        <v>1.97</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>KUSUMGAR</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>1.55</v>
+        <v>608</v>
       </c>
       <c r="C195" t="n">
-        <v>1.58</v>
+        <v>620</v>
       </c>
       <c r="D195" t="n">
-        <v>1.94</v>
+        <v>1.97</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CRSL</t>
+          <t>DCI</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>2.06</v>
+        <v>345.2</v>
       </c>
       <c r="C196" t="n">
-        <v>2.1</v>
+        <v>352</v>
       </c>
       <c r="D196" t="n">
-        <v>1.94</v>
+        <v>1.97</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>31.37</v>
+        <v>20.81</v>
       </c>
       <c r="C197" t="n">
-        <v>31.98</v>
+        <v>21.22</v>
       </c>
       <c r="D197" t="n">
-        <v>1.94</v>
+        <v>1.97</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ITTL</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>61.9</v>
+        <v>4.57</v>
       </c>
       <c r="C198" t="n">
-        <v>63.1</v>
+        <v>4.66</v>
       </c>
       <c r="D198" t="n">
-        <v>1.94</v>
+        <v>1.97</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>CEIGALL</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>372.8</v>
+        <v>47.56</v>
       </c>
       <c r="C199" t="n">
-        <v>380</v>
+        <v>48.49</v>
       </c>
       <c r="D199" t="n">
-        <v>1.93</v>
+        <v>1.96</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>LFIC</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>1032.45</v>
+        <v>126.22</v>
       </c>
       <c r="C200" t="n">
-        <v>1052.4</v>
+        <v>128.69</v>
       </c>
       <c r="D200" t="n">
-        <v>1.93</v>
+        <v>1.96</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>NGIL</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>56.5</v>
+        <v>37.75</v>
       </c>
       <c r="C201" t="n">
-        <v>57.59</v>
+        <v>38.49</v>
       </c>
       <c r="D201" t="n">
-        <v>1.93</v>
+        <v>1.96</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-12 11:19 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>TERAI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13.82</v>
+        <v>140.01</v>
       </c>
       <c r="C2" t="n">
-        <v>16.4</v>
+        <v>168</v>
       </c>
       <c r="D2" t="n">
-        <v>18.67</v>
+        <v>19.99</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>AMAL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.41</v>
+        <v>764.95</v>
       </c>
       <c r="C3" t="n">
-        <v>1.59</v>
+        <v>851</v>
       </c>
       <c r="D3" t="n">
-        <v>12.77</v>
+        <v>11.25</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5.61</v>
+        <v>41.23</v>
       </c>
       <c r="C4" t="n">
-        <v>6.14</v>
+        <v>45.35</v>
       </c>
       <c r="D4" t="n">
-        <v>9.449999999999999</v>
+        <v>9.99</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CEDAAR</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.7</v>
+        <v>95.7</v>
       </c>
       <c r="C5" t="n">
-        <v>13.9</v>
+        <v>105</v>
       </c>
       <c r="D5" t="n">
-        <v>9.449999999999999</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>BNAGROCHEM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>195.4</v>
+        <v>179.56</v>
       </c>
       <c r="C6" t="n">
-        <v>213</v>
+        <v>196.95</v>
       </c>
       <c r="D6" t="n">
-        <v>9.01</v>
+        <v>9.68</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GLOBALE</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11.53</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>12.55</v>
+        <v>2.19</v>
       </c>
       <c r="D7" t="n">
-        <v>8.85</v>
+        <v>9.5</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>63MOONS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>69.45999999999999</v>
+        <v>766.3</v>
       </c>
       <c r="C8" t="n">
-        <v>74.90000000000001</v>
+        <v>838.3</v>
       </c>
       <c r="D8" t="n">
-        <v>7.83</v>
+        <v>9.4</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.13</v>
+        <v>1.03</v>
       </c>
       <c r="C9" t="n">
-        <v>0.14</v>
+        <v>1.12</v>
       </c>
       <c r="D9" t="n">
-        <v>7.69</v>
+        <v>8.74</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BSHSL</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78.36</v>
+        <v>214.94</v>
       </c>
       <c r="C10" t="n">
-        <v>83.95</v>
+        <v>233.6</v>
       </c>
       <c r="D10" t="n">
-        <v>7.13</v>
+        <v>8.68</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>364.85</v>
+        <v>32</v>
       </c>
       <c r="C11" t="n">
-        <v>390</v>
+        <v>34.5</v>
       </c>
       <c r="D11" t="n">
-        <v>6.89</v>
+        <v>7.81</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CUDML</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>87.2</v>
+        <v>0.13</v>
       </c>
       <c r="C12" t="n">
-        <v>93</v>
+        <v>0.14</v>
       </c>
       <c r="D12" t="n">
-        <v>6.65</v>
+        <v>7.69</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20.63</v>
+        <v>57.95</v>
       </c>
       <c r="C13" t="n">
-        <v>22</v>
+        <v>62.28</v>
       </c>
       <c r="D13" t="n">
-        <v>6.64</v>
+        <v>7.47</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.84</v>
+        <v>15.86</v>
       </c>
       <c r="C14" t="n">
-        <v>17.76</v>
+        <v>17</v>
       </c>
       <c r="D14" t="n">
-        <v>5.46</v>
+        <v>7.19</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28.45</v>
+        <v>5.46</v>
       </c>
       <c r="C15" t="n">
-        <v>30</v>
+        <v>5.85</v>
       </c>
       <c r="D15" t="n">
-        <v>5.45</v>
+        <v>7.14</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>AGL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.31</v>
+        <v>12.24</v>
       </c>
       <c r="C16" t="n">
-        <v>1.38</v>
+        <v>13.11</v>
       </c>
       <c r="D16" t="n">
-        <v>5.34</v>
+        <v>7.11</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AATMAJ</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>22.95</v>
+        <v>142.72</v>
       </c>
       <c r="C17" t="n">
-        <v>24.15</v>
+        <v>152.45</v>
       </c>
       <c r="D17" t="n">
-        <v>5.23</v>
+        <v>6.82</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BNAGROCHEM</t>
+          <t>POONAWALLA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>199.39</v>
+        <v>447.3</v>
       </c>
       <c r="C18" t="n">
-        <v>209.65</v>
+        <v>476.9</v>
       </c>
       <c r="D18" t="n">
-        <v>5.15</v>
+        <v>6.62</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SIMCA</t>
+          <t>IVP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>338</v>
+        <v>220.31</v>
       </c>
       <c r="C19" t="n">
-        <v>354.9</v>
+        <v>234.8</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>6.58</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>ALFREDHE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>89.05</v>
+        <v>2650</v>
       </c>
       <c r="C20" t="n">
-        <v>93.5</v>
+        <v>2819.9</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>6.41</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MOBILISE</t>
+          <t>CORDELIA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>103.25</v>
+        <v>100.98</v>
       </c>
       <c r="C21" t="n">
-        <v>108.4</v>
+        <v>107.32</v>
       </c>
       <c r="D21" t="n">
-        <v>4.99</v>
+        <v>6.28</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>AUSTENG</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>32.76</v>
+        <v>153.38</v>
       </c>
       <c r="C22" t="n">
-        <v>34.39</v>
+        <v>163</v>
       </c>
       <c r="D22" t="n">
-        <v>4.98</v>
+        <v>6.27</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NOIDATOLL</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3.83</v>
+        <v>6.19</v>
       </c>
       <c r="C23" t="n">
-        <v>4.02</v>
+        <v>6.57</v>
       </c>
       <c r="D23" t="n">
-        <v>4.96</v>
+        <v>6.14</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>TWCGOLDETF</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>12.72</v>
+        <v>147.96</v>
       </c>
       <c r="C24" t="n">
-        <v>13.35</v>
+        <v>156.83</v>
       </c>
       <c r="D24" t="n">
-        <v>4.95</v>
+        <v>5.99</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>41.4</v>
+        <v>14.13</v>
       </c>
       <c r="C25" t="n">
-        <v>43.45</v>
+        <v>14.96</v>
       </c>
       <c r="D25" t="n">
-        <v>4.95</v>
+        <v>5.87</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>ESFL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6.91</v>
+        <v>116.2</v>
       </c>
       <c r="C26" t="n">
-        <v>7.25</v>
+        <v>123</v>
       </c>
       <c r="D26" t="n">
-        <v>4.92</v>
+        <v>5.85</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8.15</v>
+        <v>817.85</v>
       </c>
       <c r="C27" t="n">
-        <v>8.550000000000001</v>
+        <v>864.9</v>
       </c>
       <c r="D27" t="n">
-        <v>4.91</v>
+        <v>5.75</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ROXHITECH</t>
+          <t>BELDING</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>65.34999999999999</v>
+        <v>913.35</v>
       </c>
       <c r="C28" t="n">
-        <v>68.55</v>
+        <v>965</v>
       </c>
       <c r="D28" t="n">
-        <v>4.9</v>
+        <v>5.66</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>7.34</v>
+        <v>0.18</v>
       </c>
       <c r="C29" t="n">
-        <v>7.7</v>
+        <v>0.19</v>
       </c>
       <c r="D29" t="n">
-        <v>4.9</v>
+        <v>5.56</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SINTERCOM</t>
+          <t>DHRUV</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>73.41</v>
+        <v>23.03</v>
       </c>
       <c r="C30" t="n">
-        <v>77</v>
+        <v>24.3</v>
       </c>
       <c r="D30" t="n">
-        <v>4.89</v>
+        <v>5.51</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7.99</v>
+        <v>15.62</v>
       </c>
       <c r="C31" t="n">
-        <v>8.380000000000001</v>
+        <v>16.47</v>
       </c>
       <c r="D31" t="n">
-        <v>4.88</v>
+        <v>5.44</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>EMKAY</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>265.65</v>
+        <v>16.58</v>
       </c>
       <c r="C32" t="n">
-        <v>278.6</v>
+        <v>17.45</v>
       </c>
       <c r="D32" t="n">
-        <v>4.87</v>
+        <v>5.25</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KICL</t>
+          <t>BAJEL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4692</v>
+        <v>157.26</v>
       </c>
       <c r="C33" t="n">
-        <v>4919</v>
+        <v>165.5</v>
       </c>
       <c r="D33" t="n">
-        <v>4.84</v>
+        <v>5.24</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>SEPC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2.48</v>
+        <v>5.28</v>
       </c>
       <c r="C34" t="n">
-        <v>2.6</v>
+        <v>5.55</v>
       </c>
       <c r="D34" t="n">
-        <v>4.84</v>
+        <v>5.11</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>STARTECK</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>264.25</v>
+        <v>7.9</v>
       </c>
       <c r="C35" t="n">
-        <v>276.95</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D35" t="n">
-        <v>4.81</v>
+        <v>5.06</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>27.44</v>
+        <v>142.9</v>
       </c>
       <c r="C36" t="n">
-        <v>28.75</v>
+        <v>150.04</v>
       </c>
       <c r="D36" t="n">
-        <v>4.77</v>
+        <v>5</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CEWATER</t>
+          <t>BMISL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>254.8</v>
+        <v>139.1</v>
       </c>
       <c r="C37" t="n">
-        <v>266.9</v>
+        <v>146.05</v>
       </c>
       <c r="D37" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>10.01</v>
+        <v>38.5</v>
       </c>
       <c r="C38" t="n">
-        <v>10.48</v>
+        <v>40.42</v>
       </c>
       <c r="D38" t="n">
-        <v>4.7</v>
+        <v>4.99</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>21STCENMGM</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>41.07</v>
+        <v>50.06</v>
       </c>
       <c r="C39" t="n">
-        <v>42.95</v>
+        <v>52.56</v>
       </c>
       <c r="D39" t="n">
-        <v>4.58</v>
+        <v>4.99</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>SIMCA</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>45.92</v>
+        <v>354.9</v>
       </c>
       <c r="C40" t="n">
-        <v>48</v>
+        <v>372.6</v>
       </c>
       <c r="D40" t="n">
-        <v>4.53</v>
+        <v>4.99</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HBPOR</t>
+          <t>XTRANET</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>61.99</v>
+        <v>287.5</v>
       </c>
       <c r="C41" t="n">
-        <v>64.75</v>
+        <v>301.85</v>
       </c>
       <c r="D41" t="n">
-        <v>4.45</v>
+        <v>4.99</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DOLPHIN</t>
+          <t>EEPL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>620.05</v>
+        <v>139.65</v>
       </c>
       <c r="C42" t="n">
-        <v>647.6</v>
+        <v>146.6</v>
       </c>
       <c r="D42" t="n">
-        <v>4.44</v>
+        <v>4.98</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3.39</v>
+        <v>13.46</v>
       </c>
       <c r="C43" t="n">
-        <v>3.54</v>
+        <v>14.13</v>
       </c>
       <c r="D43" t="n">
-        <v>4.42</v>
+        <v>4.98</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AXIOMGAS</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>44.1</v>
+        <v>28.11</v>
       </c>
       <c r="C44" t="n">
-        <v>46</v>
+        <v>29.51</v>
       </c>
       <c r="D44" t="n">
-        <v>4.31</v>
+        <v>4.98</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DEEP</t>
+          <t>KORE</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>39.33</v>
+        <v>221.8</v>
       </c>
       <c r="C45" t="n">
-        <v>41</v>
+        <v>232.85</v>
       </c>
       <c r="D45" t="n">
-        <v>4.25</v>
+        <v>4.98</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>NCC</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>119.93</v>
+        <v>93.5</v>
       </c>
       <c r="C46" t="n">
-        <v>125</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="D46" t="n">
-        <v>4.23</v>
+        <v>4.97</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>HEXT</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>511.4</v>
+        <v>34.39</v>
       </c>
       <c r="C47" t="n">
-        <v>533</v>
+        <v>36.1</v>
       </c>
       <c r="D47" t="n">
-        <v>4.22</v>
+        <v>4.97</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MANIKA</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>55.46</v>
+        <v>26.43</v>
       </c>
       <c r="C48" t="n">
-        <v>57.8</v>
+        <v>27.74</v>
       </c>
       <c r="D48" t="n">
-        <v>4.22</v>
+        <v>4.96</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HIMALAYAN</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>76.8</v>
+        <v>15.75</v>
       </c>
       <c r="C49" t="n">
-        <v>80</v>
+        <v>16.53</v>
       </c>
       <c r="D49" t="n">
-        <v>4.17</v>
+        <v>4.95</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.73</v>
+        <v>43.45</v>
       </c>
       <c r="C50" t="n">
-        <v>0.76</v>
+        <v>45.6</v>
       </c>
       <c r="D50" t="n">
-        <v>4.11</v>
+        <v>4.95</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PNGJL</t>
+          <t>MICROPRO</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>586.3</v>
+        <v>17.35</v>
       </c>
       <c r="C51" t="n">
-        <v>609.9</v>
+        <v>18.2</v>
       </c>
       <c r="D51" t="n">
-        <v>4.03</v>
+        <v>4.9</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LAGNAM</t>
+          <t>COREIN</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>71.14</v>
+        <v>100.2</v>
       </c>
       <c r="C52" t="n">
-        <v>73.98999999999999</v>
+        <v>105</v>
       </c>
       <c r="D52" t="n">
-        <v>4.01</v>
+        <v>4.79</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>GSTL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>48.68</v>
+        <v>12.6</v>
       </c>
       <c r="C53" t="n">
-        <v>50.6</v>
+        <v>13.2</v>
       </c>
       <c r="D53" t="n">
-        <v>3.94</v>
+        <v>4.76</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>278.2</v>
+        <v>53.95</v>
       </c>
       <c r="C54" t="n">
-        <v>288.9</v>
+        <v>56.5</v>
       </c>
       <c r="D54" t="n">
-        <v>3.85</v>
+        <v>4.73</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>36.5</v>
+        <v>12.3</v>
       </c>
       <c r="C55" t="n">
-        <v>37.9</v>
+        <v>12.88</v>
       </c>
       <c r="D55" t="n">
-        <v>3.84</v>
+        <v>4.72</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>VETO</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>161.85</v>
+        <v>131.63</v>
       </c>
       <c r="C56" t="n">
-        <v>168</v>
+        <v>137.8</v>
       </c>
       <c r="D56" t="n">
-        <v>3.8</v>
+        <v>4.69</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>AKCAPIT</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1728.4</v>
+        <v>47.58</v>
       </c>
       <c r="C57" t="n">
-        <v>1793.9</v>
+        <v>49.8</v>
       </c>
       <c r="D57" t="n">
-        <v>3.79</v>
+        <v>4.67</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>AVPINFRA</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>53.5</v>
+        <v>23.59</v>
       </c>
       <c r="C58" t="n">
-        <v>55.5</v>
+        <v>24.69</v>
       </c>
       <c r="D58" t="n">
-        <v>3.74</v>
+        <v>4.66</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>7666</v>
+        <v>4.35</v>
       </c>
       <c r="C59" t="n">
-        <v>7950</v>
+        <v>4.55</v>
       </c>
       <c r="D59" t="n">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>KKCL</t>
+          <t>21STCENMGM</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>472.5</v>
+        <v>43.12</v>
       </c>
       <c r="C60" t="n">
-        <v>489.9</v>
+        <v>45.1</v>
       </c>
       <c r="D60" t="n">
-        <v>3.68</v>
+        <v>4.59</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>259.46</v>
+        <v>21</v>
       </c>
       <c r="C61" t="n">
-        <v>269</v>
+        <v>21.96</v>
       </c>
       <c r="D61" t="n">
-        <v>3.68</v>
+        <v>4.57</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AERONEU</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>68.40000000000001</v>
+        <v>9.94</v>
       </c>
       <c r="C62" t="n">
-        <v>70.90000000000001</v>
+        <v>10.38</v>
       </c>
       <c r="D62" t="n">
-        <v>3.65</v>
+        <v>4.43</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>OMINFRAL</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>68.86</v>
+        <v>30.17</v>
       </c>
       <c r="C63" t="n">
-        <v>71.34</v>
+        <v>31.5</v>
       </c>
       <c r="D63" t="n">
-        <v>3.6</v>
+        <v>4.41</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>18.72</v>
+        <v>272.43</v>
       </c>
       <c r="C64" t="n">
-        <v>19.39</v>
+        <v>284.4</v>
       </c>
       <c r="D64" t="n">
-        <v>3.58</v>
+        <v>4.39</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1.43</v>
+        <v>2.05</v>
       </c>
       <c r="C65" t="n">
-        <v>1.48</v>
+        <v>2.14</v>
       </c>
       <c r="D65" t="n">
-        <v>3.5</v>
+        <v>4.39</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>HEALTHX</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>292.9</v>
+        <v>17.86</v>
       </c>
       <c r="C66" t="n">
-        <v>303</v>
+        <v>18.64</v>
       </c>
       <c r="D66" t="n">
-        <v>3.45</v>
+        <v>4.37</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>200.16</v>
+        <v>3.44</v>
       </c>
       <c r="C67" t="n">
-        <v>207</v>
+        <v>3.59</v>
       </c>
       <c r="D67" t="n">
-        <v>3.42</v>
+        <v>4.36</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S&amp;SPOWER</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>275.2</v>
+        <v>16.19</v>
       </c>
       <c r="C68" t="n">
-        <v>284.6</v>
+        <v>16.89</v>
       </c>
       <c r="D68" t="n">
-        <v>3.42</v>
+        <v>4.32</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2.05</v>
+        <v>594.95</v>
       </c>
       <c r="C69" t="n">
-        <v>2.12</v>
+        <v>620.4</v>
       </c>
       <c r="D69" t="n">
-        <v>3.41</v>
+        <v>4.28</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>25.63</v>
+        <v>0.47</v>
       </c>
       <c r="C70" t="n">
-        <v>26.5</v>
+        <v>0.49</v>
       </c>
       <c r="D70" t="n">
-        <v>3.39</v>
+        <v>4.26</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>TEXMOPIPES</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>34.63</v>
+        <v>51.21</v>
       </c>
       <c r="C71" t="n">
-        <v>35.8</v>
+        <v>53.39</v>
       </c>
       <c r="D71" t="n">
-        <v>3.38</v>
+        <v>4.26</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>561.3</v>
+        <v>173.53</v>
       </c>
       <c r="C72" t="n">
-        <v>580</v>
+        <v>180.89</v>
       </c>
       <c r="D72" t="n">
-        <v>3.33</v>
+        <v>4.24</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>LOTUSCHO</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>763</v>
+        <v>565.1</v>
       </c>
       <c r="C73" t="n">
-        <v>788</v>
+        <v>589</v>
       </c>
       <c r="D73" t="n">
-        <v>3.28</v>
+        <v>4.23</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>GALLANTT</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>207.2</v>
+        <v>503.75</v>
       </c>
       <c r="C74" t="n">
-        <v>214</v>
+        <v>524.95</v>
       </c>
       <c r="D74" t="n">
-        <v>3.28</v>
+        <v>4.21</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DIFFNKG</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>427.25</v>
+        <v>6.18</v>
       </c>
       <c r="C75" t="n">
-        <v>441</v>
+        <v>6.44</v>
       </c>
       <c r="D75" t="n">
-        <v>3.22</v>
+        <v>4.21</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>49.92</v>
+        <v>12.85</v>
       </c>
       <c r="C76" t="n">
-        <v>51.5</v>
+        <v>13.39</v>
       </c>
       <c r="D76" t="n">
-        <v>3.17</v>
+        <v>4.2</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>COFFEEDAY</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>30.53</v>
+        <v>111.33</v>
       </c>
       <c r="C77" t="n">
-        <v>31.49</v>
+        <v>116</v>
       </c>
       <c r="D77" t="n">
-        <v>3.14</v>
+        <v>4.19</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>BATLIBOI</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>93.98</v>
+        <v>4.11</v>
       </c>
       <c r="C78" t="n">
-        <v>96.90000000000001</v>
+        <v>4.28</v>
       </c>
       <c r="D78" t="n">
-        <v>3.11</v>
+        <v>4.14</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>AARTECH</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>14.94</v>
+        <v>47.82</v>
       </c>
       <c r="C79" t="n">
-        <v>15.4</v>
+        <v>49.8</v>
       </c>
       <c r="D79" t="n">
-        <v>3.08</v>
+        <v>4.14</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>AMEYA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>36</v>
+        <v>170</v>
       </c>
       <c r="C80" t="n">
-        <v>37.09</v>
+        <v>177</v>
       </c>
       <c r="D80" t="n">
-        <v>3.03</v>
+        <v>4.12</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>9.699999999999999</v>
+        <v>21.9</v>
       </c>
       <c r="C81" t="n">
-        <v>9.99</v>
+        <v>22.8</v>
       </c>
       <c r="D81" t="n">
-        <v>2.99</v>
+        <v>4.11</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ASHIMASYN</t>
+          <t>AKANKSHA</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>14.08</v>
+        <v>175.9</v>
       </c>
       <c r="C82" t="n">
-        <v>14.5</v>
+        <v>183</v>
       </c>
       <c r="D82" t="n">
-        <v>2.98</v>
+        <v>4.04</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>4.36</v>
+        <v>102.85</v>
       </c>
       <c r="C83" t="n">
-        <v>4.49</v>
+        <v>107</v>
       </c>
       <c r="D83" t="n">
-        <v>2.98</v>
+        <v>4.04</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>TOYAMSL</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>49.51</v>
+        <v>0.76</v>
       </c>
       <c r="C84" t="n">
-        <v>50.98</v>
+        <v>0.79</v>
       </c>
       <c r="D84" t="n">
-        <v>2.97</v>
+        <v>3.95</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>KEC</t>
+          <t>RTSPOWR</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>349.6</v>
+        <v>119.33</v>
       </c>
       <c r="C85" t="n">
-        <v>360</v>
+        <v>123.97</v>
       </c>
       <c r="D85" t="n">
-        <v>2.97</v>
+        <v>3.89</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>ABSMARINE</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>1.69</v>
+        <v>310</v>
       </c>
       <c r="C86" t="n">
-        <v>1.74</v>
+        <v>321.95</v>
       </c>
       <c r="D86" t="n">
-        <v>2.96</v>
+        <v>3.85</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>18.11</v>
+        <v>26.3</v>
       </c>
       <c r="C87" t="n">
-        <v>18.64</v>
+        <v>27.3</v>
       </c>
       <c r="D87" t="n">
-        <v>2.93</v>
+        <v>3.8</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>23.71</v>
+        <v>215.72</v>
       </c>
       <c r="C88" t="n">
-        <v>24.39</v>
+        <v>223.9</v>
       </c>
       <c r="D88" t="n">
-        <v>2.87</v>
+        <v>3.79</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>GRAVITA</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>136.1</v>
+        <v>1466.4</v>
       </c>
       <c r="C89" t="n">
-        <v>140</v>
+        <v>1521.9</v>
       </c>
       <c r="D89" t="n">
-        <v>2.87</v>
+        <v>3.78</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>JAINREC</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>281.05</v>
+        <v>42.21</v>
       </c>
       <c r="C90" t="n">
-        <v>289.1</v>
+        <v>43.8</v>
       </c>
       <c r="D90" t="n">
-        <v>2.86</v>
+        <v>3.77</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>COMPINFO</t>
+          <t>ASHUTOSH</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1.06</v>
+        <v>142.6</v>
       </c>
       <c r="C91" t="n">
-        <v>1.09</v>
+        <v>147.95</v>
       </c>
       <c r="D91" t="n">
-        <v>2.83</v>
+        <v>3.75</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>KERNEX</t>
+          <t>VHL</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1700.5</v>
+        <v>3650</v>
       </c>
       <c r="C92" t="n">
-        <v>1748.7</v>
+        <v>3785</v>
       </c>
       <c r="D92" t="n">
-        <v>2.83</v>
+        <v>3.7</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DECCANCE</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>532.95</v>
+        <v>50.12</v>
       </c>
       <c r="C93" t="n">
-        <v>548</v>
+        <v>51.97</v>
       </c>
       <c r="D93" t="n">
-        <v>2.82</v>
+        <v>3.69</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>JYOTIRES</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>7.18</v>
+        <v>839.1</v>
       </c>
       <c r="C94" t="n">
-        <v>7.38</v>
+        <v>870</v>
       </c>
       <c r="D94" t="n">
-        <v>2.79</v>
+        <v>3.68</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>197</v>
+        <v>273.95</v>
       </c>
       <c r="C95" t="n">
-        <v>202.5</v>
+        <v>283.95</v>
       </c>
       <c r="D95" t="n">
-        <v>2.79</v>
+        <v>3.65</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>1.44</v>
+        <v>954.3</v>
       </c>
       <c r="C96" t="n">
-        <v>1.48</v>
+        <v>989</v>
       </c>
       <c r="D96" t="n">
-        <v>2.78</v>
+        <v>3.64</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>18.77</v>
+        <v>51.14</v>
       </c>
       <c r="C97" t="n">
-        <v>19.29</v>
+        <v>52.99</v>
       </c>
       <c r="D97" t="n">
-        <v>2.77</v>
+        <v>3.62</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>252.6</v>
+        <v>77.12</v>
       </c>
       <c r="C98" t="n">
-        <v>259.5</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="D98" t="n">
-        <v>2.73</v>
+        <v>3.6</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>1.83</v>
+        <v>617.8</v>
       </c>
       <c r="C99" t="n">
-        <v>1.88</v>
+        <v>640</v>
       </c>
       <c r="D99" t="n">
-        <v>2.73</v>
+        <v>3.59</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1041.5</v>
+        <v>1.68</v>
       </c>
       <c r="C100" t="n">
-        <v>1069.8</v>
+        <v>1.74</v>
       </c>
       <c r="D100" t="n">
-        <v>2.72</v>
+        <v>3.57</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>873.4</v>
+        <v>52.24</v>
       </c>
       <c r="C101" t="n">
-        <v>896.8</v>
+        <v>54.1</v>
       </c>
       <c r="D101" t="n">
-        <v>2.68</v>
+        <v>3.56</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>AMBAAUTO</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>14.6</v>
+        <v>113.95</v>
       </c>
       <c r="C102" t="n">
-        <v>14.99</v>
+        <v>118</v>
       </c>
       <c r="D102" t="n">
-        <v>2.67</v>
+        <v>3.55</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>MUNJALAU</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>5.25</v>
+        <v>101.32</v>
       </c>
       <c r="C103" t="n">
-        <v>5.39</v>
+        <v>104.87</v>
       </c>
       <c r="D103" t="n">
-        <v>2.67</v>
+        <v>3.5</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>MANINDS</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>608.6</v>
+        <v>867.9</v>
       </c>
       <c r="C104" t="n">
-        <v>624.8</v>
+        <v>898</v>
       </c>
       <c r="D104" t="n">
-        <v>2.66</v>
+        <v>3.47</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>CRSL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>19.97</v>
+        <v>2.07</v>
       </c>
       <c r="C105" t="n">
-        <v>20.5</v>
+        <v>2.14</v>
       </c>
       <c r="D105" t="n">
-        <v>2.65</v>
+        <v>3.38</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>TECHNVISN</t>
+          <t>INDOAMIN</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>4384.5</v>
+        <v>157.72</v>
       </c>
       <c r="C106" t="n">
-        <v>4500</v>
+        <v>163</v>
       </c>
       <c r="D106" t="n">
-        <v>2.63</v>
+        <v>3.35</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MAFATIND</t>
+          <t>MVGJL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>111.07</v>
+        <v>207.87</v>
       </c>
       <c r="C107" t="n">
-        <v>113.97</v>
+        <v>214.8</v>
       </c>
       <c r="D107" t="n">
-        <v>2.61</v>
+        <v>3.33</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>6.12</v>
+        <v>108.41</v>
       </c>
       <c r="C108" t="n">
-        <v>6.28</v>
+        <v>112</v>
       </c>
       <c r="D108" t="n">
-        <v>2.61</v>
+        <v>3.31</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>14.23</v>
+        <v>1015.45</v>
       </c>
       <c r="C109" t="n">
-        <v>14.6</v>
+        <v>1048.95</v>
       </c>
       <c r="D109" t="n">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>AUGMONT</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>25.14</v>
+        <v>1337.8</v>
       </c>
       <c r="C110" t="n">
-        <v>25.79</v>
+        <v>1381.8</v>
       </c>
       <c r="D110" t="n">
-        <v>2.59</v>
+        <v>3.29</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>GOACARBON</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>394.8</v>
+        <v>5.79</v>
       </c>
       <c r="C111" t="n">
-        <v>405</v>
+        <v>5.98</v>
       </c>
       <c r="D111" t="n">
-        <v>2.58</v>
+        <v>3.28</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CENTRUM</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>19.44</v>
+        <v>20.71</v>
       </c>
       <c r="C112" t="n">
-        <v>19.94</v>
+        <v>21.38</v>
       </c>
       <c r="D112" t="n">
-        <v>2.57</v>
+        <v>3.24</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>TAMBOLIIN</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>177.5</v>
+        <v>290.6</v>
       </c>
       <c r="C113" t="n">
-        <v>182</v>
+        <v>300</v>
       </c>
       <c r="D113" t="n">
-        <v>2.54</v>
+        <v>3.23</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GMBREW</t>
+          <t>DELAPLEX</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>887.45</v>
+        <v>94.75</v>
       </c>
       <c r="C114" t="n">
-        <v>910</v>
+        <v>97.8</v>
       </c>
       <c r="D114" t="n">
-        <v>2.54</v>
+        <v>3.22</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>BHANDARI</t>
+          <t>SYNGENE</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2.76</v>
+        <v>347.4</v>
       </c>
       <c r="C115" t="n">
-        <v>2.83</v>
+        <v>358.5</v>
       </c>
       <c r="D115" t="n">
-        <v>2.54</v>
+        <v>3.2</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>152.17</v>
+        <v>21.04</v>
       </c>
       <c r="C116" t="n">
-        <v>156</v>
+        <v>21.71</v>
       </c>
       <c r="D116" t="n">
-        <v>2.52</v>
+        <v>3.18</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2995,13 +2995,13 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>31.22</v>
+        <v>31.88</v>
       </c>
       <c r="C117" t="n">
-        <v>32</v>
+        <v>32.89</v>
       </c>
       <c r="D117" t="n">
-        <v>2.5</v>
+        <v>3.17</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PAUSHAKLTD</t>
+          <t>DEVIT</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>671.65</v>
+        <v>19.39</v>
       </c>
       <c r="C118" t="n">
-        <v>688.35</v>
+        <v>20</v>
       </c>
       <c r="D118" t="n">
-        <v>2.49</v>
+        <v>3.15</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>INVENTURE</t>
+          <t>MEESHO</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.8100000000000001</v>
+        <v>232.74</v>
       </c>
       <c r="C119" t="n">
-        <v>0.83</v>
+        <v>240</v>
       </c>
       <c r="D119" t="n">
-        <v>2.47</v>
+        <v>3.12</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DISHTV</t>
+          <t>ONIXSOLAR</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>2.03</v>
+        <v>380.15</v>
       </c>
       <c r="C120" t="n">
-        <v>2.08</v>
+        <v>392</v>
       </c>
       <c r="D120" t="n">
-        <v>2.46</v>
+        <v>3.12</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AUSOMENT</t>
+          <t>HLVLTD</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>143.29</v>
+        <v>6.11</v>
       </c>
       <c r="C121" t="n">
-        <v>146.8</v>
+        <v>6.3</v>
       </c>
       <c r="D121" t="n">
-        <v>2.45</v>
+        <v>3.11</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>CRAMC</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>6.23</v>
+        <v>219.95</v>
       </c>
       <c r="C122" t="n">
-        <v>6.38</v>
+        <v>226.75</v>
       </c>
       <c r="D122" t="n">
-        <v>2.41</v>
+        <v>3.09</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BIRLACORPN</t>
+          <t>POOJALOGIS</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>794.85</v>
+        <v>132.7</v>
       </c>
       <c r="C123" t="n">
-        <v>814</v>
+        <v>136.8</v>
       </c>
       <c r="D123" t="n">
-        <v>2.41</v>
+        <v>3.09</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>ZIMLAB</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>9.17</v>
+        <v>150.47</v>
       </c>
       <c r="C124" t="n">
-        <v>9.390000000000001</v>
+        <v>155.1</v>
       </c>
       <c r="D124" t="n">
-        <v>2.4</v>
+        <v>3.08</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>40.63</v>
+        <v>77.36</v>
       </c>
       <c r="C125" t="n">
-        <v>41.6</v>
+        <v>79.7</v>
       </c>
       <c r="D125" t="n">
-        <v>2.39</v>
+        <v>3.02</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>TCPLPACK</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>3994.4</v>
+        <v>5.33</v>
       </c>
       <c r="C126" t="n">
-        <v>4090</v>
+        <v>5.49</v>
       </c>
       <c r="D126" t="n">
-        <v>2.39</v>
+        <v>3</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>KHAICHEM</t>
+          <t>MICEL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>47.6</v>
+        <v>34.37</v>
       </c>
       <c r="C127" t="n">
-        <v>48.73</v>
+        <v>35.4</v>
       </c>
       <c r="D127" t="n">
-        <v>2.37</v>
+        <v>3</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>JITFINFRA</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>269.55</v>
+        <v>20.07</v>
       </c>
       <c r="C128" t="n">
-        <v>275.9</v>
+        <v>20.67</v>
       </c>
       <c r="D128" t="n">
-        <v>2.36</v>
+        <v>2.99</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>BAJAJST</t>
+          <t>TTML</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>324.3</v>
+        <v>32.89</v>
       </c>
       <c r="C129" t="n">
-        <v>331.95</v>
+        <v>33.87</v>
       </c>
       <c r="D129" t="n">
-        <v>2.36</v>
+        <v>2.98</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ELECTHERM</t>
+          <t>RMC</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>683.75</v>
+        <v>184.33</v>
       </c>
       <c r="C130" t="n">
-        <v>699.9</v>
+        <v>189.8</v>
       </c>
       <c r="D130" t="n">
-        <v>2.36</v>
+        <v>2.97</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>KOKUYOCMLN</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>8.09</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="C131" t="n">
-        <v>8.279999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="D131" t="n">
-        <v>2.35</v>
+        <v>2.96</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>ARROWGREEN</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.43</v>
+        <v>855.65</v>
       </c>
       <c r="C132" t="n">
-        <v>0.44</v>
+        <v>881</v>
       </c>
       <c r="D132" t="n">
-        <v>2.33</v>
+        <v>2.96</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ARCHIES</t>
+          <t>ASHOKA</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>12.01</v>
+        <v>102.02</v>
       </c>
       <c r="C133" t="n">
-        <v>12.29</v>
+        <v>105</v>
       </c>
       <c r="D133" t="n">
-        <v>2.33</v>
+        <v>2.92</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>VIRINCHI</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.87</v>
+        <v>12.81</v>
       </c>
       <c r="C134" t="n">
-        <v>0.89</v>
+        <v>13.18</v>
       </c>
       <c r="D134" t="n">
-        <v>2.3</v>
+        <v>2.89</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BAJAJINDEF</t>
+          <t>PRIORITY</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>199.24</v>
+        <v>325.55</v>
       </c>
       <c r="C135" t="n">
-        <v>203.8</v>
+        <v>334.95</v>
       </c>
       <c r="D135" t="n">
-        <v>2.29</v>
+        <v>2.89</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>12.79</v>
+        <v>1.74</v>
       </c>
       <c r="C136" t="n">
-        <v>13.08</v>
+        <v>1.79</v>
       </c>
       <c r="D136" t="n">
-        <v>2.27</v>
+        <v>2.87</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>AVATAR</t>
+          <t>GANESHHOU</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>183.75</v>
+        <v>699.5</v>
       </c>
       <c r="C137" t="n">
-        <v>187.9</v>
+        <v>719.5</v>
       </c>
       <c r="D137" t="n">
-        <v>2.26</v>
+        <v>2.86</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MMTC</t>
+          <t>A2ZINFRA</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>54.27</v>
+        <v>14</v>
       </c>
       <c r="C138" t="n">
-        <v>55.49</v>
+        <v>14.4</v>
       </c>
       <c r="D138" t="n">
-        <v>2.25</v>
+        <v>2.86</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>SATIA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>3.13</v>
+        <v>68.06</v>
       </c>
       <c r="C139" t="n">
-        <v>3.2</v>
+        <v>70</v>
       </c>
       <c r="D139" t="n">
-        <v>2.24</v>
+        <v>2.85</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>13.9</v>
+        <v>1676.4</v>
       </c>
       <c r="C140" t="n">
-        <v>14.21</v>
+        <v>1724</v>
       </c>
       <c r="D140" t="n">
-        <v>2.23</v>
+        <v>2.84</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>TEAMGTY</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1.8</v>
+        <v>243.02</v>
       </c>
       <c r="C141" t="n">
-        <v>1.84</v>
+        <v>249.9</v>
       </c>
       <c r="D141" t="n">
-        <v>2.22</v>
+        <v>2.83</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CRIZAC</t>
+          <t>TINNARUBR</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>159.97</v>
+        <v>885.85</v>
       </c>
       <c r="C142" t="n">
-        <v>163.5</v>
+        <v>910.95</v>
       </c>
       <c r="D142" t="n">
-        <v>2.21</v>
+        <v>2.83</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>EPACKPEB</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>256.33</v>
+        <v>279.05</v>
       </c>
       <c r="C143" t="n">
-        <v>262</v>
+        <v>286.95</v>
       </c>
       <c r="D143" t="n">
-        <v>2.21</v>
+        <v>2.83</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>TRIVENI</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>237.86</v>
+        <v>36.33</v>
       </c>
       <c r="C144" t="n">
-        <v>243.1</v>
+        <v>37.35</v>
       </c>
       <c r="D144" t="n">
-        <v>2.2</v>
+        <v>2.81</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>VEEGALAND</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>136.9</v>
+        <v>5.72</v>
       </c>
       <c r="C145" t="n">
-        <v>139.9</v>
+        <v>5.88</v>
       </c>
       <c r="D145" t="n">
-        <v>2.19</v>
+        <v>2.8</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>MOHITIND</t>
+          <t>GINNIFILA</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>22.01</v>
+        <v>40.75</v>
       </c>
       <c r="C146" t="n">
-        <v>22.49</v>
+        <v>41.89</v>
       </c>
       <c r="D146" t="n">
-        <v>2.18</v>
+        <v>2.8</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>TOLINS</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>86.56</v>
+        <v>18</v>
       </c>
       <c r="C147" t="n">
-        <v>88.45</v>
+        <v>18.5</v>
       </c>
       <c r="D147" t="n">
-        <v>2.18</v>
+        <v>2.78</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.46</v>
+        <v>0.36</v>
       </c>
       <c r="C148" t="n">
-        <v>0.47</v>
+        <v>0.37</v>
       </c>
       <c r="D148" t="n">
-        <v>2.17</v>
+        <v>2.78</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ISHANCH</t>
+          <t>IWARE</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>46.44</v>
+        <v>349.3</v>
       </c>
       <c r="C149" t="n">
-        <v>47.45</v>
+        <v>359</v>
       </c>
       <c r="D149" t="n">
-        <v>2.17</v>
+        <v>2.78</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>TRIVENI</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1.84</v>
+        <v>235.67</v>
       </c>
       <c r="C150" t="n">
-        <v>1.88</v>
+        <v>242.2</v>
       </c>
       <c r="D150" t="n">
-        <v>2.17</v>
+        <v>2.77</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AUTOIND</t>
+          <t>KOTHARIPRO</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>80.06</v>
+        <v>62.26</v>
       </c>
       <c r="C151" t="n">
-        <v>81.8</v>
+        <v>63.97</v>
       </c>
       <c r="D151" t="n">
-        <v>2.17</v>
+        <v>2.75</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DIGIDRIVE</t>
+          <t>SICAGEN</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>17.51</v>
+        <v>50.45</v>
       </c>
       <c r="C152" t="n">
-        <v>17.89</v>
+        <v>51.83</v>
       </c>
       <c r="D152" t="n">
-        <v>2.17</v>
+        <v>2.74</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>MANBA</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>146.82</v>
+        <v>105.13</v>
       </c>
       <c r="C153" t="n">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="D153" t="n">
-        <v>2.17</v>
+        <v>2.73</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>NECLIFE</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>5.56</v>
+        <v>10.13</v>
       </c>
       <c r="C154" t="n">
-        <v>5.68</v>
+        <v>10.4</v>
       </c>
       <c r="D154" t="n">
-        <v>2.16</v>
+        <v>2.67</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>RAMBHAJO</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>861.4</v>
+        <v>357.45</v>
       </c>
       <c r="C155" t="n">
-        <v>880</v>
+        <v>367</v>
       </c>
       <c r="D155" t="n">
-        <v>2.16</v>
+        <v>2.67</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>SURANAT&amp;P</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>44.48</v>
+        <v>15.54</v>
       </c>
       <c r="C156" t="n">
-        <v>45.44</v>
+        <v>15.95</v>
       </c>
       <c r="D156" t="n">
-        <v>2.16</v>
+        <v>2.64</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>APEXECO</t>
+          <t>HAZOOR</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>246.3</v>
+        <v>16.27</v>
       </c>
       <c r="C157" t="n">
-        <v>251.6</v>
+        <v>16.7</v>
       </c>
       <c r="D157" t="n">
-        <v>2.15</v>
+        <v>2.64</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>LCL</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>20.55</v>
+        <v>630.85</v>
       </c>
       <c r="C158" t="n">
-        <v>20.99</v>
+        <v>647.45</v>
       </c>
       <c r="D158" t="n">
-        <v>2.14</v>
+        <v>2.63</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SAMPANN</t>
+          <t>UCAL</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>23.78</v>
+        <v>134.36</v>
       </c>
       <c r="C159" t="n">
-        <v>24.29</v>
+        <v>137.89</v>
       </c>
       <c r="D159" t="n">
-        <v>2.14</v>
+        <v>2.63</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SWSOLAR</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>160.09</v>
+        <v>218.54</v>
       </c>
       <c r="C160" t="n">
-        <v>163.5</v>
+        <v>224.2</v>
       </c>
       <c r="D160" t="n">
-        <v>2.13</v>
+        <v>2.59</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GALLANTT</t>
+          <t>DCM</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>503.15</v>
+        <v>71.17</v>
       </c>
       <c r="C161" t="n">
-        <v>513.8</v>
+        <v>73</v>
       </c>
       <c r="D161" t="n">
-        <v>2.12</v>
+        <v>2.57</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>CENTUM</t>
+          <t>GTL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>4142.1</v>
+        <v>6.64</v>
       </c>
       <c r="C162" t="n">
-        <v>4230</v>
+        <v>6.81</v>
       </c>
       <c r="D162" t="n">
-        <v>2.12</v>
+        <v>2.56</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>MANIKA</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>108.11</v>
+        <v>54.21</v>
       </c>
       <c r="C163" t="n">
-        <v>110.4</v>
+        <v>55.6</v>
       </c>
       <c r="D163" t="n">
-        <v>2.12</v>
+        <v>2.56</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MUFTI</t>
+          <t>RISHABH</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>68.26000000000001</v>
+        <v>677.9</v>
       </c>
       <c r="C164" t="n">
-        <v>69.7</v>
+        <v>695</v>
       </c>
       <c r="D164" t="n">
-        <v>2.11</v>
+        <v>2.52</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>37.21</v>
+        <v>4.4</v>
       </c>
       <c r="C165" t="n">
-        <v>37.99</v>
+        <v>4.51</v>
       </c>
       <c r="D165" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CENTEXT</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>18.6</v>
+        <v>32.19</v>
       </c>
       <c r="C166" t="n">
-        <v>18.99</v>
+        <v>32.99</v>
       </c>
       <c r="D166" t="n">
-        <v>2.1</v>
+        <v>2.49</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>LKPSEC</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>31.63</v>
+        <v>13.63</v>
       </c>
       <c r="C167" t="n">
-        <v>32.29</v>
+        <v>13.97</v>
       </c>
       <c r="D167" t="n">
-        <v>2.09</v>
+        <v>2.49</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>GTL</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>6.71</v>
+        <v>21.27</v>
       </c>
       <c r="C168" t="n">
-        <v>6.85</v>
+        <v>21.8</v>
       </c>
       <c r="D168" t="n">
-        <v>2.09</v>
+        <v>2.49</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>HIGREEN</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>119.35</v>
+        <v>3121.7</v>
       </c>
       <c r="C169" t="n">
-        <v>121.8</v>
+        <v>3198.7</v>
       </c>
       <c r="D169" t="n">
-        <v>2.05</v>
+        <v>2.47</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ADVIKCA</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>0.98</v>
+        <v>40.6</v>
       </c>
       <c r="C170" t="n">
-        <v>1</v>
+        <v>41.6</v>
       </c>
       <c r="D170" t="n">
-        <v>2.04</v>
+        <v>2.46</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PRISMX</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.49</v>
+        <v>189.25</v>
       </c>
       <c r="C171" t="n">
-        <v>0.5</v>
+        <v>193.9</v>
       </c>
       <c r="D171" t="n">
-        <v>2.04</v>
+        <v>2.46</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>THERMAX</t>
+          <t>YOGI</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>3138.1</v>
+        <v>159.99</v>
       </c>
       <c r="C172" t="n">
-        <v>3202</v>
+        <v>163.9</v>
       </c>
       <c r="D172" t="n">
-        <v>2.04</v>
+        <v>2.44</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MIDWESTLTD</t>
+          <t>BTML</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>989.8</v>
+        <v>7.02</v>
       </c>
       <c r="C173" t="n">
-        <v>1010</v>
+        <v>7.19</v>
       </c>
       <c r="D173" t="n">
-        <v>2.04</v>
+        <v>2.42</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>SHADOWFAX</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>20.17</v>
+        <v>294.85</v>
       </c>
       <c r="C174" t="n">
-        <v>20.58</v>
+        <v>302</v>
       </c>
       <c r="D174" t="n">
-        <v>2.03</v>
+        <v>2.42</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>LINC</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>15.77</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="C175" t="n">
-        <v>16.09</v>
+        <v>83.5</v>
       </c>
       <c r="D175" t="n">
-        <v>2.03</v>
+        <v>2.4</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>AUGMONT</t>
+          <t>ASHIKAG</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>1274.1</v>
+        <v>380.8</v>
       </c>
       <c r="C176" t="n">
-        <v>1300</v>
+        <v>389.8</v>
       </c>
       <c r="D176" t="n">
-        <v>2.03</v>
+        <v>2.36</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>OSELDEVICE</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>11.91</v>
+        <v>366.35</v>
       </c>
       <c r="C177" t="n">
-        <v>12.15</v>
+        <v>375</v>
       </c>
       <c r="D177" t="n">
-        <v>2.02</v>
+        <v>2.36</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>GANECOS</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>199.47</v>
+        <v>966.1</v>
       </c>
       <c r="C178" t="n">
-        <v>203.5</v>
+        <v>988.9</v>
       </c>
       <c r="D178" t="n">
-        <v>2.02</v>
+        <v>2.36</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>53.75</v>
+        <v>55.6</v>
       </c>
       <c r="C179" t="n">
-        <v>54.83</v>
+        <v>56.9</v>
       </c>
       <c r="D179" t="n">
-        <v>2.01</v>
+        <v>2.34</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>76.26000000000001</v>
+        <v>0.86</v>
       </c>
       <c r="C180" t="n">
-        <v>77.79000000000001</v>
+        <v>0.88</v>
       </c>
       <c r="D180" t="n">
-        <v>2.01</v>
+        <v>2.33</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>ELDEHSG</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.5</v>
+        <v>786.45</v>
       </c>
       <c r="C181" t="n">
-        <v>0.51</v>
+        <v>804.8</v>
       </c>
       <c r="D181" t="n">
-        <v>2</v>
+        <v>2.33</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>NOVAAGRI</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>21.95</v>
+        <v>0.43</v>
       </c>
       <c r="C182" t="n">
-        <v>22.39</v>
+        <v>0.44</v>
       </c>
       <c r="D182" t="n">
-        <v>2</v>
+        <v>2.33</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>GEECEE</t>
+          <t>JINDALPHOT</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>352.7</v>
+        <v>1021.6</v>
       </c>
       <c r="C183" t="n">
-        <v>359.75</v>
+        <v>1045</v>
       </c>
       <c r="D183" t="n">
-        <v>2</v>
+        <v>2.29</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>SHILPAMED</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>483.25</v>
+        <v>1021.7</v>
       </c>
       <c r="C184" t="n">
-        <v>492.85</v>
+        <v>1045</v>
       </c>
       <c r="D184" t="n">
-        <v>1.99</v>
+        <v>2.28</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>VHL</t>
+          <t>RAJOOENG</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>3578.8</v>
+        <v>59.45</v>
       </c>
       <c r="C185" t="n">
-        <v>3650</v>
+        <v>60.8</v>
       </c>
       <c r="D185" t="n">
-        <v>1.99</v>
+        <v>2.27</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ORIENTCABL</t>
+          <t>RAMAPHO</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>386.85</v>
+        <v>109.52</v>
       </c>
       <c r="C186" t="n">
-        <v>394.55</v>
+        <v>112</v>
       </c>
       <c r="D186" t="n">
-        <v>1.99</v>
+        <v>2.26</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>AMJLAND</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>36.66</v>
+        <v>105.14</v>
       </c>
       <c r="C187" t="n">
-        <v>37.39</v>
+        <v>107.52</v>
       </c>
       <c r="D187" t="n">
-        <v>1.99</v>
+        <v>2.26</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MSL</t>
+          <t>ODYCORP</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>136.69</v>
+        <v>6.64</v>
       </c>
       <c r="C188" t="n">
-        <v>139.39</v>
+        <v>6.79</v>
       </c>
       <c r="D188" t="n">
-        <v>1.98</v>
+        <v>2.26</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PHOENXINTL</t>
+          <t>KSE</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>27.84</v>
+        <v>176.02</v>
       </c>
       <c r="C189" t="n">
-        <v>28.39</v>
+        <v>180</v>
       </c>
       <c r="D189" t="n">
-        <v>1.98</v>
+        <v>2.26</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>EFCIL</t>
+          <t>AMDIND</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>167.07</v>
+        <v>49.29</v>
       </c>
       <c r="C190" t="n">
-        <v>170.38</v>
+        <v>50.4</v>
       </c>
       <c r="D190" t="n">
-        <v>1.98</v>
+        <v>2.25</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>SAFEENTP</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>7.58</v>
+        <v>239.6</v>
       </c>
       <c r="C191" t="n">
-        <v>7.73</v>
+        <v>245</v>
       </c>
       <c r="D191" t="n">
-        <v>1.98</v>
+        <v>2.25</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>GKSL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>54.9</v>
+        <v>184.09</v>
       </c>
       <c r="C192" t="n">
-        <v>55.98</v>
+        <v>188.22</v>
       </c>
       <c r="D192" t="n">
-        <v>1.97</v>
+        <v>2.24</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>CGVAK</t>
+          <t>HINDALUMI</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>137.73</v>
+        <v>89.5</v>
       </c>
       <c r="C193" t="n">
-        <v>140.45</v>
+        <v>91.5</v>
       </c>
       <c r="D193" t="n">
-        <v>1.97</v>
+        <v>2.23</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>NTCIND</t>
+          <t>WATERBASE</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>135.03</v>
+        <v>44.31</v>
       </c>
       <c r="C194" t="n">
-        <v>137.69</v>
+        <v>45.3</v>
       </c>
       <c r="D194" t="n">
-        <v>1.97</v>
+        <v>2.23</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KUSUMGAR</t>
+          <t>PARAGMILK</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>608</v>
+        <v>306.4</v>
       </c>
       <c r="C195" t="n">
-        <v>620</v>
+        <v>313.2</v>
       </c>
       <c r="D195" t="n">
-        <v>1.97</v>
+        <v>2.22</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>DCI</t>
+          <t>OSWALPUMPS</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>345.2</v>
+        <v>254.35</v>
       </c>
       <c r="C196" t="n">
-        <v>352</v>
+        <v>260</v>
       </c>
       <c r="D196" t="n">
-        <v>1.97</v>
+        <v>2.22</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>20.81</v>
+        <v>11.24</v>
       </c>
       <c r="C197" t="n">
-        <v>21.22</v>
+        <v>11.49</v>
       </c>
       <c r="D197" t="n">
-        <v>1.97</v>
+        <v>2.22</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>4.57</v>
+        <v>89.5</v>
       </c>
       <c r="C198" t="n">
-        <v>4.66</v>
+        <v>91.48999999999999</v>
       </c>
       <c r="D198" t="n">
-        <v>1.97</v>
+        <v>2.22</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>KSHINTL</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>47.56</v>
+        <v>1001.5</v>
       </c>
       <c r="C199" t="n">
-        <v>48.49</v>
+        <v>1023.5</v>
       </c>
       <c r="D199" t="n">
-        <v>1.96</v>
+        <v>2.2</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>LFIC</t>
+          <t>MINDTECK</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>126.22</v>
+        <v>139.37</v>
       </c>
       <c r="C200" t="n">
-        <v>128.69</v>
+        <v>142.4</v>
       </c>
       <c r="D200" t="n">
-        <v>1.96</v>
+        <v>2.17</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>NGIL</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>37.75</v>
+        <v>1.39</v>
       </c>
       <c r="C201" t="n">
-        <v>38.49</v>
+        <v>1.42</v>
       </c>
       <c r="D201" t="n">
-        <v>1.96</v>
+        <v>2.16</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-13 11:04 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TERAI</t>
+          <t>ARTNIRMAN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>140.01</v>
+        <v>36.43</v>
       </c>
       <c r="C2" t="n">
-        <v>168</v>
+        <v>42.7</v>
       </c>
       <c r="D2" t="n">
-        <v>19.99</v>
+        <v>17.21</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMAL</t>
+          <t>PHOENXINTL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>764.95</v>
+        <v>33.44</v>
       </c>
       <c r="C3" t="n">
-        <v>851</v>
+        <v>38.49</v>
       </c>
       <c r="D3" t="n">
-        <v>11.25</v>
+        <v>15.1</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41.23</v>
+        <v>2.2</v>
       </c>
       <c r="C4" t="n">
-        <v>45.35</v>
+        <v>2.42</v>
       </c>
       <c r="D4" t="n">
-        <v>9.99</v>
+        <v>10</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>95.7</v>
+        <v>45.35</v>
       </c>
       <c r="C5" t="n">
-        <v>105</v>
+        <v>49.7</v>
       </c>
       <c r="D5" t="n">
-        <v>9.720000000000001</v>
+        <v>9.59</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BNAGROCHEM</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>179.56</v>
+        <v>265.35</v>
       </c>
       <c r="C6" t="n">
-        <v>196.95</v>
+        <v>289</v>
       </c>
       <c r="D6" t="n">
-        <v>9.68</v>
+        <v>8.91</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>AMAL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>917.9</v>
       </c>
       <c r="C7" t="n">
-        <v>2.19</v>
+        <v>990</v>
       </c>
       <c r="D7" t="n">
-        <v>9.5</v>
+        <v>7.85</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>63MOONS</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>766.3</v>
+        <v>0.13</v>
       </c>
       <c r="C8" t="n">
-        <v>838.3</v>
+        <v>0.14</v>
       </c>
       <c r="D8" t="n">
-        <v>9.4</v>
+        <v>7.69</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>DELAPLEX</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.03</v>
+        <v>113.7</v>
       </c>
       <c r="C9" t="n">
-        <v>1.12</v>
+        <v>121.6</v>
       </c>
       <c r="D9" t="n">
-        <v>8.74</v>
+        <v>6.95</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>VIKRAN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>214.94</v>
+        <v>55.66</v>
       </c>
       <c r="C10" t="n">
-        <v>233.6</v>
+        <v>59.47</v>
       </c>
       <c r="D10" t="n">
-        <v>8.68</v>
+        <v>6.85</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>SGLRES</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32</v>
+        <v>2.41</v>
       </c>
       <c r="C11" t="n">
-        <v>34.5</v>
+        <v>2.56</v>
       </c>
       <c r="D11" t="n">
-        <v>7.81</v>
+        <v>6.22</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>SIDDHICOTS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.13</v>
+        <v>27.9</v>
       </c>
       <c r="C12" t="n">
-        <v>0.14</v>
+        <v>29.6</v>
       </c>
       <c r="D12" t="n">
-        <v>7.69</v>
+        <v>6.09</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>57.95</v>
+        <v>566.35</v>
       </c>
       <c r="C13" t="n">
-        <v>62.28</v>
+        <v>600</v>
       </c>
       <c r="D13" t="n">
-        <v>7.47</v>
+        <v>5.94</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.86</v>
+        <v>0.17</v>
       </c>
       <c r="C14" t="n">
-        <v>17</v>
+        <v>0.18</v>
       </c>
       <c r="D14" t="n">
-        <v>7.19</v>
+        <v>5.88</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.46</v>
+        <v>0.19</v>
       </c>
       <c r="C15" t="n">
-        <v>5.85</v>
+        <v>0.2</v>
       </c>
       <c r="D15" t="n">
-        <v>7.14</v>
+        <v>5.26</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGL</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12.24</v>
+        <v>232.91</v>
       </c>
       <c r="C16" t="n">
-        <v>13.11</v>
+        <v>245</v>
       </c>
       <c r="D16" t="n">
-        <v>7.11</v>
+        <v>5.19</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>KKJEWELS</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>142.72</v>
+        <v>123.35</v>
       </c>
       <c r="C17" t="n">
-        <v>152.45</v>
+        <v>129.65</v>
       </c>
       <c r="D17" t="n">
-        <v>6.82</v>
+        <v>5.11</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>POONAWALLA</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>447.3</v>
+        <v>218.11</v>
       </c>
       <c r="C18" t="n">
-        <v>476.9</v>
+        <v>229.25</v>
       </c>
       <c r="D18" t="n">
-        <v>6.62</v>
+        <v>5.11</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IVP</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>220.31</v>
+        <v>33.18</v>
       </c>
       <c r="C19" t="n">
-        <v>234.8</v>
+        <v>34.85</v>
       </c>
       <c r="D19" t="n">
-        <v>6.58</v>
+        <v>5.03</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ALFREDHE</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2650</v>
+        <v>182.2</v>
       </c>
       <c r="C20" t="n">
-        <v>2819.9</v>
+        <v>191.31</v>
       </c>
       <c r="D20" t="n">
-        <v>6.41</v>
+        <v>5</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CORDELIA</t>
+          <t>AVATAR</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>100.98</v>
+        <v>183.05</v>
       </c>
       <c r="C21" t="n">
-        <v>107.32</v>
+        <v>192.2</v>
       </c>
       <c r="D21" t="n">
-        <v>6.28</v>
+        <v>5</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AUSTENG</t>
+          <t>BMISL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>153.38</v>
+        <v>146.05</v>
       </c>
       <c r="C22" t="n">
-        <v>163</v>
+        <v>153.35</v>
       </c>
       <c r="D22" t="n">
-        <v>6.27</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6.19</v>
+        <v>624.65</v>
       </c>
       <c r="C23" t="n">
-        <v>6.57</v>
+        <v>655.85</v>
       </c>
       <c r="D23" t="n">
-        <v>6.14</v>
+        <v>4.99</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TWCGOLDETF</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>147.96</v>
+        <v>36.1</v>
       </c>
       <c r="C24" t="n">
-        <v>156.83</v>
+        <v>37.9</v>
       </c>
       <c r="D24" t="n">
-        <v>5.99</v>
+        <v>4.99</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>14.13</v>
+        <v>55.87</v>
       </c>
       <c r="C25" t="n">
-        <v>14.96</v>
+        <v>58.66</v>
       </c>
       <c r="D25" t="n">
-        <v>5.87</v>
+        <v>4.99</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ESFL</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>116.2</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="C26" t="n">
-        <v>123</v>
+        <v>103.05</v>
       </c>
       <c r="D26" t="n">
-        <v>5.85</v>
+        <v>4.99</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>EEPL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>817.85</v>
+        <v>146.6</v>
       </c>
       <c r="C27" t="n">
-        <v>864.9</v>
+        <v>153.9</v>
       </c>
       <c r="D27" t="n">
-        <v>5.75</v>
+        <v>4.98</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BELDING</t>
+          <t>HBESD</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>913.35</v>
+        <v>79.44</v>
       </c>
       <c r="C28" t="n">
-        <v>965</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="D28" t="n">
-        <v>5.66</v>
+        <v>4.98</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>SUPTANERY</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.18</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="C29" t="n">
-        <v>0.19</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="D29" t="n">
-        <v>5.56</v>
+        <v>4.96</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DHRUV</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>23.03</v>
+        <v>14.13</v>
       </c>
       <c r="C30" t="n">
-        <v>24.3</v>
+        <v>14.83</v>
       </c>
       <c r="D30" t="n">
-        <v>5.51</v>
+        <v>4.95</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DIGISPICE</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>15.62</v>
+        <v>45.6</v>
       </c>
       <c r="C31" t="n">
-        <v>16.47</v>
+        <v>47.85</v>
       </c>
       <c r="D31" t="n">
-        <v>5.44</v>
+        <v>4.93</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>SAHANA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>16.58</v>
+        <v>858.85</v>
       </c>
       <c r="C32" t="n">
-        <v>17.45</v>
+        <v>900</v>
       </c>
       <c r="D32" t="n">
-        <v>5.25</v>
+        <v>4.79</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>157.26</v>
+        <v>3.55</v>
       </c>
       <c r="C33" t="n">
-        <v>165.5</v>
+        <v>3.72</v>
       </c>
       <c r="D33" t="n">
-        <v>5.24</v>
+        <v>4.79</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SEPC</t>
+          <t>EBIX</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>5.28</v>
+        <v>15.73</v>
       </c>
       <c r="C34" t="n">
-        <v>5.55</v>
+        <v>16.48</v>
       </c>
       <c r="D34" t="n">
-        <v>5.11</v>
+        <v>4.77</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>ITL</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>7.9</v>
+        <v>361.75</v>
       </c>
       <c r="C35" t="n">
-        <v>8.300000000000001</v>
+        <v>379</v>
       </c>
       <c r="D35" t="n">
-        <v>5.06</v>
+        <v>4.77</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>PATILAUTOM</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>142.9</v>
+        <v>361.8</v>
       </c>
       <c r="C36" t="n">
-        <v>150.04</v>
+        <v>379</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BMISL</t>
+          <t>CEDAAR</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>139.1</v>
+        <v>15.3</v>
       </c>
       <c r="C37" t="n">
-        <v>146.05</v>
+        <v>16</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>4.58</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>38.5</v>
+        <v>150.04</v>
       </c>
       <c r="C38" t="n">
-        <v>40.42</v>
+        <v>156.9</v>
       </c>
       <c r="D38" t="n">
-        <v>4.99</v>
+        <v>4.57</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>50.06</v>
+        <v>0.44</v>
       </c>
       <c r="C39" t="n">
-        <v>52.56</v>
+        <v>0.46</v>
       </c>
       <c r="D39" t="n">
-        <v>4.99</v>
+        <v>4.55</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SIMCA</t>
+          <t>QUINTEGRA</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>354.9</v>
+        <v>1.77</v>
       </c>
       <c r="C40" t="n">
-        <v>372.6</v>
+        <v>1.85</v>
       </c>
       <c r="D40" t="n">
-        <v>4.99</v>
+        <v>4.52</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>XTRANET</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>287.5</v>
+        <v>494.85</v>
       </c>
       <c r="C41" t="n">
-        <v>301.85</v>
+        <v>516.8</v>
       </c>
       <c r="D41" t="n">
-        <v>4.99</v>
+        <v>4.44</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>EEPL</t>
+          <t>ZSARACOM</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>139.65</v>
+        <v>9670</v>
       </c>
       <c r="C42" t="n">
-        <v>146.6</v>
+        <v>10093</v>
       </c>
       <c r="D42" t="n">
-        <v>4.98</v>
+        <v>4.37</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>COREIN</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>13.46</v>
+        <v>105.2</v>
       </c>
       <c r="C43" t="n">
-        <v>14.13</v>
+        <v>109.8</v>
       </c>
       <c r="D43" t="n">
-        <v>4.98</v>
+        <v>4.37</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>28.11</v>
+        <v>0.23</v>
       </c>
       <c r="C44" t="n">
-        <v>29.51</v>
+        <v>0.24</v>
       </c>
       <c r="D44" t="n">
-        <v>4.98</v>
+        <v>4.35</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>KORE</t>
+          <t>AMEYA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>221.8</v>
+        <v>178.5</v>
       </c>
       <c r="C45" t="n">
-        <v>232.85</v>
+        <v>186</v>
       </c>
       <c r="D45" t="n">
-        <v>4.98</v>
+        <v>4.2</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>93.5</v>
+        <v>0.49</v>
       </c>
       <c r="C46" t="n">
-        <v>98.15000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="D46" t="n">
-        <v>4.97</v>
+        <v>4.08</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>VGCL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>34.39</v>
+        <v>50</v>
       </c>
       <c r="C47" t="n">
-        <v>36.1</v>
+        <v>52</v>
       </c>
       <c r="D47" t="n">
-        <v>4.97</v>
+        <v>4</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>26.43</v>
+        <v>11.03</v>
       </c>
       <c r="C48" t="n">
-        <v>27.74</v>
+        <v>11.45</v>
       </c>
       <c r="D48" t="n">
-        <v>4.96</v>
+        <v>3.81</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>15.75</v>
+        <v>34.44</v>
       </c>
       <c r="C49" t="n">
-        <v>16.53</v>
+        <v>35.75</v>
       </c>
       <c r="D49" t="n">
-        <v>4.95</v>
+        <v>3.8</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>HAZOOR</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>43.45</v>
+        <v>16.66</v>
       </c>
       <c r="C50" t="n">
-        <v>45.6</v>
+        <v>17.28</v>
       </c>
       <c r="D50" t="n">
-        <v>4.95</v>
+        <v>3.72</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MICROPRO</t>
+          <t>LYKALABS</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>17.35</v>
+        <v>72.23</v>
       </c>
       <c r="C51" t="n">
-        <v>18.2</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D51" t="n">
-        <v>4.9</v>
+        <v>3.7</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>COREIN</t>
+          <t>AKSHARCHEM</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>100.2</v>
+        <v>390.7</v>
       </c>
       <c r="C52" t="n">
-        <v>105</v>
+        <v>405</v>
       </c>
       <c r="D52" t="n">
-        <v>4.79</v>
+        <v>3.66</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GSTL</t>
+          <t>BALPHARMA</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>12.6</v>
+        <v>97.70999999999999</v>
       </c>
       <c r="C53" t="n">
-        <v>13.2</v>
+        <v>101.2</v>
       </c>
       <c r="D53" t="n">
-        <v>4.76</v>
+        <v>3.57</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>53.95</v>
+        <v>5.99</v>
       </c>
       <c r="C54" t="n">
-        <v>56.5</v>
+        <v>6.2</v>
       </c>
       <c r="D54" t="n">
-        <v>4.73</v>
+        <v>3.51</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>ROCKINGDCE</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>12.3</v>
+        <v>222.2</v>
       </c>
       <c r="C55" t="n">
-        <v>12.88</v>
+        <v>230</v>
       </c>
       <c r="D55" t="n">
-        <v>4.72</v>
+        <v>3.51</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>VETO</t>
+          <t>PAVNAIND</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>131.63</v>
+        <v>14.96</v>
       </c>
       <c r="C56" t="n">
-        <v>137.8</v>
+        <v>15.48</v>
       </c>
       <c r="D56" t="n">
-        <v>4.69</v>
+        <v>3.48</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>ONIXSOLAR</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>47.58</v>
+        <v>376.05</v>
       </c>
       <c r="C57" t="n">
-        <v>49.8</v>
+        <v>389</v>
       </c>
       <c r="D57" t="n">
-        <v>4.67</v>
+        <v>3.44</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>KOLTEPATIL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>23.59</v>
+        <v>425.7</v>
       </c>
       <c r="C58" t="n">
-        <v>24.69</v>
+        <v>440</v>
       </c>
       <c r="D58" t="n">
-        <v>4.66</v>
+        <v>3.36</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>AHCL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>4.35</v>
+        <v>29.51</v>
       </c>
       <c r="C59" t="n">
-        <v>4.55</v>
+        <v>30.5</v>
       </c>
       <c r="D59" t="n">
-        <v>4.6</v>
+        <v>3.35</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>21STCENMGM</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>43.12</v>
+        <v>735.45</v>
       </c>
       <c r="C60" t="n">
-        <v>45.1</v>
+        <v>760</v>
       </c>
       <c r="D60" t="n">
-        <v>4.59</v>
+        <v>3.34</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>SAHYADRI</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>21</v>
+        <v>333.6</v>
       </c>
       <c r="C61" t="n">
-        <v>21.96</v>
+        <v>344.7</v>
       </c>
       <c r="D61" t="n">
-        <v>4.57</v>
+        <v>3.33</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>9.94</v>
+        <v>197.4</v>
       </c>
       <c r="C62" t="n">
-        <v>10.38</v>
+        <v>203.98</v>
       </c>
       <c r="D62" t="n">
-        <v>4.43</v>
+        <v>3.33</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>KOTARISUG</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>30.17</v>
+        <v>25.84</v>
       </c>
       <c r="C63" t="n">
-        <v>31.5</v>
+        <v>26.7</v>
       </c>
       <c r="D63" t="n">
-        <v>4.41</v>
+        <v>3.33</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>272.43</v>
+        <v>12.76</v>
       </c>
       <c r="C64" t="n">
-        <v>284.4</v>
+        <v>13.18</v>
       </c>
       <c r="D64" t="n">
-        <v>4.39</v>
+        <v>3.29</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>2.05</v>
+        <v>18.79</v>
       </c>
       <c r="C65" t="n">
-        <v>2.14</v>
+        <v>19.4</v>
       </c>
       <c r="D65" t="n">
-        <v>4.39</v>
+        <v>3.25</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>AEQUS</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>17.86</v>
+        <v>265.9</v>
       </c>
       <c r="C66" t="n">
-        <v>18.64</v>
+        <v>274.45</v>
       </c>
       <c r="D66" t="n">
-        <v>4.37</v>
+        <v>3.22</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>3.44</v>
+        <v>544.7</v>
       </c>
       <c r="C67" t="n">
-        <v>3.59</v>
+        <v>562</v>
       </c>
       <c r="D67" t="n">
-        <v>4.36</v>
+        <v>3.18</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>16.19</v>
+        <v>118.59</v>
       </c>
       <c r="C68" t="n">
-        <v>16.89</v>
+        <v>122.35</v>
       </c>
       <c r="D68" t="n">
-        <v>4.32</v>
+        <v>3.17</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>594.95</v>
+        <v>57.94</v>
       </c>
       <c r="C69" t="n">
-        <v>620.4</v>
+        <v>59.77</v>
       </c>
       <c r="D69" t="n">
-        <v>4.28</v>
+        <v>3.16</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>MAKERSL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.47</v>
+        <v>187</v>
       </c>
       <c r="C70" t="n">
-        <v>0.49</v>
+        <v>192.9</v>
       </c>
       <c r="D70" t="n">
-        <v>4.26</v>
+        <v>3.16</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TEXMOPIPES</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>51.21</v>
+        <v>18.23</v>
       </c>
       <c r="C71" t="n">
-        <v>53.39</v>
+        <v>18.8</v>
       </c>
       <c r="D71" t="n">
-        <v>4.26</v>
+        <v>3.13</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>173.53</v>
+        <v>387.1</v>
       </c>
       <c r="C72" t="n">
-        <v>180.89</v>
+        <v>398.95</v>
       </c>
       <c r="D72" t="n">
-        <v>4.24</v>
+        <v>3.06</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LOTUSCHO</t>
+          <t>GENCON</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>565.1</v>
+        <v>36.22</v>
       </c>
       <c r="C73" t="n">
-        <v>589</v>
+        <v>37.3</v>
       </c>
       <c r="D73" t="n">
-        <v>4.23</v>
+        <v>2.98</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>GALLANTT</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>503.75</v>
+        <v>76.14</v>
       </c>
       <c r="C74" t="n">
-        <v>524.95</v>
+        <v>78.39</v>
       </c>
       <c r="D74" t="n">
-        <v>4.21</v>
+        <v>2.96</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>6.18</v>
+        <v>25.88</v>
       </c>
       <c r="C75" t="n">
-        <v>6.44</v>
+        <v>26.64</v>
       </c>
       <c r="D75" t="n">
-        <v>4.21</v>
+        <v>2.94</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>AGOL</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>12.85</v>
+        <v>4.84</v>
       </c>
       <c r="C76" t="n">
-        <v>13.39</v>
+        <v>4.98</v>
       </c>
       <c r="D76" t="n">
-        <v>4.2</v>
+        <v>2.89</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>BANDHANBNK</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>111.33</v>
+        <v>157.5</v>
       </c>
       <c r="C77" t="n">
-        <v>116</v>
+        <v>162</v>
       </c>
       <c r="D77" t="n">
-        <v>4.19</v>
+        <v>2.86</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>4.11</v>
+        <v>57.71</v>
       </c>
       <c r="C78" t="n">
-        <v>4.28</v>
+        <v>59.35</v>
       </c>
       <c r="D78" t="n">
-        <v>4.14</v>
+        <v>2.84</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AARTECH</t>
+          <t>QUALIANCE</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>47.82</v>
+        <v>195.3</v>
       </c>
       <c r="C79" t="n">
-        <v>49.8</v>
+        <v>200.85</v>
       </c>
       <c r="D79" t="n">
-        <v>4.14</v>
+        <v>2.84</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AMEYA</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>170</v>
+        <v>1.41</v>
       </c>
       <c r="C80" t="n">
-        <v>177</v>
+        <v>1.45</v>
       </c>
       <c r="D80" t="n">
-        <v>4.12</v>
+        <v>2.84</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>21.9</v>
+        <v>2.14</v>
       </c>
       <c r="C81" t="n">
-        <v>22.8</v>
+        <v>2.2</v>
       </c>
       <c r="D81" t="n">
-        <v>4.11</v>
+        <v>2.8</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AKANKSHA</t>
+          <t>DBSTOCKBRO</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>175.9</v>
+        <v>31.13</v>
       </c>
       <c r="C82" t="n">
-        <v>183</v>
+        <v>32</v>
       </c>
       <c r="D82" t="n">
-        <v>4.04</v>
+        <v>2.79</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PREMIERPOL</t>
+          <t>RULKA</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>102.85</v>
+        <v>100.5</v>
       </c>
       <c r="C83" t="n">
-        <v>107</v>
+        <v>103.3</v>
       </c>
       <c r="D83" t="n">
-        <v>4.04</v>
+        <v>2.79</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TOYAMSL</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.76</v>
+        <v>0.36</v>
       </c>
       <c r="C84" t="n">
-        <v>0.79</v>
+        <v>0.37</v>
       </c>
       <c r="D84" t="n">
-        <v>3.95</v>
+        <v>2.78</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>RTSPOWR</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>119.33</v>
+        <v>6.47</v>
       </c>
       <c r="C85" t="n">
-        <v>123.97</v>
+        <v>6.65</v>
       </c>
       <c r="D85" t="n">
-        <v>3.89</v>
+        <v>2.78</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ABSMARINE</t>
+          <t>IRCON</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>310</v>
+        <v>104.73</v>
       </c>
       <c r="C86" t="n">
-        <v>321.95</v>
+        <v>107.6</v>
       </c>
       <c r="D86" t="n">
-        <v>3.85</v>
+        <v>2.74</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>AARTECH</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>26.3</v>
+        <v>46.73</v>
       </c>
       <c r="C87" t="n">
-        <v>27.3</v>
+        <v>48</v>
       </c>
       <c r="D87" t="n">
-        <v>3.8</v>
+        <v>2.72</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>215.72</v>
+        <v>208.13</v>
       </c>
       <c r="C88" t="n">
-        <v>223.9</v>
+        <v>213.8</v>
       </c>
       <c r="D88" t="n">
-        <v>3.79</v>
+        <v>2.72</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GRAVITA</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1466.4</v>
+        <v>19.18</v>
       </c>
       <c r="C89" t="n">
-        <v>1521.9</v>
+        <v>19.7</v>
       </c>
       <c r="D89" t="n">
-        <v>3.78</v>
+        <v>2.71</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>42.21</v>
+        <v>1007.8</v>
       </c>
       <c r="C90" t="n">
-        <v>43.8</v>
+        <v>1035</v>
       </c>
       <c r="D90" t="n">
-        <v>3.77</v>
+        <v>2.7</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ASHUTOSH</t>
+          <t>RISHABH</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>142.6</v>
+        <v>679.55</v>
       </c>
       <c r="C91" t="n">
-        <v>147.95</v>
+        <v>697.7</v>
       </c>
       <c r="D91" t="n">
-        <v>3.75</v>
+        <v>2.67</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>VHL</t>
+          <t>SKYGOLD</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3650</v>
+        <v>968.25</v>
       </c>
       <c r="C92" t="n">
-        <v>3785</v>
+        <v>994</v>
       </c>
       <c r="D92" t="n">
-        <v>3.7</v>
+        <v>2.66</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>GRPLTD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>50.12</v>
+        <v>1700.8</v>
       </c>
       <c r="C93" t="n">
-        <v>51.97</v>
+        <v>1745</v>
       </c>
       <c r="D93" t="n">
-        <v>3.69</v>
+        <v>2.6</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>JYOTIRES</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>839.1</v>
+        <v>72.52</v>
       </c>
       <c r="C94" t="n">
-        <v>870</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="D94" t="n">
-        <v>3.68</v>
+        <v>2.59</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>SARVESHWAR</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>273.95</v>
+        <v>3.86</v>
       </c>
       <c r="C95" t="n">
-        <v>283.95</v>
+        <v>3.96</v>
       </c>
       <c r="D95" t="n">
-        <v>3.65</v>
+        <v>2.59</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>INNOMET</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>954.3</v>
+        <v>251.5</v>
       </c>
       <c r="C96" t="n">
-        <v>989</v>
+        <v>258</v>
       </c>
       <c r="D96" t="n">
-        <v>3.64</v>
+        <v>2.58</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>RAMBHAJO</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>51.14</v>
+        <v>375.3</v>
       </c>
       <c r="C97" t="n">
-        <v>52.99</v>
+        <v>385</v>
       </c>
       <c r="D97" t="n">
-        <v>3.62</v>
+        <v>2.58</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>KONSTELEC</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>77.12</v>
+        <v>49.15</v>
       </c>
       <c r="C98" t="n">
-        <v>79.90000000000001</v>
+        <v>50.4</v>
       </c>
       <c r="D98" t="n">
-        <v>3.6</v>
+        <v>2.54</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>617.8</v>
+        <v>24.83</v>
       </c>
       <c r="C99" t="n">
-        <v>640</v>
+        <v>25.45</v>
       </c>
       <c r="D99" t="n">
-        <v>3.59</v>
+        <v>2.5</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>MAWANASUG</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1.68</v>
+        <v>168.79</v>
       </c>
       <c r="C100" t="n">
-        <v>1.74</v>
+        <v>173</v>
       </c>
       <c r="D100" t="n">
-        <v>3.57</v>
+        <v>2.49</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>AKSHOPTFBR</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>52.24</v>
+        <v>7.27</v>
       </c>
       <c r="C101" t="n">
-        <v>54.1</v>
+        <v>7.45</v>
       </c>
       <c r="D101" t="n">
-        <v>3.56</v>
+        <v>2.48</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>AMBAAUTO</t>
+          <t>TOLINS</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>113.95</v>
+        <v>85.58</v>
       </c>
       <c r="C102" t="n">
-        <v>118</v>
+        <v>87.7</v>
       </c>
       <c r="D102" t="n">
-        <v>3.55</v>
+        <v>2.48</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MUNJALAU</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>101.32</v>
+        <v>175.66</v>
       </c>
       <c r="C103" t="n">
-        <v>104.87</v>
+        <v>180</v>
       </c>
       <c r="D103" t="n">
-        <v>3.5</v>
+        <v>2.47</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MANINDS</t>
+          <t>HLVLTD</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>867.9</v>
+        <v>6.08</v>
       </c>
       <c r="C104" t="n">
-        <v>898</v>
+        <v>6.23</v>
       </c>
       <c r="D104" t="n">
-        <v>3.47</v>
+        <v>2.47</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CRSL</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>2.07</v>
+        <v>26.87</v>
       </c>
       <c r="C105" t="n">
-        <v>2.14</v>
+        <v>27.5</v>
       </c>
       <c r="D105" t="n">
-        <v>3.38</v>
+        <v>2.34</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>INDOAMIN</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>157.72</v>
+        <v>18.07</v>
       </c>
       <c r="C106" t="n">
-        <v>163</v>
+        <v>18.49</v>
       </c>
       <c r="D106" t="n">
-        <v>3.35</v>
+        <v>2.32</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MVGJL</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>207.87</v>
+        <v>50.33</v>
       </c>
       <c r="C107" t="n">
-        <v>214.8</v>
+        <v>51.5</v>
       </c>
       <c r="D107" t="n">
-        <v>3.33</v>
+        <v>2.32</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>HLEGLAS</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>108.41</v>
+        <v>406.6</v>
       </c>
       <c r="C108" t="n">
-        <v>112</v>
+        <v>416</v>
       </c>
       <c r="D108" t="n">
-        <v>3.31</v>
+        <v>2.31</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1015.45</v>
+        <v>0.87</v>
       </c>
       <c r="C109" t="n">
-        <v>1048.95</v>
+        <v>0.89</v>
       </c>
       <c r="D109" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>AUGMONT</t>
+          <t>RAJSREESUG</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1337.8</v>
+        <v>30.99</v>
       </c>
       <c r="C110" t="n">
-        <v>1381.8</v>
+        <v>31.7</v>
       </c>
       <c r="D110" t="n">
-        <v>3.29</v>
+        <v>2.29</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>5.79</v>
+        <v>41.62</v>
       </c>
       <c r="C111" t="n">
-        <v>5.98</v>
+        <v>42.57</v>
       </c>
       <c r="D111" t="n">
-        <v>3.28</v>
+        <v>2.28</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>20.71</v>
+        <v>380.35</v>
       </c>
       <c r="C112" t="n">
-        <v>21.38</v>
+        <v>389</v>
       </c>
       <c r="D112" t="n">
-        <v>3.24</v>
+        <v>2.27</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>290.6</v>
+        <v>1.33</v>
       </c>
       <c r="C113" t="n">
-        <v>300</v>
+        <v>1.36</v>
       </c>
       <c r="D113" t="n">
-        <v>3.23</v>
+        <v>2.26</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DELAPLEX</t>
+          <t>DEVX</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>94.75</v>
+        <v>41.66</v>
       </c>
       <c r="C114" t="n">
-        <v>97.8</v>
+        <v>42.6</v>
       </c>
       <c r="D114" t="n">
-        <v>3.22</v>
+        <v>2.26</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SYNGENE</t>
+          <t>KANPRPLA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>347.4</v>
+        <v>241.35</v>
       </c>
       <c r="C115" t="n">
-        <v>358.5</v>
+        <v>246.75</v>
       </c>
       <c r="D115" t="n">
-        <v>3.2</v>
+        <v>2.24</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>ALKALI</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>21.04</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="C116" t="n">
-        <v>21.71</v>
+        <v>96</v>
       </c>
       <c r="D116" t="n">
-        <v>3.18</v>
+        <v>2.24</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>31.88</v>
+        <v>4.98</v>
       </c>
       <c r="C117" t="n">
-        <v>32.89</v>
+        <v>5.09</v>
       </c>
       <c r="D117" t="n">
-        <v>3.17</v>
+        <v>2.21</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DEVIT</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>19.39</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="C118" t="n">
-        <v>20</v>
+        <v>10.19</v>
       </c>
       <c r="D118" t="n">
-        <v>3.15</v>
+        <v>2.21</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MEESHO</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>232.74</v>
+        <v>28.87</v>
       </c>
       <c r="C119" t="n">
-        <v>240</v>
+        <v>29.5</v>
       </c>
       <c r="D119" t="n">
-        <v>3.12</v>
+        <v>2.18</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ONIXSOLAR</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>380.15</v>
+        <v>20.16</v>
       </c>
       <c r="C120" t="n">
-        <v>392</v>
+        <v>20.6</v>
       </c>
       <c r="D120" t="n">
-        <v>3.12</v>
+        <v>2.18</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>HLVLTD</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>6.11</v>
+        <v>0.46</v>
       </c>
       <c r="C121" t="n">
-        <v>6.3</v>
+        <v>0.47</v>
       </c>
       <c r="D121" t="n">
-        <v>3.11</v>
+        <v>2.17</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CRAMC</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>219.95</v>
+        <v>53.83</v>
       </c>
       <c r="C122" t="n">
-        <v>226.75</v>
+        <v>55</v>
       </c>
       <c r="D122" t="n">
-        <v>3.09</v>
+        <v>2.17</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>POOJALOGIS</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>132.7</v>
+        <v>18</v>
       </c>
       <c r="C123" t="n">
-        <v>136.8</v>
+        <v>18.39</v>
       </c>
       <c r="D123" t="n">
-        <v>3.09</v>
+        <v>2.17</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ZIMLAB</t>
+          <t>SPUNWEB</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>150.47</v>
+        <v>129</v>
       </c>
       <c r="C124" t="n">
-        <v>155.1</v>
+        <v>131.8</v>
       </c>
       <c r="D124" t="n">
-        <v>3.08</v>
+        <v>2.17</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>77.36</v>
+        <v>3.26</v>
       </c>
       <c r="C125" t="n">
-        <v>79.7</v>
+        <v>3.33</v>
       </c>
       <c r="D125" t="n">
-        <v>3.02</v>
+        <v>2.15</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5.33</v>
+        <v>49.92</v>
       </c>
       <c r="C126" t="n">
-        <v>5.49</v>
+        <v>50.98</v>
       </c>
       <c r="D126" t="n">
-        <v>3</v>
+        <v>2.12</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MICEL</t>
+          <t>ELIN</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>34.37</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="C127" t="n">
-        <v>35.4</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="D127" t="n">
-        <v>3</v>
+        <v>2.11</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>TEXMOPIPES</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>20.07</v>
+        <v>51.52</v>
       </c>
       <c r="C128" t="n">
-        <v>20.67</v>
+        <v>52.6</v>
       </c>
       <c r="D128" t="n">
-        <v>2.99</v>
+        <v>2.1</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>TTML</t>
+          <t>KANCHI</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>32.89</v>
+        <v>359.4</v>
       </c>
       <c r="C129" t="n">
-        <v>33.87</v>
+        <v>366.95</v>
       </c>
       <c r="D129" t="n">
-        <v>2.98</v>
+        <v>2.1</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RMC</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>184.33</v>
+        <v>3.33</v>
       </c>
       <c r="C130" t="n">
-        <v>189.8</v>
+        <v>3.4</v>
       </c>
       <c r="D130" t="n">
-        <v>2.97</v>
+        <v>2.1</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>KOKUYOCMLN</t>
+          <t>BANSWRAS</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>72.65000000000001</v>
+        <v>100.66</v>
       </c>
       <c r="C131" t="n">
-        <v>74.8</v>
+        <v>102.75</v>
       </c>
       <c r="D131" t="n">
-        <v>2.96</v>
+        <v>2.08</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ARROWGREEN</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>855.65</v>
+        <v>6.25</v>
       </c>
       <c r="C132" t="n">
-        <v>881</v>
+        <v>6.38</v>
       </c>
       <c r="D132" t="n">
-        <v>2.96</v>
+        <v>2.08</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ASHOKA</t>
+          <t>NECLIFE</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>102.02</v>
+        <v>10.14</v>
       </c>
       <c r="C133" t="n">
-        <v>105</v>
+        <v>10.35</v>
       </c>
       <c r="D133" t="n">
-        <v>2.92</v>
+        <v>2.07</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>VIRINCHI</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>12.81</v>
+        <v>31.05</v>
       </c>
       <c r="C134" t="n">
-        <v>13.18</v>
+        <v>31.69</v>
       </c>
       <c r="D134" t="n">
-        <v>2.89</v>
+        <v>2.06</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>PRIORITY</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>325.55</v>
+        <v>670.75</v>
       </c>
       <c r="C135" t="n">
-        <v>334.95</v>
+        <v>684.6</v>
       </c>
       <c r="D135" t="n">
-        <v>2.89</v>
+        <v>2.06</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1.74</v>
+        <v>6.35</v>
       </c>
       <c r="C136" t="n">
-        <v>1.79</v>
+        <v>6.48</v>
       </c>
       <c r="D136" t="n">
-        <v>2.87</v>
+        <v>2.05</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GANESHHOU</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>699.5</v>
+        <v>41.53</v>
       </c>
       <c r="C137" t="n">
-        <v>719.5</v>
+        <v>42.38</v>
       </c>
       <c r="D137" t="n">
-        <v>2.86</v>
+        <v>2.05</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>PRISMX</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>14</v>
+        <v>0.49</v>
       </c>
       <c r="C138" t="n">
-        <v>14.4</v>
+        <v>0.5</v>
       </c>
       <c r="D138" t="n">
-        <v>2.86</v>
+        <v>2.04</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SATIA</t>
+          <t>DIGIDRIVE</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>68.06</v>
+        <v>18.7</v>
       </c>
       <c r="C139" t="n">
-        <v>70</v>
+        <v>19.08</v>
       </c>
       <c r="D139" t="n">
-        <v>2.85</v>
+        <v>2.03</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>CGVAK</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1676.4</v>
+        <v>133.78</v>
       </c>
       <c r="C140" t="n">
-        <v>1724</v>
+        <v>136.49</v>
       </c>
       <c r="D140" t="n">
-        <v>2.84</v>
+        <v>2.03</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>TEAMGTY</t>
+          <t>NICCOPAR</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>243.02</v>
+        <v>70.06999999999999</v>
       </c>
       <c r="C141" t="n">
-        <v>249.9</v>
+        <v>71.48999999999999</v>
       </c>
       <c r="D141" t="n">
-        <v>2.83</v>
+        <v>2.03</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>TINNARUBR</t>
+          <t>GENUSPAPER</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>885.85</v>
+        <v>10.38</v>
       </c>
       <c r="C142" t="n">
-        <v>910.95</v>
+        <v>10.59</v>
       </c>
       <c r="D142" t="n">
-        <v>2.83</v>
+        <v>2.02</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>ADVIKCA</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>279.05</v>
+        <v>0.99</v>
       </c>
       <c r="C143" t="n">
-        <v>286.95</v>
+        <v>1.01</v>
       </c>
       <c r="D143" t="n">
-        <v>2.83</v>
+        <v>2.02</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>INDIANCARD</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>36.33</v>
+        <v>183.99</v>
       </c>
       <c r="C144" t="n">
-        <v>37.35</v>
+        <v>187.69</v>
       </c>
       <c r="D144" t="n">
-        <v>2.81</v>
+        <v>2.01</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>5.72</v>
+        <v>35.38</v>
       </c>
       <c r="C145" t="n">
-        <v>5.88</v>
+        <v>36.09</v>
       </c>
       <c r="D145" t="n">
-        <v>2.8</v>
+        <v>2.01</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>GINNIFILA</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>40.75</v>
+        <v>48.04</v>
       </c>
       <c r="C146" t="n">
-        <v>41.89</v>
+        <v>49</v>
       </c>
       <c r="D146" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>18</v>
+        <v>209.01</v>
       </c>
       <c r="C147" t="n">
-        <v>18.5</v>
+        <v>213.19</v>
       </c>
       <c r="D147" t="n">
-        <v>2.78</v>
+        <v>2</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>VIKASECO</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.36</v>
+        <v>1</v>
       </c>
       <c r="C148" t="n">
-        <v>0.37</v>
+        <v>1.02</v>
       </c>
       <c r="D148" t="n">
-        <v>2.78</v>
+        <v>2</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>IWARE</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>349.3</v>
+        <v>21.46</v>
       </c>
       <c r="C149" t="n">
-        <v>359</v>
+        <v>21.89</v>
       </c>
       <c r="D149" t="n">
-        <v>2.78</v>
+        <v>2</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>TRIVENI</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>235.67</v>
+        <v>83.53</v>
       </c>
       <c r="C150" t="n">
-        <v>242.2</v>
+        <v>85.2</v>
       </c>
       <c r="D150" t="n">
-        <v>2.77</v>
+        <v>2</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>KOTHARIPRO</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>62.26</v>
+        <v>0.5</v>
       </c>
       <c r="C151" t="n">
-        <v>63.97</v>
+        <v>0.51</v>
       </c>
       <c r="D151" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SICAGEN</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>50.45</v>
+        <v>56.52</v>
       </c>
       <c r="C152" t="n">
-        <v>51.83</v>
+        <v>57.65</v>
       </c>
       <c r="D152" t="n">
-        <v>2.74</v>
+        <v>2</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>105.13</v>
+        <v>4</v>
       </c>
       <c r="C153" t="n">
-        <v>108</v>
+        <v>4.08</v>
       </c>
       <c r="D153" t="n">
-        <v>2.73</v>
+        <v>2</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>NECLIFE</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>10.13</v>
+        <v>20.58</v>
       </c>
       <c r="C154" t="n">
-        <v>10.4</v>
+        <v>20.99</v>
       </c>
       <c r="D154" t="n">
-        <v>2.67</v>
+        <v>1.99</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>RAMBHAJO</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>357.45</v>
+        <v>21.64</v>
       </c>
       <c r="C155" t="n">
-        <v>367</v>
+        <v>22.07</v>
       </c>
       <c r="D155" t="n">
-        <v>2.67</v>
+        <v>1.99</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SURANAT&amp;P</t>
+          <t>GTPL</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>15.54</v>
+        <v>56.77</v>
       </c>
       <c r="C156" t="n">
-        <v>15.95</v>
+        <v>57.9</v>
       </c>
       <c r="D156" t="n">
-        <v>2.64</v>
+        <v>1.99</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>HAZOOR</t>
+          <t>ZFSTEERING</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>16.27</v>
+        <v>680.9</v>
       </c>
       <c r="C157" t="n">
-        <v>16.7</v>
+        <v>694.45</v>
       </c>
       <c r="D157" t="n">
-        <v>2.64</v>
+        <v>1.99</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>LCL</t>
+          <t>BHARATRAS</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>630.85</v>
+        <v>970.6</v>
       </c>
       <c r="C158" t="n">
-        <v>647.45</v>
+        <v>989.8</v>
       </c>
       <c r="D158" t="n">
-        <v>2.63</v>
+        <v>1.98</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>UCAL</t>
+          <t>SECMARK</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>134.36</v>
+        <v>151.19</v>
       </c>
       <c r="C159" t="n">
-        <v>137.89</v>
+        <v>154.19</v>
       </c>
       <c r="D159" t="n">
-        <v>2.63</v>
+        <v>1.98</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>TEAMGTY</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>218.54</v>
+        <v>244.03</v>
       </c>
       <c r="C160" t="n">
-        <v>224.2</v>
+        <v>248.85</v>
       </c>
       <c r="D160" t="n">
-        <v>2.59</v>
+        <v>1.98</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>DCM</t>
+          <t>KHAITANLTD</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>71.17</v>
+        <v>148.08</v>
       </c>
       <c r="C161" t="n">
-        <v>73</v>
+        <v>150.99</v>
       </c>
       <c r="D161" t="n">
-        <v>2.57</v>
+        <v>1.97</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>GTL</t>
+          <t>AATMAJ</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>6.64</v>
+        <v>22.95</v>
       </c>
       <c r="C162" t="n">
-        <v>6.81</v>
+        <v>23.4</v>
       </c>
       <c r="D162" t="n">
-        <v>2.56</v>
+        <v>1.96</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>MANIKA</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>54.21</v>
+        <v>56.2</v>
       </c>
       <c r="C163" t="n">
-        <v>55.6</v>
+        <v>57.29</v>
       </c>
       <c r="D163" t="n">
-        <v>2.56</v>
+        <v>1.94</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RISHABH</t>
+          <t>UMIYA-MRO</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>677.9</v>
+        <v>94.61</v>
       </c>
       <c r="C164" t="n">
-        <v>695</v>
+        <v>96.45</v>
       </c>
       <c r="D164" t="n">
-        <v>2.52</v>
+        <v>1.94</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>4.4</v>
+        <v>107.99</v>
       </c>
       <c r="C165" t="n">
-        <v>4.51</v>
+        <v>110.09</v>
       </c>
       <c r="D165" t="n">
-        <v>2.5</v>
+        <v>1.94</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>OMAXAUTO</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>32.19</v>
+        <v>220.61</v>
       </c>
       <c r="C166" t="n">
-        <v>32.99</v>
+        <v>224.9</v>
       </c>
       <c r="D166" t="n">
-        <v>2.49</v>
+        <v>1.94</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>LKPSEC</t>
+          <t>KOTHARIPRO</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>13.63</v>
+        <v>61.7</v>
       </c>
       <c r="C167" t="n">
-        <v>13.97</v>
+        <v>62.89</v>
       </c>
       <c r="D167" t="n">
-        <v>2.49</v>
+        <v>1.93</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>JISLDVREQS</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>21.27</v>
+        <v>18.63</v>
       </c>
       <c r="C168" t="n">
-        <v>21.8</v>
+        <v>18.99</v>
       </c>
       <c r="D168" t="n">
-        <v>2.49</v>
+        <v>1.93</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>AERONEU</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>3121.7</v>
+        <v>70.53</v>
       </c>
       <c r="C169" t="n">
-        <v>3198.7</v>
+        <v>71.89</v>
       </c>
       <c r="D169" t="n">
-        <v>2.47</v>
+        <v>1.93</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>ANNU</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>40.6</v>
+        <v>46.6</v>
       </c>
       <c r="C170" t="n">
-        <v>41.6</v>
+        <v>47.5</v>
       </c>
       <c r="D170" t="n">
-        <v>2.46</v>
+        <v>1.93</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>RHETAN</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>189.25</v>
+        <v>16.67</v>
       </c>
       <c r="C171" t="n">
-        <v>193.9</v>
+        <v>16.99</v>
       </c>
       <c r="D171" t="n">
-        <v>2.46</v>
+        <v>1.92</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>YOGI</t>
+          <t>OSWALGREEN</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>159.99</v>
+        <v>18.73</v>
       </c>
       <c r="C172" t="n">
-        <v>163.9</v>
+        <v>19.09</v>
       </c>
       <c r="D172" t="n">
-        <v>2.44</v>
+        <v>1.92</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>BTML</t>
+          <t>HMT</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>7.02</v>
+        <v>54.8</v>
       </c>
       <c r="C173" t="n">
-        <v>7.19</v>
+        <v>55.85</v>
       </c>
       <c r="D173" t="n">
-        <v>2.42</v>
+        <v>1.92</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SHADOWFAX</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>294.85</v>
+        <v>4.19</v>
       </c>
       <c r="C174" t="n">
-        <v>302</v>
+        <v>4.27</v>
       </c>
       <c r="D174" t="n">
-        <v>2.42</v>
+        <v>1.91</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>LINC</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>81.54000000000001</v>
+        <v>5.77</v>
       </c>
       <c r="C175" t="n">
-        <v>83.5</v>
+        <v>5.88</v>
       </c>
       <c r="D175" t="n">
-        <v>2.4</v>
+        <v>1.91</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ASHIKAG</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>380.8</v>
+        <v>3.67</v>
       </c>
       <c r="C176" t="n">
-        <v>389.8</v>
+        <v>3.74</v>
       </c>
       <c r="D176" t="n">
-        <v>2.36</v>
+        <v>1.91</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>OSELDEVICE</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>366.35</v>
+        <v>54.66</v>
       </c>
       <c r="C177" t="n">
-        <v>375</v>
+        <v>55.7</v>
       </c>
       <c r="D177" t="n">
-        <v>2.36</v>
+        <v>1.9</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>GANECOS</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>966.1</v>
+        <v>15.88</v>
       </c>
       <c r="C178" t="n">
-        <v>988.9</v>
+        <v>16.18</v>
       </c>
       <c r="D178" t="n">
-        <v>2.36</v>
+        <v>1.89</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>55.6</v>
+        <v>140.35</v>
       </c>
       <c r="C179" t="n">
-        <v>56.9</v>
+        <v>143</v>
       </c>
       <c r="D179" t="n">
-        <v>2.34</v>
+        <v>1.89</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.86</v>
+        <v>53.48</v>
       </c>
       <c r="C180" t="n">
-        <v>0.88</v>
+        <v>54.49</v>
       </c>
       <c r="D180" t="n">
-        <v>2.33</v>
+        <v>1.89</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ELDEHSG</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>786.45</v>
+        <v>22.92</v>
       </c>
       <c r="C181" t="n">
-        <v>804.8</v>
+        <v>23.35</v>
       </c>
       <c r="D181" t="n">
-        <v>2.33</v>
+        <v>1.88</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>0.43</v>
+        <v>37.3</v>
       </c>
       <c r="C182" t="n">
-        <v>0.44</v>
+        <v>38</v>
       </c>
       <c r="D182" t="n">
-        <v>2.33</v>
+        <v>1.88</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>JINDALPHOT</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>1021.6</v>
+        <v>12.83</v>
       </c>
       <c r="C183" t="n">
-        <v>1045</v>
+        <v>13.07</v>
       </c>
       <c r="D183" t="n">
-        <v>2.29</v>
+        <v>1.87</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>SHILPAMED</t>
+          <t>MODIS</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>1021.7</v>
+        <v>417.25</v>
       </c>
       <c r="C184" t="n">
-        <v>1045</v>
+        <v>425</v>
       </c>
       <c r="D184" t="n">
-        <v>2.28</v>
+        <v>1.86</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>RAJOOENG</t>
+          <t>LATTEYS</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>59.45</v>
+        <v>20.02</v>
       </c>
       <c r="C185" t="n">
-        <v>60.8</v>
+        <v>20.39</v>
       </c>
       <c r="D185" t="n">
-        <v>2.27</v>
+        <v>1.85</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>RAMAPHO</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>109.52</v>
+        <v>17.86</v>
       </c>
       <c r="C186" t="n">
-        <v>112</v>
+        <v>18.19</v>
       </c>
       <c r="D186" t="n">
-        <v>2.26</v>
+        <v>1.85</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>105.14</v>
+        <v>10.79</v>
       </c>
       <c r="C187" t="n">
-        <v>107.52</v>
+        <v>10.99</v>
       </c>
       <c r="D187" t="n">
-        <v>2.26</v>
+        <v>1.85</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ODYCORP</t>
+          <t>SUDARCOLOR</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>6.64</v>
+        <v>362.35</v>
       </c>
       <c r="C188" t="n">
-        <v>6.79</v>
+        <v>369</v>
       </c>
       <c r="D188" t="n">
-        <v>2.26</v>
+        <v>1.84</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KSE</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>176.02</v>
+        <v>604.85</v>
       </c>
       <c r="C189" t="n">
-        <v>180</v>
+        <v>616</v>
       </c>
       <c r="D189" t="n">
-        <v>2.26</v>
+        <v>1.84</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>AMDIND</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>49.29</v>
+        <v>1223</v>
       </c>
       <c r="C190" t="n">
-        <v>50.4</v>
+        <v>1245.4</v>
       </c>
       <c r="D190" t="n">
-        <v>2.25</v>
+        <v>1.83</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>SAFEENTP</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>239.6</v>
+        <v>355.5</v>
       </c>
       <c r="C191" t="n">
-        <v>245</v>
+        <v>362</v>
       </c>
       <c r="D191" t="n">
-        <v>2.25</v>
+        <v>1.83</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>GKSL</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>184.09</v>
+        <v>6.08</v>
       </c>
       <c r="C192" t="n">
-        <v>188.22</v>
+        <v>6.19</v>
       </c>
       <c r="D192" t="n">
-        <v>2.24</v>
+        <v>1.81</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>HINDALUMI</t>
+          <t>TRF</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>89.5</v>
+        <v>227.89</v>
       </c>
       <c r="C193" t="n">
-        <v>91.5</v>
+        <v>231.99</v>
       </c>
       <c r="D193" t="n">
-        <v>2.23</v>
+        <v>1.8</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>WATERBASE</t>
+          <t>VIVOBIOT</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>44.31</v>
+        <v>14.43</v>
       </c>
       <c r="C194" t="n">
-        <v>45.3</v>
+        <v>14.69</v>
       </c>
       <c r="D194" t="n">
-        <v>2.23</v>
+        <v>1.8</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PARAGMILK</t>
+          <t>OMFREIGHT</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>306.4</v>
+        <v>107.97</v>
       </c>
       <c r="C195" t="n">
-        <v>313.2</v>
+        <v>109.9</v>
       </c>
       <c r="D195" t="n">
-        <v>2.22</v>
+        <v>1.79</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>OSWALPUMPS</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>254.35</v>
+        <v>19.15</v>
       </c>
       <c r="C196" t="n">
-        <v>260</v>
+        <v>19.49</v>
       </c>
       <c r="D196" t="n">
-        <v>2.22</v>
+        <v>1.78</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>AZAD</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>11.24</v>
+        <v>2968.4</v>
       </c>
       <c r="C197" t="n">
-        <v>11.49</v>
+        <v>3021.1</v>
       </c>
       <c r="D197" t="n">
-        <v>2.22</v>
+        <v>1.78</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>MANAKSIA</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>89.5</v>
+        <v>57.76</v>
       </c>
       <c r="C198" t="n">
-        <v>91.48999999999999</v>
+        <v>58.79</v>
       </c>
       <c r="D198" t="n">
-        <v>2.22</v>
+        <v>1.78</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KSHINTL</t>
+          <t>VGUARD</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>1001.5</v>
+        <v>288.9</v>
       </c>
       <c r="C199" t="n">
-        <v>1023.5</v>
+        <v>294</v>
       </c>
       <c r="D199" t="n">
-        <v>2.2</v>
+        <v>1.77</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MINDTECK</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>139.37</v>
+        <v>23.18</v>
       </c>
       <c r="C200" t="n">
-        <v>142.4</v>
+        <v>23.59</v>
       </c>
       <c r="D200" t="n">
-        <v>2.17</v>
+        <v>1.77</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>1.39</v>
+        <v>148.79</v>
       </c>
       <c r="C201" t="n">
-        <v>1.42</v>
+        <v>151.4</v>
       </c>
       <c r="D201" t="n">
-        <v>2.16</v>
+        <v>1.75</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-14 09:01 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ARTNIRMAN</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36.43</v>
+        <v>730</v>
       </c>
       <c r="C2" t="n">
-        <v>42.7</v>
+        <v>862.45</v>
       </c>
       <c r="D2" t="n">
-        <v>17.21</v>
+        <v>18.14</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PHOENXINTL</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33.44</v>
+        <v>52.11</v>
       </c>
       <c r="C3" t="n">
-        <v>38.49</v>
+        <v>58.99</v>
       </c>
       <c r="D3" t="n">
-        <v>15.1</v>
+        <v>13.2</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>PBMPOLY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.2</v>
+        <v>56.11</v>
       </c>
       <c r="C4" t="n">
-        <v>2.42</v>
+        <v>62.9</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>12.1</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>TARIL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>45.35</v>
+        <v>304</v>
       </c>
       <c r="C5" t="n">
-        <v>49.7</v>
+        <v>333</v>
       </c>
       <c r="D5" t="n">
-        <v>9.59</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>265.35</v>
+        <v>5.35</v>
       </c>
       <c r="C6" t="n">
-        <v>289</v>
+        <v>5.85</v>
       </c>
       <c r="D6" t="n">
-        <v>8.91</v>
+        <v>9.35</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMAL</t>
+          <t>KKJEWELS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>917.9</v>
+        <v>148</v>
       </c>
       <c r="C7" t="n">
-        <v>990</v>
+        <v>159.7</v>
       </c>
       <c r="D7" t="n">
-        <v>7.85</v>
+        <v>7.91</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DELAPLEX</t>
+          <t>ARTNIRMAN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>113.7</v>
+        <v>43.71</v>
       </c>
       <c r="C9" t="n">
-        <v>121.6</v>
+        <v>47</v>
       </c>
       <c r="D9" t="n">
-        <v>6.95</v>
+        <v>7.53</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VIKRAN</t>
+          <t>ITL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55.66</v>
+        <v>361.95</v>
       </c>
       <c r="C10" t="n">
-        <v>59.47</v>
+        <v>387.9</v>
       </c>
       <c r="D10" t="n">
-        <v>6.85</v>
+        <v>7.17</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SGLRES</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.41</v>
+        <v>23.06</v>
       </c>
       <c r="C11" t="n">
-        <v>2.56</v>
+        <v>24.7</v>
       </c>
       <c r="D11" t="n">
-        <v>6.22</v>
+        <v>7.11</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SIDDHICOTS</t>
+          <t>SAPPL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>27.9</v>
+        <v>354.95</v>
       </c>
       <c r="C12" t="n">
-        <v>29.6</v>
+        <v>379.95</v>
       </c>
       <c r="D12" t="n">
-        <v>6.09</v>
+        <v>7.04</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>566.35</v>
+        <v>9.84</v>
       </c>
       <c r="C13" t="n">
-        <v>600</v>
+        <v>10.42</v>
       </c>
       <c r="D13" t="n">
-        <v>5.94</v>
+        <v>5.89</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>AVPINFRA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.17</v>
+        <v>65.05</v>
       </c>
       <c r="C14" t="n">
-        <v>0.18</v>
+        <v>68.8</v>
       </c>
       <c r="D14" t="n">
-        <v>5.88</v>
+        <v>5.76</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>KANCOTEA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.19</v>
+        <v>61.51</v>
       </c>
       <c r="C15" t="n">
-        <v>0.2</v>
+        <v>65</v>
       </c>
       <c r="D15" t="n">
-        <v>5.26</v>
+        <v>5.67</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>232.91</v>
+        <v>0.18</v>
       </c>
       <c r="C16" t="n">
-        <v>245</v>
+        <v>0.19</v>
       </c>
       <c r="D16" t="n">
-        <v>5.19</v>
+        <v>5.56</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KKJEWELS</t>
+          <t>TRF</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>123.35</v>
+        <v>214.83</v>
       </c>
       <c r="C17" t="n">
-        <v>129.65</v>
+        <v>226.1</v>
       </c>
       <c r="D17" t="n">
-        <v>5.11</v>
+        <v>5.25</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>SHIVAMAUTO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>218.11</v>
+        <v>18.05</v>
       </c>
       <c r="C18" t="n">
-        <v>229.25</v>
+        <v>18.96</v>
       </c>
       <c r="D18" t="n">
-        <v>5.11</v>
+        <v>5.04</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>33.18</v>
+        <v>373.25</v>
       </c>
       <c r="C19" t="n">
-        <v>34.85</v>
+        <v>391.9</v>
       </c>
       <c r="D19" t="n">
-        <v>5.03</v>
+        <v>5</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,14 +857,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>GSPLTRANS</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>182.2</v>
+        <v>112.51</v>
       </c>
       <c r="C20" t="n">
-        <v>191.31</v>
+        <v>118.13</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
@@ -879,14 +879,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AVATAR</t>
+          <t>ASSAMENT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>183.05</v>
+        <v>784.65</v>
       </c>
       <c r="C21" t="n">
-        <v>192.2</v>
+        <v>823.85</v>
       </c>
       <c r="D21" t="n">
         <v>5</v>
@@ -901,14 +901,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BMISL</t>
+          <t>KORE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>146.05</v>
+        <v>244.05</v>
       </c>
       <c r="C22" t="n">
-        <v>153.35</v>
+        <v>256.25</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -923,14 +923,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>BMISL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>624.65</v>
+        <v>153.35</v>
       </c>
       <c r="C23" t="n">
-        <v>655.85</v>
+        <v>161</v>
       </c>
       <c r="D23" t="n">
         <v>4.99</v>
@@ -945,14 +945,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>AKANKSHA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>36.1</v>
+        <v>186.3</v>
       </c>
       <c r="C24" t="n">
-        <v>37.9</v>
+        <v>195.6</v>
       </c>
       <c r="D24" t="n">
         <v>4.99</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>55.87</v>
+        <v>14.83</v>
       </c>
       <c r="C25" t="n">
-        <v>58.66</v>
+        <v>15.57</v>
       </c>
       <c r="D25" t="n">
         <v>4.99</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>98.15000000000001</v>
+        <v>37.9</v>
       </c>
       <c r="C26" t="n">
-        <v>103.05</v>
+        <v>39.79</v>
       </c>
       <c r="D26" t="n">
         <v>4.99</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>EEPL</t>
+          <t>UNIVPHOTO</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>146.6</v>
+        <v>470.7</v>
       </c>
       <c r="C27" t="n">
-        <v>153.9</v>
+        <v>494.2</v>
       </c>
       <c r="D27" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,14 +1033,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>HBESD</t>
+          <t>COREIN</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>79.44</v>
+        <v>110.45</v>
       </c>
       <c r="C28" t="n">
-        <v>83.40000000000001</v>
+        <v>115.95</v>
       </c>
       <c r="D28" t="n">
         <v>4.98</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SUPTANERY</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>8.470000000000001</v>
+        <v>36.01</v>
       </c>
       <c r="C29" t="n">
-        <v>8.890000000000001</v>
+        <v>37.8</v>
       </c>
       <c r="D29" t="n">
-        <v>4.96</v>
+        <v>4.97</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>14.13</v>
+        <v>2.42</v>
       </c>
       <c r="C30" t="n">
-        <v>14.83</v>
+        <v>2.54</v>
       </c>
       <c r="D30" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>DIGJAMLMTD</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>45.6</v>
+        <v>52.41</v>
       </c>
       <c r="C31" t="n">
-        <v>47.85</v>
+        <v>55</v>
       </c>
       <c r="D31" t="n">
-        <v>4.93</v>
+        <v>4.94</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAHANA</t>
+          <t>LEENEE</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>858.85</v>
+        <v>7.1</v>
       </c>
       <c r="C32" t="n">
-        <v>900</v>
+        <v>7.45</v>
       </c>
       <c r="D32" t="n">
-        <v>4.79</v>
+        <v>4.93</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>NEWJAISA</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3.55</v>
+        <v>15.25</v>
       </c>
       <c r="C33" t="n">
-        <v>3.72</v>
+        <v>16</v>
       </c>
       <c r="D33" t="n">
-        <v>4.79</v>
+        <v>4.92</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>EBIX</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>15.73</v>
+        <v>47.85</v>
       </c>
       <c r="C34" t="n">
-        <v>16.48</v>
+        <v>50.2</v>
       </c>
       <c r="D34" t="n">
-        <v>4.77</v>
+        <v>4.91</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>KJMCFIN</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>361.75</v>
+        <v>57.22</v>
       </c>
       <c r="C35" t="n">
-        <v>379</v>
+        <v>60</v>
       </c>
       <c r="D35" t="n">
-        <v>4.77</v>
+        <v>4.86</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PATILAUTOM</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>361.8</v>
+        <v>3.72</v>
       </c>
       <c r="C36" t="n">
-        <v>379</v>
+        <v>3.9</v>
       </c>
       <c r="D36" t="n">
-        <v>4.75</v>
+        <v>4.84</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CEDAAR</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>15.3</v>
+        <v>5.81</v>
       </c>
       <c r="C37" t="n">
-        <v>16</v>
+        <v>6.09</v>
       </c>
       <c r="D37" t="n">
-        <v>4.58</v>
+        <v>4.82</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>150.04</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="C38" t="n">
-        <v>156.9</v>
+        <v>67.8</v>
       </c>
       <c r="D38" t="n">
-        <v>4.57</v>
+        <v>4.69</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.44</v>
+        <v>4.91</v>
       </c>
       <c r="C39" t="n">
-        <v>0.46</v>
+        <v>5.14</v>
       </c>
       <c r="D39" t="n">
-        <v>4.55</v>
+        <v>4.68</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>QUINTEGRA</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1.77</v>
+        <v>1.71</v>
       </c>
       <c r="C40" t="n">
-        <v>1.85</v>
+        <v>1.79</v>
       </c>
       <c r="D40" t="n">
-        <v>4.52</v>
+        <v>4.68</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>494.85</v>
+        <v>13.38</v>
       </c>
       <c r="C41" t="n">
-        <v>516.8</v>
+        <v>13.99</v>
       </c>
       <c r="D41" t="n">
-        <v>4.44</v>
+        <v>4.56</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ZSARACOM</t>
+          <t>GULFPETRO</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>9670</v>
+        <v>62.84</v>
       </c>
       <c r="C42" t="n">
-        <v>10093</v>
+        <v>65.7</v>
       </c>
       <c r="D42" t="n">
-        <v>4.37</v>
+        <v>4.55</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>COREIN</t>
+          <t>ESCONET</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>105.2</v>
+        <v>263.7</v>
       </c>
       <c r="C43" t="n">
-        <v>109.8</v>
+        <v>275.45</v>
       </c>
       <c r="D43" t="n">
-        <v>4.37</v>
+        <v>4.46</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>NAHARCAP</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.23</v>
+        <v>234.49</v>
       </c>
       <c r="C44" t="n">
-        <v>0.24</v>
+        <v>244.8</v>
       </c>
       <c r="D44" t="n">
-        <v>4.35</v>
+        <v>4.4</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AMEYA</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>178.5</v>
+        <v>7.98</v>
       </c>
       <c r="C45" t="n">
-        <v>186</v>
+        <v>8.33</v>
       </c>
       <c r="D45" t="n">
-        <v>4.2</v>
+        <v>4.39</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.49</v>
+        <v>57.35</v>
       </c>
       <c r="C46" t="n">
-        <v>0.51</v>
+        <v>59.85</v>
       </c>
       <c r="D46" t="n">
-        <v>4.08</v>
+        <v>4.36</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VGCL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>50</v>
+        <v>0.23</v>
       </c>
       <c r="C47" t="n">
-        <v>52</v>
+        <v>0.24</v>
       </c>
       <c r="D47" t="n">
-        <v>4</v>
+        <v>4.35</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>11.03</v>
+        <v>6.04</v>
       </c>
       <c r="C48" t="n">
-        <v>11.45</v>
+        <v>6.3</v>
       </c>
       <c r="D48" t="n">
-        <v>3.81</v>
+        <v>4.3</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KOTYARK</t>
+          <t>NARMADA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>34.44</v>
+        <v>10.75</v>
       </c>
       <c r="C49" t="n">
-        <v>35.75</v>
+        <v>11.2</v>
       </c>
       <c r="D49" t="n">
-        <v>3.8</v>
+        <v>4.19</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>HAZOOR</t>
+          <t>KALYANIFRG</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>16.66</v>
+        <v>835.15</v>
       </c>
       <c r="C50" t="n">
-        <v>17.28</v>
+        <v>868.85</v>
       </c>
       <c r="D50" t="n">
-        <v>3.72</v>
+        <v>4.04</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LYKALABS</t>
+          <t>CTE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>72.23</v>
+        <v>37.5</v>
       </c>
       <c r="C51" t="n">
-        <v>74.90000000000001</v>
+        <v>39</v>
       </c>
       <c r="D51" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AKSHARCHEM</t>
+          <t>SIEL</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>390.7</v>
+        <v>29.81</v>
       </c>
       <c r="C52" t="n">
-        <v>405</v>
+        <v>31</v>
       </c>
       <c r="D52" t="n">
-        <v>3.66</v>
+        <v>3.99</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BALPHARMA</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>97.70999999999999</v>
+        <v>3.26</v>
       </c>
       <c r="C53" t="n">
-        <v>101.2</v>
+        <v>3.39</v>
       </c>
       <c r="D53" t="n">
-        <v>3.57</v>
+        <v>3.99</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>5.99</v>
+        <v>27.28</v>
       </c>
       <c r="C54" t="n">
-        <v>6.2</v>
+        <v>28.35</v>
       </c>
       <c r="D54" t="n">
-        <v>3.51</v>
+        <v>3.92</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ROCKINGDCE</t>
+          <t>SAYAJIHOTL</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>222.2</v>
+        <v>302.95</v>
       </c>
       <c r="C55" t="n">
-        <v>230</v>
+        <v>314.8</v>
       </c>
       <c r="D55" t="n">
-        <v>3.51</v>
+        <v>3.91</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PAVNAIND</t>
+          <t>HEROMOTORS</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>14.96</v>
+        <v>155.19</v>
       </c>
       <c r="C56" t="n">
-        <v>15.48</v>
+        <v>161</v>
       </c>
       <c r="D56" t="n">
-        <v>3.48</v>
+        <v>3.74</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ONIXSOLAR</t>
+          <t>INDIANCARD</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>376.05</v>
+        <v>189.97</v>
       </c>
       <c r="C57" t="n">
-        <v>389</v>
+        <v>197</v>
       </c>
       <c r="D57" t="n">
-        <v>3.44</v>
+        <v>3.7</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>KOLTEPATIL</t>
+          <t>ANSALBU</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>425.7</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="C58" t="n">
-        <v>440</v>
+        <v>86.98999999999999</v>
       </c>
       <c r="D58" t="n">
-        <v>3.36</v>
+        <v>3.65</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AHCL</t>
+          <t>AGASTYAEN</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>29.51</v>
+        <v>69.33</v>
       </c>
       <c r="C59" t="n">
-        <v>30.5</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="D59" t="n">
-        <v>3.35</v>
+        <v>3.63</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>735.45</v>
+        <v>33.53</v>
       </c>
       <c r="C60" t="n">
-        <v>760</v>
+        <v>34.74</v>
       </c>
       <c r="D60" t="n">
-        <v>3.34</v>
+        <v>3.61</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SAHYADRI</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>333.6</v>
+        <v>28.4</v>
       </c>
       <c r="C61" t="n">
-        <v>344.7</v>
+        <v>29.39</v>
       </c>
       <c r="D61" t="n">
-        <v>3.33</v>
+        <v>3.49</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>PHOENXINTL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>197.4</v>
+        <v>40.12</v>
       </c>
       <c r="C62" t="n">
-        <v>203.98</v>
+        <v>41.5</v>
       </c>
       <c r="D62" t="n">
-        <v>3.33</v>
+        <v>3.44</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>KOTARISUG</t>
+          <t>21STCENMGM</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>25.84</v>
+        <v>42.06</v>
       </c>
       <c r="C63" t="n">
-        <v>26.7</v>
+        <v>43.5</v>
       </c>
       <c r="D63" t="n">
-        <v>3.33</v>
+        <v>3.42</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>NKIND</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>12.76</v>
+        <v>60.99</v>
       </c>
       <c r="C64" t="n">
-        <v>13.18</v>
+        <v>63</v>
       </c>
       <c r="D64" t="n">
-        <v>3.29</v>
+        <v>3.3</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>GSMFOILS</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>18.79</v>
+        <v>63.65</v>
       </c>
       <c r="C65" t="n">
-        <v>19.4</v>
+        <v>65.75</v>
       </c>
       <c r="D65" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,14 +1869,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AEQUS</t>
+          <t>GENCON</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>265.9</v>
+        <v>35.75</v>
       </c>
       <c r="C66" t="n">
-        <v>274.45</v>
+        <v>36.9</v>
       </c>
       <c r="D66" t="n">
         <v>3.22</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>544.7</v>
+        <v>20.98</v>
       </c>
       <c r="C67" t="n">
-        <v>562</v>
+        <v>21.65</v>
       </c>
       <c r="D67" t="n">
-        <v>3.18</v>
+        <v>3.19</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>118.59</v>
+        <v>3.53</v>
       </c>
       <c r="C68" t="n">
-        <v>122.35</v>
+        <v>3.64</v>
       </c>
       <c r="D68" t="n">
-        <v>3.17</v>
+        <v>3.12</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>EEPL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>57.94</v>
+        <v>153.9</v>
       </c>
       <c r="C69" t="n">
-        <v>59.77</v>
+        <v>158.65</v>
       </c>
       <c r="D69" t="n">
-        <v>3.16</v>
+        <v>3.09</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MAKERSL</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>187</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="C70" t="n">
-        <v>192.9</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="D70" t="n">
-        <v>3.16</v>
+        <v>3.07</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>18.23</v>
+        <v>272.69</v>
       </c>
       <c r="C71" t="n">
-        <v>18.8</v>
+        <v>281</v>
       </c>
       <c r="D71" t="n">
-        <v>3.13</v>
+        <v>3.05</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>387.1</v>
+        <v>1.32</v>
       </c>
       <c r="C72" t="n">
-        <v>398.95</v>
+        <v>1.36</v>
       </c>
       <c r="D72" t="n">
-        <v>3.06</v>
+        <v>3.03</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>GENCON</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>36.22</v>
+        <v>0.67</v>
       </c>
       <c r="C73" t="n">
-        <v>37.3</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D73" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>SSRETAIL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>76.14</v>
+        <v>691.95</v>
       </c>
       <c r="C74" t="n">
-        <v>78.39</v>
+        <v>712.6</v>
       </c>
       <c r="D74" t="n">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>DENORA</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>25.88</v>
+        <v>700.1</v>
       </c>
       <c r="C75" t="n">
-        <v>26.64</v>
+        <v>720.45</v>
       </c>
       <c r="D75" t="n">
-        <v>2.94</v>
+        <v>2.91</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,14 +2089,14 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AGOL</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4.84</v>
+        <v>72.89</v>
       </c>
       <c r="C76" t="n">
-        <v>4.98</v>
+        <v>75</v>
       </c>
       <c r="D76" t="n">
         <v>2.89</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BANDHANBNK</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>157.5</v>
+        <v>64.67</v>
       </c>
       <c r="C77" t="n">
-        <v>162</v>
+        <v>66.48999999999999</v>
       </c>
       <c r="D77" t="n">
-        <v>2.86</v>
+        <v>2.81</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>ADISOFT</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>57.71</v>
+        <v>288</v>
       </c>
       <c r="C78" t="n">
-        <v>59.35</v>
+        <v>296</v>
       </c>
       <c r="D78" t="n">
-        <v>2.84</v>
+        <v>2.78</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>QUALIANCE</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>195.3</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="C79" t="n">
-        <v>200.85</v>
+        <v>66.88</v>
       </c>
       <c r="D79" t="n">
-        <v>2.84</v>
+        <v>2.78</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1.41</v>
+        <v>89.47</v>
       </c>
       <c r="C80" t="n">
-        <v>1.45</v>
+        <v>91.95</v>
       </c>
       <c r="D80" t="n">
-        <v>2.84</v>
+        <v>2.77</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>ATALREAL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>2.14</v>
+        <v>11.28</v>
       </c>
       <c r="C81" t="n">
-        <v>2.2</v>
+        <v>11.59</v>
       </c>
       <c r="D81" t="n">
-        <v>2.8</v>
+        <v>2.75</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>DBSTOCKBRO</t>
+          <t>HILINFRA</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>31.13</v>
+        <v>52.06</v>
       </c>
       <c r="C82" t="n">
-        <v>32</v>
+        <v>53.49</v>
       </c>
       <c r="D82" t="n">
-        <v>2.79</v>
+        <v>2.75</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>RULKA</t>
+          <t>MADRASFERT</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>100.5</v>
+        <v>57.22</v>
       </c>
       <c r="C83" t="n">
-        <v>103.3</v>
+        <v>58.79</v>
       </c>
       <c r="D83" t="n">
-        <v>2.79</v>
+        <v>2.74</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>MADHURKNIT</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.36</v>
+        <v>57.45</v>
       </c>
       <c r="C84" t="n">
-        <v>0.37</v>
+        <v>59</v>
       </c>
       <c r="D84" t="n">
-        <v>2.78</v>
+        <v>2.7</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>6.47</v>
+        <v>36.47</v>
       </c>
       <c r="C85" t="n">
-        <v>6.65</v>
+        <v>37.45</v>
       </c>
       <c r="D85" t="n">
-        <v>2.78</v>
+        <v>2.69</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IRCON</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>104.73</v>
+        <v>3188.9</v>
       </c>
       <c r="C86" t="n">
-        <v>107.6</v>
+        <v>3274</v>
       </c>
       <c r="D86" t="n">
-        <v>2.74</v>
+        <v>2.67</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>AARTECH</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>46.73</v>
+        <v>492.05</v>
       </c>
       <c r="C87" t="n">
-        <v>48</v>
+        <v>505</v>
       </c>
       <c r="D87" t="n">
-        <v>2.72</v>
+        <v>2.63</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>JSIPL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>208.13</v>
+        <v>167.42</v>
       </c>
       <c r="C88" t="n">
-        <v>213.8</v>
+        <v>171.8</v>
       </c>
       <c r="D88" t="n">
-        <v>2.72</v>
+        <v>2.62</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>ECORECO</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>19.18</v>
+        <v>397.4</v>
       </c>
       <c r="C89" t="n">
-        <v>19.7</v>
+        <v>407.7</v>
       </c>
       <c r="D89" t="n">
-        <v>2.71</v>
+        <v>2.59</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1007.8</v>
+        <v>102.63</v>
       </c>
       <c r="C90" t="n">
-        <v>1035</v>
+        <v>105.29</v>
       </c>
       <c r="D90" t="n">
-        <v>2.7</v>
+        <v>2.59</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>RISHABH</t>
+          <t>PILANIINVS</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>679.55</v>
+        <v>3949.6</v>
       </c>
       <c r="C91" t="n">
-        <v>697.7</v>
+        <v>4049</v>
       </c>
       <c r="D91" t="n">
-        <v>2.67</v>
+        <v>2.52</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SKYGOLD</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>968.25</v>
+        <v>54.29</v>
       </c>
       <c r="C92" t="n">
-        <v>994</v>
+        <v>55.65</v>
       </c>
       <c r="D92" t="n">
-        <v>2.66</v>
+        <v>2.51</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>GRPLTD</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1700.8</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="C93" t="n">
-        <v>1745</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="D93" t="n">
-        <v>2.6</v>
+        <v>2.46</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>72.52</v>
+        <v>7.33</v>
       </c>
       <c r="C94" t="n">
-        <v>74.40000000000001</v>
+        <v>7.51</v>
       </c>
       <c r="D94" t="n">
-        <v>2.59</v>
+        <v>2.46</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>VTMLTD</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>3.86</v>
+        <v>41</v>
       </c>
       <c r="C95" t="n">
-        <v>3.96</v>
+        <v>42</v>
       </c>
       <c r="D95" t="n">
-        <v>2.59</v>
+        <v>2.44</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>INNOMET</t>
+          <t>HMVL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>251.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="C96" t="n">
-        <v>258</v>
+        <v>79.79000000000001</v>
       </c>
       <c r="D96" t="n">
-        <v>2.58</v>
+        <v>2.43</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>RAMBHAJO</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>375.3</v>
+        <v>34.12</v>
       </c>
       <c r="C97" t="n">
-        <v>385</v>
+        <v>34.95</v>
       </c>
       <c r="D97" t="n">
-        <v>2.58</v>
+        <v>2.43</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>KONSTELEC</t>
+          <t>EMKAY</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>49.15</v>
+        <v>269.45</v>
       </c>
       <c r="C98" t="n">
-        <v>50.4</v>
+        <v>275.9</v>
       </c>
       <c r="D98" t="n">
-        <v>2.54</v>
+        <v>2.39</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>BALKRISHNA</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>24.83</v>
+        <v>15.63</v>
       </c>
       <c r="C99" t="n">
-        <v>25.45</v>
+        <v>16</v>
       </c>
       <c r="D99" t="n">
-        <v>2.5</v>
+        <v>2.37</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MAWANASUG</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>168.79</v>
+        <v>76.02</v>
       </c>
       <c r="C100" t="n">
-        <v>173</v>
+        <v>77.8</v>
       </c>
       <c r="D100" t="n">
-        <v>2.49</v>
+        <v>2.34</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AKSHOPTFBR</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>7.27</v>
+        <v>4.29</v>
       </c>
       <c r="C101" t="n">
-        <v>7.45</v>
+        <v>4.39</v>
       </c>
       <c r="D101" t="n">
-        <v>2.48</v>
+        <v>2.33</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>TOLINS</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>85.58</v>
+        <v>11.28</v>
       </c>
       <c r="C102" t="n">
-        <v>87.7</v>
+        <v>11.54</v>
       </c>
       <c r="D102" t="n">
-        <v>2.48</v>
+        <v>2.3</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>175.66</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="C103" t="n">
-        <v>180</v>
+        <v>9.93</v>
       </c>
       <c r="D103" t="n">
-        <v>2.47</v>
+        <v>2.27</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>HLVLTD</t>
+          <t>AFIL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>6.08</v>
+        <v>8.01</v>
       </c>
       <c r="C104" t="n">
-        <v>6.23</v>
+        <v>8.19</v>
       </c>
       <c r="D104" t="n">
-        <v>2.47</v>
+        <v>2.25</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>IDBI</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>26.87</v>
+        <v>82.94</v>
       </c>
       <c r="C105" t="n">
-        <v>27.5</v>
+        <v>84.8</v>
       </c>
       <c r="D105" t="n">
-        <v>2.34</v>
+        <v>2.24</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>INNOMET</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>18.07</v>
+        <v>264.05</v>
       </c>
       <c r="C106" t="n">
-        <v>18.49</v>
+        <v>269.9</v>
       </c>
       <c r="D106" t="n">
-        <v>2.32</v>
+        <v>2.22</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>VIRTUALG</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>50.33</v>
+        <v>0.45</v>
       </c>
       <c r="C107" t="n">
-        <v>51.5</v>
+        <v>0.46</v>
       </c>
       <c r="D107" t="n">
-        <v>2.32</v>
+        <v>2.22</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>HLEGLAS</t>
+          <t>GANGESSECU</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>406.6</v>
+        <v>112.5</v>
       </c>
       <c r="C108" t="n">
-        <v>416</v>
+        <v>114.99</v>
       </c>
       <c r="D108" t="n">
-        <v>2.31</v>
+        <v>2.21</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>ONEGLOBAL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.87</v>
+        <v>549.85</v>
       </c>
       <c r="C109" t="n">
-        <v>0.89</v>
+        <v>561.9</v>
       </c>
       <c r="D109" t="n">
-        <v>2.3</v>
+        <v>2.19</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>RAJSREESUG</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>30.99</v>
+        <v>5.47</v>
       </c>
       <c r="C110" t="n">
-        <v>31.7</v>
+        <v>5.59</v>
       </c>
       <c r="D110" t="n">
-        <v>2.29</v>
+        <v>2.19</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>41.62</v>
+        <v>11.44</v>
       </c>
       <c r="C111" t="n">
-        <v>42.57</v>
+        <v>11.69</v>
       </c>
       <c r="D111" t="n">
-        <v>2.28</v>
+        <v>2.19</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>HTEL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>380.35</v>
+        <v>88.95999999999999</v>
       </c>
       <c r="C112" t="n">
-        <v>389</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="D112" t="n">
-        <v>2.27</v>
+        <v>2.18</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>1.33</v>
+        <v>0.46</v>
       </c>
       <c r="C113" t="n">
-        <v>1.36</v>
+        <v>0.47</v>
       </c>
       <c r="D113" t="n">
-        <v>2.26</v>
+        <v>2.17</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DEVX</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>41.66</v>
+        <v>1.84</v>
       </c>
       <c r="C114" t="n">
-        <v>42.6</v>
+        <v>1.88</v>
       </c>
       <c r="D114" t="n">
-        <v>2.26</v>
+        <v>2.17</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>KANPRPLA</t>
+          <t>PRISMX</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>241.35</v>
+        <v>0.46</v>
       </c>
       <c r="C115" t="n">
-        <v>246.75</v>
+        <v>0.47</v>
       </c>
       <c r="D115" t="n">
-        <v>2.24</v>
+        <v>2.17</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>ORIENTCER</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>93.90000000000001</v>
+        <v>43.06</v>
       </c>
       <c r="C116" t="n">
-        <v>96</v>
+        <v>43.99</v>
       </c>
       <c r="D116" t="n">
-        <v>2.24</v>
+        <v>2.16</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>4.98</v>
+        <v>49.43</v>
       </c>
       <c r="C117" t="n">
-        <v>5.09</v>
+        <v>50.5</v>
       </c>
       <c r="D117" t="n">
-        <v>2.21</v>
+        <v>2.16</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>ANUHPHR</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>9.970000000000001</v>
+        <v>81.27</v>
       </c>
       <c r="C118" t="n">
-        <v>10.19</v>
+        <v>83</v>
       </c>
       <c r="D118" t="n">
-        <v>2.21</v>
+        <v>2.13</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>28.87</v>
+        <v>15.46</v>
       </c>
       <c r="C119" t="n">
-        <v>29.5</v>
+        <v>15.79</v>
       </c>
       <c r="D119" t="n">
-        <v>2.18</v>
+        <v>2.13</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>SANATHAN</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>20.16</v>
+        <v>533.4</v>
       </c>
       <c r="C120" t="n">
-        <v>20.6</v>
+        <v>544.7</v>
       </c>
       <c r="D120" t="n">
-        <v>2.18</v>
+        <v>2.12</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>CRESTO</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.46</v>
+        <v>20.81</v>
       </c>
       <c r="C121" t="n">
-        <v>0.47</v>
+        <v>21.25</v>
       </c>
       <c r="D121" t="n">
-        <v>2.17</v>
+        <v>2.11</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>AHLUCONT</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>53.83</v>
+        <v>565.2</v>
       </c>
       <c r="C122" t="n">
-        <v>55</v>
+        <v>577.1</v>
       </c>
       <c r="D122" t="n">
-        <v>2.17</v>
+        <v>2.11</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>18</v>
+        <v>7.15</v>
       </c>
       <c r="C123" t="n">
-        <v>18.39</v>
+        <v>7.3</v>
       </c>
       <c r="D123" t="n">
-        <v>2.17</v>
+        <v>2.1</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SPUNWEB</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>129</v>
+        <v>42.31</v>
       </c>
       <c r="C124" t="n">
-        <v>131.8</v>
+        <v>43.19</v>
       </c>
       <c r="D124" t="n">
-        <v>2.17</v>
+        <v>2.08</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>RAMBHAJO</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>3.26</v>
+        <v>372.05</v>
       </c>
       <c r="C125" t="n">
-        <v>3.33</v>
+        <v>379.8</v>
       </c>
       <c r="D125" t="n">
-        <v>2.15</v>
+        <v>2.08</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>49.92</v>
+        <v>38</v>
       </c>
       <c r="C126" t="n">
-        <v>50.98</v>
+        <v>38.79</v>
       </c>
       <c r="D126" t="n">
-        <v>2.12</v>
+        <v>2.08</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ELIN</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>75.40000000000001</v>
+        <v>7.24</v>
       </c>
       <c r="C127" t="n">
-        <v>76.98999999999999</v>
+        <v>7.39</v>
       </c>
       <c r="D127" t="n">
-        <v>2.11</v>
+        <v>2.07</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TEXMOPIPES</t>
+          <t>SUMEDHA</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>51.52</v>
+        <v>43</v>
       </c>
       <c r="C128" t="n">
-        <v>52.6</v>
+        <v>43.89</v>
       </c>
       <c r="D128" t="n">
-        <v>2.1</v>
+        <v>2.07</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>KANCHI</t>
+          <t>RIIT</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>359.4</v>
+        <v>121.5</v>
       </c>
       <c r="C129" t="n">
-        <v>366.95</v>
+        <v>124</v>
       </c>
       <c r="D129" t="n">
-        <v>2.1</v>
+        <v>2.06</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>KARMAENG</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>3.33</v>
+        <v>34.68</v>
       </c>
       <c r="C130" t="n">
-        <v>3.4</v>
+        <v>35.39</v>
       </c>
       <c r="D130" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BANSWRAS</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>100.66</v>
+        <v>10.26</v>
       </c>
       <c r="C131" t="n">
-        <v>102.75</v>
+        <v>10.47</v>
       </c>
       <c r="D131" t="n">
-        <v>2.08</v>
+        <v>2.05</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>CGCL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>6.25</v>
+        <v>248.9</v>
       </c>
       <c r="C132" t="n">
-        <v>6.38</v>
+        <v>254</v>
       </c>
       <c r="D132" t="n">
-        <v>2.08</v>
+        <v>2.05</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>NECLIFE</t>
+          <t>LANCORHOL</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>10.14</v>
+        <v>29.39</v>
       </c>
       <c r="C133" t="n">
-        <v>10.35</v>
+        <v>29.99</v>
       </c>
       <c r="D133" t="n">
-        <v>2.07</v>
+        <v>2.04</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>31.05</v>
+        <v>10.78</v>
       </c>
       <c r="C134" t="n">
-        <v>31.69</v>
+        <v>11</v>
       </c>
       <c r="D134" t="n">
-        <v>2.06</v>
+        <v>2.04</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>670.75</v>
+        <v>48.7</v>
       </c>
       <c r="C135" t="n">
-        <v>684.6</v>
+        <v>49.69</v>
       </c>
       <c r="D135" t="n">
-        <v>2.06</v>
+        <v>2.03</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>SAGARDEEP</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>6.35</v>
+        <v>25.81</v>
       </c>
       <c r="C136" t="n">
-        <v>6.48</v>
+        <v>26.33</v>
       </c>
       <c r="D136" t="n">
-        <v>2.05</v>
+        <v>2.01</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>41.53</v>
+        <v>1.99</v>
       </c>
       <c r="C137" t="n">
-        <v>42.38</v>
+        <v>2.03</v>
       </c>
       <c r="D137" t="n">
-        <v>2.05</v>
+        <v>2.01</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PRISMX</t>
+          <t>VRAJ</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.49</v>
+        <v>119.39</v>
       </c>
       <c r="C138" t="n">
-        <v>0.5</v>
+        <v>121.79</v>
       </c>
       <c r="D138" t="n">
-        <v>2.04</v>
+        <v>2.01</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>DIGIDRIVE</t>
+          <t>TFL</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>18.7</v>
+        <v>11.95</v>
       </c>
       <c r="C139" t="n">
-        <v>19.08</v>
+        <v>12.19</v>
       </c>
       <c r="D139" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CGVAK</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>133.78</v>
+        <v>27.82</v>
       </c>
       <c r="C140" t="n">
-        <v>136.49</v>
+        <v>28.38</v>
       </c>
       <c r="D140" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>NICCOPAR</t>
+          <t>BEEKAY</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>70.06999999999999</v>
+        <v>435.85</v>
       </c>
       <c r="C141" t="n">
-        <v>71.48999999999999</v>
+        <v>444.55</v>
       </c>
       <c r="D141" t="n">
-        <v>2.03</v>
+        <v>2</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>GENUSPAPER</t>
+          <t>PARIN</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>10.38</v>
+        <v>691.15</v>
       </c>
       <c r="C142" t="n">
-        <v>10.59</v>
+        <v>704.95</v>
       </c>
       <c r="D142" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ADVIKCA</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>0.99</v>
+        <v>52.44</v>
       </c>
       <c r="C143" t="n">
-        <v>1.01</v>
+        <v>53.49</v>
       </c>
       <c r="D143" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>INDIANCARD</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>183.99</v>
+        <v>168.44</v>
       </c>
       <c r="C144" t="n">
-        <v>187.69</v>
+        <v>171.79</v>
       </c>
       <c r="D144" t="n">
-        <v>2.01</v>
+        <v>1.99</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>RAJMET</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>35.38</v>
+        <v>3.01</v>
       </c>
       <c r="C145" t="n">
-        <v>36.09</v>
+        <v>3.07</v>
       </c>
       <c r="D145" t="n">
-        <v>2.01</v>
+        <v>1.99</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>BLUECLOUDS</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>48.04</v>
+        <v>19.59</v>
       </c>
       <c r="C146" t="n">
-        <v>49</v>
+        <v>19.98</v>
       </c>
       <c r="D146" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>209.01</v>
+        <v>22.07</v>
       </c>
       <c r="C147" t="n">
-        <v>213.19</v>
+        <v>22.51</v>
       </c>
       <c r="D147" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>VIKASECO</t>
+          <t>CGVAK</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>1</v>
+        <v>134.71</v>
       </c>
       <c r="C148" t="n">
-        <v>1.02</v>
+        <v>137.39</v>
       </c>
       <c r="D148" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>MUTHOOTCAP</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>21.46</v>
+        <v>211.8</v>
       </c>
       <c r="C149" t="n">
-        <v>21.89</v>
+        <v>215.99</v>
       </c>
       <c r="D149" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>83.53</v>
+        <v>15.17</v>
       </c>
       <c r="C150" t="n">
-        <v>85.2</v>
+        <v>15.47</v>
       </c>
       <c r="D150" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>CRIZAC</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.5</v>
+        <v>157.77</v>
       </c>
       <c r="C151" t="n">
-        <v>0.51</v>
+        <v>160.9</v>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>MGEL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>56.52</v>
+        <v>16.13</v>
       </c>
       <c r="C152" t="n">
-        <v>57.65</v>
+        <v>16.45</v>
       </c>
       <c r="D152" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>SILINV</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>4</v>
+        <v>467.85</v>
       </c>
       <c r="C153" t="n">
-        <v>4.08</v>
+        <v>477</v>
       </c>
       <c r="D153" t="n">
-        <v>2</v>
+        <v>1.96</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>SPLIL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>20.58</v>
+        <v>28.04</v>
       </c>
       <c r="C154" t="n">
-        <v>20.99</v>
+        <v>28.59</v>
       </c>
       <c r="D154" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>BHAGCHEM</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>21.64</v>
+        <v>221.66</v>
       </c>
       <c r="C155" t="n">
-        <v>22.07</v>
+        <v>226</v>
       </c>
       <c r="D155" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>GTPL</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>56.77</v>
+        <v>6.11</v>
       </c>
       <c r="C156" t="n">
-        <v>57.9</v>
+        <v>6.23</v>
       </c>
       <c r="D156" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ZFSTEERING</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>680.9</v>
+        <v>58.25</v>
       </c>
       <c r="C157" t="n">
-        <v>694.45</v>
+        <v>59.39</v>
       </c>
       <c r="D157" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>BHARATRAS</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>970.6</v>
+        <v>32.26</v>
       </c>
       <c r="C158" t="n">
-        <v>989.8</v>
+        <v>32.89</v>
       </c>
       <c r="D158" t="n">
-        <v>1.98</v>
+        <v>1.95</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SECMARK</t>
+          <t>MERCURYEV</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>151.19</v>
+        <v>36.53</v>
       </c>
       <c r="C159" t="n">
-        <v>154.19</v>
+        <v>37.24</v>
       </c>
       <c r="D159" t="n">
-        <v>1.98</v>
+        <v>1.94</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>TEAMGTY</t>
+          <t>WEIZMANIND</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>244.03</v>
+        <v>71.41</v>
       </c>
       <c r="C160" t="n">
-        <v>248.85</v>
+        <v>72.79000000000001</v>
       </c>
       <c r="D160" t="n">
-        <v>1.98</v>
+        <v>1.93</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>KHAITANLTD</t>
+          <t>SHRADHA</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>148.08</v>
+        <v>30.01</v>
       </c>
       <c r="C161" t="n">
-        <v>150.99</v>
+        <v>30.59</v>
       </c>
       <c r="D161" t="n">
-        <v>1.97</v>
+        <v>1.93</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AATMAJ</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>22.95</v>
+        <v>15</v>
       </c>
       <c r="C162" t="n">
-        <v>23.4</v>
+        <v>15.29</v>
       </c>
       <c r="D162" t="n">
-        <v>1.96</v>
+        <v>1.93</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>56.2</v>
+        <v>439.45</v>
       </c>
       <c r="C163" t="n">
-        <v>57.29</v>
+        <v>447.9</v>
       </c>
       <c r="D163" t="n">
-        <v>1.94</v>
+        <v>1.92</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>UMIYA-MRO</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>94.61</v>
+        <v>1137.3</v>
       </c>
       <c r="C164" t="n">
-        <v>96.45</v>
+        <v>1159</v>
       </c>
       <c r="D164" t="n">
-        <v>1.94</v>
+        <v>1.91</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>HIMALAYAN</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>107.99</v>
+        <v>87.05</v>
       </c>
       <c r="C165" t="n">
-        <v>110.09</v>
+        <v>88.7</v>
       </c>
       <c r="D165" t="n">
-        <v>1.94</v>
+        <v>1.9</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>GKWLIMITED</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>220.61</v>
+        <v>1554.5</v>
       </c>
       <c r="C166" t="n">
-        <v>224.9</v>
+        <v>1584</v>
       </c>
       <c r="D166" t="n">
-        <v>1.94</v>
+        <v>1.9</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>KOTHARIPRO</t>
+          <t>SIGNPOST</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>61.7</v>
+        <v>250.75</v>
       </c>
       <c r="C167" t="n">
-        <v>62.89</v>
+        <v>255.5</v>
       </c>
       <c r="D167" t="n">
-        <v>1.93</v>
+        <v>1.89</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>JISLDVREQS</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>18.63</v>
+        <v>36.49</v>
       </c>
       <c r="C168" t="n">
-        <v>18.99</v>
+        <v>37.18</v>
       </c>
       <c r="D168" t="n">
-        <v>1.93</v>
+        <v>1.89</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>AERONEU</t>
+          <t>REPRO</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>70.53</v>
+        <v>312.05</v>
       </c>
       <c r="C169" t="n">
-        <v>71.89</v>
+        <v>317.95</v>
       </c>
       <c r="D169" t="n">
-        <v>1.93</v>
+        <v>1.89</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ANNU</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>46.6</v>
+        <v>15.4</v>
       </c>
       <c r="C170" t="n">
-        <v>47.5</v>
+        <v>15.69</v>
       </c>
       <c r="D170" t="n">
-        <v>1.93</v>
+        <v>1.88</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>RHETAN</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>16.67</v>
+        <v>15.01</v>
       </c>
       <c r="C171" t="n">
-        <v>16.99</v>
+        <v>15.29</v>
       </c>
       <c r="D171" t="n">
-        <v>1.92</v>
+        <v>1.87</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>OSWALGREEN</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>18.73</v>
+        <v>23.06</v>
       </c>
       <c r="C172" t="n">
-        <v>19.09</v>
+        <v>23.49</v>
       </c>
       <c r="D172" t="n">
-        <v>1.92</v>
+        <v>1.86</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>HMT</t>
+          <t>CEMPRO</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>54.8</v>
+        <v>1138.8</v>
       </c>
       <c r="C173" t="n">
-        <v>55.85</v>
+        <v>1160</v>
       </c>
       <c r="D173" t="n">
-        <v>1.92</v>
+        <v>1.86</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>BLACKROSE</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>4.19</v>
+        <v>103.53</v>
       </c>
       <c r="C174" t="n">
-        <v>4.27</v>
+        <v>105.45</v>
       </c>
       <c r="D174" t="n">
-        <v>1.91</v>
+        <v>1.85</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>5.77</v>
+        <v>4.88</v>
       </c>
       <c r="C175" t="n">
-        <v>5.88</v>
+        <v>4.97</v>
       </c>
       <c r="D175" t="n">
-        <v>1.91</v>
+        <v>1.84</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>MKEXIM</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>3.67</v>
+        <v>55.97</v>
       </c>
       <c r="C176" t="n">
-        <v>3.74</v>
+        <v>57</v>
       </c>
       <c r="D176" t="n">
-        <v>1.91</v>
+        <v>1.84</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>PAKKA</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>54.66</v>
+        <v>71.17</v>
       </c>
       <c r="C177" t="n">
-        <v>55.7</v>
+        <v>72.47</v>
       </c>
       <c r="D177" t="n">
-        <v>1.9</v>
+        <v>1.83</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>DIGISPICE</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>15.88</v>
+        <v>20.23</v>
       </c>
       <c r="C178" t="n">
-        <v>16.18</v>
+        <v>20.6</v>
       </c>
       <c r="D178" t="n">
-        <v>1.89</v>
+        <v>1.83</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>UDAYJEW</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>140.35</v>
+        <v>229.79</v>
       </c>
       <c r="C179" t="n">
-        <v>143</v>
+        <v>233.97</v>
       </c>
       <c r="D179" t="n">
-        <v>1.89</v>
+        <v>1.82</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>53.48</v>
+        <v>103.37</v>
       </c>
       <c r="C180" t="n">
-        <v>54.49</v>
+        <v>105.25</v>
       </c>
       <c r="D180" t="n">
-        <v>1.89</v>
+        <v>1.82</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>22.92</v>
+        <v>25.42</v>
       </c>
       <c r="C181" t="n">
-        <v>23.35</v>
+        <v>25.88</v>
       </c>
       <c r="D181" t="n">
-        <v>1.88</v>
+        <v>1.81</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>MCLEODRUSS</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>37.3</v>
+        <v>48.03</v>
       </c>
       <c r="C182" t="n">
-        <v>38</v>
+        <v>48.9</v>
       </c>
       <c r="D182" t="n">
-        <v>1.88</v>
+        <v>1.81</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>LATTEYS</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>12.83</v>
+        <v>21.01</v>
       </c>
       <c r="C183" t="n">
-        <v>13.07</v>
+        <v>21.39</v>
       </c>
       <c r="D183" t="n">
-        <v>1.87</v>
+        <v>1.81</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MODIS</t>
+          <t>BRAHMINFRA</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>417.25</v>
+        <v>161.12</v>
       </c>
       <c r="C184" t="n">
-        <v>425</v>
+        <v>164</v>
       </c>
       <c r="D184" t="n">
-        <v>1.86</v>
+        <v>1.79</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>LATTEYS</t>
+          <t>MKPL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>20.02</v>
+        <v>3.93</v>
       </c>
       <c r="C185" t="n">
-        <v>20.39</v>
+        <v>4</v>
       </c>
       <c r="D185" t="n">
-        <v>1.85</v>
+        <v>1.78</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>CEINSYS</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>17.86</v>
+        <v>657.6</v>
       </c>
       <c r="C186" t="n">
-        <v>18.19</v>
+        <v>668.95</v>
       </c>
       <c r="D186" t="n">
-        <v>1.85</v>
+        <v>1.73</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>LANCER</t>
+          <t>BIOFILCHEM</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>10.79</v>
+        <v>30.18</v>
       </c>
       <c r="C187" t="n">
-        <v>10.99</v>
+        <v>30.7</v>
       </c>
       <c r="D187" t="n">
-        <v>1.85</v>
+        <v>1.72</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SUDARCOLOR</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>362.35</v>
+        <v>1375.4</v>
       </c>
       <c r="C188" t="n">
-        <v>369</v>
+        <v>1398.9</v>
       </c>
       <c r="D188" t="n">
-        <v>1.84</v>
+        <v>1.71</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>BHARATCOAL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>604.85</v>
+        <v>31.11</v>
       </c>
       <c r="C189" t="n">
-        <v>616</v>
+        <v>31.64</v>
       </c>
       <c r="D189" t="n">
-        <v>1.84</v>
+        <v>1.7</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>1223</v>
+        <v>25.27</v>
       </c>
       <c r="C190" t="n">
-        <v>1245.4</v>
+        <v>25.7</v>
       </c>
       <c r="D190" t="n">
-        <v>1.83</v>
+        <v>1.7</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>355.5</v>
+        <v>146.46</v>
       </c>
       <c r="C191" t="n">
-        <v>362</v>
+        <v>148.95</v>
       </c>
       <c r="D191" t="n">
-        <v>1.83</v>
+        <v>1.7</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>ROSSELLIND</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>6.08</v>
+        <v>51.62</v>
       </c>
       <c r="C192" t="n">
-        <v>6.19</v>
+        <v>52.49</v>
       </c>
       <c r="D192" t="n">
-        <v>1.81</v>
+        <v>1.69</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>TRF</t>
+          <t>KAYA</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>227.89</v>
+        <v>311.75</v>
       </c>
       <c r="C193" t="n">
-        <v>231.99</v>
+        <v>317</v>
       </c>
       <c r="D193" t="n">
-        <v>1.8</v>
+        <v>1.68</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>VIVOBIOT</t>
+          <t>PARSVNATH</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>14.43</v>
+        <v>2.41</v>
       </c>
       <c r="C194" t="n">
-        <v>14.69</v>
+        <v>2.45</v>
       </c>
       <c r="D194" t="n">
-        <v>1.8</v>
+        <v>1.66</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>OMFREIGHT</t>
+          <t>KICL</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>107.97</v>
+        <v>4867.3</v>
       </c>
       <c r="C195" t="n">
-        <v>109.9</v>
+        <v>4948</v>
       </c>
       <c r="D195" t="n">
-        <v>1.79</v>
+        <v>1.66</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>19.15</v>
+        <v>190.82</v>
       </c>
       <c r="C196" t="n">
-        <v>19.49</v>
+        <v>193.99</v>
       </c>
       <c r="D196" t="n">
-        <v>1.78</v>
+        <v>1.66</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>AZAD</t>
+          <t>AGOL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>2968.4</v>
+        <v>4.85</v>
       </c>
       <c r="C197" t="n">
-        <v>3021.1</v>
+        <v>4.93</v>
       </c>
       <c r="D197" t="n">
-        <v>1.78</v>
+        <v>1.65</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>MANAKSIA</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>57.76</v>
+        <v>168.14</v>
       </c>
       <c r="C198" t="n">
-        <v>58.79</v>
+        <v>170.9</v>
       </c>
       <c r="D198" t="n">
-        <v>1.78</v>
+        <v>1.64</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>VGUARD</t>
+          <t>DRAGARWQ</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>288.9</v>
+        <v>5136</v>
       </c>
       <c r="C199" t="n">
-        <v>294</v>
+        <v>5220</v>
       </c>
       <c r="D199" t="n">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>HTMEDIA</t>
+          <t>ALICON</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>23.18</v>
+        <v>865.8</v>
       </c>
       <c r="C200" t="n">
-        <v>23.59</v>
+        <v>880</v>
       </c>
       <c r="D200" t="n">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>148.79</v>
+        <v>5.5</v>
       </c>
       <c r="C201" t="n">
-        <v>151.4</v>
+        <v>5.59</v>
       </c>
       <c r="D201" t="n">
-        <v>1.75</v>
+        <v>1.64</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-15 08:36 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>PBMPOLY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>730</v>
+        <v>67.33</v>
       </c>
       <c r="C2" t="n">
-        <v>862.45</v>
+        <v>77</v>
       </c>
       <c r="D2" t="n">
-        <v>18.14</v>
+        <v>14.36</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>52.11</v>
+        <v>876</v>
       </c>
       <c r="C3" t="n">
-        <v>58.99</v>
+        <v>976</v>
       </c>
       <c r="D3" t="n">
-        <v>13.2</v>
+        <v>11.42</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PBMPOLY</t>
+          <t>MODINATUR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>56.11</v>
+        <v>325.5</v>
       </c>
       <c r="C4" t="n">
-        <v>62.9</v>
+        <v>360</v>
       </c>
       <c r="D4" t="n">
-        <v>12.1</v>
+        <v>10.6</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TARIL</t>
+          <t>THELEELA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>304</v>
+        <v>591.3</v>
       </c>
       <c r="C5" t="n">
-        <v>333</v>
+        <v>650.4</v>
       </c>
       <c r="D5" t="n">
-        <v>9.539999999999999</v>
+        <v>9.99</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>HPIL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.35</v>
+        <v>132.26</v>
       </c>
       <c r="C6" t="n">
-        <v>5.85</v>
+        <v>143</v>
       </c>
       <c r="D6" t="n">
-        <v>9.35</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KKJEWELS</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148</v>
+        <v>21.67</v>
       </c>
       <c r="C7" t="n">
-        <v>159.7</v>
+        <v>23.42</v>
       </c>
       <c r="D7" t="n">
-        <v>7.91</v>
+        <v>8.08</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.13</v>
+        <v>4.71</v>
       </c>
       <c r="C8" t="n">
-        <v>0.14</v>
+        <v>5.05</v>
       </c>
       <c r="D8" t="n">
-        <v>7.69</v>
+        <v>7.22</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ARTNIRMAN</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>43.71</v>
+        <v>0.14</v>
       </c>
       <c r="C9" t="n">
-        <v>47</v>
+        <v>0.15</v>
       </c>
       <c r="D9" t="n">
-        <v>7.53</v>
+        <v>7.14</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>361.95</v>
+        <v>108.75</v>
       </c>
       <c r="C10" t="n">
-        <v>387.9</v>
+        <v>116.35</v>
       </c>
       <c r="D10" t="n">
-        <v>7.17</v>
+        <v>6.99</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>IPHL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23.06</v>
+        <v>75.8</v>
       </c>
       <c r="C11" t="n">
-        <v>24.7</v>
+        <v>81</v>
       </c>
       <c r="D11" t="n">
-        <v>7.11</v>
+        <v>6.86</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SAPPL</t>
+          <t>TERAI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>354.95</v>
+        <v>139.18</v>
       </c>
       <c r="C12" t="n">
-        <v>379.95</v>
+        <v>148.7</v>
       </c>
       <c r="D12" t="n">
-        <v>7.04</v>
+        <v>6.84</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>GERMAN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9.84</v>
+        <v>123.03</v>
       </c>
       <c r="C13" t="n">
-        <v>10.42</v>
+        <v>131.3</v>
       </c>
       <c r="D13" t="n">
-        <v>5.89</v>
+        <v>6.72</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AVPINFRA</t>
+          <t>GODAVARIB</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65.05</v>
+        <v>228.62</v>
       </c>
       <c r="C14" t="n">
-        <v>68.8</v>
+        <v>243</v>
       </c>
       <c r="D14" t="n">
-        <v>5.76</v>
+        <v>6.29</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KANCOTEA</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>61.51</v>
+        <v>38.59</v>
       </c>
       <c r="C15" t="n">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="D15" t="n">
-        <v>5.67</v>
+        <v>6.25</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>NSLNISP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.18</v>
+        <v>39.63</v>
       </c>
       <c r="C16" t="n">
-        <v>0.19</v>
+        <v>42</v>
       </c>
       <c r="D16" t="n">
-        <v>5.56</v>
+        <v>5.98</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TRF</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>214.83</v>
+        <v>688.6</v>
       </c>
       <c r="C17" t="n">
-        <v>226.1</v>
+        <v>723</v>
       </c>
       <c r="D17" t="n">
-        <v>5.25</v>
+        <v>5</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>OPTIVALUE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>18.05</v>
+        <v>231</v>
       </c>
       <c r="C18" t="n">
-        <v>18.96</v>
+        <v>242.55</v>
       </c>
       <c r="D18" t="n">
-        <v>5.04</v>
+        <v>5</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,14 +835,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>KORE</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373.25</v>
+        <v>256.25</v>
       </c>
       <c r="C19" t="n">
-        <v>391.9</v>
+        <v>269.05</v>
       </c>
       <c r="D19" t="n">
         <v>5</v>
@@ -857,14 +857,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GSPLTRANS</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>112.51</v>
+        <v>200.87</v>
       </c>
       <c r="C20" t="n">
-        <v>118.13</v>
+        <v>210.91</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
@@ -879,14 +879,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ASSAMENT</t>
+          <t>AMBANIORGO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>784.65</v>
+        <v>154</v>
       </c>
       <c r="C21" t="n">
-        <v>823.85</v>
+        <v>161.7</v>
       </c>
       <c r="D21" t="n">
         <v>5</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KORE</t>
+          <t>GULFPETRO</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>244.05</v>
+        <v>65.98</v>
       </c>
       <c r="C22" t="n">
-        <v>256.25</v>
+        <v>69.27</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,14 +923,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BMISL</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>153.35</v>
+        <v>391.9</v>
       </c>
       <c r="C23" t="n">
-        <v>161</v>
+        <v>411.45</v>
       </c>
       <c r="D23" t="n">
         <v>4.99</v>
@@ -945,14 +945,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AKANKSHA</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>186.3</v>
+        <v>32.86</v>
       </c>
       <c r="C24" t="n">
-        <v>195.6</v>
+        <v>34.5</v>
       </c>
       <c r="D24" t="n">
         <v>4.99</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>14.83</v>
+        <v>39.78</v>
       </c>
       <c r="C25" t="n">
-        <v>15.57</v>
+        <v>41.76</v>
       </c>
       <c r="D25" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>37.9</v>
+        <v>50.2</v>
       </c>
       <c r="C26" t="n">
-        <v>39.79</v>
+        <v>52.7</v>
       </c>
       <c r="D26" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>UNIVPHOTO</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>470.7</v>
+        <v>3.62</v>
       </c>
       <c r="C27" t="n">
-        <v>494.2</v>
+        <v>3.8</v>
       </c>
       <c r="D27" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>COREIN</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>110.45</v>
+        <v>15.75</v>
       </c>
       <c r="C28" t="n">
-        <v>115.95</v>
+        <v>16.53</v>
       </c>
       <c r="D28" t="n">
-        <v>4.98</v>
+        <v>4.95</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>36.01</v>
+        <v>15.57</v>
       </c>
       <c r="C29" t="n">
-        <v>37.8</v>
+        <v>16.34</v>
       </c>
       <c r="D29" t="n">
-        <v>4.97</v>
+        <v>4.95</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>DELAPLEX</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2.42</v>
+        <v>148.85</v>
       </c>
       <c r="C30" t="n">
-        <v>2.54</v>
+        <v>156.2</v>
       </c>
       <c r="D30" t="n">
-        <v>4.96</v>
+        <v>4.94</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,14 +1099,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DIGJAMLMTD</t>
+          <t>GSMFOILS</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>52.41</v>
+        <v>66.8</v>
       </c>
       <c r="C31" t="n">
-        <v>55</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="D31" t="n">
         <v>4.94</v>
@@ -1121,14 +1121,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LEENEE</t>
+          <t>ROXHITECH</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7.1</v>
+        <v>73</v>
       </c>
       <c r="C32" t="n">
-        <v>7.45</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="D32" t="n">
         <v>4.93</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NEWJAISA</t>
+          <t>BMISL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>15.25</v>
+        <v>161</v>
       </c>
       <c r="C33" t="n">
-        <v>16</v>
+        <v>168.9</v>
       </c>
       <c r="D33" t="n">
-        <v>4.92</v>
+        <v>4.91</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>PALREDTEC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>47.85</v>
+        <v>45.2</v>
       </c>
       <c r="C34" t="n">
-        <v>50.2</v>
+        <v>47.4</v>
       </c>
       <c r="D34" t="n">
-        <v>4.91</v>
+        <v>4.87</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>KJMCFIN</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>57.22</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="C35" t="n">
-        <v>60</v>
+        <v>67.25</v>
       </c>
       <c r="D35" t="n">
-        <v>4.86</v>
+        <v>4.83</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3.72</v>
+        <v>2.33</v>
       </c>
       <c r="C36" t="n">
-        <v>3.9</v>
+        <v>2.44</v>
       </c>
       <c r="D36" t="n">
-        <v>4.84</v>
+        <v>4.72</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>5.81</v>
+        <v>2.54</v>
       </c>
       <c r="C37" t="n">
-        <v>6.09</v>
+        <v>2.66</v>
       </c>
       <c r="D37" t="n">
-        <v>4.82</v>
+        <v>4.72</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>64.76000000000001</v>
+        <v>1.71</v>
       </c>
       <c r="C38" t="n">
-        <v>67.8</v>
+        <v>1.79</v>
       </c>
       <c r="D38" t="n">
-        <v>4.69</v>
+        <v>4.68</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,14 +1275,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4.91</v>
+        <v>56.36</v>
       </c>
       <c r="C39" t="n">
-        <v>5.14</v>
+        <v>59</v>
       </c>
       <c r="D39" t="n">
         <v>4.68</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1.71</v>
+        <v>11.66</v>
       </c>
       <c r="C40" t="n">
-        <v>1.79</v>
+        <v>12.2</v>
       </c>
       <c r="D40" t="n">
-        <v>4.68</v>
+        <v>4.63</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>13.38</v>
+        <v>3.9</v>
       </c>
       <c r="C41" t="n">
-        <v>13.99</v>
+        <v>4.08</v>
       </c>
       <c r="D41" t="n">
-        <v>4.56</v>
+        <v>4.62</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GULFPETRO</t>
+          <t>21STCENMGM</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>62.84</v>
+        <v>42.49</v>
       </c>
       <c r="C42" t="n">
-        <v>65.7</v>
+        <v>44.44</v>
       </c>
       <c r="D42" t="n">
-        <v>4.55</v>
+        <v>4.59</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ESCONET</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>263.7</v>
+        <v>7.91</v>
       </c>
       <c r="C43" t="n">
-        <v>275.45</v>
+        <v>8.27</v>
       </c>
       <c r="D43" t="n">
-        <v>4.46</v>
+        <v>4.55</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>NAHARCAP</t>
+          <t>KLL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>234.49</v>
+        <v>41.45</v>
       </c>
       <c r="C44" t="n">
-        <v>244.8</v>
+        <v>43.3</v>
       </c>
       <c r="D44" t="n">
-        <v>4.4</v>
+        <v>4.46</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>7.98</v>
+        <v>16.14</v>
       </c>
       <c r="C45" t="n">
-        <v>8.33</v>
+        <v>16.86</v>
       </c>
       <c r="D45" t="n">
-        <v>4.39</v>
+        <v>4.46</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>57.35</v>
+        <v>11.11</v>
       </c>
       <c r="C46" t="n">
-        <v>59.85</v>
+        <v>11.59</v>
       </c>
       <c r="D46" t="n">
-        <v>4.36</v>
+        <v>4.32</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>TRANSWORLD</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.23</v>
+        <v>159.93</v>
       </c>
       <c r="C47" t="n">
-        <v>0.24</v>
+        <v>166.5</v>
       </c>
       <c r="D47" t="n">
-        <v>4.35</v>
+        <v>4.11</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>CRSL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>6.04</v>
+        <v>1.96</v>
       </c>
       <c r="C48" t="n">
-        <v>6.3</v>
+        <v>2.04</v>
       </c>
       <c r="D48" t="n">
-        <v>4.3</v>
+        <v>4.08</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NARMADA</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>10.75</v>
+        <v>8.35</v>
       </c>
       <c r="C49" t="n">
-        <v>11.2</v>
+        <v>8.68</v>
       </c>
       <c r="D49" t="n">
-        <v>4.19</v>
+        <v>3.95</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>KALYANIFRG</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>835.15</v>
+        <v>162.5</v>
       </c>
       <c r="C50" t="n">
-        <v>868.85</v>
+        <v>168.9</v>
       </c>
       <c r="D50" t="n">
-        <v>4.04</v>
+        <v>3.94</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CTE</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>37.5</v>
+        <v>58.48</v>
       </c>
       <c r="C51" t="n">
-        <v>39</v>
+        <v>60.78</v>
       </c>
       <c r="D51" t="n">
-        <v>4</v>
+        <v>3.93</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SIEL</t>
+          <t>ALFREDHE</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>29.81</v>
+        <v>2721</v>
       </c>
       <c r="C52" t="n">
-        <v>31</v>
+        <v>2828</v>
       </c>
       <c r="D52" t="n">
-        <v>3.99</v>
+        <v>3.93</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3.26</v>
+        <v>0.77</v>
       </c>
       <c r="C53" t="n">
-        <v>3.39</v>
+        <v>0.8</v>
       </c>
       <c r="D53" t="n">
-        <v>3.99</v>
+        <v>3.9</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>ATALREAL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>27.28</v>
+        <v>11.84</v>
       </c>
       <c r="C54" t="n">
-        <v>28.35</v>
+        <v>12.3</v>
       </c>
       <c r="D54" t="n">
-        <v>3.92</v>
+        <v>3.89</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SAYAJIHOTL</t>
+          <t>ARIES</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>302.95</v>
+        <v>479.9</v>
       </c>
       <c r="C55" t="n">
-        <v>314.8</v>
+        <v>498.5</v>
       </c>
       <c r="D55" t="n">
-        <v>3.91</v>
+        <v>3.88</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>HEROMOTORS</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>155.19</v>
+        <v>1713</v>
       </c>
       <c r="C56" t="n">
-        <v>161</v>
+        <v>1779.1</v>
       </c>
       <c r="D56" t="n">
-        <v>3.74</v>
+        <v>3.86</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>INDIANCARD</t>
+          <t>TECHLABS</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>189.97</v>
+        <v>105.35</v>
       </c>
       <c r="C57" t="n">
-        <v>197</v>
+        <v>109.4</v>
       </c>
       <c r="D57" t="n">
-        <v>3.7</v>
+        <v>3.84</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ANSALBU</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>83.93000000000001</v>
+        <v>14.88</v>
       </c>
       <c r="C58" t="n">
-        <v>86.98999999999999</v>
+        <v>15.45</v>
       </c>
       <c r="D58" t="n">
-        <v>3.65</v>
+        <v>3.83</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AGASTYAEN</t>
+          <t>ADISOFT</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>69.33</v>
+        <v>302.4</v>
       </c>
       <c r="C59" t="n">
-        <v>71.84999999999999</v>
+        <v>313.95</v>
       </c>
       <c r="D59" t="n">
-        <v>3.63</v>
+        <v>3.82</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>KOTYARK</t>
+          <t>NATIONSTD</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>33.53</v>
+        <v>105.86</v>
       </c>
       <c r="C60" t="n">
-        <v>34.74</v>
+        <v>109.9</v>
       </c>
       <c r="D60" t="n">
-        <v>3.61</v>
+        <v>3.82</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>28.4</v>
+        <v>250.45</v>
       </c>
       <c r="C61" t="n">
-        <v>29.39</v>
+        <v>260</v>
       </c>
       <c r="D61" t="n">
-        <v>3.49</v>
+        <v>3.81</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PHOENXINTL</t>
+          <t>BSHSL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>40.12</v>
+        <v>95.42</v>
       </c>
       <c r="C62" t="n">
-        <v>41.5</v>
+        <v>99</v>
       </c>
       <c r="D62" t="n">
-        <v>3.44</v>
+        <v>3.75</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>21STCENMGM</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>42.06</v>
+        <v>152.21</v>
       </c>
       <c r="C63" t="n">
-        <v>43.5</v>
+        <v>157.79</v>
       </c>
       <c r="D63" t="n">
-        <v>3.42</v>
+        <v>3.67</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>NKIND</t>
+          <t>ARVEE</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>60.99</v>
+        <v>216.11</v>
       </c>
       <c r="C64" t="n">
-        <v>63</v>
+        <v>224</v>
       </c>
       <c r="D64" t="n">
-        <v>3.3</v>
+        <v>3.65</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GSMFOILS</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>63.65</v>
+        <v>181.21</v>
       </c>
       <c r="C65" t="n">
-        <v>65.75</v>
+        <v>187.75</v>
       </c>
       <c r="D65" t="n">
-        <v>3.3</v>
+        <v>3.61</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GENCON</t>
+          <t>VISHAL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>35.75</v>
+        <v>17.17</v>
       </c>
       <c r="C66" t="n">
-        <v>36.9</v>
+        <v>17.79</v>
       </c>
       <c r="D66" t="n">
-        <v>3.22</v>
+        <v>3.61</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>20.98</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="C67" t="n">
-        <v>21.65</v>
+        <v>0.58</v>
       </c>
       <c r="D67" t="n">
-        <v>3.19</v>
+        <v>3.57</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>TCL</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>3.53</v>
+        <v>128.05</v>
       </c>
       <c r="C68" t="n">
-        <v>3.64</v>
+        <v>132.5</v>
       </c>
       <c r="D68" t="n">
-        <v>3.12</v>
+        <v>3.48</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>EEPL</t>
+          <t>COREIN</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>153.9</v>
+        <v>115.95</v>
       </c>
       <c r="C69" t="n">
-        <v>158.65</v>
+        <v>119.95</v>
       </c>
       <c r="D69" t="n">
-        <v>3.09</v>
+        <v>3.45</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>8.140000000000001</v>
+        <v>6.77</v>
       </c>
       <c r="C70" t="n">
-        <v>8.390000000000001</v>
+        <v>7</v>
       </c>
       <c r="D70" t="n">
-        <v>3.07</v>
+        <v>3.4</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>272.69</v>
+        <v>184.98</v>
       </c>
       <c r="C71" t="n">
-        <v>281</v>
+        <v>191.2</v>
       </c>
       <c r="D71" t="n">
-        <v>3.05</v>
+        <v>3.36</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1.32</v>
+        <v>76.48</v>
       </c>
       <c r="C72" t="n">
-        <v>1.36</v>
+        <v>79.04000000000001</v>
       </c>
       <c r="D72" t="n">
-        <v>3.03</v>
+        <v>3.35</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>TOKYOPLAST</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.67</v>
+        <v>65.3</v>
       </c>
       <c r="C73" t="n">
-        <v>0.6899999999999999</v>
+        <v>67.48</v>
       </c>
       <c r="D73" t="n">
-        <v>2.99</v>
+        <v>3.34</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SSRETAIL</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>691.95</v>
+        <v>118.1</v>
       </c>
       <c r="C74" t="n">
-        <v>712.6</v>
+        <v>122</v>
       </c>
       <c r="D74" t="n">
-        <v>2.98</v>
+        <v>3.3</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DENORA</t>
+          <t>CKKRETAIL</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>700.1</v>
+        <v>180.05</v>
       </c>
       <c r="C75" t="n">
-        <v>720.45</v>
+        <v>186</v>
       </c>
       <c r="D75" t="n">
-        <v>2.91</v>
+        <v>3.3</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>ECOLINE</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>72.89</v>
+        <v>179.2</v>
       </c>
       <c r="C76" t="n">
-        <v>75</v>
+        <v>185</v>
       </c>
       <c r="D76" t="n">
-        <v>2.89</v>
+        <v>3.24</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>CEMPRO</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>64.67</v>
+        <v>1153.5</v>
       </c>
       <c r="C77" t="n">
-        <v>66.48999999999999</v>
+        <v>1190.2</v>
       </c>
       <c r="D77" t="n">
-        <v>2.81</v>
+        <v>3.18</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ADISOFT</t>
+          <t>AGOL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>288</v>
+        <v>4.78</v>
       </c>
       <c r="C78" t="n">
-        <v>296</v>
+        <v>4.93</v>
       </c>
       <c r="D78" t="n">
-        <v>2.78</v>
+        <v>3.14</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>65.06999999999999</v>
+        <v>1.28</v>
       </c>
       <c r="C79" t="n">
-        <v>66.88</v>
+        <v>1.32</v>
       </c>
       <c r="D79" t="n">
-        <v>2.78</v>
+        <v>3.13</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CSM</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>89.47</v>
+        <v>5.43</v>
       </c>
       <c r="C80" t="n">
-        <v>91.95</v>
+        <v>5.6</v>
       </c>
       <c r="D80" t="n">
-        <v>2.77</v>
+        <v>3.13</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ATALREAL</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>11.28</v>
+        <v>23.17</v>
       </c>
       <c r="C81" t="n">
-        <v>11.59</v>
+        <v>23.89</v>
       </c>
       <c r="D81" t="n">
-        <v>2.75</v>
+        <v>3.11</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>HILINFRA</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>52.06</v>
+        <v>2.91</v>
       </c>
       <c r="C82" t="n">
-        <v>53.49</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>2.75</v>
+        <v>3.09</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MADRASFERT</t>
+          <t>VRAJ</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>57.22</v>
+        <v>121.26</v>
       </c>
       <c r="C83" t="n">
-        <v>58.79</v>
+        <v>124.97</v>
       </c>
       <c r="D83" t="n">
-        <v>2.74</v>
+        <v>3.06</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MADHURKNIT</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>57.45</v>
+        <v>1.31</v>
       </c>
       <c r="C84" t="n">
-        <v>59</v>
+        <v>1.35</v>
       </c>
       <c r="D84" t="n">
-        <v>2.7</v>
+        <v>3.05</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>DEEP</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>36.47</v>
+        <v>39.79</v>
       </c>
       <c r="C85" t="n">
-        <v>37.45</v>
+        <v>41</v>
       </c>
       <c r="D85" t="n">
-        <v>2.69</v>
+        <v>3.04</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>MEDICAMEQ</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>3188.9</v>
+        <v>295.85</v>
       </c>
       <c r="C86" t="n">
-        <v>3274</v>
+        <v>304.75</v>
       </c>
       <c r="D86" t="n">
-        <v>2.67</v>
+        <v>3.01</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>DHOOTTRANS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>492.05</v>
+        <v>1471.7</v>
       </c>
       <c r="C87" t="n">
-        <v>505</v>
+        <v>1516</v>
       </c>
       <c r="D87" t="n">
-        <v>2.63</v>
+        <v>3.01</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>JSIPL</t>
+          <t>LYKALABS</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>167.42</v>
+        <v>79.63</v>
       </c>
       <c r="C88" t="n">
-        <v>171.8</v>
+        <v>82</v>
       </c>
       <c r="D88" t="n">
-        <v>2.62</v>
+        <v>2.98</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ECORECO</t>
+          <t>SWISSMLTRY</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>397.4</v>
+        <v>13.55</v>
       </c>
       <c r="C89" t="n">
-        <v>407.7</v>
+        <v>13.95</v>
       </c>
       <c r="D89" t="n">
-        <v>2.59</v>
+        <v>2.95</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>FASCINATE</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>102.63</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="C90" t="n">
-        <v>105.29</v>
+        <v>101.5</v>
       </c>
       <c r="D90" t="n">
-        <v>2.59</v>
+        <v>2.94</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PILANIINVS</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>3949.6</v>
+        <v>55.38</v>
       </c>
       <c r="C91" t="n">
-        <v>4049</v>
+        <v>57</v>
       </c>
       <c r="D91" t="n">
-        <v>2.52</v>
+        <v>2.93</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>54.29</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C92" t="n">
-        <v>55.65</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="D92" t="n">
-        <v>2.51</v>
+        <v>2.93</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>OMINFRAL</t>
+          <t>SHOPERSTOP</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>69.95999999999999</v>
+        <v>373.25</v>
       </c>
       <c r="C93" t="n">
-        <v>71.68000000000001</v>
+        <v>384</v>
       </c>
       <c r="D93" t="n">
-        <v>2.46</v>
+        <v>2.88</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>7.33</v>
+        <v>878</v>
       </c>
       <c r="C94" t="n">
-        <v>7.51</v>
+        <v>903</v>
       </c>
       <c r="D94" t="n">
-        <v>2.46</v>
+        <v>2.85</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>VTMLTD</t>
+          <t>ALPA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>41</v>
+        <v>57.39</v>
       </c>
       <c r="C95" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="D95" t="n">
-        <v>2.44</v>
+        <v>2.81</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>HMVL</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>77.90000000000001</v>
+        <v>5.69</v>
       </c>
       <c r="C96" t="n">
-        <v>79.79000000000001</v>
+        <v>5.85</v>
       </c>
       <c r="D96" t="n">
-        <v>2.43</v>
+        <v>2.81</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>ADVANCE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>34.12</v>
+        <v>155.67</v>
       </c>
       <c r="C97" t="n">
-        <v>34.95</v>
+        <v>160</v>
       </c>
       <c r="D97" t="n">
-        <v>2.43</v>
+        <v>2.78</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>EMKAY</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>269.45</v>
+        <v>70.84</v>
       </c>
       <c r="C98" t="n">
-        <v>275.9</v>
+        <v>72.8</v>
       </c>
       <c r="D98" t="n">
-        <v>2.39</v>
+        <v>2.77</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>BALKRISHNA</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>15.63</v>
+        <v>34.05</v>
       </c>
       <c r="C99" t="n">
-        <v>16</v>
+        <v>34.99</v>
       </c>
       <c r="D99" t="n">
-        <v>2.37</v>
+        <v>2.76</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>MAHEPC</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>76.02</v>
+        <v>99.36</v>
       </c>
       <c r="C100" t="n">
-        <v>77.8</v>
+        <v>102</v>
       </c>
       <c r="D100" t="n">
-        <v>2.34</v>
+        <v>2.66</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>AASTHA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>4.29</v>
+        <v>28.25</v>
       </c>
       <c r="C101" t="n">
-        <v>4.39</v>
+        <v>29</v>
       </c>
       <c r="D101" t="n">
-        <v>2.33</v>
+        <v>2.65</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>SONA</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>11.28</v>
+        <v>100.57</v>
       </c>
       <c r="C102" t="n">
-        <v>11.54</v>
+        <v>103.2</v>
       </c>
       <c r="D102" t="n">
-        <v>2.3</v>
+        <v>2.62</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>WEBELSOLAR</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>9.710000000000001</v>
+        <v>69.09</v>
       </c>
       <c r="C103" t="n">
-        <v>9.93</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="D103" t="n">
-        <v>2.27</v>
+        <v>2.62</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>AFIL</t>
+          <t>PHOENXINTL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>8.01</v>
+        <v>42.88</v>
       </c>
       <c r="C104" t="n">
-        <v>8.19</v>
+        <v>43.99</v>
       </c>
       <c r="D104" t="n">
-        <v>2.25</v>
+        <v>2.59</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IDBI</t>
+          <t>EMMVEE</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>82.94</v>
+        <v>299.4</v>
       </c>
       <c r="C105" t="n">
-        <v>84.8</v>
+        <v>307</v>
       </c>
       <c r="D105" t="n">
-        <v>2.24</v>
+        <v>2.54</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>INNOMET</t>
+          <t>BLUECLOUDS</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>264.05</v>
+        <v>20</v>
       </c>
       <c r="C106" t="n">
-        <v>269.9</v>
+        <v>20.5</v>
       </c>
       <c r="D106" t="n">
-        <v>2.22</v>
+        <v>2.5</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>VIRTUALG</t>
+          <t>AVPINFRA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.45</v>
+        <v>78.05</v>
       </c>
       <c r="C107" t="n">
-        <v>0.46</v>
+        <v>80</v>
       </c>
       <c r="D107" t="n">
-        <v>2.22</v>
+        <v>2.5</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>GANGESSECU</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>112.5</v>
+        <v>24.15</v>
       </c>
       <c r="C108" t="n">
-        <v>114.99</v>
+        <v>24.75</v>
       </c>
       <c r="D108" t="n">
-        <v>2.21</v>
+        <v>2.48</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ONEGLOBAL</t>
+          <t>MANAKSTEEL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>549.85</v>
+        <v>110.22</v>
       </c>
       <c r="C109" t="n">
-        <v>561.9</v>
+        <v>112.95</v>
       </c>
       <c r="D109" t="n">
-        <v>2.19</v>
+        <v>2.48</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>GTL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>5.47</v>
+        <v>6.52</v>
       </c>
       <c r="C110" t="n">
-        <v>5.59</v>
+        <v>6.68</v>
       </c>
       <c r="D110" t="n">
-        <v>2.19</v>
+        <v>2.45</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>11.44</v>
+        <v>91.27</v>
       </c>
       <c r="C111" t="n">
-        <v>11.69</v>
+        <v>93.5</v>
       </c>
       <c r="D111" t="n">
-        <v>2.19</v>
+        <v>2.44</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>HTEL</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>88.95999999999999</v>
+        <v>4.12</v>
       </c>
       <c r="C112" t="n">
-        <v>90.90000000000001</v>
+        <v>4.22</v>
       </c>
       <c r="D112" t="n">
-        <v>2.18</v>
+        <v>2.43</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.46</v>
+        <v>12.37</v>
       </c>
       <c r="C113" t="n">
-        <v>0.47</v>
+        <v>12.67</v>
       </c>
       <c r="D113" t="n">
-        <v>2.17</v>
+        <v>2.43</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>MINDTECK</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>1.84</v>
+        <v>145.27</v>
       </c>
       <c r="C114" t="n">
-        <v>1.88</v>
+        <v>148.8</v>
       </c>
       <c r="D114" t="n">
-        <v>2.17</v>
+        <v>2.43</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>PRISMX</t>
+          <t>SAIFL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.46</v>
+        <v>4.15</v>
       </c>
       <c r="C115" t="n">
-        <v>0.47</v>
+        <v>4.25</v>
       </c>
       <c r="D115" t="n">
-        <v>2.17</v>
+        <v>2.41</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ORIENTCER</t>
+          <t>NINSYS</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>43.06</v>
+        <v>820.35</v>
       </c>
       <c r="C116" t="n">
-        <v>43.99</v>
+        <v>840</v>
       </c>
       <c r="D116" t="n">
-        <v>2.16</v>
+        <v>2.4</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>MUKKA</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>49.43</v>
+        <v>28.81</v>
       </c>
       <c r="C117" t="n">
-        <v>50.5</v>
+        <v>29.5</v>
       </c>
       <c r="D117" t="n">
-        <v>2.16</v>
+        <v>2.4</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ANUHPHR</t>
+          <t>CSBBANK</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>81.27</v>
+        <v>321.3</v>
       </c>
       <c r="C118" t="n">
-        <v>83</v>
+        <v>329</v>
       </c>
       <c r="D118" t="n">
-        <v>2.13</v>
+        <v>2.4</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>CYBERMEDIA</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>15.46</v>
+        <v>17.99</v>
       </c>
       <c r="C119" t="n">
-        <v>15.79</v>
+        <v>18.42</v>
       </c>
       <c r="D119" t="n">
-        <v>2.13</v>
+        <v>2.39</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SANATHAN</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>533.4</v>
+        <v>31.26</v>
       </c>
       <c r="C120" t="n">
-        <v>544.7</v>
+        <v>32</v>
       </c>
       <c r="D120" t="n">
-        <v>2.12</v>
+        <v>2.37</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CRESTO</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>20.81</v>
+        <v>62.53</v>
       </c>
       <c r="C121" t="n">
-        <v>21.25</v>
+        <v>64</v>
       </c>
       <c r="D121" t="n">
-        <v>2.11</v>
+        <v>2.35</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>AHLUCONT</t>
+          <t>MRPL</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>565.2</v>
+        <v>185.26</v>
       </c>
       <c r="C122" t="n">
-        <v>577.1</v>
+        <v>189.6</v>
       </c>
       <c r="D122" t="n">
-        <v>2.11</v>
+        <v>2.34</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>MURUDCERA</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>7.15</v>
+        <v>27.72</v>
       </c>
       <c r="C123" t="n">
-        <v>7.3</v>
+        <v>28.37</v>
       </c>
       <c r="D123" t="n">
-        <v>2.1</v>
+        <v>2.34</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>SAKHTISUG</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>42.31</v>
+        <v>18.91</v>
       </c>
       <c r="C124" t="n">
-        <v>43.19</v>
+        <v>19.35</v>
       </c>
       <c r="D124" t="n">
-        <v>2.08</v>
+        <v>2.33</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RAMBHAJO</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>372.05</v>
+        <v>4.76</v>
       </c>
       <c r="C125" t="n">
-        <v>379.8</v>
+        <v>4.87</v>
       </c>
       <c r="D125" t="n">
-        <v>2.08</v>
+        <v>2.31</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>38</v>
+        <v>37.93</v>
       </c>
       <c r="C126" t="n">
-        <v>38.79</v>
+        <v>38.8</v>
       </c>
       <c r="D126" t="n">
-        <v>2.08</v>
+        <v>2.29</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>7.24</v>
+        <v>184.27</v>
       </c>
       <c r="C127" t="n">
-        <v>7.39</v>
+        <v>188.49</v>
       </c>
       <c r="D127" t="n">
-        <v>2.07</v>
+        <v>2.29</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SUMEDHA</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>43</v>
+        <v>6.25</v>
       </c>
       <c r="C128" t="n">
-        <v>43.89</v>
+        <v>6.39</v>
       </c>
       <c r="D128" t="n">
-        <v>2.07</v>
+        <v>2.24</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>RIIT</t>
+          <t>GRAVISSHO</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>121.5</v>
+        <v>31.8</v>
       </c>
       <c r="C129" t="n">
-        <v>124</v>
+        <v>32.5</v>
       </c>
       <c r="D129" t="n">
-        <v>2.06</v>
+        <v>2.2</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>KARMAENG</t>
+          <t>GPECO</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>34.68</v>
+        <v>410.55</v>
       </c>
       <c r="C130" t="n">
-        <v>35.39</v>
+        <v>419.45</v>
       </c>
       <c r="D130" t="n">
-        <v>2.05</v>
+        <v>2.17</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>RAMCOSYS</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>10.26</v>
+        <v>587.15</v>
       </c>
       <c r="C131" t="n">
-        <v>10.47</v>
+        <v>599.8</v>
       </c>
       <c r="D131" t="n">
-        <v>2.05</v>
+        <v>2.15</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CGCL</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>248.9</v>
+        <v>25.64</v>
       </c>
       <c r="C132" t="n">
-        <v>254</v>
+        <v>26.19</v>
       </c>
       <c r="D132" t="n">
-        <v>2.05</v>
+        <v>2.15</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>29.39</v>
+        <v>14.48</v>
       </c>
       <c r="C133" t="n">
-        <v>29.99</v>
+        <v>14.79</v>
       </c>
       <c r="D133" t="n">
-        <v>2.04</v>
+        <v>2.14</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LANCER</t>
+          <t>TEMBO</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>10.78</v>
+        <v>55.74</v>
       </c>
       <c r="C134" t="n">
-        <v>11</v>
+        <v>56.92</v>
       </c>
       <c r="D134" t="n">
-        <v>2.04</v>
+        <v>2.12</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>48.7</v>
+        <v>5019.5</v>
       </c>
       <c r="C135" t="n">
-        <v>49.69</v>
+        <v>5125</v>
       </c>
       <c r="D135" t="n">
-        <v>2.03</v>
+        <v>2.1</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>25.81</v>
+        <v>3.33</v>
       </c>
       <c r="C136" t="n">
-        <v>26.33</v>
+        <v>3.4</v>
       </c>
       <c r="D136" t="n">
-        <v>2.01</v>
+        <v>2.1</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>SWASTIKAIN</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1.99</v>
+        <v>214.52</v>
       </c>
       <c r="C137" t="n">
-        <v>2.03</v>
+        <v>219</v>
       </c>
       <c r="D137" t="n">
-        <v>2.01</v>
+        <v>2.09</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>VRAJ</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>119.39</v>
+        <v>5.77</v>
       </c>
       <c r="C138" t="n">
-        <v>121.79</v>
+        <v>5.89</v>
       </c>
       <c r="D138" t="n">
-        <v>2.01</v>
+        <v>2.08</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>TFL</t>
+          <t>ADROITIND</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>11.95</v>
+        <v>193.02</v>
       </c>
       <c r="C139" t="n">
-        <v>12.19</v>
+        <v>197</v>
       </c>
       <c r="D139" t="n">
-        <v>2.01</v>
+        <v>2.06</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>27.82</v>
+        <v>135.7</v>
       </c>
       <c r="C140" t="n">
-        <v>28.38</v>
+        <v>138.5</v>
       </c>
       <c r="D140" t="n">
-        <v>2.01</v>
+        <v>2.06</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>BEEKAY</t>
+          <t>UCOBANK</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>435.85</v>
+        <v>23.96</v>
       </c>
       <c r="C141" t="n">
-        <v>444.55</v>
+        <v>24.45</v>
       </c>
       <c r="D141" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>PARIN</t>
+          <t>CHEMCRUX</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>691.15</v>
+        <v>81.52</v>
       </c>
       <c r="C142" t="n">
-        <v>704.95</v>
+        <v>83.19</v>
       </c>
       <c r="D142" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>52.44</v>
+        <v>25.96</v>
       </c>
       <c r="C143" t="n">
-        <v>53.49</v>
+        <v>26.49</v>
       </c>
       <c r="D143" t="n">
-        <v>2</v>
+        <v>2.04</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>168.44</v>
+        <v>89.27</v>
       </c>
       <c r="C144" t="n">
-        <v>171.79</v>
+        <v>91.08</v>
       </c>
       <c r="D144" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RAJMET</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>3.01</v>
+        <v>190.64</v>
       </c>
       <c r="C145" t="n">
-        <v>3.07</v>
+        <v>194.49</v>
       </c>
       <c r="D145" t="n">
-        <v>1.99</v>
+        <v>2.02</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>BLUECLOUDS</t>
+          <t>LICI</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>19.59</v>
+        <v>394</v>
       </c>
       <c r="C146" t="n">
-        <v>19.98</v>
+        <v>401.9</v>
       </c>
       <c r="D146" t="n">
-        <v>1.99</v>
+        <v>2.01</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>AKASH</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>22.07</v>
+        <v>25.38</v>
       </c>
       <c r="C147" t="n">
-        <v>22.51</v>
+        <v>25.89</v>
       </c>
       <c r="D147" t="n">
-        <v>1.99</v>
+        <v>2.01</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CGVAK</t>
+          <t>MITCON</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>134.71</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="C148" t="n">
-        <v>137.39</v>
+        <v>78.59</v>
       </c>
       <c r="D148" t="n">
-        <v>1.99</v>
+        <v>2.01</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MUTHOOTCAP</t>
+          <t>MVELECTRO</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>211.8</v>
+        <v>977.6</v>
       </c>
       <c r="C149" t="n">
-        <v>215.99</v>
+        <v>997.15</v>
       </c>
       <c r="D149" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>15.17</v>
+        <v>0.5</v>
       </c>
       <c r="C150" t="n">
-        <v>15.47</v>
+        <v>0.51</v>
       </c>
       <c r="D150" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CRIZAC</t>
+          <t>ANUHPHR</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>157.77</v>
+        <v>87.16</v>
       </c>
       <c r="C151" t="n">
-        <v>160.9</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="D151" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MGEL</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>16.13</v>
+        <v>7.01</v>
       </c>
       <c r="C152" t="n">
-        <v>16.45</v>
+        <v>7.15</v>
       </c>
       <c r="D152" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SILINV</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>467.85</v>
+        <v>22.51</v>
       </c>
       <c r="C153" t="n">
-        <v>477</v>
+        <v>22.96</v>
       </c>
       <c r="D153" t="n">
-        <v>1.96</v>
+        <v>2</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SPLIL</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>28.04</v>
+        <v>1705.1</v>
       </c>
       <c r="C154" t="n">
-        <v>28.59</v>
+        <v>1739</v>
       </c>
       <c r="D154" t="n">
-        <v>1.96</v>
+        <v>1.99</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>BHAGCHEM</t>
+          <t>JYOTIRES</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>221.66</v>
+        <v>854.8</v>
       </c>
       <c r="C155" t="n">
-        <v>226</v>
+        <v>871.85</v>
       </c>
       <c r="D155" t="n">
-        <v>1.96</v>
+        <v>1.99</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>CRAVATEX</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>6.11</v>
+        <v>341.25</v>
       </c>
       <c r="C156" t="n">
-        <v>6.23</v>
+        <v>348.05</v>
       </c>
       <c r="D156" t="n">
-        <v>1.96</v>
+        <v>1.99</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>58.25</v>
+        <v>88.06</v>
       </c>
       <c r="C157" t="n">
-        <v>59.39</v>
+        <v>89.8</v>
       </c>
       <c r="D157" t="n">
-        <v>1.96</v>
+        <v>1.98</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>JOCIL</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>32.26</v>
+        <v>144.43</v>
       </c>
       <c r="C158" t="n">
-        <v>32.89</v>
+        <v>147.29</v>
       </c>
       <c r="D158" t="n">
-        <v>1.95</v>
+        <v>1.98</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MERCURYEV</t>
+          <t>ARCHIES</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>36.53</v>
+        <v>12.11</v>
       </c>
       <c r="C159" t="n">
-        <v>37.24</v>
+        <v>12.35</v>
       </c>
       <c r="D159" t="n">
-        <v>1.94</v>
+        <v>1.98</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>WEIZMANIND</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>71.41</v>
+        <v>217.59</v>
       </c>
       <c r="C160" t="n">
-        <v>72.79000000000001</v>
+        <v>221.9</v>
       </c>
       <c r="D160" t="n">
-        <v>1.93</v>
+        <v>1.98</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>SHRADHA</t>
+          <t>BATLIBOI</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>30.01</v>
+        <v>94.31999999999999</v>
       </c>
       <c r="C161" t="n">
-        <v>30.59</v>
+        <v>96.19</v>
       </c>
       <c r="D161" t="n">
-        <v>1.93</v>
+        <v>1.98</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>15</v>
+        <v>6.07</v>
       </c>
       <c r="C162" t="n">
-        <v>15.29</v>
+        <v>6.19</v>
       </c>
       <c r="D162" t="n">
-        <v>1.93</v>
+        <v>1.98</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>AUSTENG</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>439.45</v>
+        <v>148.96</v>
       </c>
       <c r="C163" t="n">
-        <v>447.9</v>
+        <v>151.89</v>
       </c>
       <c r="D163" t="n">
-        <v>1.92</v>
+        <v>1.97</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>AARON</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>1137.3</v>
+        <v>130.72</v>
       </c>
       <c r="C164" t="n">
-        <v>1159</v>
+        <v>133.29</v>
       </c>
       <c r="D164" t="n">
-        <v>1.91</v>
+        <v>1.97</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HIMALAYAN</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>87.05</v>
+        <v>14.31</v>
       </c>
       <c r="C165" t="n">
-        <v>88.7</v>
+        <v>14.59</v>
       </c>
       <c r="D165" t="n">
-        <v>1.9</v>
+        <v>1.96</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>GKWLIMITED</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>1554.5</v>
+        <v>681.7</v>
       </c>
       <c r="C166" t="n">
-        <v>1584</v>
+        <v>694.9</v>
       </c>
       <c r="D166" t="n">
-        <v>1.9</v>
+        <v>1.94</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SIGNPOST</t>
+          <t>APTECHT</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>250.75</v>
+        <v>86.95</v>
       </c>
       <c r="C167" t="n">
-        <v>255.5</v>
+        <v>88.64</v>
       </c>
       <c r="D167" t="n">
-        <v>1.89</v>
+        <v>1.94</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>DOLLEX</t>
+          <t>PRISMX</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>36.49</v>
+        <v>0.52</v>
       </c>
       <c r="C168" t="n">
-        <v>37.18</v>
+        <v>0.53</v>
       </c>
       <c r="D168" t="n">
-        <v>1.89</v>
+        <v>1.92</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>REPRO</t>
+          <t>OSELDEVICE</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>312.05</v>
+        <v>363.7</v>
       </c>
       <c r="C169" t="n">
-        <v>317.95</v>
+        <v>370.65</v>
       </c>
       <c r="D169" t="n">
-        <v>1.89</v>
+        <v>1.91</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>15.4</v>
+        <v>22.76</v>
       </c>
       <c r="C170" t="n">
-        <v>15.69</v>
+        <v>23.19</v>
       </c>
       <c r="D170" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>SILGO</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>15.01</v>
+        <v>69.48</v>
       </c>
       <c r="C171" t="n">
-        <v>15.29</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="D171" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>ORIENTCER</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>23.06</v>
+        <v>43.57</v>
       </c>
       <c r="C172" t="n">
-        <v>23.49</v>
+        <v>44.39</v>
       </c>
       <c r="D172" t="n">
-        <v>1.86</v>
+        <v>1.88</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>CEMPRO</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>1138.8</v>
+        <v>3857.5</v>
       </c>
       <c r="C173" t="n">
-        <v>1160</v>
+        <v>3930</v>
       </c>
       <c r="D173" t="n">
-        <v>1.86</v>
+        <v>1.88</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>BLACKROSE</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>103.53</v>
+        <v>15.95</v>
       </c>
       <c r="C174" t="n">
-        <v>105.45</v>
+        <v>16.25</v>
       </c>
       <c r="D174" t="n">
-        <v>1.85</v>
+        <v>1.88</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>4.88</v>
+        <v>6.38</v>
       </c>
       <c r="C175" t="n">
-        <v>4.97</v>
+        <v>6.5</v>
       </c>
       <c r="D175" t="n">
-        <v>1.84</v>
+        <v>1.88</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MKEXIM</t>
+          <t>K2INFRA</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>55.97</v>
+        <v>40.15</v>
       </c>
       <c r="C176" t="n">
-        <v>57</v>
+        <v>40.9</v>
       </c>
       <c r="D176" t="n">
-        <v>1.84</v>
+        <v>1.87</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PAKKA</t>
+          <t>SHREYANIND</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>71.17</v>
+        <v>137.28</v>
       </c>
       <c r="C177" t="n">
-        <v>72.47</v>
+        <v>139.85</v>
       </c>
       <c r="D177" t="n">
-        <v>1.83</v>
+        <v>1.87</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>20.23</v>
+        <v>3.77</v>
       </c>
       <c r="C178" t="n">
-        <v>20.6</v>
+        <v>3.84</v>
       </c>
       <c r="D178" t="n">
-        <v>1.83</v>
+        <v>1.86</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>UDAYJEW</t>
+          <t>ESCONET</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>229.79</v>
+        <v>276.85</v>
       </c>
       <c r="C179" t="n">
-        <v>233.97</v>
+        <v>282</v>
       </c>
       <c r="D179" t="n">
-        <v>1.82</v>
+        <v>1.86</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>103.37</v>
+        <v>4.86</v>
       </c>
       <c r="C180" t="n">
-        <v>105.25</v>
+        <v>4.95</v>
       </c>
       <c r="D180" t="n">
-        <v>1.82</v>
+        <v>1.85</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>25.42</v>
+        <v>2304.9</v>
       </c>
       <c r="C181" t="n">
-        <v>25.88</v>
+        <v>2347.2</v>
       </c>
       <c r="D181" t="n">
-        <v>1.81</v>
+        <v>1.84</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MCLEODRUSS</t>
+          <t>MADHURKNIT</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>48.03</v>
+        <v>57.4</v>
       </c>
       <c r="C182" t="n">
-        <v>48.9</v>
+        <v>58.45</v>
       </c>
       <c r="D182" t="n">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>LATTEYS</t>
+          <t>ROSSELLIND</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>21.01</v>
+        <v>50.87</v>
       </c>
       <c r="C183" t="n">
-        <v>21.39</v>
+        <v>51.8</v>
       </c>
       <c r="D183" t="n">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>BRAHMINFRA</t>
+          <t>AUTOIND</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>161.12</v>
+        <v>81.17</v>
       </c>
       <c r="C184" t="n">
-        <v>164</v>
+        <v>82.65000000000001</v>
       </c>
       <c r="D184" t="n">
-        <v>1.79</v>
+        <v>1.82</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>SECURKLOUD</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>3.93</v>
+        <v>15.41</v>
       </c>
       <c r="C185" t="n">
-        <v>4</v>
+        <v>15.69</v>
       </c>
       <c r="D185" t="n">
-        <v>1.78</v>
+        <v>1.82</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>CEINSYS</t>
+          <t>LATTEYS</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>657.6</v>
+        <v>20.31</v>
       </c>
       <c r="C186" t="n">
-        <v>668.95</v>
+        <v>20.68</v>
       </c>
       <c r="D186" t="n">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>BIOFILCHEM</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>30.18</v>
+        <v>14.82</v>
       </c>
       <c r="C187" t="n">
-        <v>30.7</v>
+        <v>15.09</v>
       </c>
       <c r="D187" t="n">
-        <v>1.72</v>
+        <v>1.82</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>JAYSREETEA</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>1375.4</v>
+        <v>86.43000000000001</v>
       </c>
       <c r="C188" t="n">
-        <v>1398.9</v>
+        <v>87.98999999999999</v>
       </c>
       <c r="D188" t="n">
-        <v>1.71</v>
+        <v>1.8</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>BHARATCOAL</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>31.11</v>
+        <v>30.16</v>
       </c>
       <c r="C189" t="n">
-        <v>31.64</v>
+        <v>30.7</v>
       </c>
       <c r="D189" t="n">
-        <v>1.7</v>
+        <v>1.79</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>MAHASTEEL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>25.27</v>
+        <v>1117.9</v>
       </c>
       <c r="C190" t="n">
-        <v>25.7</v>
+        <v>1137.9</v>
       </c>
       <c r="D190" t="n">
-        <v>1.7</v>
+        <v>1.79</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>GREENPLY</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>146.46</v>
+        <v>318.3</v>
       </c>
       <c r="C191" t="n">
-        <v>148.95</v>
+        <v>324</v>
       </c>
       <c r="D191" t="n">
-        <v>1.7</v>
+        <v>1.79</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ROSSELLIND</t>
+          <t>AAATECH</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>51.62</v>
+        <v>111.57</v>
       </c>
       <c r="C192" t="n">
-        <v>52.49</v>
+        <v>113.57</v>
       </c>
       <c r="D192" t="n">
-        <v>1.69</v>
+        <v>1.79</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>KAYA</t>
+          <t>SURANAT&amp;P</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>311.75</v>
+        <v>15.32</v>
       </c>
       <c r="C193" t="n">
-        <v>317</v>
+        <v>15.59</v>
       </c>
       <c r="D193" t="n">
-        <v>1.68</v>
+        <v>1.76</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>2.41</v>
+        <v>2.3</v>
       </c>
       <c r="C194" t="n">
-        <v>2.45</v>
+        <v>2.34</v>
       </c>
       <c r="D194" t="n">
-        <v>1.66</v>
+        <v>1.74</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KICL</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>4867.3</v>
+        <v>6.37</v>
       </c>
       <c r="C195" t="n">
-        <v>4948</v>
+        <v>6.48</v>
       </c>
       <c r="D195" t="n">
-        <v>1.66</v>
+        <v>1.73</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>190.82</v>
+        <v>15.63</v>
       </c>
       <c r="C196" t="n">
-        <v>193.99</v>
+        <v>15.9</v>
       </c>
       <c r="D196" t="n">
-        <v>1.66</v>
+        <v>1.73</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>AGOL</t>
+          <t>DENTA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>4.85</v>
+        <v>263.45</v>
       </c>
       <c r="C197" t="n">
-        <v>4.93</v>
+        <v>267.95</v>
       </c>
       <c r="D197" t="n">
-        <v>1.65</v>
+        <v>1.71</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>168.14</v>
+        <v>11.11</v>
       </c>
       <c r="C198" t="n">
-        <v>170.9</v>
+        <v>11.3</v>
       </c>
       <c r="D198" t="n">
-        <v>1.64</v>
+        <v>1.71</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>DRAGARWQ</t>
+          <t>WARDINMOBI</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>5136</v>
+        <v>4.69</v>
       </c>
       <c r="C199" t="n">
-        <v>5220</v>
+        <v>4.77</v>
       </c>
       <c r="D199" t="n">
-        <v>1.64</v>
+        <v>1.71</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ALICON</t>
+          <t>DOLLEX</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>865.8</v>
+        <v>37.35</v>
       </c>
       <c r="C200" t="n">
-        <v>880</v>
+        <v>37.99</v>
       </c>
       <c r="D200" t="n">
-        <v>1.64</v>
+        <v>1.71</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>HLEGLAS</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>5.5</v>
+        <v>414.95</v>
       </c>
       <c r="C201" t="n">
-        <v>5.59</v>
+        <v>422.05</v>
       </c>
       <c r="D201" t="n">
-        <v>1.64</v>
+        <v>1.71</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-10-16 08:30 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PBMPOLY</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>67.33</v>
+        <v>21.76</v>
       </c>
       <c r="C2" t="n">
-        <v>77</v>
+        <v>23.9</v>
       </c>
       <c r="D2" t="n">
-        <v>14.36</v>
+        <v>9.83</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>POLYSPIN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>876</v>
+        <v>29.93</v>
       </c>
       <c r="C3" t="n">
-        <v>976</v>
+        <v>32.85</v>
       </c>
       <c r="D3" t="n">
-        <v>11.42</v>
+        <v>9.76</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MODINATUR</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c 